<commit_message>
Daily portfolio update 2026-05-14
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -35,6 +35,10 @@
       <sz val="11"/>
     </font>
     <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
       <color rgb="00006100"/>
     </font>
     <font>
@@ -43,10 +47,6 @@
     <font>
       <b val="1"/>
       <color rgb="00006100"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="10"/>
     </font>
     <font>
       <color rgb="009C0006"/>
@@ -93,18 +93,18 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -480,7 +480,7 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -493,7 +493,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-05-15 00:09 IST</t>
+          <t>Generated: 2026-05-14 18:41 IST</t>
         </is>
       </c>
     </row>
@@ -539,13 +539,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4569323.0469093</v>
+        <v>4590504.1621449</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>99323.04690929968</v>
+        <v>120504.1621449003</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.02221992100879187</v>
+        <v>0.02695842553577188</v>
       </c>
     </row>
     <row r="6">
@@ -561,10 +561,10 @@
         <v>0</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>563095</v>
+        <v>560183.001449585</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>563095</v>
+        <v>560183.001449585</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>0</v>
@@ -583,13 +583,13 @@
         <v>4470000</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5132418.0469093</v>
+        <v>5150687.163594485</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>662418.0469092997</v>
+        <v>680687.1635944853</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.1481919568029753</v>
+        <v>0.1522790075155448</v>
       </c>
     </row>
     <row r="8"/>
@@ -611,16 +611,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -659,6 +660,11 @@
           <t>P&amp;L (₹)</t>
         </is>
       </c>
+      <c r="H1" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -678,13 +684,16 @@
         <v>0</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>522.05</v>
+        <v>539.75</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>41764</v>
+        <v>43180</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>41764</v>
+        <v>43180</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>539.75</v>
       </c>
     </row>
     <row r="3">
@@ -732,13 +741,16 @@
         <v>0</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1530</v>
+        <v>1561.300048828125</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>30600</v>
+        <v>31226.0009765625</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>30600</v>
+        <v>31226.0009765625</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>1561.300048828125</v>
       </c>
     </row>
     <row r="5">
@@ -759,13 +771,16 @@
         <v>0</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>677.35</v>
+        <v>649.7999877929688</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13547</v>
+        <v>12995.99975585938</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>13547</v>
+        <v>12995.99975585938</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>649.7999877929688</v>
       </c>
     </row>
     <row r="6">
@@ -786,13 +801,16 @@
         <v>0</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>417.05</v>
+        <v>401</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>16682</v>
+        <v>16040</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>16682</v>
+        <v>16040</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>401</v>
       </c>
     </row>
     <row r="7">
@@ -813,13 +831,16 @@
         <v>0</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>251.95</v>
+        <v>254.0500030517578</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>25195</v>
+        <v>25405.00030517578</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>25195</v>
+        <v>25405.00030517578</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>254.0500030517578</v>
       </c>
     </row>
     <row r="8">
@@ -867,13 +888,16 @@
         <v>0</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>19.73</v>
+        <v>17.86000061035156</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>29595</v>
+        <v>26790.00091552734</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>29595</v>
+        <v>26790.00091552734</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>17.86000061035156</v>
       </c>
     </row>
     <row r="10">
@@ -894,13 +918,16 @@
         <v>0</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>490.85</v>
+        <v>517.5499877929688</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>49085</v>
+        <v>51754.99877929688</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>49085</v>
+        <v>51754.99877929688</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>517.5499877929688</v>
       </c>
     </row>
     <row r="11">
@@ -921,13 +948,16 @@
         <v>0</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>9.380000000000001</v>
+        <v>8.510000228881836</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>9380</v>
+        <v>8510.000228881836</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>9380</v>
+        <v>8510.000228881836</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>8.510000228881836</v>
       </c>
     </row>
     <row r="12">
@@ -948,13 +978,16 @@
         <v>0</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2642.4</v>
+        <v>2888.60009765625</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>26424</v>
+        <v>28886.0009765625</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>26424</v>
+        <v>28886.0009765625</v>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>2888.60009765625</v>
       </c>
     </row>
     <row r="13">
@@ -975,13 +1008,16 @@
         <v>0</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>55.65</v>
+        <v>53.47000122070312</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>33390</v>
+        <v>32082.00073242188</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>33390</v>
+        <v>32082.00073242188</v>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>53.47000122070312</v>
       </c>
     </row>
     <row r="14">
@@ -1002,13 +1038,16 @@
         <v>0</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>809.45</v>
+        <v>757.0999755859375</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>40472.5</v>
+        <v>37854.99877929688</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>40472.5</v>
+        <v>37854.99877929688</v>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>757.0999755859375</v>
       </c>
     </row>
     <row r="15">
@@ -1083,13 +1122,16 @@
         <v>0</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>414.7</v>
+        <v>458.0499877929688</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>20735</v>
+        <v>22902.49938964844</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>20735</v>
+        <v>22902.49938964844</v>
+      </c>
+      <c r="H17" s="3" t="n">
+        <v>458.0499877929688</v>
       </c>
     </row>
     <row r="18">
@@ -1110,17 +1152,20 @@
         <v>0</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>444.55</v>
+        <v>407.8500061035156</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>44455</v>
+        <v>40785.00061035156</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>44455</v>
+        <v>40785.00061035156</v>
+      </c>
+      <c r="H18" s="3" t="n">
+        <v>407.8500061035156</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -1129,10 +1174,10 @@
         <v>0</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>563095</v>
-      </c>
-      <c r="G19" s="8" t="n">
-        <v>563095</v>
+        <v>560183.001449585</v>
+      </c>
+      <c r="G19" s="9" t="n">
+        <v>560183.001449585</v>
       </c>
     </row>
   </sheetData>
@@ -1157,7 +1202,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -1207,7 +1252,7 @@
           <t>Returns %</t>
         </is>
       </c>
-      <c r="J1" s="9" t="inlineStr">
+      <c r="J1" s="7" t="inlineStr">
         <is>
           <t>2026-05-14</t>
         </is>
@@ -1350,19 +1395,19 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.4841</v>
+        <v>9.4939</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>174072.0060008</v>
+        <v>174251.8760632</v>
       </c>
       <c r="H5" s="12" t="n">
-        <v>-35927.9939992</v>
+        <v>-35748.1239368</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1710856857104762</v>
+        <v>-0.1702291616038095</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>9.4841</v>
+        <v>9.4939</v>
       </c>
     </row>
     <row r="6">
@@ -1388,19 +1433,19 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.4071</v>
+        <v>12.5421</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>52469.34053669999</v>
+        <v>53040.2524317</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>2469.340536699994</v>
+        <v>3040.252431699999</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.04938681073399988</v>
+        <v>0.06080504863399998</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>12.4071</v>
+        <v>12.5421</v>
       </c>
     </row>
     <row r="7">
@@ -1464,19 +1509,19 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>30.5654</v>
+        <v>30.6804</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>49045.0268822</v>
+        <v>49229.5550772</v>
       </c>
       <c r="H8" s="12" t="n">
-        <v>-954.9731178000002</v>
+        <v>-770.4449228000012</v>
       </c>
       <c r="I8" s="13" t="n">
-        <v>-0.019099462356</v>
+        <v>-0.01540889845600002</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>30.5654</v>
+        <v>30.6804</v>
       </c>
     </row>
     <row r="9">
@@ -1616,19 +1661,19 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>348.354</v>
+        <v>351.157</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>162166.450788</v>
+        <v>163471.308954</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>62166.45078799999</v>
+        <v>63471.30895399998</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.6216645078799998</v>
+        <v>0.6347130895399998</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>348.354</v>
+        <v>351.157</v>
       </c>
     </row>
     <row r="13">
@@ -1654,19 +1699,19 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>19.575</v>
+        <v>19.888</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>226827.367875</v>
+        <v>230454.28824</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>26827.367875</v>
+        <v>30454.28824000002</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0.134136839375</v>
+        <v>0.1522714412000001</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>19.575</v>
+        <v>19.888</v>
       </c>
     </row>
     <row r="14">
@@ -1730,19 +1775,19 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.67</v>
+        <v>11.76</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>113711.86149</v>
+        <v>114588.81672</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>13711.86149</v>
+        <v>14588.81672</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>0.1371186149</v>
+        <v>0.1458881672</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>11.67</v>
+        <v>11.76</v>
       </c>
     </row>
     <row r="16">
@@ -1844,19 +1889,19 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>44.57</v>
+        <v>45.31</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>84078.45251999999</v>
+        <v>85474.41516</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>4078.452519999992</v>
+        <v>5474.415160000004</v>
       </c>
       <c r="I18" s="11" t="n">
-        <v>0.05098065649999989</v>
+        <v>0.06843018950000006</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>44.57</v>
+        <v>45.31</v>
       </c>
     </row>
     <row r="19">
@@ -1958,19 +2003,19 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>106.9865</v>
+        <v>107.9031</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>162540.2030035</v>
+        <v>163932.7558029</v>
       </c>
       <c r="H21" s="12" t="n">
-        <v>-7459.796996499994</v>
+        <v>-6067.244197099993</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.04388115880294114</v>
+        <v>-0.03568967174764702</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>106.9865</v>
+        <v>107.9031</v>
       </c>
     </row>
     <row r="22">
@@ -2034,19 +2079,19 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>59.785</v>
+        <v>60.3775</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>162403.979595</v>
+        <v>164013.4862925</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>12403.97959499998</v>
+        <v>14013.48629249999</v>
       </c>
       <c r="I23" s="11" t="n">
-        <v>0.08269319729999988</v>
+        <v>0.09342324194999994</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>59.785</v>
+        <v>60.3775</v>
       </c>
     </row>
     <row r="24">
@@ -2072,19 +2117,19 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>9.6252</v>
+        <v>9.717599999999999</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>34972.0669272</v>
+        <v>35307.79179359999</v>
       </c>
       <c r="H24" s="12" t="n">
-        <v>-65027.9330728</v>
+        <v>-64692.20820640001</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>-0.650279330728</v>
+        <v>-0.646922082064</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>9.6252</v>
+        <v>9.717599999999999</v>
       </c>
     </row>
     <row r="25">
@@ -2110,19 +2155,19 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.1269</v>
+        <v>11.2082</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>182722.3244306</v>
+        <v>184057.4065268</v>
       </c>
       <c r="H25" s="12" t="n">
-        <v>-17277.67556940002</v>
+        <v>-15942.59347320002</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.08638837784700008</v>
+        <v>-0.07971296736600009</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>11.1269</v>
+        <v>11.2082</v>
       </c>
     </row>
     <row r="26">
@@ -2148,19 +2193,19 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>8.6471</v>
+        <v>8.626300000000001</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>103261.2037765</v>
+        <v>103012.8161045</v>
       </c>
       <c r="H26" s="12" t="n">
-        <v>-6738.796223500001</v>
+        <v>-6987.183895499998</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>-0.06126178385000002</v>
+        <v>-0.06351985359545453</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>8.6471</v>
+        <v>8.626300000000001</v>
       </c>
     </row>
     <row r="27">
@@ -2186,19 +2231,19 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>61.4158</v>
+        <v>62.0021</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>98932.25558799999</v>
+        <v>99876.70280599999</v>
       </c>
       <c r="H27" s="12" t="n">
-        <v>-11067.74441200001</v>
+        <v>-10123.29719400001</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.1006158582909092</v>
+        <v>-0.09202997449090922</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>61.4158</v>
+        <v>62.0021</v>
       </c>
     </row>
     <row r="28">
@@ -2224,19 +2269,19 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>38.0738</v>
+        <v>38.3133</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>125896.9972866</v>
+        <v>126688.9416381</v>
       </c>
       <c r="H28" s="12" t="n">
-        <v>-254103.0027134</v>
+        <v>-253311.0583619</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.6686921124036842</v>
+        <v>-0.6666080483207895</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>38.0738</v>
+        <v>38.3133</v>
       </c>
     </row>
     <row r="29">
@@ -2262,19 +2307,19 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.9232</v>
+        <v>12.0216</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>114506.8716096</v>
+        <v>115451.8759848</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>14506.87160959998</v>
+        <v>15451.87598479999</v>
       </c>
       <c r="I29" s="11" t="n">
-        <v>0.1450687160959998</v>
+        <v>0.1545187598479999</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>11.9232</v>
+        <v>12.0216</v>
       </c>
     </row>
     <row r="30">
@@ -2300,19 +2345,19 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>14.9789</v>
+        <v>15.064</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>110781.8623329</v>
+        <v>111411.250104</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>10781.8623329</v>
+        <v>11411.25010399999</v>
       </c>
       <c r="I30" s="11" t="n">
-        <v>0.107818623329</v>
+        <v>0.1141125010399999</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>14.9789</v>
+        <v>15.064</v>
       </c>
     </row>
     <row r="31">
@@ -2338,19 +2383,19 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>409.9345</v>
+        <v>413.2552</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>109075.37176</v>
+        <v>109958.943616</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>9075.371759999995</v>
+        <v>9958.94361599999</v>
       </c>
       <c r="I31" s="11" t="n">
-        <v>0.09075371759999995</v>
+        <v>0.09958943615999989</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>409.9345</v>
+        <v>413.2552</v>
       </c>
     </row>
     <row r="32">
@@ -2376,19 +2421,19 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.03</v>
+        <v>10.1</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>212033.7988</v>
+        <v>213513.596</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>12033.79879999999</v>
+        <v>13513.59599999999</v>
       </c>
       <c r="I32" s="11" t="n">
-        <v>0.06016899399999995</v>
+        <v>0.06756797999999996</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>10.03</v>
+        <v>10.1</v>
       </c>
     </row>
     <row r="33">
@@ -2414,19 +2459,19 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>17.66</v>
+        <v>17.77</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>63287.0824</v>
+        <v>63681.28279999999</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>3287.082399999999</v>
+        <v>3681.282799999994</v>
       </c>
       <c r="I33" s="11" t="n">
-        <v>0.05478470666666665</v>
+        <v>0.06135471333333323</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>17.66</v>
+        <v>17.77</v>
       </c>
     </row>
     <row r="34">
@@ -2490,19 +2535,19 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>13.63</v>
+        <v>13.81</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>97255.81549000001</v>
+        <v>98540.19163</v>
       </c>
       <c r="H35" s="12" t="n">
-        <v>-2744.184509999992</v>
+        <v>-1459.808369999999</v>
       </c>
       <c r="I35" s="13" t="n">
-        <v>-0.02744184509999992</v>
+        <v>-0.01459808369999999</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>13.63</v>
+        <v>13.81</v>
       </c>
     </row>
     <row r="36">
@@ -2566,19 +2611,19 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>15.395</v>
+        <v>15.6</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>57929.676155</v>
+        <v>58701.0684</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>7929.676155000001</v>
+        <v>8701.068400000004</v>
       </c>
       <c r="I37" s="11" t="n">
-        <v>0.1585935231</v>
+        <v>0.1740213680000001</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>15.395</v>
+        <v>15.6</v>
       </c>
     </row>
     <row r="38">
@@ -2680,23 +2725,23 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>19.8133</v>
+        <v>19.911</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>99879.38025910001</v>
-      </c>
-      <c r="H40" s="12" t="n">
-        <v>-120.6197408999869</v>
-      </c>
-      <c r="I40" s="13" t="n">
-        <v>-0.001206197408999869</v>
+        <v>100371.888597</v>
+      </c>
+      <c r="H40" s="4" t="n">
+        <v>371.8885970000119</v>
+      </c>
+      <c r="I40" s="11" t="n">
+        <v>0.00371888597000012</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>19.8133</v>
+        <v>19.911</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="7" t="inlineStr">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -2705,13 +2750,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4569323.0469093</v>
-      </c>
-      <c r="H41" s="8" t="n">
-        <v>99323.04690929991</v>
+        <v>4590504.1621449</v>
+      </c>
+      <c r="H41" s="9" t="n">
+        <v>120504.1621449</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.02221992100879193</v>
+        <v>0.02695842553577181</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-05-15
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -485,7 +485,7 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-05-14 18:59 IST</t>
+          <t>Generated: 2026-05-15 05:54 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4808002.0794846</v>
+        <v>4815000.4556386</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>338002.0794845996</v>
+        <v>345000.4556385996</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.0756156777370469</v>
+        <v>0.07718130998626389</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>560183.001449585</v>
+        <v>558353.4982757568</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-30599.01855041506</v>
+        <v>-32428.52172424318</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.05179409243093596</v>
+        <v>-0.05489084065937413</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5368185.080934185</v>
+        <v>5373353.953914356</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>307403.0609341851</v>
+        <v>312571.9339143569</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.06074220539816593</v>
+        <v>0.06176356394705119</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-05-14</t>
+          <t>Last snapshot: 2026-05-15</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -627,6 +627,7 @@
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -670,6 +671,11 @@
           <t>2026-05-14</t>
         </is>
       </c>
+      <c r="I1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -689,17 +695,20 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>539.75</v>
+        <v>547.0499877929688</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>43180</v>
+        <v>43763.9990234375</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>-637.510000000002</v>
+        <v>-53.51097656250204</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
       </c>
+      <c r="I2" s="3" t="n">
+        <v>547.0499877929688</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -746,17 +755,20 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1561.300048828125</v>
+        <v>1571.800048828125</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>31226.0009765625</v>
+        <v>31436.0009765625</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-878.5790234375017</v>
+        <v>-668.5790234375017</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
       </c>
+      <c r="I4" s="3" t="n">
+        <v>1571.800048828125</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -776,17 +788,20 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>649.7999877929688</v>
+        <v>667.9000244140625</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>12995.99975585938</v>
+        <v>13358.00048828125</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1217.100244140625</v>
+        <v>-855.0995117187504</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
       </c>
+      <c r="I5" s="3" t="n">
+        <v>667.9000244140625</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -806,17 +821,20 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>401</v>
+        <v>402.1000061035156</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>16040</v>
+        <v>16084.00024414062</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-1462.240000000002</v>
+        <v>-1418.239755859377</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
       </c>
+      <c r="I6" s="3" t="n">
+        <v>402.1000061035156</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -836,17 +854,20 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>254.0500030517578</v>
+        <v>248</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>25405.00030517578</v>
+        <v>24800</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-1028.819694824218</v>
+        <v>-1633.82</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
       </c>
+      <c r="I7" s="3" t="n">
+        <v>248</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -893,17 +914,20 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>17.86000061035156</v>
+        <v>17.6299991607666</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>26790.00091552734</v>
+        <v>26444.9987411499</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-4260.169084472655</v>
+        <v>-4605.171258850096</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
       </c>
+      <c r="I9" s="3" t="n">
+        <v>17.6299991607666</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -923,17 +947,20 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>517.5499877929688</v>
+        <v>518.2000122070312</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>51754.99877929688</v>
+        <v>51820.00122070312</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>256.5187792968718</v>
+        <v>321.5212207031218</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
       </c>
+      <c r="I10" s="3" t="n">
+        <v>518.2000122070312</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -953,17 +980,20 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>8.510000228881836</v>
+        <v>8.449999809265137</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>8510.000228881836</v>
+        <v>8449.999809265137</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-1331.209771118163</v>
+        <v>-1391.210190734862</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
       </c>
+      <c r="I11" s="3" t="n">
+        <v>8.449999809265137</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -983,17 +1013,20 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2888.60009765625</v>
+        <v>2738.89990234375</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>28886.0009765625</v>
-      </c>
-      <c r="G12" s="4" t="n">
-        <v>1162.7509765625</v>
+        <v>27388.9990234375</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>-334.2509765625</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
       </c>
+      <c r="I12" s="3" t="n">
+        <v>2738.89990234375</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1013,17 +1046,20 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>53.47000122070312</v>
+        <v>53.61999893188477</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>32082.00073242188</v>
+        <v>32171.99935913086</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-2949.759267578127</v>
+        <v>-2859.760640869143</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
       </c>
+      <c r="I13" s="3" t="n">
+        <v>53.61999893188477</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1043,17 +1079,20 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>757.0999755859375</v>
+        <v>748.7999877929688</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>37854.99877929688</v>
+        <v>37439.99938964844</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-4607.511220703127</v>
+        <v>-5022.510610351565</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
       </c>
+      <c r="I14" s="3" t="n">
+        <v>748.7999877929688</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1127,17 +1166,20 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>458.0499877929688</v>
+        <v>452</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>22902.49938964844</v>
+        <v>22600</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>1147.969389648439</v>
+        <v>845.4700000000012</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
       </c>
+      <c r="I17" s="3" t="n">
+        <v>452</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1157,17 +1199,20 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>407.8500061035156</v>
+        <v>408.25</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>40785.00061035156</v>
+        <v>40825</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-5855.819389648437</v>
+        <v>-5815.82</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
       </c>
+      <c r="I18" s="3" t="n">
+        <v>408.25</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -1179,10 +1224,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>560183.001449585</v>
+        <v>558353.4982757568</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-30599.01855041505</v>
+        <v>-32428.52172424318</v>
       </c>
     </row>
   </sheetData>
@@ -1196,7 +1241,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:K41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1209,6 +1254,7 @@
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1262,6 +1308,11 @@
           <t>2026-05-14</t>
         </is>
       </c>
+      <c r="K1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1286,20 +1337,23 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.7408</v>
+        <v>57.2873</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>63690.52666559999</v>
+        <v>64303.9630786</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>13690.52666559999</v>
+        <v>14303.9630786</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.2738105333119999</v>
+        <v>0.286079261572</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
       </c>
+      <c r="K2" s="3" t="n">
+        <v>57.2873</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1324,20 +1378,23 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.2746</v>
+        <v>25.5426</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>62054.5264898</v>
+        <v>62712.5235738</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>2054.526489800002</v>
+        <v>2712.523573800005</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.03424210816333337</v>
+        <v>0.04520872623000008</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
       </c>
+      <c r="K3" s="3" t="n">
+        <v>25.5426</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1362,20 +1419,23 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.93</v>
+        <v>12.97</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>248334.78249</v>
+        <v>249103.02621</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>68334.78249000001</v>
+        <v>69103.02621000001</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3796376805000001</v>
+        <v>0.3839057011666667</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
       </c>
+      <c r="K4" s="3" t="n">
+        <v>12.97</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1414,6 +1474,9 @@
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
       </c>
+      <c r="K5" s="3" t="n">
+        <v>9.4939</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1452,6 +1515,9 @@
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
       </c>
+      <c r="K6" s="3" t="n">
+        <v>12.5421</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1476,20 +1542,23 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.3317</v>
+        <v>33.5802</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>73531.06346799999</v>
+        <v>74079.26440799999</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>13531.06346799999</v>
+        <v>14079.26440799999</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2255177244666665</v>
+        <v>0.2346544067999998</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
       </c>
+      <c r="K7" s="3" t="n">
+        <v>33.5802</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1528,6 +1597,9 @@
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
       </c>
+      <c r="K8" s="3" t="n">
+        <v>30.6804</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1552,20 +1624,23 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>40.758</v>
+        <v>41.3017</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>131216.019894</v>
+        <v>132966.4038681</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>31216.019894</v>
+        <v>32966.40386809999</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.31216019894</v>
+        <v>0.329664038681</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
       </c>
+      <c r="K9" s="3" t="n">
+        <v>41.3017</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1590,20 +1665,23 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>45.95</v>
+        <v>46.2328</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>130803.98105</v>
+        <v>131609.0162152</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>30803.98105000002</v>
+        <v>31609.01621520001</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3080398105000002</v>
+        <v>0.3160901621520001</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
       </c>
+      <c r="K10" s="3" t="n">
+        <v>46.2328</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1628,20 +1706,23 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>103.8679</v>
+        <v>104.9865</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31255.8246001</v>
+        <v>31592.4325935</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1255.824600100001</v>
+        <v>1592.432593500002</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.04186082000333335</v>
+        <v>0.05308108645000005</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
       </c>
+      <c r="K11" s="3" t="n">
+        <v>104.9865</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1680,6 +1761,9 @@
       <c r="J12" s="3" t="n">
         <v>218.889</v>
       </c>
+      <c r="K12" s="3" t="n">
+        <v>218.889</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1718,6 +1802,9 @@
       <c r="J13" s="3" t="n">
         <v>19.888</v>
       </c>
+      <c r="K13" s="3" t="n">
+        <v>19.888</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1756,6 +1843,9 @@
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
       </c>
+      <c r="K14" s="3" t="n">
+        <v>38.9826</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1794,6 +1884,9 @@
       <c r="J15" s="3" t="n">
         <v>11.76</v>
       </c>
+      <c r="K15" s="3" t="n">
+        <v>11.76</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1818,20 +1911,23 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.4436</v>
+        <v>24.6466</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>139888.9628608</v>
+        <v>141050.7172448</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>39888.96286080001</v>
+        <v>41050.71724480001</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.398889628608</v>
+        <v>0.4105071724480001</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
       </c>
+      <c r="K16" s="3" t="n">
+        <v>24.6466</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1856,20 +1952,23 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.7178</v>
+        <v>16.7201</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55269.9997146</v>
+        <v>55277.60364569999</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5269.999714599995</v>
+        <v>5277.603645699994</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1053999942919999</v>
+        <v>0.1055520729139999</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
       </c>
+      <c r="K17" s="3" t="n">
+        <v>16.7201</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1908,6 +2007,9 @@
       <c r="J18" s="3" t="n">
         <v>45.31</v>
       </c>
+      <c r="K18" s="3" t="n">
+        <v>45.31</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1946,6 +2048,9 @@
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
       </c>
+      <c r="K19" s="3" t="n">
+        <v>14.6788</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1984,6 +2089,9 @@
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
       </c>
+      <c r="K20" s="3" t="n">
+        <v>9.039999999999999</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2022,6 +2130,9 @@
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
       </c>
+      <c r="K21" s="3" t="n">
+        <v>107.9031</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2046,20 +2157,23 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>43.8</v>
+        <v>43.997</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>67209.348</v>
+        <v>67511.63662</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>7209.347999999998</v>
+        <v>7511.636620000005</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1201558</v>
+        <v>0.1251939436666668</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
       </c>
+      <c r="K22" s="3" t="n">
+        <v>43.997</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2098,6 +2212,9 @@
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
       </c>
+      <c r="K23" s="3" t="n">
+        <v>60.3775</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2136,6 +2253,9 @@
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
       </c>
+      <c r="K24" s="3" t="n">
+        <v>28.2458</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2174,6 +2294,9 @@
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
       </c>
+      <c r="K25" s="3" t="n">
+        <v>11.2082</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2212,6 +2335,9 @@
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
       </c>
+      <c r="K26" s="3" t="n">
+        <v>8.626300000000001</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2250,6 +2376,9 @@
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
       </c>
+      <c r="K27" s="3" t="n">
+        <v>62.0021</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2288,6 +2417,9 @@
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
       </c>
+      <c r="K28" s="3" t="n">
+        <v>104.8438</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2326,6 +2458,9 @@
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
       </c>
+      <c r="K29" s="3" t="n">
+        <v>12.0216</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2364,6 +2499,9 @@
       <c r="J30" s="3" t="n">
         <v>15.064</v>
       </c>
+      <c r="K30" s="3" t="n">
+        <v>15.064</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2402,6 +2540,9 @@
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
       </c>
+      <c r="K31" s="3" t="n">
+        <v>413.2552</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2440,6 +2581,9 @@
       <c r="J32" s="3" t="n">
         <v>10.1</v>
       </c>
+      <c r="K32" s="3" t="n">
+        <v>10.1</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2478,6 +2622,9 @@
       <c r="J33" s="3" t="n">
         <v>17.77</v>
       </c>
+      <c r="K33" s="3" t="n">
+        <v>17.77</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2502,20 +2649,23 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>207.806</v>
+        <v>207.9392</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>73050.250986</v>
+        <v>73097.07491520001</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-6949.749014000001</v>
+        <v>-6902.925084799994</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.08687186267500001</v>
+        <v>-0.08628656355999992</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
       </c>
+      <c r="K34" s="3" t="n">
+        <v>207.9392</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2554,6 +2704,9 @@
       <c r="J35" s="3" t="n">
         <v>13.81</v>
       </c>
+      <c r="K35" s="3" t="n">
+        <v>13.81</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2592,6 +2745,9 @@
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
       </c>
+      <c r="K36" s="3" t="n">
+        <v>349.0771</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2630,6 +2786,9 @@
       <c r="J37" s="3" t="n">
         <v>15.6</v>
       </c>
+      <c r="K37" s="3" t="n">
+        <v>15.6</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2668,6 +2827,9 @@
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
       </c>
+      <c r="K38" s="3" t="n">
+        <v>13.9942</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2706,6 +2868,9 @@
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
       </c>
+      <c r="K39" s="3" t="n">
+        <v>1008.9183</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2744,6 +2909,9 @@
       <c r="J40" s="3" t="n">
         <v>19.911</v>
       </c>
+      <c r="K40" s="3" t="n">
+        <v>19.911</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
@@ -2755,13 +2923,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4808002.0794846</v>
+        <v>4815000.4556386</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>338002.0794846</v>
+        <v>345000.4556386</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.07561567773704697</v>
+        <v>0.07718130998626399</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-05-16
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -484,8 +484,8 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-05-15 05:54 IST</t>
+          <t>Generated: 2026-05-16 05:26 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4815000.4556386</v>
+        <v>4791569.2173213</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>345000.4556385996</v>
+        <v>321569.2173212999</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.07718130998626389</v>
+        <v>0.07193942221953019</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>558353.4982757568</v>
+        <v>558009.0018539429</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-32428.52172424318</v>
+        <v>-32773.01814605715</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.05489084065937413</v>
+        <v>-0.05547395999975955</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5373353.953914356</v>
+        <v>5349578.219175243</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>312571.9339143569</v>
+        <v>288796.1991752433</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.06176356394705119</v>
+        <v>0.05706552821953854</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-05-15</t>
+          <t>Last snapshot: 2026-05-16</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -628,6 +628,7 @@
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="21" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -676,6 +677,11 @@
           <t>2026-05-15</t>
         </is>
       </c>
+      <c r="J1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -695,13 +701,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>547.0499877929688</v>
+        <v>526.4500122070312</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>43763.9990234375</v>
+        <v>42116.0009765625</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>-53.51097656250204</v>
+        <v>-1701.509023437502</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -709,6 +715,9 @@
       <c r="I2" s="3" t="n">
         <v>547.0499877929688</v>
       </c>
+      <c r="J2" s="3" t="n">
+        <v>526.4500122070312</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -755,13 +764,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1571.800048828125</v>
+        <v>1550.800048828125</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>31436.0009765625</v>
+        <v>31016.0009765625</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-668.5790234375017</v>
+        <v>-1088.579023437502</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -769,6 +778,9 @@
       <c r="I4" s="3" t="n">
         <v>1571.800048828125</v>
       </c>
+      <c r="J4" s="3" t="n">
+        <v>1550.800048828125</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -788,13 +800,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>667.9000244140625</v>
+        <v>669.0499877929688</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13358.00048828125</v>
+        <v>13380.99975585938</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-855.0995117187504</v>
+        <v>-832.1002441406254</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -802,6 +814,9 @@
       <c r="I5" s="3" t="n">
         <v>667.9000244140625</v>
       </c>
+      <c r="J5" s="3" t="n">
+        <v>669.0499877929688</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -821,13 +836,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>402.1000061035156</v>
+        <v>397</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>16084.00024414062</v>
+        <v>15880</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-1418.239755859377</v>
+        <v>-1622.240000000002</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -835,6 +850,9 @@
       <c r="I6" s="3" t="n">
         <v>402.1000061035156</v>
       </c>
+      <c r="J6" s="3" t="n">
+        <v>397</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -854,13 +872,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>248</v>
+        <v>246.75</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>24800</v>
+        <v>24675</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-1633.82</v>
+        <v>-1758.82</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -868,6 +886,9 @@
       <c r="I7" s="3" t="n">
         <v>248</v>
       </c>
+      <c r="J7" s="3" t="n">
+        <v>246.75</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -914,13 +935,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>17.6299991607666</v>
+        <v>19.54000091552734</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>26444.9987411499</v>
+        <v>29310.00137329102</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-4605.171258850096</v>
+        <v>-1740.168626708983</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -928,6 +949,9 @@
       <c r="I9" s="3" t="n">
         <v>17.6299991607666</v>
       </c>
+      <c r="J9" s="3" t="n">
+        <v>19.54000091552734</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -947,13 +971,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>518.2000122070312</v>
+        <v>518.2999877929688</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>51820.00122070312</v>
+        <v>51829.99877929688</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>321.5212207031218</v>
+        <v>331.5187792968718</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -961,6 +985,9 @@
       <c r="I10" s="3" t="n">
         <v>518.2000122070312</v>
       </c>
+      <c r="J10" s="3" t="n">
+        <v>518.2999877929688</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -980,13 +1007,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>8.449999809265137</v>
+        <v>8.359999656677246</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>8449.999809265137</v>
+        <v>8359.999656677246</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-1391.210190734862</v>
+        <v>-1481.210343322753</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -994,6 +1021,9 @@
       <c r="I11" s="3" t="n">
         <v>8.449999809265137</v>
       </c>
+      <c r="J11" s="3" t="n">
+        <v>8.359999656677246</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1013,13 +1043,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2738.89990234375</v>
+        <v>2693.39990234375</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>27388.9990234375</v>
+        <v>26933.9990234375</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-334.2509765625</v>
+        <v>-789.2509765625</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -1027,6 +1057,9 @@
       <c r="I12" s="3" t="n">
         <v>2738.89990234375</v>
       </c>
+      <c r="J12" s="3" t="n">
+        <v>2693.39990234375</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1046,13 +1079,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>53.61999893188477</v>
+        <v>53.84000015258789</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>32171.99935913086</v>
+        <v>32304.00009155273</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-2859.760640869143</v>
+        <v>-2727.759908447268</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -1060,6 +1093,9 @@
       <c r="I13" s="3" t="n">
         <v>53.61999893188477</v>
       </c>
+      <c r="J13" s="3" t="n">
+        <v>53.84000015258789</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1079,13 +1115,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>748.7999877929688</v>
+        <v>748.9000244140625</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>37439.99938964844</v>
+        <v>37445.00122070312</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-5022.510610351565</v>
+        <v>-5017.508779296877</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -1093,6 +1129,9 @@
       <c r="I14" s="3" t="n">
         <v>748.7999877929688</v>
       </c>
+      <c r="J14" s="3" t="n">
+        <v>748.9000244140625</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1166,13 +1205,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>452</v>
+        <v>445.75</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>22600</v>
+        <v>22287.5</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>845.4700000000012</v>
+        <v>532.9700000000012</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -1180,6 +1219,9 @@
       <c r="I17" s="3" t="n">
         <v>452</v>
       </c>
+      <c r="J17" s="3" t="n">
+        <v>445.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1199,13 +1241,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>408.25</v>
+        <v>407</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>40825</v>
+        <v>40700</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-5815.82</v>
+        <v>-5940.82</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -1213,6 +1255,9 @@
       <c r="I18" s="3" t="n">
         <v>408.25</v>
       </c>
+      <c r="J18" s="3" t="n">
+        <v>407</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -1224,10 +1269,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>558353.4982757568</v>
+        <v>558009.0018539429</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-32428.52172424318</v>
+        <v>-32773.01814605714</v>
       </c>
     </row>
   </sheetData>
@@ -1241,7 +1286,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K41"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1255,6 +1300,7 @@
     <col width="24" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1313,6 +1359,11 @@
           <t>2026-05-15</t>
         </is>
       </c>
+      <c r="L1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1337,16 +1388,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>57.2873</v>
+        <v>56.4905</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>64303.9630786</v>
+        <v>63409.56942099999</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>14303.9630786</v>
+        <v>13409.56942099999</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.286079261572</v>
+        <v>0.2681913884199998</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -1354,6 +1405,9 @@
       <c r="K2" s="3" t="n">
         <v>57.2873</v>
       </c>
+      <c r="L2" s="3" t="n">
+        <v>56.4905</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1378,16 +1432,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.5426</v>
+        <v>25.3959</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>62712.5235738</v>
+        <v>62352.34382670001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>2712.523573800005</v>
+        <v>2352.343826700009</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.04520872623000008</v>
+        <v>0.03920573044500016</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -1395,6 +1449,9 @@
       <c r="K3" s="3" t="n">
         <v>25.5426</v>
       </c>
+      <c r="L3" s="3" t="n">
+        <v>25.3959</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1419,16 +1476,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.97</v>
+        <v>12.66</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>249103.02621</v>
+        <v>243149.13738</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>69103.02621000001</v>
+        <v>63149.13738</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3839057011666667</v>
+        <v>0.350828541</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -1436,6 +1493,9 @@
       <c r="K4" s="3" t="n">
         <v>12.97</v>
       </c>
+      <c r="L4" s="3" t="n">
+        <v>12.66</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1460,16 +1520,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.4939</v>
+        <v>9.4802</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>174251.8760632</v>
+        <v>174000.4250576</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-35748.1239368</v>
+        <v>-35999.57494240001</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1702291616038095</v>
+        <v>-0.171426547344762</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -1477,6 +1537,9 @@
       <c r="K5" s="3" t="n">
         <v>9.4939</v>
       </c>
+      <c r="L5" s="3" t="n">
+        <v>9.4802</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1501,16 +1564,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.5421</v>
+        <v>12.4417</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>53040.2524317</v>
+        <v>52615.6631409</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>3040.252431699999</v>
+        <v>2615.663140900004</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.06080504863399998</v>
+        <v>0.05231326281800008</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -1518,6 +1581,9 @@
       <c r="K6" s="3" t="n">
         <v>12.5421</v>
       </c>
+      <c r="L6" s="3" t="n">
+        <v>12.4417</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1542,16 +1608,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.5802</v>
+        <v>32.8663</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>74079.26440799999</v>
+        <v>72504.37245200001</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>14079.26440799999</v>
+        <v>12504.37245200001</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2346544067999998</v>
+        <v>0.2084062075333335</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -1559,6 +1625,9 @@
       <c r="K7" s="3" t="n">
         <v>33.5802</v>
       </c>
+      <c r="L7" s="3" t="n">
+        <v>32.8663</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1583,16 +1652,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>30.6804</v>
+        <v>30.4531</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>49229.5550772</v>
+        <v>48864.8310883</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>-770.4449228000012</v>
+        <v>-1135.168911699999</v>
       </c>
       <c r="I8" s="13" t="n">
-        <v>-0.01540889845600002</v>
+        <v>-0.02270337823399998</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -1600,6 +1669,9 @@
       <c r="K8" s="3" t="n">
         <v>30.6804</v>
       </c>
+      <c r="L8" s="3" t="n">
+        <v>30.4531</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1624,16 +1696,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>41.3017</v>
+        <v>40.689</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>132966.4038681</v>
+        <v>130993.881777</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>32966.40386809999</v>
+        <v>30993.881777</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.329664038681</v>
+        <v>0.30993881777</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -1641,6 +1713,9 @@
       <c r="K9" s="3" t="n">
         <v>41.3017</v>
       </c>
+      <c r="L9" s="3" t="n">
+        <v>40.689</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1665,16 +1740,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>46.2328</v>
+        <v>45.9528</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>131609.0162152</v>
+        <v>130811.9516952</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>31609.01621520001</v>
+        <v>30811.95169520001</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3160901621520001</v>
+        <v>0.3081195169520001</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -1682,6 +1757,9 @@
       <c r="K10" s="3" t="n">
         <v>46.2328</v>
       </c>
+      <c r="L10" s="3" t="n">
+        <v>45.9528</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1706,16 +1784,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>104.9865</v>
+        <v>103.3395</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31592.4325935</v>
+        <v>31096.8190005</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1592.432593500002</v>
+        <v>1096.8190005</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.05308108645000005</v>
+        <v>0.03656063334999999</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -1723,6 +1801,9 @@
       <c r="K11" s="3" t="n">
         <v>104.9865</v>
       </c>
+      <c r="L11" s="3" t="n">
+        <v>103.3395</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1747,16 +1828,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>218.889</v>
+        <v>218.423</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>101897.645058</v>
+        <v>101680.711806</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>1897.645058000009</v>
+        <v>1680.711805999992</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.01897645058000009</v>
+        <v>0.01680711805999992</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -1764,6 +1845,9 @@
       <c r="K12" s="3" t="n">
         <v>218.889</v>
       </c>
+      <c r="L12" s="3" t="n">
+        <v>218.423</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1788,16 +1872,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>19.888</v>
+        <v>19.848</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>230454.28824</v>
+        <v>229990.78404</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>30454.28824000002</v>
+        <v>29990.78403999997</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.1522714412000001</v>
+        <v>0.1499539201999998</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -1805,6 +1889,9 @@
       <c r="K13" s="3" t="n">
         <v>19.888</v>
       </c>
+      <c r="L13" s="3" t="n">
+        <v>19.848</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1846,6 +1933,9 @@
       <c r="K14" s="3" t="n">
         <v>38.9826</v>
       </c>
+      <c r="L14" s="3" t="n">
+        <v>38.9826</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1870,16 +1960,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.76</v>
+        <v>11.74</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>114588.81672</v>
+        <v>114393.93778</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>14588.81672</v>
+        <v>14393.93778000001</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1458881672</v>
+        <v>0.1439393778000001</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -1887,6 +1977,9 @@
       <c r="K15" s="3" t="n">
         <v>11.76</v>
       </c>
+      <c r="L15" s="3" t="n">
+        <v>11.74</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1911,16 +2004,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.6466</v>
+        <v>24.3166</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>141050.7172448</v>
+        <v>139162.1510048</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>41050.71724480001</v>
+        <v>39162.15100479999</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4105071724480001</v>
+        <v>0.3916215100479999</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -1928,6 +2021,9 @@
       <c r="K16" s="3" t="n">
         <v>24.6466</v>
       </c>
+      <c r="L16" s="3" t="n">
+        <v>24.3166</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1952,16 +2048,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.7201</v>
+        <v>16.6235</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55277.60364569999</v>
+        <v>54958.23853949999</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5277.603645699994</v>
+        <v>4958.238539499995</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1055520729139999</v>
+        <v>0.0991647707899999</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -1969,6 +2065,9 @@
       <c r="K17" s="3" t="n">
         <v>16.7201</v>
       </c>
+      <c r="L17" s="3" t="n">
+        <v>16.6235</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1993,16 +2092,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>45.31</v>
+        <v>45.44</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>85474.41516</v>
+        <v>85719.65183999999</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>5474.415160000004</v>
+        <v>5719.651839999991</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.06843018950000006</v>
+        <v>0.0714956479999999</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -2010,6 +2109,9 @@
       <c r="K18" s="3" t="n">
         <v>45.31</v>
       </c>
+      <c r="L18" s="3" t="n">
+        <v>45.44</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2034,16 +2136,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>14.6788</v>
+        <v>14.8854</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>212354.7647608</v>
+        <v>215343.5986164</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>62354.7647608</v>
+        <v>65343.59861640001</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.4156984317386667</v>
+        <v>0.4356239907760001</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -2051,6 +2153,9 @@
       <c r="K19" s="3" t="n">
         <v>14.6788</v>
       </c>
+      <c r="L19" s="3" t="n">
+        <v>14.8854</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2075,16 +2180,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.039999999999999</v>
+        <v>9.07</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>237352.45912</v>
+        <v>238140.13321</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-12647.54088000002</v>
+        <v>-11859.86679</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.05059016352000006</v>
+        <v>-0.04743946716</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -2092,6 +2197,9 @@
       <c r="K20" s="3" t="n">
         <v>9.039999999999999</v>
       </c>
+      <c r="L20" s="3" t="n">
+        <v>9.07</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2116,16 +2224,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>107.9031</v>
+        <v>107.7303</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>163932.7558029</v>
+        <v>163670.2278477</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-6067.244197099993</v>
+        <v>-6329.772152299993</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.03568967174764702</v>
+        <v>-0.03723395383705878</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -2133,6 +2241,9 @@
       <c r="K21" s="3" t="n">
         <v>107.9031</v>
       </c>
+      <c r="L21" s="3" t="n">
+        <v>107.7303</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2157,16 +2268,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>43.997</v>
+        <v>42.665</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>67511.63662</v>
+        <v>65467.7359</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>7511.636620000005</v>
+        <v>5467.7359</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1251939436666668</v>
+        <v>0.09112893166666666</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -2174,6 +2285,9 @@
       <c r="K22" s="3" t="n">
         <v>43.997</v>
       </c>
+      <c r="L22" s="3" t="n">
+        <v>42.665</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2198,16 +2312,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>60.3775</v>
+        <v>60.2124</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>164013.4862925</v>
+        <v>163564.9975908</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>14013.48629249999</v>
+        <v>13564.99759080002</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.09342324194999994</v>
+        <v>0.09043331727200013</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -2215,6 +2329,9 @@
       <c r="K23" s="3" t="n">
         <v>60.3775</v>
       </c>
+      <c r="L23" s="3" t="n">
+        <v>60.2124</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2239,16 +2356,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>28.2458</v>
+        <v>27.9311</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>102627.8942788</v>
+        <v>101484.4677046</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>2627.894278799999</v>
+        <v>1484.4677046</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.02627894278799998</v>
+        <v>0.014844677046</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -2256,6 +2373,9 @@
       <c r="K24" s="3" t="n">
         <v>28.2458</v>
       </c>
+      <c r="L24" s="3" t="n">
+        <v>27.9311</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2280,16 +2400,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.2082</v>
+        <v>11.1514</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>184057.4065268</v>
+        <v>183124.6554436</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-15942.59347320002</v>
+        <v>-16875.3445564</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.07971296736600009</v>
+        <v>-0.08437672278199999</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -2297,6 +2417,9 @@
       <c r="K25" s="3" t="n">
         <v>11.2082</v>
       </c>
+      <c r="L25" s="3" t="n">
+        <v>11.1514</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2321,16 +2444,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>8.626300000000001</v>
+        <v>8.598100000000001</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>103012.8161045</v>
+        <v>102676.0597415</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>-6987.183895499998</v>
+        <v>-7323.940258499992</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>-0.06351985359545453</v>
+        <v>-0.06658127507727266</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -2338,6 +2461,9 @@
       <c r="K26" s="3" t="n">
         <v>8.626300000000001</v>
       </c>
+      <c r="L26" s="3" t="n">
+        <v>8.598100000000001</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2362,16 +2488,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>62.0021</v>
+        <v>61.7452</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>99876.70280599999</v>
+        <v>99462.87287199999</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-10123.29719400001</v>
+        <v>-10537.12712800001</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.09202997449090922</v>
+        <v>-0.09579206480000006</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -2379,6 +2505,9 @@
       <c r="K27" s="3" t="n">
         <v>62.0021</v>
       </c>
+      <c r="L27" s="3" t="n">
+        <v>61.7452</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2403,16 +2532,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>104.8438</v>
+        <v>104.7252</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>346682.4851766001</v>
+        <v>346290.3156564</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-33317.51482339995</v>
+        <v>-33709.68434360001</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.08767767058789461</v>
+        <v>-0.08870969564105265</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -2420,6 +2549,9 @@
       <c r="K28" s="3" t="n">
         <v>104.8438</v>
       </c>
+      <c r="L28" s="3" t="n">
+        <v>104.7252</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2444,16 +2576,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.0216</v>
+        <v>11.7996</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>115451.8759848</v>
+        <v>113319.8539188</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>15451.87598479999</v>
+        <v>13319.8539188</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.1545187598479999</v>
+        <v>0.133198539188</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -2461,6 +2593,9 @@
       <c r="K29" s="3" t="n">
         <v>12.0216</v>
       </c>
+      <c r="L29" s="3" t="n">
+        <v>11.7996</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2485,16 +2620,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>15.064</v>
+        <v>15.0715</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>111411.250104</v>
+        <v>111466.7190615</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>11411.25010399999</v>
+        <v>11466.7190615</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.1141125010399999</v>
+        <v>0.114667190615</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -2502,6 +2637,9 @@
       <c r="K30" s="3" t="n">
         <v>15.064</v>
       </c>
+      <c r="L30" s="3" t="n">
+        <v>15.0715</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2526,16 +2664,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>413.2552</v>
+        <v>410.7949</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>109958.943616</v>
+        <v>109304.306992</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>9958.94361599999</v>
+        <v>9304.306991999983</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.09958943615999989</v>
+        <v>0.09304306991999983</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -2543,6 +2681,9 @@
       <c r="K31" s="3" t="n">
         <v>413.2552</v>
       </c>
+      <c r="L31" s="3" t="n">
+        <v>410.7949</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2567,16 +2708,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.1</v>
+        <v>10.06</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>213513.596</v>
+        <v>212667.9976</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>13513.59599999999</v>
+        <v>12667.9976</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.06756797999999996</v>
+        <v>0.06333998800000001</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -2584,6 +2725,9 @@
       <c r="K32" s="3" t="n">
         <v>10.1</v>
       </c>
+      <c r="L32" s="3" t="n">
+        <v>10.06</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2608,16 +2752,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>17.77</v>
+        <v>17.68</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>63681.28279999999</v>
+        <v>63358.7552</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>3681.282799999994</v>
+        <v>3358.7552</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.06135471333333323</v>
+        <v>0.05597925333333333</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -2625,6 +2769,9 @@
       <c r="K33" s="3" t="n">
         <v>17.77</v>
       </c>
+      <c r="L33" s="3" t="n">
+        <v>17.68</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2649,16 +2796,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>207.9392</v>
+        <v>209.5029</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>73097.07491520001</v>
+        <v>73646.7639399</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-6902.925084799994</v>
+        <v>-6353.236060099996</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.08628656355999992</v>
+        <v>-0.07941545075124995</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -2666,6 +2813,9 @@
       <c r="K34" s="3" t="n">
         <v>207.9392</v>
       </c>
+      <c r="L34" s="3" t="n">
+        <v>209.5029</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2690,16 +2840,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>13.81</v>
+        <v>13.79</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>98540.19163</v>
+        <v>98397.48316999999</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>-1459.808369999999</v>
+        <v>-1602.516830000008</v>
       </c>
       <c r="I35" s="13" t="n">
-        <v>-0.01459808369999999</v>
+        <v>-0.01602516830000008</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -2707,6 +2857,9 @@
       <c r="K35" s="3" t="n">
         <v>13.81</v>
       </c>
+      <c r="L35" s="3" t="n">
+        <v>13.79</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2731,16 +2884,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>349.0771</v>
+        <v>347.7755</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>162567.2999326</v>
+        <v>161961.137003</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>12567.2999326</v>
+        <v>11961.13700300001</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.08378199955066666</v>
+        <v>0.0797409133533334</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -2748,6 +2901,9 @@
       <c r="K36" s="3" t="n">
         <v>349.0771</v>
       </c>
+      <c r="L36" s="3" t="n">
+        <v>347.7755</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2772,16 +2928,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>15.6</v>
+        <v>15.62</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>58701.0684</v>
+        <v>58776.32618</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>8701.068400000004</v>
+        <v>8776.326179999996</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.1740213680000001</v>
+        <v>0.1755265235999999</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -2789,6 +2945,9 @@
       <c r="K37" s="3" t="n">
         <v>15.6</v>
       </c>
+      <c r="L37" s="3" t="n">
+        <v>15.62</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2813,16 +2972,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.9942</v>
+        <v>13.9433</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>83692.0612044</v>
+        <v>83387.65467060001</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>3692.061204400001</v>
+        <v>3387.654670600008</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.04615076505500001</v>
+        <v>0.0423456833825001</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -2830,6 +2989,9 @@
       <c r="K38" s="3" t="n">
         <v>13.9942</v>
       </c>
+      <c r="L38" s="3" t="n">
+        <v>13.9433</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2854,16 +3016,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1008.9183</v>
+        <v>1007.1406</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50325.8537223</v>
+        <v>50237.1802686</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>325.8537223000021</v>
+        <v>237.180268600001</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.006517074446000043</v>
+        <v>0.00474360537200002</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -2871,6 +3033,9 @@
       <c r="K39" s="3" t="n">
         <v>1008.9183</v>
       </c>
+      <c r="L39" s="3" t="n">
+        <v>1007.1406</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2895,16 +3060,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>19.911</v>
+        <v>19.7344</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>100371.888597</v>
-      </c>
-      <c r="H40" s="4" t="n">
-        <v>371.8885970000119</v>
-      </c>
-      <c r="I40" s="12" t="n">
-        <v>0.00371888597000012</v>
+        <v>99481.64322880001</v>
+      </c>
+      <c r="H40" s="6" t="n">
+        <v>-518.3567711999931</v>
+      </c>
+      <c r="I40" s="13" t="n">
+        <v>-0.005183567711999931</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -2912,6 +3077,9 @@
       <c r="K40" s="3" t="n">
         <v>19.911</v>
       </c>
+      <c r="L40" s="3" t="n">
+        <v>19.7344</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
@@ -2923,13 +3091,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4815000.4556386</v>
+        <v>4791569.2173213</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>345000.4556386</v>
+        <v>321569.2173213</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.07718130998626399</v>
+        <v>0.0719394222195302</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-05-17
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-05-16 05:26 IST</t>
+          <t>Generated: 2026-05-17 05:47 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4791569.2173213</v>
+        <v>4788357.0049389</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>321569.2173212999</v>
+        <v>318357.0049388995</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.07193942221953019</v>
+        <v>0.07122080647402675</v>
       </c>
     </row>
     <row r="6">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5349578.219175243</v>
+        <v>5346366.006792842</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>288796.1991752433</v>
+        <v>285583.9867928429</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.05706552821953854</v>
+        <v>0.05643080173463841</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-05-16</t>
+          <t>Last snapshot: 2026-05-17</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -629,6 +629,7 @@
     <col width="21" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
     <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -682,6 +683,11 @@
           <t>2026-05-16</t>
         </is>
       </c>
+      <c r="K1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -718,6 +724,9 @@
       <c r="J2" s="3" t="n">
         <v>526.4500122070312</v>
       </c>
+      <c r="K2" s="3" t="n">
+        <v>526.4500122070312</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -781,6 +790,9 @@
       <c r="J4" s="3" t="n">
         <v>1550.800048828125</v>
       </c>
+      <c r="K4" s="3" t="n">
+        <v>1550.800048828125</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -817,6 +829,9 @@
       <c r="J5" s="3" t="n">
         <v>669.0499877929688</v>
       </c>
+      <c r="K5" s="3" t="n">
+        <v>669.0499877929688</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -853,6 +868,9 @@
       <c r="J6" s="3" t="n">
         <v>397</v>
       </c>
+      <c r="K6" s="3" t="n">
+        <v>397</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -889,6 +907,9 @@
       <c r="J7" s="3" t="n">
         <v>246.75</v>
       </c>
+      <c r="K7" s="3" t="n">
+        <v>246.75</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -952,6 +973,9 @@
       <c r="J9" s="3" t="n">
         <v>19.54000091552734</v>
       </c>
+      <c r="K9" s="3" t="n">
+        <v>19.54000091552734</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -988,6 +1012,9 @@
       <c r="J10" s="3" t="n">
         <v>518.2999877929688</v>
       </c>
+      <c r="K10" s="3" t="n">
+        <v>518.2999877929688</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1024,6 +1051,9 @@
       <c r="J11" s="3" t="n">
         <v>8.359999656677246</v>
       </c>
+      <c r="K11" s="3" t="n">
+        <v>8.359999656677246</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1060,6 +1090,9 @@
       <c r="J12" s="3" t="n">
         <v>2693.39990234375</v>
       </c>
+      <c r="K12" s="3" t="n">
+        <v>2693.39990234375</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1096,6 +1129,9 @@
       <c r="J13" s="3" t="n">
         <v>53.84000015258789</v>
       </c>
+      <c r="K13" s="3" t="n">
+        <v>53.84000015258789</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1132,6 +1168,9 @@
       <c r="J14" s="3" t="n">
         <v>748.9000244140625</v>
       </c>
+      <c r="K14" s="3" t="n">
+        <v>748.9000244140625</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1222,6 +1261,9 @@
       <c r="J17" s="3" t="n">
         <v>445.75</v>
       </c>
+      <c r="K17" s="3" t="n">
+        <v>445.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1256,6 +1298,9 @@
         <v>408.25</v>
       </c>
       <c r="J18" s="3" t="n">
+        <v>407</v>
+      </c>
+      <c r="K18" s="3" t="n">
         <v>407</v>
       </c>
     </row>
@@ -1286,7 +1331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:M41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1301,6 +1346,7 @@
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1364,6 +1410,11 @@
           <t>2026-05-16</t>
         </is>
       </c>
+      <c r="M1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1408,6 +1459,9 @@
       <c r="L2" s="3" t="n">
         <v>56.4905</v>
       </c>
+      <c r="M2" s="3" t="n">
+        <v>56.4905</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1452,6 +1506,9 @@
       <c r="L3" s="3" t="n">
         <v>25.3959</v>
       </c>
+      <c r="M3" s="3" t="n">
+        <v>25.3959</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1496,6 +1553,9 @@
       <c r="L4" s="3" t="n">
         <v>12.66</v>
       </c>
+      <c r="M4" s="3" t="n">
+        <v>12.66</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1540,6 +1600,9 @@
       <c r="L5" s="3" t="n">
         <v>9.4802</v>
       </c>
+      <c r="M5" s="3" t="n">
+        <v>9.4802</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1584,6 +1647,9 @@
       <c r="L6" s="3" t="n">
         <v>12.4417</v>
       </c>
+      <c r="M6" s="3" t="n">
+        <v>12.4417</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1628,6 +1694,9 @@
       <c r="L7" s="3" t="n">
         <v>32.8663</v>
       </c>
+      <c r="M7" s="3" t="n">
+        <v>32.8663</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1672,6 +1741,9 @@
       <c r="L8" s="3" t="n">
         <v>30.4531</v>
       </c>
+      <c r="M8" s="3" t="n">
+        <v>30.4531</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1716,6 +1788,9 @@
       <c r="L9" s="3" t="n">
         <v>40.689</v>
       </c>
+      <c r="M9" s="3" t="n">
+        <v>40.689</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1760,6 +1835,9 @@
       <c r="L10" s="3" t="n">
         <v>45.9528</v>
       </c>
+      <c r="M10" s="3" t="n">
+        <v>45.9528</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1804,6 +1882,9 @@
       <c r="L11" s="3" t="n">
         <v>103.3395</v>
       </c>
+      <c r="M11" s="3" t="n">
+        <v>103.3395</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1848,6 +1929,9 @@
       <c r="L12" s="3" t="n">
         <v>218.423</v>
       </c>
+      <c r="M12" s="3" t="n">
+        <v>218.423</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1892,6 +1976,9 @@
       <c r="L13" s="3" t="n">
         <v>19.848</v>
       </c>
+      <c r="M13" s="3" t="n">
+        <v>19.848</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1916,16 +2003,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>38.9826</v>
+        <v>38.0922</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>140633.8616556</v>
+        <v>137421.6492732</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>40633.86165559999</v>
+        <v>37421.64927319999</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.4063386165559999</v>
+        <v>0.3742164927319999</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -1936,6 +2023,9 @@
       <c r="L14" s="3" t="n">
         <v>38.9826</v>
       </c>
+      <c r="M14" s="3" t="n">
+        <v>38.0922</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1980,6 +2070,9 @@
       <c r="L15" s="3" t="n">
         <v>11.74</v>
       </c>
+      <c r="M15" s="3" t="n">
+        <v>11.74</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2024,6 +2117,9 @@
       <c r="L16" s="3" t="n">
         <v>24.3166</v>
       </c>
+      <c r="M16" s="3" t="n">
+        <v>24.3166</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2068,6 +2164,9 @@
       <c r="L17" s="3" t="n">
         <v>16.6235</v>
       </c>
+      <c r="M17" s="3" t="n">
+        <v>16.6235</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2112,6 +2211,9 @@
       <c r="L18" s="3" t="n">
         <v>45.44</v>
       </c>
+      <c r="M18" s="3" t="n">
+        <v>45.44</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2156,6 +2258,9 @@
       <c r="L19" s="3" t="n">
         <v>14.8854</v>
       </c>
+      <c r="M19" s="3" t="n">
+        <v>14.8854</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2200,6 +2305,9 @@
       <c r="L20" s="3" t="n">
         <v>9.07</v>
       </c>
+      <c r="M20" s="3" t="n">
+        <v>9.07</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2244,6 +2352,9 @@
       <c r="L21" s="3" t="n">
         <v>107.7303</v>
       </c>
+      <c r="M21" s="3" t="n">
+        <v>107.7303</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2288,6 +2399,9 @@
       <c r="L22" s="3" t="n">
         <v>42.665</v>
       </c>
+      <c r="M22" s="3" t="n">
+        <v>42.665</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2332,6 +2446,9 @@
       <c r="L23" s="3" t="n">
         <v>60.2124</v>
       </c>
+      <c r="M23" s="3" t="n">
+        <v>60.2124</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2376,6 +2493,9 @@
       <c r="L24" s="3" t="n">
         <v>27.9311</v>
       </c>
+      <c r="M24" s="3" t="n">
+        <v>27.9311</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2420,6 +2540,9 @@
       <c r="L25" s="3" t="n">
         <v>11.1514</v>
       </c>
+      <c r="M25" s="3" t="n">
+        <v>11.1514</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2464,6 +2587,9 @@
       <c r="L26" s="3" t="n">
         <v>8.598100000000001</v>
       </c>
+      <c r="M26" s="3" t="n">
+        <v>8.598100000000001</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2508,6 +2634,9 @@
       <c r="L27" s="3" t="n">
         <v>61.7452</v>
       </c>
+      <c r="M27" s="3" t="n">
+        <v>61.7452</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2552,6 +2681,9 @@
       <c r="L28" s="3" t="n">
         <v>104.7252</v>
       </c>
+      <c r="M28" s="3" t="n">
+        <v>104.7252</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2596,6 +2728,9 @@
       <c r="L29" s="3" t="n">
         <v>11.7996</v>
       </c>
+      <c r="M29" s="3" t="n">
+        <v>11.7996</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2640,6 +2775,9 @@
       <c r="L30" s="3" t="n">
         <v>15.0715</v>
       </c>
+      <c r="M30" s="3" t="n">
+        <v>15.0715</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2684,6 +2822,9 @@
       <c r="L31" s="3" t="n">
         <v>410.7949</v>
       </c>
+      <c r="M31" s="3" t="n">
+        <v>410.7949</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2728,6 +2869,9 @@
       <c r="L32" s="3" t="n">
         <v>10.06</v>
       </c>
+      <c r="M32" s="3" t="n">
+        <v>10.06</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2772,6 +2916,9 @@
       <c r="L33" s="3" t="n">
         <v>17.68</v>
       </c>
+      <c r="M33" s="3" t="n">
+        <v>17.68</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2816,6 +2963,9 @@
       <c r="L34" s="3" t="n">
         <v>209.5029</v>
       </c>
+      <c r="M34" s="3" t="n">
+        <v>209.5029</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2860,6 +3010,9 @@
       <c r="L35" s="3" t="n">
         <v>13.79</v>
       </c>
+      <c r="M35" s="3" t="n">
+        <v>13.79</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2904,6 +3057,9 @@
       <c r="L36" s="3" t="n">
         <v>347.7755</v>
       </c>
+      <c r="M36" s="3" t="n">
+        <v>347.7755</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2948,6 +3104,9 @@
       <c r="L37" s="3" t="n">
         <v>15.62</v>
       </c>
+      <c r="M37" s="3" t="n">
+        <v>15.62</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2992,6 +3151,9 @@
       <c r="L38" s="3" t="n">
         <v>13.9433</v>
       </c>
+      <c r="M38" s="3" t="n">
+        <v>13.9433</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3036,6 +3198,9 @@
       <c r="L39" s="3" t="n">
         <v>1007.1406</v>
       </c>
+      <c r="M39" s="3" t="n">
+        <v>1007.1406</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3080,6 +3245,9 @@
       <c r="L40" s="3" t="n">
         <v>19.7344</v>
       </c>
+      <c r="M40" s="3" t="n">
+        <v>19.7344</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
@@ -3091,13 +3259,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4791569.2173213</v>
+        <v>4788357.0049389</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>321569.2173213</v>
+        <v>318357.0049389</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.0719394222195302</v>
+        <v>0.07122080647402684</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-05-18
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -42,14 +42,14 @@
       <color rgb="009C0006"/>
     </font>
     <font>
-      <color rgb="00006100"/>
-    </font>
-    <font>
       <b val="1"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="009C0006"/>
+    </font>
+    <font>
+      <color rgb="00006100"/>
     </font>
     <font>
       <b val="1"/>
@@ -97,7 +97,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -106,10 +106,10 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-05-17 05:47 IST</t>
+          <t>Generated: 2026-05-18 06:12 IST</t>
         </is>
       </c>
     </row>
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>558009.0018539429</v>
+        <v>549061.9932250977</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-32773.01814605715</v>
+        <v>-41720.02677490236</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.05547395999975955</v>
+        <v>-0.07061830821273532</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5346366.006792842</v>
+        <v>5337418.998163997</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>285583.9867928429</v>
+        <v>276636.9781639976</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.05643080173463841</v>
+        <v>0.05466289144063898</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-05-17</t>
+          <t>Last snapshot: 2026-05-18</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -630,6 +630,7 @@
     <col width="21" customWidth="1" min="9" max="9"/>
     <col width="21" customWidth="1" min="10" max="10"/>
     <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -688,6 +689,11 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="L1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -707,13 +713,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>526.4500122070312</v>
+        <v>527.3499755859375</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>42116.0009765625</v>
+        <v>42187.998046875</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>-1701.509023437502</v>
+        <v>-1629.511953125002</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -727,6 +733,9 @@
       <c r="K2" s="3" t="n">
         <v>526.4500122070312</v>
       </c>
+      <c r="L2" s="3" t="n">
+        <v>527.3499755859375</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -773,13 +782,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1550.800048828125</v>
+        <v>1532.099975585938</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>31016.0009765625</v>
+        <v>30641.99951171875</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-1088.579023437502</v>
+        <v>-1462.580488281252</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -793,6 +802,9 @@
       <c r="K4" s="3" t="n">
         <v>1550.800048828125</v>
       </c>
+      <c r="L4" s="3" t="n">
+        <v>1532.099975585938</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -812,13 +824,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>669.0499877929688</v>
+        <v>657.5999755859375</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13380.99975585938</v>
+        <v>13151.99951171875</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-832.1002441406254</v>
+        <v>-1061.10048828125</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -832,6 +844,9 @@
       <c r="K5" s="3" t="n">
         <v>669.0499877929688</v>
       </c>
+      <c r="L5" s="3" t="n">
+        <v>657.5999755859375</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -851,13 +866,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>397</v>
+        <v>386.2999877929688</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15880</v>
+        <v>15451.99951171875</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-1622.240000000002</v>
+        <v>-2050.240488281252</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -871,6 +886,9 @@
       <c r="K6" s="3" t="n">
         <v>397</v>
       </c>
+      <c r="L6" s="3" t="n">
+        <v>386.2999877929688</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -890,13 +908,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>246.75</v>
+        <v>236.8999938964844</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>24675</v>
+        <v>23689.99938964844</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-1758.82</v>
+        <v>-2743.820610351562</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -910,6 +928,9 @@
       <c r="K7" s="3" t="n">
         <v>246.75</v>
       </c>
+      <c r="L7" s="3" t="n">
+        <v>236.8999938964844</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -956,13 +977,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>19.54000091552734</v>
+        <v>19.01000022888184</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>29310.00137329102</v>
+        <v>28515.00034332275</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-1740.168626708983</v>
+        <v>-2535.169656677244</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -976,6 +997,9 @@
       <c r="K9" s="3" t="n">
         <v>19.54000091552734</v>
       </c>
+      <c r="L9" s="3" t="n">
+        <v>19.01000022888184</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -995,13 +1019,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>518.2999877929688</v>
+        <v>509.75</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>51829.99877929688</v>
-      </c>
-      <c r="G10" s="4" t="n">
-        <v>331.5187792968718</v>
+        <v>50975</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>-523.4800000000032</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1015,6 +1039,9 @@
       <c r="K10" s="3" t="n">
         <v>518.2999877929688</v>
       </c>
+      <c r="L10" s="3" t="n">
+        <v>509.75</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1034,13 +1061,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>8.359999656677246</v>
+        <v>8.130000114440918</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>8359.999656677246</v>
+        <v>8130.000114440918</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-1481.210343322753</v>
+        <v>-1711.209885559081</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -1054,6 +1081,9 @@
       <c r="K11" s="3" t="n">
         <v>8.359999656677246</v>
       </c>
+      <c r="L11" s="3" t="n">
+        <v>8.130000114440918</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1073,13 +1103,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2693.39990234375</v>
+        <v>2472.39990234375</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>26933.9990234375</v>
+        <v>24723.9990234375</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-789.2509765625</v>
+        <v>-2999.2509765625</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -1093,6 +1123,9 @@
       <c r="K12" s="3" t="n">
         <v>2693.39990234375</v>
       </c>
+      <c r="L12" s="3" t="n">
+        <v>2472.39990234375</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1112,13 +1145,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>53.84000015258789</v>
+        <v>53.0099983215332</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>32304.00009155273</v>
+        <v>31805.99899291992</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-2727.759908447268</v>
+        <v>-3225.76100708008</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -1132,6 +1165,9 @@
       <c r="K13" s="3" t="n">
         <v>53.84000015258789</v>
       </c>
+      <c r="L13" s="3" t="n">
+        <v>53.0099983215332</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1151,13 +1187,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>748.9000244140625</v>
+        <v>731.2000122070312</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>37445.00122070312</v>
+        <v>36560.00061035156</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-5017.508779296877</v>
+        <v>-5902.50938964844</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -1171,6 +1207,9 @@
       <c r="K14" s="3" t="n">
         <v>748.9000244140625</v>
       </c>
+      <c r="L14" s="3" t="n">
+        <v>731.2000122070312</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1244,13 +1283,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>445.75</v>
+        <v>433.0499877929688</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>22287.5</v>
-      </c>
-      <c r="G17" s="4" t="n">
-        <v>532.9700000000012</v>
+        <v>21652.49938964844</v>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>-102.0306103515613</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -1264,6 +1303,9 @@
       <c r="K17" s="3" t="n">
         <v>445.75</v>
       </c>
+      <c r="L17" s="3" t="n">
+        <v>433.0499877929688</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1283,13 +1325,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>407</v>
+        <v>398.0499877929688</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>40700</v>
+        <v>39804.99877929688</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-5940.82</v>
+        <v>-6835.821220703125</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -1303,6 +1345,9 @@
       <c r="K18" s="3" t="n">
         <v>407</v>
       </c>
+      <c r="L18" s="3" t="n">
+        <v>398.0499877929688</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -1314,10 +1359,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>558009.0018539429</v>
+        <v>549061.9932250977</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-32773.01814605714</v>
+        <v>-41720.02677490236</v>
       </c>
     </row>
   </sheetData>
@@ -1331,7 +1376,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M41"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1347,6 +1392,7 @@
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1415,6 +1461,11 @@
           <t>2026-05-17</t>
         </is>
       </c>
+      <c r="N1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1462,6 +1513,9 @@
       <c r="M2" s="3" t="n">
         <v>56.4905</v>
       </c>
+      <c r="N2" s="3" t="n">
+        <v>56.4905</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1509,6 +1563,9 @@
       <c r="M3" s="3" t="n">
         <v>25.3959</v>
       </c>
+      <c r="N3" s="3" t="n">
+        <v>25.3959</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1556,6 +1613,9 @@
       <c r="M4" s="3" t="n">
         <v>12.66</v>
       </c>
+      <c r="N4" s="3" t="n">
+        <v>12.66</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1603,6 +1663,9 @@
       <c r="M5" s="3" t="n">
         <v>9.4802</v>
       </c>
+      <c r="N5" s="3" t="n">
+        <v>9.4802</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1650,6 +1713,9 @@
       <c r="M6" s="3" t="n">
         <v>12.4417</v>
       </c>
+      <c r="N6" s="3" t="n">
+        <v>12.4417</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1697,6 +1763,9 @@
       <c r="M7" s="3" t="n">
         <v>32.8663</v>
       </c>
+      <c r="N7" s="3" t="n">
+        <v>32.8663</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1744,6 +1813,9 @@
       <c r="M8" s="3" t="n">
         <v>30.4531</v>
       </c>
+      <c r="N8" s="3" t="n">
+        <v>30.4531</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1791,6 +1863,9 @@
       <c r="M9" s="3" t="n">
         <v>40.689</v>
       </c>
+      <c r="N9" s="3" t="n">
+        <v>40.689</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1838,6 +1913,9 @@
       <c r="M10" s="3" t="n">
         <v>45.9528</v>
       </c>
+      <c r="N10" s="3" t="n">
+        <v>45.9528</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1885,6 +1963,9 @@
       <c r="M11" s="3" t="n">
         <v>103.3395</v>
       </c>
+      <c r="N11" s="3" t="n">
+        <v>103.3395</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1932,6 +2013,9 @@
       <c r="M12" s="3" t="n">
         <v>218.423</v>
       </c>
+      <c r="N12" s="3" t="n">
+        <v>218.423</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1979,6 +2063,9 @@
       <c r="M13" s="3" t="n">
         <v>19.848</v>
       </c>
+      <c r="N13" s="3" t="n">
+        <v>19.848</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2026,6 +2113,9 @@
       <c r="M14" s="3" t="n">
         <v>38.0922</v>
       </c>
+      <c r="N14" s="3" t="n">
+        <v>38.0922</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2073,6 +2163,9 @@
       <c r="M15" s="3" t="n">
         <v>11.74</v>
       </c>
+      <c r="N15" s="3" t="n">
+        <v>11.74</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2120,6 +2213,9 @@
       <c r="M16" s="3" t="n">
         <v>24.3166</v>
       </c>
+      <c r="N16" s="3" t="n">
+        <v>24.3166</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2167,6 +2263,9 @@
       <c r="M17" s="3" t="n">
         <v>16.6235</v>
       </c>
+      <c r="N17" s="3" t="n">
+        <v>16.6235</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2214,6 +2313,9 @@
       <c r="M18" s="3" t="n">
         <v>45.44</v>
       </c>
+      <c r="N18" s="3" t="n">
+        <v>45.44</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2261,6 +2363,9 @@
       <c r="M19" s="3" t="n">
         <v>14.8854</v>
       </c>
+      <c r="N19" s="3" t="n">
+        <v>14.8854</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2308,6 +2413,9 @@
       <c r="M20" s="3" t="n">
         <v>9.07</v>
       </c>
+      <c r="N20" s="3" t="n">
+        <v>9.07</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2355,6 +2463,9 @@
       <c r="M21" s="3" t="n">
         <v>107.7303</v>
       </c>
+      <c r="N21" s="3" t="n">
+        <v>107.7303</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2402,6 +2513,9 @@
       <c r="M22" s="3" t="n">
         <v>42.665</v>
       </c>
+      <c r="N22" s="3" t="n">
+        <v>42.665</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2449,6 +2563,9 @@
       <c r="M23" s="3" t="n">
         <v>60.2124</v>
       </c>
+      <c r="N23" s="3" t="n">
+        <v>60.2124</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2496,6 +2613,9 @@
       <c r="M24" s="3" t="n">
         <v>27.9311</v>
       </c>
+      <c r="N24" s="3" t="n">
+        <v>27.9311</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2543,6 +2663,9 @@
       <c r="M25" s="3" t="n">
         <v>11.1514</v>
       </c>
+      <c r="N25" s="3" t="n">
+        <v>11.1514</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2590,6 +2713,9 @@
       <c r="M26" s="3" t="n">
         <v>8.598100000000001</v>
       </c>
+      <c r="N26" s="3" t="n">
+        <v>8.598100000000001</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2637,6 +2763,9 @@
       <c r="M27" s="3" t="n">
         <v>61.7452</v>
       </c>
+      <c r="N27" s="3" t="n">
+        <v>61.7452</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2684,6 +2813,9 @@
       <c r="M28" s="3" t="n">
         <v>104.7252</v>
       </c>
+      <c r="N28" s="3" t="n">
+        <v>104.7252</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2731,6 +2863,9 @@
       <c r="M29" s="3" t="n">
         <v>11.7996</v>
       </c>
+      <c r="N29" s="3" t="n">
+        <v>11.7996</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2778,6 +2913,9 @@
       <c r="M30" s="3" t="n">
         <v>15.0715</v>
       </c>
+      <c r="N30" s="3" t="n">
+        <v>15.0715</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2825,6 +2963,9 @@
       <c r="M31" s="3" t="n">
         <v>410.7949</v>
       </c>
+      <c r="N31" s="3" t="n">
+        <v>410.7949</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2872,6 +3013,9 @@
       <c r="M32" s="3" t="n">
         <v>10.06</v>
       </c>
+      <c r="N32" s="3" t="n">
+        <v>10.06</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2919,6 +3063,9 @@
       <c r="M33" s="3" t="n">
         <v>17.68</v>
       </c>
+      <c r="N33" s="3" t="n">
+        <v>17.68</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2966,6 +3113,9 @@
       <c r="M34" s="3" t="n">
         <v>209.5029</v>
       </c>
+      <c r="N34" s="3" t="n">
+        <v>209.5029</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3013,6 +3163,9 @@
       <c r="M35" s="3" t="n">
         <v>13.79</v>
       </c>
+      <c r="N35" s="3" t="n">
+        <v>13.79</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3060,6 +3213,9 @@
       <c r="M36" s="3" t="n">
         <v>347.7755</v>
       </c>
+      <c r="N36" s="3" t="n">
+        <v>347.7755</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3107,6 +3263,9 @@
       <c r="M37" s="3" t="n">
         <v>15.62</v>
       </c>
+      <c r="N37" s="3" t="n">
+        <v>15.62</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3154,6 +3313,9 @@
       <c r="M38" s="3" t="n">
         <v>13.9433</v>
       </c>
+      <c r="N38" s="3" t="n">
+        <v>13.9433</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3201,6 +3363,9 @@
       <c r="M39" s="3" t="n">
         <v>1007.1406</v>
       </c>
+      <c r="N39" s="3" t="n">
+        <v>1007.1406</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3246,6 +3411,9 @@
         <v>19.7344</v>
       </c>
       <c r="M40" s="3" t="n">
+        <v>19.7344</v>
+      </c>
+      <c r="N40" s="3" t="n">
         <v>19.7344</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily portfolio update 2026-05-19
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -39,6 +39,9 @@
       <sz val="10"/>
     </font>
     <font>
+      <color rgb="00006100"/>
+    </font>
+    <font>
       <color rgb="009C0006"/>
     </font>
     <font>
@@ -47,9 +50,6 @@
     <font>
       <b val="1"/>
       <color rgb="009C0006"/>
-    </font>
-    <font>
-      <color rgb="00006100"/>
     </font>
     <font>
       <b val="1"/>
@@ -97,20 +97,20 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -484,7 +484,7 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-05-18 06:12 IST</t>
+          <t>Generated: 2026-05-19 06:06 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4788357.0049389</v>
+        <v>4780932.4694812</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>318357.0049388995</v>
+        <v>310932.4694812</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.07122080647402675</v>
+        <v>0.06955983657297539</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>549061.9932250977</v>
+        <v>556466.4983062744</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-41720.02677490236</v>
+        <v>-34315.5216937256</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.07061830821273532</v>
+        <v>-0.05808491208606112</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5337418.998163997</v>
+        <v>5337398.967787474</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>276636.9781639976</v>
+        <v>276616.9477874748</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.05466289144063898</v>
+        <v>0.05465893347990413</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-05-18</t>
+          <t>Last snapshot: 2026-05-19</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -631,6 +631,7 @@
     <col width="21" customWidth="1" min="10" max="10"/>
     <col width="21" customWidth="1" min="11" max="11"/>
     <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -694,6 +695,11 @@
           <t>2026-05-18</t>
         </is>
       </c>
+      <c r="M1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -713,13 +719,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>527.3499755859375</v>
+        <v>569.4500122070312</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>42187.998046875</v>
-      </c>
-      <c r="G2" s="6" t="n">
-        <v>-1629.511953125002</v>
+        <v>45556.0009765625</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>1738.490976562498</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -736,6 +742,9 @@
       <c r="L2" s="3" t="n">
         <v>527.3499755859375</v>
       </c>
+      <c r="M2" s="3" t="n">
+        <v>569.4500122070312</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -782,13 +791,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1532.099975585938</v>
+        <v>1463.599975585938</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>30641.99951171875</v>
+        <v>29271.99951171875</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-1462.580488281252</v>
+        <v>-2832.580488281252</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -805,6 +814,9 @@
       <c r="L4" s="3" t="n">
         <v>1532.099975585938</v>
       </c>
+      <c r="M4" s="3" t="n">
+        <v>1463.599975585938</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -824,13 +836,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>657.5999755859375</v>
+        <v>671.8499755859375</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13151.99951171875</v>
+        <v>13436.99951171875</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1061.10048828125</v>
+        <v>-776.1004882812504</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -847,6 +859,9 @@
       <c r="L5" s="3" t="n">
         <v>657.5999755859375</v>
       </c>
+      <c r="M5" s="3" t="n">
+        <v>671.8499755859375</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -866,13 +881,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>386.2999877929688</v>
+        <v>391.6000061035156</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15451.99951171875</v>
+        <v>15664.00024414062</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2050.240488281252</v>
+        <v>-1838.239755859377</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -889,6 +904,9 @@
       <c r="L6" s="3" t="n">
         <v>386.2999877929688</v>
       </c>
+      <c r="M6" s="3" t="n">
+        <v>391.6000061035156</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -908,13 +926,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>236.8999938964844</v>
+        <v>247.6000061035156</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>23689.99938964844</v>
+        <v>24760.00061035156</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-2743.820610351562</v>
+        <v>-1673.819389648437</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -931,6 +949,9 @@
       <c r="L7" s="3" t="n">
         <v>236.8999938964844</v>
       </c>
+      <c r="M7" s="3" t="n">
+        <v>247.6000061035156</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -977,13 +998,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>19.01000022888184</v>
+        <v>19.06999969482422</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>28515.00034332275</v>
+        <v>28604.99954223633</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-2535.169656677244</v>
+        <v>-2445.17045776367</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1000,6 +1021,9 @@
       <c r="L9" s="3" t="n">
         <v>19.01000022888184</v>
       </c>
+      <c r="M9" s="3" t="n">
+        <v>19.06999969482422</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1019,13 +1043,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>509.75</v>
+        <v>505.3999938964844</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>50975</v>
+        <v>50539.99938964844</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-523.4800000000032</v>
+        <v>-958.4806103515657</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1042,6 +1066,9 @@
       <c r="L10" s="3" t="n">
         <v>509.75</v>
       </c>
+      <c r="M10" s="3" t="n">
+        <v>505.3999938964844</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1061,13 +1088,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>8.130000114440918</v>
+        <v>8.149999618530273</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>8130.000114440918</v>
+        <v>8149.999618530273</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-1711.209885559081</v>
+        <v>-1691.210381469726</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -1084,6 +1111,9 @@
       <c r="L11" s="3" t="n">
         <v>8.130000114440918</v>
       </c>
+      <c r="M11" s="3" t="n">
+        <v>8.149999618530273</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1103,13 +1133,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2472.39990234375</v>
+        <v>2550.89990234375</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>24723.9990234375</v>
+        <v>25508.9990234375</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2999.2509765625</v>
+        <v>-2214.2509765625</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -1126,6 +1156,9 @@
       <c r="L12" s="3" t="n">
         <v>2472.39990234375</v>
       </c>
+      <c r="M12" s="3" t="n">
+        <v>2550.89990234375</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1145,13 +1178,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>53.0099983215332</v>
+        <v>53.58000183105469</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>31805.99899291992</v>
+        <v>32148.00109863281</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-3225.76100708008</v>
+        <v>-2883.75890136719</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -1168,6 +1201,9 @@
       <c r="L13" s="3" t="n">
         <v>53.0099983215332</v>
       </c>
+      <c r="M13" s="3" t="n">
+        <v>53.58000183105469</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1187,13 +1223,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>731.2000122070312</v>
+        <v>743.5</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>36560.00061035156</v>
+        <v>37175</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-5902.50938964844</v>
+        <v>-5287.510000000002</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -1210,6 +1246,9 @@
       <c r="L14" s="3" t="n">
         <v>731.2000122070312</v>
       </c>
+      <c r="M14" s="3" t="n">
+        <v>743.5</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1283,13 +1322,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>433.0499877929688</v>
+        <v>458.5</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>21652.49938964844</v>
-      </c>
-      <c r="G17" s="6" t="n">
-        <v>-102.0306103515613</v>
+        <v>22925</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>1170.470000000001</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -1306,6 +1345,9 @@
       <c r="L17" s="3" t="n">
         <v>433.0499877929688</v>
       </c>
+      <c r="M17" s="3" t="n">
+        <v>458.5</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1325,13 +1367,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>398.0499877929688</v>
+        <v>409.5499877929688</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>39804.99877929688</v>
+        <v>40954.99877929688</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-6835.821220703125</v>
+        <v>-5685.821220703125</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -1348,6 +1390,9 @@
       <c r="L18" s="3" t="n">
         <v>398.0499877929688</v>
       </c>
+      <c r="M18" s="3" t="n">
+        <v>409.5499877929688</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -1359,10 +1404,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>549061.9932250977</v>
+        <v>556466.4983062744</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-41720.02677490236</v>
+        <v>-34315.5216937256</v>
       </c>
     </row>
   </sheetData>
@@ -1376,7 +1421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N41"/>
+  <dimension ref="A1:O41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1393,6 +1438,7 @@
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1466,6 +1512,11 @@
           <t>2026-05-18</t>
         </is>
       </c>
+      <c r="O1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1490,16 +1541,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.4905</v>
+        <v>56.5509</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>63409.56942099999</v>
+        <v>63477.36733379999</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>13409.56942099999</v>
+        <v>13477.36733379999</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.2681913884199998</v>
+        <v>0.2695473466759999</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -1516,6 +1567,9 @@
       <c r="N2" s="3" t="n">
         <v>56.4905</v>
       </c>
+      <c r="O2" s="3" t="n">
+        <v>56.5509</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1540,16 +1594,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.3959</v>
+        <v>25.6222</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>62352.34382670001</v>
+        <v>62907.9585286</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>2352.343826700009</v>
+        <v>2907.9585286</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.03920573044500016</v>
+        <v>0.04846597547666667</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -1566,6 +1620,9 @@
       <c r="N3" s="3" t="n">
         <v>25.3959</v>
       </c>
+      <c r="O3" s="3" t="n">
+        <v>25.6222</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1590,16 +1647,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.66</v>
+        <v>12.79</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>243149.13738</v>
+        <v>245645.92947</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>63149.13738</v>
+        <v>65645.92947</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.350828541</v>
+        <v>0.3646996081666667</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -1616,6 +1673,9 @@
       <c r="N4" s="3" t="n">
         <v>12.66</v>
       </c>
+      <c r="O4" s="3" t="n">
+        <v>12.79</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1640,16 +1700,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.4802</v>
+        <v>9.472</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>174000.4250576</v>
+        <v>173849.921536</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-35999.57494240001</v>
+        <v>-36150.07846400002</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.171426547344762</v>
+        <v>-0.1721432307809525</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -1666,6 +1726,9 @@
       <c r="N5" s="3" t="n">
         <v>9.4802</v>
       </c>
+      <c r="O5" s="3" t="n">
+        <v>9.472</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1690,16 +1753,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.4417</v>
+        <v>12.3444</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>52615.6631409</v>
+        <v>52204.1836788</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>2615.663140900004</v>
+        <v>2204.1836788</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.05231326281800008</v>
+        <v>0.044083673576</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -1716,6 +1779,9 @@
       <c r="N6" s="3" t="n">
         <v>12.4417</v>
       </c>
+      <c r="O6" s="3" t="n">
+        <v>12.3444</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1740,16 +1806,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>32.8663</v>
+        <v>33.2738</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>72504.37245200001</v>
+        <v>73403.33375200001</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>12504.37245200001</v>
+        <v>13403.33375200001</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2084062075333335</v>
+        <v>0.2233888958666668</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -1766,6 +1832,9 @@
       <c r="N7" s="3" t="n">
         <v>32.8663</v>
       </c>
+      <c r="O7" s="3" t="n">
+        <v>33.2738</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1790,16 +1859,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>30.4531</v>
+        <v>30.0521</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>48864.8310883</v>
+        <v>48221.3892953</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>-1135.168911699999</v>
+        <v>-1778.610704699997</v>
       </c>
       <c r="I8" s="13" t="n">
-        <v>-0.02270337823399998</v>
+        <v>-0.03557221409399994</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -1816,6 +1885,9 @@
       <c r="N8" s="3" t="n">
         <v>30.4531</v>
       </c>
+      <c r="O8" s="3" t="n">
+        <v>30.0521</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1840,16 +1912,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>40.689</v>
+        <v>40.9818</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>130993.881777</v>
+        <v>131936.5200474</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>30993.881777</v>
+        <v>31936.5200474</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.30993881777</v>
+        <v>0.319365200474</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -1866,6 +1938,9 @@
       <c r="N9" s="3" t="n">
         <v>40.689</v>
       </c>
+      <c r="O9" s="3" t="n">
+        <v>40.9818</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1890,16 +1965,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>45.9528</v>
+        <v>46.1686</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>130811.9516952</v>
+        <v>131426.2607074</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>30811.95169520001</v>
+        <v>31426.26070740001</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3081195169520001</v>
+        <v>0.3142626070740001</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -1916,6 +1991,9 @@
       <c r="N10" s="3" t="n">
         <v>45.9528</v>
       </c>
+      <c r="O10" s="3" t="n">
+        <v>46.1686</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1940,16 +2018,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>103.3395</v>
+        <v>103.1594</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31096.8190005</v>
+        <v>31042.6234886</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1096.8190005</v>
+        <v>1042.623488599998</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.03656063334999999</v>
+        <v>0.03475411628666662</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -1966,6 +2044,9 @@
       <c r="N11" s="3" t="n">
         <v>103.3395</v>
       </c>
+      <c r="O11" s="3" t="n">
+        <v>103.1594</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1990,16 +2071,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>218.423</v>
+        <v>217.978</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>101680.711806</v>
+        <v>101473.554516</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>1680.711805999992</v>
+        <v>1473.554516000004</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.01680711805999992</v>
+        <v>0.01473554516000004</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -2016,6 +2097,9 @@
       <c r="N12" s="3" t="n">
         <v>218.423</v>
       </c>
+      <c r="O12" s="3" t="n">
+        <v>217.978</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2040,16 +2124,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>19.848</v>
+        <v>19.89</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>229990.78404</v>
+        <v>230477.46345</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>29990.78403999997</v>
+        <v>30477.46345000001</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.1499539201999998</v>
+        <v>0.15238731725</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -2066,6 +2150,9 @@
       <c r="N13" s="3" t="n">
         <v>19.848</v>
       </c>
+      <c r="O13" s="3" t="n">
+        <v>19.89</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2090,16 +2177,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>38.0922</v>
+        <v>38.0354</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>137421.6492732</v>
+        <v>137216.7372524</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>37421.64927319999</v>
+        <v>37216.73725240002</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.3742164927319999</v>
+        <v>0.3721673725240002</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -2116,6 +2203,9 @@
       <c r="N14" s="3" t="n">
         <v>38.0922</v>
       </c>
+      <c r="O14" s="3" t="n">
+        <v>38.0354</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2140,16 +2230,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.74</v>
+        <v>11.6</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>114393.93778</v>
+        <v>113029.7852</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>14393.93778000001</v>
+        <v>13029.7852</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1439393778000001</v>
+        <v>0.130297852</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -2166,6 +2256,9 @@
       <c r="N15" s="3" t="n">
         <v>11.74</v>
       </c>
+      <c r="O15" s="3" t="n">
+        <v>11.6</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2190,16 +2283,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.3166</v>
+        <v>24.3001</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>139162.1510048</v>
+        <v>139067.7226928</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>39162.15100479999</v>
+        <v>39067.72269279999</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.3916215100479999</v>
+        <v>0.3906772269279999</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -2216,6 +2309,9 @@
       <c r="N16" s="3" t="n">
         <v>24.3166</v>
       </c>
+      <c r="O16" s="3" t="n">
+        <v>24.3001</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2240,16 +2336,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.6235</v>
+        <v>16.6438</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>54958.23853949999</v>
+        <v>55025.35149659999</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>4958.238539499995</v>
+        <v>5025.351496599993</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.0991647707899999</v>
+        <v>0.1005070299319999</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -2266,6 +2362,9 @@
       <c r="N17" s="3" t="n">
         <v>16.6235</v>
       </c>
+      <c r="O17" s="3" t="n">
+        <v>16.6438</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2290,16 +2389,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>45.44</v>
+        <v>45.38</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>85719.65183999999</v>
+        <v>85606.46568000001</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>5719.651839999991</v>
+        <v>5606.465680000008</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.0714956479999999</v>
+        <v>0.0700808210000001</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -2316,6 +2415,9 @@
       <c r="N18" s="3" t="n">
         <v>45.44</v>
       </c>
+      <c r="O18" s="3" t="n">
+        <v>45.38</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2340,16 +2442,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>14.8854</v>
+        <v>14.6525</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>215343.5986164</v>
+        <v>211974.288815</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>65343.59861640001</v>
+        <v>61974.28881499998</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.4356239907760001</v>
+        <v>0.4131619254333332</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -2366,6 +2468,9 @@
       <c r="N19" s="3" t="n">
         <v>14.8854</v>
       </c>
+      <c r="O19" s="3" t="n">
+        <v>14.6525</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2390,16 +2495,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.07</v>
+        <v>9.19</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>238140.13321</v>
+        <v>241290.82957</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-11859.86679</v>
+        <v>-8709.170430000027</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.04743946716</v>
+        <v>-0.03483668172000011</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -2416,6 +2521,9 @@
       <c r="N20" s="3" t="n">
         <v>9.07</v>
       </c>
+      <c r="O20" s="3" t="n">
+        <v>9.19</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2440,16 +2548,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>107.7303</v>
+        <v>106.959</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>163670.2278477</v>
+        <v>162498.423381</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-6329.772152299993</v>
+        <v>-7501.576618999999</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.03723395383705878</v>
+        <v>-0.04412692128823529</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -2466,6 +2574,9 @@
       <c r="N21" s="3" t="n">
         <v>107.7303</v>
       </c>
+      <c r="O21" s="3" t="n">
+        <v>106.959</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2516,6 +2627,9 @@
       <c r="N22" s="3" t="n">
         <v>42.665</v>
       </c>
+      <c r="O22" s="3" t="n">
+        <v>42.665</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2540,16 +2654,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>60.2124</v>
+        <v>59.6323</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>163564.9975908</v>
+        <v>161989.1750841</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>13564.99759080002</v>
+        <v>11989.17508410002</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.09043331727200013</v>
+        <v>0.07992783389400011</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -2566,6 +2680,9 @@
       <c r="N23" s="3" t="n">
         <v>60.2124</v>
       </c>
+      <c r="O23" s="3" t="n">
+        <v>59.6323</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2590,16 +2707,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>27.9311</v>
+        <v>27.5481</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>101484.4677046</v>
+        <v>100092.8808666</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>1484.4677046</v>
+        <v>92.88086660001136</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.014844677046</v>
+        <v>0.0009288086660001136</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -2616,6 +2733,9 @@
       <c r="N24" s="3" t="n">
         <v>27.9311</v>
       </c>
+      <c r="O24" s="3" t="n">
+        <v>27.5481</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2640,16 +2760,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.1514</v>
+        <v>11.147</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>183124.6554436</v>
+        <v>183052.400078</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-16875.3445564</v>
+        <v>-16947.59992199999</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.08437672278199999</v>
+        <v>-0.08473799960999998</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -2666,6 +2786,9 @@
       <c r="N25" s="3" t="n">
         <v>11.1514</v>
       </c>
+      <c r="O25" s="3" t="n">
+        <v>11.147</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2690,16 +2813,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>8.598100000000001</v>
+        <v>8.582599999999999</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>102676.0597415</v>
+        <v>102490.963159</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>-7323.940258499992</v>
+        <v>-7509.036841000008</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>-0.06658127507727266</v>
+        <v>-0.06826397128181826</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -2716,6 +2839,9 @@
       <c r="N26" s="3" t="n">
         <v>8.598100000000001</v>
       </c>
+      <c r="O26" s="3" t="n">
+        <v>8.582599999999999</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2740,16 +2866,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>61.7452</v>
+        <v>61.4908</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>99462.87287199999</v>
+        <v>99053.07008799999</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-10537.12712800001</v>
+        <v>-10946.92991200001</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.09579206480000006</v>
+        <v>-0.09951754465454551</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -2766,6 +2892,9 @@
       <c r="N27" s="3" t="n">
         <v>61.7452</v>
       </c>
+      <c r="O27" s="3" t="n">
+        <v>61.4908</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2790,16 +2919,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>104.7252</v>
+        <v>104.8093</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>346290.3156564</v>
+        <v>346568.4055101</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-33709.68434360001</v>
+        <v>-33431.59448989999</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.08870969564105265</v>
+        <v>-0.08797788023657892</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -2816,6 +2945,9 @@
       <c r="N28" s="3" t="n">
         <v>104.7252</v>
       </c>
+      <c r="O28" s="3" t="n">
+        <v>104.8093</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2840,16 +2972,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.7996</v>
+        <v>11.7385</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>113319.8539188</v>
+        <v>112733.0676655</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>13319.8539188</v>
+        <v>12733.0676655</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.133198539188</v>
+        <v>0.127330676655</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -2866,6 +2998,9 @@
       <c r="N29" s="3" t="n">
         <v>11.7996</v>
       </c>
+      <c r="O29" s="3" t="n">
+        <v>11.7385</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2890,16 +3025,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>15.0715</v>
+        <v>14.7715</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>111466.7190615</v>
+        <v>109247.9607615</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>11466.7190615</v>
+        <v>9247.960761499999</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.114667190615</v>
+        <v>0.09247960761499999</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -2916,6 +3051,9 @@
       <c r="N30" s="3" t="n">
         <v>15.0715</v>
       </c>
+      <c r="O30" s="3" t="n">
+        <v>14.7715</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2940,16 +3078,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>410.7949</v>
+        <v>405.4624</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>109304.306992</v>
+        <v>107885.435392</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>9304.306991999983</v>
+        <v>7885.435391999999</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.09304306991999983</v>
+        <v>0.07885435391999999</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -2966,6 +3104,9 @@
       <c r="N31" s="3" t="n">
         <v>410.7949</v>
       </c>
+      <c r="O31" s="3" t="n">
+        <v>405.4624</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2990,16 +3131,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.06</v>
+        <v>10</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>212667.9976</v>
+        <v>211399.6</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>12667.9976</v>
+        <v>11399.59999999998</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.06333998800000001</v>
+        <v>0.05699799999999988</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -3016,6 +3157,9 @@
       <c r="N32" s="3" t="n">
         <v>10.06</v>
       </c>
+      <c r="O32" s="3" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3040,16 +3184,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>17.68</v>
+        <v>17.5</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>63358.7552</v>
+        <v>62713.7</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>3358.7552</v>
+        <v>2713.699999999997</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.05597925333333333</v>
+        <v>0.04522833333333329</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -3066,6 +3210,9 @@
       <c r="N33" s="3" t="n">
         <v>17.68</v>
       </c>
+      <c r="O33" s="3" t="n">
+        <v>17.5</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3090,16 +3237,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>209.5029</v>
+        <v>212.5389</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>73646.7639399</v>
+        <v>74714.01205590001</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-6353.236060099996</v>
+        <v>-5285.987944099994</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.07941545075124995</v>
+        <v>-0.06607484930124992</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -3116,6 +3263,9 @@
       <c r="N34" s="3" t="n">
         <v>209.5029</v>
       </c>
+      <c r="O34" s="3" t="n">
+        <v>212.5389</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3140,16 +3290,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>13.79</v>
+        <v>13.67</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>98397.48316999999</v>
+        <v>97541.23241</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>-1602.516830000008</v>
+        <v>-2458.767590000003</v>
       </c>
       <c r="I35" s="13" t="n">
-        <v>-0.01602516830000008</v>
+        <v>-0.02458767590000003</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -3166,6 +3316,9 @@
       <c r="N35" s="3" t="n">
         <v>13.79</v>
       </c>
+      <c r="O35" s="3" t="n">
+        <v>13.67</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3190,16 +3343,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>347.7755</v>
+        <v>349.9214</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>161961.137003</v>
+        <v>162960.4955084</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>11961.13700300001</v>
+        <v>12960.4955084</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.0797409133533334</v>
+        <v>0.0864033033893333</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -3216,6 +3369,9 @@
       <c r="N36" s="3" t="n">
         <v>347.7755</v>
       </c>
+      <c r="O36" s="3" t="n">
+        <v>349.9214</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3240,16 +3396,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>15.62</v>
+        <v>15.633</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>58776.32618</v>
+        <v>58825.243737</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>8776.326179999996</v>
+        <v>8825.243736999997</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.1755265235999999</v>
+        <v>0.1765048747399999</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -3266,6 +3422,9 @@
       <c r="N37" s="3" t="n">
         <v>15.62</v>
       </c>
+      <c r="O37" s="3" t="n">
+        <v>15.633</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3290,16 +3449,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.9433</v>
+        <v>13.9157</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>83387.65467060001</v>
+        <v>83222.5933674</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>3387.654670600008</v>
+        <v>3222.593367399997</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.0423456833825001</v>
+        <v>0.04028241709249997</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -3316,6 +3475,9 @@
       <c r="N38" s="3" t="n">
         <v>13.9433</v>
       </c>
+      <c r="O38" s="3" t="n">
+        <v>13.9157</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3340,16 +3502,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1007.1406</v>
+        <v>1006.5403</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50237.1802686</v>
+        <v>50207.2367043</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>237.180268600001</v>
+        <v>207.2367042999977</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.00474360537200002</v>
+        <v>0.004144734085999953</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -3366,6 +3528,9 @@
       <c r="N39" s="3" t="n">
         <v>1007.1406</v>
       </c>
+      <c r="O39" s="3" t="n">
+        <v>1006.5403</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3390,16 +3555,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>19.7344</v>
+        <v>19.6371</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>99481.64322880001</v>
+        <v>98991.1513017</v>
       </c>
       <c r="H40" s="6" t="n">
-        <v>-518.3567711999931</v>
+        <v>-1008.848698300004</v>
       </c>
       <c r="I40" s="13" t="n">
-        <v>-0.005183567711999931</v>
+        <v>-0.01008848698300004</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -3416,6 +3581,9 @@
       <c r="N40" s="3" t="n">
         <v>19.7344</v>
       </c>
+      <c r="O40" s="3" t="n">
+        <v>19.6371</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
@@ -3427,13 +3595,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4788357.0049389</v>
+        <v>4780932.4694812</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>318357.0049389</v>
+        <v>310932.4694812</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.07122080647402684</v>
+        <v>0.06955983657297539</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-05-20
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -484,7 +484,7 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-05-19 06:06 IST</t>
+          <t>Generated: 2026-05-20 06:06 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4780932.4694812</v>
+        <v>4788622.6908943</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>310932.4694812</v>
+        <v>318622.6908943001</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.06955983657297539</v>
+        <v>0.07128024404794187</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>556466.4983062744</v>
+        <v>554636.0047988892</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-34315.5216937256</v>
+        <v>-36146.01520111086</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.05808491208606112</v>
+        <v>-0.06118333662407474</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5337398.967787474</v>
+        <v>5343258.695693189</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>276616.9477874748</v>
+        <v>282476.6756931897</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.05465893347990413</v>
+        <v>0.05581680352499943</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-05-19</t>
+          <t>Last snapshot: 2026-05-20</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -632,6 +632,7 @@
     <col width="21" customWidth="1" min="11" max="11"/>
     <col width="21" customWidth="1" min="12" max="12"/>
     <col width="21" customWidth="1" min="13" max="13"/>
+    <col width="21" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -700,6 +701,11 @@
           <t>2026-05-19</t>
         </is>
       </c>
+      <c r="N1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -719,13 +725,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>569.4500122070312</v>
+        <v>576.6500244140625</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>45556.0009765625</v>
+        <v>46132.001953125</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1738.490976562498</v>
+        <v>2314.491953124998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -745,6 +751,9 @@
       <c r="M2" s="3" t="n">
         <v>569.4500122070312</v>
       </c>
+      <c r="N2" s="3" t="n">
+        <v>576.6500244140625</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -791,13 +800,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1463.599975585938</v>
+        <v>1447</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>29271.99951171875</v>
+        <v>28940</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-2832.580488281252</v>
+        <v>-3164.580000000002</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -817,6 +826,9 @@
       <c r="M4" s="3" t="n">
         <v>1463.599975585938</v>
       </c>
+      <c r="N4" s="3" t="n">
+        <v>1447</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -836,13 +848,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>671.8499755859375</v>
+        <v>670.4000244140625</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13436.99951171875</v>
+        <v>13408.00048828125</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-776.1004882812504</v>
+        <v>-805.0995117187504</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -862,6 +874,9 @@
       <c r="M5" s="3" t="n">
         <v>671.8499755859375</v>
       </c>
+      <c r="N5" s="3" t="n">
+        <v>670.4000244140625</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -881,13 +896,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>391.6000061035156</v>
+        <v>384.8500061035156</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15664.00024414062</v>
+        <v>15394.00024414062</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-1838.239755859377</v>
+        <v>-2108.239755859377</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -907,6 +922,9 @@
       <c r="M6" s="3" t="n">
         <v>391.6000061035156</v>
       </c>
+      <c r="N6" s="3" t="n">
+        <v>384.8500061035156</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -926,13 +944,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>247.6000061035156</v>
+        <v>241.8000030517578</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>24760.00061035156</v>
+        <v>24180.00030517578</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-1673.819389648437</v>
+        <v>-2253.819694824218</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -952,6 +970,9 @@
       <c r="M7" s="3" t="n">
         <v>247.6000061035156</v>
       </c>
+      <c r="N7" s="3" t="n">
+        <v>241.8000030517578</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -998,13 +1019,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>19.06999969482422</v>
+        <v>18.85000038146973</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>28604.99954223633</v>
+        <v>28275.00057220459</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-2445.17045776367</v>
+        <v>-2775.169427795408</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1024,6 +1045,9 @@
       <c r="M9" s="3" t="n">
         <v>19.06999969482422</v>
       </c>
+      <c r="N9" s="3" t="n">
+        <v>18.85000038146973</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1043,13 +1067,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>505.3999938964844</v>
+        <v>507.7999877929688</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>50539.99938964844</v>
+        <v>50779.99877929688</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-958.4806103515657</v>
+        <v>-718.4812207031282</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1069,6 +1093,9 @@
       <c r="M10" s="3" t="n">
         <v>505.3999938964844</v>
       </c>
+      <c r="N10" s="3" t="n">
+        <v>507.7999877929688</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1114,6 +1141,9 @@
       <c r="M11" s="3" t="n">
         <v>8.149999618530273</v>
       </c>
+      <c r="N11" s="3" t="n">
+        <v>8.149999618530273</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1133,13 +1163,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2550.89990234375</v>
+        <v>2508.300048828125</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25508.9990234375</v>
+        <v>25083.00048828125</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2214.2509765625</v>
+        <v>-2640.24951171875</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -1159,6 +1189,9 @@
       <c r="M12" s="3" t="n">
         <v>2550.89990234375</v>
       </c>
+      <c r="N12" s="3" t="n">
+        <v>2508.300048828125</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1178,13 +1211,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>53.58000183105469</v>
+        <v>52.40999984741211</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>32148.00109863281</v>
+        <v>31445.99990844727</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-2883.75890136719</v>
+        <v>-3585.760091552736</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -1204,6 +1237,9 @@
       <c r="M13" s="3" t="n">
         <v>53.58000183105469</v>
       </c>
+      <c r="N13" s="3" t="n">
+        <v>52.40999984741211</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1223,13 +1259,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>743.5</v>
+        <v>729.1500244140625</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>37175</v>
+        <v>36457.50122070312</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-5287.510000000002</v>
+        <v>-6005.008779296877</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -1249,6 +1285,9 @@
       <c r="M14" s="3" t="n">
         <v>743.5</v>
       </c>
+      <c r="N14" s="3" t="n">
+        <v>729.1500244140625</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1322,13 +1361,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>458.5</v>
+        <v>464.2000122070312</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>22925</v>
+        <v>23210.00061035156</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>1170.470000000001</v>
+        <v>1455.470610351564</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -1348,6 +1387,9 @@
       <c r="M17" s="3" t="n">
         <v>458.5</v>
       </c>
+      <c r="N17" s="3" t="n">
+        <v>464.2000122070312</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1367,13 +1409,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>409.5499877929688</v>
+        <v>414.1000061035156</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>40954.99877929688</v>
+        <v>41410.00061035156</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-5685.821220703125</v>
+        <v>-5230.819389648437</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -1393,6 +1435,9 @@
       <c r="M18" s="3" t="n">
         <v>409.5499877929688</v>
       </c>
+      <c r="N18" s="3" t="n">
+        <v>414.1000061035156</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -1404,10 +1449,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>556466.4983062744</v>
+        <v>554636.0047988892</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-34315.5216937256</v>
+        <v>-36146.01520111085</v>
       </c>
     </row>
   </sheetData>
@@ -1421,7 +1466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O41"/>
+  <dimension ref="A1:P41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1439,6 +1484,7 @@
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="13" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1517,6 +1563,11 @@
           <t>2026-05-19</t>
         </is>
       </c>
+      <c r="P1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1541,16 +1592,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.5509</v>
+        <v>56.3099</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>63477.36733379999</v>
+        <v>63206.8491718</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>13477.36733379999</v>
+        <v>13206.8491718</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.2695473466759999</v>
+        <v>0.264136983436</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -1570,6 +1621,9 @@
       <c r="O2" s="3" t="n">
         <v>56.5509</v>
       </c>
+      <c r="P2" s="3" t="n">
+        <v>56.3099</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1594,16 +1648,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.6222</v>
+        <v>25.5901</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>62907.9585286</v>
+        <v>62829.1461913</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>2907.9585286</v>
+        <v>2829.146191300002</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.04846597547666667</v>
+        <v>0.0471524365216667</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -1623,6 +1677,9 @@
       <c r="O3" s="3" t="n">
         <v>25.6222</v>
       </c>
+      <c r="P3" s="3" t="n">
+        <v>25.5901</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1647,16 +1704,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.79</v>
+        <v>12.48</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>245645.92947</v>
+        <v>239692.04064</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>65645.92947</v>
+        <v>59692.04064000002</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3646996081666667</v>
+        <v>0.3316224480000001</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -1676,6 +1733,9 @@
       <c r="O4" s="3" t="n">
         <v>12.79</v>
       </c>
+      <c r="P4" s="3" t="n">
+        <v>12.48</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1700,16 +1760,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.472</v>
+        <v>9.542999999999999</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>173849.921536</v>
+        <v>175153.061784</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-36150.07846400002</v>
+        <v>-34846.93821600001</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1721432307809525</v>
+        <v>-0.1659378010285715</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -1729,6 +1789,9 @@
       <c r="O5" s="3" t="n">
         <v>9.472</v>
       </c>
+      <c r="P5" s="3" t="n">
+        <v>9.542999999999999</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1753,16 +1816,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.3444</v>
+        <v>12.3769</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>52204.1836788</v>
+        <v>52341.6254313</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>2204.1836788</v>
+        <v>2341.625431299995</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.044083673576</v>
+        <v>0.04683250862599991</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -1782,6 +1845,9 @@
       <c r="O6" s="3" t="n">
         <v>12.3444</v>
       </c>
+      <c r="P6" s="3" t="n">
+        <v>12.3769</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1806,16 +1872,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.2738</v>
+        <v>33.2956</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>73403.33375200001</v>
+        <v>73451.425424</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>13403.33375200001</v>
+        <v>13451.425424</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2233888958666668</v>
+        <v>0.2241904237333333</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -1835,6 +1901,9 @@
       <c r="O7" s="3" t="n">
         <v>33.2738</v>
       </c>
+      <c r="P7" s="3" t="n">
+        <v>33.2956</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1859,16 +1928,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>30.0521</v>
+        <v>30.1484</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>48221.3892953</v>
+        <v>48375.9116012</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>-1778.610704699997</v>
+        <v>-1624.088398799999</v>
       </c>
       <c r="I8" s="13" t="n">
-        <v>-0.03557221409399994</v>
+        <v>-0.03248176797599998</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -1888,6 +1957,9 @@
       <c r="O8" s="3" t="n">
         <v>30.0521</v>
       </c>
+      <c r="P8" s="3" t="n">
+        <v>30.1484</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1912,16 +1984,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>40.9818</v>
+        <v>40.1932</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>131936.5200474</v>
+        <v>129397.7067276</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>31936.5200474</v>
+        <v>29397.70672759999</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.319365200474</v>
+        <v>0.2939770672759999</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -1941,6 +2013,9 @@
       <c r="O9" s="3" t="n">
         <v>40.9818</v>
       </c>
+      <c r="P9" s="3" t="n">
+        <v>40.1932</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1965,16 +2040,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>46.1686</v>
+        <v>45.9545</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>131426.2607074</v>
+        <v>130816.7910155</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>31426.26070740001</v>
+        <v>30816.79101550001</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3142626070740001</v>
+        <v>0.3081679101550001</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -1994,6 +2069,9 @@
       <c r="O10" s="3" t="n">
         <v>46.1686</v>
       </c>
+      <c r="P10" s="3" t="n">
+        <v>45.9545</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2018,16 +2096,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>103.1594</v>
+        <v>102.5398</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31042.6234886</v>
+        <v>30856.1740762</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1042.623488599998</v>
+        <v>856.1740761999972</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.03475411628666662</v>
+        <v>0.02853913587333324</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -2047,6 +2125,9 @@
       <c r="O11" s="3" t="n">
         <v>103.1594</v>
       </c>
+      <c r="P11" s="3" t="n">
+        <v>102.5398</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2071,16 +2152,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>217.978</v>
+        <v>219.799</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>101473.554516</v>
+        <v>102321.270078</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>1473.554516000004</v>
+        <v>2321.270078000001</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.01473554516000004</v>
+        <v>0.02321270078000002</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -2100,6 +2181,9 @@
       <c r="O12" s="3" t="n">
         <v>217.978</v>
       </c>
+      <c r="P12" s="3" t="n">
+        <v>219.799</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2124,16 +2208,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>19.89</v>
+        <v>20.034</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>230477.46345</v>
+        <v>232146.07857</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>30477.46345000001</v>
+        <v>32146.07856999998</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.15238731725</v>
+        <v>0.1607303928499999</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -2153,6 +2237,9 @@
       <c r="O13" s="3" t="n">
         <v>19.89</v>
       </c>
+      <c r="P13" s="3" t="n">
+        <v>20.034</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2177,16 +2264,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>38.0354</v>
+        <v>37.4905</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>137216.7372524</v>
+        <v>135250.952743</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>37216.73725240002</v>
+        <v>35250.952743</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.3721673725240002</v>
+        <v>0.35250952743</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -2206,6 +2293,9 @@
       <c r="O14" s="3" t="n">
         <v>38.0354</v>
       </c>
+      <c r="P14" s="3" t="n">
+        <v>37.4905</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2230,16 +2320,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.6</v>
+        <v>11.65</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>113029.7852</v>
+        <v>113516.98255</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>13029.7852</v>
+        <v>13516.98255</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.130297852</v>
+        <v>0.1351698255</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -2259,6 +2349,9 @@
       <c r="O15" s="3" t="n">
         <v>11.6</v>
       </c>
+      <c r="P15" s="3" t="n">
+        <v>11.65</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2283,16 +2376,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.3001</v>
+        <v>24.1654</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>139067.7226928</v>
+        <v>138296.8442912</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>39067.72269279999</v>
+        <v>38296.84429120002</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.3906772269279999</v>
+        <v>0.3829684429120002</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -2312,6 +2405,9 @@
       <c r="O16" s="3" t="n">
         <v>24.3001</v>
       </c>
+      <c r="P16" s="3" t="n">
+        <v>24.1654</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2336,16 +2432,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.6438</v>
+        <v>16.6456</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55025.35149659999</v>
+        <v>55031.3023992</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5025.351496599993</v>
+        <v>5031.302399200002</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1005070299319999</v>
+        <v>0.100626047984</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -2365,6 +2461,9 @@
       <c r="O17" s="3" t="n">
         <v>16.6438</v>
       </c>
+      <c r="P17" s="3" t="n">
+        <v>16.6456</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2389,16 +2488,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>45.38</v>
+        <v>45.6</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>85606.46568000001</v>
+        <v>86021.4816</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>5606.465680000008</v>
+        <v>6021.481599999999</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.0700808210000001</v>
+        <v>0.07526851999999999</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -2418,6 +2517,9 @@
       <c r="O18" s="3" t="n">
         <v>45.38</v>
       </c>
+      <c r="P18" s="3" t="n">
+        <v>45.6</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2442,16 +2544,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>14.6525</v>
+        <v>14.1914</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>211974.288815</v>
+        <v>205303.6630124</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>61974.28881499998</v>
+        <v>55303.66301239998</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.4131619254333332</v>
+        <v>0.3686910867493332</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -2471,6 +2573,9 @@
       <c r="O19" s="3" t="n">
         <v>14.6525</v>
       </c>
+      <c r="P19" s="3" t="n">
+        <v>14.1914</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2495,16 +2600,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.19</v>
+        <v>9.4</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>241290.82957</v>
+        <v>246804.5482</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-8709.170430000027</v>
+        <v>-3195.451799999981</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.03483668172000011</v>
+        <v>-0.01278180719999992</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -2524,6 +2629,9 @@
       <c r="O20" s="3" t="n">
         <v>9.19</v>
       </c>
+      <c r="P20" s="3" t="n">
+        <v>9.4</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2548,16 +2656,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>106.959</v>
+        <v>107.4649</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>162498.423381</v>
+        <v>163267.0165091</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-7501.576618999999</v>
+        <v>-6732.983490899991</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.04412692128823529</v>
+        <v>-0.03960578524058819</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -2577,6 +2685,9 @@
       <c r="O21" s="3" t="n">
         <v>106.959</v>
       </c>
+      <c r="P21" s="3" t="n">
+        <v>107.4649</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2601,16 +2712,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>42.665</v>
+        <v>42.192</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>65467.7359</v>
+        <v>64741.93632</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>5467.7359</v>
+        <v>4741.936320000001</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.09112893166666666</v>
+        <v>0.07903227200000001</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -2630,6 +2741,9 @@
       <c r="O22" s="3" t="n">
         <v>42.665</v>
       </c>
+      <c r="P22" s="3" t="n">
+        <v>42.192</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2654,16 +2768,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>59.6323</v>
+        <v>59.7524</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>161989.1750841</v>
+        <v>162315.4227708</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>11989.17508410002</v>
+        <v>12315.42277080001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.07992783389400011</v>
+        <v>0.08210281847200007</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -2683,6 +2797,9 @@
       <c r="O23" s="3" t="n">
         <v>59.6323</v>
       </c>
+      <c r="P23" s="3" t="n">
+        <v>59.7524</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2707,16 +2824,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>27.5481</v>
+        <v>27.747</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>100092.8808666</v>
+        <v>100815.561342</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>92.88086660001136</v>
+        <v>815.5613420000009</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.0009288086660001136</v>
+        <v>0.00815561342000001</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -2736,6 +2853,9 @@
       <c r="O24" s="3" t="n">
         <v>27.5481</v>
       </c>
+      <c r="P24" s="3" t="n">
+        <v>27.747</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2760,16 +2880,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.147</v>
+        <v>11.2647</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>183052.400078</v>
+        <v>184985.2311078</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-16947.59992199999</v>
+        <v>-15014.76889220002</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.08473799960999998</v>
+        <v>-0.07507384446100011</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -2789,6 +2909,9 @@
       <c r="O25" s="3" t="n">
         <v>11.147</v>
       </c>
+      <c r="P25" s="3" t="n">
+        <v>11.2647</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2813,16 +2936,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>8.582599999999999</v>
+        <v>8.805400000000001</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>102490.963159</v>
+        <v>105151.577261</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>-7509.036841000008</v>
+        <v>-4848.422738999987</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>-0.06826397128181826</v>
+        <v>-0.04407657035454533</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -2842,6 +2965,9 @@
       <c r="O26" s="3" t="n">
         <v>8.582599999999999</v>
       </c>
+      <c r="P26" s="3" t="n">
+        <v>8.805400000000001</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2866,16 +2992,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>61.4908</v>
+        <v>61.8656</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>99053.07008799999</v>
+        <v>99656.82041599999</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-10946.92991200001</v>
+        <v>-10343.17958400001</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.09951754465454551</v>
+        <v>-0.09402890530909103</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -2895,6 +3021,9 @@
       <c r="O27" s="3" t="n">
         <v>61.4908</v>
       </c>
+      <c r="P27" s="3" t="n">
+        <v>61.8656</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2919,16 +3048,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>104.8093</v>
+        <v>105.9515</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>346568.4055101</v>
+        <v>350345.2691355</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-33431.59448989999</v>
+        <v>-29654.73086449999</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.08797788023657892</v>
+        <v>-0.0780387654328947</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -2948,6 +3077,9 @@
       <c r="O28" s="3" t="n">
         <v>104.8093</v>
       </c>
+      <c r="P28" s="3" t="n">
+        <v>105.9515</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2972,16 +3104,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.7385</v>
+        <v>11.6947</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>112733.0676655</v>
+        <v>112312.4254741</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>12733.0676655</v>
+        <v>12312.42547409999</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.127330676655</v>
+        <v>0.1231242547409999</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -3001,6 +3133,9 @@
       <c r="O29" s="3" t="n">
         <v>11.7385</v>
       </c>
+      <c r="P29" s="3" t="n">
+        <v>11.6947</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3025,16 +3160,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>14.7715</v>
+        <v>14.8786</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>109247.9607615</v>
+        <v>110040.0574746</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>9247.960761499999</v>
+        <v>10040.05747460001</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.09247960761499999</v>
+        <v>0.1004005747460001</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -3054,6 +3189,9 @@
       <c r="O30" s="3" t="n">
         <v>14.7715</v>
       </c>
+      <c r="P30" s="3" t="n">
+        <v>14.8786</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3078,16 +3216,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>405.4624</v>
+        <v>407.1528</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>107885.435392</v>
+        <v>108335.217024</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>7885.435391999999</v>
+        <v>8335.217023999998</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.07885435391999999</v>
+        <v>0.08335217023999998</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -3107,6 +3245,9 @@
       <c r="O31" s="3" t="n">
         <v>405.4624</v>
       </c>
+      <c r="P31" s="3" t="n">
+        <v>407.1528</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3131,16 +3272,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10</v>
+        <v>10.05</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>211399.6</v>
+        <v>212456.598</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>11399.59999999998</v>
+        <v>12456.598</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.05699799999999988</v>
+        <v>0.06228298999999999</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -3160,6 +3301,9 @@
       <c r="O32" s="3" t="n">
         <v>10</v>
       </c>
+      <c r="P32" s="3" t="n">
+        <v>10.05</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3184,16 +3328,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>17.5</v>
+        <v>17.69</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>62713.7</v>
+        <v>63394.5916</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>2713.699999999997</v>
+        <v>3394.5916</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.04522833333333329</v>
+        <v>0.05657652666666666</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -3213,6 +3357,9 @@
       <c r="O33" s="3" t="n">
         <v>17.5</v>
       </c>
+      <c r="P33" s="3" t="n">
+        <v>17.69</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3237,16 +3384,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>212.5389</v>
+        <v>215.9582</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>74714.01205590001</v>
+        <v>75916.0020042</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-5285.987944099994</v>
+        <v>-4083.997995800004</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.06607484930124992</v>
+        <v>-0.05104997494750005</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -3266,6 +3413,9 @@
       <c r="O34" s="3" t="n">
         <v>212.5389</v>
       </c>
+      <c r="P34" s="3" t="n">
+        <v>215.9582</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3319,6 +3469,9 @@
       <c r="O35" s="3" t="n">
         <v>13.67</v>
       </c>
+      <c r="P35" s="3" t="n">
+        <v>13.67</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3343,16 +3496,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>349.9214</v>
+        <v>352.2352</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>162960.4955084</v>
+        <v>164038.0460512</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>12960.4955084</v>
+        <v>14038.04605120001</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.0864033033893333</v>
+        <v>0.09358697367466676</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -3372,6 +3525,9 @@
       <c r="O36" s="3" t="n">
         <v>349.9214</v>
       </c>
+      <c r="P36" s="3" t="n">
+        <v>352.2352</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3396,16 +3552,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>15.633</v>
+        <v>15.742</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>58825.243737</v>
+        <v>59235.39863800001</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>8825.243736999997</v>
+        <v>9235.398638000006</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.1765048747399999</v>
+        <v>0.1847079727600001</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -3425,6 +3581,9 @@
       <c r="O37" s="3" t="n">
         <v>15.633</v>
       </c>
+      <c r="P37" s="3" t="n">
+        <v>15.742</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3449,16 +3608,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.9157</v>
+        <v>13.9705</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>83222.5933674</v>
+        <v>83550.323781</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>3222.593367399997</v>
+        <v>3550.323780999999</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.04028241709249997</v>
+        <v>0.04437904726249999</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -3478,6 +3637,9 @@
       <c r="O38" s="3" t="n">
         <v>13.9157</v>
       </c>
+      <c r="P38" s="3" t="n">
+        <v>13.9705</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3502,16 +3664,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1006.5403</v>
+        <v>1007.0063</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50207.2367043</v>
+        <v>50230.4812503</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>207.2367042999977</v>
+        <v>230.4812502999994</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.004144734085999953</v>
+        <v>0.004609625005999988</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -3531,6 +3693,9 @@
       <c r="O39" s="3" t="n">
         <v>1006.5403</v>
       </c>
+      <c r="P39" s="3" t="n">
+        <v>1007.0063</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3555,16 +3720,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>19.6371</v>
+        <v>19.734</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>98991.1513017</v>
+        <v>99479.626818</v>
       </c>
       <c r="H40" s="6" t="n">
-        <v>-1008.848698300004</v>
+        <v>-520.3731819999957</v>
       </c>
       <c r="I40" s="13" t="n">
-        <v>-0.01008848698300004</v>
+        <v>-0.005203731819999957</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -3584,6 +3749,9 @@
       <c r="O40" s="3" t="n">
         <v>19.6371</v>
       </c>
+      <c r="P40" s="3" t="n">
+        <v>19.734</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
@@ -3595,13 +3763,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4780932.4694812</v>
+        <v>4788622.6908943</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>310932.4694812</v>
+        <v>318622.6908943</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.06955983657297539</v>
+        <v>0.07128024404794184</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-05-21
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-05-20 06:06 IST</t>
+          <t>Generated: 2026-05-21 06:09 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4788622.6908943</v>
+        <v>4815373.626656</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>318622.6908943001</v>
+        <v>345373.6266559996</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.07128024404794187</v>
+        <v>0.07726479343534666</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>554636.0047988892</v>
+        <v>555583.4997634888</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-36146.01520111086</v>
+        <v>-35198.52023651125</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.06118333662407474</v>
+        <v>-0.05957953872142427</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5343258.695693189</v>
+        <v>5370957.126419488</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>282476.6756931897</v>
+        <v>310175.1064194888</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.05581680352499943</v>
+        <v>0.06128995581981</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-05-20</t>
+          <t>Last snapshot: 2026-05-21</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:O19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -633,6 +633,7 @@
     <col width="21" customWidth="1" min="12" max="12"/>
     <col width="21" customWidth="1" min="13" max="13"/>
     <col width="21" customWidth="1" min="14" max="14"/>
+    <col width="21" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -706,6 +707,11 @@
           <t>2026-05-20</t>
         </is>
       </c>
+      <c r="O1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -725,13 +731,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>576.6500244140625</v>
+        <v>572</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>46132.001953125</v>
+        <v>45760</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>2314.491953124998</v>
+        <v>1942.489999999998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -754,6 +760,9 @@
       <c r="N2" s="3" t="n">
         <v>576.6500244140625</v>
       </c>
+      <c r="O2" s="3" t="n">
+        <v>572</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -800,13 +809,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1447</v>
+        <v>1475.5</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>28940</v>
+        <v>29510</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-3164.580000000002</v>
+        <v>-2594.580000000002</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -829,6 +838,9 @@
       <c r="N4" s="3" t="n">
         <v>1447</v>
       </c>
+      <c r="O4" s="3" t="n">
+        <v>1475.5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -848,13 +860,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>670.4000244140625</v>
+        <v>658.6500244140625</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13408.00048828125</v>
+        <v>13173.00048828125</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-805.0995117187504</v>
+        <v>-1040.09951171875</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -877,6 +889,9 @@
       <c r="N5" s="3" t="n">
         <v>670.4000244140625</v>
       </c>
+      <c r="O5" s="3" t="n">
+        <v>658.6500244140625</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -896,13 +911,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>384.8500061035156</v>
+        <v>386.5</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15394.00024414062</v>
+        <v>15460</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2108.239755859377</v>
+        <v>-2042.240000000002</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -925,6 +940,9 @@
       <c r="N6" s="3" t="n">
         <v>384.8500061035156</v>
       </c>
+      <c r="O6" s="3" t="n">
+        <v>386.5</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -944,13 +962,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>241.8000030517578</v>
+        <v>240.1999969482422</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>24180.00030517578</v>
+        <v>24019.99969482422</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-2253.819694824218</v>
+        <v>-2413.820305175781</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -973,6 +991,9 @@
       <c r="N7" s="3" t="n">
         <v>241.8000030517578</v>
       </c>
+      <c r="O7" s="3" t="n">
+        <v>240.1999969482422</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1019,13 +1040,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>18.85000038146973</v>
+        <v>19.01000022888184</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>28275.00057220459</v>
+        <v>28515.00034332275</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-2775.169427795408</v>
+        <v>-2535.169656677244</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1048,6 +1069,9 @@
       <c r="N9" s="3" t="n">
         <v>18.85000038146973</v>
       </c>
+      <c r="O9" s="3" t="n">
+        <v>19.01000022888184</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1067,13 +1091,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>507.7999877929688</v>
+        <v>502.5</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>50779.99877929688</v>
+        <v>50250</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-718.4812207031282</v>
+        <v>-1248.480000000003</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1096,6 +1120,9 @@
       <c r="N10" s="3" t="n">
         <v>507.7999877929688</v>
       </c>
+      <c r="O10" s="3" t="n">
+        <v>502.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1115,13 +1142,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>8.149999618530273</v>
+        <v>8.319999694824219</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>8149.999618530273</v>
+        <v>8319.999694824219</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-1691.210381469726</v>
+        <v>-1521.21030517578</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -1144,6 +1171,9 @@
       <c r="N11" s="3" t="n">
         <v>8.149999618530273</v>
       </c>
+      <c r="O11" s="3" t="n">
+        <v>8.319999694824219</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1163,13 +1193,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2508.300048828125</v>
+        <v>2525</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25083.00048828125</v>
+        <v>25250</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2640.24951171875</v>
+        <v>-2473.25</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -1192,6 +1222,9 @@
       <c r="N12" s="3" t="n">
         <v>2508.300048828125</v>
       </c>
+      <c r="O12" s="3" t="n">
+        <v>2525</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1211,13 +1244,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>52.40999984741211</v>
+        <v>53.45000076293945</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>31445.99990844727</v>
+        <v>32070.00045776367</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-3585.760091552736</v>
+        <v>-2961.75954223633</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -1240,6 +1273,9 @@
       <c r="N13" s="3" t="n">
         <v>52.40999984741211</v>
       </c>
+      <c r="O13" s="3" t="n">
+        <v>53.45000076293945</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1259,13 +1295,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>729.1500244140625</v>
+        <v>735</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>36457.50122070312</v>
+        <v>36750</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-6005.008779296877</v>
+        <v>-5712.510000000002</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -1288,6 +1324,9 @@
       <c r="N14" s="3" t="n">
         <v>729.1500244140625</v>
       </c>
+      <c r="O14" s="3" t="n">
+        <v>735</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1361,13 +1400,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>464.2000122070312</v>
+        <v>472.6000061035156</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>23210.00061035156</v>
+        <v>23630.00030517578</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>1455.470610351564</v>
+        <v>1875.470305175782</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -1390,6 +1429,9 @@
       <c r="N17" s="3" t="n">
         <v>464.2000122070312</v>
       </c>
+      <c r="O17" s="3" t="n">
+        <v>472.6000061035156</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1409,13 +1451,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>414.1000061035156</v>
+        <v>411.0499877929688</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>41410.00061035156</v>
+        <v>41104.99877929688</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-5230.819389648437</v>
+        <v>-5535.821220703125</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -1438,6 +1480,9 @@
       <c r="N18" s="3" t="n">
         <v>414.1000061035156</v>
       </c>
+      <c r="O18" s="3" t="n">
+        <v>411.0499877929688</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -1449,10 +1494,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>554636.0047988892</v>
+        <v>555583.4997634888</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-36146.01520111085</v>
+        <v>-35198.52023651124</v>
       </c>
     </row>
   </sheetData>
@@ -1466,7 +1511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P41"/>
+  <dimension ref="A1:Q41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1485,6 +1530,7 @@
     <col width="13" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1568,6 +1614,11 @@
           <t>2026-05-20</t>
         </is>
       </c>
+      <c r="Q1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1592,16 +1643,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.3099</v>
+        <v>56.9033</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>63206.8491718</v>
+        <v>63872.9299906</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>13206.8491718</v>
+        <v>13872.9299906</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.264136983436</v>
+        <v>0.2774585998120001</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -1624,6 +1675,9 @@
       <c r="P2" s="3" t="n">
         <v>56.3099</v>
       </c>
+      <c r="Q2" s="3" t="n">
+        <v>56.9033</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1648,16 +1702,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.5901</v>
+        <v>25.5927</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>62829.1461913</v>
+        <v>62835.52974510001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>2829.146191300002</v>
+        <v>2835.529745100008</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.0471524365216667</v>
+        <v>0.04725882908500013</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -1680,6 +1734,9 @@
       <c r="P3" s="3" t="n">
         <v>25.5901</v>
       </c>
+      <c r="Q3" s="3" t="n">
+        <v>25.5927</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1704,16 +1761,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.48</v>
+        <v>12.64</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>239692.04064</v>
+        <v>242765.01552</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>59692.04064000002</v>
+        <v>62765.01552000002</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3316224480000001</v>
+        <v>0.3486945306666668</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -1736,6 +1793,9 @@
       <c r="P4" s="3" t="n">
         <v>12.48</v>
       </c>
+      <c r="Q4" s="3" t="n">
+        <v>12.64</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1760,16 +1820,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.542999999999999</v>
+        <v>9.527799999999999</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>175153.061784</v>
+        <v>174874.0796464</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-34846.93821600001</v>
+        <v>-35125.92035360003</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1659378010285715</v>
+        <v>-0.1672662873980954</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -1792,6 +1852,9 @@
       <c r="P5" s="3" t="n">
         <v>9.542999999999999</v>
       </c>
+      <c r="Q5" s="3" t="n">
+        <v>9.527799999999999</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1816,16 +1879,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.3769</v>
+        <v>12.5431</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>52341.6254313</v>
+        <v>53044.4814087</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>2341.625431299995</v>
+        <v>3044.481408700005</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.04683250862599991</v>
+        <v>0.0608896281740001</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -1848,6 +1911,9 @@
       <c r="P6" s="3" t="n">
         <v>12.3769</v>
       </c>
+      <c r="Q6" s="3" t="n">
+        <v>12.5431</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1872,16 +1938,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.2956</v>
+        <v>33.5886</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>73451.425424</v>
+        <v>74097.795144</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>13451.425424</v>
+        <v>14097.795144</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2241904237333333</v>
+        <v>0.2349632524</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -1904,6 +1970,9 @@
       <c r="P7" s="3" t="n">
         <v>33.2956</v>
       </c>
+      <c r="Q7" s="3" t="n">
+        <v>33.5886</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1928,16 +1997,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>30.1484</v>
+        <v>30.2942</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>48375.9116012</v>
+        <v>48609.8612606</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>-1624.088398799999</v>
+        <v>-1390.138739399998</v>
       </c>
       <c r="I8" s="13" t="n">
-        <v>-0.03248176797599998</v>
+        <v>-0.02780277478799995</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -1960,6 +2029,9 @@
       <c r="P8" s="3" t="n">
         <v>30.1484</v>
       </c>
+      <c r="Q8" s="3" t="n">
+        <v>30.2942</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1984,16 +2056,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>40.1932</v>
+        <v>40.8338</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>129397.7067276</v>
+        <v>131460.0498834</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>29397.70672759999</v>
+        <v>31460.0498834</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.2939770672759999</v>
+        <v>0.314600498834</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -2016,6 +2088,9 @@
       <c r="P9" s="3" t="n">
         <v>40.1932</v>
       </c>
+      <c r="Q9" s="3" t="n">
+        <v>40.8338</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2040,16 +2115,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>45.9545</v>
+        <v>46.3181</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>130816.7910155</v>
+        <v>131851.8362279</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>30816.79101550001</v>
+        <v>31851.8362279</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3081679101550001</v>
+        <v>0.318518362279</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -2072,6 +2147,9 @@
       <c r="P10" s="3" t="n">
         <v>45.9545</v>
       </c>
+      <c r="Q10" s="3" t="n">
+        <v>46.3181</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2096,16 +2174,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>102.5398</v>
+        <v>104.5549</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>30856.1740762</v>
+        <v>31462.5559531</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>856.1740761999972</v>
+        <v>1462.5559531</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.02853913587333324</v>
+        <v>0.04875186510333333</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -2128,6 +2206,9 @@
       <c r="P11" s="3" t="n">
         <v>102.5398</v>
       </c>
+      <c r="Q11" s="3" t="n">
+        <v>104.5549</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2152,16 +2233,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>219.799</v>
+        <v>220.391</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>102321.270078</v>
+        <v>102596.859102</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>2321.270078000001</v>
+        <v>2596.859101999988</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.02321270078000002</v>
+        <v>0.02596859101999988</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -2184,6 +2265,9 @@
       <c r="P12" s="3" t="n">
         <v>219.799</v>
       </c>
+      <c r="Q12" s="3" t="n">
+        <v>220.391</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2208,16 +2292,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>20.034</v>
+        <v>20.091</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>232146.07857</v>
+        <v>232806.572055</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>32146.07856999998</v>
+        <v>32806.572055</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.1607303928499999</v>
+        <v>0.164032860275</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -2240,6 +2324,9 @@
       <c r="P13" s="3" t="n">
         <v>20.034</v>
       </c>
+      <c r="Q13" s="3" t="n">
+        <v>20.091</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2264,16 +2351,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>37.4905</v>
+        <v>37.7689</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>135250.952743</v>
+        <v>136255.3102534</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>35250.952743</v>
+        <v>36255.31025340001</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.35250952743</v>
+        <v>0.3625531025340001</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -2296,6 +2383,9 @@
       <c r="P14" s="3" t="n">
         <v>37.4905</v>
       </c>
+      <c r="Q14" s="3" t="n">
+        <v>37.7689</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2320,16 +2410,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.65</v>
+        <v>11.75</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>113516.98255</v>
+        <v>114491.37725</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>13516.98255</v>
+        <v>14491.37725000001</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1351698255</v>
+        <v>0.1449137725</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -2352,6 +2442,9 @@
       <c r="P15" s="3" t="n">
         <v>11.65</v>
       </c>
+      <c r="Q15" s="3" t="n">
+        <v>11.75</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2376,16 +2469,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.1654</v>
+        <v>24.694</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>138296.8442912</v>
+        <v>141321.984032</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>38296.84429120002</v>
+        <v>41321.98403199998</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.3829684429120002</v>
+        <v>0.4132198403199998</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -2408,6 +2501,9 @@
       <c r="P16" s="3" t="n">
         <v>24.1654</v>
       </c>
+      <c r="Q16" s="3" t="n">
+        <v>24.694</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2432,16 +2528,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.6456</v>
+        <v>16.7399</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55031.3023992</v>
+        <v>55343.06357429999</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5031.302399200002</v>
+        <v>5343.063574299995</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.100626047984</v>
+        <v>0.1068612714859999</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -2464,6 +2560,9 @@
       <c r="P17" s="3" t="n">
         <v>16.6456</v>
       </c>
+      <c r="Q17" s="3" t="n">
+        <v>16.7399</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2488,16 +2587,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>45.6</v>
+        <v>45.56</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>86021.4816</v>
+        <v>85946.02416</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>6021.481599999999</v>
+        <v>5946.024160000001</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.07526851999999999</v>
+        <v>0.07432530200000001</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -2520,6 +2619,9 @@
       <c r="P18" s="3" t="n">
         <v>45.6</v>
       </c>
+      <c r="Q18" s="3" t="n">
+        <v>45.56</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2544,16 +2646,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>14.1914</v>
+        <v>14.1822</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>205303.6630124</v>
+        <v>205170.5687652</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>55303.66301239998</v>
+        <v>55170.56876520001</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.3686910867493332</v>
+        <v>0.367803791768</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -2576,6 +2678,9 @@
       <c r="P19" s="3" t="n">
         <v>14.1914</v>
       </c>
+      <c r="Q19" s="3" t="n">
+        <v>14.1822</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2600,16 +2705,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.4</v>
+        <v>9.42</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>246804.5482</v>
+        <v>247329.66426</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-3195.451799999981</v>
+        <v>-2670.33574000001</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.01278180719999992</v>
+        <v>-0.01068134296000004</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -2632,6 +2737,9 @@
       <c r="P20" s="3" t="n">
         <v>9.4</v>
       </c>
+      <c r="Q20" s="3" t="n">
+        <v>9.42</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2656,16 +2764,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>107.4649</v>
+        <v>107.6398</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>163267.0165091</v>
+        <v>163532.7349082</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-6732.983490899991</v>
+        <v>-6467.265091800014</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.03960578524058819</v>
+        <v>-0.03804273583411773</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -2688,6 +2796,9 @@
       <c r="P21" s="3" t="n">
         <v>107.4649</v>
       </c>
+      <c r="Q21" s="3" t="n">
+        <v>107.6398</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2712,16 +2823,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>42.192</v>
+        <v>42.493</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>64741.93632</v>
+        <v>65203.80878000001</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>4741.936320000001</v>
+        <v>5203.808780000007</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.07903227200000001</v>
+        <v>0.08673014633333344</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -2744,6 +2855,9 @@
       <c r="P22" s="3" t="n">
         <v>42.192</v>
       </c>
+      <c r="Q22" s="3" t="n">
+        <v>42.493</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2768,16 +2882,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>59.7524</v>
+        <v>60.2688</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>162315.4227708</v>
+        <v>163718.2063296</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>12315.42277080001</v>
+        <v>13718.20632960001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.08210281847200007</v>
+        <v>0.09145470886400009</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -2800,6 +2914,9 @@
       <c r="P23" s="3" t="n">
         <v>59.7524</v>
       </c>
+      <c r="Q23" s="3" t="n">
+        <v>60.2688</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2824,16 +2941,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>27.747</v>
+        <v>27.9943</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>100815.561342</v>
+        <v>101714.0976998</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>815.5613420000009</v>
+        <v>1714.097699799997</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.00815561342000001</v>
+        <v>0.01714097699799997</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -2856,6 +2973,9 @@
       <c r="P24" s="3" t="n">
         <v>27.747</v>
       </c>
+      <c r="Q24" s="3" t="n">
+        <v>27.9943</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2880,16 +3000,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.2647</v>
+        <v>11.279</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>184985.2311078</v>
+        <v>185220.061046</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-15014.76889220002</v>
+        <v>-14779.93895400001</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.07507384446100011</v>
+        <v>-0.07389969477000007</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -2912,6 +3032,9 @@
       <c r="P25" s="3" t="n">
         <v>11.2647</v>
       </c>
+      <c r="Q25" s="3" t="n">
+        <v>11.279</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2936,16 +3059,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>8.805400000000001</v>
+        <v>8.816000000000001</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>105151.577261</v>
+        <v>105278.15944</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>-4848.422738999987</v>
+        <v>-4721.840559999997</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>-0.04407657035454533</v>
+        <v>-0.04292582327272725</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -2968,6 +3091,9 @@
       <c r="P26" s="3" t="n">
         <v>8.805400000000001</v>
       </c>
+      <c r="Q26" s="3" t="n">
+        <v>8.816000000000001</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2992,16 +3118,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>61.8656</v>
+        <v>62.0396</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>99656.82041599999</v>
+        <v>99937.11005599999</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-10343.17958400001</v>
+        <v>-10062.88994400001</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.09402890530909103</v>
+        <v>-0.09148081767272737</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -3024,6 +3150,9 @@
       <c r="P27" s="3" t="n">
         <v>61.8656</v>
       </c>
+      <c r="Q27" s="3" t="n">
+        <v>62.0396</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3048,16 +3177,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>105.9515</v>
+        <v>106.352</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>350345.2691355</v>
+        <v>351669.5852640001</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-29654.73086449999</v>
+        <v>-28330.41473599995</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.0780387654328947</v>
+        <v>-0.07455372298947355</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -3080,6 +3209,9 @@
       <c r="P28" s="3" t="n">
         <v>105.9515</v>
       </c>
+      <c r="Q28" s="3" t="n">
+        <v>106.352</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3104,16 +3236,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.6947</v>
+        <v>11.7867</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>112312.4254741</v>
+        <v>113195.9661501</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>12312.42547409999</v>
+        <v>13195.96615009999</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.1231242547409999</v>
+        <v>0.1319596615009999</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -3136,6 +3268,9 @@
       <c r="P29" s="3" t="n">
         <v>11.6947</v>
       </c>
+      <c r="Q29" s="3" t="n">
+        <v>11.7867</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3160,16 +3295,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>14.8786</v>
+        <v>14.928</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>110040.0574746</v>
+        <v>110405.413008</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>10040.05747460001</v>
+        <v>10405.413008</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.1004005747460001</v>
+        <v>0.10405413008</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -3192,6 +3327,9 @@
       <c r="P30" s="3" t="n">
         <v>14.8786</v>
       </c>
+      <c r="Q30" s="3" t="n">
+        <v>14.928</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3216,16 +3354,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>407.1528</v>
+        <v>410.0316</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>108335.217024</v>
+        <v>109101.208128</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>8335.217023999998</v>
+        <v>9101.208127999998</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.08335217023999998</v>
+        <v>0.09101208127999999</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -3248,6 +3386,9 @@
       <c r="P31" s="3" t="n">
         <v>407.1528</v>
       </c>
+      <c r="Q31" s="3" t="n">
+        <v>410.0316</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3272,16 +3413,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.05</v>
+        <v>10.1</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>212456.598</v>
+        <v>213513.596</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>12456.598</v>
+        <v>13513.59599999999</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.06228298999999999</v>
+        <v>0.06756797999999996</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -3304,6 +3445,9 @@
       <c r="P32" s="3" t="n">
         <v>10.05</v>
       </c>
+      <c r="Q32" s="3" t="n">
+        <v>10.1</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3328,16 +3472,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>17.69</v>
+        <v>17.77</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>63394.5916</v>
+        <v>63681.28279999999</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>3394.5916</v>
+        <v>3681.282799999994</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.05657652666666666</v>
+        <v>0.06135471333333323</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -3360,6 +3504,9 @@
       <c r="P33" s="3" t="n">
         <v>17.69</v>
       </c>
+      <c r="Q33" s="3" t="n">
+        <v>17.77</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3384,16 +3531,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>215.9582</v>
+        <v>215.7276</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>75916.0020042</v>
+        <v>75834.9389556</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-4083.997995800004</v>
+        <v>-4165.061044400005</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.05104997494750005</v>
+        <v>-0.05206326305500006</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -3416,6 +3563,9 @@
       <c r="P34" s="3" t="n">
         <v>215.9582</v>
       </c>
+      <c r="Q34" s="3" t="n">
+        <v>215.7276</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3440,16 +3590,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>13.67</v>
+        <v>13.9</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>97541.23241</v>
+        <v>99182.3797</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>-2458.767590000003</v>
+        <v>-817.620299999995</v>
       </c>
       <c r="I35" s="13" t="n">
-        <v>-0.02458767590000003</v>
+        <v>-0.00817620299999995</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -3472,6 +3622,9 @@
       <c r="P35" s="3" t="n">
         <v>13.67</v>
       </c>
+      <c r="Q35" s="3" t="n">
+        <v>13.9</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3496,16 +3649,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>352.2352</v>
+        <v>352.6471</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>164038.0460512</v>
+        <v>164229.8703526</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>14038.04605120001</v>
+        <v>14229.8703526</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.09358697367466676</v>
+        <v>0.09486580235066669</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -3528,6 +3681,9 @@
       <c r="P36" s="3" t="n">
         <v>352.2352</v>
       </c>
+      <c r="Q36" s="3" t="n">
+        <v>352.6471</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3552,16 +3708,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>15.742</v>
+        <v>15.758</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>59235.39863800001</v>
+        <v>59295.604862</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>9235.398638000006</v>
+        <v>9295.604862</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.1847079727600001</v>
+        <v>0.18591209724</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -3584,6 +3740,9 @@
       <c r="P37" s="3" t="n">
         <v>15.742</v>
       </c>
+      <c r="Q37" s="3" t="n">
+        <v>15.758</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3608,16 +3767,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.9705</v>
+        <v>14.0135</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>83550.323781</v>
+        <v>83807.484507</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>3550.323780999999</v>
+        <v>3807.484507000001</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.04437904726249999</v>
+        <v>0.04759355633750002</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -3640,6 +3799,9 @@
       <c r="P38" s="3" t="n">
         <v>13.9705</v>
       </c>
+      <c r="Q38" s="3" t="n">
+        <v>14.0135</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3664,16 +3826,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1007.0063</v>
+        <v>1007.3754</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50230.4812503</v>
+        <v>50248.8923274</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>230.4812502999994</v>
+        <v>248.8923274000044</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.004609625005999988</v>
+        <v>0.004977846548000089</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -3696,6 +3858,9 @@
       <c r="P39" s="3" t="n">
         <v>1007.0063</v>
       </c>
+      <c r="Q39" s="3" t="n">
+        <v>1007.3754</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3720,16 +3885,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>19.734</v>
+        <v>19.93</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>99479.626818</v>
-      </c>
-      <c r="H40" s="6" t="n">
-        <v>-520.3731819999957</v>
-      </c>
-      <c r="I40" s="13" t="n">
-        <v>-0.005203731819999957</v>
+        <v>100467.66811</v>
+      </c>
+      <c r="H40" s="4" t="n">
+        <v>467.6681099999987</v>
+      </c>
+      <c r="I40" s="12" t="n">
+        <v>0.004676681099999987</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -3752,6 +3917,9 @@
       <c r="P40" s="3" t="n">
         <v>19.734</v>
       </c>
+      <c r="Q40" s="3" t="n">
+        <v>19.93</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
@@ -3763,13 +3931,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4788622.6908943</v>
+        <v>4815373.626656</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>318622.6908943</v>
+        <v>345373.626656</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.07128024404794184</v>
+        <v>0.07726479343534676</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-05-22
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -485,7 +485,7 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-05-21 06:09 IST</t>
+          <t>Generated: 2026-05-22 06:04 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4815373.626656</v>
+        <v>4827372.0145348</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>345373.6266559996</v>
+        <v>357372.0145348003</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.07726479343534666</v>
+        <v>0.07994899654022379</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>555583.4997634888</v>
+        <v>554357.9995422363</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-35198.52023651125</v>
+        <v>-36424.02045776369</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.05957953872142427</v>
+        <v>-0.061653908251581</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5370957.126419488</v>
+        <v>5381730.014077037</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>310175.1064194888</v>
+        <v>320947.9940770371</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.06128995581981</v>
+        <v>0.06341865601179106</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-05-21</t>
+          <t>Last snapshot: 2026-05-22</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O19"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -634,6 +634,7 @@
     <col width="21" customWidth="1" min="13" max="13"/>
     <col width="21" customWidth="1" min="14" max="14"/>
     <col width="21" customWidth="1" min="15" max="15"/>
+    <col width="21" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -712,6 +713,11 @@
           <t>2026-05-21</t>
         </is>
       </c>
+      <c r="P1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -731,13 +737,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>572</v>
+        <v>564.7000122070312</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>45760</v>
+        <v>45176.0009765625</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1942.489999999998</v>
+        <v>1358.490976562498</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -763,6 +769,9 @@
       <c r="O2" s="3" t="n">
         <v>572</v>
       </c>
+      <c r="P2" s="3" t="n">
+        <v>564.7000122070312</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -809,13 +818,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1475.5</v>
+        <v>1541.699951171875</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>29510</v>
+        <v>30833.9990234375</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-2594.580000000002</v>
+        <v>-1270.580976562502</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -841,6 +850,9 @@
       <c r="O4" s="3" t="n">
         <v>1475.5</v>
       </c>
+      <c r="P4" s="3" t="n">
+        <v>1541.699951171875</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -860,13 +872,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>658.6500244140625</v>
+        <v>654</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13173.00048828125</v>
+        <v>13080</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1040.09951171875</v>
+        <v>-1133.1</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -892,6 +904,9 @@
       <c r="O5" s="3" t="n">
         <v>658.6500244140625</v>
       </c>
+      <c r="P5" s="3" t="n">
+        <v>654</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -911,13 +926,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>386.5</v>
+        <v>383.6499938964844</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15460</v>
+        <v>15345.99975585938</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2042.240000000002</v>
+        <v>-2156.240244140627</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -943,6 +958,9 @@
       <c r="O6" s="3" t="n">
         <v>386.5</v>
       </c>
+      <c r="P6" s="3" t="n">
+        <v>383.6499938964844</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -962,13 +980,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>240.1999969482422</v>
+        <v>222.1499938964844</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>24019.99969482422</v>
+        <v>22214.99938964844</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-2413.820305175781</v>
+        <v>-4218.820610351562</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -994,6 +1012,9 @@
       <c r="O7" s="3" t="n">
         <v>240.1999969482422</v>
       </c>
+      <c r="P7" s="3" t="n">
+        <v>222.1499938964844</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1040,13 +1061,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>19.01000022888184</v>
+        <v>18.86000061035156</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>28515.00034332275</v>
+        <v>28290.00091552734</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-2535.169656677244</v>
+        <v>-2760.169084472655</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1072,6 +1093,9 @@
       <c r="O9" s="3" t="n">
         <v>19.01000022888184</v>
       </c>
+      <c r="P9" s="3" t="n">
+        <v>18.86000061035156</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1091,13 +1115,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>502.5</v>
+        <v>501.7999877929688</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>50250</v>
+        <v>50179.99877929688</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-1248.480000000003</v>
+        <v>-1318.481220703128</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1123,6 +1147,9 @@
       <c r="O10" s="3" t="n">
         <v>502.5</v>
       </c>
+      <c r="P10" s="3" t="n">
+        <v>501.7999877929688</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1142,13 +1169,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>8.319999694824219</v>
+        <v>8.340000152587891</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>8319.999694824219</v>
+        <v>8340.000152587891</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-1521.21030517578</v>
+        <v>-1501.209847412109</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -1174,6 +1201,9 @@
       <c r="O11" s="3" t="n">
         <v>8.319999694824219</v>
       </c>
+      <c r="P11" s="3" t="n">
+        <v>8.340000152587891</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1193,13 +1223,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2525</v>
+        <v>2524.10009765625</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25250</v>
+        <v>25241.0009765625</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2473.25</v>
+        <v>-2482.2490234375</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -1225,6 +1255,9 @@
       <c r="O12" s="3" t="n">
         <v>2525</v>
       </c>
+      <c r="P12" s="3" t="n">
+        <v>2524.10009765625</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1244,13 +1277,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>53.45000076293945</v>
+        <v>53.27999877929688</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>32070.00045776367</v>
+        <v>31967.99926757812</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-2961.75954223633</v>
+        <v>-3063.760732421877</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -1276,6 +1309,9 @@
       <c r="O13" s="3" t="n">
         <v>53.45000076293945</v>
       </c>
+      <c r="P13" s="3" t="n">
+        <v>53.27999877929688</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1295,13 +1331,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>735</v>
+        <v>749.7999877929688</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>36750</v>
+        <v>37489.99938964844</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-5712.510000000002</v>
+        <v>-4972.510610351565</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -1327,6 +1363,9 @@
       <c r="O14" s="3" t="n">
         <v>735</v>
       </c>
+      <c r="P14" s="3" t="n">
+        <v>749.7999877929688</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1400,13 +1439,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>472.6000061035156</v>
+        <v>472.1499938964844</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>23630.00030517578</v>
+        <v>23607.49969482422</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>1875.470305175782</v>
+        <v>1852.96969482422</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -1432,6 +1471,9 @@
       <c r="O17" s="3" t="n">
         <v>472.6000061035156</v>
       </c>
+      <c r="P17" s="3" t="n">
+        <v>472.1499938964844</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1451,13 +1493,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>411.0499877929688</v>
+        <v>408.2000122070312</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>41104.99877929688</v>
+        <v>40820.00122070312</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-5535.821220703125</v>
+        <v>-5820.818779296875</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -1483,6 +1525,9 @@
       <c r="O18" s="3" t="n">
         <v>411.0499877929688</v>
       </c>
+      <c r="P18" s="3" t="n">
+        <v>408.2000122070312</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -1494,10 +1539,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>555583.4997634888</v>
+        <v>554357.9995422363</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-35198.52023651124</v>
+        <v>-36424.02045776368</v>
       </c>
     </row>
   </sheetData>
@@ -1511,7 +1556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q41"/>
+  <dimension ref="A1:R41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1531,6 +1576,7 @@
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="16" max="16"/>
     <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1619,6 +1665,11 @@
           <t>2026-05-21</t>
         </is>
       </c>
+      <c r="R1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1643,16 +1694,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.9033</v>
+        <v>57.0304</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>63872.9299906</v>
+        <v>64015.5974528</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>13872.9299906</v>
+        <v>14015.5974528</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.2774585998120001</v>
+        <v>0.280311949056</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -1678,6 +1729,9 @@
       <c r="Q2" s="3" t="n">
         <v>56.9033</v>
       </c>
+      <c r="R2" s="3" t="n">
+        <v>57.0304</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1702,16 +1756,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.5927</v>
+        <v>25.5036</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>62835.52974510001</v>
+        <v>62616.7702668</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>2835.529745100008</v>
+        <v>2616.770266799998</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.04725882908500013</v>
+        <v>0.04361283777999998</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -1737,6 +1791,9 @@
       <c r="Q3" s="3" t="n">
         <v>25.5927</v>
       </c>
+      <c r="R3" s="3" t="n">
+        <v>25.5036</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1761,16 +1818,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.64</v>
+        <v>12.53</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>242765.01552</v>
+        <v>240652.34529</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>62765.01552000002</v>
+        <v>60652.34529</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3486945306666668</v>
+        <v>0.3369574738333333</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -1796,6 +1853,9 @@
       <c r="Q4" s="3" t="n">
         <v>12.64</v>
       </c>
+      <c r="R4" s="3" t="n">
+        <v>12.53</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1820,16 +1880,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.527799999999999</v>
+        <v>9.5405</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>174874.0796464</v>
+        <v>175107.176564</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-35125.92035360003</v>
+        <v>-34892.82343600001</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1672662873980954</v>
+        <v>-0.1661563020761905</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -1855,6 +1915,9 @@
       <c r="Q5" s="3" t="n">
         <v>9.527799999999999</v>
       </c>
+      <c r="R5" s="3" t="n">
+        <v>9.5405</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1879,16 +1942,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.5431</v>
+        <v>12.5454</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>53044.4814087</v>
+        <v>53054.2080558</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>3044.481408700005</v>
+        <v>3054.208055800002</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.0608896281740001</v>
+        <v>0.06108416111600003</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -1914,6 +1977,9 @@
       <c r="Q6" s="3" t="n">
         <v>12.5431</v>
       </c>
+      <c r="R6" s="3" t="n">
+        <v>12.5454</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1938,16 +2004,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.5886</v>
+        <v>33.8152</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>74097.795144</v>
+        <v>74597.68380799999</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>14097.795144</v>
+        <v>14597.68380799999</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2349632524</v>
+        <v>0.2432947301333331</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -1973,6 +2039,9 @@
       <c r="Q7" s="3" t="n">
         <v>33.5886</v>
       </c>
+      <c r="R7" s="3" t="n">
+        <v>33.8152</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1997,16 +2066,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>30.2942</v>
+        <v>30.4158</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>48609.8612606</v>
+        <v>48804.9797694</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>-1390.138739399998</v>
+        <v>-1195.020230599999</v>
       </c>
       <c r="I8" s="13" t="n">
-        <v>-0.02780277478799995</v>
+        <v>-0.02390040461199999</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -2032,6 +2101,9 @@
       <c r="Q8" s="3" t="n">
         <v>30.2942</v>
       </c>
+      <c r="R8" s="3" t="n">
+        <v>30.4158</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2056,16 +2128,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>40.8338</v>
+        <v>41.4501</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>131460.0498834</v>
+        <v>133444.1617893</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>31460.0498834</v>
+        <v>33444.16178930001</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.314600498834</v>
+        <v>0.3344416178930001</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -2091,6 +2163,9 @@
       <c r="Q9" s="3" t="n">
         <v>40.8338</v>
       </c>
+      <c r="R9" s="3" t="n">
+        <v>41.4501</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2115,16 +2190,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>46.3181</v>
+        <v>46.115</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>131851.8362279</v>
+        <v>131273.679785</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>31851.8362279</v>
+        <v>31273.67978500001</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.318518362279</v>
+        <v>0.3127367978500001</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -2150,6 +2225,9 @@
       <c r="Q10" s="3" t="n">
         <v>46.3181</v>
       </c>
+      <c r="R10" s="3" t="n">
+        <v>46.115</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2174,16 +2252,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>104.5549</v>
+        <v>104.1779</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31462.5559531</v>
+        <v>31349.1094901</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1462.5559531</v>
+        <v>1349.109490099996</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.04875186510333333</v>
+        <v>0.04497031633666653</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -2209,6 +2287,9 @@
       <c r="Q11" s="3" t="n">
         <v>104.5549</v>
       </c>
+      <c r="R11" s="3" t="n">
+        <v>104.1779</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2233,16 +2314,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>220.391</v>
+        <v>220.534</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>102596.859102</v>
+        <v>102663.428748</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>2596.859101999988</v>
+        <v>2663.428747999991</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.02596859101999988</v>
+        <v>0.02663428747999991</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -2268,6 +2349,9 @@
       <c r="Q12" s="3" t="n">
         <v>220.391</v>
       </c>
+      <c r="R12" s="3" t="n">
+        <v>220.534</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2292,16 +2376,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>20.091</v>
+        <v>20.134</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>232806.572055</v>
+        <v>233304.83907</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>32806.572055</v>
+        <v>33304.83906999999</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.164032860275</v>
+        <v>0.1665241953499999</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -2327,6 +2411,9 @@
       <c r="Q13" s="3" t="n">
         <v>20.091</v>
       </c>
+      <c r="R13" s="3" t="n">
+        <v>20.134</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2351,16 +2438,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>37.7689</v>
+        <v>38.3982</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>136255.3102534</v>
+        <v>138525.5767092</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>36255.31025340001</v>
+        <v>38525.57670920002</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.3625531025340001</v>
+        <v>0.3852557670920002</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -2386,6 +2473,9 @@
       <c r="Q14" s="3" t="n">
         <v>37.7689</v>
       </c>
+      <c r="R14" s="3" t="n">
+        <v>38.3982</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2410,16 +2500,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.75</v>
+        <v>11.82</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>114491.37725</v>
+        <v>115173.45354</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>14491.37725000001</v>
+        <v>15173.45354</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1449137725</v>
+        <v>0.1517345354</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -2445,6 +2535,9 @@
       <c r="Q15" s="3" t="n">
         <v>11.75</v>
       </c>
+      <c r="R15" s="3" t="n">
+        <v>11.82</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2469,16 +2562,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.694</v>
+        <v>24.6116</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>141321.984032</v>
+        <v>140850.4147648</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>41321.98403199998</v>
+        <v>40850.41476479999</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4132198403199998</v>
+        <v>0.4085041476479999</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -2504,6 +2597,9 @@
       <c r="Q16" s="3" t="n">
         <v>24.694</v>
       </c>
+      <c r="R16" s="3" t="n">
+        <v>24.6116</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2528,16 +2624,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.7399</v>
+        <v>16.6948</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55343.06357429999</v>
+        <v>55193.9604036</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5343.063574299995</v>
+        <v>5193.960403600002</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1068612714859999</v>
+        <v>0.103879208072</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -2563,6 +2659,9 @@
       <c r="Q17" s="3" t="n">
         <v>16.7399</v>
       </c>
+      <c r="R17" s="3" t="n">
+        <v>16.6948</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2587,16 +2686,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>45.56</v>
+        <v>45.63</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>85946.02416</v>
+        <v>86078.07468000001</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>5946.024160000001</v>
+        <v>6078.074680000005</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.07432530200000001</v>
+        <v>0.07597593350000006</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -2622,6 +2721,9 @@
       <c r="Q18" s="3" t="n">
         <v>45.56</v>
       </c>
+      <c r="R18" s="3" t="n">
+        <v>45.63</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2646,16 +2748,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>14.1822</v>
+        <v>14.3065</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>205170.5687652</v>
+        <v>206968.787779</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>55170.56876520001</v>
+        <v>56968.78777900001</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.367803791768</v>
+        <v>0.3797919185266667</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -2681,6 +2783,9 @@
       <c r="Q19" s="3" t="n">
         <v>14.1822</v>
       </c>
+      <c r="R19" s="3" t="n">
+        <v>14.3065</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2705,16 +2810,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.42</v>
+        <v>9.35</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>247329.66426</v>
+        <v>245491.75805</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-2670.33574000001</v>
+        <v>-4508.241949999996</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.01068134296000004</v>
+        <v>-0.01803296779999998</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -2740,6 +2845,9 @@
       <c r="Q20" s="3" t="n">
         <v>9.42</v>
       </c>
+      <c r="R20" s="3" t="n">
+        <v>9.35</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2764,16 +2872,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>107.6398</v>
+        <v>107.8068</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>163532.7349082</v>
+        <v>163786.4511612</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-6467.265091800014</v>
+        <v>-6213.548838799994</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.03804273583411773</v>
+        <v>-0.03655028728705879</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -2799,6 +2907,9 @@
       <c r="Q21" s="3" t="n">
         <v>107.6398</v>
       </c>
+      <c r="R21" s="3" t="n">
+        <v>107.8068</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2823,16 +2934,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>42.493</v>
+        <v>43.324</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>65203.80878000001</v>
+        <v>66478.94503999999</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>5203.808780000007</v>
+        <v>6478.945039999991</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.08673014633333344</v>
+        <v>0.1079824173333332</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -2858,6 +2969,9 @@
       <c r="Q22" s="3" t="n">
         <v>42.493</v>
       </c>
+      <c r="R22" s="3" t="n">
+        <v>43.324</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2882,16 +2996,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>60.2688</v>
+        <v>60.7104</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>163718.2063296</v>
+        <v>164917.7981568</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>13718.20632960001</v>
+        <v>14917.79815680001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.09145470886400009</v>
+        <v>0.09945198771200008</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -2917,6 +3031,9 @@
       <c r="Q23" s="3" t="n">
         <v>60.2688</v>
       </c>
+      <c r="R23" s="3" t="n">
+        <v>60.7104</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2941,16 +3058,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>27.9943</v>
+        <v>28.0977</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>101714.0976998</v>
+        <v>102089.7898122</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>1714.097699799997</v>
+        <v>2089.789812200004</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.01714097699799997</v>
+        <v>0.02089789812200004</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -2976,6 +3093,9 @@
       <c r="Q24" s="3" t="n">
         <v>27.9943</v>
       </c>
+      <c r="R24" s="3" t="n">
+        <v>28.0977</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3000,16 +3120,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.279</v>
+        <v>11.2689</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>185220.061046</v>
+        <v>185054.2021386</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-14779.93895400001</v>
+        <v>-14945.7978614</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.07389969477000007</v>
+        <v>-0.074728989307</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -3035,6 +3155,9 @@
       <c r="Q25" s="3" t="n">
         <v>11.279</v>
       </c>
+      <c r="R25" s="3" t="n">
+        <v>11.2689</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3059,16 +3182,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>8.816000000000001</v>
+        <v>8.798500000000001</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>105278.15944</v>
+        <v>105069.1794275</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>-4721.840559999997</v>
+        <v>-4930.820572499986</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>-0.04292582327272725</v>
+        <v>-0.0448256415681817</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -3094,6 +3217,9 @@
       <c r="Q26" s="3" t="n">
         <v>8.816000000000001</v>
       </c>
+      <c r="R26" s="3" t="n">
+        <v>8.798500000000001</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3118,16 +3244,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>62.0396</v>
+        <v>62.2395</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>99937.11005599999</v>
+        <v>100259.12097</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-10062.88994400001</v>
+        <v>-9740.879030000011</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.09148081767272737</v>
+        <v>-0.08855344572727283</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -3153,6 +3279,9 @@
       <c r="Q27" s="3" t="n">
         <v>62.0396</v>
       </c>
+      <c r="R27" s="3" t="n">
+        <v>62.2395</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3177,16 +3306,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>106.352</v>
+        <v>106.249</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>351669.5852640001</v>
+        <v>351328.999593</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-28330.41473599995</v>
+        <v>-28671.00040700001</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.07455372298947355</v>
+        <v>-0.07545000107105267</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -3212,6 +3341,9 @@
       <c r="Q28" s="3" t="n">
         <v>106.352</v>
       </c>
+      <c r="R28" s="3" t="n">
+        <v>106.249</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3236,16 +3368,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.7867</v>
+        <v>11.955</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>113195.9661501</v>
+        <v>114812.269365</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>13195.96615009999</v>
+        <v>14812.269365</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.1319596615009999</v>
+        <v>0.14812269365</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -3271,6 +3403,9 @@
       <c r="Q29" s="3" t="n">
         <v>11.7867</v>
       </c>
+      <c r="R29" s="3" t="n">
+        <v>11.955</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3295,16 +3430,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>14.928</v>
+        <v>15.0861</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>110405.413008</v>
+        <v>111574.6986321</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>10405.413008</v>
+        <v>11574.6986321</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.10405413008</v>
+        <v>0.115746986321</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -3330,6 +3465,9 @@
       <c r="Q30" s="3" t="n">
         <v>14.928</v>
       </c>
+      <c r="R30" s="3" t="n">
+        <v>15.0861</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3354,16 +3492,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>410.0316</v>
+        <v>413.0441</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>109101.208128</v>
+        <v>109902.774128</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>9101.208127999998</v>
+        <v>9902.77412799999</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.09101208127999999</v>
+        <v>0.0990277412799999</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -3389,6 +3527,9 @@
       <c r="Q31" s="3" t="n">
         <v>410.0316</v>
       </c>
+      <c r="R31" s="3" t="n">
+        <v>413.0441</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3413,16 +3554,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.1</v>
+        <v>10.14</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>213513.596</v>
+        <v>214359.1944</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>13513.59599999999</v>
+        <v>14359.19440000001</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.06756797999999996</v>
+        <v>0.07179597200000004</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -3448,6 +3589,9 @@
       <c r="Q32" s="3" t="n">
         <v>10.1</v>
       </c>
+      <c r="R32" s="3" t="n">
+        <v>10.14</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3472,16 +3616,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>17.77</v>
+        <v>17.92</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>63681.28279999999</v>
+        <v>64218.8288</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>3681.282799999994</v>
+        <v>4218.828800000003</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.06135471333333323</v>
+        <v>0.07031381333333338</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -3507,6 +3651,9 @@
       <c r="Q33" s="3" t="n">
         <v>17.77</v>
       </c>
+      <c r="R33" s="3" t="n">
+        <v>17.92</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3531,16 +3678,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>215.7276</v>
+        <v>214.1576</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>75834.9389556</v>
+        <v>75283.0352856</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-4165.061044400005</v>
+        <v>-4716.964714400005</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.05206326305500006</v>
+        <v>-0.05896205893000006</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -3566,6 +3713,9 @@
       <c r="Q34" s="3" t="n">
         <v>215.7276</v>
       </c>
+      <c r="R34" s="3" t="n">
+        <v>214.1576</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3590,16 +3740,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>13.9</v>
+        <v>14.11</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>99182.3797</v>
-      </c>
-      <c r="H35" s="6" t="n">
-        <v>-817.620299999995</v>
-      </c>
-      <c r="I35" s="13" t="n">
-        <v>-0.00817620299999995</v>
+        <v>100680.81853</v>
+      </c>
+      <c r="H35" s="4" t="n">
+        <v>680.8185299999896</v>
+      </c>
+      <c r="I35" s="12" t="n">
+        <v>0.006808185299999895</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -3625,6 +3775,9 @@
       <c r="Q35" s="3" t="n">
         <v>13.9</v>
       </c>
+      <c r="R35" s="3" t="n">
+        <v>14.11</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3649,16 +3802,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>352.6471</v>
+        <v>353.6924</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>164229.8703526</v>
+        <v>164716.6728344</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>14229.8703526</v>
+        <v>14716.67283440003</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.09486580235066669</v>
+        <v>0.09811115222933353</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -3684,6 +3837,9 @@
       <c r="Q36" s="3" t="n">
         <v>352.6471</v>
       </c>
+      <c r="R36" s="3" t="n">
+        <v>353.6924</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3708,16 +3864,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>15.758</v>
+        <v>15.842</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>59295.604862</v>
+        <v>59611.68753800001</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>9295.604862</v>
+        <v>9611.687538000006</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.18591209724</v>
+        <v>0.1922337507600001</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -3743,6 +3899,9 @@
       <c r="Q37" s="3" t="n">
         <v>15.758</v>
       </c>
+      <c r="R37" s="3" t="n">
+        <v>15.842</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3767,16 +3926,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>14.0135</v>
+        <v>14.0227</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>83807.484507</v>
+        <v>83862.5049414</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>3807.484507000001</v>
+        <v>3862.504941399995</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.04759355633750002</v>
+        <v>0.04828131176749994</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -3802,6 +3961,9 @@
       <c r="Q38" s="3" t="n">
         <v>14.0135</v>
       </c>
+      <c r="R38" s="3" t="n">
+        <v>14.0227</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3826,16 +3988,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1007.3754</v>
+        <v>1005.1862</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50248.8923274</v>
+        <v>50139.6928422</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>248.8923274000044</v>
+        <v>139.6928421999983</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.004977846548000089</v>
+        <v>0.002793856843999965</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -3861,6 +4023,9 @@
       <c r="Q39" s="3" t="n">
         <v>1007.3754</v>
       </c>
+      <c r="R39" s="3" t="n">
+        <v>1005.1862</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3885,16 +4050,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>19.93</v>
+        <v>19.849</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>100467.66811</v>
+        <v>100059.344923</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>467.6681099999987</v>
+        <v>59.34492299999692</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.004676681099999987</v>
+        <v>0.0005934492299999693</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -3920,6 +4085,9 @@
       <c r="Q40" s="3" t="n">
         <v>19.93</v>
       </c>
+      <c r="R40" s="3" t="n">
+        <v>19.849</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
@@ -3931,13 +4099,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4815373.626656</v>
+        <v>4827372.0145348</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>345373.626656</v>
+        <v>357372.0145348</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.07726479343534676</v>
+        <v>0.07994899654022372</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-05-23
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -485,7 +485,7 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-05-22 06:04 IST</t>
+          <t>Generated: 2026-05-23 05:38 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4827372.0145348</v>
+        <v>4834300.7735287</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>357372.0145348003</v>
+        <v>364300.7735286998</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.07994899654022379</v>
+        <v>0.08149905448069346</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>554357.9995422363</v>
+        <v>554338.0011444092</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-36424.02045776369</v>
+        <v>-36444.01885559084</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.061653908251581</v>
+        <v>-0.06168775897342109</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5381730.014077037</v>
+        <v>5388638.774673109</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>320947.9940770371</v>
+        <v>327856.7546731094</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.06341865601179106</v>
+        <v>0.06478381273436262</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-05-22</t>
+          <t>Last snapshot: 2026-05-23</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P19"/>
+  <dimension ref="A1:Q19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -635,6 +635,7 @@
     <col width="21" customWidth="1" min="14" max="14"/>
     <col width="21" customWidth="1" min="15" max="15"/>
     <col width="21" customWidth="1" min="16" max="16"/>
+    <col width="21" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -718,6 +719,11 @@
           <t>2026-05-22</t>
         </is>
       </c>
+      <c r="Q1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -737,13 +743,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>564.7000122070312</v>
+        <v>569.9500122070312</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>45176.0009765625</v>
+        <v>45596.0009765625</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1358.490976562498</v>
+        <v>1778.490976562498</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -772,6 +778,9 @@
       <c r="P2" s="3" t="n">
         <v>564.7000122070312</v>
       </c>
+      <c r="Q2" s="3" t="n">
+        <v>569.9500122070312</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -853,6 +862,9 @@
       <c r="P4" s="3" t="n">
         <v>1541.699951171875</v>
       </c>
+      <c r="Q4" s="3" t="n">
+        <v>1541.699951171875</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -872,13 +884,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>654</v>
+        <v>653.2000122070312</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13080</v>
+        <v>13064.00024414062</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1133.1</v>
+        <v>-1149.099755859375</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -907,6 +919,9 @@
       <c r="P5" s="3" t="n">
         <v>654</v>
       </c>
+      <c r="Q5" s="3" t="n">
+        <v>653.2000122070312</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -926,13 +941,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>383.6499938964844</v>
+        <v>382.25</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15345.99975585938</v>
+        <v>15290</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2156.240244140627</v>
+        <v>-2212.240000000002</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -961,6 +976,9 @@
       <c r="P6" s="3" t="n">
         <v>383.6499938964844</v>
       </c>
+      <c r="Q6" s="3" t="n">
+        <v>382.25</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -980,13 +998,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>222.1499938964844</v>
+        <v>216</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>22214.99938964844</v>
+        <v>21600</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-4218.820610351562</v>
+        <v>-4833.82</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1015,6 +1033,9 @@
       <c r="P7" s="3" t="n">
         <v>222.1499938964844</v>
       </c>
+      <c r="Q7" s="3" t="n">
+        <v>216</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1061,13 +1082,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>18.86000061035156</v>
+        <v>18.76000022888184</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>28290.00091552734</v>
+        <v>28140.00034332275</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-2760.169084472655</v>
+        <v>-2910.169656677244</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1096,6 +1117,9 @@
       <c r="P9" s="3" t="n">
         <v>18.86000061035156</v>
       </c>
+      <c r="Q9" s="3" t="n">
+        <v>18.76000022888184</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1115,13 +1139,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>501.7999877929688</v>
+        <v>499.75</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>50179.99877929688</v>
+        <v>49975</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-1318.481220703128</v>
+        <v>-1523.480000000003</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1150,6 +1174,9 @@
       <c r="P10" s="3" t="n">
         <v>501.7999877929688</v>
       </c>
+      <c r="Q10" s="3" t="n">
+        <v>499.75</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1169,13 +1196,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>8.340000152587891</v>
+        <v>8.369999885559082</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>8340.000152587891</v>
+        <v>8369.999885559082</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-1501.209847412109</v>
+        <v>-1471.210114440917</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -1204,6 +1231,9 @@
       <c r="P11" s="3" t="n">
         <v>8.340000152587891</v>
       </c>
+      <c r="Q11" s="3" t="n">
+        <v>8.369999885559082</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1223,13 +1253,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2524.10009765625</v>
+        <v>2564.10009765625</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25241.0009765625</v>
+        <v>25641.0009765625</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2482.2490234375</v>
+        <v>-2082.2490234375</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -1258,6 +1288,9 @@
       <c r="P12" s="3" t="n">
         <v>2524.10009765625</v>
       </c>
+      <c r="Q12" s="3" t="n">
+        <v>2564.10009765625</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1277,13 +1310,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>53.27999877929688</v>
+        <v>53.75</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>31967.99926757812</v>
+        <v>32250</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-3063.760732421877</v>
+        <v>-2781.760000000002</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -1312,6 +1345,9 @@
       <c r="P13" s="3" t="n">
         <v>53.27999877929688</v>
       </c>
+      <c r="Q13" s="3" t="n">
+        <v>53.75</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1331,13 +1367,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>749.7999877929688</v>
+        <v>750.2000122070312</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>37489.99938964844</v>
+        <v>37510.00061035156</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-4972.510610351565</v>
+        <v>-4952.50938964844</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -1366,6 +1402,9 @@
       <c r="P14" s="3" t="n">
         <v>749.7999877929688</v>
       </c>
+      <c r="Q14" s="3" t="n">
+        <v>750.2000122070312</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1439,13 +1478,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>472.1499938964844</v>
+        <v>468.1499938964844</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>23607.49969482422</v>
+        <v>23407.49969482422</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>1852.96969482422</v>
+        <v>1652.96969482422</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -1474,6 +1513,9 @@
       <c r="P17" s="3" t="n">
         <v>472.1499938964844</v>
       </c>
+      <c r="Q17" s="3" t="n">
+        <v>468.1499938964844</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1493,13 +1535,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>408.2000122070312</v>
+        <v>408.8999938964844</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>40820.00122070312</v>
+        <v>40889.99938964844</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-5820.818779296875</v>
+        <v>-5750.820610351562</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -1528,6 +1570,9 @@
       <c r="P18" s="3" t="n">
         <v>408.2000122070312</v>
       </c>
+      <c r="Q18" s="3" t="n">
+        <v>408.8999938964844</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -1539,10 +1584,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>554357.9995422363</v>
+        <v>554338.0011444092</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-36424.02045776368</v>
+        <v>-36444.01885559083</v>
       </c>
     </row>
   </sheetData>
@@ -1556,7 +1601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R41"/>
+  <dimension ref="A1:S41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1577,6 +1622,7 @@
     <col width="13" customWidth="1" min="16" max="16"/>
     <col width="13" customWidth="1" min="17" max="17"/>
     <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1670,6 +1716,11 @@
           <t>2026-05-22</t>
         </is>
       </c>
+      <c r="S1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1694,16 +1745,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>57.0304</v>
+        <v>56.8797</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>64015.5974528</v>
+        <v>63846.4394154</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>14015.5974528</v>
+        <v>13846.4394154</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.280311949056</v>
+        <v>0.2769287883079999</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -1732,6 +1783,9 @@
       <c r="R2" s="3" t="n">
         <v>57.0304</v>
       </c>
+      <c r="S2" s="3" t="n">
+        <v>56.8797</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1756,16 +1810,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.5036</v>
+        <v>25.7058</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>62616.7702668</v>
+        <v>63113.21433540001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>2616.770266799998</v>
+        <v>3113.214335400007</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.04361283777999998</v>
+        <v>0.05188690559000012</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -1794,6 +1848,9 @@
       <c r="R3" s="3" t="n">
         <v>25.5036</v>
       </c>
+      <c r="S3" s="3" t="n">
+        <v>25.7058</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1818,16 +1875,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.53</v>
+        <v>12.63</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>240652.34529</v>
+        <v>242572.95459</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>60652.34529</v>
+        <v>62572.95459000004</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3369574738333333</v>
+        <v>0.3476275255000002</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -1856,6 +1913,9 @@
       <c r="R4" s="3" t="n">
         <v>12.53</v>
       </c>
+      <c r="S4" s="3" t="n">
+        <v>12.63</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1880,16 +1940,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.5405</v>
+        <v>9.544499999999999</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>175107.176564</v>
+        <v>175180.592916</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-34892.82343600001</v>
+        <v>-34819.40708400001</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1661563020761905</v>
+        <v>-0.1658067004</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -1918,6 +1978,9 @@
       <c r="R5" s="3" t="n">
         <v>9.5405</v>
       </c>
+      <c r="S5" s="3" t="n">
+        <v>9.544499999999999</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1942,16 +2005,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.5454</v>
+        <v>12.4901</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>53054.2080558</v>
+        <v>52820.3456277</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>3054.208055800002</v>
+        <v>2820.3456277</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.06108416111600003</v>
+        <v>0.05640691255400001</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -1980,6 +2043,9 @@
       <c r="R6" s="3" t="n">
         <v>12.5454</v>
       </c>
+      <c r="S6" s="3" t="n">
+        <v>12.4901</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2004,16 +2070,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.8152</v>
+        <v>33.9116</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>74597.68380799999</v>
+        <v>74810.346064</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>14597.68380799999</v>
+        <v>14810.346064</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2432947301333331</v>
+        <v>0.2468391010666666</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -2042,6 +2108,9 @@
       <c r="R7" s="3" t="n">
         <v>33.8152</v>
       </c>
+      <c r="S7" s="3" t="n">
+        <v>33.9116</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2066,16 +2135,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>30.4158</v>
+        <v>30.4549</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>48804.9797694</v>
+        <v>48867.7193557</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>-1195.020230599999</v>
+        <v>-1132.280644300001</v>
       </c>
       <c r="I8" s="13" t="n">
-        <v>-0.02390040461199999</v>
+        <v>-0.02264561288600002</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -2104,6 +2173,9 @@
       <c r="R8" s="3" t="n">
         <v>30.4158</v>
       </c>
+      <c r="S8" s="3" t="n">
+        <v>30.4549</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2128,16 +2200,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>41.4501</v>
+        <v>41.9916</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>133444.1617893</v>
+        <v>135187.4630988</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>33444.16178930001</v>
+        <v>35187.46309879998</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3344416178930001</v>
+        <v>0.3518746309879999</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -2166,6 +2238,9 @@
       <c r="R9" s="3" t="n">
         <v>41.4501</v>
       </c>
+      <c r="S9" s="3" t="n">
+        <v>41.9916</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2190,16 +2265,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>46.115</v>
+        <v>46.457</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>131273.679785</v>
+        <v>132247.237163</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>31273.67978500001</v>
+        <v>32247.23716300001</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3127367978500001</v>
+        <v>0.3224723716300001</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -2228,6 +2303,9 @@
       <c r="R10" s="3" t="n">
         <v>46.115</v>
       </c>
+      <c r="S10" s="3" t="n">
+        <v>46.457</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2290,6 +2368,9 @@
       <c r="R11" s="3" t="n">
         <v>104.1779</v>
       </c>
+      <c r="S11" s="3" t="n">
+        <v>104.1779</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2314,16 +2395,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>220.534</v>
+        <v>220.359</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>102663.428748</v>
+        <v>102581.962398</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>2663.428747999991</v>
+        <v>2581.962398000003</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.02663428747999991</v>
+        <v>0.02581962398000003</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -2352,6 +2433,9 @@
       <c r="R12" s="3" t="n">
         <v>220.534</v>
       </c>
+      <c r="S12" s="3" t="n">
+        <v>220.359</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2376,16 +2460,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>20.134</v>
+        <v>19.908</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>233304.83907</v>
+        <v>230686.04034</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>33304.83906999999</v>
+        <v>30686.04034000001</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.1665241953499999</v>
+        <v>0.1534302017</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -2414,6 +2498,9 @@
       <c r="R13" s="3" t="n">
         <v>20.134</v>
       </c>
+      <c r="S13" s="3" t="n">
+        <v>19.908</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2438,16 +2525,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>38.3982</v>
+        <v>38.499</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>138525.5767092</v>
+        <v>138889.223394</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>38525.57670920002</v>
+        <v>38889.22339400003</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.3852557670920002</v>
+        <v>0.3888922339400003</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -2476,6 +2563,9 @@
       <c r="R14" s="3" t="n">
         <v>38.3982</v>
       </c>
+      <c r="S14" s="3" t="n">
+        <v>38.499</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2500,16 +2590,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.82</v>
+        <v>11.81</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>115173.45354</v>
+        <v>115076.01407</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>15173.45354</v>
+        <v>15076.01407</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1517345354</v>
+        <v>0.1507601407</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -2538,6 +2628,9 @@
       <c r="R15" s="3" t="n">
         <v>11.82</v>
       </c>
+      <c r="S15" s="3" t="n">
+        <v>11.81</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2562,16 +2655,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.6116</v>
+        <v>24.6238</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>140850.4147648</v>
+        <v>140920.2344864</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>40850.41476479999</v>
+        <v>40920.2344864</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4085041476479999</v>
+        <v>0.409202344864</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -2600,6 +2693,9 @@
       <c r="R16" s="3" t="n">
         <v>24.6116</v>
       </c>
+      <c r="S16" s="3" t="n">
+        <v>24.6238</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2624,16 +2720,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.6948</v>
+        <v>16.7</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55193.9604036</v>
+        <v>55211.1519</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5193.960403600002</v>
+        <v>5211.151899999997</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.103879208072</v>
+        <v>0.1042230379999999</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -2662,6 +2758,9 @@
       <c r="R17" s="3" t="n">
         <v>16.6948</v>
       </c>
+      <c r="S17" s="3" t="n">
+        <v>16.7</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2686,16 +2785,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>45.63</v>
+        <v>45.34</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>86078.07468000001</v>
+        <v>85531.00824000001</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>6078.074680000005</v>
+        <v>5531.00824000001</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.07597593350000006</v>
+        <v>0.06913760300000013</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -2724,6 +2823,9 @@
       <c r="R18" s="3" t="n">
         <v>45.63</v>
       </c>
+      <c r="S18" s="3" t="n">
+        <v>45.34</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2748,16 +2850,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>14.3065</v>
+        <v>14.5354</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>206968.787779</v>
+        <v>210280.2305164</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>56968.78777900001</v>
+        <v>60280.23051639998</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.3797919185266667</v>
+        <v>0.4018682034426665</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -2786,6 +2888,9 @@
       <c r="R19" s="3" t="n">
         <v>14.3065</v>
       </c>
+      <c r="S19" s="3" t="n">
+        <v>14.5354</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2810,16 +2915,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.35</v>
+        <v>9.359999999999999</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>245491.75805</v>
+        <v>245754.31608</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-4508.241949999996</v>
+        <v>-4245.68392000001</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.01803296779999998</v>
+        <v>-0.01698273568000004</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -2848,6 +2953,9 @@
       <c r="R20" s="3" t="n">
         <v>9.35</v>
       </c>
+      <c r="S20" s="3" t="n">
+        <v>9.359999999999999</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2872,16 +2980,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>107.8068</v>
+        <v>107.6678</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>163786.4511612</v>
+        <v>163575.2741602</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-6213.548838799994</v>
+        <v>-6424.725839799998</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.03655028728705879</v>
+        <v>-0.03779250493999999</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -2910,6 +3018,9 @@
       <c r="R21" s="3" t="n">
         <v>107.8068</v>
       </c>
+      <c r="S21" s="3" t="n">
+        <v>107.6678</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2934,16 +3045,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>43.324</v>
+        <v>43.467</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>66478.94503999999</v>
+        <v>66698.37282</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>6478.945039999991</v>
+        <v>6698.372820000004</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1079824173333332</v>
+        <v>0.1116395470000001</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -2972,6 +3083,9 @@
       <c r="R22" s="3" t="n">
         <v>43.324</v>
       </c>
+      <c r="S22" s="3" t="n">
+        <v>43.467</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2996,16 +3110,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>60.7104</v>
+        <v>60.8801</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>164917.7981568</v>
+        <v>165378.7826067</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>14917.79815680001</v>
+        <v>15378.7826067</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.09945198771200008</v>
+        <v>0.102525217378</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -3034,6 +3148,9 @@
       <c r="R23" s="3" t="n">
         <v>60.7104</v>
       </c>
+      <c r="S23" s="3" t="n">
+        <v>60.8801</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3058,16 +3175,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>28.0977</v>
+        <v>28.1533</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>102089.7898122</v>
+        <v>102291.8060738</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>2089.789812200004</v>
+        <v>2291.806073800006</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.02089789812200004</v>
+        <v>0.02291806073800006</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -3096,6 +3213,9 @@
       <c r="R24" s="3" t="n">
         <v>28.0977</v>
       </c>
+      <c r="S24" s="3" t="n">
+        <v>28.1533</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3120,16 +3240,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.2689</v>
+        <v>11.3115</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>185054.2021386</v>
+        <v>185753.765451</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-14945.7978614</v>
+        <v>-14246.23454900002</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.074728989307</v>
+        <v>-0.07123117274500007</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -3158,6 +3278,9 @@
       <c r="R25" s="3" t="n">
         <v>11.2689</v>
       </c>
+      <c r="S25" s="3" t="n">
+        <v>11.3115</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3182,16 +3305,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>8.798500000000001</v>
+        <v>8.871499999999999</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>105069.1794275</v>
+        <v>105940.9246225</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>-4930.820572499986</v>
+        <v>-4059.075377500005</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>-0.0448256415681817</v>
+        <v>-0.03690068525000004</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -3220,6 +3343,9 @@
       <c r="R26" s="3" t="n">
         <v>8.798500000000001</v>
       </c>
+      <c r="S26" s="3" t="n">
+        <v>8.871499999999999</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3244,16 +3370,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>62.2395</v>
+        <v>62.4143</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>100259.12097</v>
+        <v>100540.699298</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-9740.879030000011</v>
+        <v>-9459.300702000008</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.08855344572727283</v>
+        <v>-0.08599364274545461</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -3282,6 +3408,9 @@
       <c r="R27" s="3" t="n">
         <v>62.2395</v>
       </c>
+      <c r="S27" s="3" t="n">
+        <v>62.4143</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3306,16 +3435,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>106.249</v>
+        <v>105.9949</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>351328.999593</v>
+        <v>350488.7780493</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-28671.00040700001</v>
+        <v>-29511.22195069998</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.07545000107105267</v>
+        <v>-0.0776611103965789</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -3344,6 +3473,9 @@
       <c r="R28" s="3" t="n">
         <v>106.249</v>
       </c>
+      <c r="S28" s="3" t="n">
+        <v>105.9949</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3368,16 +3500,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.955</v>
+        <v>11.9289</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>114812.269365</v>
+        <v>114561.6127167</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>14812.269365</v>
+        <v>14561.61271669999</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.14812269365</v>
+        <v>0.145616127167</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -3406,6 +3538,9 @@
       <c r="R29" s="3" t="n">
         <v>11.955</v>
       </c>
+      <c r="S29" s="3" t="n">
+        <v>11.9289</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3430,16 +3565,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>15.0861</v>
+        <v>15.0804</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>111574.6986321</v>
+        <v>111532.5422244</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>11574.6986321</v>
+        <v>11532.54222439999</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.115746986321</v>
+        <v>0.1153254222439999</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -3468,6 +3603,9 @@
       <c r="R30" s="3" t="n">
         <v>15.0861</v>
       </c>
+      <c r="S30" s="3" t="n">
+        <v>15.0804</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3492,16 +3630,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>413.0441</v>
+        <v>414.0702</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>109902.774128</v>
+        <v>110175.798816</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>9902.77412799999</v>
+        <v>10175.79881599999</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.0990277412799999</v>
+        <v>0.10175798816</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -3530,6 +3668,9 @@
       <c r="R31" s="3" t="n">
         <v>413.0441</v>
       </c>
+      <c r="S31" s="3" t="n">
+        <v>414.0702</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3554,16 +3695,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.14</v>
+        <v>10.16</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>214359.1944</v>
+        <v>214781.9936</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>14359.19440000001</v>
+        <v>14781.99359999999</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.07179597200000004</v>
+        <v>0.07390996799999994</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -3592,6 +3733,9 @@
       <c r="R32" s="3" t="n">
         <v>10.14</v>
       </c>
+      <c r="S32" s="3" t="n">
+        <v>10.16</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3616,16 +3760,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>17.92</v>
+        <v>17.85</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>64218.8288</v>
+        <v>63967.974</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>4218.828800000003</v>
+        <v>3967.974000000002</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.07031381333333338</v>
+        <v>0.06613290000000004</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -3654,6 +3798,9 @@
       <c r="R33" s="3" t="n">
         <v>17.92</v>
       </c>
+      <c r="S33" s="3" t="n">
+        <v>17.85</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3678,16 +3825,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>214.1576</v>
+        <v>213.5032</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>75283.0352856</v>
+        <v>75052.9933992</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-4716.964714400005</v>
+        <v>-4947.006600799999</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.05896205893000006</v>
+        <v>-0.06183758251</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -3716,6 +3863,9 @@
       <c r="R34" s="3" t="n">
         <v>214.1576</v>
       </c>
+      <c r="S34" s="3" t="n">
+        <v>213.5032</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3740,16 +3890,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>14.11</v>
+        <v>14.17</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>100680.81853</v>
+        <v>101108.94391</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>680.8185299999896</v>
+        <v>1108.943910000002</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.006808185299999895</v>
+        <v>0.01108943910000002</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -3778,6 +3928,9 @@
       <c r="R35" s="3" t="n">
         <v>14.11</v>
       </c>
+      <c r="S35" s="3" t="n">
+        <v>14.17</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3802,16 +3955,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>353.6924</v>
+        <v>350.9864</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>164716.6728344</v>
+        <v>163456.4723984</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>14716.67283440003</v>
+        <v>13456.47239840002</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.09811115222933353</v>
+        <v>0.08970981598933343</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -3840,6 +3993,9 @@
       <c r="R36" s="3" t="n">
         <v>353.6924</v>
       </c>
+      <c r="S36" s="3" t="n">
+        <v>350.9864</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3864,16 +4020,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>15.842</v>
+        <v>15.648</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>59611.68753800001</v>
+        <v>58881.687072</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>9611.687538000006</v>
+        <v>8881.687072000001</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.1922337507600001</v>
+        <v>0.17763374144</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -3902,6 +4058,9 @@
       <c r="R37" s="3" t="n">
         <v>15.842</v>
       </c>
+      <c r="S37" s="3" t="n">
+        <v>15.648</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3926,16 +4085,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>14.0227</v>
+        <v>14.0547</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>83862.5049414</v>
+        <v>84053.88036540001</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>3862.504941399995</v>
+        <v>4053.880365400008</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.04828131176749994</v>
+        <v>0.0506735045675001</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -3964,6 +4123,9 @@
       <c r="R38" s="3" t="n">
         <v>14.0227</v>
       </c>
+      <c r="S38" s="3" t="n">
+        <v>14.0547</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3988,16 +4150,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1005.1862</v>
+        <v>1005.0898</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50139.6928422</v>
+        <v>50134.8843138</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>139.6928421999983</v>
+        <v>134.8843138000011</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.002793856843999965</v>
+        <v>0.002697686276000022</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -4026,6 +4188,9 @@
       <c r="R39" s="3" t="n">
         <v>1005.1862</v>
       </c>
+      <c r="S39" s="3" t="n">
+        <v>1005.0898</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4050,16 +4215,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>19.849</v>
+        <v>20.0352</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>100059.344923</v>
+        <v>100997.9841504</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>59.34492299999692</v>
+        <v>997.9841503999924</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.0005934492299999693</v>
+        <v>0.009979841503999923</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -4088,6 +4253,9 @@
       <c r="R40" s="3" t="n">
         <v>19.849</v>
       </c>
+      <c r="S40" s="3" t="n">
+        <v>20.0352</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
@@ -4099,13 +4267,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4827372.0145348</v>
+        <v>4834300.7735287</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>357372.0145348</v>
+        <v>364300.7735287001</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.07994899654022372</v>
+        <v>0.08149905448069353</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-05-24
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-05-23 05:38 IST</t>
+          <t>Generated: 2026-05-24 06:00 IST</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-05-23</t>
+          <t>Last snapshot: 2026-05-24</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q19"/>
+  <dimension ref="A1:R19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -636,6 +636,7 @@
     <col width="21" customWidth="1" min="15" max="15"/>
     <col width="21" customWidth="1" min="16" max="16"/>
     <col width="21" customWidth="1" min="17" max="17"/>
+    <col width="21" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -724,6 +725,11 @@
           <t>2026-05-23</t>
         </is>
       </c>
+      <c r="R1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -781,6 +787,9 @@
       <c r="Q2" s="3" t="n">
         <v>569.9500122070312</v>
       </c>
+      <c r="R2" s="3" t="n">
+        <v>569.9500122070312</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -865,6 +874,9 @@
       <c r="Q4" s="3" t="n">
         <v>1541.699951171875</v>
       </c>
+      <c r="R4" s="3" t="n">
+        <v>1541.699951171875</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -922,6 +934,9 @@
       <c r="Q5" s="3" t="n">
         <v>653.2000122070312</v>
       </c>
+      <c r="R5" s="3" t="n">
+        <v>653.2000122070312</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -979,6 +994,9 @@
       <c r="Q6" s="3" t="n">
         <v>382.25</v>
       </c>
+      <c r="R6" s="3" t="n">
+        <v>382.25</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1036,6 +1054,9 @@
       <c r="Q7" s="3" t="n">
         <v>216</v>
       </c>
+      <c r="R7" s="3" t="n">
+        <v>216</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1120,6 +1141,9 @@
       <c r="Q9" s="3" t="n">
         <v>18.76000022888184</v>
       </c>
+      <c r="R9" s="3" t="n">
+        <v>18.76000022888184</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1177,6 +1201,9 @@
       <c r="Q10" s="3" t="n">
         <v>499.75</v>
       </c>
+      <c r="R10" s="3" t="n">
+        <v>499.75</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1234,6 +1261,9 @@
       <c r="Q11" s="3" t="n">
         <v>8.369999885559082</v>
       </c>
+      <c r="R11" s="3" t="n">
+        <v>8.369999885559082</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1291,6 +1321,9 @@
       <c r="Q12" s="3" t="n">
         <v>2564.10009765625</v>
       </c>
+      <c r="R12" s="3" t="n">
+        <v>2564.10009765625</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1348,6 +1381,9 @@
       <c r="Q13" s="3" t="n">
         <v>53.75</v>
       </c>
+      <c r="R13" s="3" t="n">
+        <v>53.75</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1405,6 +1441,9 @@
       <c r="Q14" s="3" t="n">
         <v>750.2000122070312</v>
       </c>
+      <c r="R14" s="3" t="n">
+        <v>750.2000122070312</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1516,6 +1555,9 @@
       <c r="Q17" s="3" t="n">
         <v>468.1499938964844</v>
       </c>
+      <c r="R17" s="3" t="n">
+        <v>468.1499938964844</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1571,6 +1613,9 @@
         <v>408.2000122070312</v>
       </c>
       <c r="Q18" s="3" t="n">
+        <v>408.8999938964844</v>
+      </c>
+      <c r="R18" s="3" t="n">
         <v>408.8999938964844</v>
       </c>
     </row>
@@ -1601,7 +1646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S41"/>
+  <dimension ref="A1:T41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1623,6 +1668,7 @@
     <col width="13" customWidth="1" min="17" max="17"/>
     <col width="13" customWidth="1" min="18" max="18"/>
     <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="13" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1721,6 +1767,11 @@
           <t>2026-05-23</t>
         </is>
       </c>
+      <c r="T1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1786,6 +1837,9 @@
       <c r="S2" s="3" t="n">
         <v>56.8797</v>
       </c>
+      <c r="T2" s="3" t="n">
+        <v>56.8797</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1851,6 +1905,9 @@
       <c r="S3" s="3" t="n">
         <v>25.7058</v>
       </c>
+      <c r="T3" s="3" t="n">
+        <v>25.7058</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1916,6 +1973,9 @@
       <c r="S4" s="3" t="n">
         <v>12.63</v>
       </c>
+      <c r="T4" s="3" t="n">
+        <v>12.63</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1981,6 +2041,9 @@
       <c r="S5" s="3" t="n">
         <v>9.544499999999999</v>
       </c>
+      <c r="T5" s="3" t="n">
+        <v>9.544499999999999</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2046,6 +2109,9 @@
       <c r="S6" s="3" t="n">
         <v>12.4901</v>
       </c>
+      <c r="T6" s="3" t="n">
+        <v>12.4901</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2111,6 +2177,9 @@
       <c r="S7" s="3" t="n">
         <v>33.9116</v>
       </c>
+      <c r="T7" s="3" t="n">
+        <v>33.9116</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2176,6 +2245,9 @@
       <c r="S8" s="3" t="n">
         <v>30.4549</v>
       </c>
+      <c r="T8" s="3" t="n">
+        <v>30.4549</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2241,6 +2313,9 @@
       <c r="S9" s="3" t="n">
         <v>41.9916</v>
       </c>
+      <c r="T9" s="3" t="n">
+        <v>41.9916</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2306,6 +2381,9 @@
       <c r="S10" s="3" t="n">
         <v>46.457</v>
       </c>
+      <c r="T10" s="3" t="n">
+        <v>46.457</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2371,6 +2449,9 @@
       <c r="S11" s="3" t="n">
         <v>104.1779</v>
       </c>
+      <c r="T11" s="3" t="n">
+        <v>104.1779</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2436,6 +2517,9 @@
       <c r="S12" s="3" t="n">
         <v>220.359</v>
       </c>
+      <c r="T12" s="3" t="n">
+        <v>220.359</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2501,6 +2585,9 @@
       <c r="S13" s="3" t="n">
         <v>19.908</v>
       </c>
+      <c r="T13" s="3" t="n">
+        <v>19.908</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2566,6 +2653,9 @@
       <c r="S14" s="3" t="n">
         <v>38.499</v>
       </c>
+      <c r="T14" s="3" t="n">
+        <v>38.499</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2631,6 +2721,9 @@
       <c r="S15" s="3" t="n">
         <v>11.81</v>
       </c>
+      <c r="T15" s="3" t="n">
+        <v>11.81</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2696,6 +2789,9 @@
       <c r="S16" s="3" t="n">
         <v>24.6238</v>
       </c>
+      <c r="T16" s="3" t="n">
+        <v>24.6238</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2761,6 +2857,9 @@
       <c r="S17" s="3" t="n">
         <v>16.7</v>
       </c>
+      <c r="T17" s="3" t="n">
+        <v>16.7</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2826,6 +2925,9 @@
       <c r="S18" s="3" t="n">
         <v>45.34</v>
       </c>
+      <c r="T18" s="3" t="n">
+        <v>45.34</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2891,6 +2993,9 @@
       <c r="S19" s="3" t="n">
         <v>14.5354</v>
       </c>
+      <c r="T19" s="3" t="n">
+        <v>14.5354</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2956,6 +3061,9 @@
       <c r="S20" s="3" t="n">
         <v>9.359999999999999</v>
       </c>
+      <c r="T20" s="3" t="n">
+        <v>9.359999999999999</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3021,6 +3129,9 @@
       <c r="S21" s="3" t="n">
         <v>107.6678</v>
       </c>
+      <c r="T21" s="3" t="n">
+        <v>107.6678</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3086,6 +3197,9 @@
       <c r="S22" s="3" t="n">
         <v>43.467</v>
       </c>
+      <c r="T22" s="3" t="n">
+        <v>43.467</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3151,6 +3265,9 @@
       <c r="S23" s="3" t="n">
         <v>60.8801</v>
       </c>
+      <c r="T23" s="3" t="n">
+        <v>60.8801</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3216,6 +3333,9 @@
       <c r="S24" s="3" t="n">
         <v>28.1533</v>
       </c>
+      <c r="T24" s="3" t="n">
+        <v>28.1533</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3281,6 +3401,9 @@
       <c r="S25" s="3" t="n">
         <v>11.3115</v>
       </c>
+      <c r="T25" s="3" t="n">
+        <v>11.3115</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3346,6 +3469,9 @@
       <c r="S26" s="3" t="n">
         <v>8.871499999999999</v>
       </c>
+      <c r="T26" s="3" t="n">
+        <v>8.871499999999999</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3411,6 +3537,9 @@
       <c r="S27" s="3" t="n">
         <v>62.4143</v>
       </c>
+      <c r="T27" s="3" t="n">
+        <v>62.4143</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3476,6 +3605,9 @@
       <c r="S28" s="3" t="n">
         <v>105.9949</v>
       </c>
+      <c r="T28" s="3" t="n">
+        <v>105.9949</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3541,6 +3673,9 @@
       <c r="S29" s="3" t="n">
         <v>11.9289</v>
       </c>
+      <c r="T29" s="3" t="n">
+        <v>11.9289</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3606,6 +3741,9 @@
       <c r="S30" s="3" t="n">
         <v>15.0804</v>
       </c>
+      <c r="T30" s="3" t="n">
+        <v>15.0804</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3671,6 +3809,9 @@
       <c r="S31" s="3" t="n">
         <v>414.0702</v>
       </c>
+      <c r="T31" s="3" t="n">
+        <v>414.0702</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3736,6 +3877,9 @@
       <c r="S32" s="3" t="n">
         <v>10.16</v>
       </c>
+      <c r="T32" s="3" t="n">
+        <v>10.16</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3801,6 +3945,9 @@
       <c r="S33" s="3" t="n">
         <v>17.85</v>
       </c>
+      <c r="T33" s="3" t="n">
+        <v>17.85</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3866,6 +4013,9 @@
       <c r="S34" s="3" t="n">
         <v>213.5032</v>
       </c>
+      <c r="T34" s="3" t="n">
+        <v>213.5032</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3931,6 +4081,9 @@
       <c r="S35" s="3" t="n">
         <v>14.17</v>
       </c>
+      <c r="T35" s="3" t="n">
+        <v>14.17</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3996,6 +4149,9 @@
       <c r="S36" s="3" t="n">
         <v>350.9864</v>
       </c>
+      <c r="T36" s="3" t="n">
+        <v>350.9864</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4061,6 +4217,9 @@
       <c r="S37" s="3" t="n">
         <v>15.648</v>
       </c>
+      <c r="T37" s="3" t="n">
+        <v>15.648</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4126,6 +4285,9 @@
       <c r="S38" s="3" t="n">
         <v>14.0547</v>
       </c>
+      <c r="T38" s="3" t="n">
+        <v>14.0547</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4191,6 +4353,9 @@
       <c r="S39" s="3" t="n">
         <v>1005.0898</v>
       </c>
+      <c r="T39" s="3" t="n">
+        <v>1005.0898</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4254,6 +4419,9 @@
         <v>19.849</v>
       </c>
       <c r="S40" s="3" t="n">
+        <v>20.0352</v>
+      </c>
+      <c r="T40" s="3" t="n">
         <v>20.0352</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily portfolio update 2026-05-25
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-05-24 06:00 IST</t>
+          <t>Generated: 2026-05-25 06:26 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4834300.7735287</v>
+        <v>4834270.1399745</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>364300.7735286998</v>
+        <v>364270.1399745001</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.08149905448069346</v>
+        <v>0.0814922013365772</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>554338.0011444092</v>
+        <v>558467.5000457764</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-36444.01885559084</v>
+        <v>-32314.51995422365</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.06168775897342109</v>
+        <v>-0.05469787309069367</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5388638.774673109</v>
+        <v>5392737.640020276</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>327856.7546731094</v>
+        <v>331955.6200202769</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.06478381273436262</v>
+        <v>0.06559374000073548</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-05-24</t>
+          <t>Last snapshot: 2026-05-25</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R19"/>
+  <dimension ref="A1:S19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -637,6 +637,7 @@
     <col width="21" customWidth="1" min="16" max="16"/>
     <col width="21" customWidth="1" min="17" max="17"/>
     <col width="21" customWidth="1" min="18" max="18"/>
+    <col width="21" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -730,6 +731,11 @@
           <t>2026-05-24</t>
         </is>
       </c>
+      <c r="S1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -749,13 +755,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>569.9500122070312</v>
+        <v>573.9500122070312</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>45596.0009765625</v>
+        <v>45916.0009765625</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1778.490976562498</v>
+        <v>2098.490976562498</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -790,6 +796,9 @@
       <c r="R2" s="3" t="n">
         <v>569.9500122070312</v>
       </c>
+      <c r="S2" s="3" t="n">
+        <v>573.9500122070312</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -836,13 +845,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1541.699951171875</v>
+        <v>1558.599975585938</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>30833.9990234375</v>
+        <v>31171.99951171875</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-1270.580976562502</v>
+        <v>-932.5804882812517</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -877,6 +886,9 @@
       <c r="R4" s="3" t="n">
         <v>1541.699951171875</v>
       </c>
+      <c r="S4" s="3" t="n">
+        <v>1558.599975585938</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -896,13 +908,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>653.2000122070312</v>
+        <v>638.7000122070312</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13064.00024414062</v>
+        <v>12774.00024414062</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1149.099755859375</v>
+        <v>-1439.099755859375</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -937,6 +949,9 @@
       <c r="R5" s="3" t="n">
         <v>653.2000122070312</v>
       </c>
+      <c r="S5" s="3" t="n">
+        <v>638.7000122070312</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -956,13 +971,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>382.25</v>
+        <v>382.9500122070312</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15290</v>
+        <v>15318.00048828125</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2212.240000000002</v>
+        <v>-2184.239511718752</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -997,6 +1012,9 @@
       <c r="R6" s="3" t="n">
         <v>382.25</v>
       </c>
+      <c r="S6" s="3" t="n">
+        <v>382.9500122070312</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1016,13 +1034,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>216</v>
+        <v>227.75</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>21600</v>
+        <v>22775</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-4833.82</v>
+        <v>-3658.82</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1057,6 +1075,9 @@
       <c r="R7" s="3" t="n">
         <v>216</v>
       </c>
+      <c r="S7" s="3" t="n">
+        <v>227.75</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1103,13 +1124,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>18.76000022888184</v>
+        <v>18.90999984741211</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>28140.00034332275</v>
+        <v>28364.99977111816</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-2910.169656677244</v>
+        <v>-2685.170228881834</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1144,6 +1165,9 @@
       <c r="R9" s="3" t="n">
         <v>18.76000022888184</v>
       </c>
+      <c r="S9" s="3" t="n">
+        <v>18.90999984741211</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1163,13 +1187,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>499.75</v>
+        <v>486.5</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>49975</v>
+        <v>48650</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-1523.480000000003</v>
+        <v>-2848.480000000003</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1204,6 +1228,9 @@
       <c r="R10" s="3" t="n">
         <v>499.75</v>
       </c>
+      <c r="S10" s="3" t="n">
+        <v>486.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1223,13 +1250,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>8.369999885559082</v>
+        <v>8.659999847412109</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>8369.999885559082</v>
+        <v>8659.999847412109</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-1471.210114440917</v>
+        <v>-1181.21015258789</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -1264,6 +1291,9 @@
       <c r="R11" s="3" t="n">
         <v>8.369999885559082</v>
       </c>
+      <c r="S11" s="3" t="n">
+        <v>8.659999847412109</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1283,13 +1313,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2564.10009765625</v>
+        <v>2594.699951171875</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25641.0009765625</v>
+        <v>25946.99951171875</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2082.2490234375</v>
+        <v>-1776.25048828125</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -1324,6 +1354,9 @@
       <c r="R12" s="3" t="n">
         <v>2564.10009765625</v>
       </c>
+      <c r="S12" s="3" t="n">
+        <v>2594.699951171875</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1343,13 +1376,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>53.75</v>
+        <v>54.40000152587891</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>32250</v>
+        <v>32640.00091552734</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-2781.760000000002</v>
+        <v>-2391.759084472658</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -1384,6 +1417,9 @@
       <c r="R13" s="3" t="n">
         <v>53.75</v>
       </c>
+      <c r="S13" s="3" t="n">
+        <v>54.40000152587891</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1403,13 +1439,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>750.2000122070312</v>
+        <v>781.25</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>37510.00061035156</v>
+        <v>39062.5</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-4952.50938964844</v>
+        <v>-3400.010000000002</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -1444,6 +1480,9 @@
       <c r="R14" s="3" t="n">
         <v>750.2000122070312</v>
       </c>
+      <c r="S14" s="3" t="n">
+        <v>781.25</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1517,13 +1556,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>468.1499938964844</v>
+        <v>482.5499877929688</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>23407.49969482422</v>
+        <v>24127.49938964844</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>1652.96969482422</v>
+        <v>2372.969389648439</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -1558,6 +1597,9 @@
       <c r="R17" s="3" t="n">
         <v>468.1499938964844</v>
       </c>
+      <c r="S17" s="3" t="n">
+        <v>482.5499877929688</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1577,13 +1619,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>408.8999938964844</v>
+        <v>412.8999938964844</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>40889.99938964844</v>
+        <v>41289.99938964844</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-5750.820610351562</v>
+        <v>-5350.820610351562</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -1618,6 +1660,9 @@
       <c r="R18" s="3" t="n">
         <v>408.8999938964844</v>
       </c>
+      <c r="S18" s="3" t="n">
+        <v>412.8999938964844</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -1629,10 +1674,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>554338.0011444092</v>
+        <v>558467.5000457764</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-36444.01885559083</v>
+        <v>-32314.51995422364</v>
       </c>
     </row>
   </sheetData>
@@ -1646,7 +1691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T41"/>
+  <dimension ref="A1:U41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1669,6 +1714,7 @@
     <col width="13" customWidth="1" min="18" max="18"/>
     <col width="13" customWidth="1" min="19" max="19"/>
     <col width="13" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1772,6 +1818,11 @@
           <t>2026-05-24</t>
         </is>
       </c>
+      <c r="U1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1840,6 +1891,9 @@
       <c r="T2" s="3" t="n">
         <v>56.8797</v>
       </c>
+      <c r="U2" s="3" t="n">
+        <v>56.8797</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1908,6 +1962,9 @@
       <c r="T3" s="3" t="n">
         <v>25.7058</v>
       </c>
+      <c r="U3" s="3" t="n">
+        <v>25.7058</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1976,6 +2033,9 @@
       <c r="T4" s="3" t="n">
         <v>12.63</v>
       </c>
+      <c r="U4" s="3" t="n">
+        <v>12.63</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2044,6 +2104,9 @@
       <c r="T5" s="3" t="n">
         <v>9.544499999999999</v>
       </c>
+      <c r="U5" s="3" t="n">
+        <v>9.544499999999999</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2112,6 +2175,9 @@
       <c r="T6" s="3" t="n">
         <v>12.4901</v>
       </c>
+      <c r="U6" s="3" t="n">
+        <v>12.4901</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2180,6 +2246,9 @@
       <c r="T7" s="3" t="n">
         <v>33.9116</v>
       </c>
+      <c r="U7" s="3" t="n">
+        <v>33.9116</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2248,6 +2317,9 @@
       <c r="T8" s="3" t="n">
         <v>30.4549</v>
       </c>
+      <c r="U8" s="3" t="n">
+        <v>30.4549</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2316,6 +2388,9 @@
       <c r="T9" s="3" t="n">
         <v>41.9916</v>
       </c>
+      <c r="U9" s="3" t="n">
+        <v>41.9916</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2384,6 +2459,9 @@
       <c r="T10" s="3" t="n">
         <v>46.457</v>
       </c>
+      <c r="U10" s="3" t="n">
+        <v>46.457</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2408,16 +2486,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>104.1779</v>
+        <v>104.0761</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31349.1094901</v>
+        <v>31318.4759359</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1349.109490099996</v>
+        <v>1318.475935899998</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.04497031633666653</v>
+        <v>0.04394919786333327</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -2452,6 +2530,9 @@
       <c r="T11" s="3" t="n">
         <v>104.1779</v>
       </c>
+      <c r="U11" s="3" t="n">
+        <v>104.0761</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2520,6 +2601,9 @@
       <c r="T12" s="3" t="n">
         <v>220.359</v>
       </c>
+      <c r="U12" s="3" t="n">
+        <v>220.359</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2588,6 +2672,9 @@
       <c r="T13" s="3" t="n">
         <v>19.908</v>
       </c>
+      <c r="U13" s="3" t="n">
+        <v>19.908</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2656,6 +2743,9 @@
       <c r="T14" s="3" t="n">
         <v>38.499</v>
       </c>
+      <c r="U14" s="3" t="n">
+        <v>38.499</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2724,6 +2814,9 @@
       <c r="T15" s="3" t="n">
         <v>11.81</v>
       </c>
+      <c r="U15" s="3" t="n">
+        <v>11.81</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2792,6 +2885,9 @@
       <c r="T16" s="3" t="n">
         <v>24.6238</v>
       </c>
+      <c r="U16" s="3" t="n">
+        <v>24.6238</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2860,6 +2956,9 @@
       <c r="T17" s="3" t="n">
         <v>16.7</v>
       </c>
+      <c r="U17" s="3" t="n">
+        <v>16.7</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2928,6 +3027,9 @@
       <c r="T18" s="3" t="n">
         <v>45.34</v>
       </c>
+      <c r="U18" s="3" t="n">
+        <v>45.34</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2996,6 +3098,9 @@
       <c r="T19" s="3" t="n">
         <v>14.5354</v>
       </c>
+      <c r="U19" s="3" t="n">
+        <v>14.5354</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3064,6 +3169,9 @@
       <c r="T20" s="3" t="n">
         <v>9.359999999999999</v>
       </c>
+      <c r="U20" s="3" t="n">
+        <v>9.359999999999999</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3132,6 +3240,9 @@
       <c r="T21" s="3" t="n">
         <v>107.6678</v>
       </c>
+      <c r="U21" s="3" t="n">
+        <v>107.6678</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3200,6 +3311,9 @@
       <c r="T22" s="3" t="n">
         <v>43.467</v>
       </c>
+      <c r="U22" s="3" t="n">
+        <v>43.467</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3268,6 +3382,9 @@
       <c r="T23" s="3" t="n">
         <v>60.8801</v>
       </c>
+      <c r="U23" s="3" t="n">
+        <v>60.8801</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3336,6 +3453,9 @@
       <c r="T24" s="3" t="n">
         <v>28.1533</v>
       </c>
+      <c r="U24" s="3" t="n">
+        <v>28.1533</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3404,6 +3524,9 @@
       <c r="T25" s="3" t="n">
         <v>11.3115</v>
       </c>
+      <c r="U25" s="3" t="n">
+        <v>11.3115</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3472,6 +3595,9 @@
       <c r="T26" s="3" t="n">
         <v>8.871499999999999</v>
       </c>
+      <c r="U26" s="3" t="n">
+        <v>8.871499999999999</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3540,6 +3666,9 @@
       <c r="T27" s="3" t="n">
         <v>62.4143</v>
       </c>
+      <c r="U27" s="3" t="n">
+        <v>62.4143</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3608,6 +3737,9 @@
       <c r="T28" s="3" t="n">
         <v>105.9949</v>
       </c>
+      <c r="U28" s="3" t="n">
+        <v>105.9949</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3676,6 +3808,9 @@
       <c r="T29" s="3" t="n">
         <v>11.9289</v>
       </c>
+      <c r="U29" s="3" t="n">
+        <v>11.9289</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3744,6 +3879,9 @@
       <c r="T30" s="3" t="n">
         <v>15.0804</v>
       </c>
+      <c r="U30" s="3" t="n">
+        <v>15.0804</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3812,6 +3950,9 @@
       <c r="T31" s="3" t="n">
         <v>414.0702</v>
       </c>
+      <c r="U31" s="3" t="n">
+        <v>414.0702</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3880,6 +4021,9 @@
       <c r="T32" s="3" t="n">
         <v>10.16</v>
       </c>
+      <c r="U32" s="3" t="n">
+        <v>10.16</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3948,6 +4092,9 @@
       <c r="T33" s="3" t="n">
         <v>17.85</v>
       </c>
+      <c r="U33" s="3" t="n">
+        <v>17.85</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4016,6 +4163,9 @@
       <c r="T34" s="3" t="n">
         <v>213.5032</v>
       </c>
+      <c r="U34" s="3" t="n">
+        <v>213.5032</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4084,6 +4234,9 @@
       <c r="T35" s="3" t="n">
         <v>14.17</v>
       </c>
+      <c r="U35" s="3" t="n">
+        <v>14.17</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4152,6 +4305,9 @@
       <c r="T36" s="3" t="n">
         <v>350.9864</v>
       </c>
+      <c r="U36" s="3" t="n">
+        <v>350.9864</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4220,6 +4376,9 @@
       <c r="T37" s="3" t="n">
         <v>15.648</v>
       </c>
+      <c r="U37" s="3" t="n">
+        <v>15.648</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4288,6 +4447,9 @@
       <c r="T38" s="3" t="n">
         <v>14.0547</v>
       </c>
+      <c r="U38" s="3" t="n">
+        <v>14.0547</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4356,6 +4518,9 @@
       <c r="T39" s="3" t="n">
         <v>1005.0898</v>
       </c>
+      <c r="U39" s="3" t="n">
+        <v>1005.0898</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4424,6 +4589,9 @@
       <c r="T40" s="3" t="n">
         <v>20.0352</v>
       </c>
+      <c r="U40" s="3" t="n">
+        <v>20.0352</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
@@ -4435,13 +4603,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4834300.7735287</v>
+        <v>4834270.1399745</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>364300.7735287001</v>
+        <v>364270.1399745001</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.08149905448069353</v>
+        <v>0.0814922013365772</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-05-26
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -484,7 +484,7 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-05-25 06:26 IST</t>
+          <t>Generated: 2026-05-26 06:05 IST</t>
         </is>
       </c>
     </row>
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>558467.5000457764</v>
+        <v>564468.9925460815</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-32314.51995422365</v>
+        <v>-26313.02745391848</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.05469787309069367</v>
+        <v>-0.04453931663986401</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5392737.640020276</v>
+        <v>5398739.132520582</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>331955.6200202769</v>
+        <v>337957.112520582</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.06559374000073548</v>
+        <v>0.06677962243483114</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-05-25</t>
+          <t>Last snapshot: 2026-05-26</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S19"/>
+  <dimension ref="A1:T19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -638,6 +638,7 @@
     <col width="21" customWidth="1" min="17" max="17"/>
     <col width="21" customWidth="1" min="18" max="18"/>
     <col width="21" customWidth="1" min="19" max="19"/>
+    <col width="21" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -736,6 +737,11 @@
           <t>2026-05-25</t>
         </is>
       </c>
+      <c r="T1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -755,13 +761,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>573.9500122070312</v>
+        <v>581.0999755859375</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>45916.0009765625</v>
+        <v>46487.998046875</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>2098.490976562498</v>
+        <v>2670.488046874998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -799,6 +805,9 @@
       <c r="S2" s="3" t="n">
         <v>573.9500122070312</v>
       </c>
+      <c r="T2" s="3" t="n">
+        <v>581.0999755859375</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -845,13 +854,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1558.599975585938</v>
+        <v>1557.199951171875</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>31171.99951171875</v>
+        <v>31143.9990234375</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-932.5804882812517</v>
+        <v>-960.5809765625017</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -889,6 +898,9 @@
       <c r="S4" s="3" t="n">
         <v>1558.599975585938</v>
       </c>
+      <c r="T4" s="3" t="n">
+        <v>1557.199951171875</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -908,13 +920,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>638.7000122070312</v>
+        <v>642.0499877929688</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>12774.00024414062</v>
+        <v>12840.99975585938</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1439.099755859375</v>
+        <v>-1372.100244140625</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -952,6 +964,9 @@
       <c r="S5" s="3" t="n">
         <v>638.7000122070312</v>
       </c>
+      <c r="T5" s="3" t="n">
+        <v>642.0499877929688</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -971,13 +986,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>382.9500122070312</v>
+        <v>392.7999877929688</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15318.00048828125</v>
+        <v>15711.99951171875</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2184.239511718752</v>
+        <v>-1790.240488281252</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1015,6 +1030,9 @@
       <c r="S6" s="3" t="n">
         <v>382.9500122070312</v>
       </c>
+      <c r="T6" s="3" t="n">
+        <v>392.7999877929688</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1034,13 +1052,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>227.75</v>
+        <v>229.75</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>22775</v>
+        <v>22975</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-3658.82</v>
+        <v>-3458.82</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1078,6 +1096,9 @@
       <c r="S7" s="3" t="n">
         <v>227.75</v>
       </c>
+      <c r="T7" s="3" t="n">
+        <v>229.75</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1124,13 +1145,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>18.90999984741211</v>
+        <v>19.34000015258789</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>28364.99977111816</v>
+        <v>29010.00022888184</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-2685.170228881834</v>
+        <v>-2040.169771118162</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1168,6 +1189,9 @@
       <c r="S9" s="3" t="n">
         <v>18.90999984741211</v>
       </c>
+      <c r="T9" s="3" t="n">
+        <v>19.34000015258789</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1187,13 +1211,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>486.5</v>
+        <v>494.0499877929688</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48650</v>
+        <v>49404.99877929688</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-2848.480000000003</v>
+        <v>-2093.481220703128</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1231,6 +1255,9 @@
       <c r="S10" s="3" t="n">
         <v>486.5</v>
       </c>
+      <c r="T10" s="3" t="n">
+        <v>494.0499877929688</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1250,13 +1277,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>8.659999847412109</v>
+        <v>9.189999580383301</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>8659.999847412109</v>
+        <v>9189.999580383301</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-1181.21015258789</v>
+        <v>-651.2104196166983</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -1294,6 +1321,9 @@
       <c r="S11" s="3" t="n">
         <v>8.659999847412109</v>
       </c>
+      <c r="T11" s="3" t="n">
+        <v>9.189999580383301</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1313,13 +1343,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2594.699951171875</v>
+        <v>2599.89990234375</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25946.99951171875</v>
+        <v>25998.9990234375</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-1776.25048828125</v>
+        <v>-1724.2509765625</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -1357,6 +1387,9 @@
       <c r="S12" s="3" t="n">
         <v>2594.699951171875</v>
       </c>
+      <c r="T12" s="3" t="n">
+        <v>2599.89990234375</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1376,13 +1409,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>54.40000152587891</v>
+        <v>55.16999816894531</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>32640.00091552734</v>
+        <v>33101.99890136719</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-2391.759084472658</v>
+        <v>-1929.761098632815</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -1420,6 +1453,9 @@
       <c r="S13" s="3" t="n">
         <v>54.40000152587891</v>
       </c>
+      <c r="T13" s="3" t="n">
+        <v>55.16999816894531</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1439,13 +1475,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>781.25</v>
+        <v>790.25</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>39062.5</v>
+        <v>39512.5</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-3400.010000000002</v>
+        <v>-2950.010000000002</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -1483,6 +1519,9 @@
       <c r="S14" s="3" t="n">
         <v>781.25</v>
       </c>
+      <c r="T14" s="3" t="n">
+        <v>790.25</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1556,13 +1595,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>482.5499877929688</v>
+        <v>498.3999938964844</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>24127.49938964844</v>
+        <v>24919.99969482422</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>2372.969389648439</v>
+        <v>3165.46969482422</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -1600,6 +1639,9 @@
       <c r="S17" s="3" t="n">
         <v>482.5499877929688</v>
       </c>
+      <c r="T17" s="3" t="n">
+        <v>498.3999938964844</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1619,13 +1661,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>412.8999938964844</v>
+        <v>424</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>41289.99938964844</v>
+        <v>42400</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-5350.820610351562</v>
+        <v>-4240.82</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -1663,6 +1705,9 @@
       <c r="S18" s="3" t="n">
         <v>412.8999938964844</v>
       </c>
+      <c r="T18" s="3" t="n">
+        <v>424</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -1674,10 +1719,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>558467.5000457764</v>
+        <v>564468.9925460815</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-32314.51995422364</v>
+        <v>-26313.02745391847</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-05-27
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-05-26 06:05 IST</t>
+          <t>Generated: 2026-05-27 06:19 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4834270.1399745</v>
+        <v>4893403.9578459</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>364270.1399745001</v>
+        <v>423403.9578459002</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.0814922013365772</v>
+        <v>0.09472124336597321</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>564468.9925460815</v>
+        <v>568531.9986038208</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-26313.02745391848</v>
+        <v>-22250.02139617922</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.04453931663986401</v>
+        <v>-0.03766198131110899</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5398739.132520582</v>
+        <v>5461935.956449721</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>337957.112520582</v>
+        <v>401153.9364497215</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.06677962243483114</v>
+        <v>0.07926718338477687</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-05-26</t>
+          <t>Last snapshot: 2026-05-27</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T19"/>
+  <dimension ref="A1:U19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -639,6 +639,7 @@
     <col width="21" customWidth="1" min="18" max="18"/>
     <col width="21" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
+    <col width="21" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -742,6 +743,11 @@
           <t>2026-05-26</t>
         </is>
       </c>
+      <c r="U1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -808,6 +814,9 @@
       <c r="T2" s="3" t="n">
         <v>581.0999755859375</v>
       </c>
+      <c r="U2" s="3" t="n">
+        <v>581.0999755859375</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -854,13 +863,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1557.199951171875</v>
+        <v>1583.300048828125</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>31143.9990234375</v>
+        <v>31666.0009765625</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-960.5809765625017</v>
+        <v>-438.5790234375017</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -901,6 +910,9 @@
       <c r="T4" s="3" t="n">
         <v>1557.199951171875</v>
       </c>
+      <c r="U4" s="3" t="n">
+        <v>1583.300048828125</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -920,13 +932,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>642.0499877929688</v>
+        <v>635.6500244140625</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>12840.99975585938</v>
+        <v>12713.00048828125</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1372.100244140625</v>
+        <v>-1500.09951171875</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -967,6 +979,9 @@
       <c r="T5" s="3" t="n">
         <v>642.0499877929688</v>
       </c>
+      <c r="U5" s="3" t="n">
+        <v>635.6500244140625</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -986,13 +1001,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>392.7999877929688</v>
+        <v>395.4500122070312</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15711.99951171875</v>
+        <v>15818.00048828125</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-1790.240488281252</v>
+        <v>-1684.239511718752</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1033,6 +1048,9 @@
       <c r="T6" s="3" t="n">
         <v>392.7999877929688</v>
       </c>
+      <c r="U6" s="3" t="n">
+        <v>395.4500122070312</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1052,13 +1070,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>229.75</v>
+        <v>233.6999969482422</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>22975</v>
+        <v>23369.99969482422</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-3458.82</v>
+        <v>-3063.820305175781</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1099,6 +1117,9 @@
       <c r="T7" s="3" t="n">
         <v>229.75</v>
       </c>
+      <c r="U7" s="3" t="n">
+        <v>233.6999969482422</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1145,13 +1166,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>19.34000015258789</v>
+        <v>22.32999992370605</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>29010.00022888184</v>
-      </c>
-      <c r="G9" s="6" t="n">
-        <v>-2040.169771118162</v>
+        <v>33494.99988555908</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>2444.829885559084</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1192,6 +1213,9 @@
       <c r="T9" s="3" t="n">
         <v>19.34000015258789</v>
       </c>
+      <c r="U9" s="3" t="n">
+        <v>22.32999992370605</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1211,13 +1235,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>494.0499877929688</v>
+        <v>486</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>49404.99877929688</v>
+        <v>48600</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-2093.481220703128</v>
+        <v>-2898.480000000003</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1258,6 +1282,9 @@
       <c r="T10" s="3" t="n">
         <v>494.0499877929688</v>
       </c>
+      <c r="U10" s="3" t="n">
+        <v>486</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1277,13 +1304,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>9.189999580383301</v>
+        <v>9.180000305175781</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>9189.999580383301</v>
+        <v>9180.000305175781</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-651.2104196166983</v>
+        <v>-661.2096948242179</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -1324,6 +1351,9 @@
       <c r="T11" s="3" t="n">
         <v>9.189999580383301</v>
       </c>
+      <c r="U11" s="3" t="n">
+        <v>9.180000305175781</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1343,13 +1373,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2599.89990234375</v>
+        <v>2569.89990234375</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25998.9990234375</v>
+        <v>25698.9990234375</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-1724.2509765625</v>
+        <v>-2024.2509765625</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -1390,6 +1420,9 @@
       <c r="T12" s="3" t="n">
         <v>2599.89990234375</v>
       </c>
+      <c r="U12" s="3" t="n">
+        <v>2569.89990234375</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1409,13 +1442,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>55.16999816894531</v>
+        <v>54.84999847412109</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>33101.99890136719</v>
+        <v>32909.99908447266</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-1929.761098632815</v>
+        <v>-2121.760915527346</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -1456,6 +1489,9 @@
       <c r="T13" s="3" t="n">
         <v>55.16999816894531</v>
       </c>
+      <c r="U13" s="3" t="n">
+        <v>54.84999847412109</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1475,13 +1511,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>790.25</v>
+        <v>781.25</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>39512.5</v>
+        <v>39062.5</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-2950.010000000002</v>
+        <v>-3400.010000000002</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -1522,6 +1558,9 @@
       <c r="T14" s="3" t="n">
         <v>790.25</v>
       </c>
+      <c r="U14" s="3" t="n">
+        <v>781.25</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1595,13 +1634,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>498.3999938964844</v>
+        <v>499</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>24919.99969482422</v>
+        <v>24950</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>3165.46969482422</v>
+        <v>3195.470000000001</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -1642,6 +1681,9 @@
       <c r="T17" s="3" t="n">
         <v>498.3999938964844</v>
       </c>
+      <c r="U17" s="3" t="n">
+        <v>499</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1661,13 +1703,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>424</v>
+        <v>428.1000061035156</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>42400</v>
+        <v>42810.00061035156</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-4240.82</v>
+        <v>-3830.819389648437</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -1708,6 +1750,9 @@
       <c r="T18" s="3" t="n">
         <v>424</v>
       </c>
+      <c r="U18" s="3" t="n">
+        <v>428.1000061035156</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -1719,10 +1764,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>564468.9925460815</v>
+        <v>568531.9986038208</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-26313.02745391847</v>
+        <v>-22250.02139617921</v>
       </c>
     </row>
   </sheetData>
@@ -1736,7 +1781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U41"/>
+  <dimension ref="A1:V41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1747,7 +1792,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
@@ -1760,6 +1805,7 @@
     <col width="13" customWidth="1" min="19" max="19"/>
     <col width="13" customWidth="1" min="20" max="20"/>
     <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1868,6 +1914,11 @@
           <t>2026-05-25</t>
         </is>
       </c>
+      <c r="V1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1892,16 +1943,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.8797</v>
+        <v>57.4032</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>63846.4394154</v>
+        <v>64434.0587424</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>13846.4394154</v>
+        <v>14434.0587424</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.2769287883079999</v>
+        <v>0.2886811748479999</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -1939,6 +1990,9 @@
       <c r="U2" s="3" t="n">
         <v>56.8797</v>
       </c>
+      <c r="V2" s="3" t="n">
+        <v>57.4032</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1963,16 +2017,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.7058</v>
+        <v>25.6218</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>63113.21433540001</v>
+        <v>62906.9764434</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>3113.214335400007</v>
+        <v>2906.976443400003</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.05188690559000012</v>
+        <v>0.04844960739000004</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -2010,6 +2064,9 @@
       <c r="U3" s="3" t="n">
         <v>25.7058</v>
       </c>
+      <c r="V3" s="3" t="n">
+        <v>25.6218</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2034,16 +2091,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.63</v>
+        <v>12.97</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>242572.95459</v>
+        <v>249103.02621</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>62572.95459000004</v>
+        <v>69103.02621000001</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3476275255000002</v>
+        <v>0.3839057011666667</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -2081,6 +2138,9 @@
       <c r="U4" s="3" t="n">
         <v>12.63</v>
       </c>
+      <c r="V4" s="3" t="n">
+        <v>12.97</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2105,16 +2165,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.544499999999999</v>
+        <v>9.581799999999999</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>175180.592916</v>
+        <v>175865.2003984</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-34819.40708400001</v>
+        <v>-34134.79960160001</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1658067004</v>
+        <v>-0.1625466647695239</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -2152,6 +2212,9 @@
       <c r="U5" s="3" t="n">
         <v>9.544499999999999</v>
       </c>
+      <c r="V5" s="3" t="n">
+        <v>9.581799999999999</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2176,16 +2239,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.4901</v>
+        <v>12.5608</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>52820.3456277</v>
+        <v>53119.3343016</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>2820.3456277</v>
+        <v>3119.3343016</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.05640691255400001</v>
+        <v>0.062386686032</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -2223,6 +2286,9 @@
       <c r="U6" s="3" t="n">
         <v>12.4901</v>
       </c>
+      <c r="V6" s="3" t="n">
+        <v>12.5608</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2247,16 +2313,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.9116</v>
+        <v>34.0865</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>74810.346064</v>
+        <v>75196.18246</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>14810.346064</v>
+        <v>15196.18246</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2468391010666666</v>
+        <v>0.2532697076666666</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -2294,6 +2360,9 @@
       <c r="U7" s="3" t="n">
         <v>33.9116</v>
       </c>
+      <c r="V7" s="3" t="n">
+        <v>34.0865</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2318,16 +2387,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>30.4549</v>
+        <v>31.1454</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>48867.7193557</v>
+        <v>49975.6908222</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>-1132.280644300001</v>
+        <v>-24.30917780000163</v>
       </c>
       <c r="I8" s="13" t="n">
-        <v>-0.02264561288600002</v>
+        <v>-0.0004861835560000327</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -2365,6 +2434,9 @@
       <c r="U8" s="3" t="n">
         <v>30.4549</v>
       </c>
+      <c r="V8" s="3" t="n">
+        <v>31.1454</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2389,16 +2461,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>41.9916</v>
+        <v>42.3446</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>135187.4630988</v>
+        <v>136323.9088278</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>35187.46309879998</v>
+        <v>36323.90882780001</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3518746309879999</v>
+        <v>0.3632390882780001</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -2436,6 +2508,9 @@
       <c r="U9" s="3" t="n">
         <v>41.9916</v>
       </c>
+      <c r="V9" s="3" t="n">
+        <v>42.3446</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2460,16 +2535,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>46.457</v>
+        <v>46.4459</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>132247.237163</v>
+        <v>132215.6392481</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>32247.23716300001</v>
+        <v>32215.63924810002</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3224723716300001</v>
+        <v>0.3221563924810002</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -2507,6 +2582,9 @@
       <c r="U10" s="3" t="n">
         <v>46.457</v>
       </c>
+      <c r="V10" s="3" t="n">
+        <v>46.4459</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2531,16 +2609,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>104.0761</v>
+        <v>105.3885</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31318.4759359</v>
+        <v>31713.4020315</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1318.475935899998</v>
+        <v>1713.402031499998</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.04394919786333327</v>
+        <v>0.05711340104999994</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -2578,6 +2656,9 @@
       <c r="U11" s="3" t="n">
         <v>104.0761</v>
       </c>
+      <c r="V11" s="3" t="n">
+        <v>105.3885</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2602,16 +2683,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>220.359</v>
+        <v>223.135</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>102581.962398</v>
+        <v>103874.25147</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>2581.962398000003</v>
+        <v>3874.251469999988</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.02581962398000003</v>
+        <v>0.03874251469999988</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -2649,6 +2730,9 @@
       <c r="U12" s="3" t="n">
         <v>220.359</v>
       </c>
+      <c r="V12" s="3" t="n">
+        <v>223.135</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2673,16 +2757,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>19.908</v>
+        <v>20.019</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>230686.04034</v>
+        <v>231972.264495</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>30686.04034000001</v>
+        <v>31972.26449499998</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.1534302017</v>
+        <v>0.1598613224749999</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -2720,6 +2804,9 @@
       <c r="U13" s="3" t="n">
         <v>19.908</v>
       </c>
+      <c r="V13" s="3" t="n">
+        <v>20.019</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2744,16 +2831,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>38.499</v>
+        <v>39.1893</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>138889.223394</v>
+        <v>141379.5538158</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>38889.22339400003</v>
+        <v>41379.55381580003</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.3888922339400003</v>
+        <v>0.4137955381580003</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -2791,6 +2878,9 @@
       <c r="U14" s="3" t="n">
         <v>38.499</v>
       </c>
+      <c r="V14" s="3" t="n">
+        <v>39.1893</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2815,16 +2905,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.81</v>
+        <v>11.92</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>115076.01407</v>
+        <v>116147.84824</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>15076.01407</v>
+        <v>16147.84824000001</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1507601407</v>
+        <v>0.1614784824000001</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -2862,6 +2952,9 @@
       <c r="U15" s="3" t="n">
         <v>11.81</v>
       </c>
+      <c r="V15" s="3" t="n">
+        <v>11.92</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2886,16 +2979,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.6238</v>
+        <v>24.9215</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>140920.2344864</v>
+        <v>142623.950152</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>40920.2344864</v>
+        <v>42623.950152</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.409202344864</v>
+        <v>0.4262395015200001</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -2933,6 +3026,9 @@
       <c r="U16" s="3" t="n">
         <v>24.6238</v>
       </c>
+      <c r="V16" s="3" t="n">
+        <v>24.9215</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2957,16 +3053,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.7</v>
+        <v>16.7872</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55211.1519</v>
+        <v>55499.44007039999</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5211.151899999997</v>
+        <v>5499.440070399993</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1042230379999999</v>
+        <v>0.1099888014079999</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -3004,6 +3100,9 @@
       <c r="U17" s="3" t="n">
         <v>16.7</v>
       </c>
+      <c r="V17" s="3" t="n">
+        <v>16.7872</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3028,16 +3127,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>45.34</v>
+        <v>45.62</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>85531.00824000001</v>
+        <v>86059.21032</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>5531.00824000001</v>
+        <v>6059.210319999998</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.06913760300000013</v>
+        <v>0.07574012899999998</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -3075,6 +3174,9 @@
       <c r="U18" s="3" t="n">
         <v>45.34</v>
       </c>
+      <c r="V18" s="3" t="n">
+        <v>45.62</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3099,16 +3201,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>14.5354</v>
+        <v>14.8215</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>210280.2305164</v>
+        <v>214419.172269</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>60280.23051639998</v>
+        <v>64419.172269</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.4018682034426665</v>
+        <v>0.42946114846</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -3146,6 +3248,9 @@
       <c r="U19" s="3" t="n">
         <v>14.5354</v>
       </c>
+      <c r="V19" s="3" t="n">
+        <v>14.8215</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3170,16 +3275,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.359999999999999</v>
+        <v>9.48</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>245754.31608</v>
+        <v>248905.01244</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-4245.68392000001</v>
+        <v>-1094.98755999998</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.01698273568000004</v>
+        <v>-0.004379950239999918</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -3217,6 +3322,9 @@
       <c r="U20" s="3" t="n">
         <v>9.359999999999999</v>
       </c>
+      <c r="V20" s="3" t="n">
+        <v>9.48</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3241,16 +3349,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>107.6678</v>
+        <v>108.874</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>163575.2741602</v>
+        <v>165407.804366</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-6424.725839799998</v>
+        <v>-4592.195634000003</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.03779250493999999</v>
+        <v>-0.02701291549411767</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -3288,6 +3396,9 @@
       <c r="U21" s="3" t="n">
         <v>107.6678</v>
       </c>
+      <c r="V21" s="3" t="n">
+        <v>108.874</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3312,16 +3423,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>43.467</v>
+        <v>44.368</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>66698.37282</v>
+        <v>68080.92128000001</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>6698.372820000004</v>
+        <v>8080.92128000001</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1116395470000001</v>
+        <v>0.1346820213333335</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -3359,6 +3470,9 @@
       <c r="U22" s="3" t="n">
         <v>43.467</v>
       </c>
+      <c r="V22" s="3" t="n">
+        <v>44.368</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3383,16 +3497,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>60.8801</v>
+        <v>62.1049</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>165378.7826067</v>
+        <v>168705.9113883</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>15378.7826067</v>
+        <v>18705.91138830001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.102525217378</v>
+        <v>0.1247060759220001</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -3430,6 +3544,9 @@
       <c r="U23" s="3" t="n">
         <v>60.8801</v>
       </c>
+      <c r="V23" s="3" t="n">
+        <v>62.1049</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3454,16 +3571,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>28.1533</v>
+        <v>28.7044</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>102291.8060738</v>
+        <v>104294.1650984</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>2291.806073800006</v>
+        <v>4294.165098400001</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.02291806073800006</v>
+        <v>0.042941650984</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -3501,6 +3618,9 @@
       <c r="U24" s="3" t="n">
         <v>28.1533</v>
       </c>
+      <c r="V24" s="3" t="n">
+        <v>28.7044</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3525,16 +3645,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.3115</v>
+        <v>11.4442</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>185753.765451</v>
+        <v>187932.9215908</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-14246.23454900002</v>
+        <v>-12067.07840920001</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.07123117274500007</v>
+        <v>-0.06033539204600005</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -3572,6 +3692,9 @@
       <c r="U25" s="3" t="n">
         <v>11.3115</v>
       </c>
+      <c r="V25" s="3" t="n">
+        <v>11.4442</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3596,16 +3719,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>8.871499999999999</v>
+        <v>8.964</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>105940.9246225</v>
+        <v>107045.53326</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>-4059.075377500005</v>
+        <v>-2954.466739999989</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>-0.03690068525000004</v>
+        <v>-0.02685878854545444</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -3643,6 +3766,9 @@
       <c r="U26" s="3" t="n">
         <v>8.871499999999999</v>
       </c>
+      <c r="V26" s="3" t="n">
+        <v>8.964</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3667,16 +3793,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>62.4143</v>
+        <v>63.424</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>100540.699298</v>
+        <v>102167.18464</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-9459.300702000008</v>
+        <v>-7832.815360000008</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.08599364274545461</v>
+        <v>-0.07120741236363644</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -3714,6 +3840,9 @@
       <c r="U27" s="3" t="n">
         <v>62.4143</v>
       </c>
+      <c r="V27" s="3" t="n">
+        <v>63.424</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3738,16 +3867,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>105.9949</v>
+        <v>107.5413</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>350488.7780493</v>
+        <v>355602.1924341</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-29511.22195069998</v>
+        <v>-24397.80756589997</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.0776611103965789</v>
+        <v>-0.06420475675236835</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -3785,6 +3914,9 @@
       <c r="U28" s="3" t="n">
         <v>105.9949</v>
       </c>
+      <c r="V28" s="3" t="n">
+        <v>107.5413</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3809,16 +3941,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.9289</v>
+        <v>12.1179</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>114561.6127167</v>
+        <v>116376.7125837</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>14561.61271669999</v>
+        <v>16376.71258370001</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.145616127167</v>
+        <v>0.1637671258370001</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -3856,6 +3988,9 @@
       <c r="U29" s="3" t="n">
         <v>11.9289</v>
       </c>
+      <c r="V29" s="3" t="n">
+        <v>12.1179</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3880,16 +4015,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>15.0804</v>
+        <v>15.2965</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>111532.5422244</v>
+        <v>113130.7877865</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>11532.54222439999</v>
+        <v>13130.7877865</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.1153254222439999</v>
+        <v>0.131307877865</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -3927,6 +4062,9 @@
       <c r="U30" s="3" t="n">
         <v>15.0804</v>
       </c>
+      <c r="V30" s="3" t="n">
+        <v>15.2965</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3951,16 +4089,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>414.0702</v>
+        <v>417.3064</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>110175.798816</v>
+        <v>111036.886912</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>10175.79881599999</v>
+        <v>11036.88691199999</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.10175798816</v>
+        <v>0.1103688691199999</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -3998,6 +4136,9 @@
       <c r="U31" s="3" t="n">
         <v>414.0702</v>
       </c>
+      <c r="V31" s="3" t="n">
+        <v>417.3064</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4022,16 +4163,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.16</v>
+        <v>10.25</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>214781.9936</v>
+        <v>216684.59</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>14781.99359999999</v>
+        <v>16684.59</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.07390996799999994</v>
+        <v>0.08342294999999998</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -4069,6 +4210,9 @@
       <c r="U32" s="3" t="n">
         <v>10.16</v>
       </c>
+      <c r="V32" s="3" t="n">
+        <v>10.25</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4093,16 +4237,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>17.85</v>
+        <v>18.07</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>63967.974</v>
+        <v>64756.3748</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>3967.974000000002</v>
+        <v>4756.374799999998</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.06613290000000004</v>
+        <v>0.07927291333333329</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -4140,6 +4284,9 @@
       <c r="U33" s="3" t="n">
         <v>17.85</v>
       </c>
+      <c r="V33" s="3" t="n">
+        <v>18.07</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4164,16 +4311,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>213.5032</v>
+        <v>214.9833</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>75052.9933992</v>
+        <v>75573.29443230001</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-4947.006600799999</v>
+        <v>-4426.705567699988</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.06183758251</v>
+        <v>-0.05533381959624985</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -4211,6 +4358,9 @@
       <c r="U34" s="3" t="n">
         <v>213.5032</v>
       </c>
+      <c r="V34" s="3" t="n">
+        <v>214.9833</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4235,16 +4385,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>14.17</v>
+        <v>14.41</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>101108.94391</v>
+        <v>102821.44543</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>1108.943910000002</v>
+        <v>2821.445429999992</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.01108943910000002</v>
+        <v>0.02821445429999992</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -4282,6 +4432,9 @@
       <c r="U35" s="3" t="n">
         <v>14.17</v>
       </c>
+      <c r="V35" s="3" t="n">
+        <v>14.41</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4306,16 +4459,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>350.9864</v>
+        <v>352.9091</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>163456.4723984</v>
+        <v>164351.8853246</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>13456.47239840002</v>
+        <v>14351.88532460001</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.08970981598933343</v>
+        <v>0.09567923549733338</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -4353,6 +4506,9 @@
       <c r="U36" s="3" t="n">
         <v>350.9864</v>
       </c>
+      <c r="V36" s="3" t="n">
+        <v>352.9091</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4377,16 +4533,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>15.648</v>
+        <v>15.7</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>58881.687072</v>
+        <v>59077.3573</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>8881.687072000001</v>
+        <v>9077.357299999996</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.17763374144</v>
+        <v>0.1815471459999999</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -4424,6 +4580,9 @@
       <c r="U37" s="3" t="n">
         <v>15.648</v>
       </c>
+      <c r="V37" s="3" t="n">
+        <v>15.7</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4448,16 +4607,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>14.0547</v>
+        <v>14.2181</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>84053.88036540001</v>
+        <v>85031.0911242</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>4053.880365400008</v>
+        <v>5031.0911242</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.0506735045675001</v>
+        <v>0.0628886390525</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -4495,6 +4654,9 @@
       <c r="U38" s="3" t="n">
         <v>14.0547</v>
       </c>
+      <c r="V38" s="3" t="n">
+        <v>14.2181</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4519,16 +4681,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1005.0898</v>
+        <v>1007.8869</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50134.8843138</v>
+        <v>50274.4064589</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>134.8843138000011</v>
+        <v>274.4064588999972</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.002697686276000022</v>
+        <v>0.005488129177999945</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -4566,6 +4728,9 @@
       <c r="U39" s="3" t="n">
         <v>1005.0898</v>
       </c>
+      <c r="V39" s="3" t="n">
+        <v>1007.8869</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4590,16 +4755,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>20.0352</v>
+        <v>20.4955</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>100997.9841504</v>
+        <v>103318.3688785</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>997.9841503999924</v>
+        <v>3318.368878499998</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.009979841503999923</v>
+        <v>0.03318368878499998</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -4637,6 +4802,9 @@
       <c r="U40" s="3" t="n">
         <v>20.0352</v>
       </c>
+      <c r="V40" s="3" t="n">
+        <v>20.4955</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
@@ -4648,13 +4816,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4834270.1399745</v>
+        <v>4893403.9578459</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>364270.1399745001</v>
+        <v>423403.9578459001</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.0814922013365772</v>
+        <v>0.09472124336597318</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-05-28
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-05-27 06:19 IST</t>
+          <t>Generated: 2026-05-28 06:10 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4893403.9578459</v>
+        <v>4908559.2093685</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>423403.9578459002</v>
+        <v>438559.2093684999</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.09472124336597321</v>
+        <v>0.09811167994821028</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>568531.9986038208</v>
+        <v>571530.9985427856</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-22250.02139617922</v>
+        <v>-19251.02145721437</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.03766198131110899</v>
+        <v>-0.03258565901720295</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5461935.956449721</v>
+        <v>5480090.207911286</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>401153.9364497215</v>
+        <v>419308.187911286</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.07926718338477687</v>
+        <v>0.08285442571013681</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-05-27</t>
+          <t>Last snapshot: 2026-05-28</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U19"/>
+  <dimension ref="A1:V19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -640,6 +640,7 @@
     <col width="21" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="21" customWidth="1" min="21" max="21"/>
+    <col width="21" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -748,6 +749,11 @@
           <t>2026-05-27</t>
         </is>
       </c>
+      <c r="V1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -767,13 +773,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>581.0999755859375</v>
+        <v>583</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>46487.998046875</v>
+        <v>46640</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>2670.488046874998</v>
+        <v>2822.489999999998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -817,6 +823,9 @@
       <c r="U2" s="3" t="n">
         <v>581.0999755859375</v>
       </c>
+      <c r="V2" s="3" t="n">
+        <v>583</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -863,13 +872,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1583.300048828125</v>
+        <v>1602</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>31666.0009765625</v>
+        <v>32040</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-438.5790234375017</v>
+        <v>-64.58000000000175</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -913,6 +922,9 @@
       <c r="U4" s="3" t="n">
         <v>1583.300048828125</v>
       </c>
+      <c r="V4" s="3" t="n">
+        <v>1602</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -932,13 +944,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>635.6500244140625</v>
+        <v>640</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>12713.00048828125</v>
+        <v>12800</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1500.09951171875</v>
+        <v>-1413.1</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -982,6 +994,9 @@
       <c r="U5" s="3" t="n">
         <v>635.6500244140625</v>
       </c>
+      <c r="V5" s="3" t="n">
+        <v>640</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1001,13 +1016,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>395.4500122070312</v>
+        <v>393.2000122070312</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15818.00048828125</v>
+        <v>15728.00048828125</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-1684.239511718752</v>
+        <v>-1774.239511718752</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1051,6 +1066,9 @@
       <c r="U6" s="3" t="n">
         <v>395.4500122070312</v>
       </c>
+      <c r="V6" s="3" t="n">
+        <v>393.2000122070312</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1070,13 +1088,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>233.6999969482422</v>
+        <v>235</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>23369.99969482422</v>
+        <v>23500</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-3063.820305175781</v>
+        <v>-2933.82</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1120,6 +1138,9 @@
       <c r="U7" s="3" t="n">
         <v>233.6999969482422</v>
       </c>
+      <c r="V7" s="3" t="n">
+        <v>235</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1166,13 +1187,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>22.32999992370605</v>
+        <v>22.95000076293945</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>33494.99988555908</v>
+        <v>34425.00114440918</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>2444.829885559084</v>
+        <v>3374.831144409181</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1216,6 +1237,9 @@
       <c r="U9" s="3" t="n">
         <v>22.32999992370605</v>
       </c>
+      <c r="V9" s="3" t="n">
+        <v>22.95000076293945</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1235,13 +1259,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>486</v>
+        <v>488.0499877929688</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48600</v>
+        <v>48804.99877929688</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-2898.480000000003</v>
+        <v>-2693.481220703128</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1285,6 +1309,9 @@
       <c r="U10" s="3" t="n">
         <v>486</v>
       </c>
+      <c r="V10" s="3" t="n">
+        <v>488.0499877929688</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1304,13 +1331,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>9.180000305175781</v>
+        <v>9.220000267028809</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>9180.000305175781</v>
+        <v>9220.000267028809</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-661.2096948242179</v>
+        <v>-621.2097329711905</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -1354,6 +1381,9 @@
       <c r="U11" s="3" t="n">
         <v>9.180000305175781</v>
       </c>
+      <c r="V11" s="3" t="n">
+        <v>9.220000267028809</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1373,13 +1403,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2569.89990234375</v>
+        <v>2575</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25698.9990234375</v>
+        <v>25750</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2024.2509765625</v>
+        <v>-1973.25</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -1423,6 +1453,9 @@
       <c r="U12" s="3" t="n">
         <v>2569.89990234375</v>
       </c>
+      <c r="V12" s="3" t="n">
+        <v>2575</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1442,13 +1475,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>54.84999847412109</v>
+        <v>57.75</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>32909.99908447266</v>
+        <v>34650</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-2121.760915527346</v>
+        <v>-381.760000000002</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -1492,6 +1525,9 @@
       <c r="U13" s="3" t="n">
         <v>54.84999847412109</v>
       </c>
+      <c r="V13" s="3" t="n">
+        <v>57.75</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1511,13 +1547,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>781.25</v>
+        <v>775.3499755859375</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>39062.5</v>
+        <v>38767.49877929688</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-3400.010000000002</v>
+        <v>-3695.011220703127</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -1561,6 +1597,9 @@
       <c r="U14" s="3" t="n">
         <v>781.25</v>
       </c>
+      <c r="V14" s="3" t="n">
+        <v>775.3499755859375</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1634,13 +1673,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>499</v>
+        <v>492.8999938964844</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>24950</v>
+        <v>24644.99969482422</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>3195.470000000001</v>
+        <v>2890.46969482422</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -1684,6 +1723,9 @@
       <c r="U17" s="3" t="n">
         <v>499</v>
       </c>
+      <c r="V17" s="3" t="n">
+        <v>492.8999938964844</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1703,13 +1745,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>428.1000061035156</v>
+        <v>427.8999938964844</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>42810.00061035156</v>
+        <v>42789.99938964844</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-3830.819389648437</v>
+        <v>-3850.820610351562</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -1753,6 +1795,9 @@
       <c r="U18" s="3" t="n">
         <v>428.1000061035156</v>
       </c>
+      <c r="V18" s="3" t="n">
+        <v>427.8999938964844</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -1764,10 +1809,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>568531.9986038208</v>
+        <v>571530.9985427856</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-22250.02139617921</v>
+        <v>-19251.02145721437</v>
       </c>
     </row>
   </sheetData>
@@ -1781,7 +1826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V41"/>
+  <dimension ref="A1:W41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1792,7 +1837,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
@@ -1806,6 +1851,7 @@
     <col width="13" customWidth="1" min="20" max="20"/>
     <col width="13" customWidth="1" min="21" max="21"/>
     <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="13" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1919,6 +1965,11 @@
           <t>2026-05-27</t>
         </is>
       </c>
+      <c r="W1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1943,16 +1994,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>57.4032</v>
+        <v>57.2415</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>64434.0587424</v>
+        <v>64252.553403</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>14434.0587424</v>
+        <v>14252.553403</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.2886811748479999</v>
+        <v>0.28505106806</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -1993,6 +2044,9 @@
       <c r="V2" s="3" t="n">
         <v>57.4032</v>
       </c>
+      <c r="W2" s="3" t="n">
+        <v>57.2415</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2067,6 +2121,9 @@
       <c r="V3" s="3" t="n">
         <v>25.6218</v>
       </c>
+      <c r="W3" s="3" t="n">
+        <v>25.6218</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2141,6 +2198,9 @@
       <c r="V4" s="3" t="n">
         <v>12.97</v>
       </c>
+      <c r="W4" s="3" t="n">
+        <v>12.97</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2165,16 +2225,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.581799999999999</v>
+        <v>9.6485</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>175865.2003984</v>
+        <v>177089.418068</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-34134.79960160001</v>
+        <v>-32910.581932</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1625466647695239</v>
+        <v>-0.1567170568190476</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -2215,6 +2275,9 @@
       <c r="V5" s="3" t="n">
         <v>9.581799999999999</v>
       </c>
+      <c r="W5" s="3" t="n">
+        <v>9.6485</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2239,16 +2302,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.5608</v>
+        <v>12.7525</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>53119.3343016</v>
+        <v>53930.0291925</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>3119.3343016</v>
+        <v>3930.029192499998</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.062386686032</v>
+        <v>0.07860058384999996</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -2289,6 +2352,9 @@
       <c r="V6" s="3" t="n">
         <v>12.5608</v>
       </c>
+      <c r="W6" s="3" t="n">
+        <v>12.7525</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2313,16 +2379,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>34.0865</v>
+        <v>34.1536</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>75196.18246</v>
+        <v>75344.207744</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>15196.18246</v>
+        <v>15344.207744</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2532697076666666</v>
+        <v>0.2557367957333333</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -2363,6 +2429,9 @@
       <c r="V7" s="3" t="n">
         <v>34.0865</v>
       </c>
+      <c r="W7" s="3" t="n">
+        <v>34.1536</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2387,16 +2456,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>31.1454</v>
+        <v>31.2273</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>49975.6908222</v>
-      </c>
-      <c r="H8" s="6" t="n">
-        <v>-24.30917780000163</v>
-      </c>
-      <c r="I8" s="13" t="n">
-        <v>-0.0004861835560000327</v>
+        <v>50107.1069889</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>107.1069888999991</v>
+      </c>
+      <c r="I8" s="12" t="n">
+        <v>0.002142139777999983</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -2437,6 +2506,9 @@
       <c r="V8" s="3" t="n">
         <v>31.1454</v>
       </c>
+      <c r="W8" s="3" t="n">
+        <v>31.2273</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2461,16 +2533,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>42.3446</v>
+        <v>42.3147</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>136323.9088278</v>
+        <v>136227.6489771</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>36323.90882780001</v>
+        <v>36227.64897710001</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3632390882780001</v>
+        <v>0.3622764897710001</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -2511,6 +2583,9 @@
       <c r="V9" s="3" t="n">
         <v>42.3446</v>
       </c>
+      <c r="W9" s="3" t="n">
+        <v>42.3147</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2535,16 +2610,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>46.4459</v>
+        <v>46.5909</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>132215.6392481</v>
+        <v>132628.4048031</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>32215.63924810002</v>
+        <v>32628.40480310001</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3221563924810002</v>
+        <v>0.3262840480310001</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -2585,6 +2660,9 @@
       <c r="V10" s="3" t="n">
         <v>46.4459</v>
       </c>
+      <c r="W10" s="3" t="n">
+        <v>46.5909</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2609,16 +2687,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>105.3885</v>
+        <v>105.5999</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31713.4020315</v>
+        <v>31777.0163081</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1713.402031499998</v>
+        <v>1777.016308099999</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.05711340104999994</v>
+        <v>0.05923387693666664</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -2659,6 +2737,9 @@
       <c r="V11" s="3" t="n">
         <v>105.3885</v>
       </c>
+      <c r="W11" s="3" t="n">
+        <v>105.5999</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2683,16 +2764,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>223.135</v>
+        <v>223.585</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>103874.25147</v>
+        <v>104083.73637</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>3874.251469999988</v>
+        <v>4083.736369999999</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.03874251469999988</v>
+        <v>0.04083736369999999</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -2733,6 +2814,9 @@
       <c r="V12" s="3" t="n">
         <v>223.135</v>
       </c>
+      <c r="W12" s="3" t="n">
+        <v>223.585</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2757,16 +2841,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>20.019</v>
+        <v>20.01</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>231972.264495</v>
+        <v>231867.97605</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>31972.26449499998</v>
+        <v>31867.97605</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.1598613224749999</v>
+        <v>0.15933988025</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -2807,6 +2891,9 @@
       <c r="V13" s="3" t="n">
         <v>20.019</v>
       </c>
+      <c r="W13" s="3" t="n">
+        <v>20.01</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2831,16 +2918,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>39.1893</v>
+        <v>39.8818</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>141379.5538158</v>
+        <v>143877.8209708</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>41379.55381580003</v>
+        <v>43877.82097080001</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.4137955381580003</v>
+        <v>0.4387782097080001</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -2881,6 +2968,9 @@
       <c r="V14" s="3" t="n">
         <v>39.1893</v>
       </c>
+      <c r="W14" s="3" t="n">
+        <v>39.8818</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2905,16 +2995,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.92</v>
+        <v>12.01</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>116147.84824</v>
+        <v>117024.80347</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>16147.84824000001</v>
+        <v>17024.80347</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1614784824000001</v>
+        <v>0.1702480347</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -2955,6 +3045,9 @@
       <c r="V15" s="3" t="n">
         <v>11.92</v>
       </c>
+      <c r="W15" s="3" t="n">
+        <v>12.01</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2979,16 +3072,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.9215</v>
+        <v>24.988</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>142623.950152</v>
+        <v>143004.524864</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>42623.950152</v>
+        <v>43004.52486400001</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4262395015200001</v>
+        <v>0.43004524864</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -3029,6 +3122,9 @@
       <c r="V16" s="3" t="n">
         <v>24.9215</v>
       </c>
+      <c r="W16" s="3" t="n">
+        <v>24.988</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3053,16 +3149,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.7872</v>
+        <v>16.7965</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55499.44007039999</v>
+        <v>55530.1864005</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5499.440070399993</v>
+        <v>5530.186400500002</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1099888014079999</v>
+        <v>0.1106037280100001</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -3103,6 +3199,9 @@
       <c r="V17" s="3" t="n">
         <v>16.7872</v>
       </c>
+      <c r="W17" s="3" t="n">
+        <v>16.7965</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3127,16 +3226,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>45.62</v>
+        <v>45.5</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>86059.21032</v>
+        <v>85832.838</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>6059.210319999998</v>
+        <v>5832.838000000003</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.07574012899999998</v>
+        <v>0.07291047500000004</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -3177,6 +3276,9 @@
       <c r="V18" s="3" t="n">
         <v>45.62</v>
       </c>
+      <c r="W18" s="3" t="n">
+        <v>45.5</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3251,6 +3353,9 @@
       <c r="V19" s="3" t="n">
         <v>14.8215</v>
       </c>
+      <c r="W19" s="3" t="n">
+        <v>14.8215</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3275,16 +3380,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.48</v>
+        <v>9.449999999999999</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>248905.01244</v>
+        <v>248117.33835</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-1094.98755999998</v>
+        <v>-1882.661650000024</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.004379950239999918</v>
+        <v>-0.007530646600000095</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -3325,6 +3430,9 @@
       <c r="V20" s="3" t="n">
         <v>9.48</v>
       </c>
+      <c r="W20" s="3" t="n">
+        <v>9.449999999999999</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3349,16 +3457,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>108.874</v>
+        <v>109.0748</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>165407.804366</v>
+        <v>165712.8715732</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-4592.195634000003</v>
+        <v>-4287.128426800016</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.02701291549411767</v>
+        <v>-0.02521840251058833</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -3399,6 +3507,9 @@
       <c r="V21" s="3" t="n">
         <v>108.874</v>
       </c>
+      <c r="W21" s="3" t="n">
+        <v>109.0748</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3423,16 +3534,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>44.368</v>
+        <v>45.137</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>68080.92128000001</v>
+        <v>69260.92102000001</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>8080.92128000001</v>
+        <v>9260.921020000009</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1346820213333335</v>
+        <v>0.1543486836666668</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -3473,6 +3584,9 @@
       <c r="V22" s="3" t="n">
         <v>44.368</v>
       </c>
+      <c r="W22" s="3" t="n">
+        <v>45.137</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3497,16 +3611,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>62.1049</v>
+        <v>62.8006</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>168705.9113883</v>
+        <v>170595.7574802</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>18705.91138830001</v>
+        <v>20595.7574802</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.1247060759220001</v>
+        <v>0.137305049868</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -3547,6 +3661,9 @@
       <c r="V23" s="3" t="n">
         <v>62.1049</v>
       </c>
+      <c r="W23" s="3" t="n">
+        <v>62.8006</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3571,16 +3688,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>28.7044</v>
+        <v>28.9116</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>104294.1650984</v>
+        <v>105047.0026776</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>4294.165098400001</v>
+        <v>5047.002677600001</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.042941650984</v>
+        <v>0.05047002677600002</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -3621,6 +3738,9 @@
       <c r="V24" s="3" t="n">
         <v>28.7044</v>
       </c>
+      <c r="W24" s="3" t="n">
+        <v>28.9116</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3645,16 +3765,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.4442</v>
+        <v>11.4752</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>187932.9215908</v>
+        <v>188441.9934848</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-12067.07840920001</v>
+        <v>-11558.00651520002</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.06033539204600005</v>
+        <v>-0.05779003257600009</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -3695,6 +3815,9 @@
       <c r="V25" s="3" t="n">
         <v>11.4442</v>
       </c>
+      <c r="W25" s="3" t="n">
+        <v>11.4752</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3719,16 +3842,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>8.964</v>
+        <v>8.990399999999999</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>107045.53326</v>
+        <v>107360.794536</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>-2954.466739999989</v>
+        <v>-2639.205464000013</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>-0.02685878854545444</v>
+        <v>-0.02399277694545467</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -3769,6 +3892,9 @@
       <c r="V26" s="3" t="n">
         <v>8.964</v>
       </c>
+      <c r="W26" s="3" t="n">
+        <v>8.990399999999999</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3793,16 +3919,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>63.424</v>
+        <v>64.0264</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>102167.18464</v>
+        <v>103137.566704</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-7832.815360000008</v>
+        <v>-6862.433296000017</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.07120741236363644</v>
+        <v>-0.0623857572363638</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -3843,6 +3969,9 @@
       <c r="V27" s="3" t="n">
         <v>63.424</v>
       </c>
+      <c r="W27" s="3" t="n">
+        <v>64.0264</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3867,16 +3996,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>107.5413</v>
+        <v>107.5591</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>355602.1924341</v>
+        <v>355661.0509287</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-24397.80756589997</v>
+        <v>-24338.94907129998</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.06420475675236835</v>
+        <v>-0.06404986597710521</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -3917,6 +4046,9 @@
       <c r="V28" s="3" t="n">
         <v>107.5413</v>
       </c>
+      <c r="W28" s="3" t="n">
+        <v>107.5591</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3941,16 +4073,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.1179</v>
+        <v>12.13</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>116376.7125837</v>
+        <v>116492.91739</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>16376.71258370001</v>
+        <v>16492.91739</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.1637671258370001</v>
+        <v>0.1649291739</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -3991,6 +4123,9 @@
       <c r="V29" s="3" t="n">
         <v>12.1179</v>
       </c>
+      <c r="W29" s="3" t="n">
+        <v>12.13</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4015,16 +4150,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>15.2965</v>
+        <v>15.3581</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>113130.7877865</v>
+        <v>113586.3728241</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>13130.7877865</v>
+        <v>13586.37282410001</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.131307877865</v>
+        <v>0.1358637282410001</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -4065,6 +4200,9 @@
       <c r="V30" s="3" t="n">
         <v>15.2965</v>
       </c>
+      <c r="W30" s="3" t="n">
+        <v>15.3581</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4089,16 +4227,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>417.3064</v>
+        <v>422.49</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>111036.886912</v>
+        <v>112416.1392</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>11036.88691199999</v>
+        <v>12416.13919999999</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.1103688691199999</v>
+        <v>0.1241613919999999</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -4139,6 +4277,9 @@
       <c r="V31" s="3" t="n">
         <v>417.3064</v>
       </c>
+      <c r="W31" s="3" t="n">
+        <v>422.49</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4163,16 +4304,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.25</v>
+        <v>10.28</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>216684.59</v>
+        <v>217318.7888</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>16684.59</v>
+        <v>17318.78879999998</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.08342294999999998</v>
+        <v>0.0865939439999999</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -4213,6 +4354,9 @@
       <c r="V32" s="3" t="n">
         <v>10.25</v>
       </c>
+      <c r="W32" s="3" t="n">
+        <v>10.28</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4237,16 +4381,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>18.07</v>
+        <v>18.08</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>64756.3748</v>
+        <v>64792.21119999999</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>4756.374799999998</v>
+        <v>4792.211199999991</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.07927291333333329</v>
+        <v>0.07987018666666651</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -4287,6 +4431,9 @@
       <c r="V33" s="3" t="n">
         <v>18.07</v>
       </c>
+      <c r="W33" s="3" t="n">
+        <v>18.08</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4311,16 +4458,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>214.9833</v>
+        <v>215.054</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>75573.29443230001</v>
+        <v>75598.14767400001</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-4426.705567699988</v>
+        <v>-4401.852325999993</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.05533381959624985</v>
+        <v>-0.05502315407499991</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -4361,6 +4508,9 @@
       <c r="V34" s="3" t="n">
         <v>214.9833</v>
       </c>
+      <c r="W34" s="3" t="n">
+        <v>215.054</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4385,16 +4535,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>14.41</v>
+        <v>14.55</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>102821.44543</v>
+        <v>103820.40465</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>2821.445429999992</v>
+        <v>3820.404649999997</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.02821445429999992</v>
+        <v>0.03820404649999997</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -4435,6 +4585,9 @@
       <c r="V35" s="3" t="n">
         <v>14.41</v>
       </c>
+      <c r="W35" s="3" t="n">
+        <v>14.55</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4459,16 +4612,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>352.9091</v>
+        <v>352.3059</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>164351.8853246</v>
+        <v>164070.9714654</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>14351.88532460001</v>
+        <v>14070.97146540001</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.09567923549733338</v>
+        <v>0.09380647643600008</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -4509,6 +4662,9 @@
       <c r="V36" s="3" t="n">
         <v>352.9091</v>
       </c>
+      <c r="W36" s="3" t="n">
+        <v>352.3059</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4533,16 +4689,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>15.7</v>
+        <v>15.682</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>59077.3573</v>
+        <v>59009.62529800001</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>9077.357299999996</v>
+        <v>9009.625298000006</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.1815471459999999</v>
+        <v>0.1801925059600001</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -4583,6 +4739,9 @@
       <c r="V37" s="3" t="n">
         <v>15.7</v>
       </c>
+      <c r="W37" s="3" t="n">
+        <v>15.682</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4607,16 +4766,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>14.2181</v>
+        <v>14.2639</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>85031.0911242</v>
+        <v>85304.9971998</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>5031.0911242</v>
+        <v>5304.997199799996</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.0628886390525</v>
+        <v>0.06631246499749996</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -4657,6 +4816,9 @@
       <c r="V38" s="3" t="n">
         <v>14.2181</v>
       </c>
+      <c r="W38" s="3" t="n">
+        <v>14.2639</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4681,16 +4843,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1007.8869</v>
+        <v>1008.2382</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50274.4064589</v>
+        <v>50291.9296542</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>274.4064588999972</v>
+        <v>291.9296542000011</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.005488129177999945</v>
+        <v>0.005838593084000022</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -4731,6 +4893,9 @@
       <c r="V39" s="3" t="n">
         <v>1007.8869</v>
       </c>
+      <c r="W39" s="3" t="n">
+        <v>1008.2382</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4755,16 +4920,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>20.4955</v>
+        <v>20.5343</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>103318.3688785</v>
+        <v>103513.9607261</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>3318.368878499998</v>
+        <v>3513.960726100006</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.03318368878499998</v>
+        <v>0.03513960726100006</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -4805,6 +4970,9 @@
       <c r="V40" s="3" t="n">
         <v>20.4955</v>
       </c>
+      <c r="W40" s="3" t="n">
+        <v>20.5343</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
@@ -4816,13 +4984,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4893403.9578459</v>
+        <v>4908559.2093685</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>423403.9578459001</v>
+        <v>438559.2093685</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.09472124336597318</v>
+        <v>0.09811167994821028</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-05-29
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -484,7 +484,7 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-05-28 06:10 IST</t>
+          <t>Generated: 2026-05-29 06:12 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4908559.2093685</v>
+        <v>4912053.5620727</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>438559.2093684999</v>
+        <v>442053.5620726999</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.09811167994821028</v>
+        <v>0.09889341433393734</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>571530.9985427856</v>
+        <v>571344.003112793</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-19251.02145721437</v>
+        <v>-19438.01688720705</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.03258565901720295</v>
+        <v>-0.03290218088764287</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5480090.207911286</v>
+        <v>5483397.565185493</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>419308.187911286</v>
+        <v>422615.5451854933</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.08285442571013681</v>
+        <v>0.08350795262774297</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-05-28</t>
+          <t>Last snapshot: 2026-05-29</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V19"/>
+  <dimension ref="A1:W19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -641,6 +641,7 @@
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="21" customWidth="1" min="21" max="21"/>
     <col width="21" customWidth="1" min="22" max="22"/>
+    <col width="21" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -754,6 +755,11 @@
           <t>2026-05-28</t>
         </is>
       </c>
+      <c r="W1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -773,13 +779,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>583</v>
+        <v>590.9000244140625</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>46640</v>
+        <v>47272.001953125</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>2822.489999999998</v>
+        <v>3454.491953124998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -826,6 +832,9 @@
       <c r="V2" s="3" t="n">
         <v>583</v>
       </c>
+      <c r="W2" s="3" t="n">
+        <v>590.9000244140625</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -872,13 +881,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1602</v>
+        <v>1593.199951171875</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>32040</v>
+        <v>31863.9990234375</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-64.58000000000175</v>
+        <v>-240.5809765625017</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -925,6 +934,9 @@
       <c r="V4" s="3" t="n">
         <v>1602</v>
       </c>
+      <c r="W4" s="3" t="n">
+        <v>1593.199951171875</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -944,13 +956,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>640</v>
+        <v>650.0999755859375</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>12800</v>
+        <v>13001.99951171875</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1413.1</v>
+        <v>-1211.10048828125</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -997,6 +1009,9 @@
       <c r="V5" s="3" t="n">
         <v>640</v>
       </c>
+      <c r="W5" s="3" t="n">
+        <v>650.0999755859375</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1016,13 +1031,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>393.2000122070312</v>
+        <v>376.9500122070312</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15728.00048828125</v>
+        <v>15078.00048828125</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-1774.239511718752</v>
+        <v>-2424.239511718752</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1069,6 +1084,9 @@
       <c r="V6" s="3" t="n">
         <v>393.2000122070312</v>
       </c>
+      <c r="W6" s="3" t="n">
+        <v>376.9500122070312</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1088,13 +1106,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>235</v>
+        <v>235.75</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>23500</v>
+        <v>23575</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-2933.82</v>
+        <v>-2858.82</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1141,6 +1159,9 @@
       <c r="V7" s="3" t="n">
         <v>235</v>
       </c>
+      <c r="W7" s="3" t="n">
+        <v>235.75</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1187,13 +1208,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>22.95000076293945</v>
+        <v>22.35000038146973</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>34425.00114440918</v>
+        <v>33525.00057220459</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>3374.831144409181</v>
+        <v>2474.830572204592</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1240,6 +1261,9 @@
       <c r="V9" s="3" t="n">
         <v>22.95000076293945</v>
       </c>
+      <c r="W9" s="3" t="n">
+        <v>22.35000038146973</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1259,13 +1283,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>488.0499877929688</v>
+        <v>482.6000061035156</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48804.99877929688</v>
+        <v>48260.00061035156</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-2693.481220703128</v>
+        <v>-3238.479389648441</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1312,6 +1336,9 @@
       <c r="V10" s="3" t="n">
         <v>488.0499877929688</v>
       </c>
+      <c r="W10" s="3" t="n">
+        <v>482.6000061035156</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1331,13 +1358,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>9.220000267028809</v>
+        <v>9.960000038146973</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>9220.000267028809</v>
-      </c>
-      <c r="G11" s="6" t="n">
-        <v>-621.2097329711905</v>
+        <v>9960.000038146973</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>118.7900381469735</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -1384,6 +1411,9 @@
       <c r="V11" s="3" t="n">
         <v>9.220000267028809</v>
       </c>
+      <c r="W11" s="3" t="n">
+        <v>9.960000038146973</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1403,13 +1433,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2575</v>
+        <v>2616</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25750</v>
+        <v>26160</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-1973.25</v>
+        <v>-1563.25</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -1456,6 +1486,9 @@
       <c r="V12" s="3" t="n">
         <v>2575</v>
       </c>
+      <c r="W12" s="3" t="n">
+        <v>2616</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1475,13 +1508,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>57.75</v>
+        <v>57</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>34650</v>
+        <v>34200</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-381.760000000002</v>
+        <v>-831.760000000002</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -1528,6 +1561,9 @@
       <c r="V13" s="3" t="n">
         <v>57.75</v>
       </c>
+      <c r="W13" s="3" t="n">
+        <v>57</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1547,13 +1583,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>775.3499755859375</v>
+        <v>768.1500244140625</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>38767.49877929688</v>
+        <v>38407.50122070312</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-3695.011220703127</v>
+        <v>-4055.008779296877</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -1600,6 +1636,9 @@
       <c r="V14" s="3" t="n">
         <v>775.3499755859375</v>
       </c>
+      <c r="W14" s="3" t="n">
+        <v>768.1500244140625</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1673,13 +1712,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>492.8999938964844</v>
+        <v>511.6000061035156</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>24644.99969482422</v>
+        <v>25580.00030517578</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>2890.46969482422</v>
+        <v>3825.470305175782</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -1726,6 +1765,9 @@
       <c r="V17" s="3" t="n">
         <v>492.8999938964844</v>
       </c>
+      <c r="W17" s="3" t="n">
+        <v>511.6000061035156</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1745,13 +1787,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>427.8999938964844</v>
+        <v>426.8999938964844</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>42789.99938964844</v>
+        <v>42689.99938964844</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-3850.820610351562</v>
+        <v>-3950.820610351562</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -1798,6 +1840,9 @@
       <c r="V18" s="3" t="n">
         <v>427.8999938964844</v>
       </c>
+      <c r="W18" s="3" t="n">
+        <v>426.8999938964844</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -1809,10 +1854,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>571530.9985427856</v>
+        <v>571344.003112793</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-19251.02145721437</v>
+        <v>-19438.01688720704</v>
       </c>
     </row>
   </sheetData>
@@ -1826,7 +1871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W41"/>
+  <dimension ref="A1:X41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1852,6 +1897,7 @@
     <col width="13" customWidth="1" min="21" max="21"/>
     <col width="13" customWidth="1" min="22" max="22"/>
     <col width="13" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1970,6 +2016,11 @@
           <t>2026-05-28</t>
         </is>
       </c>
+      <c r="X1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2047,6 +2098,9 @@
       <c r="W2" s="3" t="n">
         <v>57.2415</v>
       </c>
+      <c r="X2" s="3" t="n">
+        <v>57.2415</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2071,16 +2125,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.6218</v>
+        <v>25.7152</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>62906.9764434</v>
+        <v>63136.2933376</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>2906.976443400003</v>
+        <v>3136.2933376</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.04844960739000004</v>
+        <v>0.05227155562666667</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -2124,6 +2178,9 @@
       <c r="W3" s="3" t="n">
         <v>25.6218</v>
       </c>
+      <c r="X3" s="3" t="n">
+        <v>25.7152</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2148,16 +2205,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.97</v>
+        <v>13.14</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>249103.02621</v>
+        <v>252368.06202</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>69103.02621000001</v>
+        <v>72368.06202000001</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3839057011666667</v>
+        <v>0.4020447890000001</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -2201,6 +2258,9 @@
       <c r="W4" s="3" t="n">
         <v>12.97</v>
       </c>
+      <c r="X4" s="3" t="n">
+        <v>13.14</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2278,6 +2338,9 @@
       <c r="W5" s="3" t="n">
         <v>9.6485</v>
       </c>
+      <c r="X5" s="3" t="n">
+        <v>9.6485</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2355,6 +2418,9 @@
       <c r="W6" s="3" t="n">
         <v>12.7525</v>
       </c>
+      <c r="X6" s="3" t="n">
+        <v>12.7525</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2432,6 +2498,9 @@
       <c r="W7" s="3" t="n">
         <v>34.1536</v>
       </c>
+      <c r="X7" s="3" t="n">
+        <v>34.1536</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2509,6 +2578,9 @@
       <c r="W8" s="3" t="n">
         <v>31.2273</v>
       </c>
+      <c r="X8" s="3" t="n">
+        <v>31.2273</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2586,6 +2658,9 @@
       <c r="W9" s="3" t="n">
         <v>42.3147</v>
       </c>
+      <c r="X9" s="3" t="n">
+        <v>42.3147</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2663,6 +2738,9 @@
       <c r="W10" s="3" t="n">
         <v>46.5909</v>
       </c>
+      <c r="X10" s="3" t="n">
+        <v>46.5909</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2740,6 +2818,9 @@
       <c r="W11" s="3" t="n">
         <v>105.5999</v>
       </c>
+      <c r="X11" s="3" t="n">
+        <v>105.5999</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2817,6 +2898,9 @@
       <c r="W12" s="3" t="n">
         <v>223.585</v>
       </c>
+      <c r="X12" s="3" t="n">
+        <v>223.585</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2894,6 +2978,9 @@
       <c r="W13" s="3" t="n">
         <v>20.01</v>
       </c>
+      <c r="X13" s="3" t="n">
+        <v>20.01</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2971,6 +3058,9 @@
       <c r="W14" s="3" t="n">
         <v>39.8818</v>
       </c>
+      <c r="X14" s="3" t="n">
+        <v>39.8818</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3048,6 +3138,9 @@
       <c r="W15" s="3" t="n">
         <v>12.01</v>
       </c>
+      <c r="X15" s="3" t="n">
+        <v>12.01</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3125,6 +3218,9 @@
       <c r="W16" s="3" t="n">
         <v>24.988</v>
       </c>
+      <c r="X16" s="3" t="n">
+        <v>24.988</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3202,6 +3298,9 @@
       <c r="W17" s="3" t="n">
         <v>16.7965</v>
       </c>
+      <c r="X17" s="3" t="n">
+        <v>16.7965</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3279,6 +3378,9 @@
       <c r="W18" s="3" t="n">
         <v>45.5</v>
       </c>
+      <c r="X18" s="3" t="n">
+        <v>45.5</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3356,6 +3458,9 @@
       <c r="W19" s="3" t="n">
         <v>14.8215</v>
       </c>
+      <c r="X19" s="3" t="n">
+        <v>14.8215</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3433,6 +3538,9 @@
       <c r="W20" s="3" t="n">
         <v>9.449999999999999</v>
       </c>
+      <c r="X20" s="3" t="n">
+        <v>9.449999999999999</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3510,6 +3618,9 @@
       <c r="W21" s="3" t="n">
         <v>109.0748</v>
       </c>
+      <c r="X21" s="3" t="n">
+        <v>109.0748</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3587,6 +3698,9 @@
       <c r="W22" s="3" t="n">
         <v>45.137</v>
       </c>
+      <c r="X22" s="3" t="n">
+        <v>45.137</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3664,6 +3778,9 @@
       <c r="W23" s="3" t="n">
         <v>62.8006</v>
       </c>
+      <c r="X23" s="3" t="n">
+        <v>62.8006</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3741,6 +3858,9 @@
       <c r="W24" s="3" t="n">
         <v>28.9116</v>
       </c>
+      <c r="X24" s="3" t="n">
+        <v>28.9116</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3818,6 +3938,9 @@
       <c r="W25" s="3" t="n">
         <v>11.4752</v>
       </c>
+      <c r="X25" s="3" t="n">
+        <v>11.4752</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3895,6 +4018,9 @@
       <c r="W26" s="3" t="n">
         <v>8.990399999999999</v>
       </c>
+      <c r="X26" s="3" t="n">
+        <v>8.990399999999999</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3972,6 +4098,9 @@
       <c r="W27" s="3" t="n">
         <v>64.0264</v>
       </c>
+      <c r="X27" s="3" t="n">
+        <v>64.0264</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4049,6 +4178,9 @@
       <c r="W28" s="3" t="n">
         <v>107.5591</v>
       </c>
+      <c r="X28" s="3" t="n">
+        <v>107.5591</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4126,6 +4258,9 @@
       <c r="W29" s="3" t="n">
         <v>12.13</v>
       </c>
+      <c r="X29" s="3" t="n">
+        <v>12.13</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4203,6 +4338,9 @@
       <c r="W30" s="3" t="n">
         <v>15.3581</v>
       </c>
+      <c r="X30" s="3" t="n">
+        <v>15.3581</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4280,6 +4418,9 @@
       <c r="W31" s="3" t="n">
         <v>422.49</v>
       </c>
+      <c r="X31" s="3" t="n">
+        <v>422.49</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4357,6 +4498,9 @@
       <c r="W32" s="3" t="n">
         <v>10.28</v>
       </c>
+      <c r="X32" s="3" t="n">
+        <v>10.28</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4434,6 +4578,9 @@
       <c r="W33" s="3" t="n">
         <v>18.08</v>
       </c>
+      <c r="X33" s="3" t="n">
+        <v>18.08</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4511,6 +4658,9 @@
       <c r="W34" s="3" t="n">
         <v>215.054</v>
       </c>
+      <c r="X34" s="3" t="n">
+        <v>215.054</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4588,6 +4738,9 @@
       <c r="W35" s="3" t="n">
         <v>14.55</v>
       </c>
+      <c r="X35" s="3" t="n">
+        <v>14.55</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4665,6 +4818,9 @@
       <c r="W36" s="3" t="n">
         <v>352.3059</v>
       </c>
+      <c r="X36" s="3" t="n">
+        <v>352.3059</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4742,6 +4898,9 @@
       <c r="W37" s="3" t="n">
         <v>15.682</v>
       </c>
+      <c r="X37" s="3" t="n">
+        <v>15.682</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4819,6 +4978,9 @@
       <c r="W38" s="3" t="n">
         <v>14.2639</v>
       </c>
+      <c r="X38" s="3" t="n">
+        <v>14.2639</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4896,6 +5058,9 @@
       <c r="W39" s="3" t="n">
         <v>1008.2382</v>
       </c>
+      <c r="X39" s="3" t="n">
+        <v>1008.2382</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4973,6 +5138,9 @@
       <c r="W40" s="3" t="n">
         <v>20.5343</v>
       </c>
+      <c r="X40" s="3" t="n">
+        <v>20.5343</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
@@ -4984,13 +5152,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4908559.2093685</v>
+        <v>4912053.5620727</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>438559.2093685</v>
+        <v>442053.5620727</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.09811167994821028</v>
+        <v>0.09889341433393736</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-05-30
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-05-29 06:12 IST</t>
+          <t>Generated: 2026-05-30 05:47 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4912053.5620727</v>
+        <v>4890219.5606371</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>442053.5620726999</v>
+        <v>420219.5606370997</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.09889341433393734</v>
+        <v>0.09400885025438471</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>571344.003112793</v>
+        <v>567171.5012435913</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-19438.01688720705</v>
+        <v>-23610.51875640871</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.03290218088764287</v>
+        <v>-0.03996485667659403</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5483397.565185493</v>
+        <v>5457391.061880691</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>422615.5451854933</v>
+        <v>396609.0418806914</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.08350795262774297</v>
+        <v>0.07836912167196869</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-05-29</t>
+          <t>Last snapshot: 2026-05-30</t>
         </is>
       </c>
     </row>
@@ -616,14 +616,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W19"/>
+  <dimension ref="A1:X19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="21" customWidth="1" min="8" max="8"/>
@@ -642,6 +642,7 @@
     <col width="21" customWidth="1" min="21" max="21"/>
     <col width="21" customWidth="1" min="22" max="22"/>
     <col width="21" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -760,6 +761,11 @@
           <t>2026-05-29</t>
         </is>
       </c>
+      <c r="X1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -779,13 +785,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>590.9000244140625</v>
+        <v>590</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>47272.001953125</v>
+        <v>47200</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>3454.491953124998</v>
+        <v>3382.489999999998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -835,6 +841,9 @@
       <c r="W2" s="3" t="n">
         <v>590.9000244140625</v>
       </c>
+      <c r="X2" s="3" t="n">
+        <v>590</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -881,13 +890,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1593.199951171875</v>
+        <v>1578.199951171875</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>31863.9990234375</v>
+        <v>31563.9990234375</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-240.5809765625017</v>
+        <v>-540.5809765625017</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -937,6 +946,9 @@
       <c r="W4" s="3" t="n">
         <v>1593.199951171875</v>
       </c>
+      <c r="X4" s="3" t="n">
+        <v>1578.199951171875</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -956,13 +968,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>650.0999755859375</v>
+        <v>650.0499877929688</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13001.99951171875</v>
+        <v>13000.99975585938</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1211.10048828125</v>
+        <v>-1212.100244140625</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1012,6 +1024,9 @@
       <c r="W5" s="3" t="n">
         <v>650.0999755859375</v>
       </c>
+      <c r="X5" s="3" t="n">
+        <v>650.0499877929688</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1031,13 +1046,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>376.9500122070312</v>
+        <v>368.25</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15078.00048828125</v>
+        <v>14730</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2424.239511718752</v>
+        <v>-2772.240000000002</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1087,6 +1102,9 @@
       <c r="W6" s="3" t="n">
         <v>376.9500122070312</v>
       </c>
+      <c r="X6" s="3" t="n">
+        <v>368.25</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1106,13 +1124,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>235.75</v>
+        <v>231.6999969482422</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>23575</v>
+        <v>23169.99969482422</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-2858.82</v>
+        <v>-3263.820305175781</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1162,6 +1180,9 @@
       <c r="W7" s="3" t="n">
         <v>235.75</v>
       </c>
+      <c r="X7" s="3" t="n">
+        <v>231.6999969482422</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1208,13 +1229,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>22.35000038146973</v>
+        <v>21.8700008392334</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>33525.00057220459</v>
+        <v>32805.0012588501</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>2474.830572204592</v>
+        <v>1754.831258850099</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1264,6 +1285,9 @@
       <c r="W9" s="3" t="n">
         <v>22.35000038146973</v>
       </c>
+      <c r="X9" s="3" t="n">
+        <v>21.8700008392334</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1283,13 +1307,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>482.6000061035156</v>
+        <v>476.1499938964844</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48260.00061035156</v>
+        <v>47614.99938964844</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-3238.479389648441</v>
+        <v>-3883.480610351566</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1339,6 +1363,9 @@
       <c r="W10" s="3" t="n">
         <v>482.6000061035156</v>
       </c>
+      <c r="X10" s="3" t="n">
+        <v>476.1499938964844</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1358,13 +1385,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>9.960000038146973</v>
+        <v>9.600000381469727</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>9960.000038146973</v>
-      </c>
-      <c r="G11" s="4" t="n">
-        <v>118.7900381469735</v>
+        <v>9600.000381469727</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>-241.2096185302726</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -1414,6 +1441,9 @@
       <c r="W11" s="3" t="n">
         <v>9.960000038146973</v>
       </c>
+      <c r="X11" s="3" t="n">
+        <v>9.600000381469727</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1433,13 +1463,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2616</v>
+        <v>2552.699951171875</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>26160</v>
+        <v>25526.99951171875</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-1563.25</v>
+        <v>-2196.25048828125</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -1489,6 +1519,9 @@
       <c r="W12" s="3" t="n">
         <v>2616</v>
       </c>
+      <c r="X12" s="3" t="n">
+        <v>2552.699951171875</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1508,13 +1541,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>57</v>
+        <v>56.9900016784668</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>34200</v>
+        <v>34194.00100708008</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-831.760000000002</v>
+        <v>-837.7589929199239</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -1564,6 +1597,9 @@
       <c r="W13" s="3" t="n">
         <v>57</v>
       </c>
+      <c r="X13" s="3" t="n">
+        <v>56.9900016784668</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1583,13 +1619,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>768.1500244140625</v>
+        <v>758</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>38407.50122070312</v>
+        <v>37900</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-4055.008779296877</v>
+        <v>-4562.510000000002</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -1639,6 +1675,9 @@
       <c r="W14" s="3" t="n">
         <v>768.1500244140625</v>
       </c>
+      <c r="X14" s="3" t="n">
+        <v>758</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1712,13 +1751,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>511.6000061035156</v>
+        <v>520.4000244140625</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>25580.00030517578</v>
+        <v>26020.00122070312</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>3825.470305175782</v>
+        <v>4265.471220703126</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -1768,6 +1807,9 @@
       <c r="W17" s="3" t="n">
         <v>511.6000061035156</v>
       </c>
+      <c r="X17" s="3" t="n">
+        <v>520.4000244140625</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1787,13 +1829,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>426.8999938964844</v>
+        <v>420.75</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>42689.99938964844</v>
+        <v>42075</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-3950.820610351562</v>
+        <v>-4565.82</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -1843,6 +1885,9 @@
       <c r="W18" s="3" t="n">
         <v>426.8999938964844</v>
       </c>
+      <c r="X18" s="3" t="n">
+        <v>420.75</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -1854,10 +1899,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>571344.003112793</v>
+        <v>567171.5012435913</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-19438.01688720704</v>
+        <v>-23610.5187564087</v>
       </c>
     </row>
   </sheetData>
@@ -1871,7 +1916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X41"/>
+  <dimension ref="A1:Y41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1898,6 +1943,7 @@
     <col width="13" customWidth="1" min="22" max="22"/>
     <col width="13" customWidth="1" min="23" max="23"/>
     <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2021,6 +2067,11 @@
           <t>2026-05-29</t>
         </is>
       </c>
+      <c r="Y1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2045,16 +2096,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>57.2415</v>
+        <v>56.9664</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>64252.553403</v>
+        <v>63943.7586048</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>14252.553403</v>
+        <v>13943.7586048</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.28505106806</v>
+        <v>0.278875172096</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -2101,6 +2152,9 @@
       <c r="X2" s="3" t="n">
         <v>57.2415</v>
       </c>
+      <c r="Y2" s="3" t="n">
+        <v>56.9664</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2181,6 +2235,9 @@
       <c r="X3" s="3" t="n">
         <v>25.7152</v>
       </c>
+      <c r="Y3" s="3" t="n">
+        <v>25.7152</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2261,6 +2318,9 @@
       <c r="X4" s="3" t="n">
         <v>13.14</v>
       </c>
+      <c r="Y4" s="3" t="n">
+        <v>13.14</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2285,16 +2345,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.6485</v>
+        <v>9.5253</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>177089.418068</v>
+        <v>174828.1944264</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-32910.581932</v>
+        <v>-35171.8055736</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1567170568190476</v>
+        <v>-0.1674847884457143</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -2341,6 +2401,9 @@
       <c r="X5" s="3" t="n">
         <v>9.6485</v>
       </c>
+      <c r="Y5" s="3" t="n">
+        <v>9.5253</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2365,16 +2428,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.7525</v>
+        <v>12.5581</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>53930.0291925</v>
+        <v>53107.91606369999</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>3930.029192499998</v>
+        <v>3107.916063699995</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.07860058384999996</v>
+        <v>0.0621583212739999</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -2421,6 +2484,9 @@
       <c r="X6" s="3" t="n">
         <v>12.7525</v>
       </c>
+      <c r="Y6" s="3" t="n">
+        <v>12.5581</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2445,16 +2511,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>34.1536</v>
+        <v>33.8687</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>75344.207744</v>
+        <v>74715.70694799999</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>15344.207744</v>
+        <v>14715.70694799999</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2557367957333333</v>
+        <v>0.2452617824666665</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -2501,6 +2567,9 @@
       <c r="X7" s="3" t="n">
         <v>34.1536</v>
       </c>
+      <c r="Y7" s="3" t="n">
+        <v>33.8687</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2525,16 +2594,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>31.2273</v>
+        <v>31.5057</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>50107.1069889</v>
+        <v>50553.8256801</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>107.1069888999991</v>
+        <v>553.8256801000025</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.002142139777999983</v>
+        <v>0.01107651360200005</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -2581,6 +2650,9 @@
       <c r="X8" s="3" t="n">
         <v>31.2273</v>
       </c>
+      <c r="Y8" s="3" t="n">
+        <v>31.5057</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2605,16 +2677,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>42.3147</v>
+        <v>43.0068</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>136227.6489771</v>
+        <v>138455.7908724</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>36227.64897710001</v>
+        <v>38455.79087239999</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3622764897710001</v>
+        <v>0.3845579087239999</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -2661,6 +2733,9 @@
       <c r="X9" s="3" t="n">
         <v>42.3147</v>
       </c>
+      <c r="Y9" s="3" t="n">
+        <v>43.0068</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2685,16 +2760,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>46.5909</v>
+        <v>46.3408</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>132628.4048031</v>
+        <v>131916.4553872</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>32628.40480310001</v>
+        <v>31916.4553872</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3262840480310001</v>
+        <v>0.3191645538719999</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -2741,6 +2816,9 @@
       <c r="X10" s="3" t="n">
         <v>46.5909</v>
       </c>
+      <c r="Y10" s="3" t="n">
+        <v>46.3408</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2765,16 +2843,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>105.5999</v>
+        <v>106.1501</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31777.0163081</v>
+        <v>31942.5819419</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1777.016308099999</v>
+        <v>1942.581941899996</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.05923387693666664</v>
+        <v>0.06475273139666654</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -2821,6 +2899,9 @@
       <c r="X11" s="3" t="n">
         <v>105.5999</v>
       </c>
+      <c r="Y11" s="3" t="n">
+        <v>106.1501</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2845,16 +2926,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>223.585</v>
+        <v>221.322</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>104083.73637</v>
+        <v>103030.260084</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>4083.736369999999</v>
+        <v>3030.260083999994</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.04083736369999999</v>
+        <v>0.03030260083999994</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -2901,6 +2982,9 @@
       <c r="X12" s="3" t="n">
         <v>223.585</v>
       </c>
+      <c r="Y12" s="3" t="n">
+        <v>221.322</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2925,16 +3009,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>20.01</v>
+        <v>19.928</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>231867.97605</v>
+        <v>230917.79244</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>31867.97605</v>
+        <v>30917.79243999999</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.15933988025</v>
+        <v>0.1545889622</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -2981,6 +3065,9 @@
       <c r="X13" s="3" t="n">
         <v>20.01</v>
       </c>
+      <c r="Y13" s="3" t="n">
+        <v>19.928</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3005,16 +3092,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>39.8818</v>
+        <v>40.0376</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>143877.8209708</v>
+        <v>144439.8859856</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>43877.82097080001</v>
+        <v>44439.88598560001</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.4387782097080001</v>
+        <v>0.444398859856</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -3061,6 +3148,9 @@
       <c r="X14" s="3" t="n">
         <v>39.8818</v>
       </c>
+      <c r="Y14" s="3" t="n">
+        <v>40.0376</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3085,16 +3175,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>12.01</v>
+        <v>11.93</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>117024.80347</v>
+        <v>116245.28771</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>17024.80347</v>
+        <v>16245.28771</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1702480347</v>
+        <v>0.1624528771</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -3141,6 +3231,9 @@
       <c r="X15" s="3" t="n">
         <v>12.01</v>
       </c>
+      <c r="Y15" s="3" t="n">
+        <v>11.93</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3165,16 +3258,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.988</v>
+        <v>25.1815</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>143004.524864</v>
+        <v>144111.911432</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>43004.52486400001</v>
+        <v>44111.91143199999</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.43004524864</v>
+        <v>0.4411191143199999</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -3221,6 +3314,9 @@
       <c r="X16" s="3" t="n">
         <v>24.988</v>
       </c>
+      <c r="Y16" s="3" t="n">
+        <v>25.1815</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3245,16 +3341,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.7965</v>
+        <v>16.6825</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55530.1864005</v>
+        <v>55153.2959025</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5530.186400500002</v>
+        <v>5153.295902500002</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1106037280100001</v>
+        <v>0.10306591805</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -3301,6 +3397,9 @@
       <c r="X17" s="3" t="n">
         <v>16.7965</v>
       </c>
+      <c r="Y17" s="3" t="n">
+        <v>16.6825</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3325,16 +3424,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>45.5</v>
+        <v>44.93</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>85832.838</v>
+        <v>84757.56947999999</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>5832.838000000003</v>
+        <v>4757.569479999991</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.07291047500000004</v>
+        <v>0.05946961849999989</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -3381,6 +3480,9 @@
       <c r="X18" s="3" t="n">
         <v>45.5</v>
       </c>
+      <c r="Y18" s="3" t="n">
+        <v>44.93</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3405,16 +3507,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>14.8215</v>
+        <v>15.0685</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>214419.172269</v>
+        <v>217992.463471</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>64419.172269</v>
+        <v>67992.463471</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.42946114846</v>
+        <v>0.4532830898066667</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -3461,6 +3563,9 @@
       <c r="X19" s="3" t="n">
         <v>14.8215</v>
       </c>
+      <c r="Y19" s="3" t="n">
+        <v>15.0685</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3485,16 +3590,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.449999999999999</v>
+        <v>9.44</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>248117.33835</v>
+        <v>247854.78032</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-1882.661650000024</v>
+        <v>-2145.219680000009</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.007530646600000095</v>
+        <v>-0.008580878720000037</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -3541,6 +3646,9 @@
       <c r="X20" s="3" t="n">
         <v>9.449999999999999</v>
       </c>
+      <c r="Y20" s="3" t="n">
+        <v>9.44</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3565,16 +3673,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>109.0748</v>
+        <v>107.9469</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>165712.8715732</v>
+        <v>163999.2993471</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-4287.128426800016</v>
+        <v>-6000.700652900006</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.02521840251058833</v>
+        <v>-0.03529823913470592</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -3621,6 +3729,9 @@
       <c r="X21" s="3" t="n">
         <v>109.0748</v>
       </c>
+      <c r="Y21" s="3" t="n">
+        <v>107.9469</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3645,16 +3756,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>45.137</v>
+        <v>45.346</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>69260.92102000001</v>
+        <v>69581.62316</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>9260.921020000009</v>
+        <v>9581.623160000003</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1543486836666668</v>
+        <v>0.1596937193333334</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -3701,6 +3812,9 @@
       <c r="X22" s="3" t="n">
         <v>45.137</v>
       </c>
+      <c r="Y22" s="3" t="n">
+        <v>45.346</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3725,16 +3839,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>62.8006</v>
+        <v>62.2455</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>170595.7574802</v>
+        <v>169087.8466485</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>20595.7574802</v>
+        <v>19087.84664850001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.137305049868</v>
+        <v>0.1272523109900001</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -3781,6 +3895,9 @@
       <c r="X23" s="3" t="n">
         <v>62.8006</v>
       </c>
+      <c r="Y23" s="3" t="n">
+        <v>62.2455</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3805,16 +3922,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>28.9116</v>
+        <v>28.4049</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>105047.0026776</v>
+        <v>103205.9659914</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>5047.002677600001</v>
+        <v>3205.965991400008</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.05047002677600002</v>
+        <v>0.03205965991400007</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -3861,6 +3978,9 @@
       <c r="X24" s="3" t="n">
         <v>28.9116</v>
       </c>
+      <c r="Y24" s="3" t="n">
+        <v>28.4049</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3885,16 +4005,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.4752</v>
+        <v>11.3963</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>188441.9934848</v>
+        <v>187146.3234062</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-11558.00651520002</v>
+        <v>-12853.67659380002</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.05779003257600009</v>
+        <v>-0.06426838296900009</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -3941,6 +4061,9 @@
       <c r="X25" s="3" t="n">
         <v>11.4752</v>
       </c>
+      <c r="Y25" s="3" t="n">
+        <v>11.3963</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3965,16 +4088,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>8.990399999999999</v>
+        <v>8.9869</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>107360.794536</v>
+        <v>107318.9985335</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>-2639.205464000013</v>
+        <v>-2681.001466499991</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>-0.02399277694545467</v>
+        <v>-0.02437274060454537</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -4021,6 +4144,9 @@
       <c r="X26" s="3" t="n">
         <v>8.990399999999999</v>
       </c>
+      <c r="Y26" s="3" t="n">
+        <v>8.9869</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4045,16 +4171,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>64.0264</v>
+        <v>63.6173</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>103137.566704</v>
+        <v>102478.563878</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-6862.433296000017</v>
+        <v>-7521.436121999999</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.0623857572363638</v>
+        <v>-0.06837669201818181</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -4101,6 +4227,9 @@
       <c r="X27" s="3" t="n">
         <v>64.0264</v>
       </c>
+      <c r="Y27" s="3" t="n">
+        <v>63.6173</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4125,16 +4254,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>107.5591</v>
+        <v>106.2856</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>355661.0509287</v>
+        <v>351450.0232392</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-24338.94907129998</v>
+        <v>-28549.9767608</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.06404986597710521</v>
+        <v>-0.07513151779157894</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -4181,6 +4310,9 @@
       <c r="X28" s="3" t="n">
         <v>107.5591</v>
       </c>
+      <c r="Y28" s="3" t="n">
+        <v>106.2856</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4205,16 +4337,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.13</v>
+        <v>11.9376</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>116492.91739</v>
+        <v>114645.1649328</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>16492.91739</v>
+        <v>14645.16493279999</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.1649291739</v>
+        <v>0.1464516493279999</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -4261,6 +4393,9 @@
       <c r="X29" s="3" t="n">
         <v>12.13</v>
       </c>
+      <c r="Y29" s="3" t="n">
+        <v>11.9376</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4285,16 +4420,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>15.3581</v>
+        <v>15.386</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>113586.3728241</v>
+        <v>113792.717346</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>13586.37282410001</v>
+        <v>13792.71734599999</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.1358637282410001</v>
+        <v>0.1379271734599999</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -4341,6 +4476,9 @@
       <c r="X30" s="3" t="n">
         <v>15.3581</v>
       </c>
+      <c r="Y30" s="3" t="n">
+        <v>15.386</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4365,16 +4503,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>422.49</v>
+        <v>418.223</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>112416.1392</v>
+        <v>111280.77584</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>12416.13919999999</v>
+        <v>11280.77584</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.1241613919999999</v>
+        <v>0.1128077584</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -4421,6 +4559,9 @@
       <c r="X31" s="3" t="n">
         <v>422.49</v>
       </c>
+      <c r="Y31" s="3" t="n">
+        <v>418.223</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4445,16 +4586,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.28</v>
+        <v>10.16</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>217318.7888</v>
+        <v>214781.9936</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>17318.78879999998</v>
+        <v>14781.99359999999</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.0865939439999999</v>
+        <v>0.07390996799999994</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -4501,6 +4642,9 @@
       <c r="X32" s="3" t="n">
         <v>10.28</v>
       </c>
+      <c r="Y32" s="3" t="n">
+        <v>10.16</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4525,16 +4669,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>18.08</v>
+        <v>17.91</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>64792.21119999999</v>
+        <v>64182.9924</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>4792.211199999991</v>
+        <v>4182.992399999996</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.07987018666666651</v>
+        <v>0.06971653999999992</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -4581,6 +4725,9 @@
       <c r="X33" s="3" t="n">
         <v>18.08</v>
       </c>
+      <c r="Y33" s="3" t="n">
+        <v>17.91</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4605,16 +4752,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>215.054</v>
+        <v>214.6027</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>75598.14767400001</v>
+        <v>75439.5017337</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-4401.852325999993</v>
+        <v>-4560.498266299997</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.05502315407499991</v>
+        <v>-0.05700622832874996</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -4661,6 +4808,9 @@
       <c r="X34" s="3" t="n">
         <v>215.054</v>
       </c>
+      <c r="Y34" s="3" t="n">
+        <v>214.6027</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4685,16 +4835,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>14.55</v>
+        <v>14.49</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>103820.40465</v>
+        <v>103392.27927</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>3820.404649999997</v>
+        <v>3392.279269999999</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.03820404649999997</v>
+        <v>0.03392279269999999</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -4741,6 +4891,9 @@
       <c r="X35" s="3" t="n">
         <v>14.55</v>
       </c>
+      <c r="Y35" s="3" t="n">
+        <v>14.49</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4765,16 +4918,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>352.3059</v>
+        <v>349.2681</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>164070.9714654</v>
+        <v>162656.2497786</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>14070.97146540001</v>
+        <v>12656.2497786</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.09380647643600008</v>
+        <v>0.08437499852400002</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -4821,6 +4974,9 @@
       <c r="X36" s="3" t="n">
         <v>352.3059</v>
       </c>
+      <c r="Y36" s="3" t="n">
+        <v>349.2681</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4845,16 +5001,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>15.682</v>
+        <v>15.569</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>59009.62529800001</v>
+        <v>58584.41884100001</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>9009.625298000006</v>
+        <v>8584.418841000006</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.1801925059600001</v>
+        <v>0.1716883768200001</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -4901,6 +5057,9 @@
       <c r="X37" s="3" t="n">
         <v>15.682</v>
       </c>
+      <c r="Y37" s="3" t="n">
+        <v>15.569</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4925,16 +5084,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>14.2639</v>
+        <v>14.0646</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>85304.9971998</v>
+        <v>84113.0871372</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>5304.997199799996</v>
+        <v>4113.087137199997</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.06631246499749996</v>
+        <v>0.05141358921499996</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -4981,6 +5140,9 @@
       <c r="X38" s="3" t="n">
         <v>14.2639</v>
       </c>
+      <c r="Y38" s="3" t="n">
+        <v>14.0646</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5005,16 +5167,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1008.2382</v>
+        <v>1009.4228</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50291.9296542</v>
+        <v>50351.0186868</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>291.9296542000011</v>
+        <v>351.0186868000019</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.005838593084000022</v>
+        <v>0.007020373736000038</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -5061,6 +5223,9 @@
       <c r="X39" s="3" t="n">
         <v>1008.2382</v>
       </c>
+      <c r="Y39" s="3" t="n">
+        <v>1009.4228</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5085,16 +5250,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>20.5343</v>
+        <v>20.4837</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>103513.9607261</v>
+        <v>103258.8847599</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>3513.960726100006</v>
+        <v>3258.8847599</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.03513960726100006</v>
+        <v>0.032588847599</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -5141,6 +5306,9 @@
       <c r="X40" s="3" t="n">
         <v>20.5343</v>
       </c>
+      <c r="Y40" s="3" t="n">
+        <v>20.4837</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
@@ -5152,13 +5320,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4912053.5620727</v>
+        <v>4890219.5606371</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>442053.5620727</v>
+        <v>420219.5606371</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.09889341433393736</v>
+        <v>0.09400885025438478</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-05-31
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-05-30 05:47 IST</t>
+          <t>Generated: 2026-05-31 06:16 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4890219.5606371</v>
+        <v>4885284.9275033</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>420219.5606370997</v>
+        <v>415284.9275032999</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.09400885025438471</v>
+        <v>0.09290490548172257</v>
       </c>
     </row>
     <row r="6">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5457391.061880691</v>
+        <v>5452456.428746891</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>396609.0418806914</v>
+        <v>391674.4087468917</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.07836912167196869</v>
+        <v>0.07739404842947409</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-05-30</t>
+          <t>Last snapshot: 2026-05-31</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X19"/>
+  <dimension ref="A1:Y19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -643,6 +643,7 @@
     <col width="21" customWidth="1" min="22" max="22"/>
     <col width="21" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -766,6 +767,11 @@
           <t>2026-05-30</t>
         </is>
       </c>
+      <c r="Y1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -844,6 +850,9 @@
       <c r="X2" s="3" t="n">
         <v>590</v>
       </c>
+      <c r="Y2" s="3" t="n">
+        <v>590</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -949,6 +958,9 @@
       <c r="X4" s="3" t="n">
         <v>1578.199951171875</v>
       </c>
+      <c r="Y4" s="3" t="n">
+        <v>1578.199951171875</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1027,6 +1039,9 @@
       <c r="X5" s="3" t="n">
         <v>650.0499877929688</v>
       </c>
+      <c r="Y5" s="3" t="n">
+        <v>650.0499877929688</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1105,6 +1120,9 @@
       <c r="X6" s="3" t="n">
         <v>368.25</v>
       </c>
+      <c r="Y6" s="3" t="n">
+        <v>368.25</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1183,6 +1201,9 @@
       <c r="X7" s="3" t="n">
         <v>231.6999969482422</v>
       </c>
+      <c r="Y7" s="3" t="n">
+        <v>231.6999969482422</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1288,6 +1309,9 @@
       <c r="X9" s="3" t="n">
         <v>21.8700008392334</v>
       </c>
+      <c r="Y9" s="3" t="n">
+        <v>21.8700008392334</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1366,6 +1390,9 @@
       <c r="X10" s="3" t="n">
         <v>476.1499938964844</v>
       </c>
+      <c r="Y10" s="3" t="n">
+        <v>476.1499938964844</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1444,6 +1471,9 @@
       <c r="X11" s="3" t="n">
         <v>9.600000381469727</v>
       </c>
+      <c r="Y11" s="3" t="n">
+        <v>9.600000381469727</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1522,6 +1552,9 @@
       <c r="X12" s="3" t="n">
         <v>2552.699951171875</v>
       </c>
+      <c r="Y12" s="3" t="n">
+        <v>2552.699951171875</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1600,6 +1633,9 @@
       <c r="X13" s="3" t="n">
         <v>56.9900016784668</v>
       </c>
+      <c r="Y13" s="3" t="n">
+        <v>56.9900016784668</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1678,6 +1714,9 @@
       <c r="X14" s="3" t="n">
         <v>758</v>
       </c>
+      <c r="Y14" s="3" t="n">
+        <v>758</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1810,6 +1849,9 @@
       <c r="X17" s="3" t="n">
         <v>520.4000244140625</v>
       </c>
+      <c r="Y17" s="3" t="n">
+        <v>520.4000244140625</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1886,6 +1928,9 @@
         <v>426.8999938964844</v>
       </c>
       <c r="X18" s="3" t="n">
+        <v>420.75</v>
+      </c>
+      <c r="Y18" s="3" t="n">
         <v>420.75</v>
       </c>
     </row>
@@ -1916,7 +1961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y41"/>
+  <dimension ref="A1:Z41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1944,6 +1989,7 @@
     <col width="13" customWidth="1" min="23" max="23"/>
     <col width="13" customWidth="1" min="24" max="24"/>
     <col width="13" customWidth="1" min="25" max="25"/>
+    <col width="13" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2072,6 +2118,11 @@
           <t>2026-05-30</t>
         </is>
       </c>
+      <c r="Z1" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2155,6 +2206,9 @@
       <c r="Y2" s="3" t="n">
         <v>56.9664</v>
       </c>
+      <c r="Z2" s="3" t="n">
+        <v>56.9664</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2179,16 +2233,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.7152</v>
+        <v>25.5856</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>63136.2933376</v>
+        <v>62818.0977328</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>3136.2933376</v>
+        <v>2818.097732800001</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.05227155562666667</v>
+        <v>0.04696829554666668</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -2238,6 +2292,9 @@
       <c r="Y3" s="3" t="n">
         <v>25.7152</v>
       </c>
+      <c r="Z3" s="3" t="n">
+        <v>25.5856</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2262,16 +2319,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>13.14</v>
+        <v>12.9</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>252368.06202</v>
+        <v>247758.5997</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>72368.06202000001</v>
+        <v>67758.59970000002</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.4020447890000001</v>
+        <v>0.3764366650000001</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -2321,6 +2378,9 @@
       <c r="Y4" s="3" t="n">
         <v>13.14</v>
       </c>
+      <c r="Z4" s="3" t="n">
+        <v>12.9</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2345,16 +2405,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.5253</v>
+        <v>9.5251</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>174828.1944264</v>
+        <v>174824.5236088</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-35171.8055736</v>
+        <v>-35175.47639120001</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1674847884457143</v>
+        <v>-0.1675022685295238</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -2404,6 +2464,9 @@
       <c r="Y5" s="3" t="n">
         <v>9.5253</v>
       </c>
+      <c r="Z5" s="3" t="n">
+        <v>9.5251</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2487,6 +2550,9 @@
       <c r="Y6" s="3" t="n">
         <v>12.5581</v>
       </c>
+      <c r="Z6" s="3" t="n">
+        <v>12.5581</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2570,6 +2636,9 @@
       <c r="Y7" s="3" t="n">
         <v>33.8687</v>
       </c>
+      <c r="Z7" s="3" t="n">
+        <v>33.8687</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2653,6 +2722,9 @@
       <c r="Y8" s="3" t="n">
         <v>31.5057</v>
       </c>
+      <c r="Z8" s="3" t="n">
+        <v>31.5057</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2736,6 +2808,9 @@
       <c r="Y9" s="3" t="n">
         <v>43.0068</v>
       </c>
+      <c r="Z9" s="3" t="n">
+        <v>43.0068</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2819,6 +2894,9 @@
       <c r="Y10" s="3" t="n">
         <v>46.3408</v>
       </c>
+      <c r="Z10" s="3" t="n">
+        <v>46.3408</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2902,6 +2980,9 @@
       <c r="Y11" s="3" t="n">
         <v>106.1501</v>
       </c>
+      <c r="Z11" s="3" t="n">
+        <v>106.1501</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2985,6 +3066,9 @@
       <c r="Y12" s="3" t="n">
         <v>221.322</v>
       </c>
+      <c r="Z12" s="3" t="n">
+        <v>221.322</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3068,6 +3152,9 @@
       <c r="Y13" s="3" t="n">
         <v>19.928</v>
       </c>
+      <c r="Z13" s="3" t="n">
+        <v>19.928</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3151,6 +3238,9 @@
       <c r="Y14" s="3" t="n">
         <v>40.0376</v>
       </c>
+      <c r="Z14" s="3" t="n">
+        <v>40.0376</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3234,6 +3324,9 @@
       <c r="Y15" s="3" t="n">
         <v>11.93</v>
       </c>
+      <c r="Z15" s="3" t="n">
+        <v>11.93</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3317,6 +3410,9 @@
       <c r="Y16" s="3" t="n">
         <v>25.1815</v>
       </c>
+      <c r="Z16" s="3" t="n">
+        <v>25.1815</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3400,6 +3496,9 @@
       <c r="Y17" s="3" t="n">
         <v>16.6825</v>
       </c>
+      <c r="Z17" s="3" t="n">
+        <v>16.6825</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3483,6 +3582,9 @@
       <c r="Y18" s="3" t="n">
         <v>44.93</v>
       </c>
+      <c r="Z18" s="3" t="n">
+        <v>44.93</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3566,6 +3668,9 @@
       <c r="Y19" s="3" t="n">
         <v>15.0685</v>
       </c>
+      <c r="Z19" s="3" t="n">
+        <v>15.0685</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3649,6 +3754,9 @@
       <c r="Y20" s="3" t="n">
         <v>9.44</v>
       </c>
+      <c r="Z20" s="3" t="n">
+        <v>9.44</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3732,6 +3840,9 @@
       <c r="Y21" s="3" t="n">
         <v>107.9469</v>
       </c>
+      <c r="Z21" s="3" t="n">
+        <v>107.9469</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3815,6 +3926,9 @@
       <c r="Y22" s="3" t="n">
         <v>45.346</v>
       </c>
+      <c r="Z22" s="3" t="n">
+        <v>45.346</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3898,6 +4012,9 @@
       <c r="Y23" s="3" t="n">
         <v>62.2455</v>
       </c>
+      <c r="Z23" s="3" t="n">
+        <v>62.2455</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3981,6 +4098,9 @@
       <c r="Y24" s="3" t="n">
         <v>28.4049</v>
       </c>
+      <c r="Z24" s="3" t="n">
+        <v>28.4049</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4064,6 +4184,9 @@
       <c r="Y25" s="3" t="n">
         <v>11.3963</v>
       </c>
+      <c r="Z25" s="3" t="n">
+        <v>11.3963</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4147,6 +4270,9 @@
       <c r="Y26" s="3" t="n">
         <v>8.9869</v>
       </c>
+      <c r="Z26" s="3" t="n">
+        <v>8.9869</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4230,6 +4356,9 @@
       <c r="Y27" s="3" t="n">
         <v>63.6173</v>
       </c>
+      <c r="Z27" s="3" t="n">
+        <v>63.6173</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4313,6 +4442,9 @@
       <c r="Y28" s="3" t="n">
         <v>106.2856</v>
       </c>
+      <c r="Z28" s="3" t="n">
+        <v>106.2856</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4396,6 +4528,9 @@
       <c r="Y29" s="3" t="n">
         <v>11.9376</v>
       </c>
+      <c r="Z29" s="3" t="n">
+        <v>11.9376</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4479,6 +4614,9 @@
       <c r="Y30" s="3" t="n">
         <v>15.386</v>
       </c>
+      <c r="Z30" s="3" t="n">
+        <v>15.386</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4562,6 +4700,9 @@
       <c r="Y31" s="3" t="n">
         <v>418.223</v>
       </c>
+      <c r="Z31" s="3" t="n">
+        <v>418.223</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4645,6 +4786,9 @@
       <c r="Y32" s="3" t="n">
         <v>10.16</v>
       </c>
+      <c r="Z32" s="3" t="n">
+        <v>10.16</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4728,6 +4872,9 @@
       <c r="Y33" s="3" t="n">
         <v>17.91</v>
       </c>
+      <c r="Z33" s="3" t="n">
+        <v>17.91</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4752,16 +4899,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>214.6027</v>
+        <v>214.5933</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>75439.5017337</v>
+        <v>75436.1973423</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-4560.498266299997</v>
+        <v>-4563.802657699998</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.05700622832874996</v>
+        <v>-0.05704753322124998</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -4811,6 +4958,9 @@
       <c r="Y34" s="3" t="n">
         <v>214.6027</v>
       </c>
+      <c r="Z34" s="3" t="n">
+        <v>214.5933</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4894,6 +5044,9 @@
       <c r="Y35" s="3" t="n">
         <v>14.49</v>
       </c>
+      <c r="Z35" s="3" t="n">
+        <v>14.49</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4977,6 +5130,9 @@
       <c r="Y36" s="3" t="n">
         <v>349.2681</v>
       </c>
+      <c r="Z36" s="3" t="n">
+        <v>349.2681</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5060,6 +5216,9 @@
       <c r="Y37" s="3" t="n">
         <v>15.569</v>
       </c>
+      <c r="Z37" s="3" t="n">
+        <v>15.569</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5143,6 +5302,9 @@
       <c r="Y38" s="3" t="n">
         <v>14.0646</v>
       </c>
+      <c r="Z38" s="3" t="n">
+        <v>14.0646</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5226,6 +5388,9 @@
       <c r="Y39" s="3" t="n">
         <v>1009.4228</v>
       </c>
+      <c r="Z39" s="3" t="n">
+        <v>1009.4228</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5309,6 +5474,9 @@
       <c r="Y40" s="3" t="n">
         <v>20.4837</v>
       </c>
+      <c r="Z40" s="3" t="n">
+        <v>20.4837</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
@@ -5320,13 +5488,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4890219.5606371</v>
+        <v>4885284.9275033</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>420219.5606371</v>
+        <v>415284.9275033</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.09400885025438478</v>
+        <v>0.09290490548172259</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-06-01
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -484,8 +484,8 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-05-31 06:16 IST</t>
+          <t>Generated: 2026-06-01 06:53 IST</t>
         </is>
       </c>
     </row>
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>567171.5012435913</v>
+        <v>561744.0025787354</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-23610.51875640871</v>
+        <v>-29038.01742126467</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.03996485667659403</v>
+        <v>-0.04915183001213318</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5452456.428746891</v>
+        <v>5447028.930082035</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>391674.4087468917</v>
+        <v>386246.9100820357</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.07739404842947409</v>
+        <v>0.07632158598327374</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-05-31</t>
+          <t>Last snapshot: 2026-06-01</t>
         </is>
       </c>
     </row>
@@ -616,14 +616,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y19"/>
+  <dimension ref="A1:Z19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="21" customWidth="1" min="8" max="8"/>
@@ -644,6 +644,7 @@
     <col width="21" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
     <col width="20" customWidth="1" min="25" max="25"/>
+    <col width="21" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -772,6 +773,11 @@
           <t>2026-05-31</t>
         </is>
       </c>
+      <c r="Z1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -791,13 +797,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>590</v>
+        <v>584.1500244140625</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>47200</v>
+        <v>46732.001953125</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>3382.489999999998</v>
+        <v>2914.491953124998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -853,6 +859,9 @@
       <c r="Y2" s="3" t="n">
         <v>590</v>
       </c>
+      <c r="Z2" s="3" t="n">
+        <v>584.1500244140625</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -899,13 +908,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1578.199951171875</v>
+        <v>1553.400024414062</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>31563.9990234375</v>
+        <v>31068.00048828125</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-540.5809765625017</v>
+        <v>-1036.579511718752</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -961,6 +970,9 @@
       <c r="Y4" s="3" t="n">
         <v>1578.199951171875</v>
       </c>
+      <c r="Z4" s="3" t="n">
+        <v>1553.400024414062</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -980,13 +992,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>650.0499877929688</v>
+        <v>655.4000244140625</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13000.99975585938</v>
+        <v>13108.00048828125</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1212.100244140625</v>
+        <v>-1105.09951171875</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1042,6 +1054,9 @@
       <c r="Y5" s="3" t="n">
         <v>650.0499877929688</v>
       </c>
+      <c r="Z5" s="3" t="n">
+        <v>655.4000244140625</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1061,13 +1076,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>368.25</v>
+        <v>384.7999877929688</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>14730</v>
+        <v>15391.99951171875</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2772.240000000002</v>
+        <v>-2110.240488281252</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1123,6 +1138,9 @@
       <c r="Y6" s="3" t="n">
         <v>368.25</v>
       </c>
+      <c r="Z6" s="3" t="n">
+        <v>384.7999877929688</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1142,13 +1160,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>231.6999969482422</v>
+        <v>228.5</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>23169.99969482422</v>
+        <v>22850</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-3263.820305175781</v>
+        <v>-3583.82</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1204,6 +1222,9 @@
       <c r="Y7" s="3" t="n">
         <v>231.6999969482422</v>
       </c>
+      <c r="Z7" s="3" t="n">
+        <v>228.5</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1250,13 +1271,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>21.8700008392334</v>
+        <v>19.1200008392334</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>32805.0012588501</v>
-      </c>
-      <c r="G9" s="4" t="n">
-        <v>1754.831258850099</v>
+        <v>28680.0012588501</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>-2370.168741149901</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1312,6 +1333,9 @@
       <c r="Y9" s="3" t="n">
         <v>21.8700008392334</v>
       </c>
+      <c r="Z9" s="3" t="n">
+        <v>19.1200008392334</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1331,13 +1355,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>476.1499938964844</v>
+        <v>479.6499938964844</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>47614.99938964844</v>
+        <v>47964.99938964844</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-3883.480610351566</v>
+        <v>-3533.480610351566</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1393,6 +1417,9 @@
       <c r="Y10" s="3" t="n">
         <v>476.1499938964844</v>
       </c>
+      <c r="Z10" s="3" t="n">
+        <v>479.6499938964844</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1412,13 +1439,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>9.600000381469727</v>
+        <v>9.550000190734863</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>9600.000381469727</v>
+        <v>9550.000190734863</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-241.2096185302726</v>
+        <v>-291.2098092651358</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -1474,6 +1501,9 @@
       <c r="Y11" s="3" t="n">
         <v>9.600000381469727</v>
       </c>
+      <c r="Z11" s="3" t="n">
+        <v>9.550000190734863</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1493,13 +1523,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2552.699951171875</v>
+        <v>2570.5</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25526.99951171875</v>
+        <v>25705</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2196.25048828125</v>
+        <v>-2018.25</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -1555,6 +1585,9 @@
       <c r="Y12" s="3" t="n">
         <v>2552.699951171875</v>
       </c>
+      <c r="Z12" s="3" t="n">
+        <v>2570.5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1574,13 +1607,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>56.9900016784668</v>
+        <v>54.65999984741211</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>34194.00100708008</v>
+        <v>32795.99990844727</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-837.7589929199239</v>
+        <v>-2235.760091552736</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -1636,6 +1669,9 @@
       <c r="Y13" s="3" t="n">
         <v>56.9900016784668</v>
       </c>
+      <c r="Z13" s="3" t="n">
+        <v>54.65999984741211</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1655,13 +1691,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>758</v>
+        <v>749.2999877929688</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>37900</v>
+        <v>37464.99938964844</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-4562.510000000002</v>
+        <v>-4997.510610351565</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -1717,6 +1753,9 @@
       <c r="Y14" s="3" t="n">
         <v>758</v>
       </c>
+      <c r="Z14" s="3" t="n">
+        <v>749.2999877929688</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1790,13 +1829,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>520.4000244140625</v>
+        <v>532.75</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>26020.00122070312</v>
+        <v>26637.5</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>4265.471220703126</v>
+        <v>4882.970000000001</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -1852,6 +1891,9 @@
       <c r="Y17" s="3" t="n">
         <v>520.4000244140625</v>
       </c>
+      <c r="Z17" s="3" t="n">
+        <v>532.75</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1871,13 +1913,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>420.75</v>
+        <v>420.25</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>42075</v>
+        <v>42025</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-4565.82</v>
+        <v>-4615.82</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -1933,6 +1975,9 @@
       <c r="Y18" s="3" t="n">
         <v>420.75</v>
       </c>
+      <c r="Z18" s="3" t="n">
+        <v>420.25</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -1944,10 +1989,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>567171.5012435913</v>
+        <v>561744.0025787354</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-23610.5187564087</v>
+        <v>-29038.01742126466</v>
       </c>
     </row>
   </sheetData>
@@ -1961,7 +2006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z41"/>
+  <dimension ref="A1:AA41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1990,6 +2035,7 @@
     <col width="13" customWidth="1" min="24" max="24"/>
     <col width="13" customWidth="1" min="25" max="25"/>
     <col width="13" customWidth="1" min="26" max="26"/>
+    <col width="13" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2123,6 +2169,11 @@
           <t>2026-05-31</t>
         </is>
       </c>
+      <c r="AA1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2209,6 +2260,9 @@
       <c r="Z2" s="3" t="n">
         <v>56.9664</v>
       </c>
+      <c r="AA2" s="3" t="n">
+        <v>56.9664</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2295,6 +2349,9 @@
       <c r="Z3" s="3" t="n">
         <v>25.5856</v>
       </c>
+      <c r="AA3" s="3" t="n">
+        <v>25.5856</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2381,6 +2438,9 @@
       <c r="Z4" s="3" t="n">
         <v>12.9</v>
       </c>
+      <c r="AA4" s="3" t="n">
+        <v>12.9</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2467,6 +2527,9 @@
       <c r="Z5" s="3" t="n">
         <v>9.5251</v>
       </c>
+      <c r="AA5" s="3" t="n">
+        <v>9.5251</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2553,6 +2616,9 @@
       <c r="Z6" s="3" t="n">
         <v>12.5581</v>
       </c>
+      <c r="AA6" s="3" t="n">
+        <v>12.5581</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2639,6 +2705,9 @@
       <c r="Z7" s="3" t="n">
         <v>33.8687</v>
       </c>
+      <c r="AA7" s="3" t="n">
+        <v>33.8687</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2725,6 +2794,9 @@
       <c r="Z8" s="3" t="n">
         <v>31.5057</v>
       </c>
+      <c r="AA8" s="3" t="n">
+        <v>31.5057</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2811,6 +2883,9 @@
       <c r="Z9" s="3" t="n">
         <v>43.0068</v>
       </c>
+      <c r="AA9" s="3" t="n">
+        <v>43.0068</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2897,6 +2972,9 @@
       <c r="Z10" s="3" t="n">
         <v>46.3408</v>
       </c>
+      <c r="AA10" s="3" t="n">
+        <v>46.3408</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2983,6 +3061,9 @@
       <c r="Z11" s="3" t="n">
         <v>106.1501</v>
       </c>
+      <c r="AA11" s="3" t="n">
+        <v>106.1501</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3069,6 +3150,9 @@
       <c r="Z12" s="3" t="n">
         <v>221.322</v>
       </c>
+      <c r="AA12" s="3" t="n">
+        <v>221.322</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3155,6 +3239,9 @@
       <c r="Z13" s="3" t="n">
         <v>19.928</v>
       </c>
+      <c r="AA13" s="3" t="n">
+        <v>19.928</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3241,6 +3328,9 @@
       <c r="Z14" s="3" t="n">
         <v>40.0376</v>
       </c>
+      <c r="AA14" s="3" t="n">
+        <v>40.0376</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3327,6 +3417,9 @@
       <c r="Z15" s="3" t="n">
         <v>11.93</v>
       </c>
+      <c r="AA15" s="3" t="n">
+        <v>11.93</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3413,6 +3506,9 @@
       <c r="Z16" s="3" t="n">
         <v>25.1815</v>
       </c>
+      <c r="AA16" s="3" t="n">
+        <v>25.1815</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3499,6 +3595,9 @@
       <c r="Z17" s="3" t="n">
         <v>16.6825</v>
       </c>
+      <c r="AA17" s="3" t="n">
+        <v>16.6825</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3585,6 +3684,9 @@
       <c r="Z18" s="3" t="n">
         <v>44.93</v>
       </c>
+      <c r="AA18" s="3" t="n">
+        <v>44.93</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3671,6 +3773,9 @@
       <c r="Z19" s="3" t="n">
         <v>15.0685</v>
       </c>
+      <c r="AA19" s="3" t="n">
+        <v>15.0685</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3757,6 +3862,9 @@
       <c r="Z20" s="3" t="n">
         <v>9.44</v>
       </c>
+      <c r="AA20" s="3" t="n">
+        <v>9.44</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3843,6 +3951,9 @@
       <c r="Z21" s="3" t="n">
         <v>107.9469</v>
       </c>
+      <c r="AA21" s="3" t="n">
+        <v>107.9469</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3929,6 +4040,9 @@
       <c r="Z22" s="3" t="n">
         <v>45.346</v>
       </c>
+      <c r="AA22" s="3" t="n">
+        <v>45.346</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4015,6 +4129,9 @@
       <c r="Z23" s="3" t="n">
         <v>62.2455</v>
       </c>
+      <c r="AA23" s="3" t="n">
+        <v>62.2455</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4101,6 +4218,9 @@
       <c r="Z24" s="3" t="n">
         <v>28.4049</v>
       </c>
+      <c r="AA24" s="3" t="n">
+        <v>28.4049</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4187,6 +4307,9 @@
       <c r="Z25" s="3" t="n">
         <v>11.3963</v>
       </c>
+      <c r="AA25" s="3" t="n">
+        <v>11.3963</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4273,6 +4396,9 @@
       <c r="Z26" s="3" t="n">
         <v>8.9869</v>
       </c>
+      <c r="AA26" s="3" t="n">
+        <v>8.9869</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4359,6 +4485,9 @@
       <c r="Z27" s="3" t="n">
         <v>63.6173</v>
       </c>
+      <c r="AA27" s="3" t="n">
+        <v>63.6173</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4445,6 +4574,9 @@
       <c r="Z28" s="3" t="n">
         <v>106.2856</v>
       </c>
+      <c r="AA28" s="3" t="n">
+        <v>106.2856</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4531,6 +4663,9 @@
       <c r="Z29" s="3" t="n">
         <v>11.9376</v>
       </c>
+      <c r="AA29" s="3" t="n">
+        <v>11.9376</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4617,6 +4752,9 @@
       <c r="Z30" s="3" t="n">
         <v>15.386</v>
       </c>
+      <c r="AA30" s="3" t="n">
+        <v>15.386</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4703,6 +4841,9 @@
       <c r="Z31" s="3" t="n">
         <v>418.223</v>
       </c>
+      <c r="AA31" s="3" t="n">
+        <v>418.223</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4789,6 +4930,9 @@
       <c r="Z32" s="3" t="n">
         <v>10.16</v>
       </c>
+      <c r="AA32" s="3" t="n">
+        <v>10.16</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4875,6 +5019,9 @@
       <c r="Z33" s="3" t="n">
         <v>17.91</v>
       </c>
+      <c r="AA33" s="3" t="n">
+        <v>17.91</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4961,6 +5108,9 @@
       <c r="Z34" s="3" t="n">
         <v>214.5933</v>
       </c>
+      <c r="AA34" s="3" t="n">
+        <v>214.5933</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -5047,6 +5197,9 @@
       <c r="Z35" s="3" t="n">
         <v>14.49</v>
       </c>
+      <c r="AA35" s="3" t="n">
+        <v>14.49</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5133,6 +5286,9 @@
       <c r="Z36" s="3" t="n">
         <v>349.2681</v>
       </c>
+      <c r="AA36" s="3" t="n">
+        <v>349.2681</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5219,6 +5375,9 @@
       <c r="Z37" s="3" t="n">
         <v>15.569</v>
       </c>
+      <c r="AA37" s="3" t="n">
+        <v>15.569</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5305,6 +5464,9 @@
       <c r="Z38" s="3" t="n">
         <v>14.0646</v>
       </c>
+      <c r="AA38" s="3" t="n">
+        <v>14.0646</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5391,6 +5553,9 @@
       <c r="Z39" s="3" t="n">
         <v>1009.4228</v>
       </c>
+      <c r="AA39" s="3" t="n">
+        <v>1009.4228</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5475,6 +5640,9 @@
         <v>20.4837</v>
       </c>
       <c r="Z40" s="3" t="n">
+        <v>20.4837</v>
+      </c>
+      <c r="AA40" s="3" t="n">
         <v>20.4837</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily portfolio update 2026-06-02
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -484,8 +484,8 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-01 06:53 IST</t>
+          <t>Generated: 2026-06-02 06:40 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4885284.9275033</v>
+        <v>4851981.0548428</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>415284.9275032999</v>
+        <v>381981.0548427999</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.09290490548172257</v>
+        <v>0.08545437468519014</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>561744.0025787354</v>
+        <v>556288.4975891113</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-29038.01742126467</v>
+        <v>-34493.52241088869</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.04915183001213318</v>
+        <v>-0.05838620886073799</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5447028.930082035</v>
+        <v>5408269.552431911</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>386246.9100820357</v>
+        <v>347487.5324319117</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.07632158598327374</v>
+        <v>0.0686628135846704</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-06-01</t>
+          <t>Last snapshot: 2026-06-02</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z19"/>
+  <dimension ref="A1:AA19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -645,6 +645,7 @@
     <col width="20" customWidth="1" min="24" max="24"/>
     <col width="20" customWidth="1" min="25" max="25"/>
     <col width="21" customWidth="1" min="26" max="26"/>
+    <col width="21" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -778,6 +779,11 @@
           <t>2026-06-01</t>
         </is>
       </c>
+      <c r="AA1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -797,13 +803,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>584.1500244140625</v>
+        <v>590.3499755859375</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>46732.001953125</v>
+        <v>47227.998046875</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>2914.491953124998</v>
+        <v>3410.488046874998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -862,6 +868,9 @@
       <c r="Z2" s="3" t="n">
         <v>584.1500244140625</v>
       </c>
+      <c r="AA2" s="3" t="n">
+        <v>590.3499755859375</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -908,13 +917,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1553.400024414062</v>
+        <v>1494.099975585938</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>31068.00048828125</v>
+        <v>29881.99951171875</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-1036.579511718752</v>
+        <v>-2222.580488281252</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -973,6 +982,9 @@
       <c r="Z4" s="3" t="n">
         <v>1553.400024414062</v>
       </c>
+      <c r="AA4" s="3" t="n">
+        <v>1494.099975585938</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -992,13 +1004,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>655.4000244140625</v>
+        <v>663.25</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13108.00048828125</v>
+        <v>13265</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1105.09951171875</v>
+        <v>-948.1000000000004</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1057,6 +1069,9 @@
       <c r="Z5" s="3" t="n">
         <v>655.4000244140625</v>
       </c>
+      <c r="AA5" s="3" t="n">
+        <v>663.25</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1076,13 +1091,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>384.7999877929688</v>
+        <v>375.3999938964844</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15391.99951171875</v>
+        <v>15015.99975585938</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2110.240488281252</v>
+        <v>-2486.240244140627</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1141,6 +1156,9 @@
       <c r="Z6" s="3" t="n">
         <v>384.7999877929688</v>
       </c>
+      <c r="AA6" s="3" t="n">
+        <v>375.3999938964844</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1160,13 +1178,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>228.5</v>
+        <v>225.0599975585938</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>22850</v>
+        <v>22505.99975585938</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-3583.82</v>
+        <v>-3927.820244140625</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1225,6 +1243,9 @@
       <c r="Z7" s="3" t="n">
         <v>228.5</v>
       </c>
+      <c r="AA7" s="3" t="n">
+        <v>225.0599975585938</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1271,13 +1292,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>19.1200008392334</v>
+        <v>18.90999984741211</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>28680.0012588501</v>
+        <v>28364.99977111816</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-2370.168741149901</v>
+        <v>-2685.170228881834</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1336,6 +1357,9 @@
       <c r="Z9" s="3" t="n">
         <v>19.1200008392334</v>
       </c>
+      <c r="AA9" s="3" t="n">
+        <v>18.90999984741211</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1355,13 +1379,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>479.6499938964844</v>
+        <v>481.8999938964844</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>47964.99938964844</v>
+        <v>48189.99938964844</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-3533.480610351566</v>
+        <v>-3308.480610351566</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1420,6 +1444,9 @@
       <c r="Z10" s="3" t="n">
         <v>479.6499938964844</v>
       </c>
+      <c r="AA10" s="3" t="n">
+        <v>481.8999938964844</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1439,13 +1466,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>9.550000190734863</v>
+        <v>9.079999923706055</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>9550.000190734863</v>
+        <v>9079.999923706055</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-291.2098092651358</v>
+        <v>-761.2100762939444</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -1504,6 +1531,9 @@
       <c r="Z11" s="3" t="n">
         <v>9.550000190734863</v>
       </c>
+      <c r="AA11" s="3" t="n">
+        <v>9.079999923706055</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1523,13 +1553,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2570.5</v>
+        <v>2528.89990234375</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25705</v>
+        <v>25288.9990234375</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2018.25</v>
+        <v>-2434.2509765625</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -1588,6 +1618,9 @@
       <c r="Z12" s="3" t="n">
         <v>2570.5</v>
       </c>
+      <c r="AA12" s="3" t="n">
+        <v>2528.89990234375</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1607,13 +1640,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>54.65999984741211</v>
+        <v>52.86999893188477</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>32795.99990844727</v>
+        <v>31721.99935913086</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-2235.760091552736</v>
+        <v>-3309.760640869143</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -1672,6 +1705,9 @@
       <c r="Z13" s="3" t="n">
         <v>54.65999984741211</v>
       </c>
+      <c r="AA13" s="3" t="n">
+        <v>52.86999893188477</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1691,13 +1727,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>749.2999877929688</v>
+        <v>732.1500244140625</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>37464.99938964844</v>
+        <v>36607.50122070312</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-4997.510610351565</v>
+        <v>-5855.008779296877</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -1756,6 +1792,9 @@
       <c r="Z14" s="3" t="n">
         <v>749.2999877929688</v>
       </c>
+      <c r="AA14" s="3" t="n">
+        <v>732.1500244140625</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1829,13 +1868,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>532.75</v>
+        <v>527.6500244140625</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>26637.5</v>
+        <v>26382.50122070312</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>4882.970000000001</v>
+        <v>4627.971220703126</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -1894,6 +1933,9 @@
       <c r="Z17" s="3" t="n">
         <v>532.75</v>
       </c>
+      <c r="AA17" s="3" t="n">
+        <v>527.6500244140625</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1913,13 +1955,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>420.25</v>
+        <v>409.8500061035156</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>42025</v>
+        <v>40985.00061035156</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-4615.82</v>
+        <v>-5655.819389648437</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -1978,6 +2020,9 @@
       <c r="Z18" s="3" t="n">
         <v>420.25</v>
       </c>
+      <c r="AA18" s="3" t="n">
+        <v>409.8500061035156</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -1989,10 +2034,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>561744.0025787354</v>
+        <v>556288.4975891113</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-29038.01742126466</v>
+        <v>-34493.52241088868</v>
       </c>
     </row>
   </sheetData>
@@ -2006,7 +2051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA41"/>
+  <dimension ref="A1:AB41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2036,6 +2081,7 @@
     <col width="13" customWidth="1" min="25" max="25"/>
     <col width="13" customWidth="1" min="26" max="26"/>
     <col width="13" customWidth="1" min="27" max="27"/>
+    <col width="13" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2174,6 +2220,11 @@
           <t>2026-06-01</t>
         </is>
       </c>
+      <c r="AB1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2198,16 +2249,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.9664</v>
+        <v>57.1035</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>63943.7586048</v>
+        <v>64097.650887</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>13943.7586048</v>
+        <v>14097.650887</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.278875172096</v>
+        <v>0.2819530177399999</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -2263,6 +2314,9 @@
       <c r="AA2" s="3" t="n">
         <v>56.9664</v>
       </c>
+      <c r="AB2" s="3" t="n">
+        <v>57.1035</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2287,16 +2341,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.5856</v>
+        <v>25.6542</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>62818.0977328</v>
+        <v>62986.52534460001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>2818.097732800001</v>
+        <v>2986.525344600006</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.04696829554666668</v>
+        <v>0.0497754224100001</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -2352,6 +2406,9 @@
       <c r="AA3" s="3" t="n">
         <v>25.5856</v>
       </c>
+      <c r="AB3" s="3" t="n">
+        <v>25.6542</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2376,16 +2433,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.9</v>
+        <v>12.88</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>247758.5997</v>
+        <v>247374.47784</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>67758.59970000002</v>
+        <v>67374.47784000004</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3764366650000001</v>
+        <v>0.3743026546666668</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -2441,6 +2498,9 @@
       <c r="AA4" s="3" t="n">
         <v>12.9</v>
       </c>
+      <c r="AB4" s="3" t="n">
+        <v>12.88</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2465,16 +2525,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.5251</v>
+        <v>9.463900000000001</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>174824.5236088</v>
+        <v>173701.2534232</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-35175.47639120001</v>
+        <v>-36298.74657679998</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1675022685295238</v>
+        <v>-0.172851174175238</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -2530,6 +2590,9 @@
       <c r="AA5" s="3" t="n">
         <v>9.5251</v>
       </c>
+      <c r="AB5" s="3" t="n">
+        <v>9.463900000000001</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2554,16 +2617,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.5581</v>
+        <v>12.3923</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>53107.91606369999</v>
+        <v>52406.7516771</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>3107.916063699995</v>
+        <v>2406.751677100001</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.0621583212739999</v>
+        <v>0.04813503354200002</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -2619,6 +2682,9 @@
       <c r="AA6" s="3" t="n">
         <v>12.5581</v>
       </c>
+      <c r="AB6" s="3" t="n">
+        <v>12.3923</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2643,16 +2709,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.8687</v>
+        <v>33.3466</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>74715.70694799999</v>
+        <v>73563.933464</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>14715.70694799999</v>
+        <v>13563.933464</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2452617824666665</v>
+        <v>0.2260655577333334</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -2708,6 +2774,9 @@
       <c r="AA7" s="3" t="n">
         <v>33.8687</v>
       </c>
+      <c r="AB7" s="3" t="n">
+        <v>33.3466</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2732,16 +2801,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>31.5057</v>
+        <v>31.3586</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>50553.8256801</v>
+        <v>50317.7900498</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>553.8256801000025</v>
+        <v>317.7900498000017</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.01107651360200005</v>
+        <v>0.006355800996000034</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -2797,6 +2866,9 @@
       <c r="AA8" s="3" t="n">
         <v>31.5057</v>
       </c>
+      <c r="AB8" s="3" t="n">
+        <v>31.3586</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2821,16 +2893,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>43.0068</v>
+        <v>42.4297</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>138455.7908724</v>
+        <v>136597.8791721</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>38455.79087239999</v>
+        <v>36597.87917209999</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3845579087239999</v>
+        <v>0.3659787917209999</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -2886,6 +2958,9 @@
       <c r="AA9" s="3" t="n">
         <v>43.0068</v>
       </c>
+      <c r="AB9" s="3" t="n">
+        <v>42.4297</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2910,16 +2985,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>46.3408</v>
+        <v>45.961</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>131916.4553872</v>
+        <v>130835.294299</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>31916.4553872</v>
+        <v>30835.294299</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3191645538719999</v>
+        <v>0.30835294299</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -2975,6 +3050,9 @@
       <c r="AA10" s="3" t="n">
         <v>46.3408</v>
       </c>
+      <c r="AB10" s="3" t="n">
+        <v>45.961</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2999,16 +3077,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>106.1501</v>
+        <v>106.6452</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31942.5819419</v>
+        <v>32091.5669388</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1942.581941899996</v>
+        <v>2091.566938799999</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.06475273139666654</v>
+        <v>0.06971889795999996</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -3064,6 +3142,9 @@
       <c r="AA11" s="3" t="n">
         <v>106.1501</v>
       </c>
+      <c r="AB11" s="3" t="n">
+        <v>106.6452</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3088,16 +3169,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>221.322</v>
+        <v>218.882</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>103030.260084</v>
+        <v>101894.386404</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>3030.260083999994</v>
+        <v>1894.386404000004</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.03030260083999994</v>
+        <v>0.01894386404000004</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -3153,6 +3234,9 @@
       <c r="AA12" s="3" t="n">
         <v>221.322</v>
       </c>
+      <c r="AB12" s="3" t="n">
+        <v>218.882</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3177,16 +3261,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>19.928</v>
+        <v>19.775</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>230917.79244</v>
+        <v>229144.888875</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>30917.79243999999</v>
+        <v>29144.88887499998</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.1545889622</v>
+        <v>0.1457244443749999</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -3242,6 +3326,9 @@
       <c r="AA13" s="3" t="n">
         <v>19.928</v>
       </c>
+      <c r="AB13" s="3" t="n">
+        <v>19.775</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3266,16 +3353,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>40.0376</v>
+        <v>40.4207</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>144439.8859856</v>
+        <v>145821.9598442</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>44439.88598560001</v>
+        <v>45821.9598442</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.444398859856</v>
+        <v>0.458219598442</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -3331,6 +3418,9 @@
       <c r="AA14" s="3" t="n">
         <v>40.0376</v>
       </c>
+      <c r="AB14" s="3" t="n">
+        <v>40.4207</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3355,16 +3445,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.93</v>
+        <v>11.75</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>116245.28771</v>
+        <v>114491.37725</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>16245.28771</v>
+        <v>14491.37725000001</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1624528771</v>
+        <v>0.1449137725</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -3420,6 +3510,9 @@
       <c r="AA15" s="3" t="n">
         <v>11.93</v>
       </c>
+      <c r="AB15" s="3" t="n">
+        <v>11.75</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3444,16 +3537,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>25.1815</v>
+        <v>25.1994</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>144111.911432</v>
+        <v>144214.3518432</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>44111.91143199999</v>
+        <v>44214.35184320001</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4411191143199999</v>
+        <v>0.4421435184320001</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -3509,6 +3602,9 @@
       <c r="AA16" s="3" t="n">
         <v>25.1815</v>
       </c>
+      <c r="AB16" s="3" t="n">
+        <v>25.1994</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3533,16 +3629,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.6825</v>
+        <v>16.5859</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55153.2959025</v>
+        <v>54833.9307963</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5153.295902500002</v>
+        <v>4833.930796299996</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.10306591805</v>
+        <v>0.09667861592599991</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -3598,6 +3694,9 @@
       <c r="AA17" s="3" t="n">
         <v>16.6825</v>
       </c>
+      <c r="AB17" s="3" t="n">
+        <v>16.5859</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3622,16 +3721,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>44.93</v>
+        <v>44.47</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>84757.56947999999</v>
+        <v>83889.80892</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>4757.569479999991</v>
+        <v>3889.808919999996</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.05946961849999989</v>
+        <v>0.04862261149999995</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -3687,6 +3786,9 @@
       <c r="AA18" s="3" t="n">
         <v>44.93</v>
       </c>
+      <c r="AB18" s="3" t="n">
+        <v>44.47</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3776,6 +3878,9 @@
       <c r="AA19" s="3" t="n">
         <v>15.0685</v>
       </c>
+      <c r="AB19" s="3" t="n">
+        <v>15.0685</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3800,16 +3905,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.44</v>
+        <v>9.48</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>247854.78032</v>
+        <v>248905.01244</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-2145.219680000009</v>
+        <v>-1094.98755999998</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.008580878720000037</v>
+        <v>-0.004379950239999918</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -3865,6 +3970,9 @@
       <c r="AA20" s="3" t="n">
         <v>9.44</v>
       </c>
+      <c r="AB20" s="3" t="n">
+        <v>9.48</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3889,16 +3997,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>107.9469</v>
+        <v>106.8822</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>163999.2993471</v>
+        <v>162381.7442898</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-6000.700652900006</v>
+        <v>-7618.255710199999</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.03529823913470592</v>
+        <v>-0.04481326888352941</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -3954,6 +4062,9 @@
       <c r="AA21" s="3" t="n">
         <v>107.9469</v>
       </c>
+      <c r="AB21" s="3" t="n">
+        <v>106.8822</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3978,16 +4089,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>45.346</v>
+        <v>45.698</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>69581.62316</v>
+        <v>70121.75308000001</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>9581.623160000003</v>
+        <v>10121.75308000001</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1596937193333334</v>
+        <v>0.1686958846666668</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -4043,6 +4154,9 @@
       <c r="AA22" s="3" t="n">
         <v>45.346</v>
       </c>
+      <c r="AB22" s="3" t="n">
+        <v>45.698</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4067,16 +4181,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>62.2455</v>
+        <v>61.2847</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>169087.8466485</v>
+        <v>166477.8651549</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>19087.84664850001</v>
+        <v>16477.86515490001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.1272523109900001</v>
+        <v>0.109852434366</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -4132,6 +4246,9 @@
       <c r="AA23" s="3" t="n">
         <v>62.2455</v>
       </c>
+      <c r="AB23" s="3" t="n">
+        <v>61.2847</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4156,16 +4273,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>28.4049</v>
+        <v>28.2003</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>103205.9659914</v>
+        <v>102462.5752158</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>3205.965991400008</v>
+        <v>2462.575215799996</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.03205965991400007</v>
+        <v>0.02462575215799996</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -4221,6 +4338,9 @@
       <c r="AA24" s="3" t="n">
         <v>28.4049</v>
       </c>
+      <c r="AB24" s="3" t="n">
+        <v>28.2003</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4245,16 +4365,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.3963</v>
+        <v>11.2735</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>187146.3234062</v>
+        <v>185129.741839</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-12853.67659380002</v>
+        <v>-14870.25816100001</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.06426838296900009</v>
+        <v>-0.07435129080500003</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -4310,6 +4430,9 @@
       <c r="AA25" s="3" t="n">
         <v>11.3963</v>
       </c>
+      <c r="AB25" s="3" t="n">
+        <v>11.2735</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4334,16 +4457,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>8.9869</v>
+        <v>8.9907</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>107318.9985335</v>
+        <v>107364.3770505</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>-2681.001466499991</v>
+        <v>-2635.622949500001</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>-0.02437274060454537</v>
+        <v>-0.02396020863181819</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -4399,6 +4522,9 @@
       <c r="AA26" s="3" t="n">
         <v>8.9869</v>
       </c>
+      <c r="AB26" s="3" t="n">
+        <v>8.9907</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4423,16 +4549,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>63.6173</v>
+        <v>62.9285</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>102478.563878</v>
+        <v>101369.00351</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-7521.436121999999</v>
+        <v>-8630.996490000005</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.06837669201818181</v>
+        <v>-0.0784636044545455</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -4488,6 +4614,9 @@
       <c r="AA27" s="3" t="n">
         <v>63.6173</v>
       </c>
+      <c r="AB27" s="3" t="n">
+        <v>62.9285</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4512,16 +4641,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>106.2856</v>
+        <v>104.934</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>351450.0232392</v>
+        <v>346980.745638</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-28549.9767608</v>
+        <v>-33019.25436199998</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.07513151779157894</v>
+        <v>-0.08689277463684204</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -4577,6 +4706,9 @@
       <c r="AA28" s="3" t="n">
         <v>106.2856</v>
       </c>
+      <c r="AB28" s="3" t="n">
+        <v>104.934</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4601,16 +4733,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.9376</v>
+        <v>11.698</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>114645.1649328</v>
+        <v>112344.117694</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>14645.16493279999</v>
+        <v>12344.117694</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.1464516493279999</v>
+        <v>0.12344117694</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -4666,6 +4798,9 @@
       <c r="AA29" s="3" t="n">
         <v>11.9376</v>
       </c>
+      <c r="AB29" s="3" t="n">
+        <v>11.698</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4690,16 +4825,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>15.386</v>
+        <v>15.408</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>113792.717346</v>
+        <v>113955.426288</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>13792.71734599999</v>
+        <v>13955.42628799999</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.1379271734599999</v>
+        <v>0.1395542628799999</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -4755,6 +4890,9 @@
       <c r="AA30" s="3" t="n">
         <v>15.386</v>
       </c>
+      <c r="AB30" s="3" t="n">
+        <v>15.408</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4779,16 +4917,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>418.223</v>
+        <v>410.7075</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>111280.77584</v>
+        <v>109281.0516</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>11280.77584</v>
+        <v>9281.051599999992</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.1128077584</v>
+        <v>0.09281051599999991</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -4844,6 +4982,9 @@
       <c r="AA31" s="3" t="n">
         <v>418.223</v>
       </c>
+      <c r="AB31" s="3" t="n">
+        <v>410.7075</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4868,16 +5009,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.16</v>
+        <v>10.08</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>214781.9936</v>
+        <v>213090.7968</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>14781.99359999999</v>
+        <v>13090.79679999998</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.07390996799999994</v>
+        <v>0.06545398399999991</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -4933,6 +5074,9 @@
       <c r="AA32" s="3" t="n">
         <v>10.16</v>
       </c>
+      <c r="AB32" s="3" t="n">
+        <v>10.08</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4957,16 +5101,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>17.91</v>
+        <v>17.67</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>64182.9924</v>
+        <v>63322.91880000001</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>4182.992399999996</v>
+        <v>3322.918800000007</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.06971653999999992</v>
+        <v>0.05538198000000012</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -5022,6 +5166,9 @@
       <c r="AA33" s="3" t="n">
         <v>17.91</v>
       </c>
+      <c r="AB33" s="3" t="n">
+        <v>17.67</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -5046,16 +5193,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>214.5933</v>
+        <v>216.7483</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>75436.1973423</v>
+        <v>76193.74664729999</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-4563.802657699998</v>
+        <v>-3806.253352700005</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.05704753322124998</v>
+        <v>-0.04757816690875007</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -5111,6 +5258,9 @@
       <c r="AA34" s="3" t="n">
         <v>214.5933</v>
       </c>
+      <c r="AB34" s="3" t="n">
+        <v>216.7483</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -5135,16 +5285,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>14.49</v>
+        <v>14.22</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>103392.27927</v>
+        <v>101465.71506</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>3392.279269999999</v>
+        <v>1465.715060000002</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.03392279269999999</v>
+        <v>0.01465715060000002</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -5200,6 +5350,9 @@
       <c r="AA35" s="3" t="n">
         <v>14.49</v>
       </c>
+      <c r="AB35" s="3" t="n">
+        <v>14.22</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5224,16 +5377,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>349.2681</v>
+        <v>345.9498</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>162656.2497786</v>
+        <v>161110.8975588</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>12656.2497786</v>
+        <v>11110.8975588</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.08437499852400002</v>
+        <v>0.07407265039200002</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -5289,6 +5442,9 @@
       <c r="AA36" s="3" t="n">
         <v>349.2681</v>
       </c>
+      <c r="AB36" s="3" t="n">
+        <v>345.9498</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5313,16 +5469,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>15.569</v>
+        <v>15.519</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>58584.41884100001</v>
+        <v>58396.274391</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>8584.418841000006</v>
+        <v>8396.274390999999</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.1716883768200001</v>
+        <v>0.16792548782</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -5378,6 +5534,9 @@
       <c r="AA37" s="3" t="n">
         <v>15.569</v>
       </c>
+      <c r="AB37" s="3" t="n">
+        <v>15.519</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5402,16 +5561,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>14.0646</v>
+        <v>13.9077</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>84113.0871372</v>
+        <v>83174.7495114</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>4113.087137199997</v>
+        <v>3174.749511400005</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.05141358921499996</v>
+        <v>0.03968436889250006</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -5467,6 +5626,9 @@
       <c r="AA38" s="3" t="n">
         <v>14.0646</v>
       </c>
+      <c r="AB38" s="3" t="n">
+        <v>13.9077</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5491,16 +5653,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1009.4228</v>
+        <v>1009.5209</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50351.0186868</v>
+        <v>50355.9120129</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>351.0186868000019</v>
+        <v>355.9120129000003</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.007020373736000038</v>
+        <v>0.007118240258000006</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -5556,6 +5718,9 @@
       <c r="AA39" s="3" t="n">
         <v>1009.4228</v>
       </c>
+      <c r="AB39" s="3" t="n">
+        <v>1009.5209</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5580,16 +5745,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>20.4837</v>
+        <v>20.2023</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>103258.8847599</v>
+        <v>101840.3397621</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>3258.8847599</v>
+        <v>1840.339762100004</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.032588847599</v>
+        <v>0.01840339762100004</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -5645,6 +5810,9 @@
       <c r="AA40" s="3" t="n">
         <v>20.4837</v>
       </c>
+      <c r="AB40" s="3" t="n">
+        <v>20.2023</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
@@ -5656,13 +5824,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4885284.9275033</v>
+        <v>4851981.0548428</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>415284.9275033</v>
+        <v>381981.0548428001</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.09290490548172259</v>
+        <v>0.08545437468519017</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-06-03
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-02 06:40 IST</t>
+          <t>Generated: 2026-06-03 06:51 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4851981.0548428</v>
+        <v>4890641.2703557</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>381981.0548427999</v>
+        <v>420641.2703556996</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.08545437468519014</v>
+        <v>0.09410319247331086</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>556288.4975891113</v>
+        <v>558969.4989852905</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-34493.52241088869</v>
+        <v>-31812.52101470949</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.05838620886073799</v>
+        <v>-0.05384815369755073</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5408269.552431911</v>
+        <v>5449610.76934099</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>347487.5324319117</v>
+        <v>388828.7493409906</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.0686628135846704</v>
+        <v>0.07683175205024748</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-06-02</t>
+          <t>Last snapshot: 2026-06-03</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA19"/>
+  <dimension ref="A1:AB19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -646,6 +646,7 @@
     <col width="20" customWidth="1" min="25" max="25"/>
     <col width="21" customWidth="1" min="26" max="26"/>
     <col width="21" customWidth="1" min="27" max="27"/>
+    <col width="21" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -784,6 +785,11 @@
           <t>2026-06-02</t>
         </is>
       </c>
+      <c r="AB1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -803,13 +809,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>590.3499755859375</v>
+        <v>595.0499877929688</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>47227.998046875</v>
+        <v>47603.9990234375</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>3410.488046874998</v>
+        <v>3786.489023437498</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -871,6 +877,9 @@
       <c r="AA2" s="3" t="n">
         <v>590.3499755859375</v>
       </c>
+      <c r="AB2" s="3" t="n">
+        <v>595.0499877929688</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -917,13 +926,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1494.099975585938</v>
+        <v>1529.5</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>29881.99951171875</v>
+        <v>30590</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-2222.580488281252</v>
+        <v>-1514.580000000002</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -985,6 +994,9 @@
       <c r="AA4" s="3" t="n">
         <v>1494.099975585938</v>
       </c>
+      <c r="AB4" s="3" t="n">
+        <v>1529.5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1004,13 +1016,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>663.25</v>
+        <v>648</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13265</v>
+        <v>12960</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-948.1000000000004</v>
+        <v>-1253.1</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1072,6 +1084,9 @@
       <c r="AA5" s="3" t="n">
         <v>663.25</v>
       </c>
+      <c r="AB5" s="3" t="n">
+        <v>648</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1091,13 +1106,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>375.3999938964844</v>
+        <v>371.25</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15015.99975585938</v>
+        <v>14850</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2486.240244140627</v>
+        <v>-2652.240000000002</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1159,6 +1174,9 @@
       <c r="AA6" s="3" t="n">
         <v>375.3999938964844</v>
       </c>
+      <c r="AB6" s="3" t="n">
+        <v>371.25</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1178,13 +1196,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>225.0599975585938</v>
+        <v>222</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>22505.99975585938</v>
+        <v>22200</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-3927.820244140625</v>
+        <v>-4233.82</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1246,6 +1264,9 @@
       <c r="AA7" s="3" t="n">
         <v>225.0599975585938</v>
       </c>
+      <c r="AB7" s="3" t="n">
+        <v>222</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1292,13 +1313,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>18.90999984741211</v>
+        <v>18.88999938964844</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>28364.99977111816</v>
+        <v>28334.99908447266</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-2685.170228881834</v>
+        <v>-2715.170915527342</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1360,6 +1381,9 @@
       <c r="AA9" s="3" t="n">
         <v>18.90999984741211</v>
       </c>
+      <c r="AB9" s="3" t="n">
+        <v>18.88999938964844</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1379,13 +1403,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>481.8999938964844</v>
+        <v>491.1499938964844</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48189.99938964844</v>
+        <v>49114.99938964844</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-3308.480610351566</v>
+        <v>-2383.480610351566</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1447,6 +1471,9 @@
       <c r="AA10" s="3" t="n">
         <v>481.8999938964844</v>
       </c>
+      <c r="AB10" s="3" t="n">
+        <v>491.1499938964844</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1466,13 +1493,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>9.079999923706055</v>
+        <v>9.060000419616699</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>9079.999923706055</v>
+        <v>9060.000419616699</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-761.2100762939444</v>
+        <v>-781.2095803832999</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -1534,6 +1561,9 @@
       <c r="AA11" s="3" t="n">
         <v>9.079999923706055</v>
       </c>
+      <c r="AB11" s="3" t="n">
+        <v>9.060000419616699</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1553,13 +1583,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2528.89990234375</v>
+        <v>2564.300048828125</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25288.9990234375</v>
+        <v>25643.00048828125</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2434.2509765625</v>
+        <v>-2080.24951171875</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -1621,6 +1651,9 @@
       <c r="AA12" s="3" t="n">
         <v>2528.89990234375</v>
       </c>
+      <c r="AB12" s="3" t="n">
+        <v>2564.300048828125</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1640,13 +1673,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>52.86999893188477</v>
+        <v>53.36999893188477</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>31721.99935913086</v>
+        <v>32021.99935913086</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-3309.760640869143</v>
+        <v>-3009.760640869143</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -1708,6 +1741,9 @@
       <c r="AA13" s="3" t="n">
         <v>52.86999893188477</v>
       </c>
+      <c r="AB13" s="3" t="n">
+        <v>53.36999893188477</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1727,13 +1763,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>732.1500244140625</v>
+        <v>718.9000244140625</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>36607.50122070312</v>
+        <v>35945.00122070312</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-5855.008779296877</v>
+        <v>-6517.508779296877</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -1795,6 +1831,9 @@
       <c r="AA14" s="3" t="n">
         <v>732.1500244140625</v>
       </c>
+      <c r="AB14" s="3" t="n">
+        <v>718.9000244140625</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1868,13 +1907,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>527.6500244140625</v>
+        <v>560.4000244140625</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>26382.50122070312</v>
+        <v>28020.00122070312</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>4627.971220703126</v>
+        <v>6265.471220703126</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -1936,6 +1975,9 @@
       <c r="AA17" s="3" t="n">
         <v>527.6500244140625</v>
       </c>
+      <c r="AB17" s="3" t="n">
+        <v>560.4000244140625</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1955,13 +1997,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>409.8500061035156</v>
+        <v>408.5499877929688</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>40985.00061035156</v>
+        <v>40854.99877929688</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-5655.819389648437</v>
+        <v>-5785.821220703125</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -2023,6 +2065,9 @@
       <c r="AA18" s="3" t="n">
         <v>409.8500061035156</v>
       </c>
+      <c r="AB18" s="3" t="n">
+        <v>408.5499877929688</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -2034,10 +2079,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>556288.4975891113</v>
+        <v>558969.4989852905</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-34493.52241088868</v>
+        <v>-31812.52101470948</v>
       </c>
     </row>
   </sheetData>
@@ -2051,7 +2096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB41"/>
+  <dimension ref="A1:AC41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2082,6 +2127,7 @@
     <col width="13" customWidth="1" min="26" max="26"/>
     <col width="13" customWidth="1" min="27" max="27"/>
     <col width="13" customWidth="1" min="28" max="28"/>
+    <col width="13" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2225,6 +2271,11 @@
           <t>2026-06-02</t>
         </is>
       </c>
+      <c r="AC1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2249,16 +2300,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>57.1035</v>
+        <v>57.6501</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>64097.650887</v>
+        <v>64711.1995482</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>14097.650887</v>
+        <v>14711.1995482</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.2819530177399999</v>
+        <v>0.294223990964</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -2317,6 +2368,9 @@
       <c r="AB2" s="3" t="n">
         <v>57.1035</v>
       </c>
+      <c r="AC2" s="3" t="n">
+        <v>57.6501</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2341,16 +2395,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.6542</v>
+        <v>25.7192</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>62986.52534460001</v>
+        <v>63146.1141896</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>2986.525344600006</v>
+        <v>3146.114189600004</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.0497754224100001</v>
+        <v>0.05243523649333341</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -2409,6 +2463,9 @@
       <c r="AB3" s="3" t="n">
         <v>25.6542</v>
       </c>
+      <c r="AC3" s="3" t="n">
+        <v>25.7192</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2433,16 +2490,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.88</v>
+        <v>13.06</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>247374.47784</v>
+        <v>250831.57458</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>67374.47784000004</v>
+        <v>70831.57458000001</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3743026546666668</v>
+        <v>0.3935087476666668</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -2501,6 +2558,9 @@
       <c r="AB4" s="3" t="n">
         <v>12.88</v>
       </c>
+      <c r="AC4" s="3" t="n">
+        <v>13.06</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2525,16 +2585,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.463900000000001</v>
+        <v>9.5745</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>173701.2534232</v>
+        <v>175731.215556</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-36298.74657679998</v>
+        <v>-34268.78444399999</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.172851174175238</v>
+        <v>-0.1631846878285714</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -2593,6 +2653,9 @@
       <c r="AB5" s="3" t="n">
         <v>9.463900000000001</v>
       </c>
+      <c r="AC5" s="3" t="n">
+        <v>9.5745</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2617,16 +2680,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.3923</v>
+        <v>12.333</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>52406.7516771</v>
+        <v>52155.973341</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>2406.751677100001</v>
+        <v>2155.973340999997</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.04813503354200002</v>
+        <v>0.04311946681999995</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -2685,6 +2748,9 @@
       <c r="AB6" s="3" t="n">
         <v>12.3923</v>
       </c>
+      <c r="AC6" s="3" t="n">
+        <v>12.333</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2709,16 +2775,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.3466</v>
+        <v>33.6596</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>73563.933464</v>
+        <v>74254.42398399999</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>13563.933464</v>
+        <v>14254.42398399999</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2260655577333334</v>
+        <v>0.2375737330666666</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -2777,6 +2843,9 @@
       <c r="AB7" s="3" t="n">
         <v>33.3466</v>
       </c>
+      <c r="AC7" s="3" t="n">
+        <v>33.6596</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2801,16 +2870,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>31.3586</v>
+        <v>31.7475</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>50317.7900498</v>
+        <v>50941.8162675</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>317.7900498000017</v>
+        <v>941.8162674999985</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.006355800996000034</v>
+        <v>0.01883632534999997</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -2869,6 +2938,9 @@
       <c r="AB8" s="3" t="n">
         <v>31.3586</v>
       </c>
+      <c r="AC8" s="3" t="n">
+        <v>31.7475</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2893,16 +2965,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>42.4297</v>
+        <v>43.7553</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>136597.8791721</v>
+        <v>140865.5065329</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>36597.87917209999</v>
+        <v>40865.50653290001</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3659787917209999</v>
+        <v>0.4086550653290001</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -2961,6 +3033,9 @@
       <c r="AB9" s="3" t="n">
         <v>42.4297</v>
       </c>
+      <c r="AC9" s="3" t="n">
+        <v>43.7553</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2985,16 +3060,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>45.961</v>
+        <v>46.1869</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>130835.294299</v>
+        <v>131478.3545671</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>30835.294299</v>
+        <v>31478.3545671</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.30835294299</v>
+        <v>0.314783545671</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -3053,6 +3128,9 @@
       <c r="AB10" s="3" t="n">
         <v>45.961</v>
       </c>
+      <c r="AC10" s="3" t="n">
+        <v>46.1869</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3077,16 +3155,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>106.6452</v>
+        <v>107.3247</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>32091.5669388</v>
+        <v>32296.0413993</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>2091.566938799999</v>
+        <v>2296.0413993</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.06971889795999996</v>
+        <v>0.07653471331</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -3145,6 +3223,9 @@
       <c r="AB11" s="3" t="n">
         <v>106.6452</v>
       </c>
+      <c r="AC11" s="3" t="n">
+        <v>107.3247</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3169,16 +3250,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>218.882</v>
+        <v>219.673</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>101894.386404</v>
+        <v>102262.614306</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>1894.386404000004</v>
+        <v>2262.614306000003</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.01894386404000004</v>
+        <v>0.02262614306000003</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -3237,6 +3318,9 @@
       <c r="AB12" s="3" t="n">
         <v>218.882</v>
       </c>
+      <c r="AC12" s="3" t="n">
+        <v>219.673</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3261,16 +3345,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>19.775</v>
+        <v>19.779</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>229144.888875</v>
+        <v>229191.239295</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>29144.88887499998</v>
+        <v>29191.23929499998</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.1457244443749999</v>
+        <v>0.1459561964749999</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -3329,6 +3413,9 @@
       <c r="AB13" s="3" t="n">
         <v>19.775</v>
       </c>
+      <c r="AC13" s="3" t="n">
+        <v>19.779</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3353,16 +3440,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>40.4207</v>
+        <v>40.98</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>145821.9598442</v>
+        <v>147839.69388</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>45821.9598442</v>
+        <v>47839.69388000001</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.458219598442</v>
+        <v>0.4783969388000001</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -3421,6 +3508,9 @@
       <c r="AB14" s="3" t="n">
         <v>40.4207</v>
       </c>
+      <c r="AC14" s="3" t="n">
+        <v>40.98</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3445,16 +3535,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.75</v>
+        <v>11.74</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>114491.37725</v>
+        <v>114393.93778</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>14491.37725000001</v>
+        <v>14393.93778000001</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1449137725</v>
+        <v>0.1439393778000001</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -3513,6 +3603,9 @@
       <c r="AB15" s="3" t="n">
         <v>11.75</v>
       </c>
+      <c r="AC15" s="3" t="n">
+        <v>11.74</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3537,16 +3630,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>25.1994</v>
+        <v>25.3949</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>144214.3518432</v>
+        <v>145333.1842672</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>44214.35184320001</v>
+        <v>45333.18426720001</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4421435184320001</v>
+        <v>0.4533318426720001</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -3605,6 +3698,9 @@
       <c r="AB16" s="3" t="n">
         <v>25.1994</v>
       </c>
+      <c r="AC16" s="3" t="n">
+        <v>25.3949</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3629,16 +3725,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.5859</v>
+        <v>16.6895</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>54833.9307963</v>
+        <v>55176.43830149999</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>4833.930796299996</v>
+        <v>5176.438301499991</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.09667861592599991</v>
+        <v>0.1035287660299998</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -3697,6 +3793,9 @@
       <c r="AB17" s="3" t="n">
         <v>16.5859</v>
       </c>
+      <c r="AC17" s="3" t="n">
+        <v>16.6895</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3721,16 +3820,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>44.47</v>
+        <v>44.34</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>83889.80892</v>
+        <v>83644.57224000001</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>3889.808919999996</v>
+        <v>3644.572240000009</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.04862261149999995</v>
+        <v>0.04555715300000011</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -3789,6 +3888,9 @@
       <c r="AB18" s="3" t="n">
         <v>44.47</v>
       </c>
+      <c r="AC18" s="3" t="n">
+        <v>44.34</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3813,16 +3915,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>15.0685</v>
+        <v>15.2629</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>217992.463471</v>
+        <v>220804.8027814</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>67992.463471</v>
+        <v>70804.80278140001</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.4532830898066667</v>
+        <v>0.4720320185426667</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -3881,6 +3983,9 @@
       <c r="AB19" s="3" t="n">
         <v>15.0685</v>
       </c>
+      <c r="AC19" s="3" t="n">
+        <v>15.2629</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3905,16 +4010,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.48</v>
+        <v>9.65</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>248905.01244</v>
-      </c>
-      <c r="H20" s="6" t="n">
-        <v>-1094.98755999998</v>
-      </c>
-      <c r="I20" s="13" t="n">
-        <v>-0.004379950239999918</v>
+        <v>253368.49895</v>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>3368.498950000008</v>
+      </c>
+      <c r="I20" s="12" t="n">
+        <v>0.01347399580000003</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -3973,6 +4078,9 @@
       <c r="AB20" s="3" t="n">
         <v>9.48</v>
       </c>
+      <c r="AC20" s="3" t="n">
+        <v>9.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3997,16 +4105,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>106.8822</v>
+        <v>107.3466</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>162381.7442898</v>
+        <v>163087.2881694</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-7618.255710199999</v>
+        <v>-6912.711830600019</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.04481326888352941</v>
+        <v>-0.04066301076823541</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -4065,6 +4173,9 @@
       <c r="AB21" s="3" t="n">
         <v>106.8822</v>
       </c>
+      <c r="AC21" s="3" t="n">
+        <v>107.3466</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4089,16 +4200,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>45.698</v>
+        <v>46.101</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>70121.75308000001</v>
+        <v>70740.14046</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>10121.75308000001</v>
+        <v>10740.14046</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1686958846666668</v>
+        <v>0.1790023409999999</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -4157,6 +4268,9 @@
       <c r="AB22" s="3" t="n">
         <v>45.698</v>
       </c>
+      <c r="AC22" s="3" t="n">
+        <v>46.101</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4181,16 +4295,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>61.2847</v>
+        <v>61.0741</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>166477.8651549</v>
+        <v>165905.7772047</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>16477.86515490001</v>
+        <v>15905.77720470002</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.109852434366</v>
+        <v>0.1060385146980001</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -4249,6 +4363,9 @@
       <c r="AB23" s="3" t="n">
         <v>61.2847</v>
       </c>
+      <c r="AC23" s="3" t="n">
+        <v>61.0741</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4273,16 +4390,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>28.2003</v>
+        <v>28.2266</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>102462.5752158</v>
+        <v>102558.1332676</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>2462.575215799996</v>
+        <v>2558.133267600002</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.02462575215799996</v>
+        <v>0.02558133267600002</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -4341,6 +4458,9 @@
       <c r="AB24" s="3" t="n">
         <v>28.2003</v>
       </c>
+      <c r="AC24" s="3" t="n">
+        <v>28.2266</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4365,16 +4485,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.2735</v>
+        <v>11.3922</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>185129.741839</v>
+        <v>187078.9945428</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-14870.25816100001</v>
+        <v>-12921.00545719999</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.07435129080500003</v>
+        <v>-0.06460502728599997</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -4433,6 +4553,9 @@
       <c r="AB25" s="3" t="n">
         <v>11.2735</v>
       </c>
+      <c r="AC25" s="3" t="n">
+        <v>11.3922</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4457,16 +4580,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>8.9907</v>
+        <v>9.1944</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>107364.3770505</v>
+        <v>109796.904396</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>-2635.622949500001</v>
+        <v>-203.0956040000019</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>-0.02396020863181819</v>
+        <v>-0.00184632367272729</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -4525,6 +4648,9 @@
       <c r="AB26" s="3" t="n">
         <v>8.9907</v>
       </c>
+      <c r="AC26" s="3" t="n">
+        <v>9.1944</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4549,16 +4675,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>62.9285</v>
+        <v>63.5109</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>101369.00351</v>
+        <v>102307.168374</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-8630.996490000005</v>
+        <v>-7692.831626000014</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.0784636044545455</v>
+        <v>-0.06993483296363649</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -4617,6 +4743,9 @@
       <c r="AB27" s="3" t="n">
         <v>62.9285</v>
       </c>
+      <c r="AC27" s="3" t="n">
+        <v>63.5109</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4641,16 +4770,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>104.934</v>
+        <v>105.6391</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>346980.745638</v>
+        <v>349312.2694887</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-33019.25436199998</v>
+        <v>-30687.73051129997</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.08689277463684204</v>
+        <v>-0.08075718555605256</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -4709,6 +4838,9 @@
       <c r="AB28" s="3" t="n">
         <v>104.934</v>
       </c>
+      <c r="AC28" s="3" t="n">
+        <v>105.6391</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4733,16 +4865,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.698</v>
+        <v>11.7844</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>112344.117694</v>
+        <v>113173.8776332</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>12344.117694</v>
+        <v>13173.8776332</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.12344117694</v>
+        <v>0.131738776332</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -4801,6 +4933,9 @@
       <c r="AB29" s="3" t="n">
         <v>11.698</v>
       </c>
+      <c r="AC29" s="3" t="n">
+        <v>11.7844</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4825,16 +4960,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>15.408</v>
+        <v>15.6143</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>113955.426288</v>
+        <v>115481.1924123</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>13955.42628799999</v>
+        <v>15481.19241229999</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.1395542628799999</v>
+        <v>0.1548119241229999</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -4893,6 +5028,9 @@
       <c r="AB30" s="3" t="n">
         <v>15.408</v>
       </c>
+      <c r="AC30" s="3" t="n">
+        <v>15.6143</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4917,16 +5055,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>410.7075</v>
+        <v>411.9591</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>109281.0516</v>
+        <v>109614.077328</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>9281.051599999992</v>
+        <v>9614.077327999985</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.09281051599999991</v>
+        <v>0.09614077327999984</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -4985,6 +5123,9 @@
       <c r="AB31" s="3" t="n">
         <v>410.7075</v>
       </c>
+      <c r="AC31" s="3" t="n">
+        <v>411.9591</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -5009,16 +5150,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.08</v>
+        <v>10.15</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>213090.7968</v>
+        <v>214570.594</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>13090.79679999998</v>
+        <v>14570.59400000001</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.06545398399999991</v>
+        <v>0.07285297000000006</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -5077,6 +5218,9 @@
       <c r="AB32" s="3" t="n">
         <v>10.08</v>
       </c>
+      <c r="AC32" s="3" t="n">
+        <v>10.15</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -5101,16 +5245,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>17.67</v>
+        <v>17.78</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>63322.91880000001</v>
+        <v>63717.1192</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>3322.918800000007</v>
+        <v>3717.119200000001</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.05538198000000012</v>
+        <v>0.06195198666666668</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -5169,6 +5313,9 @@
       <c r="AB33" s="3" t="n">
         <v>17.67</v>
       </c>
+      <c r="AC33" s="3" t="n">
+        <v>17.78</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -5193,16 +5340,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>216.7483</v>
+        <v>220.5786</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>76193.74664729999</v>
+        <v>77540.21583659999</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-3806.253352700005</v>
+        <v>-2459.784163400007</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.04757816690875007</v>
+        <v>-0.03074730204250009</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -5261,6 +5408,9 @@
       <c r="AB34" s="3" t="n">
         <v>216.7483</v>
       </c>
+      <c r="AC34" s="3" t="n">
+        <v>220.5786</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -5285,16 +5435,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>14.22</v>
+        <v>14.37</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>101465.71506</v>
+        <v>102536.02851</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>1465.715060000002</v>
+        <v>2536.028509999989</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.01465715060000002</v>
+        <v>0.02536028509999989</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -5353,6 +5503,9 @@
       <c r="AB35" s="3" t="n">
         <v>14.22</v>
       </c>
+      <c r="AC35" s="3" t="n">
+        <v>14.37</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5377,16 +5530,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>345.9498</v>
+        <v>345.5958</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>161110.8975588</v>
+        <v>160946.0376348</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>11110.8975588</v>
+        <v>10946.03763480001</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.07407265039200002</v>
+        <v>0.07297358423200009</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -5445,6 +5598,9 @@
       <c r="AB36" s="3" t="n">
         <v>345.9498</v>
       </c>
+      <c r="AC36" s="3" t="n">
+        <v>345.5958</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5469,16 +5625,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>15.519</v>
+        <v>15.455</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>58396.274391</v>
+        <v>58155.449495</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>8396.274390999999</v>
+        <v>8155.449495000001</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.16792548782</v>
+        <v>0.1631089899</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -5537,6 +5693,9 @@
       <c r="AB37" s="3" t="n">
         <v>15.519</v>
       </c>
+      <c r="AC37" s="3" t="n">
+        <v>15.455</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5561,16 +5720,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.9077</v>
+        <v>13.9479</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>83174.7495114</v>
+        <v>83415.1648878</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>3174.749511400005</v>
+        <v>3415.164887799998</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.03968436889250006</v>
+        <v>0.04268956109749997</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -5629,6 +5788,9 @@
       <c r="AB38" s="3" t="n">
         <v>13.9077</v>
       </c>
+      <c r="AC38" s="3" t="n">
+        <v>13.9479</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5653,16 +5815,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1009.5209</v>
+        <v>1010.7179</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50355.9120129</v>
+        <v>50415.6195699</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>355.9120129000003</v>
+        <v>415.6195699000018</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.007118240258000006</v>
+        <v>0.008312391398000036</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -5721,6 +5883,9 @@
       <c r="AB39" s="3" t="n">
         <v>1009.5209</v>
       </c>
+      <c r="AC39" s="3" t="n">
+        <v>1010.7179</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5745,16 +5910,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>20.2023</v>
+        <v>20.2066</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>101840.3397621</v>
+        <v>101862.0161782</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>1840.339762100004</v>
+        <v>1862.016178200007</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.01840339762100004</v>
+        <v>0.01862016178200007</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -5813,6 +5978,9 @@
       <c r="AB40" s="3" t="n">
         <v>20.2023</v>
       </c>
+      <c r="AC40" s="3" t="n">
+        <v>20.2066</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
@@ -5824,13 +5992,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4851981.0548428</v>
+        <v>4890641.2703557</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>381981.0548428001</v>
+        <v>420641.2703557</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.08545437468519017</v>
+        <v>0.09410319247331098</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-06-04
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-03 06:51 IST</t>
+          <t>Generated: 2026-06-04 06:41 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4890641.2703557</v>
+        <v>4877136.4413211</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>420641.2703556996</v>
+        <v>407136.4413211001</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.09410319247331086</v>
+        <v>0.09108197792418347</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>558969.4989852905</v>
+        <v>567987.4966125488</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-31812.52101470949</v>
+        <v>-22794.52338745119</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.05384815369755073</v>
+        <v>-0.03858364441668551</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5449610.76934099</v>
+        <v>5445123.937933649</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>388828.7493409906</v>
+        <v>384341.9179336494</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.07683175205024748</v>
+        <v>0.07594516349740932</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-06-03</t>
+          <t>Last snapshot: 2026-06-04</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB19"/>
+  <dimension ref="A1:AC19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -647,6 +647,7 @@
     <col width="21" customWidth="1" min="26" max="26"/>
     <col width="21" customWidth="1" min="27" max="27"/>
     <col width="21" customWidth="1" min="28" max="28"/>
+    <col width="21" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -790,6 +791,11 @@
           <t>2026-06-03</t>
         </is>
       </c>
+      <c r="AC1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -809,13 +815,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>595.0499877929688</v>
+        <v>601.5</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>47603.9990234375</v>
+        <v>48120</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>3786.489023437498</v>
+        <v>4302.489999999998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -880,6 +886,9 @@
       <c r="AB2" s="3" t="n">
         <v>595.0499877929688</v>
       </c>
+      <c r="AC2" s="3" t="n">
+        <v>601.5</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -926,13 +935,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1529.5</v>
+        <v>1544.199951171875</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>30590</v>
+        <v>30883.9990234375</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-1514.580000000002</v>
+        <v>-1220.580976562502</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -997,6 +1006,9 @@
       <c r="AB4" s="3" t="n">
         <v>1529.5</v>
       </c>
+      <c r="AC4" s="3" t="n">
+        <v>1544.199951171875</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1016,13 +1028,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>648</v>
+        <v>650</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>12960</v>
+        <v>13000</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1253.1</v>
+        <v>-1213.1</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1087,6 +1099,9 @@
       <c r="AB5" s="3" t="n">
         <v>648</v>
       </c>
+      <c r="AC5" s="3" t="n">
+        <v>650</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1106,13 +1121,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>371.25</v>
+        <v>383.5</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>14850</v>
+        <v>15340</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2652.240000000002</v>
+        <v>-2162.240000000002</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1177,6 +1192,9 @@
       <c r="AB6" s="3" t="n">
         <v>371.25</v>
       </c>
+      <c r="AC6" s="3" t="n">
+        <v>383.5</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1196,13 +1214,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>222</v>
+        <v>236.3800048828125</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>22200</v>
+        <v>23638.00048828125</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-4233.82</v>
+        <v>-2795.81951171875</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1267,6 +1285,9 @@
       <c r="AB7" s="3" t="n">
         <v>222</v>
       </c>
+      <c r="AC7" s="3" t="n">
+        <v>236.3800048828125</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1313,13 +1334,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>18.88999938964844</v>
+        <v>19.22999954223633</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>28334.99908447266</v>
+        <v>28844.99931335449</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-2715.170915527342</v>
+        <v>-2205.170686645506</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1384,6 +1405,9 @@
       <c r="AB9" s="3" t="n">
         <v>18.88999938964844</v>
       </c>
+      <c r="AC9" s="3" t="n">
+        <v>19.22999954223633</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1403,13 +1427,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>491.1499938964844</v>
+        <v>490.5499877929688</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>49114.99938964844</v>
+        <v>49054.99877929688</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-2383.480610351566</v>
+        <v>-2443.481220703128</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1474,6 +1498,9 @@
       <c r="AB10" s="3" t="n">
         <v>491.1499938964844</v>
       </c>
+      <c r="AC10" s="3" t="n">
+        <v>490.5499877929688</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1493,13 +1520,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>9.060000419616699</v>
+        <v>9.420000076293945</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>9060.000419616699</v>
+        <v>9420.000076293945</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-781.2095803832999</v>
+        <v>-421.2099237060538</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -1564,6 +1591,9 @@
       <c r="AB11" s="3" t="n">
         <v>9.060000419616699</v>
       </c>
+      <c r="AC11" s="3" t="n">
+        <v>9.420000076293945</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1583,13 +1613,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2564.300048828125</v>
+        <v>2657.10009765625</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25643.00048828125</v>
+        <v>26571.0009765625</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2080.24951171875</v>
+        <v>-1152.2490234375</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -1654,6 +1684,9 @@
       <c r="AB12" s="3" t="n">
         <v>2564.300048828125</v>
       </c>
+      <c r="AC12" s="3" t="n">
+        <v>2657.10009765625</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1673,13 +1706,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>53.36999893188477</v>
+        <v>55.18999862670898</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>32021.99935913086</v>
+        <v>33113.99917602539</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-3009.760640869143</v>
+        <v>-1917.760823974611</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -1744,6 +1777,9 @@
       <c r="AB13" s="3" t="n">
         <v>53.36999893188477</v>
       </c>
+      <c r="AC13" s="3" t="n">
+        <v>55.18999862670898</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1763,13 +1799,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>718.9000244140625</v>
+        <v>724</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>35945.00122070312</v>
+        <v>36200</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-6517.508779296877</v>
+        <v>-6262.510000000002</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -1834,6 +1870,9 @@
       <c r="AB14" s="3" t="n">
         <v>718.9000244140625</v>
       </c>
+      <c r="AC14" s="3" t="n">
+        <v>724</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1907,13 +1946,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>560.4000244140625</v>
+        <v>615.2999877929688</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>28020.00122070312</v>
+        <v>30764.99938964844</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>6265.471220703126</v>
+        <v>9010.469389648439</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -1978,6 +2017,9 @@
       <c r="AB17" s="3" t="n">
         <v>560.4000244140625</v>
       </c>
+      <c r="AC17" s="3" t="n">
+        <v>615.2999877929688</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1997,13 +2039,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>408.5499877929688</v>
+        <v>412.6499938964844</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>40854.99877929688</v>
+        <v>41264.99938964844</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-5785.821220703125</v>
+        <v>-5375.820610351562</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -2068,6 +2110,9 @@
       <c r="AB18" s="3" t="n">
         <v>408.5499877929688</v>
       </c>
+      <c r="AC18" s="3" t="n">
+        <v>412.6499938964844</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -2079,10 +2124,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>558969.4989852905</v>
+        <v>567987.4966125488</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-31812.52101470948</v>
+        <v>-22794.52338745118</v>
       </c>
     </row>
   </sheetData>
@@ -2096,7 +2141,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC41"/>
+  <dimension ref="A1:AD41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2128,6 +2173,7 @@
     <col width="13" customWidth="1" min="27" max="27"/>
     <col width="13" customWidth="1" min="28" max="28"/>
     <col width="13" customWidth="1" min="29" max="29"/>
+    <col width="13" customWidth="1" min="30" max="30"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2276,6 +2322,11 @@
           <t>2026-06-03</t>
         </is>
       </c>
+      <c r="AD1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2300,16 +2351,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>57.6501</v>
+        <v>57.5427</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>64711.1995482</v>
+        <v>64590.6449814</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>14711.1995482</v>
+        <v>14590.6449814</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.294223990964</v>
+        <v>0.291812899628</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -2371,6 +2422,9 @@
       <c r="AC2" s="3" t="n">
         <v>57.6501</v>
       </c>
+      <c r="AD2" s="3" t="n">
+        <v>57.5427</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2395,16 +2449,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.7192</v>
+        <v>25.88</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>63146.1141896</v>
+        <v>63540.91244</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>3146.114189600004</v>
+        <v>3540.91244</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.05243523649333341</v>
+        <v>0.05901520733333333</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -2466,6 +2520,9 @@
       <c r="AC3" s="3" t="n">
         <v>25.7192</v>
       </c>
+      <c r="AD3" s="3" t="n">
+        <v>25.88</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2490,16 +2547,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>13.06</v>
+        <v>13.05</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>250831.57458</v>
+        <v>250639.51365</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>70831.57458000001</v>
+        <v>70639.51365000004</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3935087476666668</v>
+        <v>0.3924417425000002</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -2561,6 +2618,9 @@
       <c r="AC4" s="3" t="n">
         <v>13.06</v>
       </c>
+      <c r="AD4" s="3" t="n">
+        <v>13.05</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2585,16 +2645,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.5745</v>
+        <v>9.4147</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>175731.215556</v>
+        <v>172798.2322936</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-34268.78444399999</v>
+        <v>-37201.76770640002</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1631846878285714</v>
+        <v>-0.177151274792381</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -2656,6 +2716,9 @@
       <c r="AC5" s="3" t="n">
         <v>9.5745</v>
       </c>
+      <c r="AD5" s="3" t="n">
+        <v>9.4147</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2680,16 +2743,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.333</v>
+        <v>12.3744</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>52155.973341</v>
+        <v>52331.05298879999</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>2155.973340999997</v>
+        <v>2331.052988799995</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.04311946681999995</v>
+        <v>0.0466210597759999</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -2751,6 +2814,9 @@
       <c r="AC6" s="3" t="n">
         <v>12.333</v>
       </c>
+      <c r="AD6" s="3" t="n">
+        <v>12.3744</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2775,16 +2841,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.6596</v>
+        <v>33.754</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>74254.42398399999</v>
+        <v>74462.67416</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>14254.42398399999</v>
+        <v>14462.67416</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2375737330666666</v>
+        <v>0.2410445693333333</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -2846,6 +2912,9 @@
       <c r="AC7" s="3" t="n">
         <v>33.6596</v>
       </c>
+      <c r="AD7" s="3" t="n">
+        <v>33.754</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2870,16 +2939,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>31.7475</v>
+        <v>31.9987</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>50941.8162675</v>
+        <v>51344.8900291</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>941.8162674999985</v>
+        <v>1344.890029100003</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.01883632534999997</v>
+        <v>0.02689780058200006</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -2941,6 +3010,9 @@
       <c r="AC8" s="3" t="n">
         <v>31.7475</v>
       </c>
+      <c r="AD8" s="3" t="n">
+        <v>31.9987</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2965,16 +3037,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>43.7553</v>
+        <v>43.6943</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>140865.5065329</v>
+        <v>140669.1235599</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>40865.50653290001</v>
+        <v>40669.12355990001</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.4086550653290001</v>
+        <v>0.4066912355990001</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -3036,6 +3108,9 @@
       <c r="AC9" s="3" t="n">
         <v>43.7553</v>
       </c>
+      <c r="AD9" s="3" t="n">
+        <v>43.6943</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3060,16 +3135,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>46.1869</v>
+        <v>46.7068</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>131478.3545671</v>
+        <v>132958.3325812</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>31478.3545671</v>
+        <v>32958.3325812</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.314783545671</v>
+        <v>0.3295833258119999</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -3131,6 +3206,9 @@
       <c r="AC10" s="3" t="n">
         <v>46.1869</v>
       </c>
+      <c r="AD10" s="3" t="n">
+        <v>46.7068</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3155,16 +3233,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>107.3247</v>
+        <v>107.2915</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>32296.0413993</v>
+        <v>32286.0508885</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>2296.0413993</v>
+        <v>2286.050888499998</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.07653471331</v>
+        <v>0.07620169628333327</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -3226,6 +3304,9 @@
       <c r="AC11" s="3" t="n">
         <v>107.3247</v>
       </c>
+      <c r="AD11" s="3" t="n">
+        <v>107.2915</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3250,16 +3331,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>219.673</v>
+        <v>219.077</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>102262.614306</v>
+        <v>101985.163194</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>2262.614306000003</v>
+        <v>1985.163193999993</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.02262614306000003</v>
+        <v>0.01985163193999993</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -3321,6 +3402,9 @@
       <c r="AC12" s="3" t="n">
         <v>219.673</v>
       </c>
+      <c r="AD12" s="3" t="n">
+        <v>219.077</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3345,16 +3429,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>19.779</v>
+        <v>19.85</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>229191.239295</v>
+        <v>230013.95925</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>29191.23929499998</v>
+        <v>30013.95925000001</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.1459561964749999</v>
+        <v>0.1500697962500001</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -3416,6 +3500,9 @@
       <c r="AC13" s="3" t="n">
         <v>19.779</v>
       </c>
+      <c r="AD13" s="3" t="n">
+        <v>19.85</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3440,16 +3527,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>40.98</v>
+        <v>41.1531</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>147839.69388</v>
+        <v>148464.1704786</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>47839.69388000001</v>
+        <v>48464.17047860002</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.4783969388000001</v>
+        <v>0.4846417047860002</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -3511,6 +3598,9 @@
       <c r="AC14" s="3" t="n">
         <v>40.98</v>
       </c>
+      <c r="AD14" s="3" t="n">
+        <v>41.1531</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3535,16 +3625,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.74</v>
+        <v>11.79</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>114393.93778</v>
+        <v>114881.13513</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>14393.93778000001</v>
+        <v>14881.13513</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1439393778000001</v>
+        <v>0.1488113512999999</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -3606,6 +3696,9 @@
       <c r="AC15" s="3" t="n">
         <v>11.74</v>
       </c>
+      <c r="AD15" s="3" t="n">
+        <v>11.79</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3630,16 +3723,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>25.3949</v>
+        <v>25.4826</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>145333.1842672</v>
+        <v>145835.0850528</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>45333.18426720001</v>
+        <v>45835.08505280002</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4533318426720001</v>
+        <v>0.4583508505280002</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -3701,6 +3794,9 @@
       <c r="AC16" s="3" t="n">
         <v>25.3949</v>
       </c>
+      <c r="AD16" s="3" t="n">
+        <v>25.4826</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3725,16 +3821,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.6895</v>
+        <v>16.6458</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55176.43830149999</v>
+        <v>55031.9636106</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5176.438301499991</v>
+        <v>5031.963610600003</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1035287660299998</v>
+        <v>0.1006392722120001</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -3796,6 +3892,9 @@
       <c r="AC17" s="3" t="n">
         <v>16.6895</v>
       </c>
+      <c r="AD17" s="3" t="n">
+        <v>16.6458</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3820,16 +3919,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>44.34</v>
+        <v>44.38</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>83644.57224000001</v>
+        <v>83720.02968000001</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>3644.572240000009</v>
+        <v>3720.029680000007</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.04555715300000011</v>
+        <v>0.04650037100000009</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -3891,6 +3990,9 @@
       <c r="AC18" s="3" t="n">
         <v>44.34</v>
       </c>
+      <c r="AD18" s="3" t="n">
+        <v>44.38</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3915,16 +4017,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>15.2629</v>
+        <v>15.5427</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>220804.8027814</v>
+        <v>224852.6039082</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>70804.80278140001</v>
+        <v>74852.60390819999</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.4720320185426667</v>
+        <v>0.499017359388</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -3986,6 +4088,9 @@
       <c r="AC19" s="3" t="n">
         <v>15.2629</v>
       </c>
+      <c r="AD19" s="3" t="n">
+        <v>15.5427</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4010,16 +4115,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.65</v>
+        <v>9.380000000000001</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>253368.49895</v>
-      </c>
-      <c r="H20" s="4" t="n">
-        <v>3368.498950000008</v>
-      </c>
-      <c r="I20" s="12" t="n">
-        <v>0.01347399580000003</v>
+        <v>246279.43214</v>
+      </c>
+      <c r="H20" s="6" t="n">
+        <v>-3720.567859999981</v>
+      </c>
+      <c r="I20" s="13" t="n">
+        <v>-0.01488227143999992</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -4081,6 +4186,9 @@
       <c r="AC20" s="3" t="n">
         <v>9.65</v>
       </c>
+      <c r="AD20" s="3" t="n">
+        <v>9.380000000000001</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4105,16 +4213,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>107.3466</v>
+        <v>107.0983</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>163087.2881694</v>
+        <v>162710.0561597</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-6912.711830600019</v>
+        <v>-7289.943840299995</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.04066301076823541</v>
+        <v>-0.04288202258999997</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -4176,6 +4284,9 @@
       <c r="AC21" s="3" t="n">
         <v>107.3466</v>
       </c>
+      <c r="AD21" s="3" t="n">
+        <v>107.0983</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4200,16 +4311,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>46.101</v>
+        <v>46.295</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>70740.14046</v>
+        <v>71037.8257</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>10740.14046</v>
+        <v>11037.8257</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1790023409999999</v>
+        <v>0.1839637616666667</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -4271,6 +4382,9 @@
       <c r="AC22" s="3" t="n">
         <v>46.101</v>
       </c>
+      <c r="AD22" s="3" t="n">
+        <v>46.295</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4295,16 +4409,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>61.0741</v>
+        <v>61.1852</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>165905.7772047</v>
+        <v>166207.5766884</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>15905.77720470002</v>
+        <v>16207.5766884</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.1060385146980001</v>
+        <v>0.108050511256</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -4366,6 +4480,9 @@
       <c r="AC23" s="3" t="n">
         <v>61.0741</v>
       </c>
+      <c r="AD23" s="3" t="n">
+        <v>61.1852</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4390,16 +4507,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>28.2266</v>
+        <v>28.353</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>102558.1332676</v>
+        <v>103017.393258</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>2558.133267600002</v>
+        <v>3017.393258000011</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.02558133267600002</v>
+        <v>0.03017393258000011</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -4461,6 +4578,9 @@
       <c r="AC24" s="3" t="n">
         <v>28.2266</v>
       </c>
+      <c r="AD24" s="3" t="n">
+        <v>28.353</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4485,16 +4605,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.3922</v>
+        <v>11.2505</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>187078.9945428</v>
+        <v>184752.043337</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-12921.00545719999</v>
+        <v>-15247.95666299999</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.06460502728599997</v>
+        <v>-0.07623978331499995</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -4556,6 +4676,9 @@
       <c r="AC25" s="3" t="n">
         <v>11.3922</v>
       </c>
+      <c r="AD25" s="3" t="n">
+        <v>11.2505</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4580,16 +4703,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>9.1944</v>
+        <v>8.9903</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>109796.904396</v>
+        <v>107359.6003645</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>-203.0956040000019</v>
+        <v>-2640.399635499998</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>-0.00184632367272729</v>
+        <v>-0.02400363304999998</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -4651,6 +4774,9 @@
       <c r="AC26" s="3" t="n">
         <v>9.1944</v>
       </c>
+      <c r="AD26" s="3" t="n">
+        <v>8.9903</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4675,16 +4801,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>63.5109</v>
+        <v>63.2311</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>102307.168374</v>
+        <v>101856.449746</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-7692.831626000014</v>
+        <v>-8143.550254000016</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.06993483296363649</v>
+        <v>-0.07403227503636378</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -4746,6 +4872,9 @@
       <c r="AC27" s="3" t="n">
         <v>63.5109</v>
       </c>
+      <c r="AD27" s="3" t="n">
+        <v>63.2311</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4770,16 +4899,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>105.6391</v>
+        <v>104.1164</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>349312.2694887</v>
+        <v>344277.2228748</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-30687.73051129997</v>
+        <v>-35722.77712519997</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.08075718555605256</v>
+        <v>-0.09400730822421044</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -4841,6 +4970,9 @@
       <c r="AC28" s="3" t="n">
         <v>105.6391</v>
       </c>
+      <c r="AD28" s="3" t="n">
+        <v>104.1164</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4865,16 +4997,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.7844</v>
+        <v>11.8289</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>113173.8776332</v>
+        <v>113601.2424167</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>13173.8776332</v>
+        <v>13601.2424167</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.131738776332</v>
+        <v>0.136012424167</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -4936,6 +5068,9 @@
       <c r="AC29" s="3" t="n">
         <v>11.7844</v>
       </c>
+      <c r="AD29" s="3" t="n">
+        <v>11.8289</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4960,16 +5095,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>15.6143</v>
+        <v>15.5856</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>115481.1924123</v>
+        <v>115268.9312016</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>15481.19241229999</v>
+        <v>15268.93120159999</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.1548119241229999</v>
+        <v>0.1526893120159999</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -5031,6 +5166,9 @@
       <c r="AC30" s="3" t="n">
         <v>15.6143</v>
       </c>
+      <c r="AD30" s="3" t="n">
+        <v>15.5856</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -5055,16 +5193,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>411.9591</v>
+        <v>411.2521</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>109614.077328</v>
+        <v>109425.958768</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>9614.077327999985</v>
+        <v>9425.958767999982</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.09614077327999984</v>
+        <v>0.09425958767999983</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -5126,6 +5264,9 @@
       <c r="AC31" s="3" t="n">
         <v>411.9591</v>
       </c>
+      <c r="AD31" s="3" t="n">
+        <v>411.2521</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -5150,16 +5291,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.15</v>
+        <v>10.09</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>214570.594</v>
+        <v>213302.1964</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>14570.59400000001</v>
+        <v>13302.19639999999</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.07285297000000006</v>
+        <v>0.06651098199999993</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -5221,6 +5362,9 @@
       <c r="AC32" s="3" t="n">
         <v>10.15</v>
       </c>
+      <c r="AD32" s="3" t="n">
+        <v>10.09</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -5245,16 +5389,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>17.78</v>
+        <v>17.72</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>63717.1192</v>
+        <v>63502.10079999999</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>3717.119200000001</v>
+        <v>3502.100799999993</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.06195198666666668</v>
+        <v>0.05836834666666655</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -5316,6 +5460,9 @@
       <c r="AC33" s="3" t="n">
         <v>17.78</v>
       </c>
+      <c r="AD33" s="3" t="n">
+        <v>17.72</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -5340,16 +5487,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>220.5786</v>
+        <v>214.2688</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>77540.21583659999</v>
+        <v>75322.1255328</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-2459.784163400007</v>
+        <v>-4677.874467200003</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.03074730204250009</v>
+        <v>-0.05847343084000003</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -5411,6 +5558,9 @@
       <c r="AC34" s="3" t="n">
         <v>220.5786</v>
       </c>
+      <c r="AD34" s="3" t="n">
+        <v>214.2688</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -5435,16 +5585,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>14.37</v>
+        <v>14.52</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>102536.02851</v>
+        <v>103606.34196</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>2536.028509999989</v>
+        <v>3606.341959999991</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.02536028509999989</v>
+        <v>0.0360634195999999</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -5506,6 +5656,9 @@
       <c r="AC35" s="3" t="n">
         <v>14.37</v>
       </c>
+      <c r="AD35" s="3" t="n">
+        <v>14.52</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5530,16 +5683,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>345.5958</v>
+        <v>346.0132</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>160946.0376348</v>
+        <v>161140.4233192</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>10946.03763480001</v>
+        <v>11140.4233192</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.07297358423200009</v>
+        <v>0.07426948879466663</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -5601,6 +5754,9 @@
       <c r="AC36" s="3" t="n">
         <v>345.5958</v>
       </c>
+      <c r="AD36" s="3" t="n">
+        <v>346.0132</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5625,16 +5781,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>15.455</v>
+        <v>15.539</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>58155.449495</v>
+        <v>58471.532171</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>8155.449495000001</v>
+        <v>8471.532170999999</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.1631089899</v>
+        <v>0.16943064342</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -5696,6 +5852,9 @@
       <c r="AC37" s="3" t="n">
         <v>15.455</v>
       </c>
+      <c r="AD37" s="3" t="n">
+        <v>15.539</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5720,16 +5879,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.9479</v>
+        <v>13.8991</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>83415.1648878</v>
+        <v>83123.3173662</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>3415.164887799998</v>
+        <v>3123.317366200004</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.04268956109749997</v>
+        <v>0.03904146707750006</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -5791,6 +5950,9 @@
       <c r="AC38" s="3" t="n">
         <v>13.9479</v>
       </c>
+      <c r="AD38" s="3" t="n">
+        <v>13.8991</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5815,16 +5977,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1010.7179</v>
+        <v>1010.1103</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50415.6195699</v>
+        <v>50385.3118743</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>415.6195699000018</v>
+        <v>385.3118743000014</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.008312391398000036</v>
+        <v>0.007706237486000027</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -5886,6 +6048,9 @@
       <c r="AC39" s="3" t="n">
         <v>1010.7179</v>
       </c>
+      <c r="AD39" s="3" t="n">
+        <v>1010.1103</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5910,16 +6075,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>20.2066</v>
+        <v>20.2506</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>101862.0161782</v>
+        <v>102083.8213662</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>1862.016178200007</v>
+        <v>2083.821366199991</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.01862016178200007</v>
+        <v>0.02083821366199991</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -5981,6 +6146,9 @@
       <c r="AC40" s="3" t="n">
         <v>20.2066</v>
       </c>
+      <c r="AD40" s="3" t="n">
+        <v>20.2506</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
@@ -5992,13 +6160,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4890641.2703557</v>
+        <v>4877136.4413211</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>420641.2703557</v>
+        <v>407136.4413211001</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.09410319247331098</v>
+        <v>0.09108197792418346</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-06-05
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -484,7 +484,7 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-04 06:41 IST</t>
+          <t>Generated: 2026-06-05 06:20 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4877136.4413211</v>
+        <v>4878416.3532113</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>407136.4413211001</v>
+        <v>408416.3532113004</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.09108197792418347</v>
+        <v>0.09136831168038041</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>567987.4966125488</v>
+        <v>565908.0006484985</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-22794.52338745119</v>
+        <v>-24874.01935150148</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.03858364441668551</v>
+        <v>-0.04210354836374588</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5445123.937933649</v>
+        <v>5444324.353859799</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>384341.9179336494</v>
+        <v>383542.3338597994</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.07594516349740932</v>
+        <v>0.07578716734766605</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-06-04</t>
+          <t>Last snapshot: 2026-06-05</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC19"/>
+  <dimension ref="A1:AD19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -648,6 +648,7 @@
     <col width="21" customWidth="1" min="27" max="27"/>
     <col width="21" customWidth="1" min="28" max="28"/>
     <col width="21" customWidth="1" min="29" max="29"/>
+    <col width="21" customWidth="1" min="30" max="30"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -796,6 +797,11 @@
           <t>2026-06-04</t>
         </is>
       </c>
+      <c r="AD1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -815,13 +821,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>601.5</v>
+        <v>601.0999755859375</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>48120</v>
+        <v>48087.998046875</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>4302.489999999998</v>
+        <v>4270.488046874998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -889,6 +895,9 @@
       <c r="AC2" s="3" t="n">
         <v>601.5</v>
       </c>
+      <c r="AD2" s="3" t="n">
+        <v>601.0999755859375</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -935,13 +944,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1544.199951171875</v>
+        <v>1541.5</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>30883.9990234375</v>
+        <v>30830</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-1220.580976562502</v>
+        <v>-1274.580000000002</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1009,6 +1018,9 @@
       <c r="AC4" s="3" t="n">
         <v>1544.199951171875</v>
       </c>
+      <c r="AD4" s="3" t="n">
+        <v>1541.5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1028,13 +1040,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>650</v>
+        <v>656.4000244140625</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13000</v>
+        <v>13128.00048828125</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1213.1</v>
+        <v>-1085.09951171875</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1102,6 +1114,9 @@
       <c r="AC5" s="3" t="n">
         <v>650</v>
       </c>
+      <c r="AD5" s="3" t="n">
+        <v>656.4000244140625</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1121,13 +1136,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>383.5</v>
+        <v>389.2000122070312</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15340</v>
+        <v>15568.00048828125</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2162.240000000002</v>
+        <v>-1934.239511718752</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1195,6 +1210,9 @@
       <c r="AC6" s="3" t="n">
         <v>383.5</v>
       </c>
+      <c r="AD6" s="3" t="n">
+        <v>389.2000122070312</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1214,13 +1232,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>236.3800048828125</v>
+        <v>237.3000030517578</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>23638.00048828125</v>
+        <v>23730.00030517578</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-2795.81951171875</v>
+        <v>-2703.819694824218</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1288,6 +1306,9 @@
       <c r="AC7" s="3" t="n">
         <v>236.3800048828125</v>
       </c>
+      <c r="AD7" s="3" t="n">
+        <v>237.3000030517578</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1334,13 +1355,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>19.22999954223633</v>
+        <v>19.1200008392334</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>28844.99931335449</v>
+        <v>28680.0012588501</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-2205.170686645506</v>
+        <v>-2370.168741149901</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1408,6 +1429,9 @@
       <c r="AC9" s="3" t="n">
         <v>19.22999954223633</v>
       </c>
+      <c r="AD9" s="3" t="n">
+        <v>19.1200008392334</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1427,13 +1451,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>490.5499877929688</v>
+        <v>486.6000061035156</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>49054.99877929688</v>
+        <v>48660.00061035156</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-2443.481220703128</v>
+        <v>-2838.479389648441</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1501,6 +1525,9 @@
       <c r="AC10" s="3" t="n">
         <v>490.5499877929688</v>
       </c>
+      <c r="AD10" s="3" t="n">
+        <v>486.6000061035156</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1520,13 +1547,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>9.420000076293945</v>
+        <v>9.25</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>9420.000076293945</v>
+        <v>9250</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-421.2099237060538</v>
+        <v>-591.2099999999991</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -1594,6 +1621,9 @@
       <c r="AC11" s="3" t="n">
         <v>9.420000076293945</v>
       </c>
+      <c r="AD11" s="3" t="n">
+        <v>9.25</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1613,13 +1643,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2657.10009765625</v>
+        <v>2646.60009765625</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>26571.0009765625</v>
+        <v>26466.0009765625</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-1152.2490234375</v>
+        <v>-1257.2490234375</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -1687,6 +1717,9 @@
       <c r="AC12" s="3" t="n">
         <v>2657.10009765625</v>
       </c>
+      <c r="AD12" s="3" t="n">
+        <v>2646.60009765625</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1706,13 +1739,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>55.18999862670898</v>
+        <v>55.34999847412109</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>33113.99917602539</v>
+        <v>33209.99908447266</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-1917.760823974611</v>
+        <v>-1821.760915527346</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -1780,6 +1813,9 @@
       <c r="AC13" s="3" t="n">
         <v>55.18999862670898</v>
       </c>
+      <c r="AD13" s="3" t="n">
+        <v>55.34999847412109</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1799,13 +1835,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>724</v>
+        <v>722.25</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>36200</v>
+        <v>36112.5</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-6262.510000000002</v>
+        <v>-6350.010000000002</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -1873,6 +1909,9 @@
       <c r="AC14" s="3" t="n">
         <v>724</v>
       </c>
+      <c r="AD14" s="3" t="n">
+        <v>722.25</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1946,13 +1985,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>615.2999877929688</v>
+        <v>584.5</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>30764.99938964844</v>
+        <v>29225</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>9010.469389648439</v>
+        <v>7470.470000000001</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -2020,6 +2059,9 @@
       <c r="AC17" s="3" t="n">
         <v>615.2999877929688</v>
       </c>
+      <c r="AD17" s="3" t="n">
+        <v>584.5</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2039,13 +2081,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>412.6499938964844</v>
+        <v>411.8999938964844</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>41264.99938964844</v>
+        <v>41189.99938964844</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-5375.820610351562</v>
+        <v>-5450.820610351562</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -2113,6 +2155,9 @@
       <c r="AC18" s="3" t="n">
         <v>412.6499938964844</v>
       </c>
+      <c r="AD18" s="3" t="n">
+        <v>411.8999938964844</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -2124,10 +2169,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>567987.4966125488</v>
+        <v>565908.0006484985</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-22794.52338745118</v>
+        <v>-24874.01935150148</v>
       </c>
     </row>
   </sheetData>
@@ -2141,7 +2186,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD41"/>
+  <dimension ref="A1:AE41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2174,6 +2219,7 @@
     <col width="13" customWidth="1" min="28" max="28"/>
     <col width="13" customWidth="1" min="29" max="29"/>
     <col width="13" customWidth="1" min="30" max="30"/>
+    <col width="13" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2327,6 +2373,11 @@
           <t>2026-06-04</t>
         </is>
       </c>
+      <c r="AE1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2351,16 +2402,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>57.5427</v>
+        <v>57.6055</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>64590.6449814</v>
+        <v>64661.136851</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>14590.6449814</v>
+        <v>14661.136851</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.291812899628</v>
+        <v>0.2932227370199999</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -2425,6 +2476,9 @@
       <c r="AD2" s="3" t="n">
         <v>57.5427</v>
       </c>
+      <c r="AE2" s="3" t="n">
+        <v>57.6055</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2449,16 +2503,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.88</v>
+        <v>25.5272</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>63540.91244</v>
+        <v>62674.71329360001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>3540.91244</v>
+        <v>2674.713293600005</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.05901520733333333</v>
+        <v>0.04457855489333342</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -2523,6 +2577,9 @@
       <c r="AD3" s="3" t="n">
         <v>25.88</v>
       </c>
+      <c r="AE3" s="3" t="n">
+        <v>25.5272</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2547,16 +2604,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>13.05</v>
+        <v>12.82</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>250639.51365</v>
+        <v>246222.11226</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>70639.51365000004</v>
+        <v>66222.11226000002</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3924417425000002</v>
+        <v>0.3679006236666668</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -2621,6 +2678,9 @@
       <c r="AD4" s="3" t="n">
         <v>13.05</v>
       </c>
+      <c r="AE4" s="3" t="n">
+        <v>12.82</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2645,16 +2705,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.4147</v>
+        <v>9.4536</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>172798.2322936</v>
+        <v>173512.2063168</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-37201.76770640002</v>
+        <v>-36487.7936832</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.177151274792381</v>
+        <v>-0.1737513984914286</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -2719,6 +2779,9 @@
       <c r="AD5" s="3" t="n">
         <v>9.4147</v>
       </c>
+      <c r="AE5" s="3" t="n">
+        <v>9.4536</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2743,16 +2806,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.3744</v>
+        <v>12.4113</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>52331.05298879999</v>
+        <v>52487.1022401</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>2331.052988799995</v>
+        <v>2487.102240100001</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.0466210597759999</v>
+        <v>0.04974204480200002</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -2817,6 +2880,9 @@
       <c r="AD6" s="3" t="n">
         <v>12.3744</v>
       </c>
+      <c r="AE6" s="3" t="n">
+        <v>12.4113</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2841,16 +2907,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.754</v>
+        <v>33.7988</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>74462.67416</v>
+        <v>74561.50475199999</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>14462.67416</v>
+        <v>14561.50475199999</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2410445693333333</v>
+        <v>0.2426917458666666</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -2915,6 +2981,9 @@
       <c r="AD7" s="3" t="n">
         <v>33.754</v>
       </c>
+      <c r="AE7" s="3" t="n">
+        <v>33.7988</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2939,16 +3008,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>31.9987</v>
+        <v>32.2505</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>51344.8900291</v>
+        <v>51748.92654650001</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>1344.890029100003</v>
+        <v>1748.926546500006</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.02689780058200006</v>
+        <v>0.03497853093000013</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -3013,6 +3082,9 @@
       <c r="AD8" s="3" t="n">
         <v>31.9987</v>
       </c>
+      <c r="AE8" s="3" t="n">
+        <v>32.2505</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3037,16 +3109,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>43.6943</v>
+        <v>42.777</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>140669.1235599</v>
+        <v>137715.974361</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>40669.12355990001</v>
+        <v>37715.974361</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.4066912355990001</v>
+        <v>0.37715974361</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -3111,6 +3183,9 @@
       <c r="AD9" s="3" t="n">
         <v>43.6943</v>
       </c>
+      <c r="AE9" s="3" t="n">
+        <v>42.777</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3135,16 +3210,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>46.7068</v>
+        <v>47.0664</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>132958.3325812</v>
+        <v>133981.9911576</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>32958.3325812</v>
+        <v>33981.99115760002</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3295833258119999</v>
+        <v>0.3398199115760002</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -3209,6 +3284,9 @@
       <c r="AD10" s="3" t="n">
         <v>46.7068</v>
       </c>
+      <c r="AE10" s="3" t="n">
+        <v>47.0664</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3233,16 +3311,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>107.2915</v>
+        <v>107.6649</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>32286.0508885</v>
+        <v>32398.4140431</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>2286.050888499998</v>
+        <v>2398.414043099998</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.07620169628333327</v>
+        <v>0.07994713476999993</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -3307,6 +3385,9 @@
       <c r="AD11" s="3" t="n">
         <v>107.2915</v>
       </c>
+      <c r="AE11" s="3" t="n">
+        <v>107.6649</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3331,16 +3412,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>219.077</v>
+        <v>219.942</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>101985.163194</v>
+        <v>102387.839724</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>1985.163193999993</v>
+        <v>2387.839724000005</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.01985163193999993</v>
+        <v>0.02387839724000005</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -3405,6 +3486,9 @@
       <c r="AD12" s="3" t="n">
         <v>219.077</v>
       </c>
+      <c r="AE12" s="3" t="n">
+        <v>219.942</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3429,16 +3513,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>19.85</v>
+        <v>20.006</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>230013.95925</v>
+        <v>231821.62563</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>30013.95925000001</v>
+        <v>31821.62562999999</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.1500697962500001</v>
+        <v>0.15910812815</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -3503,6 +3587,9 @@
       <c r="AD13" s="3" t="n">
         <v>19.85</v>
       </c>
+      <c r="AE13" s="3" t="n">
+        <v>20.006</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3527,16 +3614,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>41.1531</v>
+        <v>40.4025</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>148464.1704786</v>
+        <v>145756.301415</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>48464.17047860002</v>
+        <v>45756.30141500002</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.4846417047860002</v>
+        <v>0.4575630141500002</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -3601,6 +3688,9 @@
       <c r="AD14" s="3" t="n">
         <v>41.1531</v>
       </c>
+      <c r="AE14" s="3" t="n">
+        <v>40.4025</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3625,16 +3715,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.79</v>
+        <v>11.88</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>114881.13513</v>
+        <v>115758.09036</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>14881.13513</v>
+        <v>15758.09036</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1488113512999999</v>
+        <v>0.1575809036</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -3699,6 +3789,9 @@
       <c r="AD15" s="3" t="n">
         <v>11.79</v>
       </c>
+      <c r="AE15" s="3" t="n">
+        <v>11.88</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3723,16 +3816,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>25.4826</v>
+        <v>25.3403</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>145835.0850528</v>
+        <v>145020.7123984</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>45835.08505280002</v>
+        <v>45020.71239840001</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4583508505280002</v>
+        <v>0.4502071239840001</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -3797,6 +3890,9 @@
       <c r="AD16" s="3" t="n">
         <v>25.4826</v>
       </c>
+      <c r="AE16" s="3" t="n">
+        <v>25.3403</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3821,16 +3917,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.6458</v>
+        <v>16.678</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55031.9636106</v>
+        <v>55138.418646</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5031.963610600003</v>
+        <v>5138.418645999998</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1006392722120001</v>
+        <v>0.10276837292</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -3895,6 +3991,9 @@
       <c r="AD17" s="3" t="n">
         <v>16.6458</v>
       </c>
+      <c r="AE17" s="3" t="n">
+        <v>16.678</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3919,16 +4018,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>44.38</v>
+        <v>44.41</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>83720.02968000001</v>
+        <v>83776.62275999998</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>3720.029680000007</v>
+        <v>3776.622759999984</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.04650037100000009</v>
+        <v>0.0472077844999998</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -3993,6 +4092,9 @@
       <c r="AD18" s="3" t="n">
         <v>44.38</v>
       </c>
+      <c r="AE18" s="3" t="n">
+        <v>44.41</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4017,16 +4119,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>15.5427</v>
+        <v>15.0749</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>224852.6039082</v>
+        <v>218085.0507734</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>74852.60390819999</v>
+        <v>68085.0507734</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.499017359388</v>
+        <v>0.4539003384893333</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -4091,6 +4193,9 @@
       <c r="AD19" s="3" t="n">
         <v>15.5427</v>
       </c>
+      <c r="AE19" s="3" t="n">
+        <v>15.0749</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4115,16 +4220,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.380000000000001</v>
+        <v>9.43</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>246279.43214</v>
+        <v>247592.22229</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-3720.567859999981</v>
+        <v>-2407.777709999995</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.01488227143999992</v>
+        <v>-0.009631110839999979</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -4189,6 +4294,9 @@
       <c r="AD20" s="3" t="n">
         <v>9.380000000000001</v>
       </c>
+      <c r="AE20" s="3" t="n">
+        <v>9.43</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4213,16 +4321,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>107.0983</v>
+        <v>107.2602</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>162710.0561597</v>
+        <v>162956.0241918</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-7289.943840299995</v>
+        <v>-7043.97580819999</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.04288202258999997</v>
+        <v>-0.04143515181294111</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -4287,6 +4395,9 @@
       <c r="AD21" s="3" t="n">
         <v>107.0983</v>
       </c>
+      <c r="AE21" s="3" t="n">
+        <v>107.2602</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4311,16 +4422,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>46.295</v>
+        <v>45.53</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>71037.8257</v>
+        <v>69863.9638</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>11037.8257</v>
+        <v>9863.963799999998</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1839637616666667</v>
+        <v>0.1643993966666666</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -4385,6 +4496,9 @@
       <c r="AD22" s="3" t="n">
         <v>46.295</v>
       </c>
+      <c r="AE22" s="3" t="n">
+        <v>45.53</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4409,16 +4523,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>61.1852</v>
+        <v>61.3103</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>166207.5766884</v>
+        <v>166547.4067101</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>16207.5766884</v>
+        <v>16547.40671010001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.108050511256</v>
+        <v>0.1103160447340001</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -4483,6 +4597,9 @@
       <c r="AD23" s="3" t="n">
         <v>61.1852</v>
       </c>
+      <c r="AE23" s="3" t="n">
+        <v>61.3103</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4507,16 +4624,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>28.353</v>
+        <v>28.4948</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>103017.393258</v>
+        <v>103532.6073928</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>3017.393258000011</v>
+        <v>3532.607392800011</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.03017393258000011</v>
+        <v>0.03532607392800011</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -4581,6 +4698,9 @@
       <c r="AD24" s="3" t="n">
         <v>28.353</v>
       </c>
+      <c r="AE24" s="3" t="n">
+        <v>28.4948</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4605,16 +4725,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.2505</v>
+        <v>11.4191</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>184752.043337</v>
+        <v>187520.7375734</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-15247.95666299999</v>
+        <v>-12479.26242660001</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.07623978331499995</v>
+        <v>-0.06239631213300003</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -4679,6 +4799,9 @@
       <c r="AD25" s="3" t="n">
         <v>11.2505</v>
       </c>
+      <c r="AE25" s="3" t="n">
+        <v>11.4191</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4703,16 +4826,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>8.9903</v>
+        <v>8.9727</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>107359.6003645</v>
+        <v>107149.4261805</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>-2640.399635499998</v>
+        <v>-2850.573819500001</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>-0.02400363304999998</v>
+        <v>-0.02591430745000001</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -4777,6 +4900,9 @@
       <c r="AD26" s="3" t="n">
         <v>8.9903</v>
       </c>
+      <c r="AE26" s="3" t="n">
+        <v>8.9727</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4801,16 +4927,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>63.2311</v>
+        <v>63.8198</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>101856.449746</v>
+        <v>102804.763028</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-8143.550254000016</v>
+        <v>-7195.236971999999</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.07403227503636378</v>
+        <v>-0.0654112452</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -4875,6 +5001,9 @@
       <c r="AD27" s="3" t="n">
         <v>63.2311</v>
       </c>
+      <c r="AE27" s="3" t="n">
+        <v>63.8198</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4899,16 +5028,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>104.1164</v>
+        <v>104.9468</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>344277.2228748</v>
+        <v>347023.0708476</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-35722.77712519997</v>
+        <v>-32976.9291524</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.09400730822421044</v>
+        <v>-0.08678139250631579</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -4973,6 +5102,9 @@
       <c r="AD28" s="3" t="n">
         <v>104.1164</v>
       </c>
+      <c r="AE28" s="3" t="n">
+        <v>104.9468</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4997,16 +5129,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.8289</v>
+        <v>11.885</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>113601.2424167</v>
+        <v>114140.010155</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>13601.2424167</v>
+        <v>14140.010155</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.136012424167</v>
+        <v>0.14140010155</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -5071,6 +5203,9 @@
       <c r="AD29" s="3" t="n">
         <v>11.8289</v>
       </c>
+      <c r="AE29" s="3" t="n">
+        <v>11.885</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -5095,16 +5230,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>15.5856</v>
+        <v>15.6929</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>115268.9312016</v>
+        <v>116062.5070869</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>15268.93120159999</v>
+        <v>16062.50708689999</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.1526893120159999</v>
+        <v>0.1606250708689999</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -5169,6 +5304,9 @@
       <c r="AD30" s="3" t="n">
         <v>15.5856</v>
       </c>
+      <c r="AE30" s="3" t="n">
+        <v>15.6929</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -5193,16 +5331,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>411.2521</v>
+        <v>412.6834</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>109425.958768</v>
+        <v>109806.799072</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>9425.958767999982</v>
+        <v>9806.799071999994</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.09425958767999983</v>
+        <v>0.09806799071999994</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -5267,6 +5405,9 @@
       <c r="AD31" s="3" t="n">
         <v>411.2521</v>
       </c>
+      <c r="AE31" s="3" t="n">
+        <v>412.6834</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -5291,16 +5432,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.09</v>
+        <v>10.15</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>213302.1964</v>
+        <v>214570.594</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>13302.19639999999</v>
+        <v>14570.59400000001</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.06651098199999993</v>
+        <v>0.07285297000000006</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -5365,6 +5506,9 @@
       <c r="AD32" s="3" t="n">
         <v>10.09</v>
       </c>
+      <c r="AE32" s="3" t="n">
+        <v>10.15</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -5389,16 +5533,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>17.72</v>
+        <v>17.81</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>63502.10079999999</v>
+        <v>63824.62839999999</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>3502.100799999993</v>
+        <v>3824.628399999994</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.05836834666666655</v>
+        <v>0.06374380666666657</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -5463,6 +5607,9 @@
       <c r="AD33" s="3" t="n">
         <v>17.72</v>
       </c>
+      <c r="AE33" s="3" t="n">
+        <v>17.81</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -5487,16 +5634,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>214.2688</v>
+        <v>214.3516</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>75322.1255328</v>
+        <v>75351.2322996</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-4677.874467200003</v>
+        <v>-4648.7677004</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.05847343084000003</v>
+        <v>-0.058109596255</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -5561,6 +5708,9 @@
       <c r="AD34" s="3" t="n">
         <v>214.2688</v>
       </c>
+      <c r="AE34" s="3" t="n">
+        <v>214.3516</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -5585,16 +5735,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>14.52</v>
+        <v>14.7</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>103606.34196</v>
+        <v>104890.7181</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>3606.341959999991</v>
+        <v>4890.718099999998</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.0360634195999999</v>
+        <v>0.04890718099999998</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -5659,6 +5809,9 @@
       <c r="AD35" s="3" t="n">
         <v>14.52</v>
       </c>
+      <c r="AE35" s="3" t="n">
+        <v>14.7</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5683,16 +5836,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>346.0132</v>
+        <v>347.6696</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>161140.4233192</v>
+        <v>161911.8187376</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>11140.4233192</v>
+        <v>11911.8187376</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.07426948879466663</v>
+        <v>0.07941212491733332</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -5757,6 +5910,9 @@
       <c r="AD36" s="3" t="n">
         <v>346.0132</v>
       </c>
+      <c r="AE36" s="3" t="n">
+        <v>347.6696</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5781,16 +5937,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>15.539</v>
+        <v>15.619</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>58471.532171</v>
+        <v>58772.563291</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>8471.532170999999</v>
+        <v>8772.563290999999</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.16943064342</v>
+        <v>0.17545126582</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -5855,6 +6011,9 @@
       <c r="AD37" s="3" t="n">
         <v>15.539</v>
       </c>
+      <c r="AE37" s="3" t="n">
+        <v>15.619</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5879,16 +6038,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.8991</v>
+        <v>13.9354</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>83123.3173662</v>
+        <v>83340.4088628</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>3123.317366200004</v>
+        <v>3340.408862800003</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.03904146707750006</v>
+        <v>0.04175511078500004</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -5953,6 +6112,9 @@
       <c r="AD38" s="3" t="n">
         <v>13.8991</v>
       </c>
+      <c r="AE38" s="3" t="n">
+        <v>13.9354</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5977,16 +6139,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1010.1103</v>
+        <v>1011.0558</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50385.3118743</v>
+        <v>50432.4743598</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>385.3118743000014</v>
+        <v>432.4743597999986</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.007706237486000027</v>
+        <v>0.008649487195999972</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -6051,6 +6213,9 @@
       <c r="AD39" s="3" t="n">
         <v>1010.1103</v>
       </c>
+      <c r="AE39" s="3" t="n">
+        <v>1011.0558</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -6075,16 +6240,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>20.2506</v>
+        <v>20.3557</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>102083.8213662</v>
+        <v>102613.6333039</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>2083.821366199991</v>
+        <v>2613.633303900002</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.02083821366199991</v>
+        <v>0.02613633303900002</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -6149,6 +6314,9 @@
       <c r="AD40" s="3" t="n">
         <v>20.2506</v>
       </c>
+      <c r="AE40" s="3" t="n">
+        <v>20.3557</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
@@ -6160,13 +6328,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4877136.4413211</v>
+        <v>4878416.3532113</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>407136.4413211001</v>
+        <v>408416.3532113001</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.09108197792418346</v>
+        <v>0.09136831168038033</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-06-06
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -484,7 +484,7 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-05 06:20 IST</t>
+          <t>Generated: 2026-06-06 05:53 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4878416.3532113</v>
+        <v>4847032.155924</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>408416.3532113004</v>
+        <v>377032.1559239998</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.09136831168038041</v>
+        <v>0.08434723846174494</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>565908.0006484985</v>
+        <v>563537.5043563843</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-24874.01935150148</v>
+        <v>-27244.51564361574</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.04210354836374588</v>
+        <v>-0.04611602032779491</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5444324.353859799</v>
+        <v>5410569.660280384</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>383542.3338597994</v>
+        <v>349787.6402803846</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.07578716734766605</v>
+        <v>0.06911731011097463</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-06-05</t>
+          <t>Last snapshot: 2026-06-06</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD19"/>
+  <dimension ref="A1:AE19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -649,6 +649,7 @@
     <col width="21" customWidth="1" min="28" max="28"/>
     <col width="21" customWidth="1" min="29" max="29"/>
     <col width="21" customWidth="1" min="30" max="30"/>
+    <col width="21" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -802,6 +803,11 @@
           <t>2026-06-05</t>
         </is>
       </c>
+      <c r="AE1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -821,13 +827,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>601.0999755859375</v>
+        <v>601.75</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>48087.998046875</v>
+        <v>48140</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>4270.488046874998</v>
+        <v>4322.489999999998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -898,6 +904,9 @@
       <c r="AD2" s="3" t="n">
         <v>601.0999755859375</v>
       </c>
+      <c r="AE2" s="3" t="n">
+        <v>601.75</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -944,13 +953,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1541.5</v>
+        <v>1518.800048828125</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>30830</v>
+        <v>30376.0009765625</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-1274.580000000002</v>
+        <v>-1728.579023437502</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1021,6 +1030,9 @@
       <c r="AD4" s="3" t="n">
         <v>1541.5</v>
       </c>
+      <c r="AE4" s="3" t="n">
+        <v>1518.800048828125</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1040,13 +1052,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>656.4000244140625</v>
+        <v>654.9500122070312</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13128.00048828125</v>
+        <v>13099.00024414062</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1085.09951171875</v>
+        <v>-1114.099755859375</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1117,6 +1129,9 @@
       <c r="AD5" s="3" t="n">
         <v>656.4000244140625</v>
       </c>
+      <c r="AE5" s="3" t="n">
+        <v>654.9500122070312</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1136,13 +1151,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>389.2000122070312</v>
+        <v>382.1000061035156</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15568.00048828125</v>
+        <v>15284.00024414062</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-1934.239511718752</v>
+        <v>-2218.239755859377</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1213,6 +1228,9 @@
       <c r="AD6" s="3" t="n">
         <v>389.2000122070312</v>
       </c>
+      <c r="AE6" s="3" t="n">
+        <v>382.1000061035156</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1232,13 +1250,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>237.3000030517578</v>
+        <v>237.7799987792969</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>23730.00030517578</v>
+        <v>23777.99987792969</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-2703.819694824218</v>
+        <v>-2655.820122070312</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1309,6 +1327,9 @@
       <c r="AD7" s="3" t="n">
         <v>237.3000030517578</v>
       </c>
+      <c r="AE7" s="3" t="n">
+        <v>237.7799987792969</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1355,13 +1376,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>19.1200008392334</v>
+        <v>19.03000068664551</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>28680.0012588501</v>
+        <v>28545.00102996826</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-2370.168741149901</v>
+        <v>-2505.168970031737</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1432,6 +1453,9 @@
       <c r="AD9" s="3" t="n">
         <v>19.1200008392334</v>
       </c>
+      <c r="AE9" s="3" t="n">
+        <v>19.03000068664551</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1451,13 +1475,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>486.6000061035156</v>
+        <v>483.3500061035156</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48660.00061035156</v>
+        <v>48335.00061035156</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-2838.479389648441</v>
+        <v>-3163.479389648441</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1528,6 +1552,9 @@
       <c r="AD10" s="3" t="n">
         <v>486.6000061035156</v>
       </c>
+      <c r="AE10" s="3" t="n">
+        <v>483.3500061035156</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1547,13 +1574,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>9.25</v>
+        <v>9.180000305175781</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>9250</v>
+        <v>9180.000305175781</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-591.2099999999991</v>
+        <v>-661.2096948242179</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -1624,6 +1651,9 @@
       <c r="AD11" s="3" t="n">
         <v>9.25</v>
       </c>
+      <c r="AE11" s="3" t="n">
+        <v>9.180000305175781</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1643,13 +1673,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2646.60009765625</v>
+        <v>2614.89990234375</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>26466.0009765625</v>
+        <v>26148.9990234375</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-1257.2490234375</v>
+        <v>-1574.2509765625</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -1720,6 +1750,9 @@
       <c r="AD12" s="3" t="n">
         <v>2646.60009765625</v>
       </c>
+      <c r="AE12" s="3" t="n">
+        <v>2614.89990234375</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1739,13 +1772,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>55.34999847412109</v>
+        <v>55.31000137329102</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>33209.99908447266</v>
+        <v>33186.00082397461</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-1821.760915527346</v>
+        <v>-1845.759176025393</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -1816,6 +1849,9 @@
       <c r="AD13" s="3" t="n">
         <v>55.34999847412109</v>
       </c>
+      <c r="AE13" s="3" t="n">
+        <v>55.31000137329102</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1835,13 +1871,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>722.25</v>
+        <v>719.2999877929688</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>36112.5</v>
+        <v>35964.99938964844</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-6350.010000000002</v>
+        <v>-6497.510610351565</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -1912,6 +1948,9 @@
       <c r="AD14" s="3" t="n">
         <v>722.25</v>
       </c>
+      <c r="AE14" s="3" t="n">
+        <v>719.2999877929688</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1985,13 +2024,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>584.5</v>
+        <v>576.2000122070312</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>29225</v>
+        <v>28810.00061035156</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>7470.470000000001</v>
+        <v>7055.470610351564</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -2062,6 +2101,9 @@
       <c r="AD17" s="3" t="n">
         <v>584.5</v>
       </c>
+      <c r="AE17" s="3" t="n">
+        <v>576.2000122070312</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2081,13 +2123,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>411.8999938964844</v>
+        <v>409.2000122070312</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>41189.99938964844</v>
+        <v>40920.00122070312</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-5450.820610351562</v>
+        <v>-5720.818779296875</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -2158,6 +2200,9 @@
       <c r="AD18" s="3" t="n">
         <v>411.8999938964844</v>
       </c>
+      <c r="AE18" s="3" t="n">
+        <v>409.2000122070312</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -2169,10 +2214,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>565908.0006484985</v>
+        <v>563537.5043563843</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-24874.01935150148</v>
+        <v>-27244.51564361573</v>
       </c>
     </row>
   </sheetData>
@@ -2186,7 +2231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE41"/>
+  <dimension ref="A1:AF41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2220,6 +2265,7 @@
     <col width="13" customWidth="1" min="29" max="29"/>
     <col width="13" customWidth="1" min="30" max="30"/>
     <col width="13" customWidth="1" min="31" max="31"/>
+    <col width="13" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2378,6 +2424,11 @@
           <t>2026-06-05</t>
         </is>
       </c>
+      <c r="AF1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2402,16 +2453,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>57.6055</v>
+        <v>55.7267</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>64661.136851</v>
+        <v>62552.2176694</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>14661.136851</v>
+        <v>12552.2176694</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.2932227370199999</v>
+        <v>0.251044353388</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -2479,6 +2530,9 @@
       <c r="AE2" s="3" t="n">
         <v>57.6055</v>
       </c>
+      <c r="AF2" s="3" t="n">
+        <v>55.7267</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2503,16 +2557,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.5272</v>
+        <v>25.5603</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>62674.71329360001</v>
+        <v>62755.98084390001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>2674.713293600005</v>
+        <v>2755.980843900012</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.04457855489333342</v>
+        <v>0.04593301406500019</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -2580,6 +2634,9 @@
       <c r="AE3" s="3" t="n">
         <v>25.5272</v>
       </c>
+      <c r="AF3" s="3" t="n">
+        <v>25.5603</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2604,16 +2661,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.82</v>
+        <v>12.5</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>246222.11226</v>
+        <v>240076.1625</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>66222.11226000002</v>
+        <v>60076.16250000001</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3679006236666668</v>
+        <v>0.3337564583333333</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -2681,6 +2738,9 @@
       <c r="AE4" s="3" t="n">
         <v>12.82</v>
       </c>
+      <c r="AF4" s="3" t="n">
+        <v>12.5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2705,16 +2765,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.4536</v>
+        <v>9.411099999999999</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>173512.2063168</v>
+        <v>172732.1575768</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-36487.7936832</v>
+        <v>-37267.84242320003</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1737513984914286</v>
+        <v>-0.1774659163009525</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -2782,6 +2842,9 @@
       <c r="AE5" s="3" t="n">
         <v>9.4536</v>
       </c>
+      <c r="AF5" s="3" t="n">
+        <v>9.411099999999999</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2806,16 +2869,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.4113</v>
+        <v>12.3606</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>52487.1022401</v>
+        <v>52272.6931062</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>2487.102240100001</v>
+        <v>2272.6931062</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.04974204480200002</v>
+        <v>0.04545386212400001</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -2883,6 +2946,9 @@
       <c r="AE6" s="3" t="n">
         <v>12.4113</v>
       </c>
+      <c r="AF6" s="3" t="n">
+        <v>12.3606</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2907,16 +2973,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.7988</v>
+        <v>33.6592</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>74561.50475199999</v>
+        <v>74253.541568</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>14561.50475199999</v>
+        <v>14253.541568</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2426917458666666</v>
+        <v>0.2375590261333334</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -2984,6 +3050,9 @@
       <c r="AE7" s="3" t="n">
         <v>33.7988</v>
       </c>
+      <c r="AF7" s="3" t="n">
+        <v>33.6592</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3008,16 +3077,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>32.2505</v>
+        <v>32.1815</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>51748.92654650001</v>
+        <v>51638.2096295</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>1748.926546500006</v>
+        <v>1638.209629500001</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.03497853093000013</v>
+        <v>0.03276419259000002</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -3085,6 +3154,9 @@
       <c r="AE8" s="3" t="n">
         <v>32.2505</v>
       </c>
+      <c r="AF8" s="3" t="n">
+        <v>32.1815</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3109,16 +3181,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>42.777</v>
+        <v>41.5956</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>137715.974361</v>
+        <v>133912.5834708</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>37715.974361</v>
+        <v>33912.58347079999</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.37715974361</v>
+        <v>0.3391258347079999</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -3186,6 +3258,9 @@
       <c r="AE9" s="3" t="n">
         <v>42.777</v>
       </c>
+      <c r="AF9" s="3" t="n">
+        <v>41.5956</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3210,16 +3285,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>47.0664</v>
+        <v>46.7192</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>133981.9911576</v>
+        <v>132993.6311528</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>33981.99115760002</v>
+        <v>32993.63115279999</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3398199115760002</v>
+        <v>0.329936311528</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -3287,6 +3362,9 @@
       <c r="AE10" s="3" t="n">
         <v>47.0664</v>
       </c>
+      <c r="AF10" s="3" t="n">
+        <v>46.7192</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3311,16 +3389,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>107.6649</v>
+        <v>102.5771</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>32398.4140431</v>
+        <v>30867.3983549</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>2398.414043099998</v>
+        <v>867.3983549000004</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.07994713476999993</v>
+        <v>0.02891327849666668</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -3388,6 +3466,9 @@
       <c r="AE11" s="3" t="n">
         <v>107.6649</v>
       </c>
+      <c r="AF11" s="3" t="n">
+        <v>102.5771</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3412,16 +3493,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>219.942</v>
+        <v>220.327</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>102387.839724</v>
+        <v>102567.065694</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>2387.839724000005</v>
+        <v>2567.065694000004</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.02387839724000005</v>
+        <v>0.02567065694000004</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -3489,6 +3570,9 @@
       <c r="AE12" s="3" t="n">
         <v>219.942</v>
       </c>
+      <c r="AF12" s="3" t="n">
+        <v>220.327</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3513,16 +3597,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>20.006</v>
+        <v>20.141</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>231821.62563</v>
+        <v>233385.952305</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>31821.62562999999</v>
+        <v>33385.95230499998</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.15910812815</v>
+        <v>0.1669297615249999</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -3590,6 +3674,9 @@
       <c r="AE13" s="3" t="n">
         <v>20.006</v>
       </c>
+      <c r="AF13" s="3" t="n">
+        <v>20.141</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3614,16 +3701,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>40.4025</v>
+        <v>39.0967</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>145756.301415</v>
+        <v>141045.4895002</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>45756.30141500002</v>
+        <v>41045.4895002</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.4575630141500002</v>
+        <v>0.410454895002</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -3691,6 +3778,9 @@
       <c r="AE14" s="3" t="n">
         <v>40.4025</v>
       </c>
+      <c r="AF14" s="3" t="n">
+        <v>39.0967</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3715,16 +3805,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.88</v>
+        <v>11.86</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>115758.09036</v>
+        <v>115563.21142</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>15758.09036</v>
+        <v>15563.21141999999</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1575809036</v>
+        <v>0.1556321141999999</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -3792,6 +3882,9 @@
       <c r="AE15" s="3" t="n">
         <v>11.88</v>
       </c>
+      <c r="AF15" s="3" t="n">
+        <v>11.86</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3816,16 +3909,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>25.3403</v>
+        <v>24.0484</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>145020.7123984</v>
+        <v>137627.2617152</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>45020.71239840001</v>
+        <v>37627.2617152</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4502071239840001</v>
+        <v>0.376272617152</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -3893,6 +3986,9 @@
       <c r="AE16" s="3" t="n">
         <v>25.3403</v>
       </c>
+      <c r="AF16" s="3" t="n">
+        <v>24.0484</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3917,16 +4013,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.678</v>
+        <v>16.5555</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55138.418646</v>
+        <v>54733.42666349999</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5138.418645999998</v>
+        <v>4733.426663499995</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.10276837292</v>
+        <v>0.0946685332699999</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -3994,6 +4090,9 @@
       <c r="AE17" s="3" t="n">
         <v>16.678</v>
       </c>
+      <c r="AF17" s="3" t="n">
+        <v>16.5555</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4018,16 +4117,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>44.41</v>
+        <v>44.45</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>83776.62275999998</v>
+        <v>83852.0802</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>3776.622759999984</v>
+        <v>3852.080199999997</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.0472077844999998</v>
+        <v>0.04815100249999996</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -4095,6 +4194,9 @@
       <c r="AE18" s="3" t="n">
         <v>44.41</v>
       </c>
+      <c r="AF18" s="3" t="n">
+        <v>44.45</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4119,16 +4221,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>15.0749</v>
+        <v>15.1077</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>218085.0507734</v>
+        <v>218559.5606982</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>68085.0507734</v>
+        <v>68559.56069819999</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.4539003384893333</v>
+        <v>0.4570637379879999</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -4196,6 +4298,9 @@
       <c r="AE19" s="3" t="n">
         <v>15.0749</v>
       </c>
+      <c r="AF19" s="3" t="n">
+        <v>15.1077</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4220,16 +4325,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.43</v>
+        <v>9.35</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>247592.22229</v>
+        <v>245491.75805</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-2407.777709999995</v>
+        <v>-4508.241949999996</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.009631110839999979</v>
+        <v>-0.01803296779999998</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -4297,6 +4402,9 @@
       <c r="AE20" s="3" t="n">
         <v>9.43</v>
       </c>
+      <c r="AF20" s="3" t="n">
+        <v>9.35</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4321,16 +4429,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>107.2602</v>
+        <v>107.3404</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>162956.0241918</v>
+        <v>163077.8687636</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-7043.97580819999</v>
+        <v>-6922.13123639999</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.04143515181294111</v>
+        <v>-0.040718419037647</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -4398,6 +4506,9 @@
       <c r="AE21" s="3" t="n">
         <v>107.2602</v>
       </c>
+      <c r="AF21" s="3" t="n">
+        <v>107.3404</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4422,16 +4533,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>45.53</v>
+        <v>44.024</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>69863.9638</v>
+        <v>67553.06704000001</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>9863.963799999998</v>
+        <v>7553.067040000009</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1643993966666666</v>
+        <v>0.1258844506666668</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -4499,6 +4610,9 @@
       <c r="AE22" s="3" t="n">
         <v>45.53</v>
       </c>
+      <c r="AF22" s="3" t="n">
+        <v>44.024</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4523,16 +4637,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>61.3103</v>
+        <v>61.2721</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>166547.4067101</v>
+        <v>166443.6376707</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>16547.40671010001</v>
+        <v>16443.6376707</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.1103160447340001</v>
+        <v>0.109624251138</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -4600,6 +4714,9 @@
       <c r="AE23" s="3" t="n">
         <v>61.3103</v>
       </c>
+      <c r="AF23" s="3" t="n">
+        <v>61.2721</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4624,16 +4741,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>28.4948</v>
+        <v>28.3825</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>103532.6073928</v>
+        <v>103124.578145</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>3532.607392800011</v>
+        <v>3124.578145000007</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.03532607392800011</v>
+        <v>0.03124578145000007</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -4701,6 +4818,9 @@
       <c r="AE24" s="3" t="n">
         <v>28.4948</v>
       </c>
+      <c r="AF24" s="3" t="n">
+        <v>28.3825</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4725,16 +4845,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.4191</v>
+        <v>11.4082</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>187520.7375734</v>
+        <v>187341.7413268</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-12479.26242660001</v>
+        <v>-12658.25867320001</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.06239631213300003</v>
+        <v>-0.06329129336600002</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -4802,6 +4922,9 @@
       <c r="AE25" s="3" t="n">
         <v>11.4191</v>
       </c>
+      <c r="AF25" s="3" t="n">
+        <v>11.4082</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4826,16 +4949,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>8.9727</v>
+        <v>8.976100000000001</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>107149.4261805</v>
+        <v>107190.0280115</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>-2850.573819500001</v>
+        <v>-2809.971988499994</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>-0.02591430745000001</v>
+        <v>-0.02554519989545449</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -4903,6 +5026,9 @@
       <c r="AE26" s="3" t="n">
         <v>8.9727</v>
       </c>
+      <c r="AF26" s="3" t="n">
+        <v>8.976100000000001</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4927,16 +5053,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>63.8198</v>
+        <v>63.773</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>102804.763028</v>
+        <v>102729.37478</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-7195.236971999999</v>
+        <v>-7270.625220000002</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.0654112452</v>
+        <v>-0.06609659290909092</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -5004,6 +5130,9 @@
       <c r="AE27" s="3" t="n">
         <v>63.8198</v>
       </c>
+      <c r="AF27" s="3" t="n">
+        <v>63.773</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -5028,16 +5157,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>104.9468</v>
+        <v>105.1126</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>347023.0708476</v>
+        <v>347571.3145782</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-32976.9291524</v>
+        <v>-32428.68542180001</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.08678139250631579</v>
+        <v>-0.08533864584684213</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -5105,6 +5234,9 @@
       <c r="AE28" s="3" t="n">
         <v>104.9468</v>
       </c>
+      <c r="AF28" s="3" t="n">
+        <v>105.1126</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -5129,16 +5261,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.885</v>
+        <v>11.8923</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>114140.010155</v>
+        <v>114210.1171869</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>14140.010155</v>
+        <v>14210.1171869</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.14140010155</v>
+        <v>0.142101171869</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -5206,6 +5338,9 @@
       <c r="AE29" s="3" t="n">
         <v>11.885</v>
       </c>
+      <c r="AF29" s="3" t="n">
+        <v>11.8923</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -5230,16 +5365,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>15.6929</v>
+        <v>15.5756</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>116062.5070869</v>
+        <v>115194.9725916</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>16062.50708689999</v>
+        <v>15194.9725916</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.1606250708689999</v>
+        <v>0.151949725916</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -5307,6 +5442,9 @@
       <c r="AE30" s="3" t="n">
         <v>15.6929</v>
       </c>
+      <c r="AF30" s="3" t="n">
+        <v>15.5756</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -5331,16 +5469,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>412.6834</v>
+        <v>412.3612</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>109806.799072</v>
+        <v>109721.068096</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>9806.799071999994</v>
+        <v>9721.068095999988</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.09806799071999994</v>
+        <v>0.09721068095999988</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -5408,6 +5546,9 @@
       <c r="AE31" s="3" t="n">
         <v>412.6834</v>
       </c>
+      <c r="AF31" s="3" t="n">
+        <v>412.3612</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -5432,16 +5573,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.15</v>
+        <v>10.14</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>214570.594</v>
+        <v>214359.1944</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>14570.59400000001</v>
+        <v>14359.19440000001</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.07285297000000006</v>
+        <v>0.07179597200000004</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -5509,6 +5650,9 @@
       <c r="AE32" s="3" t="n">
         <v>10.15</v>
       </c>
+      <c r="AF32" s="3" t="n">
+        <v>10.14</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -5533,16 +5677,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>17.81</v>
+        <v>17.86</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>63824.62839999999</v>
+        <v>64003.81039999999</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>3824.628399999994</v>
+        <v>4003.810399999995</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.06374380666666657</v>
+        <v>0.06673017333333325</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -5610,6 +5754,9 @@
       <c r="AE33" s="3" t="n">
         <v>17.81</v>
       </c>
+      <c r="AF33" s="3" t="n">
+        <v>17.86</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -5634,16 +5781,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>214.3516</v>
+        <v>212.8114</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>75351.2322996</v>
+        <v>74809.8042534</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-4648.7677004</v>
+        <v>-5190.195746600002</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.058109596255</v>
+        <v>-0.06487744683250003</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -5711,6 +5858,9 @@
       <c r="AE34" s="3" t="n">
         <v>214.3516</v>
       </c>
+      <c r="AF34" s="3" t="n">
+        <v>212.8114</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -5735,16 +5885,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>14.7</v>
+        <v>14.58</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>104890.7181</v>
+        <v>104034.46734</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>4890.718099999998</v>
+        <v>4034.467340000003</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.04890718099999998</v>
+        <v>0.04034467340000003</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -5812,6 +5962,9 @@
       <c r="AE35" s="3" t="n">
         <v>14.7</v>
       </c>
+      <c r="AF35" s="3" t="n">
+        <v>14.58</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5836,16 +5989,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>347.6696</v>
+        <v>349.8142</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>161911.8187376</v>
+        <v>162910.5718252</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>11911.8187376</v>
+        <v>12910.57182520002</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.07941212491733332</v>
+        <v>0.08607047883466681</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -5913,6 +6066,9 @@
       <c r="AE36" s="3" t="n">
         <v>347.6696</v>
       </c>
+      <c r="AF36" s="3" t="n">
+        <v>349.8142</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5937,16 +6093,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>15.619</v>
+        <v>15.752</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>58772.563291</v>
+        <v>59273.02752800001</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>8772.563290999999</v>
+        <v>9273.027528000006</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.17545126582</v>
+        <v>0.1854605505600001</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -6014,6 +6170,9 @@
       <c r="AE37" s="3" t="n">
         <v>15.619</v>
       </c>
+      <c r="AF37" s="3" t="n">
+        <v>15.752</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -6038,16 +6197,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.9354</v>
+        <v>13.9096</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>83340.4088628</v>
+        <v>83186.1124272</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>3340.408862800003</v>
+        <v>3186.112427200002</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.04175511078500004</v>
+        <v>0.03982640534000002</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -6115,6 +6274,9 @@
       <c r="AE38" s="3" t="n">
         <v>13.9354</v>
       </c>
+      <c r="AF38" s="3" t="n">
+        <v>13.9096</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -6139,16 +6301,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1011.0558</v>
+        <v>1014.0349</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50432.4743598</v>
+        <v>50581.0748469</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>432.4743597999986</v>
+        <v>581.0748469000027</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.008649487195999972</v>
+        <v>0.01162149693800005</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -6216,6 +6378,9 @@
       <c r="AE39" s="3" t="n">
         <v>1011.0558</v>
       </c>
+      <c r="AF39" s="3" t="n">
+        <v>1014.0349</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -6240,16 +6405,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>20.3557</v>
+        <v>20.3998</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>102613.6333039</v>
+        <v>102835.9425946</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>2613.633303900002</v>
+        <v>2835.942594599997</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.02613633303900002</v>
+        <v>0.02835942594599997</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -6317,6 +6482,9 @@
       <c r="AE40" s="3" t="n">
         <v>20.3557</v>
       </c>
+      <c r="AF40" s="3" t="n">
+        <v>20.3998</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
@@ -6328,13 +6496,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4878416.3532113</v>
+        <v>4847032.155924</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>408416.3532113001</v>
+        <v>377032.155924</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.09136831168038033</v>
+        <v>0.08434723846174495</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-06-07
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-06 05:53 IST</t>
+          <t>Generated: 2026-06-07 06:22 IST</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-06-06</t>
+          <t>Last snapshot: 2026-06-07</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE19"/>
+  <dimension ref="A1:AF19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -650,6 +650,7 @@
     <col width="21" customWidth="1" min="29" max="29"/>
     <col width="21" customWidth="1" min="30" max="30"/>
     <col width="21" customWidth="1" min="31" max="31"/>
+    <col width="21" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -808,6 +809,11 @@
           <t>2026-06-06</t>
         </is>
       </c>
+      <c r="AF1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -907,6 +913,9 @@
       <c r="AE2" s="3" t="n">
         <v>601.75</v>
       </c>
+      <c r="AF2" s="3" t="n">
+        <v>601.75</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1033,6 +1042,9 @@
       <c r="AE4" s="3" t="n">
         <v>1518.800048828125</v>
       </c>
+      <c r="AF4" s="3" t="n">
+        <v>1518.800048828125</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1132,6 +1144,9 @@
       <c r="AE5" s="3" t="n">
         <v>654.9500122070312</v>
       </c>
+      <c r="AF5" s="3" t="n">
+        <v>654.9500122070312</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1231,6 +1246,9 @@
       <c r="AE6" s="3" t="n">
         <v>382.1000061035156</v>
       </c>
+      <c r="AF6" s="3" t="n">
+        <v>382.1000061035156</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1330,6 +1348,9 @@
       <c r="AE7" s="3" t="n">
         <v>237.7799987792969</v>
       </c>
+      <c r="AF7" s="3" t="n">
+        <v>237.7799987792969</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1456,6 +1477,9 @@
       <c r="AE9" s="3" t="n">
         <v>19.03000068664551</v>
       </c>
+      <c r="AF9" s="3" t="n">
+        <v>19.03000068664551</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1555,6 +1579,9 @@
       <c r="AE10" s="3" t="n">
         <v>483.3500061035156</v>
       </c>
+      <c r="AF10" s="3" t="n">
+        <v>483.3500061035156</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1654,6 +1681,9 @@
       <c r="AE11" s="3" t="n">
         <v>9.180000305175781</v>
       </c>
+      <c r="AF11" s="3" t="n">
+        <v>9.180000305175781</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1753,6 +1783,9 @@
       <c r="AE12" s="3" t="n">
         <v>2614.89990234375</v>
       </c>
+      <c r="AF12" s="3" t="n">
+        <v>2614.89990234375</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1852,6 +1885,9 @@
       <c r="AE13" s="3" t="n">
         <v>55.31000137329102</v>
       </c>
+      <c r="AF13" s="3" t="n">
+        <v>55.31000137329102</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1951,6 +1987,9 @@
       <c r="AE14" s="3" t="n">
         <v>719.2999877929688</v>
       </c>
+      <c r="AF14" s="3" t="n">
+        <v>719.2999877929688</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2104,6 +2143,9 @@
       <c r="AE17" s="3" t="n">
         <v>576.2000122070312</v>
       </c>
+      <c r="AF17" s="3" t="n">
+        <v>576.2000122070312</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2201,6 +2243,9 @@
         <v>411.8999938964844</v>
       </c>
       <c r="AE18" s="3" t="n">
+        <v>409.2000122070312</v>
+      </c>
+      <c r="AF18" s="3" t="n">
         <v>409.2000122070312</v>
       </c>
     </row>
@@ -2231,7 +2276,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF41"/>
+  <dimension ref="A1:AG41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2266,6 +2311,7 @@
     <col width="13" customWidth="1" min="30" max="30"/>
     <col width="13" customWidth="1" min="31" max="31"/>
     <col width="13" customWidth="1" min="32" max="32"/>
+    <col width="13" customWidth="1" min="33" max="33"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2429,6 +2475,11 @@
           <t>2026-06-06</t>
         </is>
       </c>
+      <c r="AG1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2533,6 +2584,9 @@
       <c r="AF2" s="3" t="n">
         <v>55.7267</v>
       </c>
+      <c r="AG2" s="3" t="n">
+        <v>55.7267</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2637,6 +2691,9 @@
       <c r="AF3" s="3" t="n">
         <v>25.5603</v>
       </c>
+      <c r="AG3" s="3" t="n">
+        <v>25.5603</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2741,6 +2798,9 @@
       <c r="AF4" s="3" t="n">
         <v>12.5</v>
       </c>
+      <c r="AG4" s="3" t="n">
+        <v>12.5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2845,6 +2905,9 @@
       <c r="AF5" s="3" t="n">
         <v>9.411099999999999</v>
       </c>
+      <c r="AG5" s="3" t="n">
+        <v>9.411099999999999</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2949,6 +3012,9 @@
       <c r="AF6" s="3" t="n">
         <v>12.3606</v>
       </c>
+      <c r="AG6" s="3" t="n">
+        <v>12.3606</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3053,6 +3119,9 @@
       <c r="AF7" s="3" t="n">
         <v>33.6592</v>
       </c>
+      <c r="AG7" s="3" t="n">
+        <v>33.6592</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3157,6 +3226,9 @@
       <c r="AF8" s="3" t="n">
         <v>32.1815</v>
       </c>
+      <c r="AG8" s="3" t="n">
+        <v>32.1815</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3261,6 +3333,9 @@
       <c r="AF9" s="3" t="n">
         <v>41.5956</v>
       </c>
+      <c r="AG9" s="3" t="n">
+        <v>41.5956</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3365,6 +3440,9 @@
       <c r="AF10" s="3" t="n">
         <v>46.7192</v>
       </c>
+      <c r="AG10" s="3" t="n">
+        <v>46.7192</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3469,6 +3547,9 @@
       <c r="AF11" s="3" t="n">
         <v>102.5771</v>
       </c>
+      <c r="AG11" s="3" t="n">
+        <v>102.5771</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3573,6 +3654,9 @@
       <c r="AF12" s="3" t="n">
         <v>220.327</v>
       </c>
+      <c r="AG12" s="3" t="n">
+        <v>220.327</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3677,6 +3761,9 @@
       <c r="AF13" s="3" t="n">
         <v>20.141</v>
       </c>
+      <c r="AG13" s="3" t="n">
+        <v>20.141</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3781,6 +3868,9 @@
       <c r="AF14" s="3" t="n">
         <v>39.0967</v>
       </c>
+      <c r="AG14" s="3" t="n">
+        <v>39.0967</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3885,6 +3975,9 @@
       <c r="AF15" s="3" t="n">
         <v>11.86</v>
       </c>
+      <c r="AG15" s="3" t="n">
+        <v>11.86</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3989,6 +4082,9 @@
       <c r="AF16" s="3" t="n">
         <v>24.0484</v>
       </c>
+      <c r="AG16" s="3" t="n">
+        <v>24.0484</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4093,6 +4189,9 @@
       <c r="AF17" s="3" t="n">
         <v>16.5555</v>
       </c>
+      <c r="AG17" s="3" t="n">
+        <v>16.5555</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4197,6 +4296,9 @@
       <c r="AF18" s="3" t="n">
         <v>44.45</v>
       </c>
+      <c r="AG18" s="3" t="n">
+        <v>44.45</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4301,6 +4403,9 @@
       <c r="AF19" s="3" t="n">
         <v>15.1077</v>
       </c>
+      <c r="AG19" s="3" t="n">
+        <v>15.1077</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4405,6 +4510,9 @@
       <c r="AF20" s="3" t="n">
         <v>9.35</v>
       </c>
+      <c r="AG20" s="3" t="n">
+        <v>9.35</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4509,6 +4617,9 @@
       <c r="AF21" s="3" t="n">
         <v>107.3404</v>
       </c>
+      <c r="AG21" s="3" t="n">
+        <v>107.3404</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4613,6 +4724,9 @@
       <c r="AF22" s="3" t="n">
         <v>44.024</v>
       </c>
+      <c r="AG22" s="3" t="n">
+        <v>44.024</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4717,6 +4831,9 @@
       <c r="AF23" s="3" t="n">
         <v>61.2721</v>
       </c>
+      <c r="AG23" s="3" t="n">
+        <v>61.2721</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4821,6 +4938,9 @@
       <c r="AF24" s="3" t="n">
         <v>28.3825</v>
       </c>
+      <c r="AG24" s="3" t="n">
+        <v>28.3825</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4925,6 +5045,9 @@
       <c r="AF25" s="3" t="n">
         <v>11.4082</v>
       </c>
+      <c r="AG25" s="3" t="n">
+        <v>11.4082</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -5029,6 +5152,9 @@
       <c r="AF26" s="3" t="n">
         <v>8.976100000000001</v>
       </c>
+      <c r="AG26" s="3" t="n">
+        <v>8.976100000000001</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5133,6 +5259,9 @@
       <c r="AF27" s="3" t="n">
         <v>63.773</v>
       </c>
+      <c r="AG27" s="3" t="n">
+        <v>63.773</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -5237,6 +5366,9 @@
       <c r="AF28" s="3" t="n">
         <v>105.1126</v>
       </c>
+      <c r="AG28" s="3" t="n">
+        <v>105.1126</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -5341,6 +5473,9 @@
       <c r="AF29" s="3" t="n">
         <v>11.8923</v>
       </c>
+      <c r="AG29" s="3" t="n">
+        <v>11.8923</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -5445,6 +5580,9 @@
       <c r="AF30" s="3" t="n">
         <v>15.5756</v>
       </c>
+      <c r="AG30" s="3" t="n">
+        <v>15.5756</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -5549,6 +5687,9 @@
       <c r="AF31" s="3" t="n">
         <v>412.3612</v>
       </c>
+      <c r="AG31" s="3" t="n">
+        <v>412.3612</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -5653,6 +5794,9 @@
       <c r="AF32" s="3" t="n">
         <v>10.14</v>
       </c>
+      <c r="AG32" s="3" t="n">
+        <v>10.14</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -5757,6 +5901,9 @@
       <c r="AF33" s="3" t="n">
         <v>17.86</v>
       </c>
+      <c r="AG33" s="3" t="n">
+        <v>17.86</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -5861,6 +6008,9 @@
       <c r="AF34" s="3" t="n">
         <v>212.8114</v>
       </c>
+      <c r="AG34" s="3" t="n">
+        <v>212.8114</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -5965,6 +6115,9 @@
       <c r="AF35" s="3" t="n">
         <v>14.58</v>
       </c>
+      <c r="AG35" s="3" t="n">
+        <v>14.58</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -6069,6 +6222,9 @@
       <c r="AF36" s="3" t="n">
         <v>349.8142</v>
       </c>
+      <c r="AG36" s="3" t="n">
+        <v>349.8142</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -6173,6 +6329,9 @@
       <c r="AF37" s="3" t="n">
         <v>15.752</v>
       </c>
+      <c r="AG37" s="3" t="n">
+        <v>15.752</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -6277,6 +6436,9 @@
       <c r="AF38" s="3" t="n">
         <v>13.9096</v>
       </c>
+      <c r="AG38" s="3" t="n">
+        <v>13.9096</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -6381,6 +6543,9 @@
       <c r="AF39" s="3" t="n">
         <v>1014.0349</v>
       </c>
+      <c r="AG39" s="3" t="n">
+        <v>1014.0349</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -6483,6 +6648,9 @@
         <v>20.3557</v>
       </c>
       <c r="AF40" s="3" t="n">
+        <v>20.3998</v>
+      </c>
+      <c r="AG40" s="3" t="n">
         <v>20.3998</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily portfolio update 2026-06-08
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -484,7 +484,7 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-07 06:22 IST</t>
+          <t>Generated: 2026-06-08 06:41 IST</t>
         </is>
       </c>
     </row>
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>563537.5043563843</v>
+        <v>562102.4972991943</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-27244.51564361574</v>
+        <v>-28679.52270080568</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.04611602032779491</v>
+        <v>-0.04854501614792827</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5410569.660280384</v>
+        <v>5409134.653223194</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>349787.6402803846</v>
+        <v>348352.6332231946</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.06911731011097463</v>
+        <v>0.06883375570149426</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-06-07</t>
+          <t>Last snapshot: 2026-06-08</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF19"/>
+  <dimension ref="A1:AG19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -651,6 +651,7 @@
     <col width="21" customWidth="1" min="30" max="30"/>
     <col width="21" customWidth="1" min="31" max="31"/>
     <col width="21" customWidth="1" min="32" max="32"/>
+    <col width="21" customWidth="1" min="33" max="33"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -814,6 +815,11 @@
           <t>2026-06-07</t>
         </is>
       </c>
+      <c r="AG1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -833,13 +839,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>601.75</v>
+        <v>585.3499755859375</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>48140</v>
+        <v>46827.998046875</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>4322.489999999998</v>
+        <v>3010.488046874998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -915,6 +921,9 @@
       </c>
       <c r="AF2" s="3" t="n">
         <v>601.75</v>
+      </c>
+      <c r="AG2" s="3" t="n">
+        <v>585.3499755859375</v>
       </c>
     </row>
     <row r="3">
@@ -962,13 +971,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1518.800048828125</v>
+        <v>1541.599975585938</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>30376.0009765625</v>
+        <v>30831.99951171875</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-1728.579023437502</v>
+        <v>-1272.580488281252</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1044,6 +1053,9 @@
       </c>
       <c r="AF4" s="3" t="n">
         <v>1518.800048828125</v>
+      </c>
+      <c r="AG4" s="3" t="n">
+        <v>1541.599975585938</v>
       </c>
     </row>
     <row r="5">
@@ -1064,13 +1076,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>654.9500122070312</v>
+        <v>653.1500244140625</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13099.00024414062</v>
+        <v>13063.00048828125</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1114.099755859375</v>
+        <v>-1150.09951171875</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1146,6 +1158,9 @@
       </c>
       <c r="AF5" s="3" t="n">
         <v>654.9500122070312</v>
+      </c>
+      <c r="AG5" s="3" t="n">
+        <v>653.1500244140625</v>
       </c>
     </row>
     <row r="6">
@@ -1166,13 +1181,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>382.1000061035156</v>
+        <v>380.5499877929688</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15284.00024414062</v>
+        <v>15221.99951171875</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2218.239755859377</v>
+        <v>-2280.240488281252</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1248,6 +1263,9 @@
       </c>
       <c r="AF6" s="3" t="n">
         <v>382.1000061035156</v>
+      </c>
+      <c r="AG6" s="3" t="n">
+        <v>380.5499877929688</v>
       </c>
     </row>
     <row r="7">
@@ -1268,13 +1286,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>237.7799987792969</v>
+        <v>242.2799987792969</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>23777.99987792969</v>
+        <v>24227.99987792969</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-2655.820122070312</v>
+        <v>-2205.820122070312</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1350,6 +1368,9 @@
       </c>
       <c r="AF7" s="3" t="n">
         <v>237.7799987792969</v>
+      </c>
+      <c r="AG7" s="3" t="n">
+        <v>242.2799987792969</v>
       </c>
     </row>
     <row r="8">
@@ -1397,13 +1418,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>19.03000068664551</v>
+        <v>18.86000061035156</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>28545.00102996826</v>
+        <v>28290.00091552734</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-2505.168970031737</v>
+        <v>-2760.169084472655</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1479,6 +1500,9 @@
       </c>
       <c r="AF9" s="3" t="n">
         <v>19.03000068664551</v>
+      </c>
+      <c r="AG9" s="3" t="n">
+        <v>18.86000061035156</v>
       </c>
     </row>
     <row r="10">
@@ -1499,13 +1523,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>483.3500061035156</v>
+        <v>491.0499877929688</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48335.00061035156</v>
+        <v>49104.99877929688</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-3163.479389648441</v>
+        <v>-2393.481220703128</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1581,6 +1605,9 @@
       </c>
       <c r="AF10" s="3" t="n">
         <v>483.3500061035156</v>
+      </c>
+      <c r="AG10" s="3" t="n">
+        <v>491.0499877929688</v>
       </c>
     </row>
     <row r="11">
@@ -1601,13 +1628,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>9.180000305175781</v>
+        <v>8.989999771118164</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>9180.000305175781</v>
+        <v>8989.999771118164</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-661.2096948242179</v>
+        <v>-851.2102288818351</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -1683,6 +1710,9 @@
       </c>
       <c r="AF11" s="3" t="n">
         <v>9.180000305175781</v>
+      </c>
+      <c r="AG11" s="3" t="n">
+        <v>8.989999771118164</v>
       </c>
     </row>
     <row r="12">
@@ -1703,13 +1733,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2614.89990234375</v>
+        <v>2580.300048828125</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>26148.9990234375</v>
+        <v>25803.00048828125</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-1574.2509765625</v>
+        <v>-1920.24951171875</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -1785,6 +1815,9 @@
       </c>
       <c r="AF12" s="3" t="n">
         <v>2614.89990234375</v>
+      </c>
+      <c r="AG12" s="3" t="n">
+        <v>2580.300048828125</v>
       </c>
     </row>
     <row r="13">
@@ -1805,13 +1838,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>55.31000137329102</v>
+        <v>55.15999984741211</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>33186.00082397461</v>
+        <v>33095.99990844727</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-1845.759176025393</v>
+        <v>-1935.760091552736</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -1887,6 +1920,9 @@
       </c>
       <c r="AF13" s="3" t="n">
         <v>55.31000137329102</v>
+      </c>
+      <c r="AG13" s="3" t="n">
+        <v>55.15999984741211</v>
       </c>
     </row>
     <row r="14">
@@ -1907,13 +1943,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>719.2999877929688</v>
+        <v>723.0999755859375</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>35964.99938964844</v>
+        <v>36154.99877929688</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-6497.510610351565</v>
+        <v>-6307.511220703127</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -1989,6 +2025,9 @@
       </c>
       <c r="AF14" s="3" t="n">
         <v>719.2999877929688</v>
+      </c>
+      <c r="AG14" s="3" t="n">
+        <v>723.0999755859375</v>
       </c>
     </row>
     <row r="15">
@@ -2063,13 +2102,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>576.2000122070312</v>
+        <v>559.7000122070312</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>28810.00061035156</v>
+        <v>27985.00061035156</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>7055.470610351564</v>
+        <v>6230.470610351564</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -2145,6 +2184,9 @@
       </c>
       <c r="AF17" s="3" t="n">
         <v>576.2000122070312</v>
+      </c>
+      <c r="AG17" s="3" t="n">
+        <v>559.7000122070312</v>
       </c>
     </row>
     <row r="18">
@@ -2165,13 +2207,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>409.2000122070312</v>
+        <v>407.3500061035156</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>40920.00122070312</v>
+        <v>40735.00061035156</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-5720.818779296875</v>
+        <v>-5905.819389648437</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -2247,6 +2289,9 @@
       </c>
       <c r="AF18" s="3" t="n">
         <v>409.2000122070312</v>
+      </c>
+      <c r="AG18" s="3" t="n">
+        <v>407.3500061035156</v>
       </c>
     </row>
     <row r="19">
@@ -2259,10 +2304,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>563537.5043563843</v>
+        <v>562102.4972991943</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-27244.51564361573</v>
+        <v>-28679.52270080568</v>
       </c>
     </row>
   </sheetData>
@@ -2276,7 +2321,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG41"/>
+  <dimension ref="A1:AH41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2312,6 +2357,7 @@
     <col width="13" customWidth="1" min="31" max="31"/>
     <col width="13" customWidth="1" min="32" max="32"/>
     <col width="13" customWidth="1" min="33" max="33"/>
+    <col width="13" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2480,6 +2526,11 @@
           <t>2026-06-07</t>
         </is>
       </c>
+      <c r="AH1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2587,6 +2638,9 @@
       <c r="AG2" s="3" t="n">
         <v>55.7267</v>
       </c>
+      <c r="AH2" s="3" t="n">
+        <v>55.7267</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3015,6 +3069,9 @@
       <c r="AG6" s="3" t="n">
         <v>12.3606</v>
       </c>
+      <c r="AH6" s="3" t="n">
+        <v>12.3606</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3229,6 +3286,9 @@
       <c r="AG8" s="3" t="n">
         <v>32.1815</v>
       </c>
+      <c r="AH8" s="3" t="n">
+        <v>32.1815</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3657,6 +3717,9 @@
       <c r="AG12" s="3" t="n">
         <v>220.327</v>
       </c>
+      <c r="AH12" s="3" t="n">
+        <v>220.327</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3764,6 +3827,9 @@
       <c r="AG13" s="3" t="n">
         <v>20.141</v>
       </c>
+      <c r="AH13" s="3" t="n">
+        <v>20.141</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3978,6 +4044,9 @@
       <c r="AG15" s="3" t="n">
         <v>11.86</v>
       </c>
+      <c r="AH15" s="3" t="n">
+        <v>11.86</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4299,6 +4368,9 @@
       <c r="AG18" s="3" t="n">
         <v>44.45</v>
       </c>
+      <c r="AH18" s="3" t="n">
+        <v>44.45</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4513,6 +4585,9 @@
       <c r="AG20" s="3" t="n">
         <v>9.35</v>
       </c>
+      <c r="AH20" s="3" t="n">
+        <v>9.35</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4620,6 +4695,9 @@
       <c r="AG21" s="3" t="n">
         <v>107.3404</v>
       </c>
+      <c r="AH21" s="3" t="n">
+        <v>107.3404</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4834,6 +4912,9 @@
       <c r="AG23" s="3" t="n">
         <v>61.2721</v>
       </c>
+      <c r="AH23" s="3" t="n">
+        <v>61.2721</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5048,6 +5129,9 @@
       <c r="AG25" s="3" t="n">
         <v>11.4082</v>
       </c>
+      <c r="AH25" s="3" t="n">
+        <v>11.4082</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -5155,6 +5239,9 @@
       <c r="AG26" s="3" t="n">
         <v>8.976100000000001</v>
       </c>
+      <c r="AH26" s="3" t="n">
+        <v>8.976100000000001</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5262,6 +5349,9 @@
       <c r="AG27" s="3" t="n">
         <v>63.773</v>
       </c>
+      <c r="AH27" s="3" t="n">
+        <v>63.773</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -5369,6 +5459,9 @@
       <c r="AG28" s="3" t="n">
         <v>105.1126</v>
       </c>
+      <c r="AH28" s="3" t="n">
+        <v>105.1126</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -5690,6 +5783,9 @@
       <c r="AG31" s="3" t="n">
         <v>412.3612</v>
       </c>
+      <c r="AH31" s="3" t="n">
+        <v>412.3612</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -5797,6 +5893,9 @@
       <c r="AG32" s="3" t="n">
         <v>10.14</v>
       </c>
+      <c r="AH32" s="3" t="n">
+        <v>10.14</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -6011,6 +6110,9 @@
       <c r="AG34" s="3" t="n">
         <v>212.8114</v>
       </c>
+      <c r="AH34" s="3" t="n">
+        <v>212.8114</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -6118,6 +6220,9 @@
       <c r="AG35" s="3" t="n">
         <v>14.58</v>
       </c>
+      <c r="AH35" s="3" t="n">
+        <v>14.58</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -6225,6 +6330,9 @@
       <c r="AG36" s="3" t="n">
         <v>349.8142</v>
       </c>
+      <c r="AH36" s="3" t="n">
+        <v>349.8142</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -6332,6 +6440,9 @@
       <c r="AG37" s="3" t="n">
         <v>15.752</v>
       </c>
+      <c r="AH37" s="3" t="n">
+        <v>15.752</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -6651,6 +6762,9 @@
         <v>20.3998</v>
       </c>
       <c r="AG40" s="3" t="n">
+        <v>20.3998</v>
+      </c>
+      <c r="AH40" s="3" t="n">
         <v>20.3998</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily portfolio update 2026-06-09
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -484,7 +484,7 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-08 06:41 IST</t>
+          <t>Generated: 2026-06-09 06:07 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4847032.155924</v>
+        <v>4785519.4604006</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>377032.1559239998</v>
+        <v>315519.4604006</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.08434723846174494</v>
+        <v>0.07058600903816555</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>562102.4972991943</v>
+        <v>555158.5032348633</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-28679.52270080568</v>
+        <v>-35623.51676513674</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.04854501614792827</v>
+        <v>-0.06029891831362223</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5409134.653223194</v>
+        <v>5340677.963635463</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>348352.6332231946</v>
+        <v>279895.9436354637</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.06883375570149426</v>
+        <v>0.05530685623868537</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-06-08</t>
+          <t>Last snapshot: 2026-06-09</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG19"/>
+  <dimension ref="A1:AH19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -652,6 +652,7 @@
     <col width="21" customWidth="1" min="31" max="31"/>
     <col width="21" customWidth="1" min="32" max="32"/>
     <col width="21" customWidth="1" min="33" max="33"/>
+    <col width="21" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -820,6 +821,11 @@
           <t>2026-06-08</t>
         </is>
       </c>
+      <c r="AH1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -839,13 +845,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>585.3499755859375</v>
+        <v>574.1500244140625</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>46827.998046875</v>
+        <v>45932.001953125</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>3010.488046874998</v>
+        <v>2114.491953124998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -924,6 +930,9 @@
       </c>
       <c r="AG2" s="3" t="n">
         <v>585.3499755859375</v>
+      </c>
+      <c r="AH2" s="3" t="n">
+        <v>574.1500244140625</v>
       </c>
     </row>
     <row r="3">
@@ -971,13 +980,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1541.599975585938</v>
+        <v>1520.400024414062</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>30831.99951171875</v>
+        <v>30408.00048828125</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-1272.580488281252</v>
+        <v>-1696.579511718752</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1056,6 +1065,9 @@
       </c>
       <c r="AG4" s="3" t="n">
         <v>1541.599975585938</v>
+      </c>
+      <c r="AH4" s="3" t="n">
+        <v>1520.400024414062</v>
       </c>
     </row>
     <row r="5">
@@ -1076,13 +1088,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>653.1500244140625</v>
+        <v>652.3499755859375</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13063.00048828125</v>
+        <v>13046.99951171875</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1150.09951171875</v>
+        <v>-1166.10048828125</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1161,6 +1173,9 @@
       </c>
       <c r="AG5" s="3" t="n">
         <v>653.1500244140625</v>
+      </c>
+      <c r="AH5" s="3" t="n">
+        <v>652.3499755859375</v>
       </c>
     </row>
     <row r="6">
@@ -1181,13 +1196,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>380.5499877929688</v>
+        <v>380.8999938964844</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15221.99951171875</v>
+        <v>15235.99975585938</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2280.240488281252</v>
+        <v>-2266.240244140627</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1266,6 +1281,9 @@
       </c>
       <c r="AG6" s="3" t="n">
         <v>380.5499877929688</v>
+      </c>
+      <c r="AH6" s="3" t="n">
+        <v>380.8999938964844</v>
       </c>
     </row>
     <row r="7">
@@ -1286,13 +1304,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>242.2799987792969</v>
+        <v>237.2700042724609</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>24227.99987792969</v>
+        <v>23727.00042724609</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-2205.820122070312</v>
+        <v>-2706.819572753906</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1371,6 +1389,9 @@
       </c>
       <c r="AG7" s="3" t="n">
         <v>242.2799987792969</v>
+      </c>
+      <c r="AH7" s="3" t="n">
+        <v>237.2700042724609</v>
       </c>
     </row>
     <row r="8">
@@ -1418,13 +1439,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>18.86000061035156</v>
+        <v>18.48999977111816</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>28290.00091552734</v>
+        <v>27734.99965667725</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-2760.169084472655</v>
+        <v>-3315.170343322752</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1503,6 +1524,9 @@
       </c>
       <c r="AG9" s="3" t="n">
         <v>18.86000061035156</v>
+      </c>
+      <c r="AH9" s="3" t="n">
+        <v>18.48999977111816</v>
       </c>
     </row>
     <row r="10">
@@ -1523,13 +1547,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>491.0499877929688</v>
+        <v>475.7000122070312</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>49104.99877929688</v>
+        <v>47570.00122070312</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-2393.481220703128</v>
+        <v>-3928.478779296878</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1608,6 +1632,9 @@
       </c>
       <c r="AG10" s="3" t="n">
         <v>491.0499877929688</v>
+      </c>
+      <c r="AH10" s="3" t="n">
+        <v>475.7000122070312</v>
       </c>
     </row>
     <row r="11">
@@ -1628,13 +1655,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>8.989999771118164</v>
+        <v>8.890000343322754</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>8989.999771118164</v>
+        <v>8890.000343322754</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-851.2102288818351</v>
+        <v>-951.2096566772452</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -1713,6 +1740,9 @@
       </c>
       <c r="AG11" s="3" t="n">
         <v>8.989999771118164</v>
+      </c>
+      <c r="AH11" s="3" t="n">
+        <v>8.890000343322754</v>
       </c>
     </row>
     <row r="12">
@@ -1733,13 +1763,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2580.300048828125</v>
+        <v>2557.800048828125</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25803.00048828125</v>
+        <v>25578.00048828125</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-1920.24951171875</v>
+        <v>-2145.24951171875</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -1818,6 +1848,9 @@
       </c>
       <c r="AG12" s="3" t="n">
         <v>2580.300048828125</v>
+      </c>
+      <c r="AH12" s="3" t="n">
+        <v>2557.800048828125</v>
       </c>
     </row>
     <row r="13">
@@ -1838,13 +1871,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>55.15999984741211</v>
+        <v>54.75</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>33095.99990844727</v>
+        <v>32850</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-1935.760091552736</v>
+        <v>-2181.760000000002</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -1923,6 +1956,9 @@
       </c>
       <c r="AG13" s="3" t="n">
         <v>55.15999984741211</v>
+      </c>
+      <c r="AH13" s="3" t="n">
+        <v>54.75</v>
       </c>
     </row>
     <row r="14">
@@ -1943,13 +1979,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>723.0999755859375</v>
+        <v>714.0999755859375</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>36154.99877929688</v>
+        <v>35704.99877929688</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-6307.511220703127</v>
+        <v>-6757.511220703127</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -2028,6 +2064,9 @@
       </c>
       <c r="AG14" s="3" t="n">
         <v>723.0999755859375</v>
+      </c>
+      <c r="AH14" s="3" t="n">
+        <v>714.0999755859375</v>
       </c>
     </row>
     <row r="15">
@@ -2102,13 +2141,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>559.7000122070312</v>
+        <v>534.4000244140625</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>27985.00061035156</v>
+        <v>26720.00122070312</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>6230.470610351564</v>
+        <v>4965.471220703126</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -2187,6 +2226,9 @@
       </c>
       <c r="AG17" s="3" t="n">
         <v>559.7000122070312</v>
+      </c>
+      <c r="AH17" s="3" t="n">
+        <v>534.4000244140625</v>
       </c>
     </row>
     <row r="18">
@@ -2207,13 +2249,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>407.3500061035156</v>
+        <v>399.8999938964844</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>40735.00061035156</v>
+        <v>39989.99938964844</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-5905.819389648437</v>
+        <v>-6650.820610351562</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -2292,6 +2334,9 @@
       </c>
       <c r="AG18" s="3" t="n">
         <v>407.3500061035156</v>
+      </c>
+      <c r="AH18" s="3" t="n">
+        <v>399.8999938964844</v>
       </c>
     </row>
     <row r="19">
@@ -2304,10 +2349,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>562102.4972991943</v>
+        <v>555158.5032348633</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-28679.52270080568</v>
+        <v>-35623.51676513673</v>
       </c>
     </row>
   </sheetData>
@@ -2321,7 +2366,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH41"/>
+  <dimension ref="A1:AI41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2358,6 +2403,7 @@
     <col width="13" customWidth="1" min="32" max="32"/>
     <col width="13" customWidth="1" min="33" max="33"/>
     <col width="13" customWidth="1" min="34" max="34"/>
+    <col width="13" customWidth="1" min="35" max="35"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2531,6 +2577,11 @@
           <t>2026-06-08</t>
         </is>
       </c>
+      <c r="AI1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2555,16 +2606,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>55.7267</v>
+        <v>56.2466</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>62552.2176694</v>
+        <v>63135.7960612</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>12552.2176694</v>
+        <v>13135.7960612</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.251044353388</v>
+        <v>0.2627159212240001</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -2640,6 +2691,9 @@
       </c>
       <c r="AH2" s="3" t="n">
         <v>55.7267</v>
+      </c>
+      <c r="AI2" s="3" t="n">
+        <v>56.2466</v>
       </c>
     </row>
     <row r="3">
@@ -2665,16 +2719,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.5603</v>
+        <v>25.3399</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>62755.98084390001</v>
+        <v>62214.85189870001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>2755.980843900012</v>
+        <v>2214.851898700006</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.04593301406500019</v>
+        <v>0.03691419831166677</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -2747,6 +2801,9 @@
       </c>
       <c r="AG3" s="3" t="n">
         <v>25.5603</v>
+      </c>
+      <c r="AI3" s="3" t="n">
+        <v>25.3399</v>
       </c>
     </row>
     <row r="4">
@@ -2772,16 +2829,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.5</v>
+        <v>12.38</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>240076.1625</v>
+        <v>237771.43134</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>60076.16250000001</v>
+        <v>57771.43134000001</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3337564583333333</v>
+        <v>0.3209523963333334</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -2854,6 +2911,9 @@
       </c>
       <c r="AG4" s="3" t="n">
         <v>12.5</v>
+      </c>
+      <c r="AI4" s="3" t="n">
+        <v>12.38</v>
       </c>
     </row>
     <row r="5">
@@ -2879,16 +2939,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.411099999999999</v>
+        <v>9.3378</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>172732.1575768</v>
+        <v>171386.8029264</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-37267.84242320003</v>
+        <v>-38613.19707360002</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1774659163009525</v>
+        <v>-0.183872367017143</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -2961,6 +3021,9 @@
       </c>
       <c r="AG5" s="3" t="n">
         <v>9.411099999999999</v>
+      </c>
+      <c r="AI5" s="3" t="n">
+        <v>9.3378</v>
       </c>
     </row>
     <row r="6">
@@ -2986,16 +3049,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.3606</v>
+        <v>12.188</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>52272.6931062</v>
+        <v>51542.771676</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>2272.6931062</v>
+        <v>1542.771676000004</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.04545386212400001</v>
+        <v>0.03085543352000008</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -3071,6 +3134,9 @@
       </c>
       <c r="AH6" s="3" t="n">
         <v>12.3606</v>
+      </c>
+      <c r="AI6" s="3" t="n">
+        <v>12.188</v>
       </c>
     </row>
     <row r="7">
@@ -3096,16 +3162,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.6592</v>
+        <v>33.4182</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>74253.541568</v>
+        <v>73721.885928</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>14253.541568</v>
+        <v>13721.885928</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2375590261333334</v>
+        <v>0.2286980988000001</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -3178,6 +3244,9 @@
       </c>
       <c r="AG7" s="3" t="n">
         <v>33.6592</v>
+      </c>
+      <c r="AI7" s="3" t="n">
+        <v>33.4182</v>
       </c>
     </row>
     <row r="8">
@@ -3203,16 +3272,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>32.1815</v>
+        <v>31.782</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>51638.2096295</v>
+        <v>50997.174726</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>1638.209629500001</v>
+        <v>997.1747260000047</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.03276419259000002</v>
+        <v>0.01994349452000009</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -3288,6 +3357,9 @@
       </c>
       <c r="AH8" s="3" t="n">
         <v>32.1815</v>
+      </c>
+      <c r="AI8" s="3" t="n">
+        <v>31.782</v>
       </c>
     </row>
     <row r="9">
@@ -3313,16 +3385,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>41.5956</v>
+        <v>40.9882</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>133912.5834708</v>
+        <v>131957.1241626</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>33912.58347079999</v>
+        <v>31957.1241626</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3391258347079999</v>
+        <v>0.319571241626</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -3395,6 +3467,9 @@
       </c>
       <c r="AG9" s="3" t="n">
         <v>41.5956</v>
+      </c>
+      <c r="AI9" s="3" t="n">
+        <v>40.9882</v>
       </c>
     </row>
     <row r="10">
@@ -3420,16 +3495,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>46.7192</v>
+        <v>46.6879</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>132993.6311528</v>
+        <v>132904.5307261</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>32993.63115279999</v>
+        <v>32904.5307261</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.329936311528</v>
+        <v>0.329045307261</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -3502,6 +3577,9 @@
       </c>
       <c r="AG10" s="3" t="n">
         <v>46.7192</v>
+      </c>
+      <c r="AI10" s="3" t="n">
+        <v>46.6879</v>
       </c>
     </row>
     <row r="11">
@@ -3527,16 +3605,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>102.5771</v>
+        <v>104.1735</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>30867.3983549</v>
+        <v>31347.7854465</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>867.3983549000004</v>
+        <v>1347.785446499998</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.02891327849666668</v>
+        <v>0.04492618154999994</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -3609,6 +3687,9 @@
       </c>
       <c r="AG11" s="3" t="n">
         <v>102.5771</v>
+      </c>
+      <c r="AI11" s="3" t="n">
+        <v>104.1735</v>
       </c>
     </row>
     <row r="12">
@@ -3634,16 +3715,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>220.327</v>
+        <v>218</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>102567.065694</v>
+        <v>101483.796</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>2567.065694000004</v>
+        <v>1483.796000000002</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.02567065694000004</v>
+        <v>0.01483796000000002</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -3719,6 +3800,9 @@
       </c>
       <c r="AH12" s="3" t="n">
         <v>220.327</v>
+      </c>
+      <c r="AI12" s="3" t="n">
+        <v>218</v>
       </c>
     </row>
     <row r="13">
@@ -3744,16 +3828,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>20.141</v>
+        <v>20.154</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>233385.952305</v>
+        <v>233536.59117</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>33385.95230499998</v>
+        <v>33536.59117</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.1669297615249999</v>
+        <v>0.16768295585</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -3829,6 +3913,9 @@
       </c>
       <c r="AH13" s="3" t="n">
         <v>20.141</v>
+      </c>
+      <c r="AI13" s="3" t="n">
+        <v>20.154</v>
       </c>
     </row>
     <row r="14">
@@ -3854,16 +3941,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>39.0967</v>
+        <v>37.7374</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>141045.4895002</v>
+        <v>136141.6706644</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>41045.4895002</v>
+        <v>36141.67066440001</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.410454895002</v>
+        <v>0.3614167066440001</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -3936,6 +4023,9 @@
       </c>
       <c r="AG14" s="3" t="n">
         <v>39.0967</v>
+      </c>
+      <c r="AI14" s="3" t="n">
+        <v>37.7374</v>
       </c>
     </row>
     <row r="15">
@@ -3961,16 +4051,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.86</v>
+        <v>11.68</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>115563.21142</v>
+        <v>113809.30096</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>15563.21141999999</v>
+        <v>13809.30095999999</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1556321141999999</v>
+        <v>0.1380930095999999</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -4046,6 +4136,9 @@
       </c>
       <c r="AH15" s="3" t="n">
         <v>11.86</v>
+      </c>
+      <c r="AI15" s="3" t="n">
+        <v>11.68</v>
       </c>
     </row>
     <row r="16">
@@ -4071,16 +4164,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.0484</v>
+        <v>24.483</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>137627.2617152</v>
+        <v>140114.446224</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>37627.2617152</v>
+        <v>40114.44622400001</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.376272617152</v>
+        <v>0.4011444622400002</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -4153,6 +4246,9 @@
       </c>
       <c r="AG16" s="3" t="n">
         <v>24.0484</v>
+      </c>
+      <c r="AI16" s="3" t="n">
+        <v>24.483</v>
       </c>
     </row>
     <row r="17">
@@ -4178,16 +4274,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.5555</v>
+        <v>16.4809</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>54733.42666349999</v>
+        <v>54486.79481129999</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>4733.426663499995</v>
+        <v>4486.794811299987</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.0946685332699999</v>
+        <v>0.08973589622599976</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -4260,6 +4356,9 @@
       </c>
       <c r="AG17" s="3" t="n">
         <v>16.5555</v>
+      </c>
+      <c r="AI17" s="3" t="n">
+        <v>16.4809</v>
       </c>
     </row>
     <row r="18">
@@ -4285,16 +4384,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>44.45</v>
+        <v>44.4</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>83852.0802</v>
+        <v>83757.75839999999</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>3852.080199999997</v>
+        <v>3757.758399999992</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.04815100249999996</v>
+        <v>0.04697197999999989</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -4370,6 +4469,9 @@
       </c>
       <c r="AH18" s="3" t="n">
         <v>44.45</v>
+      </c>
+      <c r="AI18" s="3" t="n">
+        <v>44.4</v>
       </c>
     </row>
     <row r="19">
@@ -4395,16 +4497,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>15.1077</v>
+        <v>14.4479</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>218559.5606982</v>
+        <v>209014.3884914</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>68559.56069819999</v>
+        <v>59014.38849139999</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.4570637379879999</v>
+        <v>0.3934292566093333</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -4477,6 +4579,9 @@
       </c>
       <c r="AG19" s="3" t="n">
         <v>15.1077</v>
+      </c>
+      <c r="AI19" s="3" t="n">
+        <v>14.4479</v>
       </c>
     </row>
     <row r="20">
@@ -4502,16 +4607,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.35</v>
+        <v>9.24</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>245491.75805</v>
+        <v>242603.61972</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-4508.241949999996</v>
+        <v>-7396.380279999983</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.01803296779999998</v>
+        <v>-0.02958552111999993</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -4587,6 +4692,9 @@
       </c>
       <c r="AH20" s="3" t="n">
         <v>9.35</v>
+      </c>
+      <c r="AI20" s="3" t="n">
+        <v>9.24</v>
       </c>
     </row>
     <row r="21">
@@ -4612,16 +4720,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>107.3404</v>
+        <v>106.1369</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>163077.8687636</v>
+        <v>161249.4405571</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-6922.13123639999</v>
+        <v>-8750.559442900005</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.040718419037647</v>
+        <v>-0.05147387907588238</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -4697,6 +4805,9 @@
       </c>
       <c r="AH21" s="3" t="n">
         <v>107.3404</v>
+      </c>
+      <c r="AI21" s="3" t="n">
+        <v>106.1369</v>
       </c>
     </row>
     <row r="22">
@@ -4722,16 +4833,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>44.024</v>
+        <v>42.648</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>67553.06704000001</v>
+        <v>65441.65008000001</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>7553.067040000009</v>
+        <v>5441.650080000007</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1258844506666668</v>
+        <v>0.09069416800000012</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -4804,6 +4915,9 @@
       </c>
       <c r="AG22" s="3" t="n">
         <v>44.024</v>
+      </c>
+      <c r="AI22" s="3" t="n">
+        <v>42.648</v>
       </c>
     </row>
     <row r="23">
@@ -4829,16 +4943,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>61.2721</v>
+        <v>60.3259</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>166443.6376707</v>
+        <v>163873.3165953</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>16443.6376707</v>
+        <v>13873.31659529998</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.109624251138</v>
+        <v>0.09248877730199989</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -4914,6 +5028,9 @@
       </c>
       <c r="AH23" s="3" t="n">
         <v>61.2721</v>
+      </c>
+      <c r="AI23" s="3" t="n">
+        <v>60.3259</v>
       </c>
     </row>
     <row r="24">
@@ -4939,16 +5056,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>28.3825</v>
+        <v>27.9546</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>103124.578145</v>
+        <v>101569.8522756</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>3124.578145000007</v>
+        <v>1569.852275600002</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.03124578145000007</v>
+        <v>0.01569852275600002</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -5021,6 +5138,9 @@
       </c>
       <c r="AG24" s="3" t="n">
         <v>28.3825</v>
+      </c>
+      <c r="AI24" s="3" t="n">
+        <v>27.9546</v>
       </c>
     </row>
     <row r="25">
@@ -5046,16 +5166,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.4082</v>
+        <v>11.1803</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>187341.7413268</v>
+        <v>183599.2418222</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-12658.25867320001</v>
+        <v>-16400.75817779999</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.06329129336600002</v>
+        <v>-0.08200379088899994</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -5131,6 +5251,9 @@
       </c>
       <c r="AH25" s="3" t="n">
         <v>11.4082</v>
+      </c>
+      <c r="AI25" s="3" t="n">
+        <v>11.1803</v>
       </c>
     </row>
     <row r="26">
@@ -5156,16 +5279,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>8.976100000000001</v>
+        <v>8.773099999999999</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>107190.0280115</v>
+        <v>104765.8598665</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>-2809.971988499994</v>
+        <v>-5234.140133500012</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>-0.02554519989545449</v>
+        <v>-0.04758309212272738</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -5241,6 +5364,9 @@
       </c>
       <c r="AH26" s="3" t="n">
         <v>8.976100000000001</v>
+      </c>
+      <c r="AI26" s="3" t="n">
+        <v>8.773099999999999</v>
       </c>
     </row>
     <row r="27">
@@ -5266,16 +5392,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>63.773</v>
+        <v>62.449</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>102729.37478</v>
+        <v>100596.59614</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-7270.625220000002</v>
+        <v>-9403.403860000006</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.06609659290909092</v>
+        <v>-0.0854854896363637</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -5351,6 +5477,9 @@
       </c>
       <c r="AH27" s="3" t="n">
         <v>63.773</v>
+      </c>
+      <c r="AI27" s="3" t="n">
+        <v>62.449</v>
       </c>
     </row>
     <row r="28">
@@ -5376,16 +5505,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>105.1126</v>
+        <v>103.3172</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>347571.3145782</v>
+        <v>341634.5426004</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-32428.68542180001</v>
+        <v>-38365.45739960001</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.08533864584684213</v>
+        <v>-0.1009617299989474</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -5461,6 +5590,9 @@
       </c>
       <c r="AH28" s="3" t="n">
         <v>105.1126</v>
+      </c>
+      <c r="AI28" s="3" t="n">
+        <v>103.3172</v>
       </c>
     </row>
     <row r="29">
@@ -5486,16 +5618,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.8923</v>
+        <v>11.7668</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>114210.1171869</v>
+        <v>113004.8524604</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>14210.1171869</v>
+        <v>13004.8524604</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.142101171869</v>
+        <v>0.130048524604</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -5568,6 +5700,9 @@
       </c>
       <c r="AG29" s="3" t="n">
         <v>11.8923</v>
+      </c>
+      <c r="AI29" s="3" t="n">
+        <v>11.7668</v>
       </c>
     </row>
     <row r="30">
@@ -5593,16 +5728,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>15.5756</v>
+        <v>15.2867</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>115194.9725916</v>
+        <v>113058.3083487</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>15194.9725916</v>
+        <v>13058.3083487</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.151949725916</v>
+        <v>0.130583083487</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -5675,6 +5810,9 @@
       </c>
       <c r="AG30" s="3" t="n">
         <v>15.5756</v>
+      </c>
+      <c r="AI30" s="3" t="n">
+        <v>15.2867</v>
       </c>
     </row>
     <row r="31">
@@ -5700,16 +5838,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>412.3612</v>
+        <v>406.1331</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>109721.068096</v>
+        <v>108063.895248</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>9721.068095999988</v>
+        <v>8063.895248000001</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.09721068095999988</v>
+        <v>0.08063895248000001</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -5785,6 +5923,9 @@
       </c>
       <c r="AH31" s="3" t="n">
         <v>412.3612</v>
+      </c>
+      <c r="AI31" s="3" t="n">
+        <v>406.1331</v>
       </c>
     </row>
     <row r="32">
@@ -5810,16 +5951,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.14</v>
+        <v>10.02</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>214359.1944</v>
+        <v>211822.3992</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>14359.19440000001</v>
+        <v>11822.39919999999</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.07179597200000004</v>
+        <v>0.05911199599999992</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -5895,6 +6036,9 @@
       </c>
       <c r="AH32" s="3" t="n">
         <v>10.14</v>
+      </c>
+      <c r="AI32" s="3" t="n">
+        <v>10.02</v>
       </c>
     </row>
     <row r="33">
@@ -5920,16 +6064,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>17.86</v>
+        <v>17.67</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>64003.81039999999</v>
+        <v>63322.91880000001</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>4003.810399999995</v>
+        <v>3322.918800000007</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.06673017333333325</v>
+        <v>0.05538198000000012</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -6002,6 +6146,9 @@
       </c>
       <c r="AG33" s="3" t="n">
         <v>17.86</v>
+      </c>
+      <c r="AI33" s="3" t="n">
+        <v>17.67</v>
       </c>
     </row>
     <row r="34">
@@ -6027,16 +6174,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>212.8114</v>
+        <v>210.3821</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>74809.8042534</v>
+        <v>73955.82999510001</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-5190.195746600002</v>
+        <v>-6044.170004899992</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.06487744683250003</v>
+        <v>-0.07555212506124991</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -6112,6 +6259,9 @@
       </c>
       <c r="AH34" s="3" t="n">
         <v>212.8114</v>
+      </c>
+      <c r="AI34" s="3" t="n">
+        <v>210.3821</v>
       </c>
     </row>
     <row r="35">
@@ -6137,16 +6287,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>14.58</v>
+        <v>14.23</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>104034.46734</v>
+        <v>101537.06929</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>4034.467340000003</v>
+        <v>1537.069289999999</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.04034467340000003</v>
+        <v>0.01537069289999999</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -6222,6 +6372,9 @@
       </c>
       <c r="AH35" s="3" t="n">
         <v>14.58</v>
+      </c>
+      <c r="AI35" s="3" t="n">
+        <v>14.23</v>
       </c>
     </row>
     <row r="36">
@@ -6247,16 +6400,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>349.8142</v>
+        <v>350.0769</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>162910.5718252</v>
+        <v>163032.9127914</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>12910.57182520002</v>
+        <v>13032.91279140001</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.08607047883466681</v>
+        <v>0.08688608527600009</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -6332,6 +6485,9 @@
       </c>
       <c r="AH36" s="3" t="n">
         <v>349.8142</v>
+      </c>
+      <c r="AI36" s="3" t="n">
+        <v>350.0769</v>
       </c>
     </row>
     <row r="37">
@@ -6357,16 +6513,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>15.752</v>
+        <v>15.736</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>59273.02752800001</v>
+        <v>59212.821304</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>9273.027528000006</v>
+        <v>9212.821304000005</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.1854605505600001</v>
+        <v>0.1842564260800001</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -6442,6 +6598,9 @@
       </c>
       <c r="AH37" s="3" t="n">
         <v>15.752</v>
+      </c>
+      <c r="AI37" s="3" t="n">
+        <v>15.736</v>
       </c>
     </row>
     <row r="38">
@@ -6467,16 +6626,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.9096</v>
+        <v>13.7262</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>83186.1124272</v>
+        <v>82089.2920284</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>3186.112427200002</v>
+        <v>2089.292028399999</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.03982640534000002</v>
+        <v>0.02611615035499999</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -6549,6 +6708,9 @@
       </c>
       <c r="AG38" s="3" t="n">
         <v>13.9096</v>
+      </c>
+      <c r="AI38" s="3" t="n">
+        <v>13.7262</v>
       </c>
     </row>
     <row r="39">
@@ -6574,16 +6736,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1014.0349</v>
+        <v>1015.2599</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50581.0748469</v>
+        <v>50642.1790719</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>581.0748469000027</v>
+        <v>642.1790718999982</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.01162149693800005</v>
+        <v>0.01284358143799996</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -6656,6 +6818,9 @@
       </c>
       <c r="AG39" s="3" t="n">
         <v>1014.0349</v>
+      </c>
+      <c r="AI39" s="3" t="n">
+        <v>1015.2599</v>
       </c>
     </row>
     <row r="40">
@@ -6681,16 +6846,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>20.3998</v>
+        <v>20.059</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>102835.9425946</v>
+        <v>101117.960593</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>2835.942594599997</v>
+        <v>1117.960593000011</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.02835942594599997</v>
+        <v>0.01117960593000011</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -6766,6 +6931,9 @@
       </c>
       <c r="AH40" s="3" t="n">
         <v>20.3998</v>
+      </c>
+      <c r="AI40" s="3" t="n">
+        <v>20.059</v>
       </c>
     </row>
     <row r="41">
@@ -6778,13 +6946,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4847032.155924</v>
+        <v>4785519.4604006</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>377032.155924</v>
+        <v>315519.4604006</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.08434723846174495</v>
+        <v>0.07058600903816555</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-06-10
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -484,7 +484,7 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-09 06:07 IST</t>
+          <t>Generated: 2026-06-10 06:22 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4785519.4604006</v>
+        <v>4832524.9434292</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>315519.4604006</v>
+        <v>362524.9434292</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.07058600903816555</v>
+        <v>0.08110177705351231</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>555158.5032348633</v>
+        <v>555180.4983215332</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-35623.51676513674</v>
+        <v>-35601.52167846682</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.06029891831362223</v>
+        <v>-0.06026168785310496</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5340677.963635463</v>
+        <v>5387705.441750733</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>279895.9436354637</v>
+        <v>326923.4217507336</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.05530685623868537</v>
+        <v>0.06459938809036744</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-06-09</t>
+          <t>Last snapshot: 2026-06-10</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH19"/>
+  <dimension ref="A1:AI19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -653,6 +653,7 @@
     <col width="21" customWidth="1" min="32" max="32"/>
     <col width="21" customWidth="1" min="33" max="33"/>
     <col width="21" customWidth="1" min="34" max="34"/>
+    <col width="21" customWidth="1" min="35" max="35"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -826,6 +827,11 @@
           <t>2026-06-09</t>
         </is>
       </c>
+      <c r="AI1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -845,13 +851,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>574.1500244140625</v>
+        <v>570.2000122070312</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>45932.001953125</v>
+        <v>45616.0009765625</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>2114.491953124998</v>
+        <v>1798.490976562498</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -933,6 +939,9 @@
       </c>
       <c r="AH2" s="3" t="n">
         <v>574.1500244140625</v>
+      </c>
+      <c r="AI2" s="3" t="n">
+        <v>570.2000122070312</v>
       </c>
     </row>
     <row r="3">
@@ -980,13 +989,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1520.400024414062</v>
+        <v>1527.599975585938</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>30408.00048828125</v>
+        <v>30551.99951171875</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-1696.579511718752</v>
+        <v>-1552.580488281252</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1068,6 +1077,9 @@
       </c>
       <c r="AH4" s="3" t="n">
         <v>1520.400024414062</v>
+      </c>
+      <c r="AI4" s="3" t="n">
+        <v>1527.599975585938</v>
       </c>
     </row>
     <row r="5">
@@ -1088,13 +1100,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>652.3499755859375</v>
+        <v>670</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13046.99951171875</v>
+        <v>13400</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1166.10048828125</v>
+        <v>-813.1000000000004</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1176,6 +1188,9 @@
       </c>
       <c r="AH5" s="3" t="n">
         <v>652.3499755859375</v>
+      </c>
+      <c r="AI5" s="3" t="n">
+        <v>670</v>
       </c>
     </row>
     <row r="6">
@@ -1196,13 +1211,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>380.8999938964844</v>
+        <v>378.5499877929688</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15235.99975585938</v>
+        <v>15141.99951171875</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2266.240244140627</v>
+        <v>-2360.240488281252</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1284,6 +1299,9 @@
       </c>
       <c r="AH6" s="3" t="n">
         <v>380.8999938964844</v>
+      </c>
+      <c r="AI6" s="3" t="n">
+        <v>378.5499877929688</v>
       </c>
     </row>
     <row r="7">
@@ -1304,13 +1322,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>237.2700042724609</v>
+        <v>234.9199981689453</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>23727.00042724609</v>
+        <v>23491.99981689453</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-2706.819572753906</v>
+        <v>-2941.820183105468</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1392,6 +1410,9 @@
       </c>
       <c r="AH7" s="3" t="n">
         <v>237.2700042724609</v>
+      </c>
+      <c r="AI7" s="3" t="n">
+        <v>234.9199981689453</v>
       </c>
     </row>
     <row r="8">
@@ -1439,13 +1460,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>18.48999977111816</v>
+        <v>18.39999961853027</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>27734.99965667725</v>
+        <v>27599.99942779541</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-3315.170343322752</v>
+        <v>-3450.170572204588</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1527,6 +1548,9 @@
       </c>
       <c r="AH9" s="3" t="n">
         <v>18.48999977111816</v>
+      </c>
+      <c r="AI9" s="3" t="n">
+        <v>18.39999961853027</v>
       </c>
     </row>
     <row r="10">
@@ -1547,13 +1571,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>475.7000122070312</v>
+        <v>460.7999877929688</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>47570.00122070312</v>
+        <v>46079.99877929688</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-3928.478779296878</v>
+        <v>-5418.481220703128</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1635,6 +1659,9 @@
       </c>
       <c r="AH10" s="3" t="n">
         <v>475.7000122070312</v>
+      </c>
+      <c r="AI10" s="3" t="n">
+        <v>460.7999877929688</v>
       </c>
     </row>
     <row r="11">
@@ -1655,13 +1682,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>8.890000343322754</v>
+        <v>8.699999809265137</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>8890.000343322754</v>
+        <v>8699.999809265137</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-951.2096566772452</v>
+        <v>-1141.210190734862</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -1743,6 +1770,9 @@
       </c>
       <c r="AH11" s="3" t="n">
         <v>8.890000343322754</v>
+      </c>
+      <c r="AI11" s="3" t="n">
+        <v>8.699999809265137</v>
       </c>
     </row>
     <row r="12">
@@ -1763,13 +1793,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2557.800048828125</v>
+        <v>2551.5</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25578.00048828125</v>
+        <v>25515</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2145.24951171875</v>
+        <v>-2208.25</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -1851,6 +1881,9 @@
       </c>
       <c r="AH12" s="3" t="n">
         <v>2557.800048828125</v>
+      </c>
+      <c r="AI12" s="3" t="n">
+        <v>2551.5</v>
       </c>
     </row>
     <row r="13">
@@ -1871,13 +1904,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>54.75</v>
+        <v>54.77999877929688</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>32850</v>
+        <v>32867.99926757812</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-2181.760000000002</v>
+        <v>-2163.760732421877</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -1959,6 +1992,9 @@
       </c>
       <c r="AH13" s="3" t="n">
         <v>54.75</v>
+      </c>
+      <c r="AI13" s="3" t="n">
+        <v>54.77999877929688</v>
       </c>
     </row>
     <row r="14">
@@ -1979,13 +2015,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>714.0999755859375</v>
+        <v>734.1500244140625</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>35704.99877929688</v>
+        <v>36707.50122070312</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-6757.511220703127</v>
+        <v>-5755.008779296877</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -2067,6 +2103,9 @@
       </c>
       <c r="AH14" s="3" t="n">
         <v>714.0999755859375</v>
+      </c>
+      <c r="AI14" s="3" t="n">
+        <v>734.1500244140625</v>
       </c>
     </row>
     <row r="15">
@@ -2141,13 +2180,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>534.4000244140625</v>
+        <v>555.1500244140625</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>26720.00122070312</v>
+        <v>27757.50122070312</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>4965.471220703126</v>
+        <v>6002.971220703126</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -2229,6 +2268,9 @@
       </c>
       <c r="AH17" s="3" t="n">
         <v>534.4000244140625</v>
+      </c>
+      <c r="AI17" s="3" t="n">
+        <v>555.1500244140625</v>
       </c>
     </row>
     <row r="18">
@@ -2249,13 +2291,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>399.8999938964844</v>
+        <v>399.7999877929688</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>39989.99938964844</v>
+        <v>39979.99877929688</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-6650.820610351562</v>
+        <v>-6660.821220703125</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -2337,6 +2379,9 @@
       </c>
       <c r="AH18" s="3" t="n">
         <v>399.8999938964844</v>
+      </c>
+      <c r="AI18" s="3" t="n">
+        <v>399.7999877929688</v>
       </c>
     </row>
     <row r="19">
@@ -2349,10 +2394,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>555158.5032348633</v>
+        <v>555180.4983215332</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-35623.51676513673</v>
+        <v>-35601.52167846681</v>
       </c>
     </row>
   </sheetData>
@@ -2366,7 +2411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI41"/>
+  <dimension ref="A1:AJ41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2404,6 +2449,7 @@
     <col width="13" customWidth="1" min="33" max="33"/>
     <col width="13" customWidth="1" min="34" max="34"/>
     <col width="13" customWidth="1" min="35" max="35"/>
+    <col width="13" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2582,6 +2628,11 @@
           <t>2026-06-09</t>
         </is>
       </c>
+      <c r="AJ1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2606,16 +2657,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.2466</v>
+        <v>55.9272</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>63135.7960612</v>
+        <v>62777.2753104</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>13135.7960612</v>
+        <v>12777.2753104</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.2627159212240001</v>
+        <v>0.255545506208</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -2694,6 +2745,9 @@
       </c>
       <c r="AI2" s="3" t="n">
         <v>56.2466</v>
+      </c>
+      <c r="AJ2" s="3" t="n">
+        <v>55.9272</v>
       </c>
     </row>
     <row r="3">
@@ -2719,16 +2773,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.3399</v>
+        <v>25.3352</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>62214.85189870001</v>
+        <v>62203.31239760001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>2214.851898700006</v>
+        <v>2203.312397600006</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.03691419831166677</v>
+        <v>0.03672187329333344</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -2804,6 +2858,9 @@
       </c>
       <c r="AI3" s="3" t="n">
         <v>25.3399</v>
+      </c>
+      <c r="AJ3" s="3" t="n">
+        <v>25.3352</v>
       </c>
     </row>
     <row r="4">
@@ -2829,16 +2886,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.38</v>
+        <v>12.51</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>237771.43134</v>
+        <v>240268.22343</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>57771.43134000001</v>
+        <v>60268.22343000001</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3209523963333334</v>
+        <v>0.3348234635000001</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -2914,6 +2971,9 @@
       </c>
       <c r="AI4" s="3" t="n">
         <v>12.38</v>
+      </c>
+      <c r="AJ4" s="3" t="n">
+        <v>12.51</v>
       </c>
     </row>
     <row r="5">
@@ -2939,16 +2999,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.3378</v>
+        <v>9.392200000000001</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>171386.8029264</v>
+        <v>172385.2653136</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-38613.19707360002</v>
+        <v>-37614.73468639998</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.183872367017143</v>
+        <v>-0.1791177842209523</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -3024,6 +3084,9 @@
       </c>
       <c r="AI5" s="3" t="n">
         <v>9.3378</v>
+      </c>
+      <c r="AJ5" s="3" t="n">
+        <v>9.392200000000001</v>
       </c>
     </row>
     <row r="6">
@@ -3049,16 +3112,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.188</v>
+        <v>12.1792</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>51542.771676</v>
+        <v>51505.5566784</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>1542.771676000004</v>
+        <v>1505.556678399997</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.03085543352000008</v>
+        <v>0.03011113356799993</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -3137,6 +3200,9 @@
       </c>
       <c r="AI6" s="3" t="n">
         <v>12.188</v>
+      </c>
+      <c r="AJ6" s="3" t="n">
+        <v>12.1792</v>
       </c>
     </row>
     <row r="7">
@@ -3162,16 +3228,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.4182</v>
+        <v>33.7602</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>73721.885928</v>
+        <v>74476.351608</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>13721.885928</v>
+        <v>14476.351608</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2286980988000001</v>
+        <v>0.2412725267999999</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -3247,6 +3313,9 @@
       </c>
       <c r="AI7" s="3" t="n">
         <v>33.4182</v>
+      </c>
+      <c r="AJ7" s="3" t="n">
+        <v>33.7602</v>
       </c>
     </row>
     <row r="8">
@@ -3272,16 +3341,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>31.782</v>
+        <v>32.3294</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>50997.174726</v>
+        <v>51875.5289342</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>997.1747260000047</v>
+        <v>1875.528934200003</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.01994349452000009</v>
+        <v>0.03751057868400007</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -3360,6 +3429,9 @@
       </c>
       <c r="AI8" s="3" t="n">
         <v>31.782</v>
+      </c>
+      <c r="AJ8" s="3" t="n">
+        <v>32.3294</v>
       </c>
     </row>
     <row r="9">
@@ -3385,16 +3457,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>40.9882</v>
+        <v>41.8621</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>131957.1241626</v>
+        <v>134770.5517053</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>31957.1241626</v>
+        <v>34770.55170529999</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.319571241626</v>
+        <v>0.347705517053</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -3470,6 +3542,9 @@
       </c>
       <c r="AI9" s="3" t="n">
         <v>40.9882</v>
+      </c>
+      <c r="AJ9" s="3" t="n">
+        <v>41.8621</v>
       </c>
     </row>
     <row r="10">
@@ -3495,16 +3570,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>46.6879</v>
+        <v>46.9218</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>132904.5307261</v>
+        <v>133570.3642662</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>32904.5307261</v>
+        <v>33570.36426619999</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.329045307261</v>
+        <v>0.3357036426619999</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -3580,6 +3655,9 @@
       </c>
       <c r="AI10" s="3" t="n">
         <v>46.6879</v>
+      </c>
+      <c r="AJ10" s="3" t="n">
+        <v>46.9218</v>
       </c>
     </row>
     <row r="11">
@@ -3605,16 +3683,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>104.1735</v>
+        <v>103.2162</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31347.7854465</v>
+        <v>31059.7156878</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1347.785446499998</v>
+        <v>1059.715687799999</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.04492618154999994</v>
+        <v>0.03532385625999996</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -3690,6 +3768,9 @@
       </c>
       <c r="AI11" s="3" t="n">
         <v>104.1735</v>
+      </c>
+      <c r="AJ11" s="3" t="n">
+        <v>103.2162</v>
       </c>
     </row>
     <row r="12">
@@ -3715,16 +3796,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>218</v>
+        <v>220.409</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>101483.796</v>
+        <v>102605.238498</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>1483.796000000002</v>
+        <v>2605.238497999992</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.01483796000000002</v>
+        <v>0.02605238497999992</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -3803,6 +3884,9 @@
       </c>
       <c r="AI12" s="3" t="n">
         <v>218</v>
+      </c>
+      <c r="AJ12" s="3" t="n">
+        <v>220.409</v>
       </c>
     </row>
     <row r="13">
@@ -3828,16 +3912,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>20.154</v>
+        <v>20.274</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>233536.59117</v>
+        <v>234927.10377</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>33536.59117</v>
+        <v>34927.10377000002</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.16768295585</v>
+        <v>0.1746355188500001</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -3916,6 +4000,9 @@
       </c>
       <c r="AI13" s="3" t="n">
         <v>20.154</v>
+      </c>
+      <c r="AJ13" s="3" t="n">
+        <v>20.274</v>
       </c>
     </row>
     <row r="14">
@@ -3941,16 +4028,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>37.7374</v>
+        <v>39.0015</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>136141.6706644</v>
+        <v>140702.045409</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>36141.67066440001</v>
+        <v>40702.04540900001</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.3614167066440001</v>
+        <v>0.4070204540900001</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -4026,6 +4113,9 @@
       </c>
       <c r="AI14" s="3" t="n">
         <v>37.7374</v>
+      </c>
+      <c r="AJ14" s="3" t="n">
+        <v>39.0015</v>
       </c>
     </row>
     <row r="15">
@@ -4051,16 +4141,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.68</v>
+        <v>11.71</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>113809.30096</v>
+        <v>114101.61937</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>13809.30095999999</v>
+        <v>14101.61937000001</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1380930095999999</v>
+        <v>0.1410161937000002</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -4139,6 +4229,9 @@
       </c>
       <c r="AI15" s="3" t="n">
         <v>11.68</v>
+      </c>
+      <c r="AJ15" s="3" t="n">
+        <v>11.71</v>
       </c>
     </row>
     <row r="16">
@@ -4164,16 +4257,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.483</v>
+        <v>24.2126</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>140114.446224</v>
+        <v>138566.9664928</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>40114.44622400001</v>
+        <v>38566.96649279998</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4011444622400002</v>
+        <v>0.3856696649279998</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -4249,6 +4342,9 @@
       </c>
       <c r="AI16" s="3" t="n">
         <v>24.483</v>
+      </c>
+      <c r="AJ16" s="3" t="n">
+        <v>24.2126</v>
       </c>
     </row>
     <row r="17">
@@ -4274,16 +4370,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.4809</v>
+        <v>16.5767</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>54486.79481129999</v>
+        <v>54803.51507189999</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>4486.794811299987</v>
+        <v>4803.515071899994</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.08973589622599976</v>
+        <v>0.09607030143799988</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -4359,6 +4455,9 @@
       </c>
       <c r="AI17" s="3" t="n">
         <v>16.4809</v>
+      </c>
+      <c r="AJ17" s="3" t="n">
+        <v>16.5767</v>
       </c>
     </row>
     <row r="18">
@@ -4384,16 +4483,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>44.4</v>
+        <v>44.69</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>83757.75839999999</v>
+        <v>84304.82483999999</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>3757.758399999992</v>
+        <v>4304.824839999987</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.04697197999999989</v>
+        <v>0.05381031049999983</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -4472,6 +4571,9 @@
       </c>
       <c r="AI18" s="3" t="n">
         <v>44.4</v>
+      </c>
+      <c r="AJ18" s="3" t="n">
+        <v>44.69</v>
       </c>
     </row>
     <row r="19">
@@ -4497,16 +4599,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>14.4479</v>
+        <v>14.5769</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>209014.3884914</v>
+        <v>210880.6013054</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>59014.38849139999</v>
+        <v>60880.60130539999</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.3934292566093333</v>
+        <v>0.4058706753693333</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -4582,6 +4684,9 @@
       </c>
       <c r="AI19" s="3" t="n">
         <v>14.4479</v>
+      </c>
+      <c r="AJ19" s="3" t="n">
+        <v>14.5769</v>
       </c>
     </row>
     <row r="20">
@@ -4607,16 +4712,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.24</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>242603.61972</v>
+        <v>243916.40987</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-7396.380279999983</v>
+        <v>-6083.590130000026</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.02958552111999993</v>
+        <v>-0.0243343605200001</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -4695,6 +4800,9 @@
       </c>
       <c r="AI20" s="3" t="n">
         <v>9.24</v>
+      </c>
+      <c r="AJ20" s="3" t="n">
+        <v>9.289999999999999</v>
       </c>
     </row>
     <row r="21">
@@ -4720,16 +4828,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>106.1369</v>
+        <v>107.5499</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>161249.4405571</v>
+        <v>163396.1535241</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-8750.559442900005</v>
+        <v>-6603.846475900005</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.05147387907588238</v>
+        <v>-0.03884615574058826</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -4808,6 +4916,9 @@
       </c>
       <c r="AI21" s="3" t="n">
         <v>106.1369</v>
+      </c>
+      <c r="AJ21" s="3" t="n">
+        <v>107.5499</v>
       </c>
     </row>
     <row r="22">
@@ -4833,16 +4944,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>42.648</v>
+        <v>44.113</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>65441.65008000001</v>
+        <v>67689.63398</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>5441.650080000007</v>
+        <v>7689.633979999999</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.09069416800000012</v>
+        <v>0.1281605663333333</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -4918,6 +5029,9 @@
       </c>
       <c r="AI22" s="3" t="n">
         <v>42.648</v>
+      </c>
+      <c r="AJ22" s="3" t="n">
+        <v>44.113</v>
       </c>
     </row>
     <row r="23">
@@ -4943,16 +5057,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>60.3259</v>
+        <v>60.9661</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>163873.3165953</v>
+        <v>165612.3987687</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>13873.31659529998</v>
+        <v>15612.39876869999</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.09248877730199989</v>
+        <v>0.1040826584579999</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -5031,6 +5145,9 @@
       </c>
       <c r="AI23" s="3" t="n">
         <v>60.3259</v>
+      </c>
+      <c r="AJ23" s="3" t="n">
+        <v>60.9661</v>
       </c>
     </row>
     <row r="24">
@@ -5056,16 +5173,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>27.9546</v>
+        <v>28.377</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>101569.8522756</v>
+        <v>103104.594522</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>1569.852275600002</v>
+        <v>3104.594521999999</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.01569852275600002</v>
+        <v>0.03104594522</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -5141,6 +5258,9 @@
       </c>
       <c r="AI24" s="3" t="n">
         <v>27.9546</v>
+      </c>
+      <c r="AJ24" s="3" t="n">
+        <v>28.377</v>
       </c>
     </row>
     <row r="25">
@@ -5166,16 +5286,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.1803</v>
+        <v>11.2752</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>183599.2418222</v>
+        <v>185157.6586848</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-16400.75817779999</v>
+        <v>-14842.3413152</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.08200379088899994</v>
+        <v>-0.074211706576</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -5254,6 +5374,9 @@
       </c>
       <c r="AI25" s="3" t="n">
         <v>11.1803</v>
+      </c>
+      <c r="AJ25" s="3" t="n">
+        <v>11.2752</v>
       </c>
     </row>
     <row r="26">
@@ -5279,16 +5402,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>8.773099999999999</v>
+        <v>8.8413</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>104765.8598665</v>
+        <v>105580.2848295</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>-5234.140133500012</v>
+        <v>-4419.7151705</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>-0.04758309212272738</v>
+        <v>-0.04017922882272727</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -5367,6 +5490,9 @@
       </c>
       <c r="AI26" s="3" t="n">
         <v>8.773099999999999</v>
+      </c>
+      <c r="AJ26" s="3" t="n">
+        <v>8.8413</v>
       </c>
     </row>
     <row r="27">
@@ -5392,16 +5518,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>62.449</v>
+        <v>63.1459</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>100596.59614</v>
+        <v>101719.204474</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-9403.403860000006</v>
+        <v>-8280.795526000016</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.0854854896363637</v>
+        <v>-0.07527995932727287</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -5480,6 +5606,9 @@
       </c>
       <c r="AI27" s="3" t="n">
         <v>62.449</v>
+      </c>
+      <c r="AJ27" s="3" t="n">
+        <v>63.1459</v>
       </c>
     </row>
     <row r="28">
@@ -5505,16 +5634,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>103.3172</v>
+        <v>104.4346</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>341634.5426004</v>
+        <v>345329.4011322</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-38365.45739960001</v>
+        <v>-34670.59886779997</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.1009617299989474</v>
+        <v>-0.09123841807315781</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -5593,6 +5722,9 @@
       </c>
       <c r="AI28" s="3" t="n">
         <v>103.3172</v>
+      </c>
+      <c r="AJ28" s="3" t="n">
+        <v>104.4346</v>
       </c>
     </row>
     <row r="29">
@@ -5618,16 +5750,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.7668</v>
+        <v>11.9675</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>113004.8524604</v>
+        <v>114932.3156525</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>13004.8524604</v>
+        <v>14932.31565249999</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.130048524604</v>
+        <v>0.1493231565249999</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -5703,6 +5835,9 @@
       </c>
       <c r="AI29" s="3" t="n">
         <v>11.7668</v>
+      </c>
+      <c r="AJ29" s="3" t="n">
+        <v>11.9675</v>
       </c>
     </row>
     <row r="30">
@@ -5728,16 +5863,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>15.2867</v>
+        <v>15.4905</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>113058.3083487</v>
+        <v>114565.5848205</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>13058.3083487</v>
+        <v>14565.58482050001</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.130583083487</v>
+        <v>0.1456558482050001</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -5813,6 +5948,9 @@
       </c>
       <c r="AI30" s="3" t="n">
         <v>15.2867</v>
+      </c>
+      <c r="AJ30" s="3" t="n">
+        <v>15.4905</v>
       </c>
     </row>
     <row r="31">
@@ -5838,16 +5976,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>406.1331</v>
+        <v>408.9721</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>108063.895248</v>
+        <v>108819.296368</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>8063.895248000001</v>
+        <v>8819.296367999996</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.08063895248000001</v>
+        <v>0.08819296367999996</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -5926,6 +6064,9 @@
       </c>
       <c r="AI31" s="3" t="n">
         <v>406.1331</v>
+      </c>
+      <c r="AJ31" s="3" t="n">
+        <v>408.9721</v>
       </c>
     </row>
     <row r="32">
@@ -5951,16 +6092,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.02</v>
+        <v>10.12</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>211822.3992</v>
+        <v>213936.3952</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>11822.39919999999</v>
+        <v>13936.39519999997</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.05911199599999992</v>
+        <v>0.06968197599999985</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -6039,6 +6180,9 @@
       </c>
       <c r="AI32" s="3" t="n">
         <v>10.02</v>
+      </c>
+      <c r="AJ32" s="3" t="n">
+        <v>10.12</v>
       </c>
     </row>
     <row r="33">
@@ -6064,16 +6208,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>17.67</v>
+        <v>17.91</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>63322.91880000001</v>
+        <v>64182.9924</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>3322.918800000007</v>
+        <v>4182.992399999996</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.05538198000000012</v>
+        <v>0.06971653999999992</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -6149,6 +6293,9 @@
       </c>
       <c r="AI33" s="3" t="n">
         <v>17.67</v>
+      </c>
+      <c r="AJ33" s="3" t="n">
+        <v>17.91</v>
       </c>
     </row>
     <row r="34">
@@ -6174,16 +6321,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>210.3821</v>
+        <v>209.9767</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>73955.82999510001</v>
+        <v>73813.3193277</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-6044.170004899992</v>
+        <v>-6186.680672300005</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.07555212506124991</v>
+        <v>-0.07733350840375006</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -6262,6 +6409,9 @@
       </c>
       <c r="AI34" s="3" t="n">
         <v>210.3821</v>
+      </c>
+      <c r="AJ34" s="3" t="n">
+        <v>209.9767</v>
       </c>
     </row>
     <row r="35">
@@ -6287,16 +6437,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>14.23</v>
+        <v>14.47</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>101537.06929</v>
+        <v>103249.57081</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>1537.069289999999</v>
+        <v>3249.570810000005</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.01537069289999999</v>
+        <v>0.03249570810000005</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -6375,6 +6525,9 @@
       </c>
       <c r="AI35" s="3" t="n">
         <v>14.23</v>
+      </c>
+      <c r="AJ35" s="3" t="n">
+        <v>14.47</v>
       </c>
     </row>
     <row r="36">
@@ -6400,16 +6553,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>350.0769</v>
+        <v>354.0663</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>163032.9127914</v>
+        <v>164890.8003078</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>13032.91279140001</v>
+        <v>14890.8003078</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.08688608527600009</v>
+        <v>0.09927200205200003</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -6488,6 +6641,9 @@
       </c>
       <c r="AI36" s="3" t="n">
         <v>350.0769</v>
+      </c>
+      <c r="AJ36" s="3" t="n">
+        <v>354.0663</v>
       </c>
     </row>
     <row r="37">
@@ -6513,16 +6669,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>15.736</v>
+        <v>15.878</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>59212.821304</v>
+        <v>59747.151542</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>9212.821304000005</v>
+        <v>9747.151542</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.1842564260800001</v>
+        <v>0.19494303084</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -6601,6 +6757,9 @@
       </c>
       <c r="AI37" s="3" t="n">
         <v>15.736</v>
+      </c>
+      <c r="AJ37" s="3" t="n">
+        <v>15.878</v>
       </c>
     </row>
     <row r="38">
@@ -6626,16 +6785,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.7262</v>
+        <v>13.8652</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>82089.2920284</v>
+        <v>82920.5790264</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>2089.292028399999</v>
+        <v>2920.579026399995</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.02611615035499999</v>
+        <v>0.03650723782999994</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -6711,6 +6870,9 @@
       </c>
       <c r="AI38" s="3" t="n">
         <v>13.7262</v>
+      </c>
+      <c r="AJ38" s="3" t="n">
+        <v>13.8652</v>
       </c>
     </row>
     <row r="39">
@@ -6736,16 +6898,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1015.2599</v>
+        <v>1016.0649</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50642.1790719</v>
+        <v>50682.3332769</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>642.1790718999982</v>
+        <v>682.3332768999971</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.01284358143799996</v>
+        <v>0.01364666553799994</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -6821,6 +6983,9 @@
       </c>
       <c r="AI39" s="3" t="n">
         <v>1015.2599</v>
+      </c>
+      <c r="AJ39" s="3" t="n">
+        <v>1016.0649</v>
       </c>
     </row>
     <row r="40">
@@ -6846,16 +7011,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>20.059</v>
+        <v>20.5305</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>101117.960593</v>
+        <v>103494.8048235</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>1117.960593000011</v>
+        <v>3494.804823500002</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.01117960593000011</v>
+        <v>0.03494804823500002</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -6934,6 +7099,9 @@
       </c>
       <c r="AI40" s="3" t="n">
         <v>20.059</v>
+      </c>
+      <c r="AJ40" s="3" t="n">
+        <v>20.5305</v>
       </c>
     </row>
     <row r="41">
@@ -6946,13 +7114,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4785519.4604006</v>
+        <v>4832524.9434292</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>315519.4604006</v>
+        <v>362524.9434291999</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.07058600903816555</v>
+        <v>0.08110177705351229</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-06-11
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -484,7 +484,7 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-10 06:22 IST</t>
+          <t>Generated: 2026-06-11 06:47 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4832524.9434292</v>
+        <v>4756600.8030446</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>362524.9434292</v>
+        <v>286600.8030446004</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.08110177705351231</v>
+        <v>0.06411651074823276</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>555180.4983215332</v>
+        <v>547766.0032348633</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-35601.52167846682</v>
+        <v>-43016.01676513674</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.06026168785310496</v>
+        <v>-0.07281199377925675</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5387705.441750733</v>
+        <v>5304366.806279464</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>326923.4217507336</v>
+        <v>243584.7862794641</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.06459938809036744</v>
+        <v>0.04813184707755189</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-06-10</t>
+          <t>Last snapshot: 2026-06-11</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI19"/>
+  <dimension ref="A1:AJ19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -654,6 +654,7 @@
     <col width="21" customWidth="1" min="33" max="33"/>
     <col width="21" customWidth="1" min="34" max="34"/>
     <col width="21" customWidth="1" min="35" max="35"/>
+    <col width="21" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -832,6 +833,11 @@
           <t>2026-06-10</t>
         </is>
       </c>
+      <c r="AJ1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -851,13 +857,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>570.2000122070312</v>
+        <v>557.9000244140625</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>45616.0009765625</v>
+        <v>44632.001953125</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1798.490976562498</v>
+        <v>814.491953124998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -942,6 +948,9 @@
       </c>
       <c r="AI2" s="3" t="n">
         <v>570.2000122070312</v>
+      </c>
+      <c r="AJ2" s="3" t="n">
+        <v>557.9000244140625</v>
       </c>
     </row>
     <row r="3">
@@ -989,13 +998,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1527.599975585938</v>
+        <v>1497.199951171875</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>30551.99951171875</v>
+        <v>29943.9990234375</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-1552.580488281252</v>
+        <v>-2160.580976562502</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1080,6 +1089,9 @@
       </c>
       <c r="AI4" s="3" t="n">
         <v>1527.599975585938</v>
+      </c>
+      <c r="AJ4" s="3" t="n">
+        <v>1497.199951171875</v>
       </c>
     </row>
     <row r="5">
@@ -1100,13 +1112,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>670</v>
+        <v>672.8499755859375</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13400</v>
+        <v>13456.99951171875</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-813.1000000000004</v>
+        <v>-756.1004882812504</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1191,6 +1203,9 @@
       </c>
       <c r="AI5" s="3" t="n">
         <v>670</v>
+      </c>
+      <c r="AJ5" s="3" t="n">
+        <v>672.8499755859375</v>
       </c>
     </row>
     <row r="6">
@@ -1211,13 +1226,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>378.5499877929688</v>
+        <v>372.9500122070312</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15141.99951171875</v>
+        <v>14918.00048828125</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2360.240488281252</v>
+        <v>-2584.239511718752</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1302,6 +1317,9 @@
       </c>
       <c r="AI6" s="3" t="n">
         <v>378.5499877929688</v>
+      </c>
+      <c r="AJ6" s="3" t="n">
+        <v>372.9500122070312</v>
       </c>
     </row>
     <row r="7">
@@ -1322,13 +1340,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>234.9199981689453</v>
+        <v>227.6999969482422</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>23491.99981689453</v>
+        <v>22769.99969482422</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-2941.820183105468</v>
+        <v>-3663.820305175781</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1413,6 +1431,9 @@
       </c>
       <c r="AI7" s="3" t="n">
         <v>234.9199981689453</v>
+      </c>
+      <c r="AJ7" s="3" t="n">
+        <v>227.6999969482422</v>
       </c>
     </row>
     <row r="8">
@@ -1460,13 +1481,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>18.39999961853027</v>
+        <v>17.82999992370605</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>27599.99942779541</v>
+        <v>26744.99988555908</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-3450.170572204588</v>
+        <v>-4305.170114440916</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1551,6 +1572,9 @@
       </c>
       <c r="AI9" s="3" t="n">
         <v>18.39999961853027</v>
+      </c>
+      <c r="AJ9" s="3" t="n">
+        <v>17.82999992370605</v>
       </c>
     </row>
     <row r="10">
@@ -1571,13 +1595,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>460.7999877929688</v>
+        <v>432.4500122070312</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>46079.99877929688</v>
+        <v>43245.00122070312</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-5418.481220703128</v>
+        <v>-8253.478779296878</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1662,6 +1686,9 @@
       </c>
       <c r="AI10" s="3" t="n">
         <v>460.7999877929688</v>
+      </c>
+      <c r="AJ10" s="3" t="n">
+        <v>432.4500122070312</v>
       </c>
     </row>
     <row r="11">
@@ -1682,13 +1709,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>8.699999809265137</v>
+        <v>8.630000114440918</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>8699.999809265137</v>
+        <v>8630.000114440918</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-1141.210190734862</v>
+        <v>-1211.209885559081</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -1773,6 +1800,9 @@
       </c>
       <c r="AI11" s="3" t="n">
         <v>8.699999809265137</v>
+      </c>
+      <c r="AJ11" s="3" t="n">
+        <v>8.630000114440918</v>
       </c>
     </row>
     <row r="12">
@@ -1793,13 +1823,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2551.5</v>
+        <v>2505</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25515</v>
+        <v>25050</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2208.25</v>
+        <v>-2673.25</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -1884,6 +1914,9 @@
       </c>
       <c r="AI12" s="3" t="n">
         <v>2551.5</v>
+      </c>
+      <c r="AJ12" s="3" t="n">
+        <v>2505</v>
       </c>
     </row>
     <row r="13">
@@ -1904,13 +1937,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>54.77999877929688</v>
+        <v>53.72000122070312</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>32867.99926757812</v>
+        <v>32232.00073242188</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-2163.760732421877</v>
+        <v>-2799.759267578127</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -1995,6 +2028,9 @@
       </c>
       <c r="AI13" s="3" t="n">
         <v>54.77999877929688</v>
+      </c>
+      <c r="AJ13" s="3" t="n">
+        <v>53.72000122070312</v>
       </c>
     </row>
     <row r="14">
@@ -2015,13 +2051,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>734.1500244140625</v>
+        <v>734.8499755859375</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>36707.50122070312</v>
+        <v>36742.49877929688</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-5755.008779296877</v>
+        <v>-5720.011220703127</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -2106,6 +2142,9 @@
       </c>
       <c r="AI14" s="3" t="n">
         <v>734.1500244140625</v>
+      </c>
+      <c r="AJ14" s="3" t="n">
+        <v>734.8499755859375</v>
       </c>
     </row>
     <row r="15">
@@ -2180,13 +2219,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>555.1500244140625</v>
+        <v>571.7000122070312</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>27757.50122070312</v>
+        <v>28585.00061035156</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>6002.971220703126</v>
+        <v>6830.470610351564</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -2271,6 +2310,9 @@
       </c>
       <c r="AI17" s="3" t="n">
         <v>555.1500244140625</v>
+      </c>
+      <c r="AJ17" s="3" t="n">
+        <v>571.7000122070312</v>
       </c>
     </row>
     <row r="18">
@@ -2291,13 +2333,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>399.7999877929688</v>
+        <v>390.4500122070312</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>39979.99877929688</v>
+        <v>39045.00122070312</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-6660.821220703125</v>
+        <v>-7595.818779296875</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -2382,6 +2424,9 @@
       </c>
       <c r="AI18" s="3" t="n">
         <v>399.7999877929688</v>
+      </c>
+      <c r="AJ18" s="3" t="n">
+        <v>390.4500122070312</v>
       </c>
     </row>
     <row r="19">
@@ -2394,10 +2439,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>555180.4983215332</v>
+        <v>547766.0032348633</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-35601.52167846681</v>
+        <v>-43016.01676513673</v>
       </c>
     </row>
   </sheetData>
@@ -2411,7 +2456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ41"/>
+  <dimension ref="A1:AK41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2450,6 +2495,7 @@
     <col width="13" customWidth="1" min="34" max="34"/>
     <col width="13" customWidth="1" min="35" max="35"/>
     <col width="13" customWidth="1" min="36" max="36"/>
+    <col width="13" customWidth="1" min="37" max="37"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2633,6 +2679,11 @@
           <t>2026-06-10</t>
         </is>
       </c>
+      <c r="AK1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2657,16 +2708,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>55.9272</v>
+        <v>54.9922</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>62777.2753104</v>
+        <v>61727.75464039999</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>12777.2753104</v>
+        <v>11727.75464039999</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.255545506208</v>
+        <v>0.2345550928079999</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -2748,6 +2799,9 @@
       </c>
       <c r="AJ2" s="3" t="n">
         <v>55.9272</v>
+      </c>
+      <c r="AK2" s="3" t="n">
+        <v>54.9922</v>
       </c>
     </row>
     <row r="3">
@@ -2773,16 +2827,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.3352</v>
+        <v>25.0352</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>62203.31239760001</v>
+        <v>61466.74849760001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>2203.312397600006</v>
+        <v>1466.748497600005</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.03672187329333344</v>
+        <v>0.02444580829333342</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -2861,6 +2915,9 @@
       </c>
       <c r="AJ3" s="3" t="n">
         <v>25.3352</v>
+      </c>
+      <c r="AK3" s="3" t="n">
+        <v>25.0352</v>
       </c>
     </row>
     <row r="4">
@@ -2886,16 +2943,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.51</v>
+        <v>12.11</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>240268.22343</v>
+        <v>232585.78623</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>60268.22343000001</v>
+        <v>52585.78623</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3348234635000001</v>
+        <v>0.2921432568333333</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -2974,6 +3031,9 @@
       </c>
       <c r="AJ4" s="3" t="n">
         <v>12.51</v>
+      </c>
+      <c r="AK4" s="3" t="n">
+        <v>12.11</v>
       </c>
     </row>
     <row r="5">
@@ -2999,16 +3059,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.392200000000001</v>
+        <v>9.351699999999999</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>172385.2653136</v>
+        <v>171641.9247496</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-37614.73468639998</v>
+        <v>-38358.07525040003</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1791177842209523</v>
+        <v>-0.1826575011923811</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -3087,6 +3147,9 @@
       </c>
       <c r="AJ5" s="3" t="n">
         <v>9.392200000000001</v>
+      </c>
+      <c r="AK5" s="3" t="n">
+        <v>9.351699999999999</v>
       </c>
     </row>
     <row r="6">
@@ -3112,16 +3175,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.1792</v>
+        <v>11.9712</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>51505.5566784</v>
+        <v>50625.9294624</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>1505.556678399997</v>
+        <v>625.9294623999958</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.03011113356799993</v>
+        <v>0.01251858924799992</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -3203,6 +3266,9 @@
       </c>
       <c r="AJ6" s="3" t="n">
         <v>12.1792</v>
+      </c>
+      <c r="AK6" s="3" t="n">
+        <v>11.9712</v>
       </c>
     </row>
     <row r="7">
@@ -3228,16 +3294,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.7602</v>
+        <v>33.3424</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>74476.351608</v>
+        <v>73554.66809599999</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>14476.351608</v>
+        <v>13554.66809599999</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2412725267999999</v>
+        <v>0.2259111349333332</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -3316,6 +3382,9 @@
       </c>
       <c r="AJ7" s="3" t="n">
         <v>33.7602</v>
+      </c>
+      <c r="AK7" s="3" t="n">
+        <v>33.3424</v>
       </c>
     </row>
     <row r="8">
@@ -3341,16 +3410,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>32.3294</v>
+        <v>31.9529</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>51875.5289342</v>
+        <v>51271.3996697</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>1875.528934200003</v>
+        <v>1271.399669700004</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.03751057868400007</v>
+        <v>0.02542799339400008</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -3432,6 +3501,9 @@
       </c>
       <c r="AJ8" s="3" t="n">
         <v>32.3294</v>
+      </c>
+      <c r="AK8" s="3" t="n">
+        <v>31.9529</v>
       </c>
     </row>
     <row r="9">
@@ -3457,16 +3529,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>41.8621</v>
+        <v>40.7137</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>134770.5517053</v>
+        <v>131073.4007841</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>34770.55170529999</v>
+        <v>31073.4007841</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.347705517053</v>
+        <v>0.310734007841</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -3545,6 +3617,9 @@
       </c>
       <c r="AJ9" s="3" t="n">
         <v>41.8621</v>
+      </c>
+      <c r="AK9" s="3" t="n">
+        <v>40.7137</v>
       </c>
     </row>
     <row r="10">
@@ -3570,16 +3645,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>46.9218</v>
+        <v>46.6173</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>133570.3642662</v>
+        <v>132703.5566007</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>33570.36426619999</v>
+        <v>32703.55660070002</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3357036426619999</v>
+        <v>0.3270355660070002</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -3658,6 +3733,9 @@
       </c>
       <c r="AJ10" s="3" t="n">
         <v>46.9218</v>
+      </c>
+      <c r="AK10" s="3" t="n">
+        <v>46.6173</v>
       </c>
     </row>
     <row r="11">
@@ -3683,16 +3761,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>103.2162</v>
+        <v>101.1045</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31059.7156878</v>
+        <v>30424.2650355</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1059.715687799999</v>
+        <v>424.2650355000005</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.03532385625999996</v>
+        <v>0.01414216785000002</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -3771,6 +3849,9 @@
       </c>
       <c r="AJ11" s="3" t="n">
         <v>103.2162</v>
+      </c>
+      <c r="AK11" s="3" t="n">
+        <v>101.1045</v>
       </c>
     </row>
     <row r="12">
@@ -3796,16 +3877,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>220.409</v>
+        <v>218.508</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>102605.238498</v>
+        <v>101720.281176</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>2605.238497999992</v>
+        <v>1720.281176000004</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.02605238497999992</v>
+        <v>0.01720281176000004</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -3887,6 +3968,9 @@
       </c>
       <c r="AJ12" s="3" t="n">
         <v>220.409</v>
+      </c>
+      <c r="AK12" s="3" t="n">
+        <v>218.508</v>
       </c>
     </row>
     <row r="13">
@@ -3912,16 +3996,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>20.274</v>
+        <v>20.14</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>234927.10377</v>
+        <v>233374.3647</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>34927.10377000002</v>
+        <v>33374.36470000001</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.1746355188500001</v>
+        <v>0.1668718235</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -4003,6 +4087,9 @@
       </c>
       <c r="AJ13" s="3" t="n">
         <v>20.274</v>
+      </c>
+      <c r="AK13" s="3" t="n">
+        <v>20.14</v>
       </c>
     </row>
     <row r="14">
@@ -4028,16 +4115,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>39.0015</v>
+        <v>37.6845</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>140702.045409</v>
+        <v>135950.828307</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>40702.04540900001</v>
+        <v>35950.82830700002</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.4070204540900001</v>
+        <v>0.3595082830700002</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -4116,6 +4203,9 @@
       </c>
       <c r="AJ14" s="3" t="n">
         <v>39.0015</v>
+      </c>
+      <c r="AK14" s="3" t="n">
+        <v>37.6845</v>
       </c>
     </row>
     <row r="15">
@@ -4141,16 +4231,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.71</v>
+        <v>11.52</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>114101.61937</v>
+        <v>112250.26944</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>14101.61937000001</v>
+        <v>12250.26944</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1410161937000002</v>
+        <v>0.1225026944</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -4232,6 +4322,9 @@
       </c>
       <c r="AJ15" s="3" t="n">
         <v>11.71</v>
+      </c>
+      <c r="AK15" s="3" t="n">
+        <v>11.52</v>
       </c>
     </row>
     <row r="16">
@@ -4257,16 +4350,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.2126</v>
+        <v>23.6211</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>138566.9664928</v>
+        <v>135181.8545808</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>38566.96649279998</v>
+        <v>35181.85458079999</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.3856696649279998</v>
+        <v>0.3518185458079999</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -4345,6 +4438,9 @@
       </c>
       <c r="AJ16" s="3" t="n">
         <v>24.2126</v>
+      </c>
+      <c r="AK16" s="3" t="n">
+        <v>23.6211</v>
       </c>
     </row>
     <row r="17">
@@ -4370,16 +4466,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.5767</v>
+        <v>16.4842</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>54803.51507189999</v>
+        <v>54497.7047994</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>4803.515071899994</v>
+        <v>4497.704799400002</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.09607030143799988</v>
+        <v>0.08995409598800004</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -4458,6 +4554,9 @@
       </c>
       <c r="AJ17" s="3" t="n">
         <v>16.5767</v>
+      </c>
+      <c r="AK17" s="3" t="n">
+        <v>16.4842</v>
       </c>
     </row>
     <row r="18">
@@ -4483,16 +4582,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>44.69</v>
+        <v>44.62</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>84304.82483999999</v>
+        <v>84172.77432</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>4304.824839999987</v>
+        <v>4172.774319999997</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.05381031049999983</v>
+        <v>0.05215967899999996</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -4574,6 +4673,9 @@
       </c>
       <c r="AJ18" s="3" t="n">
         <v>44.69</v>
+      </c>
+      <c r="AK18" s="3" t="n">
+        <v>44.62</v>
       </c>
     </row>
     <row r="19">
@@ -4599,16 +4701,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>14.5769</v>
+        <v>13.9225</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>210880.6013054</v>
+        <v>201413.549635</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>60880.60130539999</v>
+        <v>51413.54963499997</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.4058706753693333</v>
+        <v>0.3427569975666665</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -4687,6 +4789,9 @@
       </c>
       <c r="AJ19" s="3" t="n">
         <v>14.5769</v>
+      </c>
+      <c r="AK19" s="3" t="n">
+        <v>13.9225</v>
       </c>
     </row>
     <row r="20">
@@ -4712,16 +4817,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.289999999999999</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>243916.40987</v>
+        <v>239978.03942</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-6083.590130000026</v>
+        <v>-10021.96057999998</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.0243343605200001</v>
+        <v>-0.04008784231999993</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -4803,6 +4908,9 @@
       </c>
       <c r="AJ20" s="3" t="n">
         <v>9.289999999999999</v>
+      </c>
+      <c r="AK20" s="3" t="n">
+        <v>9.140000000000001</v>
       </c>
     </row>
     <row r="21">
@@ -4828,16 +4936,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>107.5499</v>
+        <v>106.7909</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>163396.1535241</v>
+        <v>162243.0359431</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-6603.846475900005</v>
+        <v>-7756.964056900004</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.03884615574058826</v>
+        <v>-0.0456292003347059</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -4919,6 +5027,9 @@
       </c>
       <c r="AJ21" s="3" t="n">
         <v>107.5499</v>
+      </c>
+      <c r="AK21" s="3" t="n">
+        <v>106.7909</v>
       </c>
     </row>
     <row r="22">
@@ -4944,16 +5055,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>44.113</v>
+        <v>42.419</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>67689.63398</v>
+        <v>65090.25874</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>7689.633979999999</v>
+        <v>5090.258739999997</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1281605663333333</v>
+        <v>0.08483764566666663</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -5032,6 +5143,9 @@
       </c>
       <c r="AJ22" s="3" t="n">
         <v>44.113</v>
+      </c>
+      <c r="AK22" s="3" t="n">
+        <v>42.419</v>
       </c>
     </row>
     <row r="23">
@@ -5057,16 +5171,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>60.9661</v>
+        <v>60.3361</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>165612.3987687</v>
+        <v>163901.0245587</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>15612.39876869999</v>
+        <v>13901.02455870001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.1040826584579999</v>
+        <v>0.09267349705800007</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -5148,6 +5262,9 @@
       </c>
       <c r="AJ23" s="3" t="n">
         <v>60.9661</v>
+      </c>
+      <c r="AK23" s="3" t="n">
+        <v>60.3361</v>
       </c>
     </row>
     <row r="24">
@@ -5173,16 +5290,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>28.377</v>
+        <v>27.8585</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>103104.594522</v>
+        <v>101220.683881</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>3104.594521999999</v>
+        <v>1220.68388099999</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.03104594522</v>
+        <v>0.0122068388099999</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -5261,6 +5378,9 @@
       </c>
       <c r="AJ24" s="3" t="n">
         <v>28.377</v>
+      </c>
+      <c r="AK24" s="3" t="n">
+        <v>27.8585</v>
       </c>
     </row>
     <row r="25">
@@ -5286,16 +5406,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.2752</v>
+        <v>11.0913</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>185157.6586848</v>
+        <v>182137.7128362</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-14842.3413152</v>
+        <v>-17862.28716380001</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.074211706576</v>
+        <v>-0.08931143581900003</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -5377,6 +5497,9 @@
       </c>
       <c r="AJ25" s="3" t="n">
         <v>11.2752</v>
+      </c>
+      <c r="AK25" s="3" t="n">
+        <v>11.0913</v>
       </c>
     </row>
     <row r="26">
@@ -5402,16 +5525,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>8.8413</v>
+        <v>8.7445</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>105580.2848295</v>
+        <v>104424.3268175</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>-4419.7151705</v>
+        <v>-5575.673182499988</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>-0.04017922882272727</v>
+        <v>-0.05068793802272716</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -5493,6 +5616,9 @@
       </c>
       <c r="AJ26" s="3" t="n">
         <v>8.8413</v>
+      </c>
+      <c r="AK26" s="3" t="n">
+        <v>8.7445</v>
       </c>
     </row>
     <row r="27">
@@ -5518,16 +5644,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>63.1459</v>
+        <v>62.095</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>101719.204474</v>
+        <v>100026.3517</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-8280.795526000016</v>
+        <v>-9973.648300000015</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.07527995932727287</v>
+        <v>-0.09066953000000014</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -5609,6 +5735,9 @@
       </c>
       <c r="AJ27" s="3" t="n">
         <v>63.1459</v>
+      </c>
+      <c r="AK27" s="3" t="n">
+        <v>62.095</v>
       </c>
     </row>
     <row r="28">
@@ -5634,16 +5763,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>104.4346</v>
+        <v>102.765</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>345329.4011322</v>
+        <v>339808.606605</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-34670.59886779997</v>
+        <v>-40191.39339499996</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.09123841807315781</v>
+        <v>-0.1057668247236841</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -5725,6 +5854,9 @@
       </c>
       <c r="AJ28" s="3" t="n">
         <v>104.4346</v>
+      </c>
+      <c r="AK28" s="3" t="n">
+        <v>102.765</v>
       </c>
     </row>
     <row r="29">
@@ -5750,16 +5882,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.9675</v>
+        <v>11.7832</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>114932.3156525</v>
+        <v>113162.3531896</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>14932.31565249999</v>
+        <v>13162.35318960001</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.1493231565249999</v>
+        <v>0.1316235318960001</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -5838,6 +5970,9 @@
       </c>
       <c r="AJ29" s="3" t="n">
         <v>11.9675</v>
+      </c>
+      <c r="AK29" s="3" t="n">
+        <v>11.7832</v>
       </c>
     </row>
     <row r="30">
@@ -5863,16 +5998,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>15.4905</v>
+        <v>15.3026</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>114565.5848205</v>
+        <v>113175.9025386</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>14565.58482050001</v>
+        <v>13175.9025386</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.1456558482050001</v>
+        <v>0.131759025386</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -5951,6 +6086,9 @@
       </c>
       <c r="AJ30" s="3" t="n">
         <v>15.4905</v>
+      </c>
+      <c r="AK30" s="3" t="n">
+        <v>15.3026</v>
       </c>
     </row>
     <row r="31">
@@ -5976,16 +6114,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>408.9721</v>
+        <v>403.7669</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>108819.296368</v>
+        <v>107434.296752</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>8819.296367999996</v>
+        <v>7434.296751999995</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.08819296367999996</v>
+        <v>0.07434296751999994</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -6067,6 +6205,9 @@
       </c>
       <c r="AJ31" s="3" t="n">
         <v>408.9721</v>
+      </c>
+      <c r="AK31" s="3" t="n">
+        <v>403.7669</v>
       </c>
     </row>
     <row r="32">
@@ -6092,16 +6233,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.12</v>
+        <v>10.06</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>213936.3952</v>
+        <v>212667.9976</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>13936.39519999997</v>
+        <v>12667.9976</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.06968197599999985</v>
+        <v>0.06333998800000001</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -6183,6 +6324,9 @@
       </c>
       <c r="AJ32" s="3" t="n">
         <v>10.12</v>
+      </c>
+      <c r="AK32" s="3" t="n">
+        <v>10.06</v>
       </c>
     </row>
     <row r="33">
@@ -6208,16 +6352,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>17.91</v>
+        <v>17.79</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>64182.9924</v>
+        <v>63752.95559999999</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>4182.992399999996</v>
+        <v>3752.955599999994</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.06971653999999992</v>
+        <v>0.0625492599999999</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -6296,6 +6440,9 @@
       </c>
       <c r="AJ33" s="3" t="n">
         <v>17.91</v>
+      </c>
+      <c r="AK33" s="3" t="n">
+        <v>17.79</v>
       </c>
     </row>
     <row r="34">
@@ -6321,16 +6468,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>209.9767</v>
+        <v>207.8411</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>73813.3193277</v>
+        <v>73062.58972410001</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-6186.680672300005</v>
+        <v>-6937.410275899994</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.07733350840375006</v>
+        <v>-0.08671762844874993</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -6412,6 +6559,9 @@
       </c>
       <c r="AJ34" s="3" t="n">
         <v>209.9767</v>
+      </c>
+      <c r="AK34" s="3" t="n">
+        <v>207.8411</v>
       </c>
     </row>
     <row r="35">
@@ -6437,16 +6587,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>14.47</v>
+        <v>14.17</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>103249.57081</v>
+        <v>101108.94391</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>3249.570810000005</v>
+        <v>1108.943910000002</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.03249570810000005</v>
+        <v>0.01108943910000002</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -6528,6 +6678,9 @@
       </c>
       <c r="AJ35" s="3" t="n">
         <v>14.47</v>
+      </c>
+      <c r="AK35" s="3" t="n">
+        <v>14.17</v>
       </c>
     </row>
     <row r="36">
@@ -6553,16 +6706,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>354.0663</v>
+        <v>352.564</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>164890.8003078</v>
+        <v>164191.170184</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>14890.8003078</v>
+        <v>14191.17018400002</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.09927200205200003</v>
+        <v>0.09460780122666677</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -6644,6 +6797,9 @@
       </c>
       <c r="AJ36" s="3" t="n">
         <v>354.0663</v>
+      </c>
+      <c r="AK36" s="3" t="n">
+        <v>352.564</v>
       </c>
     </row>
     <row r="37">
@@ -6669,16 +6825,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>15.878</v>
+        <v>15.769</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>59747.151542</v>
+        <v>59336.99664100001</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>9747.151542</v>
+        <v>9336.996641000005</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.19494303084</v>
+        <v>0.1867399328200001</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -6760,6 +6916,9 @@
       </c>
       <c r="AJ37" s="3" t="n">
         <v>15.878</v>
+      </c>
+      <c r="AK37" s="3" t="n">
+        <v>15.769</v>
       </c>
     </row>
     <row r="38">
@@ -6785,16 +6944,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.8652</v>
+        <v>13.7496</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>82920.5790264</v>
+        <v>82229.2353072</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>2920.579026399995</v>
+        <v>2229.235307199997</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.03650723782999994</v>
+        <v>0.02786544133999996</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -6873,6 +7032,9 @@
       </c>
       <c r="AJ38" s="3" t="n">
         <v>13.8652</v>
+      </c>
+      <c r="AK38" s="3" t="n">
+        <v>13.7496</v>
       </c>
     </row>
     <row r="39">
@@ -6898,16 +7060,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1016.0649</v>
+        <v>1015.1705</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50682.3332769</v>
+        <v>50637.71971049999</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>682.3332768999971</v>
+        <v>637.7197104999941</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.01364666553799994</v>
+        <v>0.01275439420999988</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -6986,6 +7148,9 @@
       </c>
       <c r="AJ39" s="3" t="n">
         <v>1016.0649</v>
+      </c>
+      <c r="AK39" s="3" t="n">
+        <v>1015.1705</v>
       </c>
     </row>
     <row r="40">
@@ -7011,16 +7176,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>20.5305</v>
+        <v>20.1097</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>103494.8048235</v>
+        <v>101373.5406619</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>3494.804823500002</v>
+        <v>1373.540661899999</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.03494804823500002</v>
+        <v>0.01373540661899999</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -7102,6 +7267,9 @@
       </c>
       <c r="AJ40" s="3" t="n">
         <v>20.5305</v>
+      </c>
+      <c r="AK40" s="3" t="n">
+        <v>20.1097</v>
       </c>
     </row>
     <row r="41">
@@ -7114,13 +7282,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4832524.9434292</v>
+        <v>4756600.8030446</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>362524.9434291999</v>
+        <v>286600.8030446</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.08110177705351229</v>
+        <v>0.06411651074823266</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-06-12
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-11 06:47 IST</t>
+          <t>Generated: 2026-06-12 06:39 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4756600.8030446</v>
+        <v>4740492.4473511</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>286600.8030446004</v>
+        <v>270492.4473510999</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.06411651074823276</v>
+        <v>0.06051285175639819</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>547766.0032348633</v>
+        <v>549562.0021514893</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-43016.01676513674</v>
+        <v>-41220.01784851076</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.07281199377925675</v>
+        <v>-0.06977195725846694</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5304366.806279464</v>
+        <v>5290054.449502589</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>243584.7862794641</v>
+        <v>229272.4295025896</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.04813184707755189</v>
+        <v>0.04530375515019508</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-06-11</t>
+          <t>Last snapshot: 2026-06-12</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ19"/>
+  <dimension ref="A1:AK19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -655,6 +655,7 @@
     <col width="21" customWidth="1" min="34" max="34"/>
     <col width="21" customWidth="1" min="35" max="35"/>
     <col width="21" customWidth="1" min="36" max="36"/>
+    <col width="21" customWidth="1" min="37" max="37"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -838,6 +839,11 @@
           <t>2026-06-11</t>
         </is>
       </c>
+      <c r="AK1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -857,13 +863,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>557.9000244140625</v>
+        <v>548.7999877929688</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>44632.001953125</v>
+        <v>43903.9990234375</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>814.491953124998</v>
+        <v>86.48902343749796</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -951,6 +957,9 @@
       </c>
       <c r="AJ2" s="3" t="n">
         <v>557.9000244140625</v>
+      </c>
+      <c r="AK2" s="3" t="n">
+        <v>548.7999877929688</v>
       </c>
     </row>
     <row r="3">
@@ -998,13 +1007,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1497.199951171875</v>
+        <v>1522.800048828125</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>29943.9990234375</v>
+        <v>30456.0009765625</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-2160.580976562502</v>
+        <v>-1648.579023437502</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1092,6 +1101,9 @@
       </c>
       <c r="AJ4" s="3" t="n">
         <v>1497.199951171875</v>
+      </c>
+      <c r="AK4" s="3" t="n">
+        <v>1522.800048828125</v>
       </c>
     </row>
     <row r="5">
@@ -1112,13 +1124,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>672.8499755859375</v>
+        <v>676.3499755859375</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13456.99951171875</v>
+        <v>13526.99951171875</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-756.1004882812504</v>
+        <v>-686.1004882812504</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1206,6 +1218,9 @@
       </c>
       <c r="AJ5" s="3" t="n">
         <v>672.8499755859375</v>
+      </c>
+      <c r="AK5" s="3" t="n">
+        <v>676.3499755859375</v>
       </c>
     </row>
     <row r="6">
@@ -1226,13 +1241,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>372.9500122070312</v>
+        <v>372.3500061035156</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>14918.00048828125</v>
+        <v>14894.00024414062</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2584.239511718752</v>
+        <v>-2608.239755859377</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1320,6 +1335,9 @@
       </c>
       <c r="AJ6" s="3" t="n">
         <v>372.9500122070312</v>
+      </c>
+      <c r="AK6" s="3" t="n">
+        <v>372.3500061035156</v>
       </c>
     </row>
     <row r="7">
@@ -1340,13 +1358,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>227.6999969482422</v>
+        <v>226.7100067138672</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>22769.99969482422</v>
+        <v>22671.00067138672</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-3663.820305175781</v>
+        <v>-3762.819328613281</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1434,6 +1452,9 @@
       </c>
       <c r="AJ7" s="3" t="n">
         <v>227.6999969482422</v>
+      </c>
+      <c r="AK7" s="3" t="n">
+        <v>226.7100067138672</v>
       </c>
     </row>
     <row r="8">
@@ -1481,13 +1502,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>17.82999992370605</v>
+        <v>18.14999961853027</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>26744.99988555908</v>
+        <v>27224.99942779541</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-4305.170114440916</v>
+        <v>-3825.170572204588</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1575,6 +1596,9 @@
       </c>
       <c r="AJ9" s="3" t="n">
         <v>17.82999992370605</v>
+      </c>
+      <c r="AK9" s="3" t="n">
+        <v>18.14999961853027</v>
       </c>
     </row>
     <row r="10">
@@ -1595,13 +1619,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>432.4500122070312</v>
+        <v>419</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>43245.00122070312</v>
+        <v>41900</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-8253.478779296878</v>
+        <v>-9598.480000000003</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1689,6 +1713,9 @@
       </c>
       <c r="AJ10" s="3" t="n">
         <v>432.4500122070312</v>
+      </c>
+      <c r="AK10" s="3" t="n">
+        <v>419</v>
       </c>
     </row>
     <row r="11">
@@ -1709,13 +1736,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>8.630000114440918</v>
+        <v>8.800000190734863</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>8630.000114440918</v>
+        <v>8800.000190734863</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-1211.209885559081</v>
+        <v>-1041.209809265136</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -1803,6 +1830,9 @@
       </c>
       <c r="AJ11" s="3" t="n">
         <v>8.630000114440918</v>
+      </c>
+      <c r="AK11" s="3" t="n">
+        <v>8.800000190734863</v>
       </c>
     </row>
     <row r="12">
@@ -1823,13 +1853,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2505</v>
+        <v>2550.89990234375</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25050</v>
+        <v>25508.9990234375</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2673.25</v>
+        <v>-2214.2509765625</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -1917,6 +1947,9 @@
       </c>
       <c r="AJ12" s="3" t="n">
         <v>2505</v>
+      </c>
+      <c r="AK12" s="3" t="n">
+        <v>2550.89990234375</v>
       </c>
     </row>
     <row r="13">
@@ -1937,13 +1970,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>53.72000122070312</v>
+        <v>54.63000106811523</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>32232.00073242188</v>
+        <v>32778.00064086914</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-2799.759267578127</v>
+        <v>-2253.759359130861</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -2031,6 +2064,9 @@
       </c>
       <c r="AJ13" s="3" t="n">
         <v>53.72000122070312</v>
+      </c>
+      <c r="AK13" s="3" t="n">
+        <v>54.63000106811523</v>
       </c>
     </row>
     <row r="14">
@@ -2051,13 +2087,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>734.8499755859375</v>
+        <v>747.75</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>36742.49877929688</v>
+        <v>37387.5</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-5720.011220703127</v>
+        <v>-5075.010000000002</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -2145,6 +2181,9 @@
       </c>
       <c r="AJ14" s="3" t="n">
         <v>734.8499755859375</v>
+      </c>
+      <c r="AK14" s="3" t="n">
+        <v>747.75</v>
       </c>
     </row>
     <row r="15">
@@ -2219,13 +2258,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>571.7000122070312</v>
+        <v>594.4000244140625</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>28585.00061035156</v>
+        <v>29720.00122070312</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>6830.470610351564</v>
+        <v>7965.471220703126</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -2313,6 +2352,9 @@
       </c>
       <c r="AJ17" s="3" t="n">
         <v>571.7000122070312</v>
+      </c>
+      <c r="AK17" s="3" t="n">
+        <v>594.4000244140625</v>
       </c>
     </row>
     <row r="18">
@@ -2333,13 +2375,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>390.4500122070312</v>
+        <v>390.2000122070312</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>39045.00122070312</v>
+        <v>39020.00122070312</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-7595.818779296875</v>
+        <v>-7620.818779296875</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -2427,6 +2469,9 @@
       </c>
       <c r="AJ18" s="3" t="n">
         <v>390.4500122070312</v>
+      </c>
+      <c r="AK18" s="3" t="n">
+        <v>390.2000122070312</v>
       </c>
     </row>
     <row r="19">
@@ -2439,10 +2484,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>547766.0032348633</v>
+        <v>549562.0021514893</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-43016.01676513673</v>
+        <v>-41220.01784851075</v>
       </c>
     </row>
   </sheetData>
@@ -2456,7 +2501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK41"/>
+  <dimension ref="A1:AL41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2467,7 +2512,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
@@ -2496,6 +2541,7 @@
     <col width="13" customWidth="1" min="35" max="35"/>
     <col width="13" customWidth="1" min="36" max="36"/>
     <col width="13" customWidth="1" min="37" max="37"/>
+    <col width="13" customWidth="1" min="38" max="38"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2684,6 +2730,11 @@
           <t>2026-06-11</t>
         </is>
       </c>
+      <c r="AL1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2708,16 +2759,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>54.9922</v>
+        <v>56.154</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>61727.75464039999</v>
+        <v>63031.854228</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>11727.75464039999</v>
+        <v>13031.854228</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.2345550928079999</v>
+        <v>0.2606370845600001</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -2802,6 +2853,9 @@
       </c>
       <c r="AK2" s="3" t="n">
         <v>54.9922</v>
+      </c>
+      <c r="AL2" s="3" t="n">
+        <v>56.154</v>
       </c>
     </row>
     <row r="3">
@@ -2827,16 +2881,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.0352</v>
+        <v>25.0891</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>61466.74849760001</v>
+        <v>61599.0844783</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>1466.748497600005</v>
+        <v>1599.084478299999</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.02444580829333342</v>
+        <v>0.02665140797166666</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -2918,6 +2972,9 @@
       </c>
       <c r="AK3" s="3" t="n">
         <v>25.0352</v>
+      </c>
+      <c r="AL3" s="3" t="n">
+        <v>25.0891</v>
       </c>
     </row>
     <row r="4">
@@ -2943,16 +3000,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.11</v>
+        <v>12.12</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>232585.78623</v>
+        <v>232777.84716</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>52585.78623</v>
+        <v>52777.84716</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.2921432568333333</v>
+        <v>0.293210262</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -3034,6 +3091,9 @@
       </c>
       <c r="AK4" s="3" t="n">
         <v>12.11</v>
+      </c>
+      <c r="AL4" s="3" t="n">
+        <v>12.12</v>
       </c>
     </row>
     <row r="5">
@@ -3059,16 +3119,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.351699999999999</v>
+        <v>9.2438</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>171641.9247496</v>
+        <v>169661.5186544</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-38358.07525040003</v>
+        <v>-40338.48134560001</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1826575011923811</v>
+        <v>-0.1920880064076191</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -3150,6 +3210,9 @@
       </c>
       <c r="AK5" s="3" t="n">
         <v>9.351699999999999</v>
+      </c>
+      <c r="AL5" s="3" t="n">
+        <v>9.2438</v>
       </c>
     </row>
     <row r="6">
@@ -3175,16 +3238,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>11.9712</v>
+        <v>11.892</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>50625.9294624</v>
+        <v>50290.994484</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>625.9294623999958</v>
+        <v>290.9944839999953</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.01251858924799992</v>
+        <v>0.005819889679999905</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -3269,6 +3332,9 @@
       </c>
       <c r="AK6" s="3" t="n">
         <v>11.9712</v>
+      </c>
+      <c r="AL6" s="3" t="n">
+        <v>11.892</v>
       </c>
     </row>
     <row r="7">
@@ -3294,16 +3360,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.3424</v>
+        <v>33.675</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>73554.66809599999</v>
+        <v>74288.397</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>13554.66809599999</v>
+        <v>14288.397</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2259111349333332</v>
+        <v>0.23813995</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -3385,6 +3451,9 @@
       </c>
       <c r="AK7" s="3" t="n">
         <v>33.3424</v>
+      </c>
+      <c r="AL7" s="3" t="n">
+        <v>33.675</v>
       </c>
     </row>
     <row r="8">
@@ -3410,16 +3479,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>31.9529</v>
+        <v>31.6957</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>51271.3996697</v>
+        <v>50858.6983501</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>1271.399669700004</v>
+        <v>858.6983500999995</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.02542799339400008</v>
+        <v>0.01717396700199999</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -3504,6 +3573,9 @@
       </c>
       <c r="AK8" s="3" t="n">
         <v>31.9529</v>
+      </c>
+      <c r="AL8" s="3" t="n">
+        <v>31.6957</v>
       </c>
     </row>
     <row r="9">
@@ -3529,16 +3601,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>40.7137</v>
+        <v>40.5965</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>131073.4007841</v>
+        <v>130696.0879245</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>31073.4007841</v>
+        <v>30696.0879245</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.310734007841</v>
+        <v>0.306960879245</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -3620,6 +3692,9 @@
       </c>
       <c r="AK9" s="3" t="n">
         <v>40.7137</v>
+      </c>
+      <c r="AL9" s="3" t="n">
+        <v>40.5965</v>
       </c>
     </row>
     <row r="10">
@@ -3645,16 +3720,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>46.6173</v>
+        <v>46.5793</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>132703.5566007</v>
+        <v>132595.3835587</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>32703.55660070002</v>
+        <v>32595.38355870001</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3270355660070002</v>
+        <v>0.3259538355870001</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -3736,6 +3811,9 @@
       </c>
       <c r="AK10" s="3" t="n">
         <v>46.6173</v>
+      </c>
+      <c r="AL10" s="3" t="n">
+        <v>46.5793</v>
       </c>
     </row>
     <row r="11">
@@ -3761,16 +3839,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>101.1045</v>
+        <v>104.1766</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>30424.2650355</v>
+        <v>31348.71829539999</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>424.2650355000005</v>
+        <v>1348.718295399995</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.01414216785000002</v>
+        <v>0.04495727651333315</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -3852,6 +3930,9 @@
       </c>
       <c r="AK11" s="3" t="n">
         <v>101.1045</v>
+      </c>
+      <c r="AL11" s="3" t="n">
+        <v>104.1766</v>
       </c>
     </row>
     <row r="12">
@@ -3877,16 +3958,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>218.508</v>
+        <v>216.81</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>101720.281176</v>
+        <v>100929.82482</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>1720.281176000004</v>
+        <v>929.8248199999944</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.01720281176000004</v>
+        <v>0.009298248199999944</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -3971,6 +4052,9 @@
       </c>
       <c r="AK12" s="3" t="n">
         <v>218.508</v>
+      </c>
+      <c r="AL12" s="3" t="n">
+        <v>216.81</v>
       </c>
     </row>
     <row r="13">
@@ -3996,16 +4080,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>20.14</v>
+        <v>20.177</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>233374.3647</v>
+        <v>233803.106085</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>33374.36470000001</v>
+        <v>33803.10608499998</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.1668718235</v>
+        <v>0.1690155304249999</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -4090,6 +4174,9 @@
       </c>
       <c r="AK13" s="3" t="n">
         <v>20.14</v>
+      </c>
+      <c r="AL13" s="3" t="n">
+        <v>20.177</v>
       </c>
     </row>
     <row r="14">
@@ -4115,16 +4202,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>37.6845</v>
+        <v>37.6814</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>135950.828307</v>
+        <v>135939.6447284</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>35950.82830700002</v>
+        <v>35939.64472839999</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.3595082830700002</v>
+        <v>0.3593964472839999</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -4206,6 +4293,9 @@
       </c>
       <c r="AK14" s="3" t="n">
         <v>37.6845</v>
+      </c>
+      <c r="AL14" s="3" t="n">
+        <v>37.6814</v>
       </c>
     </row>
     <row r="15">
@@ -4231,16 +4321,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.52</v>
+        <v>11.42</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>112250.26944</v>
+        <v>111275.87474</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>12250.26944</v>
+        <v>11275.87474</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1225026944</v>
+        <v>0.1127587474</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -4325,6 +4415,9 @@
       </c>
       <c r="AK15" s="3" t="n">
         <v>11.52</v>
+      </c>
+      <c r="AL15" s="3" t="n">
+        <v>11.42</v>
       </c>
     </row>
     <row r="16">
@@ -4350,16 +4443,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>23.6211</v>
+        <v>24.5345</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>135181.8545808</v>
+        <v>140409.177016</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>35181.85458079999</v>
+        <v>40409.177016</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.3518185458079999</v>
+        <v>0.40409177016</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -4441,6 +4534,9 @@
       </c>
       <c r="AK16" s="3" t="n">
         <v>23.6211</v>
+      </c>
+      <c r="AL16" s="3" t="n">
+        <v>24.5345</v>
       </c>
     </row>
     <row r="17">
@@ -4466,16 +4562,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.4842</v>
+        <v>16.5823</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>54497.7047994</v>
+        <v>54822.0289911</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>4497.704799400002</v>
+        <v>4822.0289911</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.08995409598800004</v>
+        <v>0.09644057982199999</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -4557,6 +4653,9 @@
       </c>
       <c r="AK17" s="3" t="n">
         <v>16.4842</v>
+      </c>
+      <c r="AL17" s="3" t="n">
+        <v>16.5823</v>
       </c>
     </row>
     <row r="18">
@@ -4582,16 +4681,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>44.62</v>
+        <v>44.7</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>84172.77432</v>
+        <v>84323.68920000001</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>4172.774319999997</v>
+        <v>4323.689200000008</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.05215967899999996</v>
+        <v>0.0540461150000001</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -4676,6 +4775,9 @@
       </c>
       <c r="AK18" s="3" t="n">
         <v>44.62</v>
+      </c>
+      <c r="AL18" s="3" t="n">
+        <v>44.7</v>
       </c>
     </row>
     <row r="19">
@@ -4701,16 +4803,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>13.9225</v>
+        <v>14.0132</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>201413.549635</v>
+        <v>202725.6853112</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>51413.54963499997</v>
+        <v>52725.68531119998</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.3427569975666665</v>
+        <v>0.3515045687413332</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -4792,6 +4894,9 @@
       </c>
       <c r="AK19" s="3" t="n">
         <v>13.9225</v>
+      </c>
+      <c r="AL19" s="3" t="n">
+        <v>14.0132</v>
       </c>
     </row>
     <row r="20">
@@ -4817,16 +4922,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.140000000000001</v>
+        <v>9.06</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>239978.03942</v>
+        <v>237877.57518</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-10021.96057999998</v>
+        <v>-12122.42481999999</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.04008784231999993</v>
+        <v>-0.04848969927999994</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -4911,6 +5016,9 @@
       </c>
       <c r="AK20" s="3" t="n">
         <v>9.140000000000001</v>
+      </c>
+      <c r="AL20" s="3" t="n">
+        <v>9.06</v>
       </c>
     </row>
     <row r="21">
@@ -4936,16 +5044,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>106.7909</v>
+        <v>106.0619</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>162243.0359431</v>
+        <v>161135.4961321</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-7756.964056900004</v>
+        <v>-8864.503867899999</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.0456292003347059</v>
+        <v>-0.05214414039941176</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -5030,6 +5138,9 @@
       </c>
       <c r="AK21" s="3" t="n">
         <v>106.7909</v>
+      </c>
+      <c r="AL21" s="3" t="n">
+        <v>106.0619</v>
       </c>
     </row>
     <row r="22">
@@ -5055,16 +5166,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>42.419</v>
+        <v>42.753</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>65090.25874</v>
+        <v>65602.76838000001</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>5090.258739999997</v>
+        <v>5602.768380000009</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.08483764566666663</v>
+        <v>0.09337947300000014</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -5146,6 +5257,9 @@
       </c>
       <c r="AK22" s="3" t="n">
         <v>42.419</v>
+      </c>
+      <c r="AL22" s="3" t="n">
+        <v>42.753</v>
       </c>
     </row>
     <row r="23">
@@ -5171,16 +5285,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>60.3361</v>
+        <v>59.9</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>163901.0245587</v>
+        <v>162716.3733</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>13901.02455870001</v>
+        <v>12716.37330000001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.09267349705800007</v>
+        <v>0.08477582200000004</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -5265,6 +5379,9 @@
       </c>
       <c r="AK23" s="3" t="n">
         <v>60.3361</v>
+      </c>
+      <c r="AL23" s="3" t="n">
+        <v>59.9</v>
       </c>
     </row>
     <row r="24">
@@ -5290,16 +5407,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>27.8585</v>
+        <v>27.5108</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>101220.683881</v>
-      </c>
-      <c r="H24" s="4" t="n">
-        <v>1220.68388099999</v>
-      </c>
-      <c r="I24" s="12" t="n">
-        <v>0.0122068388099999</v>
+        <v>99957.35556880001</v>
+      </c>
+      <c r="H24" s="6" t="n">
+        <v>-42.64443119999487</v>
+      </c>
+      <c r="I24" s="13" t="n">
+        <v>-0.0004264443119999487</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -5381,6 +5498,9 @@
       </c>
       <c r="AK24" s="3" t="n">
         <v>27.8585</v>
+      </c>
+      <c r="AL24" s="3" t="n">
+        <v>27.5108</v>
       </c>
     </row>
     <row r="25">
@@ -5406,16 +5526,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.0913</v>
+        <v>10.9758</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>182137.7128362</v>
+        <v>180241.0094892</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-17862.28716380001</v>
+        <v>-19758.99051080001</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.08931143581900003</v>
+        <v>-0.09879495255400005</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -5500,6 +5620,9 @@
       </c>
       <c r="AK25" s="3" t="n">
         <v>11.0913</v>
+      </c>
+      <c r="AL25" s="3" t="n">
+        <v>10.9758</v>
       </c>
     </row>
     <row r="26">
@@ -5525,16 +5648,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>8.7445</v>
+        <v>8.6305</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>104424.3268175</v>
+        <v>103062.9713075</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>-5575.673182499988</v>
+        <v>-6937.028692499996</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>-0.05068793802272716</v>
+        <v>-0.06306389720454542</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -5619,6 +5742,9 @@
       </c>
       <c r="AK26" s="3" t="n">
         <v>8.7445</v>
+      </c>
+      <c r="AL26" s="3" t="n">
+        <v>8.6305</v>
       </c>
     </row>
     <row r="27">
@@ -5644,16 +5770,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>62.095</v>
+        <v>61.3422</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>100026.3517</v>
+        <v>98813.69629199999</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-9973.648300000015</v>
+        <v>-11186.30370800001</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.09066953000000014</v>
+        <v>-0.1016936700727273</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -5738,6 +5864,9 @@
       </c>
       <c r="AK27" s="3" t="n">
         <v>62.095</v>
+      </c>
+      <c r="AL27" s="3" t="n">
+        <v>61.3422</v>
       </c>
     </row>
     <row r="28">
@@ -5763,16 +5892,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>102.765</v>
+        <v>101.7489</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>339808.606605</v>
+        <v>336448.7124273001</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-40191.39339499996</v>
+        <v>-43551.28757269995</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.1057668247236841</v>
+        <v>-0.1146086515071051</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -5857,6 +5986,9 @@
       </c>
       <c r="AK28" s="3" t="n">
         <v>102.765</v>
+      </c>
+      <c r="AL28" s="3" t="n">
+        <v>101.7489</v>
       </c>
     </row>
     <row r="29">
@@ -5882,16 +6014,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.7832</v>
+        <v>11.5365</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>113162.3531896</v>
+        <v>110793.1196595</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>13162.35318960001</v>
+        <v>10793.11965949999</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.1316235318960001</v>
+        <v>0.1079311965949999</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -5973,6 +6105,9 @@
       </c>
       <c r="AK29" s="3" t="n">
         <v>11.7832</v>
+      </c>
+      <c r="AL29" s="3" t="n">
+        <v>11.5365</v>
       </c>
     </row>
     <row r="30">
@@ -5998,16 +6133,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>15.3026</v>
+        <v>15.1512</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>113175.9025386</v>
+        <v>112056.1691832</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>13175.9025386</v>
+        <v>12056.16918319999</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.131759025386</v>
+        <v>0.1205616918319999</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -6089,6 +6224,9 @@
       </c>
       <c r="AK30" s="3" t="n">
         <v>15.3026</v>
+      </c>
+      <c r="AL30" s="3" t="n">
+        <v>15.1512</v>
       </c>
     </row>
     <row r="31">
@@ -6114,16 +6252,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>403.7669</v>
+        <v>399.005</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>107434.296752</v>
+        <v>106167.2504</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>7434.296751999995</v>
+        <v>6167.25039999999</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.07434296751999994</v>
+        <v>0.0616725039999999</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -6208,6 +6346,9 @@
       </c>
       <c r="AK31" s="3" t="n">
         <v>403.7669</v>
+      </c>
+      <c r="AL31" s="3" t="n">
+        <v>399.005</v>
       </c>
     </row>
     <row r="32">
@@ -6233,16 +6374,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.06</v>
+        <v>10</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>212667.9976</v>
+        <v>211399.6</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>12667.9976</v>
+        <v>11399.59999999998</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.06333998800000001</v>
+        <v>0.05699799999999988</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -6327,6 +6468,9 @@
       </c>
       <c r="AK32" s="3" t="n">
         <v>10.06</v>
+      </c>
+      <c r="AL32" s="3" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="33">
@@ -6352,16 +6496,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>17.79</v>
+        <v>17.69</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>63752.95559999999</v>
+        <v>63394.5916</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>3752.955599999994</v>
+        <v>3394.5916</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.0625492599999999</v>
+        <v>0.05657652666666666</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -6443,6 +6587,9 @@
       </c>
       <c r="AK33" s="3" t="n">
         <v>17.79</v>
+      </c>
+      <c r="AL33" s="3" t="n">
+        <v>17.69</v>
       </c>
     </row>
     <row r="34">
@@ -6468,16 +6615,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>207.8411</v>
+        <v>206.0169</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>73062.58972410001</v>
+        <v>72421.32687390001</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-6937.410275899994</v>
+        <v>-7578.673126099995</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.08671762844874993</v>
+        <v>-0.09473341407624994</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -6562,6 +6709,9 @@
       </c>
       <c r="AK34" s="3" t="n">
         <v>207.8411</v>
+      </c>
+      <c r="AL34" s="3" t="n">
+        <v>206.0169</v>
       </c>
     </row>
     <row r="35">
@@ -6587,16 +6737,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>14.17</v>
+        <v>14</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>101108.94391</v>
-      </c>
-      <c r="H35" s="4" t="n">
-        <v>1108.943910000002</v>
-      </c>
-      <c r="I35" s="12" t="n">
-        <v>0.01108943910000002</v>
+        <v>99895.92199999999</v>
+      </c>
+      <c r="H35" s="6" t="n">
+        <v>-104.0780000000086</v>
+      </c>
+      <c r="I35" s="13" t="n">
+        <v>-0.001040780000000086</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -6681,6 +6831,9 @@
       </c>
       <c r="AK35" s="3" t="n">
         <v>14.17</v>
+      </c>
+      <c r="AL35" s="3" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="36">
@@ -6706,16 +6859,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>352.564</v>
+        <v>353.3227</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>164191.170184</v>
+        <v>164544.5013262</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>14191.17018400002</v>
+        <v>14544.5013262</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.09460780122666677</v>
+        <v>0.09696334217466666</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -6800,6 +6953,9 @@
       </c>
       <c r="AK36" s="3" t="n">
         <v>352.564</v>
+      </c>
+      <c r="AL36" s="3" t="n">
+        <v>353.3227</v>
       </c>
     </row>
     <row r="37">
@@ -6825,16 +6981,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>15.769</v>
+        <v>15.81</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>59336.99664100001</v>
+        <v>59491.27509</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>9336.996641000005</v>
+        <v>9491.275090000003</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.1867399328200001</v>
+        <v>0.1898255018</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -6919,6 +7075,9 @@
       </c>
       <c r="AK37" s="3" t="n">
         <v>15.769</v>
+      </c>
+      <c r="AL37" s="3" t="n">
+        <v>15.81</v>
       </c>
     </row>
     <row r="38">
@@ -6944,16 +7103,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.7496</v>
+        <v>13.6629</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>82229.2353072</v>
+        <v>81710.7275178</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>2229.235307199997</v>
+        <v>1710.727517799998</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.02786544133999996</v>
+        <v>0.02138409397249998</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -7035,6 +7194,9 @@
       </c>
       <c r="AK38" s="3" t="n">
         <v>13.7496</v>
+      </c>
+      <c r="AL38" s="3" t="n">
+        <v>13.6629</v>
       </c>
     </row>
     <row r="39">
@@ -7060,16 +7222,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1015.1705</v>
+        <v>1015.8523</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50637.71971049999</v>
+        <v>50671.7285763</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>637.7197104999941</v>
+        <v>671.7285763000036</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.01275439420999988</v>
+        <v>0.01343457152600007</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -7151,6 +7313,9 @@
       </c>
       <c r="AK39" s="3" t="n">
         <v>1015.1705</v>
+      </c>
+      <c r="AL39" s="3" t="n">
+        <v>1015.8523</v>
       </c>
     </row>
     <row r="40">
@@ -7176,16 +7341,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>20.1097</v>
+        <v>19.9786</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>101373.5406619</v>
+        <v>100712.6620222</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>1373.540661899999</v>
+        <v>712.6620222000056</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.01373540661899999</v>
+        <v>0.007126620222000056</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -7270,6 +7435,9 @@
       </c>
       <c r="AK40" s="3" t="n">
         <v>20.1097</v>
+      </c>
+      <c r="AL40" s="3" t="n">
+        <v>19.9786</v>
       </c>
     </row>
     <row r="41">
@@ -7282,13 +7450,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4756600.8030446</v>
+        <v>4740492.4473511</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>286600.8030446</v>
+        <v>270492.4473511</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.06411651074823266</v>
+        <v>0.06051285175639821</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-06-13
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-12 06:39 IST</t>
+          <t>Generated: 2026-06-13 06:15 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4740492.4473511</v>
+        <v>4822717.2647319</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>270492.4473510999</v>
+        <v>352717.2647318998</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.06051285175639819</v>
+        <v>0.07890766548812077</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>549562.0021514893</v>
+        <v>551575.4942779541</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-41220.01784851076</v>
+        <v>-39206.52572204592</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.06977195725846694</v>
+        <v>-0.0663637761386948</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5290054.449502589</v>
+        <v>5374292.759009854</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>229272.4295025896</v>
+        <v>313510.7390098544</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.04530375515019508</v>
+        <v>0.06194906988107234</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-06-12</t>
+          <t>Last snapshot: 2026-06-13</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK19"/>
+  <dimension ref="A1:AL19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -656,6 +656,7 @@
     <col width="21" customWidth="1" min="35" max="35"/>
     <col width="21" customWidth="1" min="36" max="36"/>
     <col width="21" customWidth="1" min="37" max="37"/>
+    <col width="21" customWidth="1" min="38" max="38"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -844,6 +845,11 @@
           <t>2026-06-12</t>
         </is>
       </c>
+      <c r="AL1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -863,13 +869,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>548.7999877929688</v>
+        <v>548.2999877929688</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>43903.9990234375</v>
+        <v>43863.9990234375</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>86.48902343749796</v>
+        <v>46.48902343749796</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -960,6 +966,9 @@
       </c>
       <c r="AK2" s="3" t="n">
         <v>548.7999877929688</v>
+      </c>
+      <c r="AL2" s="3" t="n">
+        <v>548.2999877929688</v>
       </c>
     </row>
     <row r="3">
@@ -1007,13 +1016,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1522.800048828125</v>
+        <v>1508.599975585938</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>30456.0009765625</v>
+        <v>30171.99951171875</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-1648.579023437502</v>
+        <v>-1932.580488281252</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1104,6 +1113,9 @@
       </c>
       <c r="AK4" s="3" t="n">
         <v>1522.800048828125</v>
+      </c>
+      <c r="AL4" s="3" t="n">
+        <v>1508.599975585938</v>
       </c>
     </row>
     <row r="5">
@@ -1124,13 +1136,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>676.3499755859375</v>
+        <v>673.7999877929688</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13526.99951171875</v>
+        <v>13475.99975585938</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-686.1004882812504</v>
+        <v>-737.1002441406254</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1221,6 +1233,9 @@
       </c>
       <c r="AK5" s="3" t="n">
         <v>676.3499755859375</v>
+      </c>
+      <c r="AL5" s="3" t="n">
+        <v>673.7999877929688</v>
       </c>
     </row>
     <row r="6">
@@ -1241,13 +1256,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>372.3500061035156</v>
+        <v>377.2999877929688</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>14894.00024414062</v>
+        <v>15091.99951171875</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2608.239755859377</v>
+        <v>-2410.240488281252</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1338,6 +1353,9 @@
       </c>
       <c r="AK6" s="3" t="n">
         <v>372.3500061035156</v>
+      </c>
+      <c r="AL6" s="3" t="n">
+        <v>377.2999877929688</v>
       </c>
     </row>
     <row r="7">
@@ -1358,13 +1376,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>226.7100067138672</v>
+        <v>234.6799926757812</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>22671.00067138672</v>
+        <v>23467.99926757812</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-3762.819328613281</v>
+        <v>-2965.820732421875</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1455,6 +1473,9 @@
       </c>
       <c r="AK7" s="3" t="n">
         <v>226.7100067138672</v>
+      </c>
+      <c r="AL7" s="3" t="n">
+        <v>234.6799926757812</v>
       </c>
     </row>
     <row r="8">
@@ -1502,13 +1523,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>18.14999961853027</v>
+        <v>18.38999938964844</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>27224.99942779541</v>
+        <v>27584.99908447266</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-3825.170572204588</v>
+        <v>-3465.170915527342</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1599,6 +1620,9 @@
       </c>
       <c r="AK9" s="3" t="n">
         <v>18.14999961853027</v>
+      </c>
+      <c r="AL9" s="3" t="n">
+        <v>18.38999938964844</v>
       </c>
     </row>
     <row r="10">
@@ -1619,13 +1643,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>419</v>
+        <v>417.7999877929688</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>41900</v>
+        <v>41779.99877929688</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-9598.480000000003</v>
+        <v>-9718.481220703128</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1716,6 +1740,9 @@
       </c>
       <c r="AK10" s="3" t="n">
         <v>419</v>
+      </c>
+      <c r="AL10" s="3" t="n">
+        <v>417.7999877929688</v>
       </c>
     </row>
     <row r="11">
@@ -1736,13 +1763,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>8.800000190734863</v>
+        <v>8.920000076293945</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>8800.000190734863</v>
+        <v>8920.000076293945</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-1041.209809265136</v>
+        <v>-921.2099237060538</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -1833,6 +1860,9 @@
       </c>
       <c r="AK11" s="3" t="n">
         <v>8.800000190734863</v>
+      </c>
+      <c r="AL11" s="3" t="n">
+        <v>8.920000076293945</v>
       </c>
     </row>
     <row r="12">
@@ -1853,13 +1883,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2550.89990234375</v>
+        <v>2580.5</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25508.9990234375</v>
+        <v>25805</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2214.2509765625</v>
+        <v>-1918.25</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -1950,6 +1980,9 @@
       </c>
       <c r="AK12" s="3" t="n">
         <v>2550.89990234375</v>
+      </c>
+      <c r="AL12" s="3" t="n">
+        <v>2580.5</v>
       </c>
     </row>
     <row r="13">
@@ -1970,13 +2003,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>54.63000106811523</v>
+        <v>55.08000183105469</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>32778.00064086914</v>
+        <v>33048.00109863281</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-2253.759359130861</v>
+        <v>-1983.75890136719</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -2067,6 +2100,9 @@
       </c>
       <c r="AK13" s="3" t="n">
         <v>54.63000106811523</v>
+      </c>
+      <c r="AL13" s="3" t="n">
+        <v>55.08000183105469</v>
       </c>
     </row>
     <row r="14">
@@ -2087,13 +2123,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>747.75</v>
+        <v>745.9500122070312</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>37387.5</v>
+        <v>37297.50061035156</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-5075.010000000002</v>
+        <v>-5165.00938964844</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -2184,6 +2220,9 @@
       </c>
       <c r="AK14" s="3" t="n">
         <v>747.75</v>
+      </c>
+      <c r="AL14" s="3" t="n">
+        <v>745.9500122070312</v>
       </c>
     </row>
     <row r="15">
@@ -2258,13 +2297,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>594.4000244140625</v>
+        <v>598.8499755859375</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>29720.00122070312</v>
+        <v>29942.49877929688</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>7965.471220703126</v>
+        <v>8187.968779296876</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -2355,6 +2394,9 @@
       </c>
       <c r="AK17" s="3" t="n">
         <v>594.4000244140625</v>
+      </c>
+      <c r="AL17" s="3" t="n">
+        <v>598.8499755859375</v>
       </c>
     </row>
     <row r="18">
@@ -2375,13 +2417,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>390.2000122070312</v>
+        <v>393.5499877929688</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>39020.00122070312</v>
+        <v>39354.99877929688</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-7620.818779296875</v>
+        <v>-7285.821220703125</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -2472,6 +2514,9 @@
       </c>
       <c r="AK18" s="3" t="n">
         <v>390.2000122070312</v>
+      </c>
+      <c r="AL18" s="3" t="n">
+        <v>393.5499877929688</v>
       </c>
     </row>
     <row r="19">
@@ -2484,10 +2529,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>549562.0021514893</v>
+        <v>551575.4942779541</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-41220.01784851075</v>
+        <v>-39206.52572204591</v>
       </c>
     </row>
   </sheetData>
@@ -2501,7 +2546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL41"/>
+  <dimension ref="A1:AM41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2512,7 +2557,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
@@ -2542,6 +2587,7 @@
     <col width="13" customWidth="1" min="36" max="36"/>
     <col width="13" customWidth="1" min="37" max="37"/>
     <col width="13" customWidth="1" min="38" max="38"/>
+    <col width="13" customWidth="1" min="39" max="39"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2735,6 +2781,11 @@
           <t>2026-06-12</t>
         </is>
       </c>
+      <c r="AM1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2759,16 +2810,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.154</v>
+        <v>56.4319</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>63031.854228</v>
+        <v>63343.7919758</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>13031.854228</v>
+        <v>13343.7919758</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.2606370845600001</v>
+        <v>0.266875839516</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -2856,6 +2907,9 @@
       </c>
       <c r="AL2" s="3" t="n">
         <v>56.154</v>
+      </c>
+      <c r="AM2" s="3" t="n">
+        <v>56.4319</v>
       </c>
     </row>
     <row r="3">
@@ -2976,6 +3030,9 @@
       <c r="AL3" s="3" t="n">
         <v>25.0891</v>
       </c>
+      <c r="AM3" s="3" t="n">
+        <v>25.0891</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3095,6 +3152,9 @@
       <c r="AL4" s="3" t="n">
         <v>12.12</v>
       </c>
+      <c r="AM4" s="3" t="n">
+        <v>12.12</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3119,16 +3179,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.2438</v>
+        <v>9.326700000000001</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>169661.5186544</v>
+        <v>171183.0725496</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-40338.48134560001</v>
+        <v>-38816.92745039999</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1920880064076191</v>
+        <v>-0.1848425116685714</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -3213,6 +3273,9 @@
       </c>
       <c r="AL5" s="3" t="n">
         <v>9.2438</v>
+      </c>
+      <c r="AM5" s="3" t="n">
+        <v>9.326700000000001</v>
       </c>
     </row>
     <row r="6">
@@ -3238,16 +3301,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>11.892</v>
+        <v>12.0487</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>50290.994484</v>
+        <v>50953.6751799</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>290.9944839999953</v>
+        <v>953.6751798999976</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.005819889679999905</v>
+        <v>0.01907350359799995</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -3335,6 +3398,9 @@
       </c>
       <c r="AL6" s="3" t="n">
         <v>11.892</v>
+      </c>
+      <c r="AM6" s="3" t="n">
+        <v>12.0487</v>
       </c>
     </row>
     <row r="7">
@@ -3360,16 +3426,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.675</v>
+        <v>34.0781</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>74288.397</v>
+        <v>75177.651724</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>14288.397</v>
+        <v>15177.651724</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.23813995</v>
+        <v>0.2529608620666666</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -3454,6 +3520,9 @@
       </c>
       <c r="AL7" s="3" t="n">
         <v>33.675</v>
+      </c>
+      <c r="AM7" s="3" t="n">
+        <v>34.0781</v>
       </c>
     </row>
     <row r="8">
@@ -3479,16 +3548,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>31.6957</v>
+        <v>32.2764</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>50858.6983501</v>
+        <v>51790.48550520001</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>858.6983500999995</v>
+        <v>1790.485505200006</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.01717396700199999</v>
+        <v>0.03580971010400012</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -3576,6 +3645,9 @@
       </c>
       <c r="AL8" s="3" t="n">
         <v>31.6957</v>
+      </c>
+      <c r="AM8" s="3" t="n">
+        <v>32.2764</v>
       </c>
     </row>
     <row r="9">
@@ -3601,16 +3673,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>40.5965</v>
+        <v>41.3929</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>130696.0879245</v>
+        <v>133260.0125097</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>30696.0879245</v>
+        <v>33260.0125097</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.306960879245</v>
+        <v>0.332600125097</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -3695,6 +3767,9 @@
       </c>
       <c r="AL9" s="3" t="n">
         <v>40.5965</v>
+      </c>
+      <c r="AM9" s="3" t="n">
+        <v>41.3929</v>
       </c>
     </row>
     <row r="10">
@@ -3720,16 +3795,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>46.5793</v>
+        <v>46.9497</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>132595.3835587</v>
+        <v>133649.7860523</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>32595.38355870001</v>
+        <v>33649.78605230001</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3259538355870001</v>
+        <v>0.3364978605230001</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -3814,6 +3889,9 @@
       </c>
       <c r="AL10" s="3" t="n">
         <v>46.5793</v>
+      </c>
+      <c r="AM10" s="3" t="n">
+        <v>46.9497</v>
       </c>
     </row>
     <row r="11">
@@ -3839,16 +3917,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>104.1766</v>
+        <v>104.0296</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31348.71829539999</v>
+        <v>31304.4832024</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1348.718295399995</v>
+        <v>1304.483202399999</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.04495727651333315</v>
+        <v>0.04348277341333329</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -3933,6 +4011,9 @@
       </c>
       <c r="AL11" s="3" t="n">
         <v>104.1766</v>
+      </c>
+      <c r="AM11" s="3" t="n">
+        <v>104.0296</v>
       </c>
     </row>
     <row r="12">
@@ -3958,16 +4039,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>216.81</v>
+        <v>220.156</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>100929.82482</v>
+        <v>102487.461432</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>929.8248199999944</v>
+        <v>2487.461431999996</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.009298248199999944</v>
+        <v>0.02487461431999996</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -4055,6 +4136,9 @@
       </c>
       <c r="AL12" s="3" t="n">
         <v>216.81</v>
+      </c>
+      <c r="AM12" s="3" t="n">
+        <v>220.156</v>
       </c>
     </row>
     <row r="13">
@@ -4080,16 +4164,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>20.177</v>
+        <v>20.313</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>233803.106085</v>
+        <v>235379.020365</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>33803.10608499998</v>
+        <v>35379.02036499997</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.1690155304249999</v>
+        <v>0.1768951018249999</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -4177,6 +4261,9 @@
       </c>
       <c r="AL13" s="3" t="n">
         <v>20.177</v>
+      </c>
+      <c r="AM13" s="3" t="n">
+        <v>20.313</v>
       </c>
     </row>
     <row r="14">
@@ -4202,16 +4289,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>37.6814</v>
+        <v>38.7849</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>135939.6447284</v>
+        <v>139920.6379494</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>35939.64472839999</v>
+        <v>39920.6379494</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.3593964472839999</v>
+        <v>0.399206379494</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -4296,6 +4383,9 @@
       </c>
       <c r="AL14" s="3" t="n">
         <v>37.6814</v>
+      </c>
+      <c r="AM14" s="3" t="n">
+        <v>38.7849</v>
       </c>
     </row>
     <row r="15">
@@ -4321,16 +4411,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.42</v>
+        <v>11.66</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>111275.87474</v>
+        <v>113614.42202</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>11275.87474</v>
+        <v>13614.42202</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1127587474</v>
+        <v>0.1361442202</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -4418,6 +4508,9 @@
       </c>
       <c r="AL15" s="3" t="n">
         <v>11.42</v>
+      </c>
+      <c r="AM15" s="3" t="n">
+        <v>11.66</v>
       </c>
     </row>
     <row r="16">
@@ -4443,16 +4536,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.5345</v>
+        <v>24.6055</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>140409.177016</v>
+        <v>140815.504904</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>40409.177016</v>
+        <v>40815.504904</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.40409177016</v>
+        <v>0.40815504904</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -4537,6 +4630,9 @@
       </c>
       <c r="AL16" s="3" t="n">
         <v>24.5345</v>
+      </c>
+      <c r="AM16" s="3" t="n">
+        <v>24.6055</v>
       </c>
     </row>
     <row r="17">
@@ -4562,16 +4658,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.5823</v>
+        <v>16.7283</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>54822.0289911</v>
+        <v>55304.7133131</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>4822.0289911</v>
+        <v>5304.713313100001</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.09644057982199999</v>
+        <v>0.106094266262</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -4656,6 +4752,9 @@
       </c>
       <c r="AL17" s="3" t="n">
         <v>16.5823</v>
+      </c>
+      <c r="AM17" s="3" t="n">
+        <v>16.7283</v>
       </c>
     </row>
     <row r="18">
@@ -4681,16 +4780,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>44.7</v>
+        <v>45.09</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>84323.68920000001</v>
+        <v>85059.39924</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>4323.689200000008</v>
+        <v>5059.399239999999</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.0540461150000001</v>
+        <v>0.06324249049999998</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -4778,6 +4877,9 @@
       </c>
       <c r="AL18" s="3" t="n">
         <v>44.7</v>
+      </c>
+      <c r="AM18" s="3" t="n">
+        <v>45.09</v>
       </c>
     </row>
     <row r="19">
@@ -4803,16 +4905,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>14.0132</v>
+        <v>14.3784</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>202725.6853112</v>
+        <v>208008.9482544</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>52725.68531119998</v>
+        <v>58008.94825439999</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.3515045687413332</v>
+        <v>0.386726321696</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -4897,6 +4999,9 @@
       </c>
       <c r="AL19" s="3" t="n">
         <v>14.0132</v>
+      </c>
+      <c r="AM19" s="3" t="n">
+        <v>14.3784</v>
       </c>
     </row>
     <row r="20">
@@ -4922,16 +5027,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.06</v>
+        <v>9.17</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>237877.57518</v>
+        <v>240765.71351</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-12122.42481999999</v>
+        <v>-9234.286489999999</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.04848969927999994</v>
+        <v>-0.03693714595999999</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -5019,6 +5124,9 @@
       </c>
       <c r="AL20" s="3" t="n">
         <v>9.06</v>
+      </c>
+      <c r="AM20" s="3" t="n">
+        <v>9.17</v>
       </c>
     </row>
     <row r="21">
@@ -5044,16 +5152,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>106.0619</v>
+        <v>108.3559</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>161135.4961321</v>
+        <v>164620.6762781</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-8864.503867899999</v>
+        <v>-5379.3237219</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.05214414039941176</v>
+        <v>-0.03164308071705883</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -5141,6 +5249,9 @@
       </c>
       <c r="AL21" s="3" t="n">
         <v>106.0619</v>
+      </c>
+      <c r="AM21" s="3" t="n">
+        <v>108.3559</v>
       </c>
     </row>
     <row r="22">
@@ -5166,16 +5277,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>42.753</v>
+        <v>44.011</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>65602.76838000001</v>
+        <v>67533.11906000001</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>5602.768380000009</v>
+        <v>7533.119060000012</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.09337947300000014</v>
+        <v>0.1255519843333335</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -5260,6 +5371,9 @@
       </c>
       <c r="AL22" s="3" t="n">
         <v>42.753</v>
+      </c>
+      <c r="AM22" s="3" t="n">
+        <v>44.011</v>
       </c>
     </row>
     <row r="23">
@@ -5285,16 +5399,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>59.9</v>
+        <v>61.3411</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>162716.3733</v>
+        <v>166631.0738937</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>12716.37330000001</v>
+        <v>16631.0738937</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.08477582200000004</v>
+        <v>0.110873825958</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -5382,6 +5496,9 @@
       </c>
       <c r="AL23" s="3" t="n">
         <v>59.9</v>
+      </c>
+      <c r="AM23" s="3" t="n">
+        <v>61.3411</v>
       </c>
     </row>
     <row r="24">
@@ -5407,16 +5524,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>27.5108</v>
+        <v>28.1701</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>99957.35556880001</v>
-      </c>
-      <c r="H24" s="6" t="n">
-        <v>-42.64443119999487</v>
-      </c>
-      <c r="I24" s="13" t="n">
-        <v>-0.0004264443119999487</v>
+        <v>102352.8469586</v>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>2352.846958599999</v>
+      </c>
+      <c r="I24" s="12" t="n">
+        <v>0.02352846958599999</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -5501,6 +5618,9 @@
       </c>
       <c r="AL24" s="3" t="n">
         <v>27.5108</v>
+      </c>
+      <c r="AM24" s="3" t="n">
+        <v>28.1701</v>
       </c>
     </row>
     <row r="25">
@@ -5526,16 +5646,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>10.9758</v>
+        <v>11.2619</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>180241.0094892</v>
+        <v>184939.2504206</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-19758.99051080001</v>
+        <v>-15060.7495794</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.09879495255400005</v>
+        <v>-0.07530374789699999</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -5623,6 +5743,9 @@
       </c>
       <c r="AL25" s="3" t="n">
         <v>10.9758</v>
+      </c>
+      <c r="AM25" s="3" t="n">
+        <v>11.2619</v>
       </c>
     </row>
     <row r="26">
@@ -5648,16 +5771,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>8.6305</v>
+        <v>8.8187</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>103062.9713075</v>
+        <v>105310.4020705</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>-6937.028692499996</v>
+        <v>-4689.5979295</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>-0.06306389720454542</v>
+        <v>-0.04263270845</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -5745,6 +5868,9 @@
       </c>
       <c r="AL26" s="3" t="n">
         <v>8.6305</v>
+      </c>
+      <c r="AM26" s="3" t="n">
+        <v>8.8187</v>
       </c>
     </row>
     <row r="27">
@@ -5770,16 +5896,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>61.3422</v>
+        <v>62.6305</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>98813.69629199999</v>
+        <v>100888.96723</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-11186.30370800001</v>
+        <v>-9111.032770000005</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.1016936700727273</v>
+        <v>-0.08282757063636369</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -5867,6 +5993,9 @@
       </c>
       <c r="AL27" s="3" t="n">
         <v>61.3422</v>
+      </c>
+      <c r="AM27" s="3" t="n">
+        <v>62.6305</v>
       </c>
     </row>
     <row r="28">
@@ -5892,16 +6021,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>101.7489</v>
+        <v>104.5676</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>336448.7124273001</v>
+        <v>345769.1865132</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-43551.28757269995</v>
+        <v>-34230.81348680001</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.1146086515071051</v>
+        <v>-0.0900810881231579</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -5989,6 +6118,9 @@
       </c>
       <c r="AL28" s="3" t="n">
         <v>101.7489</v>
+      </c>
+      <c r="AM28" s="3" t="n">
+        <v>104.5676</v>
       </c>
     </row>
     <row r="29">
@@ -6014,16 +6146,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.5365</v>
+        <v>11.79</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>110793.1196595</v>
+        <v>113227.65837</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>10793.11965949999</v>
+        <v>13227.65836999999</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.1079311965949999</v>
+        <v>0.1322765836999999</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -6108,6 +6240,9 @@
       </c>
       <c r="AL29" s="3" t="n">
         <v>11.5365</v>
+      </c>
+      <c r="AM29" s="3" t="n">
+        <v>11.79</v>
       </c>
     </row>
     <row r="30">
@@ -6133,16 +6268,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>15.1512</v>
+        <v>15.5484</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>112056.1691832</v>
+        <v>114993.8051724</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>12056.16918319999</v>
+        <v>14993.80517240001</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.1205616918319999</v>
+        <v>0.1499380517240001</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -6227,6 +6362,9 @@
       </c>
       <c r="AL30" s="3" t="n">
         <v>15.1512</v>
+      </c>
+      <c r="AM30" s="3" t="n">
+        <v>15.5484</v>
       </c>
     </row>
     <row r="31">
@@ -6252,16 +6390,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>399.005</v>
+        <v>409.1495</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>106167.2504</v>
+        <v>108866.49896</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>6167.25039999999</v>
+        <v>8866.498959999997</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.0616725039999999</v>
+        <v>0.08866498959999997</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -6349,6 +6487,9 @@
       </c>
       <c r="AL31" s="3" t="n">
         <v>399.005</v>
+      </c>
+      <c r="AM31" s="3" t="n">
+        <v>409.1495</v>
       </c>
     </row>
     <row r="32">
@@ -6374,16 +6515,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10</v>
+        <v>10.2</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>211399.6</v>
+        <v>215627.592</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>11399.59999999998</v>
+        <v>15627.59199999998</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.05699799999999988</v>
+        <v>0.07813795999999988</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -6471,6 +6612,9 @@
       </c>
       <c r="AL32" s="3" t="n">
         <v>10</v>
+      </c>
+      <c r="AM32" s="3" t="n">
+        <v>10.2</v>
       </c>
     </row>
     <row r="33">
@@ -6496,16 +6640,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>17.69</v>
+        <v>18.13</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>63394.5916</v>
+        <v>64971.39319999999</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>3394.5916</v>
+        <v>4971.393199999991</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.05657652666666666</v>
+        <v>0.08285655333333319</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -6590,6 +6734,9 @@
       </c>
       <c r="AL33" s="3" t="n">
         <v>17.69</v>
+      </c>
+      <c r="AM33" s="3" t="n">
+        <v>18.13</v>
       </c>
     </row>
     <row r="34">
@@ -6615,16 +6762,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>206.0169</v>
+        <v>208.1454</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>72421.32687390001</v>
+        <v>73169.5606074</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-7578.673126099995</v>
+        <v>-6830.439392600005</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.09473341407624994</v>
+        <v>-0.08538049240750006</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -6712,6 +6859,9 @@
       </c>
       <c r="AL34" s="3" t="n">
         <v>206.0169</v>
+      </c>
+      <c r="AM34" s="3" t="n">
+        <v>208.1454</v>
       </c>
     </row>
     <row r="35">
@@ -6737,16 +6887,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>14</v>
+        <v>14.43</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>99895.92199999999</v>
-      </c>
-      <c r="H35" s="6" t="n">
-        <v>-104.0780000000086</v>
-      </c>
-      <c r="I35" s="13" t="n">
-        <v>-0.001040780000000086</v>
+        <v>102964.15389</v>
+      </c>
+      <c r="H35" s="4" t="n">
+        <v>2964.153890000001</v>
+      </c>
+      <c r="I35" s="12" t="n">
+        <v>0.02964153890000001</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -6834,6 +6984,9 @@
       </c>
       <c r="AL35" s="3" t="n">
         <v>14</v>
+      </c>
+      <c r="AM35" s="3" t="n">
+        <v>14.43</v>
       </c>
     </row>
     <row r="36">
@@ -6859,16 +7012,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>353.3227</v>
+        <v>355.9597</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>164544.5013262</v>
+        <v>165772.5680482</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>14544.5013262</v>
+        <v>15772.56804820002</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.09696334217466666</v>
+        <v>0.1051504536546668</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -6956,6 +7109,9 @@
       </c>
       <c r="AL36" s="3" t="n">
         <v>353.3227</v>
+      </c>
+      <c r="AM36" s="3" t="n">
+        <v>355.9597</v>
       </c>
     </row>
     <row r="37">
@@ -6981,16 +7137,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>15.81</v>
+        <v>15.947</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>59491.27509</v>
+        <v>60006.790883</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>9491.275090000003</v>
+        <v>10006.790883</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.1898255018</v>
+        <v>0.20013581766</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -7078,6 +7234,9 @@
       </c>
       <c r="AL37" s="3" t="n">
         <v>15.81</v>
+      </c>
+      <c r="AM37" s="3" t="n">
+        <v>15.947</v>
       </c>
     </row>
     <row r="38">
@@ -7103,16 +7262,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.6629</v>
+        <v>13.9727</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>81710.7275178</v>
+        <v>83563.4808414</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>1710.727517799998</v>
+        <v>3563.4808414</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.02138409397249998</v>
+        <v>0.0445435105175</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -7197,6 +7356,9 @@
       </c>
       <c r="AL38" s="3" t="n">
         <v>13.6629</v>
+      </c>
+      <c r="AM38" s="3" t="n">
+        <v>13.9727</v>
       </c>
     </row>
     <row r="39">
@@ -7222,16 +7384,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1015.8523</v>
+        <v>1016.6971</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50671.7285763</v>
+        <v>50713.8680451</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>671.7285763000036</v>
+        <v>713.8680450999964</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.01343457152600007</v>
+        <v>0.01427736090199993</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -7316,6 +7478,9 @@
       </c>
       <c r="AL39" s="3" t="n">
         <v>1015.8523</v>
+      </c>
+      <c r="AM39" s="3" t="n">
+        <v>1016.6971</v>
       </c>
     </row>
     <row r="40">
@@ -7341,16 +7506,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>19.9786</v>
+        <v>20.7098</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>100712.6620222</v>
+        <v>104398.6609646</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>712.6620222000056</v>
+        <v>4398.660964600014</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.007126620222000056</v>
+        <v>0.04398660964600015</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -7438,6 +7603,9 @@
       </c>
       <c r="AL40" s="3" t="n">
         <v>19.9786</v>
+      </c>
+      <c r="AM40" s="3" t="n">
+        <v>20.7098</v>
       </c>
     </row>
     <row r="41">
@@ -7450,13 +7618,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4740492.4473511</v>
+        <v>4822717.2647319</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>270492.4473511</v>
+        <v>352717.2647319</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.06051285175639821</v>
+        <v>0.0789076654881208</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-06-14
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -485,7 +485,7 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-13 06:15 IST</t>
+          <t>Generated: 2026-06-14 06:38 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4822717.2647319</v>
+        <v>4826546.0174467</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>352717.2647318998</v>
+        <v>356546.0174466996</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.07890766548812077</v>
+        <v>0.07976420971961959</v>
       </c>
     </row>
     <row r="6">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5374292.759009854</v>
+        <v>5378121.511724654</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>313510.7390098544</v>
+        <v>317339.4917246541</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.06194906988107234</v>
+        <v>0.06270562345316232</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-06-13</t>
+          <t>Last snapshot: 2026-06-14</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL19"/>
+  <dimension ref="A1:AM19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -657,6 +657,7 @@
     <col width="21" customWidth="1" min="36" max="36"/>
     <col width="21" customWidth="1" min="37" max="37"/>
     <col width="21" customWidth="1" min="38" max="38"/>
+    <col width="21" customWidth="1" min="39" max="39"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -850,6 +851,11 @@
           <t>2026-06-13</t>
         </is>
       </c>
+      <c r="AM1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -970,6 +976,9 @@
       <c r="AL2" s="3" t="n">
         <v>548.2999877929688</v>
       </c>
+      <c r="AM2" s="3" t="n">
+        <v>548.2999877929688</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1117,6 +1126,9 @@
       <c r="AL4" s="3" t="n">
         <v>1508.599975585938</v>
       </c>
+      <c r="AM4" s="3" t="n">
+        <v>1508.599975585938</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1237,6 +1249,9 @@
       <c r="AL5" s="3" t="n">
         <v>673.7999877929688</v>
       </c>
+      <c r="AM5" s="3" t="n">
+        <v>673.7999877929688</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1357,6 +1372,9 @@
       <c r="AL6" s="3" t="n">
         <v>377.2999877929688</v>
       </c>
+      <c r="AM6" s="3" t="n">
+        <v>377.2999877929688</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1477,6 +1495,9 @@
       <c r="AL7" s="3" t="n">
         <v>234.6799926757812</v>
       </c>
+      <c r="AM7" s="3" t="n">
+        <v>234.6799926757812</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1624,6 +1645,9 @@
       <c r="AL9" s="3" t="n">
         <v>18.38999938964844</v>
       </c>
+      <c r="AM9" s="3" t="n">
+        <v>18.38999938964844</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1744,6 +1768,9 @@
       <c r="AL10" s="3" t="n">
         <v>417.7999877929688</v>
       </c>
+      <c r="AM10" s="3" t="n">
+        <v>417.7999877929688</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1864,6 +1891,9 @@
       <c r="AL11" s="3" t="n">
         <v>8.920000076293945</v>
       </c>
+      <c r="AM11" s="3" t="n">
+        <v>8.920000076293945</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1984,6 +2014,9 @@
       <c r="AL12" s="3" t="n">
         <v>2580.5</v>
       </c>
+      <c r="AM12" s="3" t="n">
+        <v>2580.5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2104,6 +2137,9 @@
       <c r="AL13" s="3" t="n">
         <v>55.08000183105469</v>
       </c>
+      <c r="AM13" s="3" t="n">
+        <v>55.08000183105469</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2224,6 +2260,9 @@
       <c r="AL14" s="3" t="n">
         <v>745.9500122070312</v>
       </c>
+      <c r="AM14" s="3" t="n">
+        <v>745.9500122070312</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2398,6 +2437,9 @@
       <c r="AL17" s="3" t="n">
         <v>598.8499755859375</v>
       </c>
+      <c r="AM17" s="3" t="n">
+        <v>598.8499755859375</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2516,6 +2558,9 @@
         <v>390.2000122070312</v>
       </c>
       <c r="AL18" s="3" t="n">
+        <v>393.5499877929688</v>
+      </c>
+      <c r="AM18" s="3" t="n">
         <v>393.5499877929688</v>
       </c>
     </row>
@@ -2546,7 +2591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM41"/>
+  <dimension ref="A1:AN41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2588,6 +2633,7 @@
     <col width="13" customWidth="1" min="37" max="37"/>
     <col width="13" customWidth="1" min="38" max="38"/>
     <col width="13" customWidth="1" min="39" max="39"/>
+    <col width="13" customWidth="1" min="40" max="40"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2786,6 +2832,11 @@
           <t>2026-06-13</t>
         </is>
       </c>
+      <c r="AN1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2911,6 +2962,9 @@
       <c r="AM2" s="3" t="n">
         <v>56.4319</v>
       </c>
+      <c r="AN2" s="3" t="n">
+        <v>56.4319</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2935,16 +2989,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.0891</v>
+        <v>25.3187</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>61599.0844783</v>
+        <v>62162.80138310001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>1599.084478299999</v>
+        <v>2162.801383100006</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.02665140797166666</v>
+        <v>0.03604668971833343</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -3032,6 +3086,9 @@
       </c>
       <c r="AM3" s="3" t="n">
         <v>25.0891</v>
+      </c>
+      <c r="AN3" s="3" t="n">
+        <v>25.3187</v>
       </c>
     </row>
     <row r="4">
@@ -3057,16 +3114,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.12</v>
+        <v>12.29</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>232777.84716</v>
+        <v>236042.88297</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>52777.84716</v>
+        <v>56042.88297000001</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.293210262</v>
+        <v>0.3113493498333333</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -3154,6 +3211,9 @@
       </c>
       <c r="AM4" s="3" t="n">
         <v>12.12</v>
+      </c>
+      <c r="AN4" s="3" t="n">
+        <v>12.29</v>
       </c>
     </row>
     <row r="5">
@@ -3277,6 +3337,9 @@
       <c r="AM5" s="3" t="n">
         <v>9.326700000000001</v>
       </c>
+      <c r="AN5" s="3" t="n">
+        <v>9.326700000000001</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3402,6 +3465,9 @@
       <c r="AM6" s="3" t="n">
         <v>12.0487</v>
       </c>
+      <c r="AN6" s="3" t="n">
+        <v>12.0487</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3524,6 +3590,9 @@
       <c r="AM7" s="3" t="n">
         <v>34.0781</v>
       </c>
+      <c r="AN7" s="3" t="n">
+        <v>34.0781</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3649,6 +3718,9 @@
       <c r="AM8" s="3" t="n">
         <v>32.2764</v>
       </c>
+      <c r="AN8" s="3" t="n">
+        <v>32.2764</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3771,6 +3843,9 @@
       <c r="AM9" s="3" t="n">
         <v>41.3929</v>
       </c>
+      <c r="AN9" s="3" t="n">
+        <v>41.3929</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3893,6 +3968,9 @@
       <c r="AM10" s="3" t="n">
         <v>46.9497</v>
       </c>
+      <c r="AN10" s="3" t="n">
+        <v>46.9497</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4015,6 +4093,9 @@
       <c r="AM11" s="3" t="n">
         <v>104.0296</v>
       </c>
+      <c r="AN11" s="3" t="n">
+        <v>104.0296</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4140,6 +4221,9 @@
       <c r="AM12" s="3" t="n">
         <v>220.156</v>
       </c>
+      <c r="AN12" s="3" t="n">
+        <v>220.156</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4265,6 +4349,9 @@
       <c r="AM13" s="3" t="n">
         <v>20.313</v>
       </c>
+      <c r="AN13" s="3" t="n">
+        <v>20.313</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4387,6 +4474,9 @@
       <c r="AM14" s="3" t="n">
         <v>38.7849</v>
       </c>
+      <c r="AN14" s="3" t="n">
+        <v>38.7849</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4512,6 +4602,9 @@
       <c r="AM15" s="3" t="n">
         <v>11.66</v>
       </c>
+      <c r="AN15" s="3" t="n">
+        <v>11.66</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4634,6 +4727,9 @@
       <c r="AM16" s="3" t="n">
         <v>24.6055</v>
       </c>
+      <c r="AN16" s="3" t="n">
+        <v>24.6055</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4756,6 +4852,9 @@
       <c r="AM17" s="3" t="n">
         <v>16.7283</v>
       </c>
+      <c r="AN17" s="3" t="n">
+        <v>16.7283</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4881,6 +4980,9 @@
       <c r="AM18" s="3" t="n">
         <v>45.09</v>
       </c>
+      <c r="AN18" s="3" t="n">
+        <v>45.09</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5003,6 +5105,9 @@
       <c r="AM19" s="3" t="n">
         <v>14.3784</v>
       </c>
+      <c r="AN19" s="3" t="n">
+        <v>14.3784</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5128,6 +5233,9 @@
       <c r="AM20" s="3" t="n">
         <v>9.17</v>
       </c>
+      <c r="AN20" s="3" t="n">
+        <v>9.17</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5253,6 +5361,9 @@
       <c r="AM21" s="3" t="n">
         <v>108.3559</v>
       </c>
+      <c r="AN21" s="3" t="n">
+        <v>108.3559</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5375,6 +5486,9 @@
       <c r="AM22" s="3" t="n">
         <v>44.011</v>
       </c>
+      <c r="AN22" s="3" t="n">
+        <v>44.011</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5500,6 +5614,9 @@
       <c r="AM23" s="3" t="n">
         <v>61.3411</v>
       </c>
+      <c r="AN23" s="3" t="n">
+        <v>61.3411</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5622,6 +5739,9 @@
       <c r="AM24" s="3" t="n">
         <v>28.1701</v>
       </c>
+      <c r="AN24" s="3" t="n">
+        <v>28.1701</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5747,6 +5867,9 @@
       <c r="AM25" s="3" t="n">
         <v>11.2619</v>
       </c>
+      <c r="AN25" s="3" t="n">
+        <v>11.2619</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -5872,6 +5995,9 @@
       <c r="AM26" s="3" t="n">
         <v>8.8187</v>
       </c>
+      <c r="AN26" s="3" t="n">
+        <v>8.8187</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5997,6 +6123,9 @@
       <c r="AM27" s="3" t="n">
         <v>62.6305</v>
       </c>
+      <c r="AN27" s="3" t="n">
+        <v>62.6305</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6122,6 +6251,9 @@
       <c r="AM28" s="3" t="n">
         <v>104.5676</v>
       </c>
+      <c r="AN28" s="3" t="n">
+        <v>104.5676</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -6244,6 +6376,9 @@
       <c r="AM29" s="3" t="n">
         <v>11.79</v>
       </c>
+      <c r="AN29" s="3" t="n">
+        <v>11.79</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -6366,6 +6501,9 @@
       <c r="AM30" s="3" t="n">
         <v>15.5484</v>
       </c>
+      <c r="AN30" s="3" t="n">
+        <v>15.5484</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -6491,6 +6629,9 @@
       <c r="AM31" s="3" t="n">
         <v>409.1495</v>
       </c>
+      <c r="AN31" s="3" t="n">
+        <v>409.1495</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -6616,6 +6757,9 @@
       <c r="AM32" s="3" t="n">
         <v>10.2</v>
       </c>
+      <c r="AN32" s="3" t="n">
+        <v>10.2</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -6738,6 +6882,9 @@
       <c r="AM33" s="3" t="n">
         <v>18.13</v>
       </c>
+      <c r="AN33" s="3" t="n">
+        <v>18.13</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -6863,6 +7010,9 @@
       <c r="AM34" s="3" t="n">
         <v>208.1454</v>
       </c>
+      <c r="AN34" s="3" t="n">
+        <v>208.1454</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -6988,6 +7138,9 @@
       <c r="AM35" s="3" t="n">
         <v>14.43</v>
       </c>
+      <c r="AN35" s="3" t="n">
+        <v>14.43</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -7113,6 +7266,9 @@
       <c r="AM36" s="3" t="n">
         <v>355.9597</v>
       </c>
+      <c r="AN36" s="3" t="n">
+        <v>355.9597</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -7238,6 +7394,9 @@
       <c r="AM37" s="3" t="n">
         <v>15.947</v>
       </c>
+      <c r="AN37" s="3" t="n">
+        <v>15.947</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -7360,6 +7519,9 @@
       <c r="AM38" s="3" t="n">
         <v>13.9727</v>
       </c>
+      <c r="AN38" s="3" t="n">
+        <v>13.9727</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -7482,6 +7644,9 @@
       <c r="AM39" s="3" t="n">
         <v>1016.6971</v>
       </c>
+      <c r="AN39" s="3" t="n">
+        <v>1016.6971</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -7607,6 +7772,9 @@
       <c r="AM40" s="3" t="n">
         <v>20.7098</v>
       </c>
+      <c r="AN40" s="3" t="n">
+        <v>20.7098</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
@@ -7618,13 +7786,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4822717.2647319</v>
+        <v>4826546.0174467</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>352717.2647319</v>
+        <v>356546.0174467</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.0789076654881208</v>
+        <v>0.07976420971961967</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-06-15
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -485,7 +485,7 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-14 06:38 IST</t>
+          <t>Generated: 2026-06-15 07:16 IST</t>
         </is>
       </c>
     </row>
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>551575.4942779541</v>
+        <v>554199.0009765625</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-39206.52572204592</v>
+        <v>-36583.01902343752</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.0663637761386948</v>
+        <v>-0.06192304062238983</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5378121.511724654</v>
+        <v>5380745.018423262</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>317339.4917246541</v>
+        <v>319962.9984232625</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.06270562345316232</v>
+        <v>0.06322402291953735</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-06-14</t>
+          <t>Last snapshot: 2026-06-15</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM19"/>
+  <dimension ref="A1:AN19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -658,6 +658,7 @@
     <col width="21" customWidth="1" min="37" max="37"/>
     <col width="21" customWidth="1" min="38" max="38"/>
     <col width="21" customWidth="1" min="39" max="39"/>
+    <col width="21" customWidth="1" min="40" max="40"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -856,6 +857,11 @@
           <t>2026-06-14</t>
         </is>
       </c>
+      <c r="AN1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -875,13 +881,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>548.2999877929688</v>
+        <v>549</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>43863.9990234375</v>
+        <v>43920</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>46.48902343749796</v>
+        <v>102.489999999998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -978,6 +984,9 @@
       </c>
       <c r="AM2" s="3" t="n">
         <v>548.2999877929688</v>
+      </c>
+      <c r="AN2" s="3" t="n">
+        <v>549</v>
       </c>
     </row>
     <row r="3">
@@ -1025,13 +1034,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1508.599975585938</v>
+        <v>1541</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>30171.99951171875</v>
+        <v>30820</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-1932.580488281252</v>
+        <v>-1284.580000000002</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1128,6 +1137,9 @@
       </c>
       <c r="AM4" s="3" t="n">
         <v>1508.599975585938</v>
+      </c>
+      <c r="AN4" s="3" t="n">
+        <v>1541</v>
       </c>
     </row>
     <row r="5">
@@ -1148,13 +1160,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>673.7999877929688</v>
+        <v>670</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13475.99975585938</v>
+        <v>13400</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-737.1002441406254</v>
+        <v>-813.1000000000004</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1251,6 +1263,9 @@
       </c>
       <c r="AM5" s="3" t="n">
         <v>673.7999877929688</v>
+      </c>
+      <c r="AN5" s="3" t="n">
+        <v>670</v>
       </c>
     </row>
     <row r="6">
@@ -1271,13 +1286,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>377.2999877929688</v>
+        <v>389.1499938964844</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15091.99951171875</v>
+        <v>15565.99975585938</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2410.240488281252</v>
+        <v>-1936.240244140627</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1374,6 +1389,9 @@
       </c>
       <c r="AM6" s="3" t="n">
         <v>377.2999877929688</v>
+      </c>
+      <c r="AN6" s="3" t="n">
+        <v>389.1499938964844</v>
       </c>
     </row>
     <row r="7">
@@ -1394,13 +1412,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>234.6799926757812</v>
+        <v>237.3200073242188</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>23467.99926757812</v>
+        <v>23732.00073242188</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-2965.820732421875</v>
+        <v>-2701.819267578125</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1497,6 +1515,9 @@
       </c>
       <c r="AM7" s="3" t="n">
         <v>234.6799926757812</v>
+      </c>
+      <c r="AN7" s="3" t="n">
+        <v>237.3200073242188</v>
       </c>
     </row>
     <row r="8">
@@ -1544,13 +1565,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>18.38999938964844</v>
+        <v>18.54999923706055</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>27584.99908447266</v>
+        <v>27824.99885559082</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-3465.170915527342</v>
+        <v>-3225.171144409178</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1647,6 +1668,9 @@
       </c>
       <c r="AM9" s="3" t="n">
         <v>18.38999938964844</v>
+      </c>
+      <c r="AN9" s="3" t="n">
+        <v>18.54999923706055</v>
       </c>
     </row>
     <row r="10">
@@ -1667,13 +1691,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>417.7999877929688</v>
+        <v>418.3500061035156</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>41779.99877929688</v>
+        <v>41835.00061035156</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-9718.481220703128</v>
+        <v>-9663.479389648441</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1770,6 +1794,9 @@
       </c>
       <c r="AM10" s="3" t="n">
         <v>417.7999877929688</v>
+      </c>
+      <c r="AN10" s="3" t="n">
+        <v>418.3500061035156</v>
       </c>
     </row>
     <row r="11">
@@ -1790,13 +1817,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>8.920000076293945</v>
+        <v>9.260000228881836</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>8920.000076293945</v>
+        <v>9260.000228881836</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-921.2099237060538</v>
+        <v>-581.2097711181632</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -1893,6 +1920,9 @@
       </c>
       <c r="AM11" s="3" t="n">
         <v>8.920000076293945</v>
+      </c>
+      <c r="AN11" s="3" t="n">
+        <v>9.260000228881836</v>
       </c>
     </row>
     <row r="12">
@@ -1913,13 +1943,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2580.5</v>
+        <v>2586.5</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25805</v>
+        <v>25865</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-1918.25</v>
+        <v>-1858.25</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -2016,6 +2046,9 @@
       </c>
       <c r="AM12" s="3" t="n">
         <v>2580.5</v>
+      </c>
+      <c r="AN12" s="3" t="n">
+        <v>2586.5</v>
       </c>
     </row>
     <row r="13">
@@ -2036,13 +2069,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>55.08000183105469</v>
+        <v>55.93000030517578</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>33048.00109863281</v>
+        <v>33558.00018310547</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-1983.75890136719</v>
+        <v>-1473.759816894533</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -2139,6 +2172,9 @@
       </c>
       <c r="AM13" s="3" t="n">
         <v>55.08000183105469</v>
+      </c>
+      <c r="AN13" s="3" t="n">
+        <v>55.93000030517578</v>
       </c>
     </row>
     <row r="14">
@@ -2159,13 +2195,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>745.9500122070312</v>
+        <v>741.1500244140625</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>37297.50061035156</v>
+        <v>37057.50122070312</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-5165.00938964844</v>
+        <v>-5405.008779296877</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -2262,6 +2298,9 @@
       </c>
       <c r="AM14" s="3" t="n">
         <v>745.9500122070312</v>
+      </c>
+      <c r="AN14" s="3" t="n">
+        <v>741.1500244140625</v>
       </c>
     </row>
     <row r="15">
@@ -2336,13 +2375,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>598.8499755859375</v>
+        <v>596.7000122070312</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>29942.49877929688</v>
+        <v>29835.00061035156</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>8187.968779296876</v>
+        <v>8080.470610351564</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -2439,6 +2478,9 @@
       </c>
       <c r="AM17" s="3" t="n">
         <v>598.8499755859375</v>
+      </c>
+      <c r="AN17" s="3" t="n">
+        <v>596.7000122070312</v>
       </c>
     </row>
     <row r="18">
@@ -2459,13 +2501,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>393.5499877929688</v>
+        <v>397.5499877929688</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>39354.99877929688</v>
+        <v>39754.99877929688</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-7285.821220703125</v>
+        <v>-6885.821220703125</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -2562,6 +2604,9 @@
       </c>
       <c r="AM18" s="3" t="n">
         <v>393.5499877929688</v>
+      </c>
+      <c r="AN18" s="3" t="n">
+        <v>397.5499877929688</v>
       </c>
     </row>
     <row r="19">
@@ -2574,10 +2619,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>551575.4942779541</v>
+        <v>554199.0009765625</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-39206.52572204591</v>
+        <v>-36583.01902343751</v>
       </c>
     </row>
   </sheetData>
@@ -2591,7 +2636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN41"/>
+  <dimension ref="A1:AO41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2634,6 +2679,7 @@
     <col width="13" customWidth="1" min="38" max="38"/>
     <col width="13" customWidth="1" min="39" max="39"/>
     <col width="13" customWidth="1" min="40" max="40"/>
+    <col width="13" customWidth="1" min="41" max="41"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2837,6 +2883,11 @@
           <t>2026-06-14</t>
         </is>
       </c>
+      <c r="AO1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2965,6 +3016,9 @@
       <c r="AN2" s="3" t="n">
         <v>56.4319</v>
       </c>
+      <c r="AO2" s="3" t="n">
+        <v>56.4319</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3468,6 +3522,9 @@
       <c r="AN6" s="3" t="n">
         <v>12.0487</v>
       </c>
+      <c r="AO6" s="3" t="n">
+        <v>12.0487</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3721,6 +3778,9 @@
       <c r="AN8" s="3" t="n">
         <v>32.2764</v>
       </c>
+      <c r="AO8" s="3" t="n">
+        <v>32.2764</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4224,6 +4284,9 @@
       <c r="AN12" s="3" t="n">
         <v>220.156</v>
       </c>
+      <c r="AO12" s="3" t="n">
+        <v>220.156</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4352,6 +4415,9 @@
       <c r="AN13" s="3" t="n">
         <v>20.313</v>
       </c>
+      <c r="AO13" s="3" t="n">
+        <v>20.313</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4605,6 +4671,9 @@
       <c r="AN15" s="3" t="n">
         <v>11.66</v>
       </c>
+      <c r="AO15" s="3" t="n">
+        <v>11.66</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4983,6 +5052,9 @@
       <c r="AN18" s="3" t="n">
         <v>45.09</v>
       </c>
+      <c r="AO18" s="3" t="n">
+        <v>45.09</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5236,6 +5308,9 @@
       <c r="AN20" s="3" t="n">
         <v>9.17</v>
       </c>
+      <c r="AO20" s="3" t="n">
+        <v>9.17</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5364,6 +5439,9 @@
       <c r="AN21" s="3" t="n">
         <v>108.3559</v>
       </c>
+      <c r="AO21" s="3" t="n">
+        <v>108.3559</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5617,6 +5695,9 @@
       <c r="AN23" s="3" t="n">
         <v>61.3411</v>
       </c>
+      <c r="AO23" s="3" t="n">
+        <v>61.3411</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -6126,6 +6207,9 @@
       <c r="AN27" s="3" t="n">
         <v>62.6305</v>
       </c>
+      <c r="AO27" s="3" t="n">
+        <v>62.6305</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6254,6 +6338,9 @@
       <c r="AN28" s="3" t="n">
         <v>104.5676</v>
       </c>
+      <c r="AO28" s="3" t="n">
+        <v>104.5676</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -6758,6 +6845,9 @@
         <v>10.2</v>
       </c>
       <c r="AN32" s="3" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="AO32" s="3" t="n">
         <v>10.2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily portfolio update 2026-06-16
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -485,7 +485,7 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-15 07:16 IST</t>
+          <t>Generated: 2026-06-16 07:25 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4826546.0174467</v>
+        <v>4897378.0183038</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>356546.0174466996</v>
+        <v>427378.0183038004</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.07976420971961959</v>
+        <v>0.09561029492255042</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>554199.0009765625</v>
+        <v>553627.0022659302</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-36583.01902343752</v>
+        <v>-37155.01773406984</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.06192304062238983</v>
+        <v>-0.06289124664638548</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5380745.018423262</v>
+        <v>5451005.020569731</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>319962.9984232625</v>
+        <v>390223.000569731</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.06322402291953735</v>
+        <v>0.07710725319280419</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-06-15</t>
+          <t>Last snapshot: 2026-06-16</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN19"/>
+  <dimension ref="A1:AO19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -659,6 +659,7 @@
     <col width="21" customWidth="1" min="38" max="38"/>
     <col width="21" customWidth="1" min="39" max="39"/>
     <col width="21" customWidth="1" min="40" max="40"/>
+    <col width="21" customWidth="1" min="41" max="41"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -862,6 +863,11 @@
           <t>2026-06-15</t>
         </is>
       </c>
+      <c r="AO1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -881,13 +887,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>549</v>
+        <v>552.6500244140625</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>43920</v>
+        <v>44212.001953125</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>102.489999999998</v>
+        <v>394.491953124998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -987,6 +993,9 @@
       </c>
       <c r="AN2" s="3" t="n">
         <v>549</v>
+      </c>
+      <c r="AO2" s="3" t="n">
+        <v>552.6500244140625</v>
       </c>
     </row>
     <row r="3">
@@ -1034,13 +1043,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1541</v>
+        <v>1569.599975585938</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>30820</v>
+        <v>31391.99951171875</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-1284.580000000002</v>
+        <v>-712.5804882812517</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1140,6 +1149,9 @@
       </c>
       <c r="AN4" s="3" t="n">
         <v>1541</v>
+      </c>
+      <c r="AO4" s="3" t="n">
+        <v>1569.599975585938</v>
       </c>
     </row>
     <row r="5">
@@ -1160,13 +1172,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>670</v>
+        <v>673.6500244140625</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13400</v>
+        <v>13473.00048828125</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-813.1000000000004</v>
+        <v>-740.0995117187504</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1266,6 +1278,9 @@
       </c>
       <c r="AN5" s="3" t="n">
         <v>670</v>
+      </c>
+      <c r="AO5" s="3" t="n">
+        <v>673.6500244140625</v>
       </c>
     </row>
     <row r="6">
@@ -1286,13 +1301,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>389.1499938964844</v>
+        <v>388.7000122070312</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15565.99975585938</v>
+        <v>15548.00048828125</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-1936.240244140627</v>
+        <v>-1954.239511718752</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1392,6 +1407,9 @@
       </c>
       <c r="AN6" s="3" t="n">
         <v>389.1499938964844</v>
+      </c>
+      <c r="AO6" s="3" t="n">
+        <v>388.7000122070312</v>
       </c>
     </row>
     <row r="7">
@@ -1412,13 +1430,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>237.3200073242188</v>
+        <v>234.0899963378906</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>23732.00073242188</v>
+        <v>23408.99963378906</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-2701.819267578125</v>
+        <v>-3024.820366210937</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1518,6 +1536,9 @@
       </c>
       <c r="AN7" s="3" t="n">
         <v>237.3200073242188</v>
+      </c>
+      <c r="AO7" s="3" t="n">
+        <v>234.0899963378906</v>
       </c>
     </row>
     <row r="8">
@@ -1565,13 +1586,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>18.54999923706055</v>
+        <v>17.8700008392334</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>27824.99885559082</v>
+        <v>26805.0012588501</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-3225.171144409178</v>
+        <v>-4245.168741149901</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1671,6 +1692,9 @@
       </c>
       <c r="AN9" s="3" t="n">
         <v>18.54999923706055</v>
+      </c>
+      <c r="AO9" s="3" t="n">
+        <v>17.8700008392334</v>
       </c>
     </row>
     <row r="10">
@@ -1691,13 +1715,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>418.3500061035156</v>
+        <v>419.3999938964844</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>41835.00061035156</v>
+        <v>41939.99938964844</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-9663.479389648441</v>
+        <v>-9558.480610351566</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1797,6 +1821,9 @@
       </c>
       <c r="AN10" s="3" t="n">
         <v>418.3500061035156</v>
+      </c>
+      <c r="AO10" s="3" t="n">
+        <v>419.3999938964844</v>
       </c>
     </row>
     <row r="11">
@@ -1817,13 +1844,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>9.260000228881836</v>
+        <v>9.090000152587891</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>9260.000228881836</v>
+        <v>9090.000152587891</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-581.2097711181632</v>
+        <v>-751.2098474121085</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -1923,6 +1950,9 @@
       </c>
       <c r="AN11" s="3" t="n">
         <v>9.260000228881836</v>
+      </c>
+      <c r="AO11" s="3" t="n">
+        <v>9.090000152587891</v>
       </c>
     </row>
     <row r="12">
@@ -1943,13 +1973,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2586.5</v>
+        <v>2588.5</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25865</v>
+        <v>25885</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-1858.25</v>
+        <v>-1838.25</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -2049,6 +2079,9 @@
       </c>
       <c r="AN12" s="3" t="n">
         <v>2586.5</v>
+      </c>
+      <c r="AO12" s="3" t="n">
+        <v>2588.5</v>
       </c>
     </row>
     <row r="13">
@@ -2069,13 +2102,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>55.93000030517578</v>
+        <v>58</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>33558.00018310547</v>
+        <v>34800</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-1473.759816894533</v>
+        <v>-231.760000000002</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -2175,6 +2208,9 @@
       </c>
       <c r="AN13" s="3" t="n">
         <v>55.93000030517578</v>
+      </c>
+      <c r="AO13" s="3" t="n">
+        <v>58</v>
       </c>
     </row>
     <row r="14">
@@ -2195,13 +2231,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>741.1500244140625</v>
+        <v>726.1500244140625</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>37057.50122070312</v>
+        <v>36307.50122070312</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-5405.008779296877</v>
+        <v>-6155.008779296877</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -2301,6 +2337,9 @@
       </c>
       <c r="AN14" s="3" t="n">
         <v>741.1500244140625</v>
+      </c>
+      <c r="AO14" s="3" t="n">
+        <v>726.1500244140625</v>
       </c>
     </row>
     <row r="15">
@@ -2375,13 +2414,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>596.7000122070312</v>
+        <v>578.2999877929688</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>29835.00061035156</v>
+        <v>28914.99938964844</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>8080.470610351564</v>
+        <v>7160.469389648439</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -2481,6 +2520,9 @@
       </c>
       <c r="AN17" s="3" t="n">
         <v>596.7000122070312</v>
+      </c>
+      <c r="AO17" s="3" t="n">
+        <v>578.2999877929688</v>
       </c>
     </row>
     <row r="18">
@@ -2501,13 +2543,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>397.5499877929688</v>
+        <v>400.7999877929688</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>39754.99877929688</v>
+        <v>40079.99877929688</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-6885.821220703125</v>
+        <v>-6560.821220703125</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -2607,6 +2649,9 @@
       </c>
       <c r="AN18" s="3" t="n">
         <v>397.5499877929688</v>
+      </c>
+      <c r="AO18" s="3" t="n">
+        <v>400.7999877929688</v>
       </c>
     </row>
     <row r="19">
@@ -2619,10 +2664,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>554199.0009765625</v>
+        <v>553627.0022659302</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-36583.01902343751</v>
+        <v>-37155.01773406984</v>
       </c>
     </row>
   </sheetData>
@@ -2636,7 +2681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO41"/>
+  <dimension ref="A1:AP41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2680,6 +2725,7 @@
     <col width="13" customWidth="1" min="39" max="39"/>
     <col width="13" customWidth="1" min="40" max="40"/>
     <col width="13" customWidth="1" min="41" max="41"/>
+    <col width="13" customWidth="1" min="42" max="42"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2888,6 +2934,11 @@
           <t>2026-06-15</t>
         </is>
       </c>
+      <c r="AP1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2912,16 +2963,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.4319</v>
+        <v>57.3828</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>63343.7919758</v>
+        <v>64411.1601096</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>13343.7919758</v>
+        <v>14411.1601096</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.266875839516</v>
+        <v>0.288223202192</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -3018,6 +3069,9 @@
       </c>
       <c r="AO2" s="3" t="n">
         <v>56.4319</v>
+      </c>
+      <c r="AP2" s="3" t="n">
+        <v>57.3828</v>
       </c>
     </row>
     <row r="3">
@@ -3043,16 +3097,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.3187</v>
+        <v>25.5977</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>62162.80138310001</v>
+        <v>62847.80581010001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>2162.801383100006</v>
+        <v>2847.805810100006</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.03604668971833343</v>
+        <v>0.04746343016833343</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -3143,6 +3197,9 @@
       </c>
       <c r="AN3" s="3" t="n">
         <v>25.3187</v>
+      </c>
+      <c r="AP3" s="3" t="n">
+        <v>25.5977</v>
       </c>
     </row>
     <row r="4">
@@ -3168,16 +3225,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.29</v>
+        <v>12.54</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>236042.88297</v>
+        <v>240844.40622</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>56042.88297000001</v>
+        <v>60844.40622</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3113493498333333</v>
+        <v>0.338024479</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -3268,6 +3325,9 @@
       </c>
       <c r="AN4" s="3" t="n">
         <v>12.29</v>
+      </c>
+      <c r="AP4" s="3" t="n">
+        <v>12.54</v>
       </c>
     </row>
     <row r="5">
@@ -3293,16 +3353,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.326700000000001</v>
+        <v>9.404500000000001</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>171183.0725496</v>
+        <v>172611.020596</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-38816.92745039999</v>
+        <v>-37388.97940399998</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1848425116685714</v>
+        <v>-0.1780427590666666</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -3393,6 +3453,9 @@
       </c>
       <c r="AN5" s="3" t="n">
         <v>9.326700000000001</v>
+      </c>
+      <c r="AP5" s="3" t="n">
+        <v>9.404500000000001</v>
       </c>
     </row>
     <row r="6">
@@ -3418,16 +3481,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.0487</v>
+        <v>12.147</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>50953.6751799</v>
+        <v>51369.383619</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>953.6751798999976</v>
+        <v>1369.383619</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.01907350359799995</v>
+        <v>0.02738767238</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -3524,6 +3587,9 @@
       </c>
       <c r="AO6" s="3" t="n">
         <v>12.0487</v>
+      </c>
+      <c r="AP6" s="3" t="n">
+        <v>12.147</v>
       </c>
     </row>
     <row r="7">
@@ -3549,16 +3615,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>34.0781</v>
+        <v>34.2063</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>75177.651724</v>
+        <v>75460.466052</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>15177.651724</v>
+        <v>15460.466052</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2529608620666666</v>
+        <v>0.2576744342000001</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -3649,6 +3715,9 @@
       </c>
       <c r="AN7" s="3" t="n">
         <v>34.0781</v>
+      </c>
+      <c r="AP7" s="3" t="n">
+        <v>34.2063</v>
       </c>
     </row>
     <row r="8">
@@ -3674,16 +3743,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>32.2764</v>
+        <v>32.6846</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>51790.48550520001</v>
+        <v>52445.48036780001</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>1790.485505200006</v>
+        <v>2445.48036780001</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.03580971010400012</v>
+        <v>0.0489096073560002</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -3780,6 +3849,9 @@
       </c>
       <c r="AO8" s="3" t="n">
         <v>32.2764</v>
+      </c>
+      <c r="AP8" s="3" t="n">
+        <v>32.6846</v>
       </c>
     </row>
     <row r="9">
@@ -3805,16 +3877,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>41.3929</v>
+        <v>42.775</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>133260.0125097</v>
+        <v>137709.535575</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>33260.0125097</v>
+        <v>37709.53557499999</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.332600125097</v>
+        <v>0.3770953557499999</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -3905,6 +3977,9 @@
       </c>
       <c r="AN9" s="3" t="n">
         <v>41.3929</v>
+      </c>
+      <c r="AP9" s="3" t="n">
+        <v>42.775</v>
       </c>
     </row>
     <row r="10">
@@ -3930,16 +4005,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>46.9497</v>
+        <v>47.3815</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>133649.7860523</v>
+        <v>134878.9734085</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>33649.78605230001</v>
+        <v>34878.97340850002</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3364978605230001</v>
+        <v>0.3487897340850002</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -4030,6 +4105,9 @@
       </c>
       <c r="AN10" s="3" t="n">
         <v>46.9497</v>
+      </c>
+      <c r="AP10" s="3" t="n">
+        <v>47.3815</v>
       </c>
     </row>
     <row r="11">
@@ -4055,16 +4133,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>104.0296</v>
+        <v>106.8136</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31304.4832024</v>
+        <v>32142.2416984</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1304.483202399999</v>
+        <v>2142.241698399997</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.04348277341333329</v>
+        <v>0.07140805661333324</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -4155,6 +4233,9 @@
       </c>
       <c r="AN11" s="3" t="n">
         <v>104.0296</v>
+      </c>
+      <c r="AP11" s="3" t="n">
+        <v>106.8136</v>
       </c>
     </row>
     <row r="12">
@@ -4180,16 +4261,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>220.156</v>
+        <v>223.036</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>102487.461432</v>
+        <v>103828.164792</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>2487.461431999996</v>
+        <v>3828.164791999996</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.02487461431999996</v>
+        <v>0.03828164791999996</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -4286,6 +4367,9 @@
       </c>
       <c r="AO12" s="3" t="n">
         <v>220.156</v>
+      </c>
+      <c r="AP12" s="3" t="n">
+        <v>223.036</v>
       </c>
     </row>
     <row r="13">
@@ -4311,16 +4395,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>20.313</v>
+        <v>20.169</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>235379.020365</v>
+        <v>233710.405245</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>35379.02036499997</v>
+        <v>33710.405245</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.1768951018249999</v>
+        <v>0.168552026225</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -4417,6 +4501,9 @@
       </c>
       <c r="AO13" s="3" t="n">
         <v>20.313</v>
+      </c>
+      <c r="AP13" s="3" t="n">
+        <v>20.169</v>
       </c>
     </row>
     <row r="14">
@@ -4442,16 +4529,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>38.7849</v>
+        <v>39.549</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>139920.6379494</v>
+        <v>142677.209694</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>39920.6379494</v>
+        <v>42677.20969400002</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.399206379494</v>
+        <v>0.4267720969400002</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -4542,6 +4629,9 @@
       </c>
       <c r="AN14" s="3" t="n">
         <v>38.7849</v>
+      </c>
+      <c r="AP14" s="3" t="n">
+        <v>39.549</v>
       </c>
     </row>
     <row r="15">
@@ -4567,16 +4657,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.66</v>
+        <v>11.75</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>113614.42202</v>
+        <v>114491.37725</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>13614.42202</v>
+        <v>14491.37725000001</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1361442202</v>
+        <v>0.1449137725</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -4673,6 +4763,9 @@
       </c>
       <c r="AO15" s="3" t="n">
         <v>11.66</v>
+      </c>
+      <c r="AP15" s="3" t="n">
+        <v>11.75</v>
       </c>
     </row>
     <row r="16">
@@ -4698,16 +4791,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.6055</v>
+        <v>25.1724</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>140815.504904</v>
+        <v>144059.8327872</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>40815.504904</v>
+        <v>44059.83278719999</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.40815504904</v>
+        <v>0.4405983278719999</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -4798,6 +4891,9 @@
       </c>
       <c r="AN16" s="3" t="n">
         <v>24.6055</v>
+      </c>
+      <c r="AP16" s="3" t="n">
+        <v>25.1724</v>
       </c>
     </row>
     <row r="17">
@@ -4823,16 +4919,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.7283</v>
+        <v>16.8258</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55304.7133131</v>
+        <v>55627.0538706</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5304.713313100001</v>
+        <v>5627.053870600001</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.106094266262</v>
+        <v>0.112541077412</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -4923,6 +5019,9 @@
       </c>
       <c r="AN17" s="3" t="n">
         <v>16.7283</v>
+      </c>
+      <c r="AP17" s="3" t="n">
+        <v>16.8258</v>
       </c>
     </row>
     <row r="18">
@@ -4948,16 +5047,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>45.09</v>
+        <v>45.05</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>85059.39924</v>
+        <v>84983.94179999999</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>5059.399239999999</v>
+        <v>4983.941799999986</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.06324249049999998</v>
+        <v>0.06229927249999982</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -5054,6 +5153,9 @@
       </c>
       <c r="AO18" s="3" t="n">
         <v>45.09</v>
+      </c>
+      <c r="AP18" s="3" t="n">
+        <v>45.05</v>
       </c>
     </row>
     <row r="19">
@@ -5079,16 +5181,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>14.3784</v>
+        <v>14.7403</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>208008.9482544</v>
+        <v>213244.4708698</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>58008.94825439999</v>
+        <v>63244.47086979999</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.386726321696</v>
+        <v>0.4216298057986666</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -5179,6 +5281,9 @@
       </c>
       <c r="AN19" s="3" t="n">
         <v>14.3784</v>
+      </c>
+      <c r="AP19" s="3" t="n">
+        <v>14.7403</v>
       </c>
     </row>
     <row r="20">
@@ -5204,16 +5309,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.17</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>240765.71351</v>
+        <v>243916.40987</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-9234.286489999999</v>
+        <v>-6083.590130000026</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.03693714595999999</v>
+        <v>-0.0243343605200001</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -5310,6 +5415,9 @@
       </c>
       <c r="AO20" s="3" t="n">
         <v>9.17</v>
+      </c>
+      <c r="AP20" s="3" t="n">
+        <v>9.289999999999999</v>
       </c>
     </row>
     <row r="21">
@@ -5335,16 +5443,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>108.3559</v>
+        <v>109.8342</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>164620.6762781</v>
+        <v>166866.5968578</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-5379.3237219</v>
+        <v>-3133.403142199997</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.03164308071705883</v>
+        <v>-0.01843178318941175</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -5441,6 +5549,9 @@
       </c>
       <c r="AO21" s="3" t="n">
         <v>108.3559</v>
+      </c>
+      <c r="AP21" s="3" t="n">
+        <v>109.8342</v>
       </c>
     </row>
     <row r="22">
@@ -5466,16 +5577,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>44.011</v>
+        <v>44.969</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>67533.11906000001</v>
+        <v>69003.13174</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>7533.119060000012</v>
+        <v>9003.131739999997</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1255519843333335</v>
+        <v>0.1500521956666666</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -5566,6 +5677,9 @@
       </c>
       <c r="AN22" s="3" t="n">
         <v>44.011</v>
+      </c>
+      <c r="AP22" s="3" t="n">
+        <v>44.969</v>
       </c>
     </row>
     <row r="23">
@@ -5591,16 +5705,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>61.3411</v>
+        <v>62.3803</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>166631.0738937</v>
+        <v>169454.0264001</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>16631.0738937</v>
+        <v>19454.0264001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.110873825958</v>
+        <v>0.129693509334</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -5697,6 +5811,9 @@
       </c>
       <c r="AO23" s="3" t="n">
         <v>61.3411</v>
+      </c>
+      <c r="AP23" s="3" t="n">
+        <v>62.3803</v>
       </c>
     </row>
     <row r="24">
@@ -5722,16 +5839,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>28.1701</v>
+        <v>28.4706</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>102352.8469586</v>
+        <v>103444.6794516</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>2352.846958599999</v>
+        <v>3444.679451600008</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.02352846958599999</v>
+        <v>0.03444679451600008</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -5822,6 +5939,9 @@
       </c>
       <c r="AN24" s="3" t="n">
         <v>28.1701</v>
+      </c>
+      <c r="AP24" s="3" t="n">
+        <v>28.4706</v>
       </c>
     </row>
     <row r="25">
@@ -5847,16 +5967,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.2619</v>
+        <v>11.56</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>184939.2504206</v>
+        <v>189834.55144</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-15060.7495794</v>
+        <v>-10165.44855999999</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.07530374789699999</v>
+        <v>-0.05082724279999995</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -5950,6 +6070,9 @@
       </c>
       <c r="AN25" s="3" t="n">
         <v>11.2619</v>
+      </c>
+      <c r="AP25" s="3" t="n">
+        <v>11.56</v>
       </c>
     </row>
     <row r="26">
@@ -5975,16 +6098,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>8.8187</v>
+        <v>8.985300000000001</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>105310.4020705</v>
+        <v>107299.8917895</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>-4689.5979295</v>
+        <v>-2700.108210499995</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>-0.04263270845</v>
+        <v>-0.02454643827727268</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -6078,6 +6201,9 @@
       </c>
       <c r="AN26" s="3" t="n">
         <v>8.8187</v>
+      </c>
+      <c r="AP26" s="3" t="n">
+        <v>8.985300000000001</v>
       </c>
     </row>
     <row r="27">
@@ -6103,16 +6229,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>62.6305</v>
+        <v>64.0227</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>100888.96723</v>
+        <v>103131.606522</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-9111.032770000005</v>
+        <v>-6868.393478000013</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.08282757063636369</v>
+        <v>-0.06243994070909102</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -6209,6 +6335,9 @@
       </c>
       <c r="AO27" s="3" t="n">
         <v>62.6305</v>
+      </c>
+      <c r="AP27" s="3" t="n">
+        <v>64.0227</v>
       </c>
     </row>
     <row r="28">
@@ -6234,16 +6363,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>104.5676</v>
+        <v>107.7604</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>345769.1865132</v>
+        <v>356326.6809828</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-34230.81348680001</v>
+        <v>-23673.31901719997</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.0900810881231579</v>
+        <v>-0.06229820793999993</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -6340,6 +6469,9 @@
       </c>
       <c r="AO28" s="3" t="n">
         <v>104.5676</v>
+      </c>
+      <c r="AP28" s="3" t="n">
+        <v>107.7604</v>
       </c>
     </row>
     <row r="29">
@@ -6365,16 +6497,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.79</v>
+        <v>11.966</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>113227.65837</v>
+        <v>114917.910098</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>13227.65836999999</v>
+        <v>14917.91009799999</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.1322765836999999</v>
+        <v>0.1491791009799999</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -6465,6 +6597,9 @@
       </c>
       <c r="AN29" s="3" t="n">
         <v>11.79</v>
+      </c>
+      <c r="AP29" s="3" t="n">
+        <v>11.966</v>
       </c>
     </row>
     <row r="30">
@@ -6490,16 +6625,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>15.5484</v>
+        <v>15.8643</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>114993.8051724</v>
+        <v>117330.1576623</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>14993.80517240001</v>
+        <v>17330.1576623</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.1499380517240001</v>
+        <v>0.173301576623</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -6590,6 +6725,9 @@
       </c>
       <c r="AN30" s="3" t="n">
         <v>15.5484</v>
+      </c>
+      <c r="AP30" s="3" t="n">
+        <v>15.8643</v>
       </c>
     </row>
     <row r="31">
@@ -6615,16 +6753,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>409.1495</v>
+        <v>414.7285</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>108866.49896</v>
+        <v>110350.95928</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>8866.498959999997</v>
+        <v>10350.95928</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.08866498959999997</v>
+        <v>0.1035095928</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -6718,6 +6856,9 @@
       </c>
       <c r="AN31" s="3" t="n">
         <v>409.1495</v>
+      </c>
+      <c r="AP31" s="3" t="n">
+        <v>414.7285</v>
       </c>
     </row>
     <row r="32">
@@ -6743,16 +6884,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.2</v>
+        <v>10.33</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>215627.592</v>
+        <v>218375.7868</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>15627.59199999998</v>
+        <v>18375.7868</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.07813795999999988</v>
+        <v>0.09187893400000001</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -6849,6 +6990,9 @@
       </c>
       <c r="AO32" s="3" t="n">
         <v>10.2</v>
+      </c>
+      <c r="AP32" s="3" t="n">
+        <v>10.33</v>
       </c>
     </row>
     <row r="33">
@@ -6874,16 +7018,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>18.13</v>
+        <v>18.29</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>64971.39319999999</v>
+        <v>65544.77559999999</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>4971.393199999991</v>
+        <v>5544.775599999994</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.08285655333333319</v>
+        <v>0.09241292666666656</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -6974,6 +7118,9 @@
       </c>
       <c r="AN33" s="3" t="n">
         <v>18.13</v>
+      </c>
+      <c r="AP33" s="3" t="n">
+        <v>18.29</v>
       </c>
     </row>
     <row r="34">
@@ -6999,16 +7146,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>208.1454</v>
+        <v>210.1009</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>73169.5606074</v>
+        <v>73856.97947789999</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-6830.439392600005</v>
+        <v>-6143.020522100007</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.08538049240750006</v>
+        <v>-0.07678775652625008</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -7102,6 +7249,9 @@
       </c>
       <c r="AN34" s="3" t="n">
         <v>208.1454</v>
+      </c>
+      <c r="AP34" s="3" t="n">
+        <v>210.1009</v>
       </c>
     </row>
     <row r="35">
@@ -7127,16 +7277,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>14.43</v>
+        <v>14.64</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>102964.15389</v>
+        <v>104462.59272</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>2964.153890000001</v>
+        <v>4462.592720000001</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.02964153890000001</v>
+        <v>0.04462592720000001</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -7230,6 +7380,9 @@
       </c>
       <c r="AN35" s="3" t="n">
         <v>14.43</v>
+      </c>
+      <c r="AP35" s="3" t="n">
+        <v>14.64</v>
       </c>
     </row>
     <row r="36">
@@ -7255,16 +7408,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>355.9597</v>
+        <v>354.4978</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>165772.5680482</v>
+        <v>165091.7524468</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>15772.56804820002</v>
+        <v>15091.7524468</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1051504536546668</v>
+        <v>0.1006116829786667</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -7358,6 +7511,9 @@
       </c>
       <c r="AN36" s="3" t="n">
         <v>355.9597</v>
+      </c>
+      <c r="AP36" s="3" t="n">
+        <v>354.4978</v>
       </c>
     </row>
     <row r="37">
@@ -7383,16 +7539,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>15.947</v>
+        <v>15.837</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>60006.790883</v>
+        <v>59592.873093</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>10006.790883</v>
+        <v>9592.873093000002</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.20013581766</v>
+        <v>0.1918574618600001</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -7486,6 +7642,9 @@
       </c>
       <c r="AN37" s="3" t="n">
         <v>15.947</v>
+      </c>
+      <c r="AP37" s="3" t="n">
+        <v>15.837</v>
       </c>
     </row>
     <row r="38">
@@ -7511,16 +7670,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13.9727</v>
+        <v>14.1626</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>83563.4808414</v>
+        <v>84699.1743732</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>3563.4808414</v>
+        <v>4699.174373200003</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.0445435105175</v>
+        <v>0.05873967966500004</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -7611,6 +7770,9 @@
       </c>
       <c r="AN38" s="3" t="n">
         <v>13.9727</v>
+      </c>
+      <c r="AP38" s="3" t="n">
+        <v>14.1626</v>
       </c>
     </row>
     <row r="39">
@@ -7636,16 +7798,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1016.6971</v>
+        <v>1018.0503</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50713.8680451</v>
+        <v>50781.3670143</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>713.8680450999964</v>
+        <v>781.3670142999981</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.01427736090199993</v>
+        <v>0.01562734028599996</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -7736,6 +7898,9 @@
       </c>
       <c r="AN39" s="3" t="n">
         <v>1016.6971</v>
+      </c>
+      <c r="AP39" s="3" t="n">
+        <v>1018.0503</v>
       </c>
     </row>
     <row r="40">
@@ -7761,16 +7926,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>20.7098</v>
+        <v>20.9785</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>104398.6609646</v>
+        <v>105753.1849195</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>4398.660964600014</v>
+        <v>5753.184919499996</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.04398660964600015</v>
+        <v>0.05753184919499996</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -7864,6 +8029,9 @@
       </c>
       <c r="AN40" s="3" t="n">
         <v>20.7098</v>
+      </c>
+      <c r="AP40" s="3" t="n">
+        <v>20.9785</v>
       </c>
     </row>
     <row r="41">
@@ -7876,13 +8044,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4826546.0174467</v>
+        <v>4897378.0183038</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>356546.0174467</v>
+        <v>427378.0183038</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.07976420971961967</v>
+        <v>0.09561029492255034</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-06-17
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -484,7 +484,7 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-16 07:25 IST</t>
+          <t>Generated: 2026-06-17 07:07 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4897378.0183038</v>
+        <v>4916306.1372329</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>427378.0183038004</v>
+        <v>446306.1372328997</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.09561029492255042</v>
+        <v>0.09984477343017889</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>553627.0022659302</v>
+        <v>555423.002784729</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-37155.01773406984</v>
+        <v>-35359.01721527101</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.06289124664638548</v>
+        <v>-0.05985120741364305</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5451005.020569731</v>
+        <v>5471729.140017629</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>390223.000569731</v>
+        <v>410947.1200176291</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.07710725319280419</v>
+        <v>0.08120229608656987</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-06-16</t>
+          <t>Last snapshot: 2026-06-17</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO19"/>
+  <dimension ref="A1:AP19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -660,6 +660,7 @@
     <col width="21" customWidth="1" min="39" max="39"/>
     <col width="21" customWidth="1" min="40" max="40"/>
     <col width="21" customWidth="1" min="41" max="41"/>
+    <col width="21" customWidth="1" min="42" max="42"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -868,6 +869,11 @@
           <t>2026-06-16</t>
         </is>
       </c>
+      <c r="AP1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -887,13 +893,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>552.6500244140625</v>
+        <v>559.4500122070312</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>44212.001953125</v>
+        <v>44756.0009765625</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>394.491953124998</v>
+        <v>938.490976562498</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -996,6 +1002,9 @@
       </c>
       <c r="AO2" s="3" t="n">
         <v>552.6500244140625</v>
+      </c>
+      <c r="AP2" s="3" t="n">
+        <v>559.4500122070312</v>
       </c>
     </row>
     <row r="3">
@@ -1043,13 +1052,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1569.599975585938</v>
+        <v>1555.599975585938</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>31391.99951171875</v>
+        <v>31111.99951171875</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-712.5804882812517</v>
+        <v>-992.5804882812517</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1152,6 +1161,9 @@
       </c>
       <c r="AO4" s="3" t="n">
         <v>1569.599975585938</v>
+      </c>
+      <c r="AP4" s="3" t="n">
+        <v>1555.599975585938</v>
       </c>
     </row>
     <row r="5">
@@ -1172,13 +1184,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>673.6500244140625</v>
+        <v>659.4500122070312</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13473.00048828125</v>
+        <v>13189.00024414062</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-740.0995117187504</v>
+        <v>-1024.099755859375</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1281,6 +1293,9 @@
       </c>
       <c r="AO5" s="3" t="n">
         <v>673.6500244140625</v>
+      </c>
+      <c r="AP5" s="3" t="n">
+        <v>659.4500122070312</v>
       </c>
     </row>
     <row r="6">
@@ -1301,13 +1316,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>388.7000122070312</v>
+        <v>383.25</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15548.00048828125</v>
+        <v>15330</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-1954.239511718752</v>
+        <v>-2172.240000000002</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1410,6 +1425,9 @@
       </c>
       <c r="AO6" s="3" t="n">
         <v>388.7000122070312</v>
+      </c>
+      <c r="AP6" s="3" t="n">
+        <v>383.25</v>
       </c>
     </row>
     <row r="7">
@@ -1430,13 +1448,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>234.0899963378906</v>
+        <v>241.6000061035156</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>23408.99963378906</v>
+        <v>24160.00061035156</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-3024.820366210937</v>
+        <v>-2273.819389648437</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1539,6 +1557,9 @@
       </c>
       <c r="AO7" s="3" t="n">
         <v>234.0899963378906</v>
+      </c>
+      <c r="AP7" s="3" t="n">
+        <v>241.6000061035156</v>
       </c>
     </row>
     <row r="8">
@@ -1586,13 +1607,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>17.8700008392334</v>
+        <v>18.21999931335449</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>26805.0012588501</v>
+        <v>27329.99897003174</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-4245.168741149901</v>
+        <v>-3720.17102996826</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1695,6 +1716,9 @@
       </c>
       <c r="AO9" s="3" t="n">
         <v>17.8700008392334</v>
+      </c>
+      <c r="AP9" s="3" t="n">
+        <v>18.21999931335449</v>
       </c>
     </row>
     <row r="10">
@@ -1715,13 +1739,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>419.3999938964844</v>
+        <v>415.2000122070312</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>41939.99938964844</v>
+        <v>41520.00122070312</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-9558.480610351566</v>
+        <v>-9978.478779296878</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1824,6 +1848,9 @@
       </c>
       <c r="AO10" s="3" t="n">
         <v>419.3999938964844</v>
+      </c>
+      <c r="AP10" s="3" t="n">
+        <v>415.2000122070312</v>
       </c>
     </row>
     <row r="11">
@@ -1844,13 +1871,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>9.090000152587891</v>
+        <v>9.020000457763672</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>9090.000152587891</v>
+        <v>9020.000457763672</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-751.2098474121085</v>
+        <v>-821.2095422363273</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -1953,6 +1980,9 @@
       </c>
       <c r="AO11" s="3" t="n">
         <v>9.090000152587891</v>
+      </c>
+      <c r="AP11" s="3" t="n">
+        <v>9.020000457763672</v>
       </c>
     </row>
     <row r="12">
@@ -1973,13 +2003,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2588.5</v>
+        <v>2633</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25885</v>
+        <v>26330</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-1838.25</v>
+        <v>-1393.25</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -2082,6 +2112,9 @@
       </c>
       <c r="AO12" s="3" t="n">
         <v>2588.5</v>
+      </c>
+      <c r="AP12" s="3" t="n">
+        <v>2633</v>
       </c>
     </row>
     <row r="13">
@@ -2102,13 +2135,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>58</v>
+        <v>57.93000030517578</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>34800</v>
+        <v>34758.00018310547</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-231.760000000002</v>
+        <v>-273.7598168945333</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -2211,6 +2244,9 @@
       </c>
       <c r="AO13" s="3" t="n">
         <v>58</v>
+      </c>
+      <c r="AP13" s="3" t="n">
+        <v>57.93000030517578</v>
       </c>
     </row>
     <row r="14">
@@ -2231,13 +2267,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>726.1500244140625</v>
+        <v>729.2000122070312</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>36307.50122070312</v>
+        <v>36460.00061035156</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-6155.008779296877</v>
+        <v>-6002.50938964844</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -2340,6 +2376,9 @@
       </c>
       <c r="AO14" s="3" t="n">
         <v>726.1500244140625</v>
+      </c>
+      <c r="AP14" s="3" t="n">
+        <v>729.2000122070312</v>
       </c>
     </row>
     <row r="15">
@@ -2414,13 +2453,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>578.2999877929688</v>
+        <v>592.25</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>28914.99938964844</v>
+        <v>29612.5</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>7160.469389648439</v>
+        <v>7857.970000000001</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -2523,6 +2562,9 @@
       </c>
       <c r="AO17" s="3" t="n">
         <v>578.2999877929688</v>
+      </c>
+      <c r="AP17" s="3" t="n">
+        <v>592.25</v>
       </c>
     </row>
     <row r="18">
@@ -2543,13 +2585,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>400.7999877929688</v>
+        <v>400.75</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>40079.99877929688</v>
+        <v>40075</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-6560.821220703125</v>
+        <v>-6565.82</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -2652,6 +2694,9 @@
       </c>
       <c r="AO18" s="3" t="n">
         <v>400.7999877929688</v>
+      </c>
+      <c r="AP18" s="3" t="n">
+        <v>400.75</v>
       </c>
     </row>
     <row r="19">
@@ -2664,10 +2709,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>553627.0022659302</v>
+        <v>555423.002784729</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-37155.01773406984</v>
+        <v>-35359.01721527101</v>
       </c>
     </row>
   </sheetData>
@@ -2681,7 +2726,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP41"/>
+  <dimension ref="A1:AQ41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2726,6 +2771,7 @@
     <col width="13" customWidth="1" min="40" max="40"/>
     <col width="13" customWidth="1" min="41" max="41"/>
     <col width="13" customWidth="1" min="42" max="42"/>
+    <col width="13" customWidth="1" min="43" max="43"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2939,6 +2985,11 @@
           <t>2026-06-16</t>
         </is>
       </c>
+      <c r="AQ1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2963,16 +3014,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>57.3828</v>
+        <v>57.0887</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>64411.1601096</v>
+        <v>64081.0381534</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>14411.1601096</v>
+        <v>14081.0381534</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.288223202192</v>
+        <v>0.2816207630680001</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -3072,6 +3123,9 @@
       </c>
       <c r="AP2" s="3" t="n">
         <v>57.3828</v>
+      </c>
+      <c r="AQ2" s="3" t="n">
+        <v>57.0887</v>
       </c>
     </row>
     <row r="3">
@@ -3097,16 +3151,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.5977</v>
+        <v>25.6215</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>62847.80581010001</v>
+        <v>62906.2398795</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>2847.805810100006</v>
+        <v>2906.239879500004</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.04746343016833343</v>
+        <v>0.04843733132500008</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -3200,6 +3254,9 @@
       </c>
       <c r="AP3" s="3" t="n">
         <v>25.5977</v>
+      </c>
+      <c r="AQ3" s="3" t="n">
+        <v>25.6215</v>
       </c>
     </row>
     <row r="4">
@@ -3225,16 +3282,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.54</v>
+        <v>12.41</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>240844.40622</v>
+        <v>238347.61413</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>60844.40622</v>
+        <v>58347.61413</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.338024479</v>
+        <v>0.3241534118333333</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -3328,6 +3385,9 @@
       </c>
       <c r="AP4" s="3" t="n">
         <v>12.54</v>
+      </c>
+      <c r="AQ4" s="3" t="n">
+        <v>12.41</v>
       </c>
     </row>
     <row r="5">
@@ -3353,16 +3413,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.404500000000001</v>
+        <v>9.488300000000001</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>172611.020596</v>
+        <v>174149.0931704</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-37388.97940399998</v>
+        <v>-35850.90682959999</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1780427590666666</v>
+        <v>-0.1707186039504761</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -3456,6 +3516,9 @@
       </c>
       <c r="AP5" s="3" t="n">
         <v>9.404500000000001</v>
+      </c>
+      <c r="AQ5" s="3" t="n">
+        <v>9.488300000000001</v>
       </c>
     </row>
     <row r="6">
@@ -3481,16 +3544,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.147</v>
+        <v>12.2281</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>51369.383619</v>
+        <v>51712.3536537</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>1369.383619</v>
+        <v>1712.353653699996</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.02738767238</v>
+        <v>0.03424707307399993</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -3590,6 +3653,9 @@
       </c>
       <c r="AP6" s="3" t="n">
         <v>12.147</v>
+      </c>
+      <c r="AQ6" s="3" t="n">
+        <v>12.2281</v>
       </c>
     </row>
     <row r="7">
@@ -3615,16 +3681,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>34.2063</v>
+        <v>34.2288</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>75460.466052</v>
+        <v>75510.101952</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>15460.466052</v>
+        <v>15510.101952</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2576744342000001</v>
+        <v>0.2585016991999999</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -3718,6 +3784,9 @@
       </c>
       <c r="AP7" s="3" t="n">
         <v>34.2063</v>
+      </c>
+      <c r="AQ7" s="3" t="n">
+        <v>34.2288</v>
       </c>
     </row>
     <row r="8">
@@ -3743,16 +3812,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>32.6846</v>
+        <v>32.7202</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>52445.48036780001</v>
+        <v>52502.6038786</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>2445.48036780001</v>
+        <v>2502.603878599999</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.0489096073560002</v>
+        <v>0.05005207757199998</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -3852,6 +3921,9 @@
       </c>
       <c r="AP8" s="3" t="n">
         <v>32.6846</v>
+      </c>
+      <c r="AQ8" s="3" t="n">
+        <v>32.7202</v>
       </c>
     </row>
     <row r="9">
@@ -3877,16 +3949,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>42.775</v>
+        <v>43.0981</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>137709.535575</v>
+        <v>138749.7214533</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>37709.53557499999</v>
+        <v>38749.72145330001</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3770953557499999</v>
+        <v>0.3874972145330001</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -3980,6 +4052,9 @@
       </c>
       <c r="AP9" s="3" t="n">
         <v>42.775</v>
+      </c>
+      <c r="AQ9" s="3" t="n">
+        <v>43.0981</v>
       </c>
     </row>
     <row r="10">
@@ -4005,16 +4080,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>47.3815</v>
+        <v>47.5456</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>134878.9734085</v>
+        <v>135346.1101504</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>34878.97340850002</v>
+        <v>35346.1101504</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3487897340850002</v>
+        <v>0.353461101504</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -4108,6 +4183,9 @@
       </c>
       <c r="AP10" s="3" t="n">
         <v>47.3815</v>
+      </c>
+      <c r="AQ10" s="3" t="n">
+        <v>47.5456</v>
       </c>
     </row>
     <row r="11">
@@ -4133,16 +4211,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>106.8136</v>
+        <v>105.4261</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>32142.2416984</v>
+        <v>31724.7165859</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>2142.241698399997</v>
+        <v>1724.716585900002</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.07140805661333324</v>
+        <v>0.05749055286333338</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -4236,6 +4314,9 @@
       </c>
       <c r="AP11" s="3" t="n">
         <v>106.8136</v>
+      </c>
+      <c r="AQ11" s="3" t="n">
+        <v>105.4261</v>
       </c>
     </row>
     <row r="12">
@@ -4261,16 +4342,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>223.036</v>
+        <v>223.292</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>103828.164792</v>
+        <v>103947.338424</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>3828.164791999996</v>
+        <v>3947.338424000001</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.03828164791999996</v>
+        <v>0.03947338424000001</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -4370,6 +4451,9 @@
       </c>
       <c r="AP12" s="3" t="n">
         <v>223.036</v>
+      </c>
+      <c r="AQ12" s="3" t="n">
+        <v>223.292</v>
       </c>
     </row>
     <row r="13">
@@ -4395,16 +4479,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>20.169</v>
+        <v>20.152</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>233710.405245</v>
+        <v>233513.41596</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>33710.405245</v>
+        <v>33513.41596000001</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.168552026225</v>
+        <v>0.1675670798000001</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -4504,6 +4588,9 @@
       </c>
       <c r="AP13" s="3" t="n">
         <v>20.169</v>
+      </c>
+      <c r="AQ13" s="3" t="n">
+        <v>20.152</v>
       </c>
     </row>
     <row r="14">
@@ -4529,16 +4616,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>39.549</v>
+        <v>39.8038</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>142677.209694</v>
+        <v>143596.4277028</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>42677.20969400002</v>
+        <v>43596.42770280002</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.4267720969400002</v>
+        <v>0.4359642770280002</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -4632,6 +4719,9 @@
       </c>
       <c r="AP14" s="3" t="n">
         <v>39.549</v>
+      </c>
+      <c r="AQ14" s="3" t="n">
+        <v>39.8038</v>
       </c>
     </row>
     <row r="15">
@@ -4657,16 +4747,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.75</v>
+        <v>11.85</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>114491.37725</v>
+        <v>115465.77195</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>14491.37725000001</v>
+        <v>15465.77194999999</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1449137725</v>
+        <v>0.1546577195</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -4766,6 +4856,9 @@
       </c>
       <c r="AP15" s="3" t="n">
         <v>11.75</v>
+      </c>
+      <c r="AQ15" s="3" t="n">
+        <v>11.85</v>
       </c>
     </row>
     <row r="16">
@@ -4791,16 +4884,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>25.1724</v>
+        <v>24.7039</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>144059.8327872</v>
+        <v>141378.6410192</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>44059.83278719999</v>
+        <v>41378.6410192</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4405983278719999</v>
+        <v>0.413786410192</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -4894,6 +4987,9 @@
       </c>
       <c r="AP16" s="3" t="n">
         <v>25.1724</v>
+      </c>
+      <c r="AQ16" s="3" t="n">
+        <v>24.7039</v>
       </c>
     </row>
     <row r="17">
@@ -4919,16 +5015,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.8258</v>
+        <v>16.8624</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55627.0538706</v>
+        <v>55748.0555568</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5627.053870600001</v>
+        <v>5748.055556799998</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.112541077412</v>
+        <v>0.114961111136</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -5022,6 +5118,9 @@
       </c>
       <c r="AP17" s="3" t="n">
         <v>16.8258</v>
+      </c>
+      <c r="AQ17" s="3" t="n">
+        <v>16.8624</v>
       </c>
     </row>
     <row r="18">
@@ -5047,16 +5146,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>45.05</v>
+        <v>45</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>84983.94179999999</v>
+        <v>84889.62</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>4983.941799999986</v>
+        <v>4889.619999999995</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.06229927249999982</v>
+        <v>0.06112024999999994</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -5156,6 +5255,9 @@
       </c>
       <c r="AP18" s="3" t="n">
         <v>45.05</v>
+      </c>
+      <c r="AQ18" s="3" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="19">
@@ -5181,16 +5283,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>14.7403</v>
+        <v>15.055</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>213244.4708698</v>
+        <v>217797.16213</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>63244.47086979999</v>
+        <v>67797.16212999998</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.4216298057986666</v>
+        <v>0.4519810808666666</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -5284,6 +5386,9 @@
       </c>
       <c r="AP19" s="3" t="n">
         <v>14.7403</v>
+      </c>
+      <c r="AQ19" s="3" t="n">
+        <v>15.055</v>
       </c>
     </row>
     <row r="20">
@@ -5309,16 +5414,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.289999999999999</v>
+        <v>9.43</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>243916.40987</v>
+        <v>247592.22229</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-6083.590130000026</v>
+        <v>-2407.777709999995</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.0243343605200001</v>
+        <v>-0.009631110839999979</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -5418,6 +5523,9 @@
       </c>
       <c r="AP20" s="3" t="n">
         <v>9.289999999999999</v>
+      </c>
+      <c r="AQ20" s="3" t="n">
+        <v>9.43</v>
       </c>
     </row>
     <row r="21">
@@ -5443,16 +5551,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>109.8342</v>
+        <v>110.1175</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>166866.5968578</v>
+        <v>167297.0029325</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-3133.403142199997</v>
+        <v>-2702.997067499993</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.01843178318941175</v>
+        <v>-0.01589998274999996</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -5552,6 +5660,9 @@
       </c>
       <c r="AP21" s="3" t="n">
         <v>109.8342</v>
+      </c>
+      <c r="AQ21" s="3" t="n">
+        <v>110.1175</v>
       </c>
     </row>
     <row r="22">
@@ -5577,16 +5688,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>44.969</v>
+        <v>45.445</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>69003.13174</v>
+        <v>69733.5347</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>9003.131739999997</v>
+        <v>9733.534700000004</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1500521956666666</v>
+        <v>0.1622255783333334</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -5680,6 +5791,9 @@
       </c>
       <c r="AP22" s="3" t="n">
         <v>44.969</v>
+      </c>
+      <c r="AQ22" s="3" t="n">
+        <v>45.445</v>
       </c>
     </row>
     <row r="23">
@@ -5705,16 +5819,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>62.3803</v>
+        <v>62.4481</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>169454.0264001</v>
+        <v>169638.2028627</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>19454.0264001</v>
+        <v>19638.20286270001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.129693509334</v>
+        <v>0.1309213524180001</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -5814,6 +5928,9 @@
       </c>
       <c r="AP23" s="3" t="n">
         <v>62.3803</v>
+      </c>
+      <c r="AQ23" s="3" t="n">
+        <v>62.4481</v>
       </c>
     </row>
     <row r="24">
@@ -5839,16 +5956,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>28.4706</v>
+        <v>28.4686</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>103444.6794516</v>
+        <v>103437.4126796</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>3444.679451600008</v>
+        <v>3437.412679599991</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.03444679451600008</v>
+        <v>0.03437412679599991</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -5942,6 +6059,9 @@
       </c>
       <c r="AP24" s="3" t="n">
         <v>28.4706</v>
+      </c>
+      <c r="AQ24" s="3" t="n">
+        <v>28.4686</v>
       </c>
     </row>
     <row r="25">
@@ -5967,16 +6087,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.56</v>
+        <v>11.6532</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>189834.55144</v>
+        <v>191365.0514568</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-10165.44855999999</v>
+        <v>-8634.948543200007</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.05082724279999995</v>
+        <v>-0.04317474271600004</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -6073,6 +6193,9 @@
       </c>
       <c r="AP25" s="3" t="n">
         <v>11.56</v>
+      </c>
+      <c r="AQ25" s="3" t="n">
+        <v>11.6532</v>
       </c>
     </row>
     <row r="26">
@@ -6098,16 +6221,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>8.985300000000001</v>
+        <v>9.1904</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>107299.8917895</v>
+        <v>109749.137536</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>-2700.108210499995</v>
+        <v>-250.8624639999907</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>-0.02454643827727268</v>
+        <v>-0.00228056785454537</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -6204,6 +6327,9 @@
       </c>
       <c r="AP26" s="3" t="n">
         <v>8.985300000000001</v>
+      </c>
+      <c r="AQ26" s="3" t="n">
+        <v>9.1904</v>
       </c>
     </row>
     <row r="27">
@@ -6229,16 +6355,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>64.0227</v>
+        <v>64.2837</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>103131.606522</v>
+        <v>103552.040982</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-6868.393478000013</v>
+        <v>-6447.959018000009</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.06243994070909102</v>
+        <v>-0.05861780925454553</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -6338,6 +6464,9 @@
       </c>
       <c r="AP27" s="3" t="n">
         <v>64.0227</v>
+      </c>
+      <c r="AQ27" s="3" t="n">
+        <v>64.2837</v>
       </c>
     </row>
     <row r="28">
@@ -6363,16 +6492,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>107.7604</v>
+        <v>108.2352</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>356326.6809828</v>
+        <v>357896.6817264</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-23673.31901719997</v>
+        <v>-22103.31827359996</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.06229820793999993</v>
+        <v>-0.05816662703578936</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -6472,6 +6601,9 @@
       </c>
       <c r="AP28" s="3" t="n">
         <v>107.7604</v>
+      </c>
+      <c r="AQ28" s="3" t="n">
+        <v>108.2352</v>
       </c>
     </row>
     <row r="29">
@@ -6497,16 +6629,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.966</v>
+        <v>11.9672</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>114917.910098</v>
+        <v>114929.4345416</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>14917.91009799999</v>
+        <v>14929.4345416</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.1491791009799999</v>
+        <v>0.149294345416</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -6600,6 +6732,9 @@
       </c>
       <c r="AP29" s="3" t="n">
         <v>11.966</v>
+      </c>
+      <c r="AQ29" s="3" t="n">
+        <v>11.9672</v>
       </c>
     </row>
     <row r="30">
@@ -6625,16 +6760,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>15.8643</v>
+        <v>16.0338</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>117330.1576623</v>
+        <v>118583.7561018</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>17330.1576623</v>
+        <v>18583.7561018</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.173301576623</v>
+        <v>0.185837561018</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -6728,6 +6863,9 @@
       </c>
       <c r="AP30" s="3" t="n">
         <v>15.8643</v>
+      </c>
+      <c r="AQ30" s="3" t="n">
+        <v>16.0338</v>
       </c>
     </row>
     <row r="31">
@@ -6753,16 +6891,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>414.7285</v>
+        <v>416.9249</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>110350.95928</v>
+        <v>110935.377392</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>10350.95928</v>
+        <v>10935.37739199999</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.1035095928</v>
+        <v>0.10935377392</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -6859,6 +6997,9 @@
       </c>
       <c r="AP31" s="3" t="n">
         <v>414.7285</v>
+      </c>
+      <c r="AQ31" s="3" t="n">
+        <v>416.9249</v>
       </c>
     </row>
     <row r="32">
@@ -6884,16 +7025,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.33</v>
+        <v>10.36</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>218375.7868</v>
+        <v>219009.9856</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>18375.7868</v>
+        <v>19009.98559999999</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.09187893400000001</v>
+        <v>0.09504992799999992</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -6993,6 +7134,9 @@
       </c>
       <c r="AP32" s="3" t="n">
         <v>10.33</v>
+      </c>
+      <c r="AQ32" s="3" t="n">
+        <v>10.36</v>
       </c>
     </row>
     <row r="33">
@@ -7018,16 +7162,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>18.29</v>
+        <v>18.32</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>65544.77559999999</v>
+        <v>65652.28479999999</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>5544.775599999994</v>
+        <v>5652.284799999994</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.09241292666666656</v>
+        <v>0.09420474666666656</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -7121,6 +7265,9 @@
       </c>
       <c r="AP33" s="3" t="n">
         <v>18.29</v>
+      </c>
+      <c r="AQ33" s="3" t="n">
+        <v>18.32</v>
       </c>
     </row>
     <row r="34">
@@ -7146,16 +7293,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>210.1009</v>
+        <v>212.2212</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>73856.97947789999</v>
+        <v>74602.3306572</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-6143.020522100007</v>
+        <v>-5397.6693428</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.07678775652625008</v>
+        <v>-0.067470866785</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -7252,6 +7399,9 @@
       </c>
       <c r="AP34" s="3" t="n">
         <v>210.1009</v>
+      </c>
+      <c r="AQ34" s="3" t="n">
+        <v>212.2212</v>
       </c>
     </row>
     <row r="35">
@@ -7277,16 +7427,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>14.64</v>
+        <v>14.62</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>104462.59272</v>
+        <v>104319.88426</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>4462.592720000001</v>
+        <v>4319.884259999992</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.04462592720000001</v>
+        <v>0.04319884259999992</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -7383,6 +7533,9 @@
       </c>
       <c r="AP35" s="3" t="n">
         <v>14.64</v>
+      </c>
+      <c r="AQ35" s="3" t="n">
+        <v>14.62</v>
       </c>
     </row>
     <row r="36">
@@ -7408,16 +7561,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>354.4978</v>
+        <v>354.8719</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>165091.7524468</v>
+        <v>165265.9730614</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>15091.7524468</v>
+        <v>15265.9730614</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1006116829786667</v>
+        <v>0.1017731537426667</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -7514,6 +7667,9 @@
       </c>
       <c r="AP36" s="3" t="n">
         <v>354.4978</v>
+      </c>
+      <c r="AQ36" s="3" t="n">
+        <v>354.8719</v>
       </c>
     </row>
     <row r="37">
@@ -7539,16 +7695,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>15.837</v>
+        <v>15.789</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>59592.873093</v>
+        <v>59412.254421</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>9592.873093000002</v>
+        <v>9412.254420999998</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.1918574618600001</v>
+        <v>0.18824508842</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -7645,6 +7801,9 @@
       </c>
       <c r="AP37" s="3" t="n">
         <v>15.837</v>
+      </c>
+      <c r="AQ37" s="3" t="n">
+        <v>15.789</v>
       </c>
     </row>
     <row r="38">
@@ -7670,16 +7829,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>14.1626</v>
+        <v>14.2243</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>84699.1743732</v>
+        <v>85068.1701126</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>4699.174373200003</v>
+        <v>5068.170112599997</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.05873967966500004</v>
+        <v>0.06335212640749996</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -7773,6 +7932,9 @@
       </c>
       <c r="AP38" s="3" t="n">
         <v>14.1626</v>
+      </c>
+      <c r="AQ38" s="3" t="n">
+        <v>14.2243</v>
       </c>
     </row>
     <row r="39">
@@ -7798,16 +7960,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1018.0503</v>
+        <v>1018.1888</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50781.3670143</v>
+        <v>50788.2755328</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>781.3670142999981</v>
+        <v>788.2755327999985</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.01562734028599996</v>
+        <v>0.01576551065599997</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -7901,6 +8063,9 @@
       </c>
       <c r="AP39" s="3" t="n">
         <v>1018.0503</v>
+      </c>
+      <c r="AQ39" s="3" t="n">
+        <v>1018.1888</v>
       </c>
     </row>
     <row r="40">
@@ -7926,16 +8091,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>20.9785</v>
+        <v>21.0495</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>105753.1849195</v>
+        <v>106111.0978365</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>5753.184919499996</v>
+        <v>6111.09783649999</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.05753184919499996</v>
+        <v>0.0611109783649999</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -8032,6 +8197,9 @@
       </c>
       <c r="AP40" s="3" t="n">
         <v>20.9785</v>
+      </c>
+      <c r="AQ40" s="3" t="n">
+        <v>21.0495</v>
       </c>
     </row>
     <row r="41">
@@ -8044,13 +8212,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4897378.0183038</v>
+        <v>4916306.1372329</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>427378.0183038</v>
+        <v>446306.1372329</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.09561029492255034</v>
+        <v>0.09984477343017897</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-06-18
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -484,8 +484,8 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-17 07:07 IST</t>
+          <t>Generated: 2026-06-18 06:50 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4916306.1372329</v>
+        <v>4933199.4012336</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>446306.1372328997</v>
+        <v>463199.4012336005</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.09984477343017889</v>
+        <v>0.1036240271216108</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>555423.002784729</v>
+        <v>557826.4984207153</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-35359.01721527101</v>
+        <v>-32955.52157928469</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.05985120741364305</v>
+        <v>-0.05578287839444519</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5471729.140017629</v>
+        <v>5491025.899654316</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>410947.1200176291</v>
+        <v>430243.8796543162</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.08120229608656987</v>
+        <v>0.08501529565075325</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-06-17</t>
+          <t>Last snapshot: 2026-06-18</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP19"/>
+  <dimension ref="A1:AQ19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -661,6 +661,7 @@
     <col width="21" customWidth="1" min="40" max="40"/>
     <col width="21" customWidth="1" min="41" max="41"/>
     <col width="21" customWidth="1" min="42" max="42"/>
+    <col width="21" customWidth="1" min="43" max="43"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -874,6 +875,11 @@
           <t>2026-06-17</t>
         </is>
       </c>
+      <c r="AQ1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -893,13 +899,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>559.4500122070312</v>
+        <v>557.5999755859375</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>44756.0009765625</v>
+        <v>44607.998046875</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>938.490976562498</v>
+        <v>790.488046874998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1005,6 +1011,9 @@
       </c>
       <c r="AP2" s="3" t="n">
         <v>559.4500122070312</v>
+      </c>
+      <c r="AQ2" s="3" t="n">
+        <v>557.5999755859375</v>
       </c>
     </row>
     <row r="3">
@@ -1052,13 +1061,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1555.599975585938</v>
+        <v>1571.099975585938</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>31111.99951171875</v>
+        <v>31421.99951171875</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-992.5804882812517</v>
+        <v>-682.5804882812517</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1164,6 +1173,9 @@
       </c>
       <c r="AP4" s="3" t="n">
         <v>1555.599975585938</v>
+      </c>
+      <c r="AQ4" s="3" t="n">
+        <v>1571.099975585938</v>
       </c>
     </row>
     <row r="5">
@@ -1184,13 +1196,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>659.4500122070312</v>
+        <v>659.5</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13189.00024414062</v>
+        <v>13190</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1024.099755859375</v>
+        <v>-1023.1</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1296,6 +1308,9 @@
       </c>
       <c r="AP5" s="3" t="n">
         <v>659.4500122070312</v>
+      </c>
+      <c r="AQ5" s="3" t="n">
+        <v>659.5</v>
       </c>
     </row>
     <row r="6">
@@ -1316,13 +1331,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>383.25</v>
+        <v>395.9500122070312</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15330</v>
+        <v>15838.00048828125</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2172.240000000002</v>
+        <v>-1664.239511718752</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1428,6 +1443,9 @@
       </c>
       <c r="AP6" s="3" t="n">
         <v>383.25</v>
+      </c>
+      <c r="AQ6" s="3" t="n">
+        <v>395.9500122070312</v>
       </c>
     </row>
     <row r="7">
@@ -1448,13 +1466,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>241.6000061035156</v>
+        <v>243.1100006103516</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>24160.00061035156</v>
+        <v>24311.00006103516</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-2273.819389648437</v>
+        <v>-2122.819938964843</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1560,6 +1578,9 @@
       </c>
       <c r="AP7" s="3" t="n">
         <v>241.6000061035156</v>
+      </c>
+      <c r="AQ7" s="3" t="n">
+        <v>243.1100006103516</v>
       </c>
     </row>
     <row r="8">
@@ -1607,13 +1628,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>18.21999931335449</v>
+        <v>18</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>27329.99897003174</v>
+        <v>27000</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-3720.17102996826</v>
+        <v>-4050.169999999998</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1719,6 +1740,9 @@
       </c>
       <c r="AP9" s="3" t="n">
         <v>18.21999931335449</v>
+      </c>
+      <c r="AQ9" s="3" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="10">
@@ -1739,13 +1763,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>415.2000122070312</v>
+        <v>421.5499877929688</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>41520.00122070312</v>
+        <v>42154.99877929688</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-9978.478779296878</v>
+        <v>-9343.481220703128</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1851,6 +1875,9 @@
       </c>
       <c r="AP10" s="3" t="n">
         <v>415.2000122070312</v>
+      </c>
+      <c r="AQ10" s="3" t="n">
+        <v>421.5499877929688</v>
       </c>
     </row>
     <row r="11">
@@ -1871,13 +1898,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>9.020000457763672</v>
+        <v>8.939999580383301</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>9020.000457763672</v>
+        <v>8939.999580383301</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-821.2095422363273</v>
+        <v>-901.2104196166983</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -1983,6 +2010,9 @@
       </c>
       <c r="AP11" s="3" t="n">
         <v>9.020000457763672</v>
+      </c>
+      <c r="AQ11" s="3" t="n">
+        <v>8.939999580383301</v>
       </c>
     </row>
     <row r="12">
@@ -2003,13 +2033,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2633</v>
+        <v>2639.10009765625</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>26330</v>
+        <v>26391.0009765625</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-1393.25</v>
+        <v>-1332.2490234375</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -2115,6 +2145,9 @@
       </c>
       <c r="AP12" s="3" t="n">
         <v>2633</v>
+      </c>
+      <c r="AQ12" s="3" t="n">
+        <v>2639.10009765625</v>
       </c>
     </row>
     <row r="13">
@@ -2135,13 +2168,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>57.93000030517578</v>
+        <v>58.86000061035156</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>34758.00018310547</v>
-      </c>
-      <c r="G13" s="6" t="n">
-        <v>-273.7598168945333</v>
+        <v>35316.00036621094</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>284.2403662109355</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -2247,6 +2280,9 @@
       </c>
       <c r="AP13" s="3" t="n">
         <v>57.93000030517578</v>
+      </c>
+      <c r="AQ13" s="3" t="n">
+        <v>58.86000061035156</v>
       </c>
     </row>
     <row r="14">
@@ -2267,13 +2303,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>729.2000122070312</v>
+        <v>728</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>36460.00061035156</v>
+        <v>36400</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-6002.50938964844</v>
+        <v>-6062.510000000002</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -2379,6 +2415,9 @@
       </c>
       <c r="AP14" s="3" t="n">
         <v>729.2000122070312</v>
+      </c>
+      <c r="AQ14" s="3" t="n">
+        <v>728</v>
       </c>
     </row>
     <row r="15">
@@ -2453,13 +2492,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>592.25</v>
+        <v>609.7000122070312</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>29612.5</v>
+        <v>30485.00061035156</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>7857.970000000001</v>
+        <v>8730.470610351564</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -2565,6 +2604,9 @@
       </c>
       <c r="AP17" s="3" t="n">
         <v>592.25</v>
+      </c>
+      <c r="AQ17" s="3" t="n">
+        <v>609.7000122070312</v>
       </c>
     </row>
     <row r="18">
@@ -2585,13 +2627,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>400.75</v>
+        <v>400</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>40075</v>
+        <v>40000</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-6565.82</v>
+        <v>-6640.82</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -2697,6 +2739,9 @@
       </c>
       <c r="AP18" s="3" t="n">
         <v>400.75</v>
+      </c>
+      <c r="AQ18" s="3" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="19">
@@ -2709,10 +2754,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>555423.002784729</v>
+        <v>557826.4984207153</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-35359.01721527101</v>
+        <v>-32955.52157928468</v>
       </c>
     </row>
   </sheetData>
@@ -2726,7 +2771,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ41"/>
+  <dimension ref="A1:AR41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2772,6 +2817,7 @@
     <col width="13" customWidth="1" min="41" max="41"/>
     <col width="13" customWidth="1" min="42" max="42"/>
     <col width="13" customWidth="1" min="43" max="43"/>
+    <col width="13" customWidth="1" min="44" max="44"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2990,6 +3036,11 @@
           <t>2026-06-17</t>
         </is>
       </c>
+      <c r="AR1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3014,16 +3065,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>57.0887</v>
+        <v>56.6859</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>64081.0381534</v>
+        <v>63628.90240379999</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>14081.0381534</v>
+        <v>13628.90240379999</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.2816207630680001</v>
+        <v>0.2725780480759998</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -3126,6 +3177,9 @@
       </c>
       <c r="AQ2" s="3" t="n">
         <v>57.0887</v>
+      </c>
+      <c r="AR2" s="3" t="n">
+        <v>56.6859</v>
       </c>
     </row>
     <row r="3">
@@ -3151,16 +3205,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.6215</v>
+        <v>25.5243</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>62906.2398795</v>
+        <v>62667.59317590001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>2906.239879500004</v>
+        <v>2667.593175900009</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.04843733132500008</v>
+        <v>0.04445988626500014</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -3257,6 +3311,9 @@
       </c>
       <c r="AQ3" s="3" t="n">
         <v>25.6215</v>
+      </c>
+      <c r="AR3" s="3" t="n">
+        <v>25.5243</v>
       </c>
     </row>
     <row r="4">
@@ -3282,16 +3339,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.41</v>
+        <v>12.37</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>238347.61413</v>
+        <v>237579.37041</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>58347.61413</v>
+        <v>57579.37041</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3241534118333333</v>
+        <v>0.3198853911666667</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -3388,6 +3445,9 @@
       </c>
       <c r="AQ4" s="3" t="n">
         <v>12.41</v>
+      </c>
+      <c r="AR4" s="3" t="n">
+        <v>12.37</v>
       </c>
     </row>
     <row r="5">
@@ -3413,16 +3473,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.488300000000001</v>
+        <v>9.5829</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>174149.0931704</v>
+        <v>175885.3898952</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-35850.90682959999</v>
+        <v>-34114.6101048</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1707186039504761</v>
+        <v>-0.1624505243085714</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -3519,6 +3579,9 @@
       </c>
       <c r="AQ5" s="3" t="n">
         <v>9.488300000000001</v>
+      </c>
+      <c r="AR5" s="3" t="n">
+        <v>9.5829</v>
       </c>
     </row>
     <row r="6">
@@ -3544,16 +3607,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.2281</v>
+        <v>12.3308</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>51712.3536537</v>
+        <v>52146.6695916</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>1712.353653699996</v>
+        <v>2146.669591599995</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.03424707307399993</v>
+        <v>0.04293339183199991</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -3656,6 +3719,9 @@
       </c>
       <c r="AQ6" s="3" t="n">
         <v>12.2281</v>
+      </c>
+      <c r="AR6" s="3" t="n">
+        <v>12.3308</v>
       </c>
     </row>
     <row r="7">
@@ -3681,16 +3747,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>34.2288</v>
+        <v>34.3099</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>75510.101952</v>
+        <v>75689.01179599999</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>15510.101952</v>
+        <v>15689.01179599999</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2585016991999999</v>
+        <v>0.2614835299333332</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -3787,6 +3853,9 @@
       </c>
       <c r="AQ7" s="3" t="n">
         <v>34.2288</v>
+      </c>
+      <c r="AR7" s="3" t="n">
+        <v>34.3099</v>
       </c>
     </row>
     <row r="8">
@@ -3812,16 +3881,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>32.7202</v>
+        <v>32.8508</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>52502.6038786</v>
+        <v>52712.1637244</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>2502.603878599999</v>
+        <v>2712.163724400001</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.05005207757199998</v>
+        <v>0.05424327448800002</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -3924,6 +3993,9 @@
       </c>
       <c r="AQ8" s="3" t="n">
         <v>32.7202</v>
+      </c>
+      <c r="AR8" s="3" t="n">
+        <v>32.8508</v>
       </c>
     </row>
     <row r="9">
@@ -3949,16 +4021,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>43.0981</v>
+        <v>42.004</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>138749.7214533</v>
+        <v>135227.383572</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>38749.72145330001</v>
+        <v>35227.38357199999</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3874972145330001</v>
+        <v>0.3522738357199999</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -4055,6 +4127,9 @@
       </c>
       <c r="AQ9" s="3" t="n">
         <v>43.0981</v>
+      </c>
+      <c r="AR9" s="3" t="n">
+        <v>42.004</v>
       </c>
     </row>
     <row r="10">
@@ -4080,16 +4155,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>47.5456</v>
+        <v>47.3381</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>135346.1101504</v>
+        <v>134755.4284079</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>35346.1101504</v>
+        <v>34755.42840790001</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.353461101504</v>
+        <v>0.3475542840790001</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -4186,6 +4261,9 @@
       </c>
       <c r="AQ10" s="3" t="n">
         <v>47.5456</v>
+      </c>
+      <c r="AR10" s="3" t="n">
+        <v>47.3381</v>
       </c>
     </row>
     <row r="11">
@@ -4211,16 +4289,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>105.4261</v>
+        <v>104.304</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31724.7165859</v>
+        <v>31387.055376</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1724.716585900002</v>
+        <v>1387.055376</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.05749055286333338</v>
+        <v>0.04623517920000001</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -4317,6 +4395,9 @@
       </c>
       <c r="AQ11" s="3" t="n">
         <v>105.4261</v>
+      </c>
+      <c r="AR11" s="3" t="n">
+        <v>104.304</v>
       </c>
     </row>
     <row r="12">
@@ -4342,16 +4423,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>223.292</v>
+        <v>224.28</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>103947.338424</v>
+        <v>104407.27416</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>3947.338424000001</v>
+        <v>4407.274160000001</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.03947338424000001</v>
+        <v>0.04407274160000001</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -4454,6 +4535,9 @@
       </c>
       <c r="AQ12" s="3" t="n">
         <v>223.292</v>
+      </c>
+      <c r="AR12" s="3" t="n">
+        <v>224.28</v>
       </c>
     </row>
     <row r="13">
@@ -4479,16 +4563,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>20.152</v>
+        <v>20.199</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>233513.41596</v>
+        <v>234058.033395</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>33513.41596000001</v>
+        <v>34058.03339500001</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.1675670798000001</v>
+        <v>0.170290166975</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -4591,6 +4675,9 @@
       </c>
       <c r="AQ13" s="3" t="n">
         <v>20.152</v>
+      </c>
+      <c r="AR13" s="3" t="n">
+        <v>20.199</v>
       </c>
     </row>
     <row r="14">
@@ -4616,16 +4703,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>39.8038</v>
+        <v>40.0228</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>143596.4277028</v>
+        <v>144386.4934168</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>43596.42770280002</v>
+        <v>44386.49341679999</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.4359642770280002</v>
+        <v>0.4438649341679999</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -4722,6 +4809,9 @@
       </c>
       <c r="AQ14" s="3" t="n">
         <v>39.8038</v>
+      </c>
+      <c r="AR14" s="3" t="n">
+        <v>40.0228</v>
       </c>
     </row>
     <row r="15">
@@ -4747,16 +4837,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.85</v>
+        <v>11.96</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>115465.77195</v>
+        <v>116537.60612</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>15465.77194999999</v>
+        <v>16537.60612000001</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1546577195</v>
+        <v>0.1653760612000001</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -4859,6 +4949,9 @@
       </c>
       <c r="AQ15" s="3" t="n">
         <v>11.85</v>
+      </c>
+      <c r="AR15" s="3" t="n">
+        <v>11.96</v>
       </c>
     </row>
     <row r="16">
@@ -4884,16 +4977,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.7039</v>
+        <v>24.3754</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>141378.6410192</v>
+        <v>139498.6591712</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>41378.6410192</v>
+        <v>39498.65917119998</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.413786410192</v>
+        <v>0.3949865917119998</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -4990,6 +5083,9 @@
       </c>
       <c r="AQ16" s="3" t="n">
         <v>24.7039</v>
+      </c>
+      <c r="AR16" s="3" t="n">
+        <v>24.3754</v>
       </c>
     </row>
     <row r="17">
@@ -5015,16 +5111,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.8624</v>
+        <v>16.8181</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55748.0555568</v>
+        <v>55601.5972317</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5748.055556799998</v>
+        <v>5601.597231699998</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.114961111136</v>
+        <v>0.112031944634</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -5121,6 +5217,9 @@
       </c>
       <c r="AQ17" s="3" t="n">
         <v>16.8624</v>
+      </c>
+      <c r="AR17" s="3" t="n">
+        <v>16.8181</v>
       </c>
     </row>
     <row r="18">
@@ -5146,16 +5245,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>45</v>
+        <v>44.89</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>84889.62</v>
+        <v>84682.11203999999</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>4889.619999999995</v>
+        <v>4682.112039999993</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.06112024999999994</v>
+        <v>0.05852640049999991</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -5258,6 +5357,9 @@
       </c>
       <c r="AQ18" s="3" t="n">
         <v>45</v>
+      </c>
+      <c r="AR18" s="3" t="n">
+        <v>44.89</v>
       </c>
     </row>
     <row r="19">
@@ -5283,16 +5385,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>15.055</v>
+        <v>14.9529</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>217797.16213</v>
+        <v>216320.1053214</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>67797.16212999998</v>
+        <v>66320.10532139998</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.4519810808666666</v>
+        <v>0.4421340354759999</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -5389,6 +5491,9 @@
       </c>
       <c r="AQ19" s="3" t="n">
         <v>15.055</v>
+      </c>
+      <c r="AR19" s="3" t="n">
+        <v>14.9529</v>
       </c>
     </row>
     <row r="20">
@@ -5414,16 +5519,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.43</v>
+        <v>9.48</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>247592.22229</v>
+        <v>248905.01244</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-2407.777709999995</v>
+        <v>-1094.98755999998</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.009631110839999979</v>
+        <v>-0.004379950239999918</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -5526,6 +5631,9 @@
       </c>
       <c r="AQ20" s="3" t="n">
         <v>9.43</v>
+      </c>
+      <c r="AR20" s="3" t="n">
+        <v>9.48</v>
       </c>
     </row>
     <row r="21">
@@ -5551,16 +5659,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>110.1175</v>
+        <v>110.4811</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>167297.0029325</v>
+        <v>167849.4055049</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-2702.997067499993</v>
+        <v>-2150.594495099998</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.01589998274999996</v>
+        <v>-0.0126505558535294</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -5663,6 +5771,9 @@
       </c>
       <c r="AQ21" s="3" t="n">
         <v>110.1175</v>
+      </c>
+      <c r="AR21" s="3" t="n">
+        <v>110.4811</v>
       </c>
     </row>
     <row r="22">
@@ -5688,16 +5799,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>45.445</v>
+        <v>45.447</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>69733.5347</v>
+        <v>69736.60362000001</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>9733.534700000004</v>
+        <v>9736.603620000009</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1622255783333334</v>
+        <v>0.1622767270000001</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -5794,6 +5905,9 @@
       </c>
       <c r="AQ22" s="3" t="n">
         <v>45.445</v>
+      </c>
+      <c r="AR22" s="3" t="n">
+        <v>45.447</v>
       </c>
     </row>
     <row r="23">
@@ -5819,16 +5933,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>62.4481</v>
+        <v>62.8831</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>169638.2028627</v>
+        <v>170819.8660077</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>19638.20286270001</v>
+        <v>20819.86600770001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.1309213524180001</v>
+        <v>0.1387991067180001</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -5931,6 +6045,9 @@
       </c>
       <c r="AQ23" s="3" t="n">
         <v>62.4481</v>
+      </c>
+      <c r="AR23" s="3" t="n">
+        <v>62.8831</v>
       </c>
     </row>
     <row r="24">
@@ -5956,16 +6073,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>28.4686</v>
+        <v>28.4869</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>103437.4126796</v>
+        <v>103503.9036434</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>3437.412679599991</v>
+        <v>3503.903643400001</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.03437412679599991</v>
+        <v>0.03503903643400001</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -6062,6 +6179,9 @@
       </c>
       <c r="AQ24" s="3" t="n">
         <v>28.4686</v>
+      </c>
+      <c r="AR24" s="3" t="n">
+        <v>28.4869</v>
       </c>
     </row>
     <row r="25">
@@ -6087,16 +6207,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.6532</v>
+        <v>11.7368</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>191365.0514568</v>
+        <v>192737.9034032</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-8634.948543200007</v>
+        <v>-7262.096596799995</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.04317474271600004</v>
+        <v>-0.03631048298399997</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -6196,6 +6316,9 @@
       </c>
       <c r="AQ25" s="3" t="n">
         <v>11.6532</v>
+      </c>
+      <c r="AR25" s="3" t="n">
+        <v>11.7368</v>
       </c>
     </row>
     <row r="26">
@@ -6221,16 +6344,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>9.1904</v>
+        <v>9.2788</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>109749.137536</v>
-      </c>
-      <c r="H26" s="6" t="n">
-        <v>-250.8624639999907</v>
-      </c>
-      <c r="I26" s="13" t="n">
-        <v>-0.00228056785454537</v>
+        <v>110804.785142</v>
+      </c>
+      <c r="H26" s="4" t="n">
+        <v>804.7851420000079</v>
+      </c>
+      <c r="I26" s="12" t="n">
+        <v>0.007316228563636435</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -6330,6 +6453,9 @@
       </c>
       <c r="AQ26" s="3" t="n">
         <v>9.1904</v>
+      </c>
+      <c r="AR26" s="3" t="n">
+        <v>9.2788</v>
       </c>
     </row>
     <row r="27">
@@ -6355,16 +6481,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>64.2837</v>
+        <v>64.8507</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>103552.040982</v>
+        <v>104465.398602</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-6447.959018000009</v>
+        <v>-5534.601397999999</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.05861780925454553</v>
+        <v>-0.05031455816363636</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -6467,6 +6593,9 @@
       </c>
       <c r="AQ27" s="3" t="n">
         <v>64.2837</v>
+      </c>
+      <c r="AR27" s="3" t="n">
+        <v>64.8507</v>
       </c>
     </row>
     <row r="28">
@@ -6492,16 +6621,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>108.2352</v>
+        <v>108.9451</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>357896.6817264</v>
+        <v>360244.0775307</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-22103.31827359996</v>
+        <v>-19755.92246929999</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.05816662703578936</v>
+        <v>-0.05198926965605259</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -6604,6 +6733,9 @@
       </c>
       <c r="AQ28" s="3" t="n">
         <v>108.2352</v>
+      </c>
+      <c r="AR28" s="3" t="n">
+        <v>108.9451</v>
       </c>
     </row>
     <row r="29">
@@ -6629,16 +6761,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>11.9672</v>
+        <v>12.4346</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>114929.4345416</v>
+        <v>119418.2053238</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>14929.4345416</v>
+        <v>19418.20532379999</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.149294345416</v>
+        <v>0.1941820532379999</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -6735,6 +6867,9 @@
       </c>
       <c r="AQ29" s="3" t="n">
         <v>11.9672</v>
+      </c>
+      <c r="AR29" s="3" t="n">
+        <v>12.4346</v>
       </c>
     </row>
     <row r="30">
@@ -6760,16 +6895,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>16.0338</v>
+        <v>16.1495</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>118583.7561018</v>
+        <v>119439.4572195</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>18583.7561018</v>
+        <v>19439.45721949999</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.185837561018</v>
+        <v>0.1943945721949999</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -6866,6 +7001,9 @@
       </c>
       <c r="AQ30" s="3" t="n">
         <v>16.0338</v>
+      </c>
+      <c r="AR30" s="3" t="n">
+        <v>16.1495</v>
       </c>
     </row>
     <row r="31">
@@ -6891,16 +7029,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>416.9249</v>
+        <v>420.3835</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>110935.377392</v>
+        <v>111855.64168</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>10935.37739199999</v>
+        <v>11855.64168</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.10935377392</v>
+        <v>0.1185564168</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -7000,6 +7138,9 @@
       </c>
       <c r="AQ31" s="3" t="n">
         <v>416.9249</v>
+      </c>
+      <c r="AR31" s="3" t="n">
+        <v>420.3835</v>
       </c>
     </row>
     <row r="32">
@@ -7025,16 +7166,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.36</v>
+        <v>10.46</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>219009.9856</v>
+        <v>221123.9816</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>19009.98559999999</v>
+        <v>21123.9816</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.09504992799999992</v>
+        <v>0.105619908</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -7137,6 +7278,9 @@
       </c>
       <c r="AQ32" s="3" t="n">
         <v>10.36</v>
+      </c>
+      <c r="AR32" s="3" t="n">
+        <v>10.46</v>
       </c>
     </row>
     <row r="33">
@@ -7162,16 +7306,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>18.32</v>
+        <v>18.57</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>65652.28479999999</v>
+        <v>66548.1948</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>5652.284799999994</v>
+        <v>6548.194799999997</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.09420474666666656</v>
+        <v>0.10913658</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -7268,6 +7412,9 @@
       </c>
       <c r="AQ33" s="3" t="n">
         <v>18.32</v>
+      </c>
+      <c r="AR33" s="3" t="n">
+        <v>18.57</v>
       </c>
     </row>
     <row r="34">
@@ -7293,16 +7440,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>212.2212</v>
+        <v>213.7101</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>74602.3306572</v>
+        <v>75125.72516310001</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-5397.6693428</v>
+        <v>-4874.274836899989</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.067470866785</v>
+        <v>-0.06092843546124987</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -7402,6 +7549,9 @@
       </c>
       <c r="AQ34" s="3" t="n">
         <v>212.2212</v>
+      </c>
+      <c r="AR34" s="3" t="n">
+        <v>213.7101</v>
       </c>
     </row>
     <row r="35">
@@ -7427,16 +7577,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>14.62</v>
+        <v>14.79</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>104319.88426</v>
+        <v>105532.90617</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>4319.884259999992</v>
+        <v>5532.906169999987</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.04319884259999992</v>
+        <v>0.05532906169999988</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -7536,6 +7686,9 @@
       </c>
       <c r="AQ35" s="3" t="n">
         <v>14.62</v>
+      </c>
+      <c r="AR35" s="3" t="n">
+        <v>14.79</v>
       </c>
     </row>
     <row r="36">
@@ -7561,16 +7714,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>354.8719</v>
+        <v>355.3036</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>165265.9730614</v>
+        <v>165467.0183416</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>15265.9730614</v>
+        <v>15467.01834160002</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1017731537426667</v>
+        <v>0.1031134556106668</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -7670,6 +7823,9 @@
       </c>
       <c r="AQ36" s="3" t="n">
         <v>354.8719</v>
+      </c>
+      <c r="AR36" s="3" t="n">
+        <v>355.3036</v>
       </c>
     </row>
     <row r="37">
@@ -7695,16 +7851,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>15.789</v>
+        <v>15.813</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>59412.254421</v>
+        <v>59502.563757</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>9412.254420999998</v>
+        <v>9502.563757000004</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.18824508842</v>
+        <v>0.1900512751400001</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -7804,6 +7960,9 @@
       </c>
       <c r="AQ37" s="3" t="n">
         <v>15.789</v>
+      </c>
+      <c r="AR37" s="3" t="n">
+        <v>15.813</v>
       </c>
     </row>
     <row r="38">
@@ -7829,16 +7988,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>14.2243</v>
+        <v>14.2923</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>85068.1701126</v>
+        <v>85474.84288859999</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>5068.170112599997</v>
+        <v>5474.842888599989</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.06335212640749996</v>
+        <v>0.06843553610749986</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -7935,6 +8094,9 @@
       </c>
       <c r="AQ38" s="3" t="n">
         <v>14.2243</v>
+      </c>
+      <c r="AR38" s="3" t="n">
+        <v>14.2923</v>
       </c>
     </row>
     <row r="39">
@@ -7960,16 +8122,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1018.1888</v>
+        <v>1018.7854</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50788.2755328</v>
+        <v>50818.0345374</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>788.2755327999985</v>
+        <v>818.0345374000026</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.01576551065599997</v>
+        <v>0.01636069074800005</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -8066,6 +8228,9 @@
       </c>
       <c r="AQ39" s="3" t="n">
         <v>1018.1888</v>
+      </c>
+      <c r="AR39" s="3" t="n">
+        <v>1018.7854</v>
       </c>
     </row>
     <row r="40">
@@ -8091,16 +8256,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>21.0495</v>
+        <v>21.1574</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>106111.0978365</v>
+        <v>106655.0246498</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>6111.09783649999</v>
+        <v>6655.024649799991</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.0611109783649999</v>
+        <v>0.06655024649799991</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -8200,6 +8365,9 @@
       </c>
       <c r="AQ40" s="3" t="n">
         <v>21.0495</v>
+      </c>
+      <c r="AR40" s="3" t="n">
+        <v>21.1574</v>
       </c>
     </row>
     <row r="41">
@@ -8212,13 +8380,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4916306.1372329</v>
+        <v>4933199.4012336</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>446306.1372329</v>
+        <v>463199.4012336</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.09984477343017897</v>
+        <v>0.1036240271216107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-06-19
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -485,7 +485,7 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-18 06:50 IST</t>
+          <t>Generated: 2026-06-19 07:04 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4933199.4012336</v>
+        <v>4951334.5140237</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>463199.4012336005</v>
+        <v>481334.5140236998</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1036240271216108</v>
+        <v>0.107681099334161</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>557826.4984207153</v>
+        <v>557439.0023498535</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-32955.52157928469</v>
+        <v>-33343.0176501465</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.05578287839444519</v>
+        <v>-0.05643878202343819</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5491025.899654316</v>
+        <v>5508773.516373553</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>430243.8796543162</v>
+        <v>447991.4963735538</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.08501529565075325</v>
+        <v>0.08852218779688792</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-06-18</t>
+          <t>Last snapshot: 2026-06-19</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ19"/>
+  <dimension ref="A1:AR19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -662,6 +662,7 @@
     <col width="21" customWidth="1" min="41" max="41"/>
     <col width="21" customWidth="1" min="42" max="42"/>
     <col width="21" customWidth="1" min="43" max="43"/>
+    <col width="21" customWidth="1" min="44" max="44"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -880,6 +881,11 @@
           <t>2026-06-18</t>
         </is>
       </c>
+      <c r="AR1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -899,13 +905,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>557.5999755859375</v>
+        <v>549.9500122070312</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>44607.998046875</v>
+        <v>43996.0009765625</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>790.488046874998</v>
+        <v>178.490976562498</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1014,6 +1020,9 @@
       </c>
       <c r="AQ2" s="3" t="n">
         <v>557.5999755859375</v>
+      </c>
+      <c r="AR2" s="3" t="n">
+        <v>549.9500122070312</v>
       </c>
     </row>
     <row r="3">
@@ -1061,13 +1070,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1571.099975585938</v>
+        <v>1544.300048828125</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>31421.99951171875</v>
+        <v>30886.0009765625</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-682.5804882812517</v>
+        <v>-1218.579023437502</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1176,6 +1185,9 @@
       </c>
       <c r="AQ4" s="3" t="n">
         <v>1571.099975585938</v>
+      </c>
+      <c r="AR4" s="3" t="n">
+        <v>1544.300048828125</v>
       </c>
     </row>
     <row r="5">
@@ -1196,13 +1208,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>659.5</v>
+        <v>659</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13190</v>
+        <v>13180</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1023.1</v>
+        <v>-1033.1</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1311,6 +1323,9 @@
       </c>
       <c r="AQ5" s="3" t="n">
         <v>659.5</v>
+      </c>
+      <c r="AR5" s="3" t="n">
+        <v>659</v>
       </c>
     </row>
     <row r="6">
@@ -1331,13 +1346,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>395.9500122070312</v>
+        <v>390.25</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15838.00048828125</v>
+        <v>15610</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-1664.239511718752</v>
+        <v>-1892.240000000002</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1446,6 +1461,9 @@
       </c>
       <c r="AQ6" s="3" t="n">
         <v>395.9500122070312</v>
+      </c>
+      <c r="AR6" s="3" t="n">
+        <v>390.25</v>
       </c>
     </row>
     <row r="7">
@@ -1466,13 +1484,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>243.1100006103516</v>
+        <v>251.6600036621094</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>24311.00006103516</v>
+        <v>25166.00036621094</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-2122.819938964843</v>
+        <v>-1267.819633789062</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1581,6 +1599,9 @@
       </c>
       <c r="AQ7" s="3" t="n">
         <v>243.1100006103516</v>
+      </c>
+      <c r="AR7" s="3" t="n">
+        <v>251.6600036621094</v>
       </c>
     </row>
     <row r="8">
@@ -1628,13 +1649,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>18</v>
+        <v>18.06999969482422</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>27000</v>
+        <v>27104.99954223633</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-4050.169999999998</v>
+        <v>-3945.17045776367</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1743,6 +1764,9 @@
       </c>
       <c r="AQ9" s="3" t="n">
         <v>18</v>
+      </c>
+      <c r="AR9" s="3" t="n">
+        <v>18.06999969482422</v>
       </c>
     </row>
     <row r="10">
@@ -1763,13 +1787,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>421.5499877929688</v>
+        <v>418.6499938964844</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>42154.99877929688</v>
+        <v>41864.99938964844</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-9343.481220703128</v>
+        <v>-9633.480610351566</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1878,6 +1902,9 @@
       </c>
       <c r="AQ10" s="3" t="n">
         <v>421.5499877929688</v>
+      </c>
+      <c r="AR10" s="3" t="n">
+        <v>418.6499938964844</v>
       </c>
     </row>
     <row r="11">
@@ -1898,13 +1925,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>8.939999580383301</v>
+        <v>8.930000305175781</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>8939.999580383301</v>
+        <v>8930.000305175781</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-901.2104196166983</v>
+        <v>-911.2096948242179</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -2013,6 +2040,9 @@
       </c>
       <c r="AQ11" s="3" t="n">
         <v>8.939999580383301</v>
+      </c>
+      <c r="AR11" s="3" t="n">
+        <v>8.930000305175781</v>
       </c>
     </row>
     <row r="12">
@@ -2033,13 +2063,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2639.10009765625</v>
+        <v>2607.60009765625</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>26391.0009765625</v>
+        <v>26076.0009765625</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-1332.2490234375</v>
+        <v>-1647.2490234375</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -2148,6 +2178,9 @@
       </c>
       <c r="AQ12" s="3" t="n">
         <v>2639.10009765625</v>
+      </c>
+      <c r="AR12" s="3" t="n">
+        <v>2607.60009765625</v>
       </c>
     </row>
     <row r="13">
@@ -2168,13 +2201,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>58.86000061035156</v>
+        <v>59.81999969482422</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>35316.00036621094</v>
+        <v>35891.99981689453</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>284.2403662109355</v>
+        <v>860.2398168945292</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -2283,6 +2316,9 @@
       </c>
       <c r="AQ13" s="3" t="n">
         <v>58.86000061035156</v>
+      </c>
+      <c r="AR13" s="3" t="n">
+        <v>59.81999969482422</v>
       </c>
     </row>
     <row r="14">
@@ -2303,13 +2339,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>728</v>
+        <v>725.5</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>36400</v>
+        <v>36275</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-6062.510000000002</v>
+        <v>-6187.510000000002</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -2418,6 +2454,9 @@
       </c>
       <c r="AQ14" s="3" t="n">
         <v>728</v>
+      </c>
+      <c r="AR14" s="3" t="n">
+        <v>725.5</v>
       </c>
     </row>
     <row r="15">
@@ -2492,13 +2531,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>609.7000122070312</v>
+        <v>611.25</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>30485.00061035156</v>
+        <v>30562.5</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>8730.470610351564</v>
+        <v>8807.970000000001</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -2607,6 +2646,9 @@
       </c>
       <c r="AQ17" s="3" t="n">
         <v>609.7000122070312</v>
+      </c>
+      <c r="AR17" s="3" t="n">
+        <v>611.25</v>
       </c>
     </row>
     <row r="18">
@@ -2627,13 +2669,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>400</v>
+        <v>401.25</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>40000</v>
+        <v>40125</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-6640.82</v>
+        <v>-6515.82</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -2742,6 +2784,9 @@
       </c>
       <c r="AQ18" s="3" t="n">
         <v>400</v>
+      </c>
+      <c r="AR18" s="3" t="n">
+        <v>401.25</v>
       </c>
     </row>
     <row r="19">
@@ -2754,10 +2799,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>557826.4984207153</v>
+        <v>557439.0023498535</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-32955.52157928468</v>
+        <v>-33343.0176501465</v>
       </c>
     </row>
   </sheetData>
@@ -2771,7 +2816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR41"/>
+  <dimension ref="A1:AS41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2818,6 +2863,7 @@
     <col width="13" customWidth="1" min="42" max="42"/>
     <col width="13" customWidth="1" min="43" max="43"/>
     <col width="13" customWidth="1" min="44" max="44"/>
+    <col width="13" customWidth="1" min="45" max="45"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3041,6 +3087,11 @@
           <t>2026-06-18</t>
         </is>
       </c>
+      <c r="AS1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3065,16 +3116,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.6859</v>
+        <v>57.1227</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>63628.90240379999</v>
+        <v>64119.2025414</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>13628.90240379999</v>
+        <v>14119.2025414</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.2725780480759998</v>
+        <v>0.2823840508280001</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -3180,6 +3231,9 @@
       </c>
       <c r="AR2" s="3" t="n">
         <v>56.6859</v>
+      </c>
+      <c r="AS2" s="3" t="n">
+        <v>57.1227</v>
       </c>
     </row>
     <row r="3">
@@ -3205,16 +3259,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.5243</v>
+        <v>25.31</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>62667.59317590001</v>
+        <v>62141.44103</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>2667.593175900009</v>
+        <v>2141.441030000002</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.04445988626500014</v>
+        <v>0.03569068383333336</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -3314,6 +3368,9 @@
       </c>
       <c r="AR3" s="3" t="n">
         <v>25.5243</v>
+      </c>
+      <c r="AS3" s="3" t="n">
+        <v>25.31</v>
       </c>
     </row>
     <row r="4">
@@ -3449,6 +3506,9 @@
       <c r="AR4" s="3" t="n">
         <v>12.37</v>
       </c>
+      <c r="AS4" s="3" t="n">
+        <v>12.37</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3473,16 +3533,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.5829</v>
+        <v>9.5838</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>175885.3898952</v>
+        <v>175901.9085744</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-34114.6101048</v>
+        <v>-34098.0914256</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1624505243085714</v>
+        <v>-0.1623718639314286</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -3582,6 +3642,9 @@
       </c>
       <c r="AR5" s="3" t="n">
         <v>9.5829</v>
+      </c>
+      <c r="AS5" s="3" t="n">
+        <v>9.5838</v>
       </c>
     </row>
     <row r="6">
@@ -3607,16 +3670,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.3308</v>
+        <v>12.3967</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>52146.6695916</v>
+        <v>52425.3591759</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>2146.669591599995</v>
+        <v>2425.359175899997</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.04293339183199991</v>
+        <v>0.04850718351799994</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -3722,6 +3785,9 @@
       </c>
       <c r="AR6" s="3" t="n">
         <v>12.3308</v>
+      </c>
+      <c r="AS6" s="3" t="n">
+        <v>12.3967</v>
       </c>
     </row>
     <row r="7">
@@ -3747,16 +3813,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>34.3099</v>
+        <v>33.9637</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>75689.01179599999</v>
+        <v>74925.280748</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>15689.01179599999</v>
+        <v>14925.280748</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2614835299333332</v>
+        <v>0.2487546791333334</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -3856,6 +3922,9 @@
       </c>
       <c r="AR7" s="3" t="n">
         <v>34.3099</v>
+      </c>
+      <c r="AS7" s="3" t="n">
+        <v>33.9637</v>
       </c>
     </row>
     <row r="8">
@@ -3881,16 +3950,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>32.8508</v>
+        <v>33.0896</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>52712.1637244</v>
+        <v>53095.3405328</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>2712.163724400001</v>
+        <v>3095.340532800001</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.05424327448800002</v>
+        <v>0.06190681065600002</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -3996,6 +4065,9 @@
       </c>
       <c r="AR8" s="3" t="n">
         <v>32.8508</v>
+      </c>
+      <c r="AS8" s="3" t="n">
+        <v>33.0896</v>
       </c>
     </row>
     <row r="9">
@@ -4021,16 +4093,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>42.004</v>
+        <v>42.1536</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>135227.383572</v>
+        <v>135709.0047648</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>35227.38357199999</v>
+        <v>35709.00476479999</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3522738357199999</v>
+        <v>0.3570900476479999</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -4130,6 +4202,9 @@
       </c>
       <c r="AR9" s="3" t="n">
         <v>42.004</v>
+      </c>
+      <c r="AS9" s="3" t="n">
+        <v>42.1536</v>
       </c>
     </row>
     <row r="10">
@@ -4155,16 +4230,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>47.3381</v>
+        <v>47.2455</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>134755.4284079</v>
+        <v>134491.8277845</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>34755.42840790001</v>
+        <v>34491.8277845</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3475542840790001</v>
+        <v>0.344918277845</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -4264,6 +4339,9 @@
       </c>
       <c r="AR10" s="3" t="n">
         <v>47.3381</v>
+      </c>
+      <c r="AS10" s="3" t="n">
+        <v>47.2455</v>
       </c>
     </row>
     <row r="11">
@@ -4289,16 +4367,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>104.304</v>
+        <v>105.991</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31387.055376</v>
+        <v>31894.705729</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1387.055376</v>
+        <v>1894.705728999998</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.04623517920000001</v>
+        <v>0.06315685763333324</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -4398,6 +4476,9 @@
       </c>
       <c r="AR11" s="3" t="n">
         <v>104.304</v>
+      </c>
+      <c r="AS11" s="3" t="n">
+        <v>105.991</v>
       </c>
     </row>
     <row r="12">
@@ -4423,16 +4504,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>224.28</v>
+        <v>225.63</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>104407.27416</v>
+        <v>105035.72886</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>4407.274160000001</v>
+        <v>5035.728860000003</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.04407274160000001</v>
+        <v>0.05035728860000003</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -4538,6 +4619,9 @@
       </c>
       <c r="AR12" s="3" t="n">
         <v>224.28</v>
+      </c>
+      <c r="AS12" s="3" t="n">
+        <v>225.63</v>
       </c>
     </row>
     <row r="13">
@@ -4563,16 +4647,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>20.199</v>
+        <v>20.414</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>234058.033395</v>
+        <v>236549.36847</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>34058.03339500001</v>
+        <v>36549.36847000002</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.170290166975</v>
+        <v>0.1827468423500001</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -4678,6 +4762,9 @@
       </c>
       <c r="AR13" s="3" t="n">
         <v>20.199</v>
+      </c>
+      <c r="AS13" s="3" t="n">
+        <v>20.414</v>
       </c>
     </row>
     <row r="14">
@@ -4703,16 +4790,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>40.0228</v>
+        <v>40.1296</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>144386.4934168</v>
+        <v>144771.7857376</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>44386.49341679999</v>
+        <v>44771.78573760003</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.4438649341679999</v>
+        <v>0.4477178573760003</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -4812,6 +4899,9 @@
       </c>
       <c r="AR14" s="3" t="n">
         <v>40.0228</v>
+      </c>
+      <c r="AS14" s="3" t="n">
+        <v>40.1296</v>
       </c>
     </row>
     <row r="15">
@@ -4837,16 +4927,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.96</v>
+        <v>11.99</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>116537.60612</v>
+        <v>116829.92453</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>16537.60612000001</v>
+        <v>16829.92453</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1653760612000001</v>
+        <v>0.1682992453</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -4952,6 +5042,9 @@
       </c>
       <c r="AR15" s="3" t="n">
         <v>11.96</v>
+      </c>
+      <c r="AS15" s="3" t="n">
+        <v>11.99</v>
       </c>
     </row>
     <row r="16">
@@ -4977,16 +5070,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.3754</v>
+        <v>24.9541</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>139498.6591712</v>
+        <v>142810.5176048</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>39498.65917119998</v>
+        <v>42810.5176048</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.3949865917119998</v>
+        <v>0.428105176048</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -5086,6 +5179,9 @@
       </c>
       <c r="AR16" s="3" t="n">
         <v>24.3754</v>
+      </c>
+      <c r="AS16" s="3" t="n">
+        <v>24.9541</v>
       </c>
     </row>
     <row r="17">
@@ -5111,16 +5207,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.8181</v>
+        <v>16.8426</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55601.5972317</v>
+        <v>55682.5956282</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5601.597231699998</v>
+        <v>5682.595628199997</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.112031944634</v>
+        <v>0.1136519125639999</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -5220,6 +5316,9 @@
       </c>
       <c r="AR17" s="3" t="n">
         <v>16.8181</v>
+      </c>
+      <c r="AS17" s="3" t="n">
+        <v>16.8426</v>
       </c>
     </row>
     <row r="18">
@@ -5245,16 +5344,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>44.89</v>
+        <v>45.18</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>84682.11203999999</v>
+        <v>85229.17848</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>4682.112039999993</v>
+        <v>5229.178480000002</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.05852640049999991</v>
+        <v>0.06536473100000002</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -5360,6 +5459,9 @@
       </c>
       <c r="AR18" s="3" t="n">
         <v>44.89</v>
+      </c>
+      <c r="AS18" s="3" t="n">
+        <v>45.18</v>
       </c>
     </row>
     <row r="19">
@@ -5385,16 +5487,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>14.9529</v>
+        <v>15.0267</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>216320.1053214</v>
+        <v>217387.7526522</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>66320.10532139998</v>
+        <v>67387.7526522</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.4421340354759999</v>
+        <v>0.449251684348</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -5494,6 +5596,9 @@
       </c>
       <c r="AR19" s="3" t="n">
         <v>14.9529</v>
+      </c>
+      <c r="AS19" s="3" t="n">
+        <v>15.0267</v>
       </c>
     </row>
     <row r="20">
@@ -5519,16 +5624,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.48</v>
+        <v>9.470000000000001</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>248905.01244</v>
+        <v>248642.45441</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-1094.98755999998</v>
+        <v>-1357.545589999994</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.004379950239999918</v>
+        <v>-0.005430182359999977</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -5634,6 +5739,9 @@
       </c>
       <c r="AR20" s="3" t="n">
         <v>9.48</v>
+      </c>
+      <c r="AS20" s="3" t="n">
+        <v>9.470000000000001</v>
       </c>
     </row>
     <row r="21">
@@ -5659,16 +5767,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>110.4811</v>
+        <v>111.103</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>167849.4055049</v>
+        <v>168794.232677</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-2150.594495099998</v>
+        <v>-1205.767323000007</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.0126505558535294</v>
+        <v>-0.007092748958823572</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -5774,6 +5882,9 @@
       </c>
       <c r="AR21" s="3" t="n">
         <v>110.4811</v>
+      </c>
+      <c r="AS21" s="3" t="n">
+        <v>111.103</v>
       </c>
     </row>
     <row r="22">
@@ -5799,16 +5910,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>45.447</v>
+        <v>45.796</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>69736.60362000001</v>
+        <v>70272.13016</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>9736.603620000009</v>
+        <v>10272.13016</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1622767270000001</v>
+        <v>0.1712021693333333</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -5908,6 +6019,9 @@
       </c>
       <c r="AR22" s="3" t="n">
         <v>45.447</v>
+      </c>
+      <c r="AS22" s="3" t="n">
+        <v>45.796</v>
       </c>
     </row>
     <row r="23">
@@ -5933,16 +6047,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>62.8831</v>
+        <v>63.3739</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>170819.8660077</v>
+        <v>172153.1080113</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>20819.86600770001</v>
+        <v>22153.10801130001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.1387991067180001</v>
+        <v>0.147687386742</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -6048,6 +6162,9 @@
       </c>
       <c r="AR23" s="3" t="n">
         <v>62.8831</v>
+      </c>
+      <c r="AS23" s="3" t="n">
+        <v>63.3739</v>
       </c>
     </row>
     <row r="24">
@@ -6073,16 +6190,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>28.4869</v>
+        <v>28.5713</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>103503.9036434</v>
+        <v>103810.5614218</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>3503.903643400001</v>
+        <v>3810.561421799997</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.03503903643400001</v>
+        <v>0.03810561421799998</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -6182,6 +6299,9 @@
       </c>
       <c r="AR24" s="3" t="n">
         <v>28.4869</v>
+      </c>
+      <c r="AS24" s="3" t="n">
+        <v>28.5713</v>
       </c>
     </row>
     <row r="25">
@@ -6207,16 +6327,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.7368</v>
+        <v>11.7456</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>192737.9034032</v>
+        <v>192882.4141344</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-7262.096596799995</v>
+        <v>-7117.585865600005</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.03631048298399997</v>
+        <v>-0.03558792932800003</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -6319,6 +6439,9 @@
       </c>
       <c r="AR25" s="3" t="n">
         <v>11.7368</v>
+      </c>
+      <c r="AS25" s="3" t="n">
+        <v>11.7456</v>
       </c>
     </row>
     <row r="26">
@@ -6344,16 +6467,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>9.2788</v>
+        <v>9.249000000000001</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>110804.785142</v>
+        <v>110448.922035</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>804.7851420000079</v>
+        <v>448.9220350000105</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.007316228563636435</v>
+        <v>0.004081109409091004</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -6456,6 +6579,9 @@
       </c>
       <c r="AR26" s="3" t="n">
         <v>9.2788</v>
+      </c>
+      <c r="AS26" s="3" t="n">
+        <v>9.249000000000001</v>
       </c>
     </row>
     <row r="27">
@@ -6481,16 +6607,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>64.8507</v>
+        <v>65.11799999999999</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>104465.398602</v>
+        <v>104895.98148</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-5534.601397999999</v>
+        <v>-5104.018520000012</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.05031455816363636</v>
+        <v>-0.04640016836363647</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -6596,6 +6722,9 @@
       </c>
       <c r="AR27" s="3" t="n">
         <v>64.8507</v>
+      </c>
+      <c r="AS27" s="3" t="n">
+        <v>65.11799999999999</v>
       </c>
     </row>
     <row r="28">
@@ -6621,16 +6750,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>108.9451</v>
+        <v>108.8399</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>360244.0775307</v>
+        <v>359896.2172143</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-19755.92246929999</v>
+        <v>-20103.78278569999</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.05198926965605259</v>
+        <v>-0.05290469154131577</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -6736,6 +6865,9 @@
       </c>
       <c r="AR28" s="3" t="n">
         <v>108.9451</v>
+      </c>
+      <c r="AS28" s="3" t="n">
+        <v>108.8399</v>
       </c>
     </row>
     <row r="29">
@@ -6761,16 +6893,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.4346</v>
+        <v>12.4813</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>119418.2053238</v>
+        <v>119866.6982539</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>19418.20532379999</v>
+        <v>19866.69825389999</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.1941820532379999</v>
+        <v>0.1986669825389999</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -6870,6 +7002,9 @@
       </c>
       <c r="AR29" s="3" t="n">
         <v>12.4346</v>
+      </c>
+      <c r="AS29" s="3" t="n">
+        <v>12.4813</v>
       </c>
     </row>
     <row r="30">
@@ -6895,16 +7030,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>16.1495</v>
+        <v>16.257</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>119439.4572195</v>
+        <v>120234.512277</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>19439.45721949999</v>
+        <v>20234.512277</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.1943945721949999</v>
+        <v>0.20234512277</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -7004,6 +7139,9 @@
       </c>
       <c r="AR30" s="3" t="n">
         <v>16.1495</v>
+      </c>
+      <c r="AS30" s="3" t="n">
+        <v>16.257</v>
       </c>
     </row>
     <row r="31">
@@ -7029,16 +7167,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>420.3835</v>
+        <v>422.2204</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>111855.64168</v>
+        <v>112344.404032</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>11855.64168</v>
+        <v>12344.40403199999</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.1185564168</v>
+        <v>0.1234440403199999</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -7141,6 +7279,9 @@
       </c>
       <c r="AR31" s="3" t="n">
         <v>420.3835</v>
+      </c>
+      <c r="AS31" s="3" t="n">
+        <v>422.2204</v>
       </c>
     </row>
     <row r="32">
@@ -7166,16 +7307,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.46</v>
+        <v>10.52</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>221123.9816</v>
+        <v>222392.3792</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>21123.9816</v>
+        <v>22392.3792</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.105619908</v>
+        <v>0.111961896</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -7281,6 +7422,9 @@
       </c>
       <c r="AR32" s="3" t="n">
         <v>10.46</v>
+      </c>
+      <c r="AS32" s="3" t="n">
+        <v>10.52</v>
       </c>
     </row>
     <row r="33">
@@ -7306,16 +7450,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>18.57</v>
+        <v>18.66</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>66548.1948</v>
+        <v>66870.7224</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>6548.194799999997</v>
+        <v>6870.722399999999</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.10913658</v>
+        <v>0.11451204</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -7415,6 +7559,9 @@
       </c>
       <c r="AR33" s="3" t="n">
         <v>18.57</v>
+      </c>
+      <c r="AS33" s="3" t="n">
+        <v>18.66</v>
       </c>
     </row>
     <row r="34">
@@ -7440,16 +7587,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>213.7101</v>
+        <v>211.6903</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>75125.72516310001</v>
+        <v>74415.70284930001</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-4874.274836899989</v>
+        <v>-5584.297150699989</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.06092843546124987</v>
+        <v>-0.06980371438374987</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -7552,6 +7699,9 @@
       </c>
       <c r="AR34" s="3" t="n">
         <v>213.7101</v>
+      </c>
+      <c r="AS34" s="3" t="n">
+        <v>211.6903</v>
       </c>
     </row>
     <row r="35">
@@ -7577,16 +7727,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>14.79</v>
+        <v>14.91</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>105532.90617</v>
+        <v>106389.15693</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>5532.906169999987</v>
+        <v>6389.156929999997</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.05532906169999988</v>
+        <v>0.06389156929999998</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -7689,6 +7839,9 @@
       </c>
       <c r="AR35" s="3" t="n">
         <v>14.79</v>
+      </c>
+      <c r="AS35" s="3" t="n">
+        <v>14.91</v>
       </c>
     </row>
     <row r="36">
@@ -7714,16 +7867,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>355.3036</v>
+        <v>358.0491</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>165467.0183416</v>
+        <v>166745.6141646</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>15467.01834160002</v>
+        <v>16745.6141646</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1031134556106668</v>
+        <v>0.111637427764</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -7826,6 +7979,9 @@
       </c>
       <c r="AR36" s="3" t="n">
         <v>355.3036</v>
+      </c>
+      <c r="AS36" s="3" t="n">
+        <v>358.0491</v>
       </c>
     </row>
     <row r="37">
@@ -7851,16 +8007,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>15.813</v>
+        <v>15.951</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>59502.563757</v>
+        <v>60021.84243900001</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>9502.563757000004</v>
+        <v>10021.84243900001</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.1900512751400001</v>
+        <v>0.2004368487800001</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -7963,6 +8119,9 @@
       </c>
       <c r="AR37" s="3" t="n">
         <v>15.813</v>
+      </c>
+      <c r="AS37" s="3" t="n">
+        <v>15.951</v>
       </c>
     </row>
     <row r="38">
@@ -7988,16 +8147,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>14.2923</v>
+        <v>14.3524</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>85474.84288859999</v>
+        <v>85834.26985679999</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>5474.842888599989</v>
+        <v>5834.269856799991</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.06843553610749986</v>
+        <v>0.07292837320999988</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -8097,6 +8256,9 @@
       </c>
       <c r="AR38" s="3" t="n">
         <v>14.2923</v>
+      </c>
+      <c r="AS38" s="3" t="n">
+        <v>14.3524</v>
       </c>
     </row>
     <row r="39">
@@ -8122,16 +8284,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1018.7854</v>
+        <v>1019.0851</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50818.0345374</v>
+        <v>50832.9838731</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>818.0345374000026</v>
+        <v>832.9838730999982</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.01636069074800005</v>
+        <v>0.01665967746199996</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -8231,6 +8393,9 @@
       </c>
       <c r="AR39" s="3" t="n">
         <v>1018.7854</v>
+      </c>
+      <c r="AS39" s="3" t="n">
+        <v>1019.0851</v>
       </c>
     </row>
     <row r="40">
@@ -8256,16 +8421,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>21.1574</v>
+        <v>21.2278</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>106655.0246498</v>
+        <v>107009.9129506</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>6655.024649799991</v>
+        <v>7009.912950599988</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.06655024649799991</v>
+        <v>0.07009912950599988</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -8368,6 +8533,9 @@
       </c>
       <c r="AR40" s="3" t="n">
         <v>21.1574</v>
+      </c>
+      <c r="AS40" s="3" t="n">
+        <v>21.2278</v>
       </c>
     </row>
     <row r="41">
@@ -8380,13 +8548,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4933199.4012336</v>
+        <v>4951334.5140237</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>463199.4012336</v>
+        <v>481334.5140237</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1036240271216107</v>
+        <v>0.1076810993341611</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-06-20
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -484,8 +484,8 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-19 07:04 IST</t>
+          <t>Generated: 2026-06-20 06:19 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4951334.5140237</v>
+        <v>4960163.8993248</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>481334.5140236998</v>
+        <v>490163.8993247999</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.107681099334161</v>
+        <v>0.10965635331651</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>557439.0023498535</v>
+        <v>559848.5002975464</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-33343.0176501465</v>
+        <v>-30933.51970245363</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.05643878202343819</v>
+        <v>-0.0523602930611423</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5508773.516373553</v>
+        <v>5520012.399622346</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>447991.4963735538</v>
+        <v>459230.3796223467</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.08852218779688792</v>
+        <v>0.0907429677483613</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-06-19</t>
+          <t>Last snapshot: 2026-06-20</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR19"/>
+  <dimension ref="A1:AS19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -663,6 +663,7 @@
     <col width="21" customWidth="1" min="42" max="42"/>
     <col width="21" customWidth="1" min="43" max="43"/>
     <col width="21" customWidth="1" min="44" max="44"/>
+    <col width="21" customWidth="1" min="45" max="45"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -886,6 +887,11 @@
           <t>2026-06-19</t>
         </is>
       </c>
+      <c r="AS1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1024,6 +1030,9 @@
       <c r="AR2" s="3" t="n">
         <v>549.9500122070312</v>
       </c>
+      <c r="AS2" s="3" t="n">
+        <v>549.9500122070312</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1070,13 +1079,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1544.300048828125</v>
+        <v>1542.099975585938</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>30886.0009765625</v>
+        <v>30841.99951171875</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-1218.579023437502</v>
+        <v>-1262.580488281252</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1188,6 +1197,9 @@
       </c>
       <c r="AR4" s="3" t="n">
         <v>1544.300048828125</v>
+      </c>
+      <c r="AS4" s="3" t="n">
+        <v>1542.099975585938</v>
       </c>
     </row>
     <row r="5">
@@ -1208,13 +1220,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>659</v>
+        <v>660.2000122070312</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13180</v>
+        <v>13204.00024414062</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1033.1</v>
+        <v>-1009.099755859375</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1326,6 +1338,9 @@
       </c>
       <c r="AR5" s="3" t="n">
         <v>659</v>
+      </c>
+      <c r="AS5" s="3" t="n">
+        <v>660.2000122070312</v>
       </c>
     </row>
     <row r="6">
@@ -1346,13 +1361,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>390.25</v>
+        <v>390.2000122070312</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15610</v>
+        <v>15608.00048828125</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-1892.240000000002</v>
+        <v>-1894.239511718752</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1464,6 +1479,9 @@
       </c>
       <c r="AR6" s="3" t="n">
         <v>390.25</v>
+      </c>
+      <c r="AS6" s="3" t="n">
+        <v>390.2000122070312</v>
       </c>
     </row>
     <row r="7">
@@ -1484,13 +1502,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>251.6600036621094</v>
+        <v>250.7400054931641</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>25166.00036621094</v>
+        <v>25074.00054931641</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-1267.819633789062</v>
+        <v>-1359.819450683593</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1602,6 +1620,9 @@
       </c>
       <c r="AR7" s="3" t="n">
         <v>251.6600036621094</v>
+      </c>
+      <c r="AS7" s="3" t="n">
+        <v>250.7400054931641</v>
       </c>
     </row>
     <row r="8">
@@ -1649,13 +1670,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>18.06999969482422</v>
+        <v>18.05999946594238</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>27104.99954223633</v>
+        <v>27089.99919891357</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-3945.17045776367</v>
+        <v>-3960.170801086424</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1767,6 +1788,9 @@
       </c>
       <c r="AR9" s="3" t="n">
         <v>18.06999969482422</v>
+      </c>
+      <c r="AS9" s="3" t="n">
+        <v>18.05999946594238</v>
       </c>
     </row>
     <row r="10">
@@ -1787,13 +1811,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>418.6499938964844</v>
+        <v>418.1499938964844</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>41864.99938964844</v>
+        <v>41814.99938964844</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-9633.480610351566</v>
+        <v>-9683.480610351566</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1905,6 +1929,9 @@
       </c>
       <c r="AR10" s="3" t="n">
         <v>418.6499938964844</v>
+      </c>
+      <c r="AS10" s="3" t="n">
+        <v>418.1499938964844</v>
       </c>
     </row>
     <row r="11">
@@ -1925,13 +1952,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>8.930000305175781</v>
+        <v>8.909999847412109</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>8930.000305175781</v>
+        <v>8909.999847412109</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-911.2096948242179</v>
+        <v>-931.2101525878898</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -2043,6 +2070,9 @@
       </c>
       <c r="AR11" s="3" t="n">
         <v>8.930000305175781</v>
+      </c>
+      <c r="AS11" s="3" t="n">
+        <v>8.909999847412109</v>
       </c>
     </row>
     <row r="12">
@@ -2063,13 +2093,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2607.60009765625</v>
+        <v>2770.89990234375</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>26076.0009765625</v>
+        <v>27708.9990234375</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-1647.2490234375</v>
+        <v>-14.2509765625</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -2181,6 +2211,9 @@
       </c>
       <c r="AR12" s="3" t="n">
         <v>2607.60009765625</v>
+      </c>
+      <c r="AS12" s="3" t="n">
+        <v>2770.89990234375</v>
       </c>
     </row>
     <row r="13">
@@ -2201,13 +2234,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>59.81999969482422</v>
+        <v>59.20000076293945</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>35891.99981689453</v>
+        <v>35520.00045776367</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>860.2398168945292</v>
+        <v>488.2404577636698</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -2319,6 +2352,9 @@
       </c>
       <c r="AR13" s="3" t="n">
         <v>59.81999969482422</v>
+      </c>
+      <c r="AS13" s="3" t="n">
+        <v>59.20000076293945</v>
       </c>
     </row>
     <row r="14">
@@ -2339,13 +2375,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>725.5</v>
+        <v>729.1500244140625</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>36275</v>
+        <v>36457.50122070312</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-6187.510000000002</v>
+        <v>-6005.008779296877</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -2457,6 +2493,9 @@
       </c>
       <c r="AR14" s="3" t="n">
         <v>725.5</v>
+      </c>
+      <c r="AS14" s="3" t="n">
+        <v>729.1500244140625</v>
       </c>
     </row>
     <row r="15">
@@ -2531,13 +2570,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>611.25</v>
+        <v>632.3499755859375</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>30562.5</v>
+        <v>31617.49877929688</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>8807.970000000001</v>
+        <v>9862.968779296876</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -2649,6 +2688,9 @@
       </c>
       <c r="AR17" s="3" t="n">
         <v>611.25</v>
+      </c>
+      <c r="AS17" s="3" t="n">
+        <v>632.3499755859375</v>
       </c>
     </row>
     <row r="18">
@@ -2669,13 +2711,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>401.25</v>
+        <v>402.3500061035156</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>40125</v>
+        <v>40235.00061035156</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-6515.82</v>
+        <v>-6405.819389648437</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -2787,6 +2829,9 @@
       </c>
       <c r="AR18" s="3" t="n">
         <v>401.25</v>
+      </c>
+      <c r="AS18" s="3" t="n">
+        <v>402.3500061035156</v>
       </c>
     </row>
     <row r="19">
@@ -2799,10 +2844,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>557439.0023498535</v>
+        <v>559848.5002975464</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-33343.0176501465</v>
+        <v>-30933.51970245362</v>
       </c>
     </row>
   </sheetData>
@@ -2816,7 +2861,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS41"/>
+  <dimension ref="A1:AT41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2864,6 +2909,7 @@
     <col width="13" customWidth="1" min="43" max="43"/>
     <col width="13" customWidth="1" min="44" max="44"/>
     <col width="13" customWidth="1" min="45" max="45"/>
+    <col width="13" customWidth="1" min="46" max="46"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3092,6 +3138,11 @@
           <t>2026-06-19</t>
         </is>
       </c>
+      <c r="AT1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3116,16 +3167,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>57.1227</v>
+        <v>57.0703</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>64119.2025414</v>
+        <v>64060.3844846</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>14119.2025414</v>
+        <v>14060.3844846</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.2823840508280001</v>
+        <v>0.281207689692</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -3234,6 +3285,9 @@
       </c>
       <c r="AS2" s="3" t="n">
         <v>57.1227</v>
+      </c>
+      <c r="AT2" s="3" t="n">
+        <v>57.0703</v>
       </c>
     </row>
     <row r="3">
@@ -3372,6 +3426,9 @@
       <c r="AS3" s="3" t="n">
         <v>25.31</v>
       </c>
+      <c r="AT3" s="3" t="n">
+        <v>25.31</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3509,6 +3566,9 @@
       <c r="AS4" s="3" t="n">
         <v>12.37</v>
       </c>
+      <c r="AT4" s="3" t="n">
+        <v>12.37</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3533,16 +3593,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.5838</v>
+        <v>9.5047</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>175901.9085744</v>
+        <v>174450.1002136</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-34098.0914256</v>
+        <v>-35549.8997864</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1623718639314286</v>
+        <v>-0.1692852370780952</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -3645,6 +3705,9 @@
       </c>
       <c r="AS5" s="3" t="n">
         <v>9.5838</v>
+      </c>
+      <c r="AT5" s="3" t="n">
+        <v>9.5047</v>
       </c>
     </row>
     <row r="6">
@@ -3670,16 +3733,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.3967</v>
+        <v>12.4233</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>52425.3591759</v>
+        <v>52537.84996409999</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>2425.359175899997</v>
+        <v>2537.849964099994</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.04850718351799994</v>
+        <v>0.05075699928199989</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -3788,6 +3851,9 @@
       </c>
       <c r="AS6" s="3" t="n">
         <v>12.3967</v>
+      </c>
+      <c r="AT6" s="3" t="n">
+        <v>12.4233</v>
       </c>
     </row>
     <row r="7">
@@ -3813,16 +3879,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.9637</v>
+        <v>33.9176</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>74925.280748</v>
+        <v>74823.582304</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>14925.280748</v>
+        <v>14823.582304</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2487546791333334</v>
+        <v>0.2470597050666666</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -3925,6 +3991,9 @@
       </c>
       <c r="AS7" s="3" t="n">
         <v>33.9637</v>
+      </c>
+      <c r="AT7" s="3" t="n">
+        <v>33.9176</v>
       </c>
     </row>
     <row r="8">
@@ -3950,16 +4019,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>33.0896</v>
+        <v>33.4768</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>53095.3405328</v>
+        <v>53716.6389424</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>3095.340532800001</v>
+        <v>3716.638942400001</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.06190681065600002</v>
+        <v>0.07433277884800002</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -4068,6 +4137,9 @@
       </c>
       <c r="AS8" s="3" t="n">
         <v>33.0896</v>
+      </c>
+      <c r="AT8" s="3" t="n">
+        <v>33.4768</v>
       </c>
     </row>
     <row r="9">
@@ -4206,6 +4278,9 @@
       <c r="AS9" s="3" t="n">
         <v>42.1536</v>
       </c>
+      <c r="AT9" s="3" t="n">
+        <v>42.1536</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4343,6 +4418,9 @@
       <c r="AS10" s="3" t="n">
         <v>47.2455</v>
       </c>
+      <c r="AT10" s="3" t="n">
+        <v>47.2455</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4480,6 +4558,9 @@
       <c r="AS11" s="3" t="n">
         <v>105.991</v>
       </c>
+      <c r="AT11" s="3" t="n">
+        <v>105.991</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4504,16 +4585,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>225.63</v>
+        <v>226.497</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>105035.72886</v>
+        <v>105439.336434</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>5035.728860000003</v>
+        <v>5439.336434000012</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.05035728860000003</v>
+        <v>0.05439336434000012</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -4622,6 +4703,9 @@
       </c>
       <c r="AS12" s="3" t="n">
         <v>225.63</v>
+      </c>
+      <c r="AT12" s="3" t="n">
+        <v>226.497</v>
       </c>
     </row>
     <row r="13">
@@ -4647,16 +4731,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>20.414</v>
+        <v>20.615</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>236549.36847</v>
+        <v>238878.477075</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>36549.36847000002</v>
+        <v>38878.47707499997</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.1827468423500001</v>
+        <v>0.1943923853749999</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -4765,6 +4849,9 @@
       </c>
       <c r="AS13" s="3" t="n">
         <v>20.414</v>
+      </c>
+      <c r="AT13" s="3" t="n">
+        <v>20.615</v>
       </c>
     </row>
     <row r="14">
@@ -4903,6 +4990,9 @@
       <c r="AS14" s="3" t="n">
         <v>40.1296</v>
       </c>
+      <c r="AT14" s="3" t="n">
+        <v>40.1296</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4927,16 +5017,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.99</v>
+        <v>12.03</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>116829.92453</v>
+        <v>117219.68241</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>16829.92453</v>
+        <v>17219.68240999999</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1682992453</v>
+        <v>0.1721968241</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -5045,6 +5135,9 @@
       </c>
       <c r="AS15" s="3" t="n">
         <v>11.99</v>
+      </c>
+      <c r="AT15" s="3" t="n">
+        <v>12.03</v>
       </c>
     </row>
     <row r="16">
@@ -5183,6 +5276,9 @@
       <c r="AS16" s="3" t="n">
         <v>24.9541</v>
       </c>
+      <c r="AT16" s="3" t="n">
+        <v>24.9541</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5320,6 +5416,9 @@
       <c r="AS17" s="3" t="n">
         <v>16.8426</v>
       </c>
+      <c r="AT17" s="3" t="n">
+        <v>16.8426</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5344,16 +5443,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>45.18</v>
+        <v>45.33</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>85229.17848</v>
+        <v>85512.14387999999</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>5229.178480000002</v>
+        <v>5512.143879999989</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.06536473100000002</v>
+        <v>0.06890179849999986</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -5462,6 +5561,9 @@
       </c>
       <c r="AS18" s="3" t="n">
         <v>45.18</v>
+      </c>
+      <c r="AT18" s="3" t="n">
+        <v>45.33</v>
       </c>
     </row>
     <row r="19">
@@ -5600,6 +5702,9 @@
       <c r="AS19" s="3" t="n">
         <v>15.0267</v>
       </c>
+      <c r="AT19" s="3" t="n">
+        <v>15.0267</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5624,16 +5729,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.470000000000001</v>
+        <v>9.41</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>248642.45441</v>
+        <v>247067.10623</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-1357.545589999994</v>
+        <v>-2932.893769999995</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.005430182359999977</v>
+        <v>-0.01173157507999998</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -5742,6 +5847,9 @@
       </c>
       <c r="AS20" s="3" t="n">
         <v>9.470000000000001</v>
+      </c>
+      <c r="AT20" s="3" t="n">
+        <v>9.41</v>
       </c>
     </row>
     <row r="21">
@@ -5767,16 +5875,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>111.103</v>
+        <v>111.1739</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>168794.232677</v>
+        <v>168901.9481401</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-1205.767323000007</v>
+        <v>-1098.051859900006</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.007092748958823572</v>
+        <v>-0.006459128587647095</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -5885,6 +5993,9 @@
       </c>
       <c r="AS21" s="3" t="n">
         <v>111.103</v>
+      </c>
+      <c r="AT21" s="3" t="n">
+        <v>111.1739</v>
       </c>
     </row>
     <row r="22">
@@ -5910,16 +6021,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>45.796</v>
+        <v>45.876</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>70272.13016</v>
+        <v>70394.88696</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>10272.13016</v>
+        <v>10394.88696</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1712021693333333</v>
+        <v>0.1732481160000001</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -6022,6 +6133,9 @@
       </c>
       <c r="AS22" s="3" t="n">
         <v>45.796</v>
+      </c>
+      <c r="AT22" s="3" t="n">
+        <v>45.876</v>
       </c>
     </row>
     <row r="23">
@@ -6047,16 +6161,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>63.3739</v>
+        <v>63.7762</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>172153.1080113</v>
+        <v>173245.9426854</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>22153.10801130001</v>
+        <v>23245.94268540002</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.147687386742</v>
+        <v>0.1549729512360001</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -6165,6 +6279,9 @@
       </c>
       <c r="AS23" s="3" t="n">
         <v>63.3739</v>
+      </c>
+      <c r="AT23" s="3" t="n">
+        <v>63.7762</v>
       </c>
     </row>
     <row r="24">
@@ -6190,16 +6307,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>28.5713</v>
+        <v>28.3764</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>103810.5614218</v>
+        <v>103102.4144904</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>3810.561421799997</v>
+        <v>3102.414490399999</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.03810561421799998</v>
+        <v>0.03102414490399999</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -6302,6 +6419,9 @@
       </c>
       <c r="AS24" s="3" t="n">
         <v>28.5713</v>
+      </c>
+      <c r="AT24" s="3" t="n">
+        <v>28.3764</v>
       </c>
     </row>
     <row r="25">
@@ -6327,16 +6447,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.7456</v>
+        <v>11.7358</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>192882.4141344</v>
+        <v>192721.4817292</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-7117.585865600005</v>
+        <v>-7278.518270800036</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.03558792932800003</v>
+        <v>-0.03639259135400018</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -6442,6 +6562,9 @@
       </c>
       <c r="AS25" s="3" t="n">
         <v>11.7456</v>
+      </c>
+      <c r="AT25" s="3" t="n">
+        <v>11.7358</v>
       </c>
     </row>
     <row r="26">
@@ -6467,16 +6590,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>9.249000000000001</v>
+        <v>9.218</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>110448.922035</v>
+        <v>110078.72887</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>448.9220350000105</v>
+        <v>78.72887000000628</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.004081109409091004</v>
+        <v>0.0007157170000000571</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -6582,6 +6705,9 @@
       </c>
       <c r="AS26" s="3" t="n">
         <v>9.249000000000001</v>
+      </c>
+      <c r="AT26" s="3" t="n">
+        <v>9.218</v>
       </c>
     </row>
     <row r="27">
@@ -6607,16 +6733,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>65.11799999999999</v>
+        <v>65.55629999999999</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>104895.98148</v>
+        <v>105602.021418</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-5104.018520000012</v>
+        <v>-4397.978582000011</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.04640016836363647</v>
+        <v>-0.03998162347272737</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -6725,6 +6851,9 @@
       </c>
       <c r="AS27" s="3" t="n">
         <v>65.11799999999999</v>
+      </c>
+      <c r="AT27" s="3" t="n">
+        <v>65.55629999999999</v>
       </c>
     </row>
     <row r="28">
@@ -6750,16 +6879,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>108.8399</v>
+        <v>109.0277</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>359896.2172143</v>
+        <v>360517.2073989</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-20103.78278569999</v>
+        <v>-19482.79260109999</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.05290469154131577</v>
+        <v>-0.05127050684499999</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -6868,6 +6997,9 @@
       </c>
       <c r="AS28" s="3" t="n">
         <v>108.8399</v>
+      </c>
+      <c r="AT28" s="3" t="n">
+        <v>109.0277</v>
       </c>
     </row>
     <row r="29">
@@ -6893,16 +7025,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.4813</v>
+        <v>12.5655</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>119866.6982539</v>
+        <v>120675.3300465</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>19866.69825389999</v>
+        <v>20675.33004649999</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.1986669825389999</v>
+        <v>0.2067533004649999</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -7005,6 +7137,9 @@
       </c>
       <c r="AS29" s="3" t="n">
         <v>12.4813</v>
+      </c>
+      <c r="AT29" s="3" t="n">
+        <v>12.5655</v>
       </c>
     </row>
     <row r="30">
@@ -7030,16 +7165,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>16.257</v>
+        <v>16.475</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>120234.512277</v>
+        <v>121846.809975</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>20234.512277</v>
+        <v>21846.80997500001</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.20234512277</v>
+        <v>0.2184680997500001</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -7142,6 +7277,9 @@
       </c>
       <c r="AS30" s="3" t="n">
         <v>16.257</v>
+      </c>
+      <c r="AT30" s="3" t="n">
+        <v>16.475</v>
       </c>
     </row>
     <row r="31">
@@ -7167,16 +7305,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>422.2204</v>
+        <v>423.5517</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>112344.404032</v>
+        <v>112698.636336</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>12344.40403199999</v>
+        <v>12698.63633599998</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.1234440403199999</v>
+        <v>0.1269863633599998</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -7282,6 +7420,9 @@
       </c>
       <c r="AS31" s="3" t="n">
         <v>422.2204</v>
+      </c>
+      <c r="AT31" s="3" t="n">
+        <v>423.5517</v>
       </c>
     </row>
     <row r="32">
@@ -7307,16 +7448,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.52</v>
+        <v>10.54</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>222392.3792</v>
+        <v>222815.1784</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>22392.3792</v>
+        <v>22815.17839999998</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.111961896</v>
+        <v>0.1140758919999999</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -7425,6 +7566,9 @@
       </c>
       <c r="AS32" s="3" t="n">
         <v>10.52</v>
+      </c>
+      <c r="AT32" s="3" t="n">
+        <v>10.54</v>
       </c>
     </row>
     <row r="33">
@@ -7450,16 +7594,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>18.66</v>
+        <v>18.74</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>66870.7224</v>
+        <v>67157.41359999999</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>6870.722399999999</v>
+        <v>7157.413599999985</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.11451204</v>
+        <v>0.1192902266666664</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -7562,6 +7706,9 @@
       </c>
       <c r="AS33" s="3" t="n">
         <v>18.66</v>
+      </c>
+      <c r="AT33" s="3" t="n">
+        <v>18.74</v>
       </c>
     </row>
     <row r="34">
@@ -7587,16 +7734,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>211.6903</v>
+        <v>209.7188</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>74415.70284930001</v>
+        <v>73722.65948279999</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-5584.297150699989</v>
+        <v>-6277.340517200006</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.06980371438374987</v>
+        <v>-0.07846675646500006</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -7702,6 +7849,9 @@
       </c>
       <c r="AS34" s="3" t="n">
         <v>211.6903</v>
+      </c>
+      <c r="AT34" s="3" t="n">
+        <v>209.7188</v>
       </c>
     </row>
     <row r="35">
@@ -7727,16 +7877,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>14.91</v>
+        <v>15.06</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>106389.15693</v>
+        <v>107459.47038</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>6389.156929999997</v>
+        <v>7459.470379999999</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.06389156929999998</v>
+        <v>0.0745947038</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -7842,6 +7992,9 @@
       </c>
       <c r="AS35" s="3" t="n">
         <v>14.91</v>
+      </c>
+      <c r="AT35" s="3" t="n">
+        <v>15.06</v>
       </c>
     </row>
     <row r="36">
@@ -7867,16 +8020,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>358.0491</v>
+        <v>360.6164</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>166745.6141646</v>
+        <v>167941.2211784</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>16745.6141646</v>
+        <v>17941.22117840001</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.111637427764</v>
+        <v>0.1196081411893334</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -7982,6 +8135,9 @@
       </c>
       <c r="AS36" s="3" t="n">
         <v>358.0491</v>
+      </c>
+      <c r="AT36" s="3" t="n">
+        <v>360.6164</v>
       </c>
     </row>
     <row r="37">
@@ -8007,16 +8163,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>15.951</v>
+        <v>16.095</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>60021.84243900001</v>
+        <v>60563.698455</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>10021.84243900001</v>
+        <v>10563.698455</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.2004368487800001</v>
+        <v>0.2112739691</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -8122,6 +8278,9 @@
       </c>
       <c r="AS37" s="3" t="n">
         <v>15.951</v>
+      </c>
+      <c r="AT37" s="3" t="n">
+        <v>16.095</v>
       </c>
     </row>
     <row r="38">
@@ -8147,16 +8306,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>14.3524</v>
+        <v>14.3497</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>85834.26985679999</v>
+        <v>85818.1225554</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>5834.269856799991</v>
+        <v>5818.122555399998</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.07292837320999988</v>
+        <v>0.07272653194249996</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -8259,6 +8418,9 @@
       </c>
       <c r="AS38" s="3" t="n">
         <v>14.3524</v>
+      </c>
+      <c r="AT38" s="3" t="n">
+        <v>14.3497</v>
       </c>
     </row>
     <row r="39">
@@ -8284,16 +8446,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1019.0851</v>
+        <v>1019.0919</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50832.9838731</v>
+        <v>50833.3230639</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>832.9838730999982</v>
+        <v>833.323063900003</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.01665967746199996</v>
+        <v>0.01666646127800006</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -8396,6 +8558,9 @@
       </c>
       <c r="AS39" s="3" t="n">
         <v>1019.0851</v>
+      </c>
+      <c r="AT39" s="3" t="n">
+        <v>1019.0919</v>
       </c>
     </row>
     <row r="40">
@@ -8421,16 +8586,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>21.2278</v>
+        <v>21.403</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>107009.9129506</v>
+        <v>107893.100881</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>7009.912950599988</v>
+        <v>7893.100880999991</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.07009912950599988</v>
+        <v>0.07893100880999991</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -8536,6 +8701,9 @@
       </c>
       <c r="AS40" s="3" t="n">
         <v>21.2278</v>
+      </c>
+      <c r="AT40" s="3" t="n">
+        <v>21.403</v>
       </c>
     </row>
     <row r="41">
@@ -8548,13 +8716,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4951334.5140237</v>
+        <v>4960163.8993248</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>481334.5140237</v>
+        <v>490163.8993247999</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1076810993341611</v>
+        <v>0.10965635331651</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-06-21
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-20 06:19 IST</t>
+          <t>Generated: 2026-06-21 06:50 IST</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-06-20</t>
+          <t>Last snapshot: 2026-06-21</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS19"/>
+  <dimension ref="A1:AT19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -664,6 +664,7 @@
     <col width="21" customWidth="1" min="43" max="43"/>
     <col width="21" customWidth="1" min="44" max="44"/>
     <col width="21" customWidth="1" min="45" max="45"/>
+    <col width="21" customWidth="1" min="46" max="46"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -892,6 +893,11 @@
           <t>2026-06-20</t>
         </is>
       </c>
+      <c r="AT1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1033,6 +1039,9 @@
       <c r="AS2" s="3" t="n">
         <v>549.9500122070312</v>
       </c>
+      <c r="AT2" s="3" t="n">
+        <v>549.9500122070312</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1201,6 +1210,9 @@
       <c r="AS4" s="3" t="n">
         <v>1542.099975585938</v>
       </c>
+      <c r="AT4" s="3" t="n">
+        <v>1542.099975585938</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1342,6 +1354,9 @@
       <c r="AS5" s="3" t="n">
         <v>660.2000122070312</v>
       </c>
+      <c r="AT5" s="3" t="n">
+        <v>660.2000122070312</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1483,6 +1498,9 @@
       <c r="AS6" s="3" t="n">
         <v>390.2000122070312</v>
       </c>
+      <c r="AT6" s="3" t="n">
+        <v>390.2000122070312</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1624,6 +1642,9 @@
       <c r="AS7" s="3" t="n">
         <v>250.7400054931641</v>
       </c>
+      <c r="AT7" s="3" t="n">
+        <v>250.7400054931641</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1792,6 +1813,9 @@
       <c r="AS9" s="3" t="n">
         <v>18.05999946594238</v>
       </c>
+      <c r="AT9" s="3" t="n">
+        <v>18.05999946594238</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1933,6 +1957,9 @@
       <c r="AS10" s="3" t="n">
         <v>418.1499938964844</v>
       </c>
+      <c r="AT10" s="3" t="n">
+        <v>418.1499938964844</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2074,6 +2101,9 @@
       <c r="AS11" s="3" t="n">
         <v>8.909999847412109</v>
       </c>
+      <c r="AT11" s="3" t="n">
+        <v>8.909999847412109</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2215,6 +2245,9 @@
       <c r="AS12" s="3" t="n">
         <v>2770.89990234375</v>
       </c>
+      <c r="AT12" s="3" t="n">
+        <v>2770.89990234375</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2356,6 +2389,9 @@
       <c r="AS13" s="3" t="n">
         <v>59.20000076293945</v>
       </c>
+      <c r="AT13" s="3" t="n">
+        <v>59.20000076293945</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2497,6 +2533,9 @@
       <c r="AS14" s="3" t="n">
         <v>729.1500244140625</v>
       </c>
+      <c r="AT14" s="3" t="n">
+        <v>729.1500244140625</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2692,6 +2731,9 @@
       <c r="AS17" s="3" t="n">
         <v>632.3499755859375</v>
       </c>
+      <c r="AT17" s="3" t="n">
+        <v>632.3499755859375</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2831,6 +2873,9 @@
         <v>401.25</v>
       </c>
       <c r="AS18" s="3" t="n">
+        <v>402.3500061035156</v>
+      </c>
+      <c r="AT18" s="3" t="n">
         <v>402.3500061035156</v>
       </c>
     </row>
@@ -2861,7 +2906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT41"/>
+  <dimension ref="A1:AU41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2910,6 +2955,7 @@
     <col width="13" customWidth="1" min="44" max="44"/>
     <col width="13" customWidth="1" min="45" max="45"/>
     <col width="13" customWidth="1" min="46" max="46"/>
+    <col width="13" customWidth="1" min="47" max="47"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3143,6 +3189,11 @@
           <t>2026-06-20</t>
         </is>
       </c>
+      <c r="AU1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3289,6 +3340,9 @@
       <c r="AT2" s="3" t="n">
         <v>57.0703</v>
       </c>
+      <c r="AU2" s="3" t="n">
+        <v>57.0703</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3429,6 +3483,9 @@
       <c r="AT3" s="3" t="n">
         <v>25.31</v>
       </c>
+      <c r="AU3" s="3" t="n">
+        <v>25.31</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3569,6 +3626,9 @@
       <c r="AT4" s="3" t="n">
         <v>12.37</v>
       </c>
+      <c r="AU4" s="3" t="n">
+        <v>12.37</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3709,6 +3769,9 @@
       <c r="AT5" s="3" t="n">
         <v>9.5047</v>
       </c>
+      <c r="AU5" s="3" t="n">
+        <v>9.5047</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3855,6 +3918,9 @@
       <c r="AT6" s="3" t="n">
         <v>12.4233</v>
       </c>
+      <c r="AU6" s="3" t="n">
+        <v>12.4233</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3995,6 +4061,9 @@
       <c r="AT7" s="3" t="n">
         <v>33.9176</v>
       </c>
+      <c r="AU7" s="3" t="n">
+        <v>33.9176</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4141,6 +4210,9 @@
       <c r="AT8" s="3" t="n">
         <v>33.4768</v>
       </c>
+      <c r="AU8" s="3" t="n">
+        <v>33.4768</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4281,6 +4353,9 @@
       <c r="AT9" s="3" t="n">
         <v>42.1536</v>
       </c>
+      <c r="AU9" s="3" t="n">
+        <v>42.1536</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4421,6 +4496,9 @@
       <c r="AT10" s="3" t="n">
         <v>47.2455</v>
       </c>
+      <c r="AU10" s="3" t="n">
+        <v>47.2455</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4561,6 +4639,9 @@
       <c r="AT11" s="3" t="n">
         <v>105.991</v>
       </c>
+      <c r="AU11" s="3" t="n">
+        <v>105.991</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4707,6 +4788,9 @@
       <c r="AT12" s="3" t="n">
         <v>226.497</v>
       </c>
+      <c r="AU12" s="3" t="n">
+        <v>226.497</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4853,6 +4937,9 @@
       <c r="AT13" s="3" t="n">
         <v>20.615</v>
       </c>
+      <c r="AU13" s="3" t="n">
+        <v>20.615</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4993,6 +5080,9 @@
       <c r="AT14" s="3" t="n">
         <v>40.1296</v>
       </c>
+      <c r="AU14" s="3" t="n">
+        <v>40.1296</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5139,6 +5229,9 @@
       <c r="AT15" s="3" t="n">
         <v>12.03</v>
       </c>
+      <c r="AU15" s="3" t="n">
+        <v>12.03</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5279,6 +5372,9 @@
       <c r="AT16" s="3" t="n">
         <v>24.9541</v>
       </c>
+      <c r="AU16" s="3" t="n">
+        <v>24.9541</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5419,6 +5515,9 @@
       <c r="AT17" s="3" t="n">
         <v>16.8426</v>
       </c>
+      <c r="AU17" s="3" t="n">
+        <v>16.8426</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5565,6 +5664,9 @@
       <c r="AT18" s="3" t="n">
         <v>45.33</v>
       </c>
+      <c r="AU18" s="3" t="n">
+        <v>45.33</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5705,6 +5807,9 @@
       <c r="AT19" s="3" t="n">
         <v>15.0267</v>
       </c>
+      <c r="AU19" s="3" t="n">
+        <v>15.0267</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5851,6 +5956,9 @@
       <c r="AT20" s="3" t="n">
         <v>9.41</v>
       </c>
+      <c r="AU20" s="3" t="n">
+        <v>9.41</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5997,6 +6105,9 @@
       <c r="AT21" s="3" t="n">
         <v>111.1739</v>
       </c>
+      <c r="AU21" s="3" t="n">
+        <v>111.1739</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -6137,6 +6248,9 @@
       <c r="AT22" s="3" t="n">
         <v>45.876</v>
       </c>
+      <c r="AU22" s="3" t="n">
+        <v>45.876</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -6283,6 +6397,9 @@
       <c r="AT23" s="3" t="n">
         <v>63.7762</v>
       </c>
+      <c r="AU23" s="3" t="n">
+        <v>63.7762</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -6423,6 +6540,9 @@
       <c r="AT24" s="3" t="n">
         <v>28.3764</v>
       </c>
+      <c r="AU24" s="3" t="n">
+        <v>28.3764</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -6566,6 +6686,9 @@
       <c r="AT25" s="3" t="n">
         <v>11.7358</v>
       </c>
+      <c r="AU25" s="3" t="n">
+        <v>11.7358</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -6709,6 +6832,9 @@
       <c r="AT26" s="3" t="n">
         <v>9.218</v>
       </c>
+      <c r="AU26" s="3" t="n">
+        <v>9.218</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6855,6 +6981,9 @@
       <c r="AT27" s="3" t="n">
         <v>65.55629999999999</v>
       </c>
+      <c r="AU27" s="3" t="n">
+        <v>65.55629999999999</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -7001,6 +7130,9 @@
       <c r="AT28" s="3" t="n">
         <v>109.0277</v>
       </c>
+      <c r="AU28" s="3" t="n">
+        <v>109.0277</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -7141,6 +7273,9 @@
       <c r="AT29" s="3" t="n">
         <v>12.5655</v>
       </c>
+      <c r="AU29" s="3" t="n">
+        <v>12.5655</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -7281,6 +7416,9 @@
       <c r="AT30" s="3" t="n">
         <v>16.475</v>
       </c>
+      <c r="AU30" s="3" t="n">
+        <v>16.475</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -7424,6 +7562,9 @@
       <c r="AT31" s="3" t="n">
         <v>423.5517</v>
       </c>
+      <c r="AU31" s="3" t="n">
+        <v>423.5517</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -7570,6 +7711,9 @@
       <c r="AT32" s="3" t="n">
         <v>10.54</v>
       </c>
+      <c r="AU32" s="3" t="n">
+        <v>10.54</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -7710,6 +7854,9 @@
       <c r="AT33" s="3" t="n">
         <v>18.74</v>
       </c>
+      <c r="AU33" s="3" t="n">
+        <v>18.74</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -7853,6 +8000,9 @@
       <c r="AT34" s="3" t="n">
         <v>209.7188</v>
       </c>
+      <c r="AU34" s="3" t="n">
+        <v>209.7188</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -7996,6 +8146,9 @@
       <c r="AT35" s="3" t="n">
         <v>15.06</v>
       </c>
+      <c r="AU35" s="3" t="n">
+        <v>15.06</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -8139,6 +8292,9 @@
       <c r="AT36" s="3" t="n">
         <v>360.6164</v>
       </c>
+      <c r="AU36" s="3" t="n">
+        <v>360.6164</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -8282,6 +8438,9 @@
       <c r="AT37" s="3" t="n">
         <v>16.095</v>
       </c>
+      <c r="AU37" s="3" t="n">
+        <v>16.095</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -8422,6 +8581,9 @@
       <c r="AT38" s="3" t="n">
         <v>14.3497</v>
       </c>
+      <c r="AU38" s="3" t="n">
+        <v>14.3497</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -8562,6 +8724,9 @@
       <c r="AT39" s="3" t="n">
         <v>1019.0919</v>
       </c>
+      <c r="AU39" s="3" t="n">
+        <v>1019.0919</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -8703,6 +8868,9 @@
         <v>21.2278</v>
       </c>
       <c r="AT40" s="3" t="n">
+        <v>21.403</v>
+      </c>
+      <c r="AU40" s="3" t="n">
         <v>21.403</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily portfolio update 2026-06-22
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -485,7 +485,7 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-21 06:50 IST</t>
+          <t>Generated: 2026-06-22 07:22 IST</t>
         </is>
       </c>
     </row>
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>559848.5002975464</v>
+        <v>563004.5028381348</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-30933.51970245363</v>
+        <v>-27777.51716186525</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.0523602930611423</v>
+        <v>-0.04701821690826889</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5520012.399622346</v>
+        <v>5523168.402162935</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>459230.3796223467</v>
+        <v>462386.3821629351</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.0907429677483613</v>
+        <v>0.0913665872854439</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-06-21</t>
+          <t>Last snapshot: 2026-06-22</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT19"/>
+  <dimension ref="A1:AU19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -665,6 +665,7 @@
     <col width="21" customWidth="1" min="44" max="44"/>
     <col width="21" customWidth="1" min="45" max="45"/>
     <col width="21" customWidth="1" min="46" max="46"/>
+    <col width="21" customWidth="1" min="47" max="47"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -898,6 +899,11 @@
           <t>2026-06-21</t>
         </is>
       </c>
+      <c r="AU1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -917,13 +923,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>549.9500122070312</v>
+        <v>564</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>43996.0009765625</v>
+        <v>45120</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>178.490976562498</v>
+        <v>1302.489999999998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1041,6 +1047,9 @@
       </c>
       <c r="AT2" s="3" t="n">
         <v>549.9500122070312</v>
+      </c>
+      <c r="AU2" s="3" t="n">
+        <v>564</v>
       </c>
     </row>
     <row r="3">
@@ -1088,13 +1097,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1542.099975585938</v>
+        <v>1560.300048828125</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>30841.99951171875</v>
+        <v>31206.0009765625</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-1262.580488281252</v>
+        <v>-898.5790234375017</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1212,6 +1221,9 @@
       </c>
       <c r="AT4" s="3" t="n">
         <v>1542.099975585938</v>
+      </c>
+      <c r="AU4" s="3" t="n">
+        <v>1560.300048828125</v>
       </c>
     </row>
     <row r="5">
@@ -1232,13 +1244,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>660.2000122070312</v>
+        <v>665.7000122070312</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13204.00024414062</v>
+        <v>13314.00024414062</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1009.099755859375</v>
+        <v>-899.0997558593754</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1356,6 +1368,9 @@
       </c>
       <c r="AT5" s="3" t="n">
         <v>660.2000122070312</v>
+      </c>
+      <c r="AU5" s="3" t="n">
+        <v>665.7000122070312</v>
       </c>
     </row>
     <row r="6">
@@ -1376,13 +1391,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>390.2000122070312</v>
+        <v>389.8500061035156</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15608.00048828125</v>
+        <v>15594.00024414062</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-1894.239511718752</v>
+        <v>-1908.239755859377</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1500,6 +1515,9 @@
       </c>
       <c r="AT6" s="3" t="n">
         <v>390.2000122070312</v>
+      </c>
+      <c r="AU6" s="3" t="n">
+        <v>389.8500061035156</v>
       </c>
     </row>
     <row r="7">
@@ -1520,13 +1538,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>250.7400054931641</v>
+        <v>258.4200134277344</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>25074.00054931641</v>
+        <v>25842.00134277344</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-1359.819450683593</v>
+        <v>-591.8186572265622</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1644,6 +1662,9 @@
       </c>
       <c r="AT7" s="3" t="n">
         <v>250.7400054931641</v>
+      </c>
+      <c r="AU7" s="3" t="n">
+        <v>258.4200134277344</v>
       </c>
     </row>
     <row r="8">
@@ -1691,13 +1712,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>18.05999946594238</v>
+        <v>18.51000022888184</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>27089.99919891357</v>
+        <v>27765.00034332275</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-3960.170801086424</v>
+        <v>-3285.169656677244</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1815,6 +1836,9 @@
       </c>
       <c r="AT9" s="3" t="n">
         <v>18.05999946594238</v>
+      </c>
+      <c r="AU9" s="3" t="n">
+        <v>18.51000022888184</v>
       </c>
     </row>
     <row r="10">
@@ -1835,13 +1859,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>418.1499938964844</v>
+        <v>418.3999938964844</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>41814.99938964844</v>
+        <v>41839.99938964844</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-9683.480610351566</v>
+        <v>-9658.480610351566</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1959,6 +1983,9 @@
       </c>
       <c r="AT10" s="3" t="n">
         <v>418.1499938964844</v>
+      </c>
+      <c r="AU10" s="3" t="n">
+        <v>418.3999938964844</v>
       </c>
     </row>
     <row r="11">
@@ -1979,13 +2006,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>8.909999847412109</v>
+        <v>8.949999809265137</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>8909.999847412109</v>
+        <v>8949.999809265137</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-931.2101525878898</v>
+        <v>-891.2101907348624</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -2103,6 +2130,9 @@
       </c>
       <c r="AT11" s="3" t="n">
         <v>8.909999847412109</v>
+      </c>
+      <c r="AU11" s="3" t="n">
+        <v>8.949999809265137</v>
       </c>
     </row>
     <row r="12">
@@ -2123,13 +2153,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2770.89990234375</v>
+        <v>2767.800048828125</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>27708.9990234375</v>
+        <v>27678.00048828125</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-14.2509765625</v>
+        <v>-45.24951171875</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -2247,6 +2277,9 @@
       </c>
       <c r="AT12" s="3" t="n">
         <v>2770.89990234375</v>
+      </c>
+      <c r="AU12" s="3" t="n">
+        <v>2767.800048828125</v>
       </c>
     </row>
     <row r="13">
@@ -2267,13 +2300,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>59.20000076293945</v>
+        <v>59.5</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>35520.00045776367</v>
+        <v>35700</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>488.2404577636698</v>
+        <v>668.239999999998</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -2391,6 +2424,9 @@
       </c>
       <c r="AT13" s="3" t="n">
         <v>59.20000076293945</v>
+      </c>
+      <c r="AU13" s="3" t="n">
+        <v>59.5</v>
       </c>
     </row>
     <row r="14">
@@ -2411,13 +2447,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>729.1500244140625</v>
+        <v>726.4000244140625</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>36457.50122070312</v>
+        <v>36320.00122070312</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-6005.008779296877</v>
+        <v>-6142.508779296877</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -2535,6 +2571,9 @@
       </c>
       <c r="AT14" s="3" t="n">
         <v>729.1500244140625</v>
+      </c>
+      <c r="AU14" s="3" t="n">
+        <v>726.4000244140625</v>
       </c>
     </row>
     <row r="15">
@@ -2609,13 +2648,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>632.3499755859375</v>
+        <v>629.0999755859375</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>31617.49877929688</v>
+        <v>31454.99877929688</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>9862.968779296876</v>
+        <v>9700.468779296876</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -2733,6 +2772,9 @@
       </c>
       <c r="AT17" s="3" t="n">
         <v>632.3499755859375</v>
+      </c>
+      <c r="AU17" s="3" t="n">
+        <v>629.0999755859375</v>
       </c>
     </row>
     <row r="18">
@@ -2753,13 +2795,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>402.3500061035156</v>
+        <v>404.5</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>40235.00061035156</v>
+        <v>40450</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-6405.819389648437</v>
+        <v>-6190.82</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -2877,6 +2919,9 @@
       </c>
       <c r="AT18" s="3" t="n">
         <v>402.3500061035156</v>
+      </c>
+      <c r="AU18" s="3" t="n">
+        <v>404.5</v>
       </c>
     </row>
     <row r="19">
@@ -2889,10 +2934,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>559848.5002975464</v>
+        <v>563004.5028381348</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-30933.51970245362</v>
+        <v>-27777.51716186525</v>
       </c>
     </row>
   </sheetData>
@@ -2906,7 +2951,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU41"/>
+  <dimension ref="A1:AV41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2956,6 +3001,7 @@
     <col width="13" customWidth="1" min="45" max="45"/>
     <col width="13" customWidth="1" min="46" max="46"/>
     <col width="13" customWidth="1" min="47" max="47"/>
+    <col width="13" customWidth="1" min="48" max="48"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3194,6 +3240,11 @@
           <t>2026-06-21</t>
         </is>
       </c>
+      <c r="AV1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3343,6 +3394,9 @@
       <c r="AU2" s="3" t="n">
         <v>57.0703</v>
       </c>
+      <c r="AV2" s="3" t="n">
+        <v>57.0703</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3486,6 +3540,9 @@
       <c r="AU3" s="3" t="n">
         <v>25.31</v>
       </c>
+      <c r="AV3" s="3" t="n">
+        <v>25.31</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3629,6 +3686,9 @@
       <c r="AU4" s="3" t="n">
         <v>12.37</v>
       </c>
+      <c r="AV4" s="3" t="n">
+        <v>12.37</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3772,6 +3832,9 @@
       <c r="AU5" s="3" t="n">
         <v>9.5047</v>
       </c>
+      <c r="AV5" s="3" t="n">
+        <v>9.5047</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3921,6 +3984,9 @@
       <c r="AU6" s="3" t="n">
         <v>12.4233</v>
       </c>
+      <c r="AV6" s="3" t="n">
+        <v>12.4233</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4064,6 +4130,9 @@
       <c r="AU7" s="3" t="n">
         <v>33.9176</v>
       </c>
+      <c r="AV7" s="3" t="n">
+        <v>33.9176</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4213,6 +4282,9 @@
       <c r="AU8" s="3" t="n">
         <v>33.4768</v>
       </c>
+      <c r="AV8" s="3" t="n">
+        <v>33.4768</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4356,6 +4428,9 @@
       <c r="AU9" s="3" t="n">
         <v>42.1536</v>
       </c>
+      <c r="AV9" s="3" t="n">
+        <v>42.1536</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4499,6 +4574,9 @@
       <c r="AU10" s="3" t="n">
         <v>47.2455</v>
       </c>
+      <c r="AV10" s="3" t="n">
+        <v>47.2455</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4642,6 +4720,9 @@
       <c r="AU11" s="3" t="n">
         <v>105.991</v>
       </c>
+      <c r="AV11" s="3" t="n">
+        <v>105.991</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4791,6 +4872,9 @@
       <c r="AU12" s="3" t="n">
         <v>226.497</v>
       </c>
+      <c r="AV12" s="3" t="n">
+        <v>226.497</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4940,6 +5024,9 @@
       <c r="AU13" s="3" t="n">
         <v>20.615</v>
       </c>
+      <c r="AV13" s="3" t="n">
+        <v>20.615</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5083,6 +5170,9 @@
       <c r="AU14" s="3" t="n">
         <v>40.1296</v>
       </c>
+      <c r="AV14" s="3" t="n">
+        <v>40.1296</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5232,6 +5322,9 @@
       <c r="AU15" s="3" t="n">
         <v>12.03</v>
       </c>
+      <c r="AV15" s="3" t="n">
+        <v>12.03</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5375,6 +5468,9 @@
       <c r="AU16" s="3" t="n">
         <v>24.9541</v>
       </c>
+      <c r="AV16" s="3" t="n">
+        <v>24.9541</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5518,6 +5614,9 @@
       <c r="AU17" s="3" t="n">
         <v>16.8426</v>
       </c>
+      <c r="AV17" s="3" t="n">
+        <v>16.8426</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5667,6 +5766,9 @@
       <c r="AU18" s="3" t="n">
         <v>45.33</v>
       </c>
+      <c r="AV18" s="3" t="n">
+        <v>45.33</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5810,6 +5912,9 @@
       <c r="AU19" s="3" t="n">
         <v>15.0267</v>
       </c>
+      <c r="AV19" s="3" t="n">
+        <v>15.0267</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5959,6 +6064,9 @@
       <c r="AU20" s="3" t="n">
         <v>9.41</v>
       </c>
+      <c r="AV20" s="3" t="n">
+        <v>9.41</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -6108,6 +6216,9 @@
       <c r="AU21" s="3" t="n">
         <v>111.1739</v>
       </c>
+      <c r="AV21" s="3" t="n">
+        <v>111.1739</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -6251,6 +6362,9 @@
       <c r="AU22" s="3" t="n">
         <v>45.876</v>
       </c>
+      <c r="AV22" s="3" t="n">
+        <v>45.876</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -6400,6 +6514,9 @@
       <c r="AU23" s="3" t="n">
         <v>63.7762</v>
       </c>
+      <c r="AV23" s="3" t="n">
+        <v>63.7762</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -6543,6 +6660,9 @@
       <c r="AU24" s="3" t="n">
         <v>28.3764</v>
       </c>
+      <c r="AV24" s="3" t="n">
+        <v>28.3764</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -6689,6 +6809,9 @@
       <c r="AU25" s="3" t="n">
         <v>11.7358</v>
       </c>
+      <c r="AV25" s="3" t="n">
+        <v>11.7358</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -6835,6 +6958,9 @@
       <c r="AU26" s="3" t="n">
         <v>9.218</v>
       </c>
+      <c r="AV26" s="3" t="n">
+        <v>9.218</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6984,6 +7110,9 @@
       <c r="AU27" s="3" t="n">
         <v>65.55629999999999</v>
       </c>
+      <c r="AV27" s="3" t="n">
+        <v>65.55629999999999</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -7133,6 +7262,9 @@
       <c r="AU28" s="3" t="n">
         <v>109.0277</v>
       </c>
+      <c r="AV28" s="3" t="n">
+        <v>109.0277</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -7276,6 +7408,9 @@
       <c r="AU29" s="3" t="n">
         <v>12.5655</v>
       </c>
+      <c r="AV29" s="3" t="n">
+        <v>12.5655</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -7419,6 +7554,9 @@
       <c r="AU30" s="3" t="n">
         <v>16.475</v>
       </c>
+      <c r="AV30" s="3" t="n">
+        <v>16.475</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -7565,6 +7703,9 @@
       <c r="AU31" s="3" t="n">
         <v>423.5517</v>
       </c>
+      <c r="AV31" s="3" t="n">
+        <v>423.5517</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -7714,6 +7855,9 @@
       <c r="AU32" s="3" t="n">
         <v>10.54</v>
       </c>
+      <c r="AV32" s="3" t="n">
+        <v>10.54</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -7857,6 +8001,9 @@
       <c r="AU33" s="3" t="n">
         <v>18.74</v>
       </c>
+      <c r="AV33" s="3" t="n">
+        <v>18.74</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -8003,6 +8150,9 @@
       <c r="AU34" s="3" t="n">
         <v>209.7188</v>
       </c>
+      <c r="AV34" s="3" t="n">
+        <v>209.7188</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -8149,6 +8299,9 @@
       <c r="AU35" s="3" t="n">
         <v>15.06</v>
       </c>
+      <c r="AV35" s="3" t="n">
+        <v>15.06</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -8295,6 +8448,9 @@
       <c r="AU36" s="3" t="n">
         <v>360.6164</v>
       </c>
+      <c r="AV36" s="3" t="n">
+        <v>360.6164</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -8441,6 +8597,9 @@
       <c r="AU37" s="3" t="n">
         <v>16.095</v>
       </c>
+      <c r="AV37" s="3" t="n">
+        <v>16.095</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -8584,6 +8743,9 @@
       <c r="AU38" s="3" t="n">
         <v>14.3497</v>
       </c>
+      <c r="AV38" s="3" t="n">
+        <v>14.3497</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -8727,6 +8889,9 @@
       <c r="AU39" s="3" t="n">
         <v>1019.0919</v>
       </c>
+      <c r="AV39" s="3" t="n">
+        <v>1019.0919</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -8871,6 +9036,9 @@
         <v>21.403</v>
       </c>
       <c r="AU40" s="3" t="n">
+        <v>21.403</v>
+      </c>
+      <c r="AV40" s="3" t="n">
         <v>21.403</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily portfolio update 2026-06-23
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-22 07:22 IST</t>
+          <t>Generated: 2026-06-23 06:05 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4960163.8993248</v>
+        <v>4996454.8331916</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>490163.8993247999</v>
+        <v>526454.8331915997</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.10965635331651</v>
+        <v>0.1177751304679194</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>563004.5028381348</v>
+        <v>561157.5029830933</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-27777.51716186525</v>
+        <v>-29624.51701690676</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.04701821690826889</v>
+        <v>-0.05014458127365954</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5523168.402162935</v>
+        <v>5557612.336174693</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>462386.3821629351</v>
+        <v>496830.3161746934</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.0913665872854439</v>
+        <v>0.09817263699784751</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-06-22</t>
+          <t>Last snapshot: 2026-06-23</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU19"/>
+  <dimension ref="A1:AV19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -666,6 +666,7 @@
     <col width="21" customWidth="1" min="45" max="45"/>
     <col width="21" customWidth="1" min="46" max="46"/>
     <col width="21" customWidth="1" min="47" max="47"/>
+    <col width="21" customWidth="1" min="48" max="48"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -904,6 +905,11 @@
           <t>2026-06-22</t>
         </is>
       </c>
+      <c r="AV1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -923,13 +929,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>564</v>
+        <v>564.75</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>45120</v>
+        <v>45180</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1302.489999999998</v>
+        <v>1362.489999999998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1050,6 +1056,9 @@
       </c>
       <c r="AU2" s="3" t="n">
         <v>564</v>
+      </c>
+      <c r="AV2" s="3" t="n">
+        <v>564.75</v>
       </c>
     </row>
     <row r="3">
@@ -1225,6 +1234,9 @@
       <c r="AU4" s="3" t="n">
         <v>1560.300048828125</v>
       </c>
+      <c r="AV4" s="3" t="n">
+        <v>1560.300048828125</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1244,13 +1256,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>665.7000122070312</v>
+        <v>659.2999877929688</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13314.00024414062</v>
+        <v>13185.99975585938</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-899.0997558593754</v>
+        <v>-1027.100244140625</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1371,6 +1383,9 @@
       </c>
       <c r="AU5" s="3" t="n">
         <v>665.7000122070312</v>
+      </c>
+      <c r="AV5" s="3" t="n">
+        <v>659.2999877929688</v>
       </c>
     </row>
     <row r="6">
@@ -1391,13 +1406,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>389.8500061035156</v>
+        <v>383.6000061035156</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15594.00024414062</v>
+        <v>15344.00024414062</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-1908.239755859377</v>
+        <v>-2158.239755859377</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1518,6 +1533,9 @@
       </c>
       <c r="AU6" s="3" t="n">
         <v>389.8500061035156</v>
+      </c>
+      <c r="AV6" s="3" t="n">
+        <v>383.6000061035156</v>
       </c>
     </row>
     <row r="7">
@@ -1538,13 +1556,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>258.4200134277344</v>
+        <v>262.989990234375</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>25842.00134277344</v>
+        <v>26298.9990234375</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-591.8186572265622</v>
+        <v>-134.8209765624997</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1665,6 +1683,9 @@
       </c>
       <c r="AU7" s="3" t="n">
         <v>258.4200134277344</v>
+      </c>
+      <c r="AV7" s="3" t="n">
+        <v>262.989990234375</v>
       </c>
     </row>
     <row r="8">
@@ -1712,13 +1733,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>18.51000022888184</v>
+        <v>18.02000045776367</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>27765.00034332275</v>
+        <v>27030.00068664551</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-3285.169656677244</v>
+        <v>-4020.16931335449</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1839,6 +1860,9 @@
       </c>
       <c r="AU9" s="3" t="n">
         <v>18.51000022888184</v>
+      </c>
+      <c r="AV9" s="3" t="n">
+        <v>18.02000045776367</v>
       </c>
     </row>
     <row r="10">
@@ -1859,13 +1883,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>418.3999938964844</v>
+        <v>418.2000122070312</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>41839.99938964844</v>
+        <v>41820.00122070312</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-9658.480610351566</v>
+        <v>-9678.478779296878</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -1986,6 +2010,9 @@
       </c>
       <c r="AU10" s="3" t="n">
         <v>418.3999938964844</v>
+      </c>
+      <c r="AV10" s="3" t="n">
+        <v>418.2000122070312</v>
       </c>
     </row>
     <row r="11">
@@ -2006,13 +2033,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>8.949999809265137</v>
+        <v>8.890000343322754</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>8949.999809265137</v>
+        <v>8890.000343322754</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-891.2101907348624</v>
+        <v>-951.2096566772452</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -2133,6 +2160,9 @@
       </c>
       <c r="AU11" s="3" t="n">
         <v>8.949999809265137</v>
+      </c>
+      <c r="AV11" s="3" t="n">
+        <v>8.890000343322754</v>
       </c>
     </row>
     <row r="12">
@@ -2153,13 +2183,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2767.800048828125</v>
+        <v>2730.10009765625</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>27678.00048828125</v>
+        <v>27301.0009765625</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-45.24951171875</v>
+        <v>-422.2490234375</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -2280,6 +2310,9 @@
       </c>
       <c r="AU12" s="3" t="n">
         <v>2767.800048828125</v>
+      </c>
+      <c r="AV12" s="3" t="n">
+        <v>2730.10009765625</v>
       </c>
     </row>
     <row r="13">
@@ -2300,13 +2333,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>59.5</v>
+        <v>59.11000061035156</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>35700</v>
+        <v>35466.00036621094</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>668.239999999998</v>
+        <v>434.2403662109355</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -2427,6 +2460,9 @@
       </c>
       <c r="AU13" s="3" t="n">
         <v>59.5</v>
+      </c>
+      <c r="AV13" s="3" t="n">
+        <v>59.11000061035156</v>
       </c>
     </row>
     <row r="14">
@@ -2447,13 +2483,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>726.4000244140625</v>
+        <v>731.0999755859375</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>36320.00122070312</v>
+        <v>36554.99877929688</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-6142.508779296877</v>
+        <v>-5907.511220703127</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -2574,6 +2610,9 @@
       </c>
       <c r="AU14" s="3" t="n">
         <v>726.4000244140625</v>
+      </c>
+      <c r="AV14" s="3" t="n">
+        <v>731.0999755859375</v>
       </c>
     </row>
     <row r="15">
@@ -2648,13 +2687,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>629.0999755859375</v>
+        <v>621.2000122070312</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>31454.99877929688</v>
+        <v>31060.00061035156</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>9700.468779296876</v>
+        <v>9305.470610351564</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -2775,6 +2814,9 @@
       </c>
       <c r="AU17" s="3" t="n">
         <v>629.0999755859375</v>
+      </c>
+      <c r="AV17" s="3" t="n">
+        <v>621.2000122070312</v>
       </c>
     </row>
     <row r="18">
@@ -2795,13 +2837,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>404.5</v>
+        <v>400.5</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>40450</v>
+        <v>40050</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-6190.82</v>
+        <v>-6590.82</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -2922,6 +2964,9 @@
       </c>
       <c r="AU18" s="3" t="n">
         <v>404.5</v>
+      </c>
+      <c r="AV18" s="3" t="n">
+        <v>400.5</v>
       </c>
     </row>
     <row r="19">
@@ -2934,10 +2979,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>563004.5028381348</v>
+        <v>561157.5029830933</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-27777.51716186525</v>
+        <v>-29624.51701690675</v>
       </c>
     </row>
   </sheetData>
@@ -2951,7 +2996,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV41"/>
+  <dimension ref="A1:AW41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3002,6 +3047,7 @@
     <col width="13" customWidth="1" min="46" max="46"/>
     <col width="13" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
+    <col width="13" customWidth="1" min="49" max="49"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3245,6 +3291,11 @@
           <t>2026-06-22</t>
         </is>
       </c>
+      <c r="AW1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3269,16 +3320,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>57.0703</v>
+        <v>57.1333</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>64060.3844846</v>
+        <v>64131.1008506</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>14060.3844846</v>
+        <v>14131.1008506</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.281207689692</v>
+        <v>0.282622017012</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -3396,6 +3447,9 @@
       </c>
       <c r="AV2" s="3" t="n">
         <v>57.0703</v>
+      </c>
+      <c r="AW2" s="3" t="n">
+        <v>57.1333</v>
       </c>
     </row>
     <row r="3">
@@ -3421,16 +3475,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.31</v>
+        <v>25.3824</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>62141.44103</v>
+        <v>62319.19845120001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>2141.441030000002</v>
+        <v>2319.198451200005</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.03569068383333336</v>
+        <v>0.03865330752000009</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -3542,6 +3596,9 @@
       </c>
       <c r="AV3" s="3" t="n">
         <v>25.31</v>
+      </c>
+      <c r="AW3" s="3" t="n">
+        <v>25.3824</v>
       </c>
     </row>
     <row r="4">
@@ -3567,16 +3624,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.37</v>
+        <v>12.59</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>237579.37041</v>
+        <v>241804.71087</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>57579.37041</v>
+        <v>61804.71087000001</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3198853911666667</v>
+        <v>0.3433595048333334</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -3688,6 +3745,9 @@
       </c>
       <c r="AV4" s="3" t="n">
         <v>12.37</v>
+      </c>
+      <c r="AW4" s="3" t="n">
+        <v>12.59</v>
       </c>
     </row>
     <row r="5">
@@ -3713,16 +3773,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.5047</v>
+        <v>9.4948</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>174450.1002136</v>
+        <v>174268.3947424</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-35549.8997864</v>
+        <v>-35731.60525760002</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1692852370780952</v>
+        <v>-0.1701505012266668</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -3834,6 +3894,9 @@
       </c>
       <c r="AV5" s="3" t="n">
         <v>9.5047</v>
+      </c>
+      <c r="AW5" s="3" t="n">
+        <v>9.4948</v>
       </c>
     </row>
     <row r="6">
@@ -3859,16 +3922,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.4233</v>
+        <v>12.4869</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>52537.84996409999</v>
+        <v>52806.8129013</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>2537.849964099994</v>
+        <v>2806.8129013</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.05075699928199989</v>
+        <v>0.056136258026</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -3986,6 +4049,9 @@
       </c>
       <c r="AV6" s="3" t="n">
         <v>12.4233</v>
+      </c>
+      <c r="AW6" s="3" t="n">
+        <v>12.4869</v>
       </c>
     </row>
     <row r="7">
@@ -4011,16 +4077,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.9176</v>
+        <v>34.1109</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>74823.582304</v>
+        <v>75250.009836</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>14823.582304</v>
+        <v>15250.009836</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2470597050666666</v>
+        <v>0.2541668305999999</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -4132,6 +4198,9 @@
       </c>
       <c r="AV7" s="3" t="n">
         <v>33.9176</v>
+      </c>
+      <c r="AW7" s="3" t="n">
+        <v>34.1109</v>
       </c>
     </row>
     <row r="8">
@@ -4157,16 +4226,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>33.4768</v>
+        <v>33.5894</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>53716.6389424</v>
+        <v>53897.3161142</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>3716.638942400001</v>
+        <v>3897.316114199995</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.07433277884800002</v>
+        <v>0.07794632228399991</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -4284,6 +4353,9 @@
       </c>
       <c r="AV8" s="3" t="n">
         <v>33.4768</v>
+      </c>
+      <c r="AW8" s="3" t="n">
+        <v>33.5894</v>
       </c>
     </row>
     <row r="9">
@@ -4309,16 +4381,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>42.1536</v>
+        <v>43.6783</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>135709.0047648</v>
+        <v>140617.6132719</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>35709.00476479999</v>
+        <v>40617.61327190002</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3570900476479999</v>
+        <v>0.4061761327190002</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -4430,6 +4502,9 @@
       </c>
       <c r="AV9" s="3" t="n">
         <v>42.1536</v>
+      </c>
+      <c r="AW9" s="3" t="n">
+        <v>43.6783</v>
       </c>
     </row>
     <row r="10">
@@ -4455,16 +4530,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>47.2455</v>
+        <v>47.3715</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>134491.8277845</v>
+        <v>134850.5068185</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>34491.8277845</v>
+        <v>34850.5068185</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.344918277845</v>
+        <v>0.348505068185</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -4576,6 +4651,9 @@
       </c>
       <c r="AV10" s="3" t="n">
         <v>47.2455</v>
+      </c>
+      <c r="AW10" s="3" t="n">
+        <v>47.3715</v>
       </c>
     </row>
     <row r="11">
@@ -4601,16 +4679,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>105.991</v>
+        <v>105.2956</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31894.705729</v>
+        <v>31685.4466564</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1894.705728999998</v>
+        <v>1685.446656399996</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.06315685763333324</v>
+        <v>0.05618155521333319</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -4722,6 +4800,9 @@
       </c>
       <c r="AV11" s="3" t="n">
         <v>105.991</v>
+      </c>
+      <c r="AW11" s="3" t="n">
+        <v>105.2956</v>
       </c>
     </row>
     <row r="12">
@@ -4747,16 +4828,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>226.497</v>
+        <v>227.616</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>105439.336434</v>
+        <v>105960.255552</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>5439.336434000012</v>
+        <v>5960.255552000002</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.05439336434000012</v>
+        <v>0.05960255552000002</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -4874,6 +4955,9 @@
       </c>
       <c r="AV12" s="3" t="n">
         <v>226.497</v>
+      </c>
+      <c r="AW12" s="3" t="n">
+        <v>227.616</v>
       </c>
     </row>
     <row r="13">
@@ -4899,16 +4983,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>20.615</v>
+        <v>20.655</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>238878.477075</v>
+        <v>239341.981275</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>38878.47707499997</v>
+        <v>39341.981275</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.1943923853749999</v>
+        <v>0.196709906375</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -5026,6 +5110,9 @@
       </c>
       <c r="AV13" s="3" t="n">
         <v>20.615</v>
+      </c>
+      <c r="AW13" s="3" t="n">
+        <v>20.655</v>
       </c>
     </row>
     <row r="14">
@@ -5051,16 +5138,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>40.1296</v>
+        <v>40.4924</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>144771.7857376</v>
+        <v>146080.6251944</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>44771.78573760003</v>
+        <v>46080.62519440003</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.4477178573760003</v>
+        <v>0.4608062519440003</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -5172,6 +5259,9 @@
       </c>
       <c r="AV14" s="3" t="n">
         <v>40.1296</v>
+      </c>
+      <c r="AW14" s="3" t="n">
+        <v>40.4924</v>
       </c>
     </row>
     <row r="15">
@@ -5197,16 +5287,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>12.03</v>
+        <v>12.21</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>117219.68241</v>
+        <v>118973.59287</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>17219.68240999999</v>
+        <v>18973.59287000001</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1721968241</v>
+        <v>0.1897359287000001</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -5324,6 +5414,9 @@
       </c>
       <c r="AV15" s="3" t="n">
         <v>12.03</v>
+      </c>
+      <c r="AW15" s="3" t="n">
+        <v>12.21</v>
       </c>
     </row>
     <row r="16">
@@ -5349,16 +5442,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.9541</v>
+        <v>24.9618</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>142810.5176048</v>
+        <v>142854.5841504</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>42810.5176048</v>
+        <v>42854.58415040001</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.428105176048</v>
+        <v>0.4285458415040001</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -5470,6 +5563,9 @@
       </c>
       <c r="AV16" s="3" t="n">
         <v>24.9541</v>
+      </c>
+      <c r="AW16" s="3" t="n">
+        <v>24.9618</v>
       </c>
     </row>
     <row r="17">
@@ -5495,16 +5591,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.8426</v>
+        <v>16.8589</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55682.5956282</v>
+        <v>55736.48435729999</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5682.595628199997</v>
+        <v>5736.484357299989</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1136519125639999</v>
+        <v>0.1147296871459998</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -5616,6 +5712,9 @@
       </c>
       <c r="AV17" s="3" t="n">
         <v>16.8426</v>
+      </c>
+      <c r="AW17" s="3" t="n">
+        <v>16.8589</v>
       </c>
     </row>
     <row r="18">
@@ -5641,16 +5740,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>45.33</v>
+        <v>45.88</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>85512.14387999999</v>
+        <v>86549.68368</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>5512.143879999989</v>
+        <v>6549.683680000002</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.06890179849999986</v>
+        <v>0.08187104600000003</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -5768,6 +5867,9 @@
       </c>
       <c r="AV18" s="3" t="n">
         <v>45.33</v>
+      </c>
+      <c r="AW18" s="3" t="n">
+        <v>45.88</v>
       </c>
     </row>
     <row r="19">
@@ -5793,16 +5895,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>15.0267</v>
+        <v>15.286</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>217387.7526522</v>
+        <v>221138.985076</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>67387.7526522</v>
+        <v>71138.98507599998</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.449251684348</v>
+        <v>0.4742599005066666</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -5914,6 +6016,9 @@
       </c>
       <c r="AV19" s="3" t="n">
         <v>15.0267</v>
+      </c>
+      <c r="AW19" s="3" t="n">
+        <v>15.286</v>
       </c>
     </row>
     <row r="20">
@@ -5939,16 +6044,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.41</v>
+        <v>9.48</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>247067.10623</v>
+        <v>248905.01244</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-2932.893769999995</v>
+        <v>-1094.98755999998</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.01173157507999998</v>
+        <v>-0.004379950239999918</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -6066,6 +6171,9 @@
       </c>
       <c r="AV20" s="3" t="n">
         <v>9.41</v>
+      </c>
+      <c r="AW20" s="3" t="n">
+        <v>9.48</v>
       </c>
     </row>
     <row r="21">
@@ -6091,16 +6199,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>111.1739</v>
+        <v>111.8294</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>168901.9481401</v>
+        <v>169897.8224146</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-1098.051859900006</v>
+        <v>-102.1775854000007</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.006459128587647095</v>
+        <v>-0.000601044620000004</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -6218,6 +6326,9 @@
       </c>
       <c r="AV21" s="3" t="n">
         <v>111.1739</v>
+      </c>
+      <c r="AW21" s="3" t="n">
+        <v>111.8294</v>
       </c>
     </row>
     <row r="22">
@@ -6243,16 +6354,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>45.876</v>
+        <v>46.26</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>70394.88696</v>
+        <v>70984.11960000001</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>10394.88696</v>
+        <v>10984.11960000001</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1732481160000001</v>
+        <v>0.1830686600000001</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -6364,6 +6475,9 @@
       </c>
       <c r="AV22" s="3" t="n">
         <v>45.876</v>
+      </c>
+      <c r="AW22" s="3" t="n">
+        <v>46.26</v>
       </c>
     </row>
     <row r="23">
@@ -6389,16 +6503,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>63.7762</v>
+        <v>64.56019999999999</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>173245.9426854</v>
+        <v>175375.6528134</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>23245.94268540002</v>
+        <v>25375.6528134</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.1549729512360001</v>
+        <v>0.169171018756</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -6516,6 +6630,9 @@
       </c>
       <c r="AV23" s="3" t="n">
         <v>63.7762</v>
+      </c>
+      <c r="AW23" s="3" t="n">
+        <v>64.56019999999999</v>
       </c>
     </row>
     <row r="24">
@@ -6541,16 +6658,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>28.3764</v>
+        <v>28.5126</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>103102.4144904</v>
+        <v>103597.2816636</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>3102.414490399999</v>
+        <v>3597.281663599992</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.03102414490399999</v>
+        <v>0.03597281663599992</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -6662,6 +6779,9 @@
       </c>
       <c r="AV24" s="3" t="n">
         <v>28.3764</v>
+      </c>
+      <c r="AW24" s="3" t="n">
+        <v>28.5126</v>
       </c>
     </row>
     <row r="25">
@@ -6687,16 +6807,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.7358</v>
+        <v>11.7959</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>192721.4817292</v>
+        <v>193708.4243366</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-7278.518270800036</v>
+        <v>-6291.575663400028</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.03639259135400018</v>
+        <v>-0.03145787831700014</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -6811,6 +6931,9 @@
       </c>
       <c r="AV25" s="3" t="n">
         <v>11.7358</v>
+      </c>
+      <c r="AW25" s="3" t="n">
+        <v>11.7959</v>
       </c>
     </row>
     <row r="26">
@@ -6836,16 +6959,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>9.218</v>
+        <v>9.2803</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>110078.72887</v>
+        <v>110822.6977145</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>78.72887000000628</v>
+        <v>822.6977145000128</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.0007157170000000571</v>
+        <v>0.007479070131818298</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -6960,6 +7083,9 @@
       </c>
       <c r="AV26" s="3" t="n">
         <v>9.218</v>
+      </c>
+      <c r="AW26" s="3" t="n">
+        <v>9.2803</v>
       </c>
     </row>
     <row r="27">
@@ -6985,16 +7111,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>65.55629999999999</v>
+        <v>65.3536</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>105602.021418</v>
+        <v>105275.500096</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-4397.978582000011</v>
+        <v>-4724.499904000011</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.03998162347272737</v>
+        <v>-0.04294999912727283</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -7112,6 +7238,9 @@
       </c>
       <c r="AV27" s="3" t="n">
         <v>65.55629999999999</v>
+      </c>
+      <c r="AW27" s="3" t="n">
+        <v>65.3536</v>
       </c>
     </row>
     <row r="28">
@@ -7137,16 +7266,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>109.0277</v>
+        <v>109.4567</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>360517.2073989</v>
+        <v>361935.7632519</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-19482.79260109999</v>
+        <v>-18064.23674809997</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.05127050684499999</v>
+        <v>-0.04753746512657886</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -7264,6 +7393,9 @@
       </c>
       <c r="AV28" s="3" t="n">
         <v>109.0277</v>
+      </c>
+      <c r="AW28" s="3" t="n">
+        <v>109.4567</v>
       </c>
     </row>
     <row r="29">
@@ -7289,16 +7421,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.5655</v>
+        <v>12.7503</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>120675.3300465</v>
+        <v>122450.0943609</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>20675.33004649999</v>
+        <v>22450.09436089998</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.2067533004649999</v>
+        <v>0.2245009436089998</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -7410,6 +7542,9 @@
       </c>
       <c r="AV29" s="3" t="n">
         <v>12.5655</v>
+      </c>
+      <c r="AW29" s="3" t="n">
+        <v>12.7503</v>
       </c>
     </row>
     <row r="30">
@@ -7435,16 +7570,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>16.475</v>
+        <v>16.5965</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>121846.809975</v>
+        <v>122745.4070865</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>21846.80997500001</v>
+        <v>22745.4070865</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.2184680997500001</v>
+        <v>0.227454070865</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -7556,6 +7691,9 @@
       </c>
       <c r="AV30" s="3" t="n">
         <v>16.475</v>
+      </c>
+      <c r="AW30" s="3" t="n">
+        <v>16.5965</v>
       </c>
     </row>
     <row r="31">
@@ -7581,16 +7719,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>423.5517</v>
+        <v>427.8476</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>112698.636336</v>
+        <v>113841.689408</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>12698.63633599998</v>
+        <v>13841.68940799999</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.1269863633599998</v>
+        <v>0.1384168940799999</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -7705,6 +7843,9 @@
       </c>
       <c r="AV31" s="3" t="n">
         <v>423.5517</v>
+      </c>
+      <c r="AW31" s="3" t="n">
+        <v>427.8476</v>
       </c>
     </row>
     <row r="32">
@@ -7730,16 +7871,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.54</v>
+        <v>10.61</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>222815.1784</v>
+        <v>224294.9756</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>22815.17839999998</v>
+        <v>24294.97559999998</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.1140758919999999</v>
+        <v>0.1214748779999999</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -7857,6 +7998,9 @@
       </c>
       <c r="AV32" s="3" t="n">
         <v>10.54</v>
+      </c>
+      <c r="AW32" s="3" t="n">
+        <v>10.61</v>
       </c>
     </row>
     <row r="33">
@@ -7882,16 +8026,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>18.74</v>
+        <v>18.94</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>67157.41359999999</v>
+        <v>67874.1416</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>7157.413599999985</v>
+        <v>7874.141600000003</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.1192902266666664</v>
+        <v>0.1312356933333334</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -8003,6 +8147,9 @@
       </c>
       <c r="AV33" s="3" t="n">
         <v>18.74</v>
+      </c>
+      <c r="AW33" s="3" t="n">
+        <v>18.94</v>
       </c>
     </row>
     <row r="34">
@@ -8028,16 +8175,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>209.7188</v>
+        <v>210.1832</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>73722.65948279999</v>
+        <v>73885.9104792</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-6277.340517200006</v>
+        <v>-6114.0895208</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.07846675646500006</v>
+        <v>-0.07642611901</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -8152,6 +8299,9 @@
       </c>
       <c r="AV34" s="3" t="n">
         <v>209.7188</v>
+      </c>
+      <c r="AW34" s="3" t="n">
+        <v>210.1832</v>
       </c>
     </row>
     <row r="35">
@@ -8177,16 +8327,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>15.06</v>
+        <v>15.18</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>107459.47038</v>
+        <v>108315.72114</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>7459.470379999999</v>
+        <v>8315.721139999994</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.0745947038</v>
+        <v>0.08315721139999994</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -8301,6 +8451,9 @@
       </c>
       <c r="AV35" s="3" t="n">
         <v>15.06</v>
+      </c>
+      <c r="AW35" s="3" t="n">
+        <v>15.18</v>
       </c>
     </row>
     <row r="36">
@@ -8326,16 +8479,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>360.6164</v>
+        <v>362.1997</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>167941.2211784</v>
+        <v>168678.5734882</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>17941.22117840001</v>
+        <v>18678.5734882</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1196081411893334</v>
+        <v>0.1245238232546666</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -8450,6 +8603,9 @@
       </c>
       <c r="AV36" s="3" t="n">
         <v>360.6164</v>
+      </c>
+      <c r="AW36" s="3" t="n">
+        <v>362.1997</v>
       </c>
     </row>
     <row r="37">
@@ -8475,16 +8631,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>16.095</v>
+        <v>16.177</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>60563.698455</v>
+        <v>60872.255353</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>10563.698455</v>
+        <v>10872.255353</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.2112739691</v>
+        <v>0.21744510706</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -8599,6 +8755,9 @@
       </c>
       <c r="AV37" s="3" t="n">
         <v>16.095</v>
+      </c>
+      <c r="AW37" s="3" t="n">
+        <v>16.177</v>
       </c>
     </row>
     <row r="38">
@@ -8624,16 +8783,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>14.3497</v>
+        <v>14.4161</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>85818.1225554</v>
+        <v>86215.2265602</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>5818.122555399998</v>
+        <v>6215.226560199997</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.07272653194249996</v>
+        <v>0.07769033200249996</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -8745,6 +8904,9 @@
       </c>
       <c r="AV38" s="3" t="n">
         <v>14.3497</v>
+      </c>
+      <c r="AW38" s="3" t="n">
+        <v>14.4161</v>
       </c>
     </row>
     <row r="39">
@@ -8770,16 +8932,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1019.0919</v>
+        <v>1019.7809</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50833.3230639</v>
+        <v>50867.6910729</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>833.323063900003</v>
+        <v>867.691072900001</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.01666646127800006</v>
+        <v>0.01735382145800002</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -8891,6 +9053,9 @@
       </c>
       <c r="AV39" s="3" t="n">
         <v>1019.0919</v>
+      </c>
+      <c r="AW39" s="3" t="n">
+        <v>1019.7809</v>
       </c>
     </row>
     <row r="40">
@@ -8916,16 +9081,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>21.403</v>
+        <v>21.3535</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>107893.100881</v>
+        <v>107643.5700445</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>7893.100880999991</v>
+        <v>7643.570044499997</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.07893100880999991</v>
+        <v>0.07643570044499996</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -9040,6 +9205,9 @@
       </c>
       <c r="AV40" s="3" t="n">
         <v>21.403</v>
+      </c>
+      <c r="AW40" s="3" t="n">
+        <v>21.3535</v>
       </c>
     </row>
     <row r="41">
@@ -9052,13 +9220,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4960163.8993248</v>
+        <v>4996454.8331916</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>490163.8993247999</v>
+        <v>526454.8331915999</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.10965635331651</v>
+        <v>0.1177751304679194</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-06-24
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-23 06:05 IST</t>
+          <t>Generated: 2026-06-24 06:05 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4996454.8331916</v>
+        <v>4944604.1767516</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>526454.8331915997</v>
+        <v>474604.1767515996</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1177751304679194</v>
+        <v>0.1061754310406263</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>561157.5029830933</v>
+        <v>556358.5018234253</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-29624.51701690676</v>
+        <v>-34423.51817657473</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.05014458127365954</v>
+        <v>-0.05826771467516009</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5557612.336174693</v>
+        <v>5500962.678575025</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>496830.3161746934</v>
+        <v>440180.6585750254</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.09817263699784751</v>
+        <v>0.08697878249556092</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-06-23</t>
+          <t>Last snapshot: 2026-06-24</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV19"/>
+  <dimension ref="A1:AW19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -667,6 +667,7 @@
     <col width="21" customWidth="1" min="46" max="46"/>
     <col width="21" customWidth="1" min="47" max="47"/>
     <col width="21" customWidth="1" min="48" max="48"/>
+    <col width="21" customWidth="1" min="49" max="49"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -910,6 +911,11 @@
           <t>2026-06-23</t>
         </is>
       </c>
+      <c r="AW1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -929,13 +935,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>564.75</v>
+        <v>552.2000122070312</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>45180</v>
+        <v>44176.0009765625</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1362.489999999998</v>
+        <v>358.490976562498</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1059,6 +1065,9 @@
       </c>
       <c r="AV2" s="3" t="n">
         <v>564.75</v>
+      </c>
+      <c r="AW2" s="3" t="n">
+        <v>552.2000122070312</v>
       </c>
     </row>
     <row r="3">
@@ -1106,13 +1115,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1560.300048828125</v>
+        <v>1531.199951171875</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>31206.0009765625</v>
+        <v>30623.9990234375</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-898.5790234375017</v>
+        <v>-1480.580976562502</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1236,6 +1245,9 @@
       </c>
       <c r="AV4" s="3" t="n">
         <v>1560.300048828125</v>
+      </c>
+      <c r="AW4" s="3" t="n">
+        <v>1531.199951171875</v>
       </c>
     </row>
     <row r="5">
@@ -1256,13 +1268,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>659.2999877929688</v>
+        <v>655.3499755859375</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13185.99975585938</v>
+        <v>13106.99951171875</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1027.100244140625</v>
+        <v>-1106.10048828125</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1386,6 +1398,9 @@
       </c>
       <c r="AV5" s="3" t="n">
         <v>659.2999877929688</v>
+      </c>
+      <c r="AW5" s="3" t="n">
+        <v>655.3499755859375</v>
       </c>
     </row>
     <row r="6">
@@ -1406,13 +1421,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>383.6000061035156</v>
+        <v>382.25</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15344.00024414062</v>
+        <v>15290</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2158.239755859377</v>
+        <v>-2212.240000000002</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1536,6 +1551,9 @@
       </c>
       <c r="AV6" s="3" t="n">
         <v>383.6000061035156</v>
+      </c>
+      <c r="AW6" s="3" t="n">
+        <v>382.25</v>
       </c>
     </row>
     <row r="7">
@@ -1556,13 +1574,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>262.989990234375</v>
+        <v>254.8999938964844</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>26298.9990234375</v>
+        <v>25489.99938964844</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-134.8209765624997</v>
+        <v>-943.8206103515622</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1686,6 +1704,9 @@
       </c>
       <c r="AV7" s="3" t="n">
         <v>262.989990234375</v>
+      </c>
+      <c r="AW7" s="3" t="n">
+        <v>254.8999938964844</v>
       </c>
     </row>
     <row r="8">
@@ -1733,13 +1754,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>18.02000045776367</v>
+        <v>17.82999992370605</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>27030.00068664551</v>
+        <v>26744.99988555908</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-4020.16931335449</v>
+        <v>-4305.170114440916</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1863,6 +1884,9 @@
       </c>
       <c r="AV9" s="3" t="n">
         <v>18.02000045776367</v>
+      </c>
+      <c r="AW9" s="3" t="n">
+        <v>17.82999992370605</v>
       </c>
     </row>
     <row r="10">
@@ -1883,13 +1907,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>418.2000122070312</v>
+        <v>414.6000061035156</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>41820.00122070312</v>
+        <v>41460.00061035156</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-9678.478779296878</v>
+        <v>-10038.47938964844</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -2013,6 +2037,9 @@
       </c>
       <c r="AV10" s="3" t="n">
         <v>418.2000122070312</v>
+      </c>
+      <c r="AW10" s="3" t="n">
+        <v>414.6000061035156</v>
       </c>
     </row>
     <row r="11">
@@ -2033,13 +2060,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>8.890000343322754</v>
+        <v>8.829999923706055</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>8890.000343322754</v>
+        <v>8829.999923706055</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-951.2096566772452</v>
+        <v>-1011.210076293944</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -2163,6 +2190,9 @@
       </c>
       <c r="AV11" s="3" t="n">
         <v>8.890000343322754</v>
+      </c>
+      <c r="AW11" s="3" t="n">
+        <v>8.829999923706055</v>
       </c>
     </row>
     <row r="12">
@@ -2183,13 +2213,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2730.10009765625</v>
+        <v>2741.60009765625</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>27301.0009765625</v>
+        <v>27416.0009765625</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-422.2490234375</v>
+        <v>-307.2490234375</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -2313,6 +2343,9 @@
       </c>
       <c r="AV12" s="3" t="n">
         <v>2730.10009765625</v>
+      </c>
+      <c r="AW12" s="3" t="n">
+        <v>2741.60009765625</v>
       </c>
     </row>
     <row r="13">
@@ -2333,13 +2366,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>59.11000061035156</v>
+        <v>57.90000152587891</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>35466.00036621094</v>
-      </c>
-      <c r="G13" s="4" t="n">
-        <v>434.2403662109355</v>
+        <v>34740.00091552734</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>-291.7590844726583</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -2463,6 +2496,9 @@
       </c>
       <c r="AV13" s="3" t="n">
         <v>59.11000061035156</v>
+      </c>
+      <c r="AW13" s="3" t="n">
+        <v>57.90000152587891</v>
       </c>
     </row>
     <row r="14">
@@ -2483,13 +2519,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>731.0999755859375</v>
+        <v>725.5</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>36554.99877929688</v>
+        <v>36275</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-5907.511220703127</v>
+        <v>-6187.510000000002</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -2613,6 +2649,9 @@
       </c>
       <c r="AV14" s="3" t="n">
         <v>731.0999755859375</v>
+      </c>
+      <c r="AW14" s="3" t="n">
+        <v>725.5</v>
       </c>
     </row>
     <row r="15">
@@ -2687,13 +2726,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>621.2000122070312</v>
+        <v>618.2999877929688</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>31060.00061035156</v>
+        <v>30914.99938964844</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>9305.470610351564</v>
+        <v>9160.469389648439</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -2817,6 +2856,9 @@
       </c>
       <c r="AV17" s="3" t="n">
         <v>621.2000122070312</v>
+      </c>
+      <c r="AW17" s="3" t="n">
+        <v>618.2999877929688</v>
       </c>
     </row>
     <row r="18">
@@ -2837,13 +2879,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>400.5</v>
+        <v>395.2000122070312</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>40050</v>
+        <v>39520.00122070312</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-6590.82</v>
+        <v>-7120.818779296875</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -2967,6 +3009,9 @@
       </c>
       <c r="AV18" s="3" t="n">
         <v>400.5</v>
+      </c>
+      <c r="AW18" s="3" t="n">
+        <v>395.2000122070312</v>
       </c>
     </row>
     <row r="19">
@@ -2979,10 +3024,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>561157.5029830933</v>
+        <v>556358.5018234253</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-29624.51701690675</v>
+        <v>-34423.51817657472</v>
       </c>
     </row>
   </sheetData>
@@ -2996,7 +3041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW41"/>
+  <dimension ref="A1:AX41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3007,7 +3052,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
@@ -3048,6 +3093,7 @@
     <col width="13" customWidth="1" min="47" max="47"/>
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="13" customWidth="1" min="49" max="49"/>
+    <col width="13" customWidth="1" min="50" max="50"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3296,6 +3342,11 @@
           <t>2026-06-23</t>
         </is>
       </c>
+      <c r="AX1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3320,16 +3371,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>57.1333</v>
+        <v>56.0437</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>64131.1008506</v>
+        <v>62908.0444634</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>14131.1008506</v>
+        <v>12908.0444634</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.282622017012</v>
+        <v>0.258160889268</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -3450,6 +3501,9 @@
       </c>
       <c r="AW2" s="3" t="n">
         <v>57.1333</v>
+      </c>
+      <c r="AX2" s="3" t="n">
+        <v>56.0437</v>
       </c>
     </row>
     <row r="3">
@@ -3475,16 +3529,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.3824</v>
+        <v>24.9866</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>62319.19845120001</v>
+        <v>61347.4251458</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>2319.198451200005</v>
+        <v>1347.4251458</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.03865330752000009</v>
+        <v>0.02245708576333333</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -3599,6 +3653,9 @@
       </c>
       <c r="AW3" s="3" t="n">
         <v>25.3824</v>
+      </c>
+      <c r="AX3" s="3" t="n">
+        <v>24.9866</v>
       </c>
     </row>
     <row r="4">
@@ -3624,16 +3681,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.59</v>
+        <v>12.12</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>241804.71087</v>
+        <v>232777.84716</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>61804.71087000001</v>
+        <v>52777.84716</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3433595048333334</v>
+        <v>0.293210262</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -3748,6 +3805,9 @@
       </c>
       <c r="AW4" s="3" t="n">
         <v>12.59</v>
+      </c>
+      <c r="AX4" s="3" t="n">
+        <v>12.12</v>
       </c>
     </row>
     <row r="5">
@@ -3773,16 +3833,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.4948</v>
+        <v>9.404</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>174268.3947424</v>
+        <v>172601.843552</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-35731.60525760002</v>
+        <v>-37398.15644799999</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1701505012266668</v>
+        <v>-0.1780864592761905</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -3897,6 +3957,9 @@
       </c>
       <c r="AW5" s="3" t="n">
         <v>9.4948</v>
+      </c>
+      <c r="AX5" s="3" t="n">
+        <v>9.404</v>
       </c>
     </row>
     <row r="6">
@@ -3922,16 +3985,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.4869</v>
+        <v>12.3758</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>52806.8129013</v>
+        <v>52336.97355659999</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>2806.8129013</v>
+        <v>2336.973556599994</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.056136258026</v>
+        <v>0.04673947113199989</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -4052,6 +4115,9 @@
       </c>
       <c r="AW6" s="3" t="n">
         <v>12.4869</v>
+      </c>
+      <c r="AX6" s="3" t="n">
+        <v>12.3758</v>
       </c>
     </row>
     <row r="7">
@@ -4077,16 +4143,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>34.1109</v>
+        <v>33.8215</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>75250.009836</v>
+        <v>74611.58186000001</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>15250.009836</v>
+        <v>14611.58186000001</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2541668305999999</v>
+        <v>0.2435263643333334</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -4201,6 +4267,9 @@
       </c>
       <c r="AW7" s="3" t="n">
         <v>34.1109</v>
+      </c>
+      <c r="AX7" s="3" t="n">
+        <v>33.8215</v>
       </c>
     </row>
     <row r="8">
@@ -4226,16 +4295,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>33.5894</v>
+        <v>33.521</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>53897.3161142</v>
+        <v>53787.561953</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>3897.316114199995</v>
+        <v>3787.561953000004</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.07794632228399991</v>
+        <v>0.07575123906000009</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -4356,6 +4425,9 @@
       </c>
       <c r="AW8" s="3" t="n">
         <v>33.5894</v>
+      </c>
+      <c r="AX8" s="3" t="n">
+        <v>33.521</v>
       </c>
     </row>
     <row r="9">
@@ -4381,16 +4453,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>43.6783</v>
+        <v>42.0059</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>140617.6132719</v>
+        <v>135233.5004187</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>40617.61327190002</v>
+        <v>35233.50041869999</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.4061761327190002</v>
+        <v>0.3523350041869999</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -4505,6 +4577,9 @@
       </c>
       <c r="AW9" s="3" t="n">
         <v>43.6783</v>
+      </c>
+      <c r="AX9" s="3" t="n">
+        <v>42.0059</v>
       </c>
     </row>
     <row r="10">
@@ -4530,16 +4605,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>47.3715</v>
+        <v>47.0175</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>134850.5068185</v>
+        <v>133842.7895325</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>34850.5068185</v>
+        <v>33842.7895325</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.348505068185</v>
+        <v>0.338427895325</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -4654,6 +4729,9 @@
       </c>
       <c r="AW10" s="3" t="n">
         <v>47.3715</v>
+      </c>
+      <c r="AX10" s="3" t="n">
+        <v>47.0175</v>
       </c>
     </row>
     <row r="11">
@@ -4679,16 +4757,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>105.2956</v>
+        <v>102.7625</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31685.4466564</v>
+        <v>30923.1887375</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1685.446656399996</v>
+        <v>923.1887375000006</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.05618155521333319</v>
+        <v>0.03077295791666669</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -4803,6 +4881,9 @@
       </c>
       <c r="AW11" s="3" t="n">
         <v>105.2956</v>
+      </c>
+      <c r="AX11" s="3" t="n">
+        <v>102.7625</v>
       </c>
     </row>
     <row r="12">
@@ -4828,16 +4909,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>227.616</v>
+        <v>226.634</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>105960.255552</v>
+        <v>105503.112948</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>5960.255552000002</v>
+        <v>5503.112947999995</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.05960255552000002</v>
+        <v>0.05503112947999995</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -4958,6 +5039,9 @@
       </c>
       <c r="AW12" s="3" t="n">
         <v>227.616</v>
+      </c>
+      <c r="AX12" s="3" t="n">
+        <v>226.634</v>
       </c>
     </row>
     <row r="13">
@@ -4983,16 +5067,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>20.655</v>
+        <v>20.789</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>239341.981275</v>
+        <v>240894.720345</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>39341.981275</v>
+        <v>40894.72034500001</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.196709906375</v>
+        <v>0.204473601725</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -5113,6 +5197,9 @@
       </c>
       <c r="AW13" s="3" t="n">
         <v>20.655</v>
+      </c>
+      <c r="AX13" s="3" t="n">
+        <v>20.789</v>
       </c>
     </row>
     <row r="14">
@@ -5263,6 +5350,9 @@
       <c r="AW14" s="3" t="n">
         <v>40.4924</v>
       </c>
+      <c r="AX14" s="3" t="n">
+        <v>40.4924</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5287,16 +5377,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>12.21</v>
+        <v>12.14</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>118973.59287</v>
+        <v>118291.51658</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>18973.59287000001</v>
+        <v>18291.51658000001</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1897359287000001</v>
+        <v>0.1829151658000001</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -5417,6 +5507,9 @@
       </c>
       <c r="AW15" s="3" t="n">
         <v>12.21</v>
+      </c>
+      <c r="AX15" s="3" t="n">
+        <v>12.14</v>
       </c>
     </row>
     <row r="16">
@@ -5442,16 +5535,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.9618</v>
+        <v>24.1943</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>142854.5841504</v>
+        <v>138462.2369104</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>42854.58415040001</v>
+        <v>38462.23691039998</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4285458415040001</v>
+        <v>0.3846223691039998</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -5566,6 +5659,9 @@
       </c>
       <c r="AW16" s="3" t="n">
         <v>24.9618</v>
+      </c>
+      <c r="AX16" s="3" t="n">
+        <v>24.1943</v>
       </c>
     </row>
     <row r="17">
@@ -5591,16 +5687,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.8589</v>
+        <v>16.7199</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55736.48435729999</v>
+        <v>55276.94243429999</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5736.484357299989</v>
+        <v>5276.942434299992</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1147296871459998</v>
+        <v>0.1055388486859998</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -5715,6 +5811,9 @@
       </c>
       <c r="AW17" s="3" t="n">
         <v>16.8589</v>
+      </c>
+      <c r="AX17" s="3" t="n">
+        <v>16.7199</v>
       </c>
     </row>
     <row r="18">
@@ -5740,16 +5839,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>45.88</v>
+        <v>46.25</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>86549.68368</v>
+        <v>87247.66499999999</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>6549.683680000002</v>
+        <v>7247.664999999994</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.08187104600000003</v>
+        <v>0.09059581249999991</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -5870,6 +5969,9 @@
       </c>
       <c r="AW18" s="3" t="n">
         <v>45.88</v>
+      </c>
+      <c r="AX18" s="3" t="n">
+        <v>46.25</v>
       </c>
     </row>
     <row r="19">
@@ -6020,6 +6122,9 @@
       <c r="AW19" s="3" t="n">
         <v>15.286</v>
       </c>
+      <c r="AX19" s="3" t="n">
+        <v>15.286</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -6044,16 +6149,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.48</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>248905.01244</v>
+        <v>246016.87411</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-1094.98755999998</v>
+        <v>-3983.125890000025</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.004379950239999918</v>
+        <v>-0.0159325035600001</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -6174,6 +6279,9 @@
       </c>
       <c r="AW20" s="3" t="n">
         <v>9.48</v>
+      </c>
+      <c r="AX20" s="3" t="n">
+        <v>9.369999999999999</v>
       </c>
     </row>
     <row r="21">
@@ -6199,16 +6307,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>111.8294</v>
+        <v>111.0276</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>169897.8224146</v>
+        <v>168679.6805484</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-102.1775854000007</v>
+        <v>-1320.319451599993</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.000601044620000004</v>
+        <v>-0.007766585009411723</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -6329,6 +6437,9 @@
       </c>
       <c r="AW21" s="3" t="n">
         <v>111.8294</v>
+      </c>
+      <c r="AX21" s="3" t="n">
+        <v>111.0276</v>
       </c>
     </row>
     <row r="22">
@@ -6354,16 +6465,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>46.26</v>
+        <v>44.405</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>70984.11960000001</v>
+        <v>68137.69630000001</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>10984.11960000001</v>
+        <v>8137.696300000011</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1830686600000001</v>
+        <v>0.1356282716666669</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -6478,6 +6589,9 @@
       </c>
       <c r="AW22" s="3" t="n">
         <v>46.26</v>
+      </c>
+      <c r="AX22" s="3" t="n">
+        <v>44.405</v>
       </c>
     </row>
     <row r="23">
@@ -6503,16 +6617,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>64.56019999999999</v>
+        <v>64.1322</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>175375.6528134</v>
+        <v>174213.0049374</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>25375.6528134</v>
+        <v>24213.00493739999</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.169171018756</v>
+        <v>0.161420032916</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -6633,6 +6747,9 @@
       </c>
       <c r="AW23" s="3" t="n">
         <v>64.56019999999999</v>
+      </c>
+      <c r="AX23" s="3" t="n">
+        <v>64.1322</v>
       </c>
     </row>
     <row r="24">
@@ -6658,16 +6775,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>28.5126</v>
+        <v>28.0795</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>103597.2816636</v>
+        <v>102023.662187</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>3597.281663599992</v>
+        <v>2023.662186999994</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.03597281663599992</v>
+        <v>0.02023662186999994</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -6782,6 +6899,9 @@
       </c>
       <c r="AW24" s="3" t="n">
         <v>28.5126</v>
+      </c>
+      <c r="AX24" s="3" t="n">
+        <v>28.0795</v>
       </c>
     </row>
     <row r="25">
@@ -6807,16 +6927,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.7959</v>
+        <v>11.6442</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>193708.4243366</v>
+        <v>191217.2563908</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-6291.575663400028</v>
+        <v>-8782.743609200028</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.03145787831700014</v>
+        <v>-0.04391371804600014</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -6934,6 +7054,9 @@
       </c>
       <c r="AW25" s="3" t="n">
         <v>11.7959</v>
+      </c>
+      <c r="AX25" s="3" t="n">
+        <v>11.6442</v>
       </c>
     </row>
     <row r="26">
@@ -6959,16 +7082,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>9.2803</v>
+        <v>9.1143</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>110822.6977145</v>
-      </c>
-      <c r="H26" s="4" t="n">
-        <v>822.6977145000128</v>
-      </c>
-      <c r="I26" s="12" t="n">
-        <v>0.007479070131818298</v>
+        <v>108840.3730245</v>
+      </c>
+      <c r="H26" s="6" t="n">
+        <v>-1159.626975499996</v>
+      </c>
+      <c r="I26" s="13" t="n">
+        <v>-0.01054206341363633</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -7086,6 +7209,9 @@
       </c>
       <c r="AW26" s="3" t="n">
         <v>9.2803</v>
+      </c>
+      <c r="AX26" s="3" t="n">
+        <v>9.1143</v>
       </c>
     </row>
     <row r="27">
@@ -7111,16 +7237,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>65.3536</v>
+        <v>64.65130000000001</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>105275.500096</v>
+        <v>104144.193118</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-4724.499904000011</v>
+        <v>-5855.80688199999</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.04294999912727283</v>
+        <v>-0.05323460801818172</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -7241,6 +7367,9 @@
       </c>
       <c r="AW27" s="3" t="n">
         <v>65.3536</v>
+      </c>
+      <c r="AX27" s="3" t="n">
+        <v>64.65130000000001</v>
       </c>
     </row>
     <row r="28">
@@ -7266,16 +7395,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>109.4567</v>
+        <v>108.0557</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>361935.7632519</v>
+        <v>357303.1367949</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-18064.23674809997</v>
+        <v>-22696.8632051</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.04753746512657886</v>
+        <v>-0.05972858738184211</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -7396,6 +7525,9 @@
       </c>
       <c r="AW28" s="3" t="n">
         <v>109.4567</v>
+      </c>
+      <c r="AX28" s="3" t="n">
+        <v>108.0557</v>
       </c>
     </row>
     <row r="29">
@@ -7421,16 +7553,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.7503</v>
+        <v>12.6508</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>122450.0943609</v>
+        <v>121494.5259124</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>22450.09436089998</v>
+        <v>21494.5259124</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.2245009436089998</v>
+        <v>0.214945259124</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -7545,6 +7677,9 @@
       </c>
       <c r="AW29" s="3" t="n">
         <v>12.7503</v>
+      </c>
+      <c r="AX29" s="3" t="n">
+        <v>12.6508</v>
       </c>
     </row>
     <row r="30">
@@ -7570,16 +7705,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>16.5965</v>
+        <v>16.4926</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>122745.4070865</v>
+        <v>121976.9771286</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>22745.4070865</v>
+        <v>21976.97712859999</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.227454070865</v>
+        <v>0.2197697712859999</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -7694,6 +7829,9 @@
       </c>
       <c r="AW30" s="3" t="n">
         <v>16.5965</v>
+      </c>
+      <c r="AX30" s="3" t="n">
+        <v>16.4926</v>
       </c>
     </row>
     <row r="31">
@@ -7719,16 +7857,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>427.8476</v>
+        <v>423.4812</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>113841.689408</v>
+        <v>112679.877696</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>13841.68940799999</v>
+        <v>12679.877696</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.1384168940799999</v>
+        <v>0.12679877696</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -7846,6 +7984,9 @@
       </c>
       <c r="AW31" s="3" t="n">
         <v>427.8476</v>
+      </c>
+      <c r="AX31" s="3" t="n">
+        <v>423.4812</v>
       </c>
     </row>
     <row r="32">
@@ -7871,16 +8012,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.61</v>
+        <v>10.54</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>224294.9756</v>
+        <v>222815.1784</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>24294.97559999998</v>
+        <v>22815.17839999998</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.1214748779999999</v>
+        <v>0.1140758919999999</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -8001,6 +8142,9 @@
       </c>
       <c r="AW32" s="3" t="n">
         <v>10.61</v>
+      </c>
+      <c r="AX32" s="3" t="n">
+        <v>10.54</v>
       </c>
     </row>
     <row r="33">
@@ -8026,16 +8170,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>18.94</v>
+        <v>18.88</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>67874.1416</v>
+        <v>67659.12319999999</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>7874.141600000003</v>
+        <v>7659.123199999987</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.1312356933333334</v>
+        <v>0.1276520533333331</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -8150,6 +8294,9 @@
       </c>
       <c r="AW33" s="3" t="n">
         <v>18.94</v>
+      </c>
+      <c r="AX33" s="3" t="n">
+        <v>18.88</v>
       </c>
     </row>
     <row r="34">
@@ -8175,16 +8322,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>210.1832</v>
+        <v>207.1779</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>73885.9104792</v>
+        <v>72829.4543649</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-6114.0895208</v>
+        <v>-7170.545635100003</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.07642611901</v>
+        <v>-0.08963182043875004</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -8302,6 +8449,9 @@
       </c>
       <c r="AW34" s="3" t="n">
         <v>210.1832</v>
+      </c>
+      <c r="AX34" s="3" t="n">
+        <v>207.1779</v>
       </c>
     </row>
     <row r="35">
@@ -8327,16 +8477,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>15.18</v>
+        <v>15.07</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>108315.72114</v>
+        <v>107530.82461</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>8315.721139999994</v>
+        <v>7530.824609999996</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.08315721139999994</v>
+        <v>0.07530824609999996</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -8454,6 +8604,9 @@
       </c>
       <c r="AW35" s="3" t="n">
         <v>15.18</v>
+      </c>
+      <c r="AX35" s="3" t="n">
+        <v>15.07</v>
       </c>
     </row>
     <row r="36">
@@ -8479,16 +8632,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>362.1997</v>
+        <v>364.5574</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>168678.5734882</v>
+        <v>169776.5685244</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>18678.5734882</v>
+        <v>19776.56852440001</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1245238232546666</v>
+        <v>0.1318437901626667</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -8606,6 +8759,9 @@
       </c>
       <c r="AW36" s="3" t="n">
         <v>362.1997</v>
+      </c>
+      <c r="AX36" s="3" t="n">
+        <v>364.5574</v>
       </c>
     </row>
     <row r="37">
@@ -8631,16 +8787,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>16.177</v>
+        <v>16.323</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>60872.255353</v>
+        <v>61421.637147</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>10872.255353</v>
+        <v>11421.637147</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.21744510706</v>
+        <v>0.22843274294</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -8758,6 +8914,9 @@
       </c>
       <c r="AW37" s="3" t="n">
         <v>16.177</v>
+      </c>
+      <c r="AX37" s="3" t="n">
+        <v>16.323</v>
       </c>
     </row>
     <row r="38">
@@ -8783,16 +8942,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>14.4161</v>
+        <v>14.2652</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>86215.2265602</v>
+        <v>85312.7718264</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>6215.226560199997</v>
+        <v>5312.7718264</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.07769033200249996</v>
+        <v>0.06640964782999999</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -8907,6 +9066,9 @@
       </c>
       <c r="AW38" s="3" t="n">
         <v>14.4161</v>
+      </c>
+      <c r="AX38" s="3" t="n">
+        <v>14.2652</v>
       </c>
     </row>
     <row r="39">
@@ -8932,16 +9094,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1019.7809</v>
+        <v>1020.6133</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50867.6910729</v>
+        <v>50909.2120173</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>867.691072900001</v>
+        <v>909.2120173000003</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.01735382145800002</v>
+        <v>0.01818424034600001</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -9056,6 +9218,9 @@
       </c>
       <c r="AW39" s="3" t="n">
         <v>1019.7809</v>
+      </c>
+      <c r="AX39" s="3" t="n">
+        <v>1020.6133</v>
       </c>
     </row>
     <row r="40">
@@ -9081,16 +9246,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>21.3535</v>
+        <v>21.098</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>107643.5700445</v>
+        <v>106355.587646</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>7643.570044499997</v>
+        <v>6355.587646</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.07643570044499996</v>
+        <v>0.06355587645999999</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -9208,6 +9373,9 @@
       </c>
       <c r="AW40" s="3" t="n">
         <v>21.3535</v>
+      </c>
+      <c r="AX40" s="3" t="n">
+        <v>21.098</v>
       </c>
     </row>
     <row r="41">
@@ -9220,13 +9388,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4996454.8331916</v>
+        <v>4944604.1767516</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>526454.8331915999</v>
+        <v>474604.1767515999</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1177751304679194</v>
+        <v>0.1061754310406264</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-06-25
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -484,8 +484,8 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-24 06:05 IST</t>
+          <t>Generated: 2026-06-25 06:05 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4944604.1767516</v>
+        <v>4930922.4790445</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>474604.1767515996</v>
+        <v>460922.4790444998</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1061754310406263</v>
+        <v>0.1031146485558165</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>556358.5018234253</v>
+        <v>555417.5009231567</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-34423.51817657473</v>
+        <v>-35364.51907684328</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.05826771467516009</v>
+        <v>-0.05986052025896672</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5500962.678575025</v>
+        <v>5486339.979967657</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>440180.6585750254</v>
+        <v>425557.959967657</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.08697878249556092</v>
+        <v>0.084089367668054</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-06-24</t>
+          <t>Last snapshot: 2026-06-25</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW19"/>
+  <dimension ref="A1:AX19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -668,6 +668,7 @@
     <col width="21" customWidth="1" min="47" max="47"/>
     <col width="21" customWidth="1" min="48" max="48"/>
     <col width="21" customWidth="1" min="49" max="49"/>
+    <col width="21" customWidth="1" min="50" max="50"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -916,6 +917,11 @@
           <t>2026-06-24</t>
         </is>
       </c>
+      <c r="AX1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -935,13 +941,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>552.2000122070312</v>
+        <v>552.6500244140625</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>44176.0009765625</v>
+        <v>44212.001953125</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>358.490976562498</v>
+        <v>394.491953124998</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1068,6 +1074,9 @@
       </c>
       <c r="AW2" s="3" t="n">
         <v>552.2000122070312</v>
+      </c>
+      <c r="AX2" s="3" t="n">
+        <v>552.6500244140625</v>
       </c>
     </row>
     <row r="3">
@@ -1115,13 +1124,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1531.199951171875</v>
+        <v>1501.599975585938</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>30623.9990234375</v>
+        <v>30031.99951171875</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-1480.580976562502</v>
+        <v>-2072.580488281252</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1248,6 +1257,9 @@
       </c>
       <c r="AW4" s="3" t="n">
         <v>1531.199951171875</v>
+      </c>
+      <c r="AX4" s="3" t="n">
+        <v>1501.599975585938</v>
       </c>
     </row>
     <row r="5">
@@ -1268,13 +1280,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>655.3499755859375</v>
+        <v>645</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13106.99951171875</v>
+        <v>12900</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1106.10048828125</v>
+        <v>-1313.1</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1401,6 +1413,9 @@
       </c>
       <c r="AW5" s="3" t="n">
         <v>655.3499755859375</v>
+      </c>
+      <c r="AX5" s="3" t="n">
+        <v>645</v>
       </c>
     </row>
     <row r="6">
@@ -1421,13 +1436,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>382.25</v>
+        <v>377.2999877929688</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15290</v>
+        <v>15091.99951171875</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2212.240000000002</v>
+        <v>-2410.240488281252</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1554,6 +1569,9 @@
       </c>
       <c r="AW6" s="3" t="n">
         <v>382.25</v>
+      </c>
+      <c r="AX6" s="3" t="n">
+        <v>377.2999877929688</v>
       </c>
     </row>
     <row r="7">
@@ -1574,13 +1592,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>254.8999938964844</v>
+        <v>251.6399993896484</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>25489.99938964844</v>
+        <v>25163.99993896484</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-943.8206103515622</v>
+        <v>-1269.820061035156</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1707,6 +1725,9 @@
       </c>
       <c r="AW7" s="3" t="n">
         <v>254.8999938964844</v>
+      </c>
+      <c r="AX7" s="3" t="n">
+        <v>251.6399993896484</v>
       </c>
     </row>
     <row r="8">
@@ -1754,13 +1775,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>17.82999992370605</v>
+        <v>17.93000030517578</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>26744.99988555908</v>
+        <v>26895.00045776367</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-4305.170114440916</v>
+        <v>-4155.169542236326</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1887,6 +1908,9 @@
       </c>
       <c r="AW9" s="3" t="n">
         <v>17.82999992370605</v>
+      </c>
+      <c r="AX9" s="3" t="n">
+        <v>17.93000030517578</v>
       </c>
     </row>
     <row r="10">
@@ -1907,13 +1931,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>414.6000061035156</v>
+        <v>409.6499938964844</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>41460.00061035156</v>
+        <v>40964.99938964844</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-10038.47938964844</v>
+        <v>-10533.48061035157</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -2040,6 +2064,9 @@
       </c>
       <c r="AW10" s="3" t="n">
         <v>414.6000061035156</v>
+      </c>
+      <c r="AX10" s="3" t="n">
+        <v>409.6499938964844</v>
       </c>
     </row>
     <row r="11">
@@ -2060,13 +2087,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>8.829999923706055</v>
+        <v>8.640000343322754</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>8829.999923706055</v>
+        <v>8640.000343322754</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-1011.210076293944</v>
+        <v>-1201.209656677245</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -2193,6 +2220,9 @@
       </c>
       <c r="AW11" s="3" t="n">
         <v>8.829999923706055</v>
+      </c>
+      <c r="AX11" s="3" t="n">
+        <v>8.640000343322754</v>
       </c>
     </row>
     <row r="12">
@@ -2213,13 +2243,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2741.60009765625</v>
+        <v>2695.39990234375</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>27416.0009765625</v>
+        <v>26953.9990234375</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-307.2490234375</v>
+        <v>-769.2509765625</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -2346,6 +2376,9 @@
       </c>
       <c r="AW12" s="3" t="n">
         <v>2741.60009765625</v>
+      </c>
+      <c r="AX12" s="3" t="n">
+        <v>2695.39990234375</v>
       </c>
     </row>
     <row r="13">
@@ -2366,13 +2399,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>57.90000152587891</v>
+        <v>57.93000030517578</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>34740.00091552734</v>
+        <v>34758.00018310547</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-291.7590844726583</v>
+        <v>-273.7598168945333</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -2499,6 +2532,9 @@
       </c>
       <c r="AW13" s="3" t="n">
         <v>57.90000152587891</v>
+      </c>
+      <c r="AX13" s="3" t="n">
+        <v>57.93000030517578</v>
       </c>
     </row>
     <row r="14">
@@ -2519,13 +2555,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>725.5</v>
+        <v>748</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>36275</v>
+        <v>37400</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-6187.510000000002</v>
+        <v>-5062.510000000002</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -2652,6 +2688,9 @@
       </c>
       <c r="AW14" s="3" t="n">
         <v>725.5</v>
+      </c>
+      <c r="AX14" s="3" t="n">
+        <v>748</v>
       </c>
     </row>
     <row r="15">
@@ -2726,13 +2765,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>618.2999877929688</v>
+        <v>624.9000244140625</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>30914.99938964844</v>
+        <v>31245.00122070312</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>9160.469389648439</v>
+        <v>9490.471220703126</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -2859,6 +2898,9 @@
       </c>
       <c r="AW17" s="3" t="n">
         <v>618.2999877929688</v>
+      </c>
+      <c r="AX17" s="3" t="n">
+        <v>624.9000244140625</v>
       </c>
     </row>
     <row r="18">
@@ -2879,13 +2921,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>395.2000122070312</v>
+        <v>393.8999938964844</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>39520.00122070312</v>
+        <v>39389.99938964844</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-7120.818779296875</v>
+        <v>-7250.820610351562</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -3012,6 +3054,9 @@
       </c>
       <c r="AW18" s="3" t="n">
         <v>395.2000122070312</v>
+      </c>
+      <c r="AX18" s="3" t="n">
+        <v>393.8999938964844</v>
       </c>
     </row>
     <row r="19">
@@ -3024,10 +3069,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>556358.5018234253</v>
+        <v>555417.5009231567</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-34423.51817657472</v>
+        <v>-35364.51907684327</v>
       </c>
     </row>
   </sheetData>
@@ -3041,7 +3086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX41"/>
+  <dimension ref="A1:AY41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3094,6 +3139,7 @@
     <col width="13" customWidth="1" min="48" max="48"/>
     <col width="13" customWidth="1" min="49" max="49"/>
     <col width="13" customWidth="1" min="50" max="50"/>
+    <col width="13" customWidth="1" min="51" max="51"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3347,6 +3393,11 @@
           <t>2026-06-24</t>
         </is>
       </c>
+      <c r="AY1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3371,16 +3422,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.0437</v>
+        <v>55.9638</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>62908.0444634</v>
+        <v>62818.3581516</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>12908.0444634</v>
+        <v>12818.3581516</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.258160889268</v>
+        <v>0.256367163032</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -3504,6 +3555,9 @@
       </c>
       <c r="AX2" s="3" t="n">
         <v>56.0437</v>
+      </c>
+      <c r="AY2" s="3" t="n">
+        <v>55.9638</v>
       </c>
     </row>
     <row r="3">
@@ -3529,16 +3583,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>24.9866</v>
+        <v>25.0245</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>61347.4251458</v>
+        <v>61440.47771850001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>1347.4251458</v>
+        <v>1440.477718500006</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.02245708576333333</v>
+        <v>0.0240079619750001</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -3656,6 +3710,9 @@
       </c>
       <c r="AX3" s="3" t="n">
         <v>24.9866</v>
+      </c>
+      <c r="AY3" s="3" t="n">
+        <v>25.0245</v>
       </c>
     </row>
     <row r="4">
@@ -3681,16 +3738,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.12</v>
+        <v>12.01</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>232777.84716</v>
+        <v>230665.17693</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>52777.84716</v>
+        <v>50665.17693000002</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.293210262</v>
+        <v>0.2814732051666667</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -3808,6 +3865,9 @@
       </c>
       <c r="AX4" s="3" t="n">
         <v>12.12</v>
+      </c>
+      <c r="AY4" s="3" t="n">
+        <v>12.01</v>
       </c>
     </row>
     <row r="5">
@@ -3833,16 +3893,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.404</v>
+        <v>9.3818</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>172601.843552</v>
+        <v>172194.3827984</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-37398.15644799999</v>
+        <v>-37805.61720159999</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1780864592761905</v>
+        <v>-0.1800267485790476</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -3960,6 +4020,9 @@
       </c>
       <c r="AX5" s="3" t="n">
         <v>9.404</v>
+      </c>
+      <c r="AY5" s="3" t="n">
+        <v>9.3818</v>
       </c>
     </row>
     <row r="6">
@@ -3985,16 +4048,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.3758</v>
+        <v>12.2529</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>52336.97355659999</v>
+        <v>51817.2322833</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>2336.973556599994</v>
+        <v>1817.2322833</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.04673947113199989</v>
+        <v>0.036344645666</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -4118,6 +4181,9 @@
       </c>
       <c r="AX6" s="3" t="n">
         <v>12.3758</v>
+      </c>
+      <c r="AY6" s="3" t="n">
+        <v>12.2529</v>
       </c>
     </row>
     <row r="7">
@@ -4143,16 +4209,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.8215</v>
+        <v>33.662</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>74611.58186000001</v>
+        <v>74259.71848</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>14611.58186000001</v>
+        <v>14259.71848</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2435263643333334</v>
+        <v>0.2376619746666666</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -4270,6 +4336,9 @@
       </c>
       <c r="AX7" s="3" t="n">
         <v>33.8215</v>
+      </c>
+      <c r="AY7" s="3" t="n">
+        <v>33.662</v>
       </c>
     </row>
     <row r="8">
@@ -4295,16 +4364,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>33.521</v>
+        <v>33.575</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>53787.561953</v>
+        <v>53874.20997500001</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>3787.561953000004</v>
+        <v>3874.209975000005</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.07575123906000009</v>
+        <v>0.0774841995000001</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -4428,6 +4497,9 @@
       </c>
       <c r="AX8" s="3" t="n">
         <v>33.521</v>
+      </c>
+      <c r="AY8" s="3" t="n">
+        <v>33.575</v>
       </c>
     </row>
     <row r="9">
@@ -4453,16 +4525,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>42.0059</v>
+        <v>41.4979</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>135233.5004187</v>
+        <v>133598.0487747</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>35233.50041869999</v>
+        <v>33598.0487747</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3523350041869999</v>
+        <v>0.335980487747</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -4580,6 +4652,9 @@
       </c>
       <c r="AX9" s="3" t="n">
         <v>42.0059</v>
+      </c>
+      <c r="AY9" s="3" t="n">
+        <v>41.4979</v>
       </c>
     </row>
     <row r="10">
@@ -4605,16 +4680,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>47.0175</v>
+        <v>47.1751</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>133842.7895325</v>
+        <v>134291.4229909</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>33842.7895325</v>
+        <v>34291.4229909</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.338427895325</v>
+        <v>0.342914229909</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -4732,6 +4807,9 @@
       </c>
       <c r="AX10" s="3" t="n">
         <v>47.0175</v>
+      </c>
+      <c r="AY10" s="3" t="n">
+        <v>47.1751</v>
       </c>
     </row>
     <row r="11">
@@ -4757,16 +4835,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>102.7625</v>
+        <v>102.8893</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>30923.1887375</v>
+        <v>30961.3452667</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>923.1887375000006</v>
+        <v>961.3452666999983</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.03077295791666669</v>
+        <v>0.03204484222333328</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -4884,6 +4962,9 @@
       </c>
       <c r="AX11" s="3" t="n">
         <v>102.7625</v>
+      </c>
+      <c r="AY11" s="3" t="n">
+        <v>102.8893</v>
       </c>
     </row>
     <row r="12">
@@ -4909,16 +4990,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>226.634</v>
+        <v>227.898</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>105503.112948</v>
+        <v>106091.532756</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>5503.112947999995</v>
+        <v>6091.532756000001</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.05503112947999995</v>
+        <v>0.06091532756</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -5042,6 +5123,9 @@
       </c>
       <c r="AX12" s="3" t="n">
         <v>226.634</v>
+      </c>
+      <c r="AY12" s="3" t="n">
+        <v>227.898</v>
       </c>
     </row>
     <row r="13">
@@ -5067,16 +5151,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>20.789</v>
+        <v>20.806</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>240894.720345</v>
+        <v>241091.70963</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>40894.72034500001</v>
+        <v>41091.70963</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.204473601725</v>
+        <v>0.20545854815</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -5200,6 +5284,9 @@
       </c>
       <c r="AX13" s="3" t="n">
         <v>20.789</v>
+      </c>
+      <c r="AY13" s="3" t="n">
+        <v>20.806</v>
       </c>
     </row>
     <row r="14">
@@ -5225,16 +5312,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>40.4924</v>
+        <v>38.8375</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>146080.6251944</v>
+        <v>140110.398025</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>46080.62519440003</v>
+        <v>40110.398025</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.4608062519440003</v>
+        <v>0.40110398025</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -5352,6 +5439,9 @@
       </c>
       <c r="AX14" s="3" t="n">
         <v>40.4924</v>
+      </c>
+      <c r="AY14" s="3" t="n">
+        <v>38.8375</v>
       </c>
     </row>
     <row r="15">
@@ -5377,16 +5467,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>12.14</v>
+        <v>12.06</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>118291.51658</v>
+        <v>117512.00082</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>18291.51658000001</v>
+        <v>17512.00082</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1829151658000001</v>
+        <v>0.1751200082</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -5510,6 +5600,9 @@
       </c>
       <c r="AX15" s="3" t="n">
         <v>12.14</v>
+      </c>
+      <c r="AY15" s="3" t="n">
+        <v>12.06</v>
       </c>
     </row>
     <row r="16">
@@ -5535,16 +5628,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.1943</v>
+        <v>24.0874</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>138462.2369104</v>
+        <v>137850.4559072</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>38462.23691039998</v>
+        <v>37850.4559072</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.3846223691039998</v>
+        <v>0.378504559072</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -5662,6 +5755,9 @@
       </c>
       <c r="AX16" s="3" t="n">
         <v>24.1943</v>
+      </c>
+      <c r="AY16" s="3" t="n">
+        <v>24.0874</v>
       </c>
     </row>
     <row r="17">
@@ -5687,16 +5783,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.7199</v>
+        <v>16.7713</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55276.94243429999</v>
+        <v>55446.8737641</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5276.942434299992</v>
+        <v>5446.873764099997</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1055388486859998</v>
+        <v>0.1089374752819999</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -5814,6 +5910,9 @@
       </c>
       <c r="AX17" s="3" t="n">
         <v>16.7199</v>
+      </c>
+      <c r="AY17" s="3" t="n">
+        <v>16.7713</v>
       </c>
     </row>
     <row r="18">
@@ -5839,16 +5938,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>46.25</v>
+        <v>46.43</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>87247.66499999999</v>
+        <v>87587.22348</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>7247.664999999994</v>
+        <v>7587.223480000001</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.09059581249999991</v>
+        <v>0.09484029350000001</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -5972,6 +6071,9 @@
       </c>
       <c r="AX18" s="3" t="n">
         <v>46.25</v>
+      </c>
+      <c r="AY18" s="3" t="n">
+        <v>46.43</v>
       </c>
     </row>
     <row r="19">
@@ -5997,16 +6099,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>15.286</v>
+        <v>14.7103</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>221138.985076</v>
+        <v>212810.4678898</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>71138.98507599998</v>
+        <v>62810.4678898</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.4742599005066666</v>
+        <v>0.4187364525986667</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -6124,6 +6226,9 @@
       </c>
       <c r="AX19" s="3" t="n">
         <v>15.286</v>
+      </c>
+      <c r="AY19" s="3" t="n">
+        <v>14.7103</v>
       </c>
     </row>
     <row r="20">
@@ -6149,16 +6254,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.369999999999999</v>
+        <v>9.42</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>246016.87411</v>
+        <v>247329.66426</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-3983.125890000025</v>
+        <v>-2670.33574000001</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.0159325035600001</v>
+        <v>-0.01068134296000004</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -6282,6 +6387,9 @@
       </c>
       <c r="AX20" s="3" t="n">
         <v>9.369999999999999</v>
+      </c>
+      <c r="AY20" s="3" t="n">
+        <v>9.42</v>
       </c>
     </row>
     <row r="21">
@@ -6307,16 +6415,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>111.0276</v>
+        <v>111.9808</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>168679.6805484</v>
-      </c>
-      <c r="H21" s="6" t="n">
-        <v>-1320.319451599993</v>
-      </c>
-      <c r="I21" s="13" t="n">
-        <v>-0.007766585009411723</v>
+        <v>170127.8382272</v>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>127.8382272000017</v>
+      </c>
+      <c r="I21" s="12" t="n">
+        <v>0.000751989571764716</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -6440,6 +6548,9 @@
       </c>
       <c r="AX21" s="3" t="n">
         <v>111.0276</v>
+      </c>
+      <c r="AY21" s="3" t="n">
+        <v>111.9808</v>
       </c>
     </row>
     <row r="22">
@@ -6465,16 +6576,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>44.405</v>
+        <v>44.337</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>68137.69630000001</v>
+        <v>68033.35302000001</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>8137.696300000011</v>
+        <v>8033.35302000001</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1356282716666669</v>
+        <v>0.1338892170000002</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -6592,6 +6703,9 @@
       </c>
       <c r="AX22" s="3" t="n">
         <v>44.405</v>
+      </c>
+      <c r="AY22" s="3" t="n">
+        <v>44.337</v>
       </c>
     </row>
     <row r="23">
@@ -6617,16 +6731,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>64.1322</v>
+        <v>63.8971</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>174213.0049374</v>
+        <v>173574.3635457</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>24213.00493739999</v>
+        <v>23574.36354570001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.161420032916</v>
+        <v>0.157162423638</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -6750,6 +6864,9 @@
       </c>
       <c r="AX23" s="3" t="n">
         <v>64.1322</v>
+      </c>
+      <c r="AY23" s="3" t="n">
+        <v>63.8971</v>
       </c>
     </row>
     <row r="24">
@@ -6775,16 +6892,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>28.0795</v>
+        <v>28.2167</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>102023.662187</v>
+        <v>102522.1627462</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>2023.662186999994</v>
+        <v>2522.162746200003</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.02023662186999994</v>
+        <v>0.02522162746200003</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -6902,6 +7019,9 @@
       </c>
       <c r="AX24" s="3" t="n">
         <v>28.0795</v>
+      </c>
+      <c r="AY24" s="3" t="n">
+        <v>28.2167</v>
       </c>
     </row>
     <row r="25">
@@ -6927,16 +7047,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.6442</v>
+        <v>11.7077</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>191217.2563908</v>
+        <v>192260.0326898</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-8782.743609200028</v>
+        <v>-7739.967310200009</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.04391371804600014</v>
+        <v>-0.03869983655100005</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -7057,6 +7177,9 @@
       </c>
       <c r="AX25" s="3" t="n">
         <v>11.6442</v>
+      </c>
+      <c r="AY25" s="3" t="n">
+        <v>11.7077</v>
       </c>
     </row>
     <row r="26">
@@ -7082,16 +7205,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>9.1143</v>
+        <v>9.1891</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>108840.3730245</v>
+        <v>109733.6133065</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>-1159.626975499996</v>
+        <v>-266.3866934999969</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>-0.01054206341363633</v>
+        <v>-0.002421697213636336</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -7212,6 +7335,9 @@
       </c>
       <c r="AX26" s="3" t="n">
         <v>9.1143</v>
+      </c>
+      <c r="AY26" s="3" t="n">
+        <v>9.1891</v>
       </c>
     </row>
     <row r="27">
@@ -7237,16 +7363,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>64.65130000000001</v>
+        <v>64.5823</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>104144.193118</v>
+        <v>104033.043778</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-5855.80688199999</v>
+        <v>-5966.956221999993</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.05323460801818172</v>
+        <v>-0.0542450565636363</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -7370,6 +7496,9 @@
       </c>
       <c r="AX27" s="3" t="n">
         <v>64.65130000000001</v>
+      </c>
+      <c r="AY27" s="3" t="n">
+        <v>64.5823</v>
       </c>
     </row>
     <row r="28">
@@ -7395,16 +7524,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>108.0557</v>
+        <v>108.4143</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>357303.1367949</v>
+        <v>358488.9039951</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-22696.8632051</v>
+        <v>-21511.0960049</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.05972858738184211</v>
+        <v>-0.05660814738131579</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -7528,6 +7657,9 @@
       </c>
       <c r="AX28" s="3" t="n">
         <v>108.0557</v>
+      </c>
+      <c r="AY28" s="3" t="n">
+        <v>108.4143</v>
       </c>
     </row>
     <row r="29">
@@ -7553,16 +7685,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.6508</v>
+        <v>12.4011</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>121494.5259124</v>
+        <v>119096.4812733</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>21494.5259124</v>
+        <v>19096.48127329999</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.214945259124</v>
+        <v>0.1909648127329999</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -7680,6 +7812,9 @@
       </c>
       <c r="AX29" s="3" t="n">
         <v>12.6508</v>
+      </c>
+      <c r="AY29" s="3" t="n">
+        <v>12.4011</v>
       </c>
     </row>
     <row r="30">
@@ -7705,16 +7840,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>16.4926</v>
+        <v>16.5525</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>121976.9771286</v>
+        <v>122419.9892025</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>21976.97712859999</v>
+        <v>22419.98920249999</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.2197697712859999</v>
+        <v>0.2241998920249999</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -7832,6 +7967,9 @@
       </c>
       <c r="AX30" s="3" t="n">
         <v>16.4926</v>
+      </c>
+      <c r="AY30" s="3" t="n">
+        <v>16.5525</v>
       </c>
     </row>
     <row r="31">
@@ -7857,16 +7995,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>423.4812</v>
+        <v>421.3574</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>112679.877696</v>
+        <v>112114.776992</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>12679.877696</v>
+        <v>12114.77699199998</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.12679877696</v>
+        <v>0.1211477699199998</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -7987,6 +8125,9 @@
       </c>
       <c r="AX31" s="3" t="n">
         <v>423.4812</v>
+      </c>
+      <c r="AY31" s="3" t="n">
+        <v>421.3574</v>
       </c>
     </row>
     <row r="32">
@@ -8146,6 +8287,9 @@
       <c r="AX32" s="3" t="n">
         <v>10.54</v>
       </c>
+      <c r="AY32" s="3" t="n">
+        <v>10.54</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -8170,16 +8314,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>18.88</v>
+        <v>18.87</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>67659.12319999999</v>
+        <v>67623.2868</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>7659.123199999987</v>
+        <v>7623.286800000002</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.1276520533333331</v>
+        <v>0.12705478</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -8297,6 +8441,9 @@
       </c>
       <c r="AX33" s="3" t="n">
         <v>18.88</v>
+      </c>
+      <c r="AY33" s="3" t="n">
+        <v>18.87</v>
       </c>
     </row>
     <row r="34">
@@ -8322,16 +8469,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>207.1779</v>
+        <v>208.2005</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>72829.4543649</v>
+        <v>73188.92996550001</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-7170.545635100003</v>
+        <v>-6811.070034499993</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.08963182043875004</v>
+        <v>-0.08513837543124991</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -8452,6 +8599,9 @@
       </c>
       <c r="AX34" s="3" t="n">
         <v>207.1779</v>
+      </c>
+      <c r="AY34" s="3" t="n">
+        <v>208.2005</v>
       </c>
     </row>
     <row r="35">
@@ -8477,16 +8627,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>15.07</v>
+        <v>14.93</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>107530.82461</v>
+        <v>106531.86539</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>7530.824609999996</v>
+        <v>6531.865389999992</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.07530824609999996</v>
+        <v>0.06531865389999991</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -8607,6 +8757,9 @@
       </c>
       <c r="AX35" s="3" t="n">
         <v>15.07</v>
+      </c>
+      <c r="AY35" s="3" t="n">
+        <v>14.93</v>
       </c>
     </row>
     <row r="36">
@@ -8632,16 +8785,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>364.5574</v>
+        <v>366.4301</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>169776.5685244</v>
+        <v>170648.6961506</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>19776.56852440001</v>
+        <v>20648.69615060001</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1318437901626667</v>
+        <v>0.1376579743373334</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -8762,6 +8915,9 @@
       </c>
       <c r="AX36" s="3" t="n">
         <v>364.5574</v>
+      </c>
+      <c r="AY36" s="3" t="n">
+        <v>366.4301</v>
       </c>
     </row>
     <row r="37">
@@ -8787,16 +8943,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>16.323</v>
+        <v>16.343</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>61421.637147</v>
+        <v>61496.894927</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>11421.637147</v>
+        <v>11496.894927</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.22843274294</v>
+        <v>0.22993789854</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -8917,6 +9073,9 @@
       </c>
       <c r="AX37" s="3" t="n">
         <v>16.323</v>
+      </c>
+      <c r="AY37" s="3" t="n">
+        <v>16.343</v>
       </c>
     </row>
     <row r="38">
@@ -8942,16 +9101,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>14.2652</v>
+        <v>14.3177</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>85312.7718264</v>
+        <v>85626.7471314</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>5312.7718264</v>
+        <v>5626.747131399999</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.06640964782999999</v>
+        <v>0.07033433914249999</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -9069,6 +9228,9 @@
       </c>
       <c r="AX38" s="3" t="n">
         <v>14.2652</v>
+      </c>
+      <c r="AY38" s="3" t="n">
+        <v>14.3177</v>
       </c>
     </row>
     <row r="39">
@@ -9094,16 +9256,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1020.6133</v>
+        <v>1021.3417</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50909.2120173</v>
+        <v>50945.54533769999</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>909.2120173000003</v>
+        <v>945.545337699994</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.01818424034600001</v>
+        <v>0.01891090675399988</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -9221,6 +9383,9 @@
       </c>
       <c r="AX39" s="3" t="n">
         <v>1020.6133</v>
+      </c>
+      <c r="AY39" s="3" t="n">
+        <v>1021.3417</v>
       </c>
     </row>
     <row r="40">
@@ -9246,16 +9411,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>21.098</v>
+        <v>21.4024</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>106355.587646</v>
+        <v>107890.0762648</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>6355.587646</v>
+        <v>7890.076264799995</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.06355587645999999</v>
+        <v>0.07890076264799994</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -9376,6 +9541,9 @@
       </c>
       <c r="AX40" s="3" t="n">
         <v>21.098</v>
+      </c>
+      <c r="AY40" s="3" t="n">
+        <v>21.4024</v>
       </c>
     </row>
     <row r="41">
@@ -9388,13 +9556,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4944604.1767516</v>
+        <v>4930922.4790445</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>474604.1767515999</v>
+        <v>460922.4790445</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1061754310406264</v>
+        <v>0.1031146485558165</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-06-26
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -39,10 +39,10 @@
       <sz val="10"/>
     </font>
     <font>
-      <color rgb="00006100"/>
+      <color rgb="009C0006"/>
     </font>
     <font>
-      <color rgb="009C0006"/>
+      <color rgb="00006100"/>
     </font>
     <font>
       <b val="1"/>
@@ -97,9 +97,9 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -109,8 +109,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -484,8 +484,8 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-25 06:05 IST</t>
+          <t>Generated: 2026-06-26 06:08 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4930922.4790445</v>
+        <v>4919461.156848</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>460922.4790444998</v>
+        <v>449461.1568480004</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1031146485558165</v>
+        <v>0.1005505943731544</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>555417.5009231567</v>
+        <v>551210.4988937378</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-35364.51907684328</v>
+        <v>-39571.52110626223</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.05986052025896672</v>
+        <v>-0.06698159349240558</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5486339.979967657</v>
+        <v>5470671.655741738</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>425557.959967657</v>
+        <v>409889.6357417386</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.084089367668054</v>
+        <v>0.08099333939337278</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-06-25</t>
+          <t>Last snapshot: 2026-06-26</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX19"/>
+  <dimension ref="A1:AY19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -669,6 +669,7 @@
     <col width="21" customWidth="1" min="48" max="48"/>
     <col width="21" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
+    <col width="21" customWidth="1" min="51" max="51"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -922,6 +923,11 @@
           <t>2026-06-25</t>
         </is>
       </c>
+      <c r="AY1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -941,13 +947,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>552.6500244140625</v>
+        <v>533.7000122070312</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>44212.001953125</v>
-      </c>
-      <c r="G2" s="4" t="n">
-        <v>394.491953124998</v>
+        <v>42696.0009765625</v>
+      </c>
+      <c r="G2" s="6" t="n">
+        <v>-1121.509023437502</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1077,6 +1083,9 @@
       </c>
       <c r="AX2" s="3" t="n">
         <v>552.6500244140625</v>
+      </c>
+      <c r="AY2" s="3" t="n">
+        <v>533.7000122070312</v>
       </c>
     </row>
     <row r="3">
@@ -1124,13 +1133,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1501.599975585938</v>
+        <v>1490</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>30031.99951171875</v>
+        <v>29800</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-2072.580488281252</v>
+        <v>-2304.580000000002</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1260,6 +1269,9 @@
       </c>
       <c r="AX4" s="3" t="n">
         <v>1501.599975585938</v>
+      </c>
+      <c r="AY4" s="3" t="n">
+        <v>1490</v>
       </c>
     </row>
     <row r="5">
@@ -1280,13 +1292,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>645</v>
+        <v>640</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>12900</v>
+        <v>12800</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1313.1</v>
+        <v>-1413.1</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1416,6 +1428,9 @@
       </c>
       <c r="AX5" s="3" t="n">
         <v>645</v>
+      </c>
+      <c r="AY5" s="3" t="n">
+        <v>640</v>
       </c>
     </row>
     <row r="6">
@@ -1436,13 +1451,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>377.2999877929688</v>
+        <v>379</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15091.99951171875</v>
+        <v>15160</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2410.240488281252</v>
+        <v>-2342.240000000002</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1572,6 +1587,9 @@
       </c>
       <c r="AX6" s="3" t="n">
         <v>377.2999877929688</v>
+      </c>
+      <c r="AY6" s="3" t="n">
+        <v>379</v>
       </c>
     </row>
     <row r="7">
@@ -1592,13 +1610,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>251.6399993896484</v>
+        <v>251.8800048828125</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>25163.99993896484</v>
+        <v>25188.00048828125</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-1269.820061035156</v>
+        <v>-1245.81951171875</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1728,6 +1746,9 @@
       </c>
       <c r="AX7" s="3" t="n">
         <v>251.6399993896484</v>
+      </c>
+      <c r="AY7" s="3" t="n">
+        <v>251.8800048828125</v>
       </c>
     </row>
     <row r="8">
@@ -1775,13 +1796,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>17.93000030517578</v>
+        <v>17.8799991607666</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>26895.00045776367</v>
+        <v>26819.9987411499</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-4155.169542236326</v>
+        <v>-4230.171258850096</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1911,6 +1932,9 @@
       </c>
       <c r="AX9" s="3" t="n">
         <v>17.93000030517578</v>
+      </c>
+      <c r="AY9" s="3" t="n">
+        <v>17.8799991607666</v>
       </c>
     </row>
     <row r="10">
@@ -1931,13 +1955,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>409.6499938964844</v>
+        <v>405.9500122070312</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>40964.99938964844</v>
+        <v>40595.00122070312</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-10533.48061035157</v>
+        <v>-10903.47877929688</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -2067,6 +2091,9 @@
       </c>
       <c r="AX10" s="3" t="n">
         <v>409.6499938964844</v>
+      </c>
+      <c r="AY10" s="3" t="n">
+        <v>405.9500122070312</v>
       </c>
     </row>
     <row r="11">
@@ -2087,13 +2114,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>8.640000343322754</v>
+        <v>8.569999694824219</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>8640.000343322754</v>
+        <v>8569.999694824219</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-1201.209656677245</v>
+        <v>-1271.21030517578</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -2223,6 +2250,9 @@
       </c>
       <c r="AX11" s="3" t="n">
         <v>8.640000343322754</v>
+      </c>
+      <c r="AY11" s="3" t="n">
+        <v>8.569999694824219</v>
       </c>
     </row>
     <row r="12">
@@ -2243,13 +2273,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2695.39990234375</v>
+        <v>2650</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>26953.9990234375</v>
+        <v>26500</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-769.2509765625</v>
+        <v>-1223.25</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -2379,6 +2409,9 @@
       </c>
       <c r="AX12" s="3" t="n">
         <v>2695.39990234375</v>
+      </c>
+      <c r="AY12" s="3" t="n">
+        <v>2650</v>
       </c>
     </row>
     <row r="13">
@@ -2399,13 +2432,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>57.93000030517578</v>
+        <v>57.0099983215332</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>34758.00018310547</v>
+        <v>34205.99899291992</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-273.7598168945333</v>
+        <v>-825.7610070800802</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -2535,6 +2568,9 @@
       </c>
       <c r="AX13" s="3" t="n">
         <v>57.93000030517578</v>
+      </c>
+      <c r="AY13" s="3" t="n">
+        <v>57.0099983215332</v>
       </c>
     </row>
     <row r="14">
@@ -2555,13 +2591,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>748</v>
+        <v>745</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>37400</v>
+        <v>37250</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-5062.510000000002</v>
+        <v>-5212.510000000002</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -2691,6 +2727,9 @@
       </c>
       <c r="AX14" s="3" t="n">
         <v>748</v>
+      </c>
+      <c r="AY14" s="3" t="n">
+        <v>745</v>
       </c>
     </row>
     <row r="15">
@@ -2765,13 +2804,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>624.9000244140625</v>
+        <v>620</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>31245.00122070312</v>
+        <v>31000</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>9490.471220703126</v>
+        <v>9245.470000000001</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -2901,6 +2940,9 @@
       </c>
       <c r="AX17" s="3" t="n">
         <v>624.9000244140625</v>
+      </c>
+      <c r="AY17" s="3" t="n">
+        <v>620</v>
       </c>
     </row>
     <row r="18">
@@ -2921,13 +2963,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>393.8999938964844</v>
+        <v>388.5499877929688</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>39389.99938964844</v>
+        <v>38854.99877929688</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-7250.820610351562</v>
+        <v>-7785.821220703125</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -3057,6 +3099,9 @@
       </c>
       <c r="AX18" s="3" t="n">
         <v>393.8999938964844</v>
+      </c>
+      <c r="AY18" s="3" t="n">
+        <v>388.5499877929688</v>
       </c>
     </row>
     <row r="19">
@@ -3069,10 +3114,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>555417.5009231567</v>
+        <v>551210.4988937378</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-35364.51907684327</v>
+        <v>-39571.52110626222</v>
       </c>
     </row>
   </sheetData>
@@ -3086,7 +3131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY41"/>
+  <dimension ref="A1:AZ41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3140,6 +3185,7 @@
     <col width="13" customWidth="1" min="49" max="49"/>
     <col width="13" customWidth="1" min="50" max="50"/>
     <col width="13" customWidth="1" min="51" max="51"/>
+    <col width="13" customWidth="1" min="52" max="52"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3398,6 +3444,11 @@
           <t>2026-06-25</t>
         </is>
       </c>
+      <c r="AZ1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3422,16 +3473,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>55.9638</v>
+        <v>56.0634</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>62818.3581516</v>
+        <v>62930.1573588</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>12818.3581516</v>
+        <v>12930.1573588</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.256367163032</v>
+        <v>0.2586031471760001</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -3558,6 +3609,9 @@
       </c>
       <c r="AY2" s="3" t="n">
         <v>55.9638</v>
+      </c>
+      <c r="AZ2" s="3" t="n">
+        <v>56.0634</v>
       </c>
     </row>
     <row r="3">
@@ -3714,6 +3768,9 @@
       <c r="AY3" s="3" t="n">
         <v>25.0245</v>
       </c>
+      <c r="AZ3" s="3" t="n">
+        <v>25.0245</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3869,6 +3926,9 @@
       <c r="AY4" s="3" t="n">
         <v>12.01</v>
       </c>
+      <c r="AZ4" s="3" t="n">
+        <v>12.01</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3893,16 +3953,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.3818</v>
+        <v>9.372</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>172194.3827984</v>
+        <v>172014.512736</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-37805.61720159999</v>
+        <v>-37985.487264</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1800267485790476</v>
+        <v>-0.1808832726857143</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -4023,6 +4083,9 @@
       </c>
       <c r="AY5" s="3" t="n">
         <v>9.3818</v>
+      </c>
+      <c r="AZ5" s="3" t="n">
+        <v>9.372</v>
       </c>
     </row>
     <row r="6">
@@ -4048,16 +4111,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.2529</v>
+        <v>12.148</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>51817.2322833</v>
+        <v>51373.612596</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>1817.2322833</v>
+        <v>1373.612595999999</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.036344645666</v>
+        <v>0.02747225191999998</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -4184,6 +4247,9 @@
       </c>
       <c r="AY6" s="3" t="n">
         <v>12.2529</v>
+      </c>
+      <c r="AZ6" s="3" t="n">
+        <v>12.148</v>
       </c>
     </row>
     <row r="7">
@@ -4209,16 +4275,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.662</v>
+        <v>33.621</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>74259.71848</v>
+        <v>74169.27084</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>14259.71848</v>
+        <v>14169.27084</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2376619746666666</v>
+        <v>0.236154514</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -4339,6 +4405,9 @@
       </c>
       <c r="AY7" s="3" t="n">
         <v>33.662</v>
+      </c>
+      <c r="AZ7" s="3" t="n">
+        <v>33.621</v>
       </c>
     </row>
     <row r="8">
@@ -4364,16 +4433,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>33.575</v>
+        <v>33.2869</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>53874.20997500001</v>
+        <v>53411.9267317</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>3874.209975000005</v>
+        <v>3411.926731700005</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.0774841995000001</v>
+        <v>0.06823853463400009</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -4500,6 +4569,9 @@
       </c>
       <c r="AY8" s="3" t="n">
         <v>33.575</v>
+      </c>
+      <c r="AZ8" s="3" t="n">
+        <v>33.2869</v>
       </c>
     </row>
     <row r="9">
@@ -4525,16 +4597,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>41.4979</v>
+        <v>40.8271</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>133598.0487747</v>
+        <v>131438.4799503</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>33598.0487747</v>
+        <v>31438.47995030001</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.335980487747</v>
+        <v>0.3143847995030001</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -4655,6 +4727,9 @@
       </c>
       <c r="AY9" s="3" t="n">
         <v>41.4979</v>
+      </c>
+      <c r="AZ9" s="3" t="n">
+        <v>40.8271</v>
       </c>
     </row>
     <row r="10">
@@ -4680,16 +4755,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>47.1751</v>
+        <v>47.4092</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>134291.4229909</v>
+        <v>134957.8258628</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>34291.4229909</v>
+        <v>34957.8258628</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.342914229909</v>
+        <v>0.349578258628</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -4810,6 +4885,9 @@
       </c>
       <c r="AY10" s="3" t="n">
         <v>47.1751</v>
+      </c>
+      <c r="AZ10" s="3" t="n">
+        <v>47.4092</v>
       </c>
     </row>
     <row r="11">
@@ -4835,16 +4913,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>102.8893</v>
+        <v>102.6766</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>30961.3452667</v>
+        <v>30897.3397954</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>961.3452666999983</v>
+        <v>897.3397953999956</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.03204484222333328</v>
+        <v>0.02991132651333319</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -4965,6 +5043,9 @@
       </c>
       <c r="AY11" s="3" t="n">
         <v>102.8893</v>
+      </c>
+      <c r="AZ11" s="3" t="n">
+        <v>102.6766</v>
       </c>
     </row>
     <row r="12">
@@ -4990,16 +5071,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>227.898</v>
+        <v>226.915</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>106091.532756</v>
+        <v>105633.92463</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>6091.532756000001</v>
+        <v>5633.924629999994</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.06091532756</v>
+        <v>0.05633924629999994</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -5126,6 +5207,9 @@
       </c>
       <c r="AY12" s="3" t="n">
         <v>227.898</v>
+      </c>
+      <c r="AZ12" s="3" t="n">
+        <v>226.915</v>
       </c>
     </row>
     <row r="13">
@@ -5151,16 +5235,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>20.806</v>
+        <v>20.753</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>241091.70963</v>
+        <v>240477.566565</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>41091.70963</v>
+        <v>40477.56656499999</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.20545854815</v>
+        <v>0.2023878328249999</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -5287,6 +5371,9 @@
       </c>
       <c r="AY13" s="3" t="n">
         <v>20.806</v>
+      </c>
+      <c r="AZ13" s="3" t="n">
+        <v>20.753</v>
       </c>
     </row>
     <row r="14">
@@ -5312,16 +5399,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>38.8375</v>
+        <v>39.3784</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>140110.398025</v>
+        <v>142061.7521104</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>40110.398025</v>
+        <v>42061.7521104</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.40110398025</v>
+        <v>0.420617521104</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -5442,6 +5529,9 @@
       </c>
       <c r="AY14" s="3" t="n">
         <v>38.8375</v>
+      </c>
+      <c r="AZ14" s="3" t="n">
+        <v>39.3784</v>
       </c>
     </row>
     <row r="15">
@@ -5467,16 +5557,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>12.06</v>
+        <v>11.94</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>117512.00082</v>
+        <v>116342.72718</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>17512.00082</v>
+        <v>16342.72718</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1751200082</v>
+        <v>0.1634272718</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -5603,6 +5693,9 @@
       </c>
       <c r="AY15" s="3" t="n">
         <v>12.06</v>
+      </c>
+      <c r="AZ15" s="3" t="n">
+        <v>11.94</v>
       </c>
     </row>
     <row r="16">
@@ -5628,16 +5721,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.0874</v>
+        <v>24.2127</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>137850.4559072</v>
+        <v>138567.5387856</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>37850.4559072</v>
+        <v>38567.53878560002</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.378504559072</v>
+        <v>0.3856753878560001</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -5758,6 +5851,9 @@
       </c>
       <c r="AY16" s="3" t="n">
         <v>24.0874</v>
+      </c>
+      <c r="AZ16" s="3" t="n">
+        <v>24.2127</v>
       </c>
     </row>
     <row r="17">
@@ -5783,16 +5879,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.7713</v>
+        <v>16.796</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55446.8737641</v>
+        <v>55528.53337199999</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5446.873764099997</v>
+        <v>5528.533371999991</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1089374752819999</v>
+        <v>0.1105706674399998</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -5913,6 +6009,9 @@
       </c>
       <c r="AY17" s="3" t="n">
         <v>16.7713</v>
+      </c>
+      <c r="AZ17" s="3" t="n">
+        <v>16.796</v>
       </c>
     </row>
     <row r="18">
@@ -5938,16 +6037,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>46.43</v>
+        <v>46.28</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>87587.22348</v>
+        <v>87304.25808</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>7587.223480000001</v>
+        <v>7304.25808</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.09484029350000001</v>
+        <v>0.091303226</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -6074,6 +6173,9 @@
       </c>
       <c r="AY18" s="3" t="n">
         <v>46.43</v>
+      </c>
+      <c r="AZ18" s="3" t="n">
+        <v>46.28</v>
       </c>
     </row>
     <row r="19">
@@ -6099,16 +6201,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>14.7103</v>
+        <v>14.7596</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>212810.4678898</v>
+        <v>213523.6794536</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>62810.4678898</v>
+        <v>63523.67945359999</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.4187364525986667</v>
+        <v>0.4234911963573333</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -6229,6 +6331,9 @@
       </c>
       <c r="AY19" s="3" t="n">
         <v>14.7103</v>
+      </c>
+      <c r="AZ19" s="3" t="n">
+        <v>14.7596</v>
       </c>
     </row>
     <row r="20">
@@ -6254,16 +6359,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.42</v>
+        <v>9.31</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>247329.66426</v>
+        <v>244441.52593</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-2670.33574000001</v>
+        <v>-5558.474069999997</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.01068134296000004</v>
+        <v>-0.02223389627999999</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -6390,6 +6495,9 @@
       </c>
       <c r="AY20" s="3" t="n">
         <v>9.42</v>
+      </c>
+      <c r="AZ20" s="3" t="n">
+        <v>9.31</v>
       </c>
     </row>
     <row r="21">
@@ -6415,16 +6523,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>111.9808</v>
+        <v>111.8968</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>170127.8382272</v>
+        <v>170000.2204712</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>127.8382272000017</v>
+        <v>0.2204712000093423</v>
       </c>
       <c r="I21" s="12" t="n">
-        <v>0.000751989571764716</v>
+        <v>1.29688941181966e-06</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -6551,6 +6659,9 @@
       </c>
       <c r="AY21" s="3" t="n">
         <v>111.9808</v>
+      </c>
+      <c r="AZ21" s="3" t="n">
+        <v>111.8968</v>
       </c>
     </row>
     <row r="22">
@@ -6576,16 +6687,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>44.337</v>
+        <v>45.142</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>68033.35302000001</v>
+        <v>69268.59332</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>8033.35302000001</v>
+        <v>9268.59332</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1338892170000002</v>
+        <v>0.1544765553333333</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -6706,6 +6817,9 @@
       </c>
       <c r="AY22" s="3" t="n">
         <v>44.337</v>
+      </c>
+      <c r="AZ22" s="3" t="n">
+        <v>45.142</v>
       </c>
     </row>
     <row r="23">
@@ -6731,16 +6845,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>63.8971</v>
+        <v>63.8459</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>173574.3635457</v>
+        <v>173435.2804353</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>23574.36354570001</v>
+        <v>23435.2804353</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.157162423638</v>
+        <v>0.156235202902</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -6867,6 +6981,9 @@
       </c>
       <c r="AY23" s="3" t="n">
         <v>63.8971</v>
+      </c>
+      <c r="AZ23" s="3" t="n">
+        <v>63.8459</v>
       </c>
     </row>
     <row r="24">
@@ -6892,16 +7009,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>28.2167</v>
+        <v>27.957</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>102522.1627462</v>
+        <v>101578.572402</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>2522.162746200003</v>
+        <v>1578.572402000005</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.02522162746200003</v>
+        <v>0.01578572402000005</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -7022,6 +7139,9 @@
       </c>
       <c r="AY24" s="3" t="n">
         <v>28.2167</v>
+      </c>
+      <c r="AZ24" s="3" t="n">
+        <v>27.957</v>
       </c>
     </row>
     <row r="25">
@@ -7047,16 +7167,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.7077</v>
+        <v>11.6432</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>192260.0326898</v>
+        <v>191200.8347168</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-7739.967310200009</v>
+        <v>-8799.165283200011</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.03869983655100005</v>
+        <v>-0.04399582641600006</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -7180,6 +7300,9 @@
       </c>
       <c r="AY25" s="3" t="n">
         <v>11.7077</v>
+      </c>
+      <c r="AZ25" s="3" t="n">
+        <v>11.6432</v>
       </c>
     </row>
     <row r="26">
@@ -7205,16 +7328,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>9.1891</v>
+        <v>9.124599999999999</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>109733.6133065</v>
+        <v>108963.372689</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>-266.3866934999969</v>
+        <v>-1036.627311000004</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>-0.002421697213636336</v>
+        <v>-0.009423884645454581</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -7338,6 +7461,9 @@
       </c>
       <c r="AY26" s="3" t="n">
         <v>9.1891</v>
+      </c>
+      <c r="AZ26" s="3" t="n">
+        <v>9.124599999999999</v>
       </c>
     </row>
     <row r="27">
@@ -7363,16 +7489,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>64.5823</v>
+        <v>64.77970000000001</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>104033.043778</v>
+        <v>104351.027542</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-5966.956221999993</v>
+        <v>-5648.972458000004</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.0542450565636363</v>
+        <v>-0.0513542950727273</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -7499,6 +7625,9 @@
       </c>
       <c r="AY27" s="3" t="n">
         <v>64.5823</v>
+      </c>
+      <c r="AZ27" s="3" t="n">
+        <v>64.77970000000001</v>
       </c>
     </row>
     <row r="28">
@@ -7524,16 +7653,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>108.4143</v>
+        <v>108.3414</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>358488.9039951</v>
+        <v>358247.8486998</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-21511.0960049</v>
+        <v>-21752.15130020003</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.05660814738131579</v>
+        <v>-0.05724250342157902</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -7660,6 +7789,9 @@
       </c>
       <c r="AY28" s="3" t="n">
         <v>108.4143</v>
+      </c>
+      <c r="AZ28" s="3" t="n">
+        <v>108.3414</v>
       </c>
     </row>
     <row r="29">
@@ -7685,16 +7817,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.4011</v>
+        <v>12.314</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>119096.4812733</v>
+        <v>118259.998742</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>19096.48127329999</v>
+        <v>18259.998742</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.1909648127329999</v>
+        <v>0.18259998742</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -7815,6 +7947,9 @@
       </c>
       <c r="AY29" s="3" t="n">
         <v>12.4011</v>
+      </c>
+      <c r="AZ29" s="3" t="n">
+        <v>12.314</v>
       </c>
     </row>
     <row r="30">
@@ -7840,16 +7975,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>16.5525</v>
+        <v>16.5235</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>122419.9892025</v>
+        <v>122205.5092335</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>22419.98920249999</v>
+        <v>22205.50923349999</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.2241998920249999</v>
+        <v>0.2220550923349999</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -7970,6 +8105,9 @@
       </c>
       <c r="AY30" s="3" t="n">
         <v>16.5525</v>
+      </c>
+      <c r="AZ30" s="3" t="n">
+        <v>16.5235</v>
       </c>
     </row>
     <row r="31">
@@ -7995,16 +8133,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>421.3574</v>
+        <v>420.0282</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>112114.776992</v>
+        <v>111761.103456</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>12114.77699199998</v>
+        <v>11761.103456</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.1211477699199998</v>
+        <v>0.11761103456</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -8128,6 +8266,9 @@
       </c>
       <c r="AY31" s="3" t="n">
         <v>421.3574</v>
+      </c>
+      <c r="AZ31" s="3" t="n">
+        <v>420.0282</v>
       </c>
     </row>
     <row r="32">
@@ -8153,16 +8294,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.54</v>
+        <v>10.51</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>222815.1784</v>
+        <v>222180.9796</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>22815.17839999998</v>
+        <v>22180.97959999999</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.1140758919999999</v>
+        <v>0.110904898</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -8289,6 +8430,9 @@
       </c>
       <c r="AY32" s="3" t="n">
         <v>10.54</v>
+      </c>
+      <c r="AZ32" s="3" t="n">
+        <v>10.51</v>
       </c>
     </row>
     <row r="33">
@@ -8314,16 +8458,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>18.87</v>
+        <v>18.69</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>67623.2868</v>
+        <v>66978.2316</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>7623.286800000002</v>
+        <v>6978.231599999999</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.12705478</v>
+        <v>0.11630386</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -8444,6 +8588,9 @@
       </c>
       <c r="AY33" s="3" t="n">
         <v>18.87</v>
+      </c>
+      <c r="AZ33" s="3" t="n">
+        <v>18.69</v>
       </c>
     </row>
     <row r="34">
@@ -8469,16 +8616,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>208.2005</v>
+        <v>205.4291</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>73188.92996550001</v>
+        <v>72214.6969521</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-6811.070034499993</v>
+        <v>-7785.303047900001</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.08513837543124991</v>
+        <v>-0.09731628809875001</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -8602,6 +8749,9 @@
       </c>
       <c r="AY34" s="3" t="n">
         <v>208.2005</v>
+      </c>
+      <c r="AZ34" s="3" t="n">
+        <v>205.4291</v>
       </c>
     </row>
     <row r="35">
@@ -8627,16 +8777,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>14.93</v>
+        <v>14.96</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>106531.86539</v>
+        <v>106745.92808</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>6531.865389999992</v>
+        <v>6745.928079999998</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.06531865389999991</v>
+        <v>0.06745928079999998</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -8760,6 +8910,9 @@
       </c>
       <c r="AY35" s="3" t="n">
         <v>14.93</v>
+      </c>
+      <c r="AZ35" s="3" t="n">
+        <v>14.96</v>
       </c>
     </row>
     <row r="36">
@@ -8785,16 +8938,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>366.4301</v>
+        <v>364.9704</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>170648.6961506</v>
+        <v>169968.9051024</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>20648.69615060001</v>
+        <v>19968.90510239999</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1376579743373334</v>
+        <v>0.133126034016</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -8918,6 +9071,9 @@
       </c>
       <c r="AY36" s="3" t="n">
         <v>366.4301</v>
+      </c>
+      <c r="AZ36" s="3" t="n">
+        <v>364.9704</v>
       </c>
     </row>
     <row r="37">
@@ -8943,16 +9099,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>16.343</v>
+        <v>16.306</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>61496.894927</v>
+        <v>61357.668034</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>11496.894927</v>
+        <v>11357.668034</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.22993789854</v>
+        <v>0.2271533606800001</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -9076,6 +9232,9 @@
       </c>
       <c r="AY37" s="3" t="n">
         <v>16.343</v>
+      </c>
+      <c r="AZ37" s="3" t="n">
+        <v>16.306</v>
       </c>
     </row>
     <row r="38">
@@ -9101,16 +9260,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>14.3177</v>
+        <v>14.2898</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>85626.7471314</v>
+        <v>85459.8916836</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>5626.747131399999</v>
+        <v>5459.891683599999</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.07033433914249999</v>
+        <v>0.06824864604499999</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -9231,6 +9390,9 @@
       </c>
       <c r="AY38" s="3" t="n">
         <v>14.3177</v>
+      </c>
+      <c r="AZ38" s="3" t="n">
+        <v>14.2898</v>
       </c>
     </row>
     <row r="39">
@@ -9256,16 +9418,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1021.3417</v>
+        <v>1021.4944</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50945.54533769999</v>
+        <v>50953.1621664</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>945.545337699994</v>
+        <v>953.1621664000049</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.01891090675399988</v>
+        <v>0.0190632433280001</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -9386,6 +9548,9 @@
       </c>
       <c r="AY39" s="3" t="n">
         <v>1021.3417</v>
+      </c>
+      <c r="AZ39" s="3" t="n">
+        <v>1021.4944</v>
       </c>
     </row>
     <row r="40">
@@ -9411,16 +9576,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>21.4024</v>
+        <v>21.2554</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>107890.0762648</v>
+        <v>107149.0452958</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>7890.076264799995</v>
+        <v>7149.04529580001</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.07890076264799994</v>
+        <v>0.07149045295800009</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -9544,6 +9709,9 @@
       </c>
       <c r="AY40" s="3" t="n">
         <v>21.4024</v>
+      </c>
+      <c r="AZ40" s="3" t="n">
+        <v>21.2554</v>
       </c>
     </row>
     <row r="41">
@@ -9556,13 +9724,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4930922.4790445</v>
+        <v>4919461.156848</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>460922.4790445</v>
+        <v>449461.156848</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1031146485558165</v>
+        <v>0.1005505943731543</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-06-27
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -483,7 +483,7 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-26 06:08 IST</t>
+          <t>Generated: 2026-06-27 05:52 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4919461.156848</v>
+        <v>4920365.1738469</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>449461.1568480004</v>
+        <v>450365.1738468995</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1005505943731544</v>
+        <v>0.1007528353125055</v>
       </c>
     </row>
     <row r="6">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5470671.655741738</v>
+        <v>5471575.672740637</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>409889.6357417386</v>
+        <v>410793.6527406378</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.08099333939337278</v>
+        <v>0.08117197127187031</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-06-26</t>
+          <t>Last snapshot: 2026-06-27</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY19"/>
+  <dimension ref="A1:AZ19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -670,6 +670,7 @@
     <col width="21" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
     <col width="21" customWidth="1" min="51" max="51"/>
+    <col width="21" customWidth="1" min="52" max="52"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -928,6 +929,11 @@
           <t>2026-06-26</t>
         </is>
       </c>
+      <c r="AZ1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1273,6 +1279,9 @@
       <c r="AY4" s="3" t="n">
         <v>1490</v>
       </c>
+      <c r="AZ4" s="3" t="n">
+        <v>1490</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1432,6 +1441,9 @@
       <c r="AY5" s="3" t="n">
         <v>640</v>
       </c>
+      <c r="AZ5" s="3" t="n">
+        <v>640</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1591,6 +1603,9 @@
       <c r="AY6" s="3" t="n">
         <v>379</v>
       </c>
+      <c r="AZ6" s="3" t="n">
+        <v>379</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1750,6 +1765,9 @@
       <c r="AY7" s="3" t="n">
         <v>251.8800048828125</v>
       </c>
+      <c r="AZ7" s="3" t="n">
+        <v>251.8800048828125</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1936,6 +1954,9 @@
       <c r="AY9" s="3" t="n">
         <v>17.8799991607666</v>
       </c>
+      <c r="AZ9" s="3" t="n">
+        <v>17.8799991607666</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2095,6 +2116,9 @@
       <c r="AY10" s="3" t="n">
         <v>405.9500122070312</v>
       </c>
+      <c r="AZ10" s="3" t="n">
+        <v>405.9500122070312</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2254,6 +2278,9 @@
       <c r="AY11" s="3" t="n">
         <v>8.569999694824219</v>
       </c>
+      <c r="AZ11" s="3" t="n">
+        <v>8.569999694824219</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2413,6 +2440,9 @@
       <c r="AY12" s="3" t="n">
         <v>2650</v>
       </c>
+      <c r="AZ12" s="3" t="n">
+        <v>2650</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2572,6 +2602,9 @@
       <c r="AY13" s="3" t="n">
         <v>57.0099983215332</v>
       </c>
+      <c r="AZ13" s="3" t="n">
+        <v>57.0099983215332</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2731,6 +2764,9 @@
       <c r="AY14" s="3" t="n">
         <v>745</v>
       </c>
+      <c r="AZ14" s="3" t="n">
+        <v>745</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2944,6 +2980,9 @@
       <c r="AY17" s="3" t="n">
         <v>620</v>
       </c>
+      <c r="AZ17" s="3" t="n">
+        <v>620</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3101,6 +3140,9 @@
         <v>393.8999938964844</v>
       </c>
       <c r="AY18" s="3" t="n">
+        <v>388.5499877929688</v>
+      </c>
+      <c r="AZ18" s="3" t="n">
         <v>388.5499877929688</v>
       </c>
     </row>
@@ -3131,7 +3173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ41"/>
+  <dimension ref="A1:BA41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3186,6 +3228,7 @@
     <col width="13" customWidth="1" min="50" max="50"/>
     <col width="13" customWidth="1" min="51" max="51"/>
     <col width="13" customWidth="1" min="52" max="52"/>
+    <col width="13" customWidth="1" min="53" max="53"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3449,6 +3492,11 @@
           <t>2026-06-26</t>
         </is>
       </c>
+      <c r="BA1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3613,6 +3661,9 @@
       <c r="AZ2" s="3" t="n">
         <v>56.0634</v>
       </c>
+      <c r="BA2" s="3" t="n">
+        <v>56.0634</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3637,16 +3688,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.0245</v>
+        <v>25.0798</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>61440.47771850001</v>
+        <v>61576.2509974</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>1440.477718500006</v>
+        <v>1576.250997399999</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.0240079619750001</v>
+        <v>0.02627084995666664</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -3770,6 +3821,9 @@
       </c>
       <c r="AZ3" s="3" t="n">
         <v>25.0245</v>
+      </c>
+      <c r="BA3" s="3" t="n">
+        <v>25.0798</v>
       </c>
     </row>
     <row r="4">
@@ -3795,16 +3849,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.01</v>
+        <v>12.05</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>230665.17693</v>
+        <v>231433.42065</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>50665.17693000002</v>
+        <v>51433.42065000001</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.2814732051666667</v>
+        <v>0.2857412258333334</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -3928,6 +3982,9 @@
       </c>
       <c r="AZ4" s="3" t="n">
         <v>12.01</v>
+      </c>
+      <c r="BA4" s="3" t="n">
+        <v>12.05</v>
       </c>
     </row>
     <row r="5">
@@ -4087,6 +4144,9 @@
       <c r="AZ5" s="3" t="n">
         <v>9.372</v>
       </c>
+      <c r="BA5" s="3" t="n">
+        <v>9.372</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4251,6 +4311,9 @@
       <c r="AZ6" s="3" t="n">
         <v>12.148</v>
       </c>
+      <c r="BA6" s="3" t="n">
+        <v>12.148</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4409,6 +4472,9 @@
       <c r="AZ7" s="3" t="n">
         <v>33.621</v>
       </c>
+      <c r="BA7" s="3" t="n">
+        <v>33.621</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4573,6 +4639,9 @@
       <c r="AZ8" s="3" t="n">
         <v>33.2869</v>
       </c>
+      <c r="BA8" s="3" t="n">
+        <v>33.2869</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4731,6 +4800,9 @@
       <c r="AZ9" s="3" t="n">
         <v>40.8271</v>
       </c>
+      <c r="BA9" s="3" t="n">
+        <v>40.8271</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4889,6 +4961,9 @@
       <c r="AZ10" s="3" t="n">
         <v>47.4092</v>
       </c>
+      <c r="BA10" s="3" t="n">
+        <v>47.4092</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5047,6 +5122,9 @@
       <c r="AZ11" s="3" t="n">
         <v>102.6766</v>
       </c>
+      <c r="BA11" s="3" t="n">
+        <v>102.6766</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5211,6 +5289,9 @@
       <c r="AZ12" s="3" t="n">
         <v>226.915</v>
       </c>
+      <c r="BA12" s="3" t="n">
+        <v>226.915</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5375,6 +5456,9 @@
       <c r="AZ13" s="3" t="n">
         <v>20.753</v>
       </c>
+      <c r="BA13" s="3" t="n">
+        <v>20.753</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5533,6 +5617,9 @@
       <c r="AZ14" s="3" t="n">
         <v>39.3784</v>
       </c>
+      <c r="BA14" s="3" t="n">
+        <v>39.3784</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5697,6 +5784,9 @@
       <c r="AZ15" s="3" t="n">
         <v>11.94</v>
       </c>
+      <c r="BA15" s="3" t="n">
+        <v>11.94</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5855,6 +5945,9 @@
       <c r="AZ16" s="3" t="n">
         <v>24.2127</v>
       </c>
+      <c r="BA16" s="3" t="n">
+        <v>24.2127</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -6013,6 +6106,9 @@
       <c r="AZ17" s="3" t="n">
         <v>16.796</v>
       </c>
+      <c r="BA17" s="3" t="n">
+        <v>16.796</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -6177,6 +6273,9 @@
       <c r="AZ18" s="3" t="n">
         <v>46.28</v>
       </c>
+      <c r="BA18" s="3" t="n">
+        <v>46.28</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -6335,6 +6434,9 @@
       <c r="AZ19" s="3" t="n">
         <v>14.7596</v>
       </c>
+      <c r="BA19" s="3" t="n">
+        <v>14.7596</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -6499,6 +6601,9 @@
       <c r="AZ20" s="3" t="n">
         <v>9.31</v>
       </c>
+      <c r="BA20" s="3" t="n">
+        <v>9.31</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -6663,6 +6768,9 @@
       <c r="AZ21" s="3" t="n">
         <v>111.8968</v>
       </c>
+      <c r="BA21" s="3" t="n">
+        <v>111.8968</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -6821,6 +6929,9 @@
       <c r="AZ22" s="3" t="n">
         <v>45.142</v>
       </c>
+      <c r="BA22" s="3" t="n">
+        <v>45.142</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -6985,6 +7096,9 @@
       <c r="AZ23" s="3" t="n">
         <v>63.8459</v>
       </c>
+      <c r="BA23" s="3" t="n">
+        <v>63.8459</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -7143,6 +7257,9 @@
       <c r="AZ24" s="3" t="n">
         <v>27.957</v>
       </c>
+      <c r="BA24" s="3" t="n">
+        <v>27.957</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -7304,6 +7421,9 @@
       <c r="AZ25" s="3" t="n">
         <v>11.6432</v>
       </c>
+      <c r="BA25" s="3" t="n">
+        <v>11.6432</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -7465,6 +7585,9 @@
       <c r="AZ26" s="3" t="n">
         <v>9.124599999999999</v>
       </c>
+      <c r="BA26" s="3" t="n">
+        <v>9.124599999999999</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -7629,6 +7752,9 @@
       <c r="AZ27" s="3" t="n">
         <v>64.77970000000001</v>
       </c>
+      <c r="BA27" s="3" t="n">
+        <v>64.77970000000001</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -7793,6 +7919,9 @@
       <c r="AZ28" s="3" t="n">
         <v>108.3414</v>
       </c>
+      <c r="BA28" s="3" t="n">
+        <v>108.3414</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -7951,6 +8080,9 @@
       <c r="AZ29" s="3" t="n">
         <v>12.314</v>
       </c>
+      <c r="BA29" s="3" t="n">
+        <v>12.314</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -8109,6 +8241,9 @@
       <c r="AZ30" s="3" t="n">
         <v>16.5235</v>
       </c>
+      <c r="BA30" s="3" t="n">
+        <v>16.5235</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -8270,6 +8405,9 @@
       <c r="AZ31" s="3" t="n">
         <v>420.0282</v>
       </c>
+      <c r="BA31" s="3" t="n">
+        <v>420.0282</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -8434,6 +8572,9 @@
       <c r="AZ32" s="3" t="n">
         <v>10.51</v>
       </c>
+      <c r="BA32" s="3" t="n">
+        <v>10.51</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -8592,6 +8733,9 @@
       <c r="AZ33" s="3" t="n">
         <v>18.69</v>
       </c>
+      <c r="BA33" s="3" t="n">
+        <v>18.69</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -8753,6 +8897,9 @@
       <c r="AZ34" s="3" t="n">
         <v>205.4291</v>
       </c>
+      <c r="BA34" s="3" t="n">
+        <v>205.4291</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -8914,6 +9061,9 @@
       <c r="AZ35" s="3" t="n">
         <v>14.96</v>
       </c>
+      <c r="BA35" s="3" t="n">
+        <v>14.96</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -9075,6 +9225,9 @@
       <c r="AZ36" s="3" t="n">
         <v>364.9704</v>
       </c>
+      <c r="BA36" s="3" t="n">
+        <v>364.9704</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -9236,6 +9389,9 @@
       <c r="AZ37" s="3" t="n">
         <v>16.306</v>
       </c>
+      <c r="BA37" s="3" t="n">
+        <v>16.306</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -9394,6 +9550,9 @@
       <c r="AZ38" s="3" t="n">
         <v>14.2898</v>
       </c>
+      <c r="BA38" s="3" t="n">
+        <v>14.2898</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -9552,6 +9711,9 @@
       <c r="AZ39" s="3" t="n">
         <v>1021.4944</v>
       </c>
+      <c r="BA39" s="3" t="n">
+        <v>1021.4944</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -9713,6 +9875,9 @@
       <c r="AZ40" s="3" t="n">
         <v>21.2554</v>
       </c>
+      <c r="BA40" s="3" t="n">
+        <v>21.2554</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
@@ -9724,13 +9889,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4919461.156848</v>
+        <v>4920365.1738469</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>449461.156848</v>
+        <v>450365.1738469</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1005505943731543</v>
+        <v>0.1007528353125056</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-06-28
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-27 05:52 IST</t>
+          <t>Generated: 2026-06-28 06:15 IST</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-06-27</t>
+          <t>Last snapshot: 2026-06-28</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ19"/>
+  <dimension ref="A1:BA19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -671,6 +671,7 @@
     <col width="21" customWidth="1" min="50" max="50"/>
     <col width="21" customWidth="1" min="51" max="51"/>
     <col width="21" customWidth="1" min="52" max="52"/>
+    <col width="21" customWidth="1" min="53" max="53"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -934,6 +935,11 @@
           <t>2026-06-27</t>
         </is>
       </c>
+      <c r="BA1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1093,6 +1099,9 @@
       <c r="AY2" s="3" t="n">
         <v>533.7000122070312</v>
       </c>
+      <c r="BA2" s="3" t="n">
+        <v>533.7000122070312</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1282,6 +1291,9 @@
       <c r="AZ4" s="3" t="n">
         <v>1490</v>
       </c>
+      <c r="BA4" s="3" t="n">
+        <v>1490</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1444,6 +1456,9 @@
       <c r="AZ5" s="3" t="n">
         <v>640</v>
       </c>
+      <c r="BA5" s="3" t="n">
+        <v>640</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1606,6 +1621,9 @@
       <c r="AZ6" s="3" t="n">
         <v>379</v>
       </c>
+      <c r="BA6" s="3" t="n">
+        <v>379</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1768,6 +1786,9 @@
       <c r="AZ7" s="3" t="n">
         <v>251.8800048828125</v>
       </c>
+      <c r="BA7" s="3" t="n">
+        <v>251.8800048828125</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1957,6 +1978,9 @@
       <c r="AZ9" s="3" t="n">
         <v>17.8799991607666</v>
       </c>
+      <c r="BA9" s="3" t="n">
+        <v>17.8799991607666</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2119,6 +2143,9 @@
       <c r="AZ10" s="3" t="n">
         <v>405.9500122070312</v>
       </c>
+      <c r="BA10" s="3" t="n">
+        <v>405.9500122070312</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2281,6 +2308,9 @@
       <c r="AZ11" s="3" t="n">
         <v>8.569999694824219</v>
       </c>
+      <c r="BA11" s="3" t="n">
+        <v>8.569999694824219</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2443,6 +2473,9 @@
       <c r="AZ12" s="3" t="n">
         <v>2650</v>
       </c>
+      <c r="BA12" s="3" t="n">
+        <v>2650</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2605,6 +2638,9 @@
       <c r="AZ13" s="3" t="n">
         <v>57.0099983215332</v>
       </c>
+      <c r="BA13" s="3" t="n">
+        <v>57.0099983215332</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2767,6 +2803,9 @@
       <c r="AZ14" s="3" t="n">
         <v>745</v>
       </c>
+      <c r="BA14" s="3" t="n">
+        <v>745</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2983,6 +3022,9 @@
       <c r="AZ17" s="3" t="n">
         <v>620</v>
       </c>
+      <c r="BA17" s="3" t="n">
+        <v>620</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3143,6 +3185,9 @@
         <v>388.5499877929688</v>
       </c>
       <c r="AZ18" s="3" t="n">
+        <v>388.5499877929688</v>
+      </c>
+      <c r="BA18" s="3" t="n">
         <v>388.5499877929688</v>
       </c>
     </row>
@@ -3173,7 +3218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA41"/>
+  <dimension ref="A1:BB41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3229,6 +3274,7 @@
     <col width="13" customWidth="1" min="51" max="51"/>
     <col width="13" customWidth="1" min="52" max="52"/>
     <col width="13" customWidth="1" min="53" max="53"/>
+    <col width="13" customWidth="1" min="54" max="54"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3497,6 +3543,11 @@
           <t>2026-06-27</t>
         </is>
       </c>
+      <c r="BB1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3664,6 +3715,9 @@
       <c r="BA2" s="3" t="n">
         <v>56.0634</v>
       </c>
+      <c r="BB2" s="3" t="n">
+        <v>56.0634</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3825,6 +3879,9 @@
       <c r="BA3" s="3" t="n">
         <v>25.0798</v>
       </c>
+      <c r="BB3" s="3" t="n">
+        <v>25.0798</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3986,6 +4043,9 @@
       <c r="BA4" s="3" t="n">
         <v>12.05</v>
       </c>
+      <c r="BB4" s="3" t="n">
+        <v>12.05</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4147,6 +4207,9 @@
       <c r="BA5" s="3" t="n">
         <v>9.372</v>
       </c>
+      <c r="BB5" s="3" t="n">
+        <v>9.372</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4314,6 +4377,9 @@
       <c r="BA6" s="3" t="n">
         <v>12.148</v>
       </c>
+      <c r="BB6" s="3" t="n">
+        <v>12.148</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4475,6 +4541,9 @@
       <c r="BA7" s="3" t="n">
         <v>33.621</v>
       </c>
+      <c r="BB7" s="3" t="n">
+        <v>33.621</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4642,6 +4711,9 @@
       <c r="BA8" s="3" t="n">
         <v>33.2869</v>
       </c>
+      <c r="BB8" s="3" t="n">
+        <v>33.2869</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4803,6 +4875,9 @@
       <c r="BA9" s="3" t="n">
         <v>40.8271</v>
       </c>
+      <c r="BB9" s="3" t="n">
+        <v>40.8271</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4964,6 +5039,9 @@
       <c r="BA10" s="3" t="n">
         <v>47.4092</v>
       </c>
+      <c r="BB10" s="3" t="n">
+        <v>47.4092</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5125,6 +5203,9 @@
       <c r="BA11" s="3" t="n">
         <v>102.6766</v>
       </c>
+      <c r="BB11" s="3" t="n">
+        <v>102.6766</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5292,6 +5373,9 @@
       <c r="BA12" s="3" t="n">
         <v>226.915</v>
       </c>
+      <c r="BB12" s="3" t="n">
+        <v>226.915</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5459,6 +5543,9 @@
       <c r="BA13" s="3" t="n">
         <v>20.753</v>
       </c>
+      <c r="BB13" s="3" t="n">
+        <v>20.753</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5620,6 +5707,9 @@
       <c r="BA14" s="3" t="n">
         <v>39.3784</v>
       </c>
+      <c r="BB14" s="3" t="n">
+        <v>39.3784</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5787,6 +5877,9 @@
       <c r="BA15" s="3" t="n">
         <v>11.94</v>
       </c>
+      <c r="BB15" s="3" t="n">
+        <v>11.94</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5948,6 +6041,9 @@
       <c r="BA16" s="3" t="n">
         <v>24.2127</v>
       </c>
+      <c r="BB16" s="3" t="n">
+        <v>24.2127</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -6109,6 +6205,9 @@
       <c r="BA17" s="3" t="n">
         <v>16.796</v>
       </c>
+      <c r="BB17" s="3" t="n">
+        <v>16.796</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -6276,6 +6375,9 @@
       <c r="BA18" s="3" t="n">
         <v>46.28</v>
       </c>
+      <c r="BB18" s="3" t="n">
+        <v>46.28</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -6437,6 +6539,9 @@
       <c r="BA19" s="3" t="n">
         <v>14.7596</v>
       </c>
+      <c r="BB19" s="3" t="n">
+        <v>14.7596</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -6604,6 +6709,9 @@
       <c r="BA20" s="3" t="n">
         <v>9.31</v>
       </c>
+      <c r="BB20" s="3" t="n">
+        <v>9.31</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -6771,6 +6879,9 @@
       <c r="BA21" s="3" t="n">
         <v>111.8968</v>
       </c>
+      <c r="BB21" s="3" t="n">
+        <v>111.8968</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -6932,6 +7043,9 @@
       <c r="BA22" s="3" t="n">
         <v>45.142</v>
       </c>
+      <c r="BB22" s="3" t="n">
+        <v>45.142</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -7099,6 +7213,9 @@
       <c r="BA23" s="3" t="n">
         <v>63.8459</v>
       </c>
+      <c r="BB23" s="3" t="n">
+        <v>63.8459</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -7260,6 +7377,9 @@
       <c r="BA24" s="3" t="n">
         <v>27.957</v>
       </c>
+      <c r="BB24" s="3" t="n">
+        <v>27.957</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -7424,6 +7544,9 @@
       <c r="BA25" s="3" t="n">
         <v>11.6432</v>
       </c>
+      <c r="BB25" s="3" t="n">
+        <v>11.6432</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -7588,6 +7711,9 @@
       <c r="BA26" s="3" t="n">
         <v>9.124599999999999</v>
       </c>
+      <c r="BB26" s="3" t="n">
+        <v>9.124599999999999</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -7755,6 +7881,9 @@
       <c r="BA27" s="3" t="n">
         <v>64.77970000000001</v>
       </c>
+      <c r="BB27" s="3" t="n">
+        <v>64.77970000000001</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -7922,6 +8051,9 @@
       <c r="BA28" s="3" t="n">
         <v>108.3414</v>
       </c>
+      <c r="BB28" s="3" t="n">
+        <v>108.3414</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -8083,6 +8215,9 @@
       <c r="BA29" s="3" t="n">
         <v>12.314</v>
       </c>
+      <c r="BB29" s="3" t="n">
+        <v>12.314</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -8244,6 +8379,9 @@
       <c r="BA30" s="3" t="n">
         <v>16.5235</v>
       </c>
+      <c r="BB30" s="3" t="n">
+        <v>16.5235</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -8408,6 +8546,9 @@
       <c r="BA31" s="3" t="n">
         <v>420.0282</v>
       </c>
+      <c r="BB31" s="3" t="n">
+        <v>420.0282</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -8575,6 +8716,9 @@
       <c r="BA32" s="3" t="n">
         <v>10.51</v>
       </c>
+      <c r="BB32" s="3" t="n">
+        <v>10.51</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -8736,6 +8880,9 @@
       <c r="BA33" s="3" t="n">
         <v>18.69</v>
       </c>
+      <c r="BB33" s="3" t="n">
+        <v>18.69</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -8900,6 +9047,9 @@
       <c r="BA34" s="3" t="n">
         <v>205.4291</v>
       </c>
+      <c r="BB34" s="3" t="n">
+        <v>205.4291</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -9064,6 +9214,9 @@
       <c r="BA35" s="3" t="n">
         <v>14.96</v>
       </c>
+      <c r="BB35" s="3" t="n">
+        <v>14.96</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -9228,6 +9381,9 @@
       <c r="BA36" s="3" t="n">
         <v>364.9704</v>
       </c>
+      <c r="BB36" s="3" t="n">
+        <v>364.9704</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -9392,6 +9548,9 @@
       <c r="BA37" s="3" t="n">
         <v>16.306</v>
       </c>
+      <c r="BB37" s="3" t="n">
+        <v>16.306</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -9553,6 +9712,9 @@
       <c r="BA38" s="3" t="n">
         <v>14.2898</v>
       </c>
+      <c r="BB38" s="3" t="n">
+        <v>14.2898</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -9714,6 +9876,9 @@
       <c r="BA39" s="3" t="n">
         <v>1021.4944</v>
       </c>
+      <c r="BB39" s="3" t="n">
+        <v>1021.4944</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -9876,6 +10041,9 @@
         <v>21.2554</v>
       </c>
       <c r="BA40" s="3" t="n">
+        <v>21.2554</v>
+      </c>
+      <c r="BB40" s="3" t="n">
         <v>21.2554</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily portfolio update 2026-06-29
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -484,8 +484,8 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-28 06:15 IST</t>
+          <t>Generated: 2026-06-29 06:44 IST</t>
         </is>
       </c>
     </row>
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>551210.4988937378</v>
+        <v>546206.5051727295</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-39571.52110626223</v>
+        <v>-44575.51482727053</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.06698159349240558</v>
+        <v>-0.0754517119990729</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5471575.672740637</v>
+        <v>5466571.679019629</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>410793.6527406378</v>
+        <v>405789.6590196295</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.08117197127187031</v>
+        <v>0.08018319252162327</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-06-28</t>
+          <t>Last snapshot: 2026-06-29</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA19"/>
+  <dimension ref="A1:BB19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -672,6 +672,7 @@
     <col width="21" customWidth="1" min="51" max="51"/>
     <col width="21" customWidth="1" min="52" max="52"/>
     <col width="21" customWidth="1" min="53" max="53"/>
+    <col width="21" customWidth="1" min="54" max="54"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -940,6 +941,11 @@
           <t>2026-06-28</t>
         </is>
       </c>
+      <c r="BB1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -959,13 +965,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>533.7000122070312</v>
+        <v>539.9000244140625</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>42696.0009765625</v>
+        <v>43192.001953125</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>-1121.509023437502</v>
+        <v>-625.508046875002</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1101,6 +1107,9 @@
       </c>
       <c r="BA2" s="3" t="n">
         <v>533.7000122070312</v>
+      </c>
+      <c r="BB2" s="3" t="n">
+        <v>539.9000244140625</v>
       </c>
     </row>
     <row r="3">
@@ -1148,13 +1157,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1490</v>
+        <v>1358</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>29800</v>
+        <v>27160</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-2304.580000000002</v>
+        <v>-4944.580000000002</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1293,6 +1302,9 @@
       </c>
       <c r="BA4" s="3" t="n">
         <v>1490</v>
+      </c>
+      <c r="BB4" s="3" t="n">
+        <v>1358</v>
       </c>
     </row>
     <row r="5">
@@ -1313,13 +1325,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>640</v>
+        <v>642.4500122070312</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>12800</v>
+        <v>12849.00024414062</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1413.1</v>
+        <v>-1364.099755859375</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1458,6 +1470,9 @@
       </c>
       <c r="BA5" s="3" t="n">
         <v>640</v>
+      </c>
+      <c r="BB5" s="3" t="n">
+        <v>642.4500122070312</v>
       </c>
     </row>
     <row r="6">
@@ -1478,13 +1493,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>379</v>
+        <v>374.3999938964844</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>15160</v>
+        <v>14975.99975585938</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2342.240000000002</v>
+        <v>-2526.240244140627</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1623,6 +1638,9 @@
       </c>
       <c r="BA6" s="3" t="n">
         <v>379</v>
+      </c>
+      <c r="BB6" s="3" t="n">
+        <v>374.3999938964844</v>
       </c>
     </row>
     <row r="7">
@@ -1643,13 +1661,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>251.8800048828125</v>
+        <v>244.5299987792969</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>25188.00048828125</v>
+        <v>24452.99987792969</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-1245.81951171875</v>
+        <v>-1980.820122070312</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1788,6 +1806,9 @@
       </c>
       <c r="BA7" s="3" t="n">
         <v>251.8800048828125</v>
+      </c>
+      <c r="BB7" s="3" t="n">
+        <v>244.5299987792969</v>
       </c>
     </row>
     <row r="8">
@@ -1835,13 +1856,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>17.8799991607666</v>
+        <v>17.79999923706055</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>26819.9987411499</v>
+        <v>26699.99885559082</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-4230.171258850096</v>
+        <v>-4350.171144409178</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -1980,6 +2001,9 @@
       </c>
       <c r="BA9" s="3" t="n">
         <v>17.8799991607666</v>
+      </c>
+      <c r="BB9" s="3" t="n">
+        <v>17.79999923706055</v>
       </c>
     </row>
     <row r="10">
@@ -2000,13 +2024,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>405.9500122070312</v>
+        <v>411.2000122070312</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>40595.00122070312</v>
+        <v>41120.00122070312</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-10903.47877929688</v>
+        <v>-10378.47877929688</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -2145,6 +2169,9 @@
       </c>
       <c r="BA10" s="3" t="n">
         <v>405.9500122070312</v>
+      </c>
+      <c r="BB10" s="3" t="n">
+        <v>411.2000122070312</v>
       </c>
     </row>
     <row r="11">
@@ -2165,13 +2192,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>8.569999694824219</v>
+        <v>8.520000457763672</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>8569.999694824219</v>
+        <v>8520.000457763672</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-1271.21030517578</v>
+        <v>-1321.209542236327</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -2310,6 +2337,9 @@
       </c>
       <c r="BA11" s="3" t="n">
         <v>8.569999694824219</v>
+      </c>
+      <c r="BB11" s="3" t="n">
+        <v>8.520000457763672</v>
       </c>
     </row>
     <row r="12">
@@ -2330,13 +2360,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2650</v>
+        <v>2553.60009765625</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>26500</v>
+        <v>25536.0009765625</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-1223.25</v>
+        <v>-2187.2490234375</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -2475,6 +2505,9 @@
       </c>
       <c r="BA12" s="3" t="n">
         <v>2650</v>
+      </c>
+      <c r="BB12" s="3" t="n">
+        <v>2553.60009765625</v>
       </c>
     </row>
     <row r="13">
@@ -2495,13 +2528,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>57.0099983215332</v>
+        <v>57.25</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>34205.99899291992</v>
+        <v>34350</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-825.7610070800802</v>
+        <v>-681.760000000002</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -2640,6 +2673,9 @@
       </c>
       <c r="BA13" s="3" t="n">
         <v>57.0099983215332</v>
+      </c>
+      <c r="BB13" s="3" t="n">
+        <v>57.25</v>
       </c>
     </row>
     <row r="14">
@@ -2660,13 +2696,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>745</v>
+        <v>729.9000244140625</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>37250</v>
+        <v>36495.00122070312</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-5212.510000000002</v>
+        <v>-5967.508779296877</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -2805,6 +2841,9 @@
       </c>
       <c r="BA14" s="3" t="n">
         <v>745</v>
+      </c>
+      <c r="BB14" s="3" t="n">
+        <v>729.9000244140625</v>
       </c>
     </row>
     <row r="15">
@@ -2879,13 +2918,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>620</v>
+        <v>602.7999877929688</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>31000</v>
+        <v>30139.99938964844</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>9245.470000000001</v>
+        <v>8385.469389648439</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -3024,6 +3063,9 @@
       </c>
       <c r="BA17" s="3" t="n">
         <v>620</v>
+      </c>
+      <c r="BB17" s="3" t="n">
+        <v>602.7999877929688</v>
       </c>
     </row>
     <row r="18">
@@ -3044,13 +3086,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>388.5499877929688</v>
+        <v>389.4500122070312</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>38854.99877929688</v>
+        <v>38945.00122070312</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-7785.821220703125</v>
+        <v>-7695.818779296875</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -3189,6 +3231,9 @@
       </c>
       <c r="BA18" s="3" t="n">
         <v>388.5499877929688</v>
+      </c>
+      <c r="BB18" s="3" t="n">
+        <v>389.4500122070312</v>
       </c>
     </row>
     <row r="19">
@@ -3201,10 +3246,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>551210.4988937378</v>
+        <v>546206.5051727295</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-39571.52110626222</v>
+        <v>-44575.51482727052</v>
       </c>
     </row>
   </sheetData>
@@ -3218,7 +3263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB41"/>
+  <dimension ref="A1:BC41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3275,6 +3320,7 @@
     <col width="13" customWidth="1" min="52" max="52"/>
     <col width="13" customWidth="1" min="53" max="53"/>
     <col width="13" customWidth="1" min="54" max="54"/>
+    <col width="13" customWidth="1" min="55" max="55"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3548,6 +3594,11 @@
           <t>2026-06-28</t>
         </is>
       </c>
+      <c r="BC1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3718,6 +3769,9 @@
       <c r="BB2" s="3" t="n">
         <v>56.0634</v>
       </c>
+      <c r="BC2" s="3" t="n">
+        <v>56.0634</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3882,6 +3936,9 @@
       <c r="BB3" s="3" t="n">
         <v>25.0798</v>
       </c>
+      <c r="BC3" s="3" t="n">
+        <v>25.0798</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4046,6 +4103,9 @@
       <c r="BB4" s="3" t="n">
         <v>12.05</v>
       </c>
+      <c r="BC4" s="3" t="n">
+        <v>12.05</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4210,6 +4270,9 @@
       <c r="BB5" s="3" t="n">
         <v>9.372</v>
       </c>
+      <c r="BC5" s="3" t="n">
+        <v>9.372</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4380,6 +4443,9 @@
       <c r="BB6" s="3" t="n">
         <v>12.148</v>
       </c>
+      <c r="BC6" s="3" t="n">
+        <v>12.148</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4544,6 +4610,9 @@
       <c r="BB7" s="3" t="n">
         <v>33.621</v>
       </c>
+      <c r="BC7" s="3" t="n">
+        <v>33.621</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4714,6 +4783,9 @@
       <c r="BB8" s="3" t="n">
         <v>33.2869</v>
       </c>
+      <c r="BC8" s="3" t="n">
+        <v>33.2869</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4878,6 +4950,9 @@
       <c r="BB9" s="3" t="n">
         <v>40.8271</v>
       </c>
+      <c r="BC9" s="3" t="n">
+        <v>40.8271</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5042,6 +5117,9 @@
       <c r="BB10" s="3" t="n">
         <v>47.4092</v>
       </c>
+      <c r="BC10" s="3" t="n">
+        <v>47.4092</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5206,6 +5284,9 @@
       <c r="BB11" s="3" t="n">
         <v>102.6766</v>
       </c>
+      <c r="BC11" s="3" t="n">
+        <v>102.6766</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5376,6 +5457,9 @@
       <c r="BB12" s="3" t="n">
         <v>226.915</v>
       </c>
+      <c r="BC12" s="3" t="n">
+        <v>226.915</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5546,6 +5630,9 @@
       <c r="BB13" s="3" t="n">
         <v>20.753</v>
       </c>
+      <c r="BC13" s="3" t="n">
+        <v>20.753</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5710,6 +5797,9 @@
       <c r="BB14" s="3" t="n">
         <v>39.3784</v>
       </c>
+      <c r="BC14" s="3" t="n">
+        <v>39.3784</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5880,6 +5970,9 @@
       <c r="BB15" s="3" t="n">
         <v>11.94</v>
       </c>
+      <c r="BC15" s="3" t="n">
+        <v>11.94</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -6044,6 +6137,9 @@
       <c r="BB16" s="3" t="n">
         <v>24.2127</v>
       </c>
+      <c r="BC16" s="3" t="n">
+        <v>24.2127</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -6208,6 +6304,9 @@
       <c r="BB17" s="3" t="n">
         <v>16.796</v>
       </c>
+      <c r="BC17" s="3" t="n">
+        <v>16.796</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -6378,6 +6477,9 @@
       <c r="BB18" s="3" t="n">
         <v>46.28</v>
       </c>
+      <c r="BC18" s="3" t="n">
+        <v>46.28</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -6542,6 +6644,9 @@
       <c r="BB19" s="3" t="n">
         <v>14.7596</v>
       </c>
+      <c r="BC19" s="3" t="n">
+        <v>14.7596</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -6712,6 +6817,9 @@
       <c r="BB20" s="3" t="n">
         <v>9.31</v>
       </c>
+      <c r="BC20" s="3" t="n">
+        <v>9.31</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -6882,6 +6990,9 @@
       <c r="BB21" s="3" t="n">
         <v>111.8968</v>
       </c>
+      <c r="BC21" s="3" t="n">
+        <v>111.8968</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -7046,6 +7157,9 @@
       <c r="BB22" s="3" t="n">
         <v>45.142</v>
       </c>
+      <c r="BC22" s="3" t="n">
+        <v>45.142</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -7216,6 +7330,9 @@
       <c r="BB23" s="3" t="n">
         <v>63.8459</v>
       </c>
+      <c r="BC23" s="3" t="n">
+        <v>63.8459</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -7380,6 +7497,9 @@
       <c r="BB24" s="3" t="n">
         <v>27.957</v>
       </c>
+      <c r="BC24" s="3" t="n">
+        <v>27.957</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -7547,6 +7667,9 @@
       <c r="BB25" s="3" t="n">
         <v>11.6432</v>
       </c>
+      <c r="BC25" s="3" t="n">
+        <v>11.6432</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -7714,6 +7837,9 @@
       <c r="BB26" s="3" t="n">
         <v>9.124599999999999</v>
       </c>
+      <c r="BC26" s="3" t="n">
+        <v>9.124599999999999</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -7884,6 +8010,9 @@
       <c r="BB27" s="3" t="n">
         <v>64.77970000000001</v>
       </c>
+      <c r="BC27" s="3" t="n">
+        <v>64.77970000000001</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -8054,6 +8183,9 @@
       <c r="BB28" s="3" t="n">
         <v>108.3414</v>
       </c>
+      <c r="BC28" s="3" t="n">
+        <v>108.3414</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -8218,6 +8350,9 @@
       <c r="BB29" s="3" t="n">
         <v>12.314</v>
       </c>
+      <c r="BC29" s="3" t="n">
+        <v>12.314</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -8382,6 +8517,9 @@
       <c r="BB30" s="3" t="n">
         <v>16.5235</v>
       </c>
+      <c r="BC30" s="3" t="n">
+        <v>16.5235</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -8549,6 +8687,9 @@
       <c r="BB31" s="3" t="n">
         <v>420.0282</v>
       </c>
+      <c r="BC31" s="3" t="n">
+        <v>420.0282</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -8719,6 +8860,9 @@
       <c r="BB32" s="3" t="n">
         <v>10.51</v>
       </c>
+      <c r="BC32" s="3" t="n">
+        <v>10.51</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -8883,6 +9027,9 @@
       <c r="BB33" s="3" t="n">
         <v>18.69</v>
       </c>
+      <c r="BC33" s="3" t="n">
+        <v>18.69</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -9050,6 +9197,9 @@
       <c r="BB34" s="3" t="n">
         <v>205.4291</v>
       </c>
+      <c r="BC34" s="3" t="n">
+        <v>205.4291</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -9217,6 +9367,9 @@
       <c r="BB35" s="3" t="n">
         <v>14.96</v>
       </c>
+      <c r="BC35" s="3" t="n">
+        <v>14.96</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -9384,6 +9537,9 @@
       <c r="BB36" s="3" t="n">
         <v>364.9704</v>
       </c>
+      <c r="BC36" s="3" t="n">
+        <v>364.9704</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -9551,6 +9707,9 @@
       <c r="BB37" s="3" t="n">
         <v>16.306</v>
       </c>
+      <c r="BC37" s="3" t="n">
+        <v>16.306</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -9715,6 +9874,9 @@
       <c r="BB38" s="3" t="n">
         <v>14.2898</v>
       </c>
+      <c r="BC38" s="3" t="n">
+        <v>14.2898</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -9879,6 +10041,9 @@
       <c r="BB39" s="3" t="n">
         <v>1021.4944</v>
       </c>
+      <c r="BC39" s="3" t="n">
+        <v>1021.4944</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -10044,6 +10209,9 @@
         <v>21.2554</v>
       </c>
       <c r="BB40" s="3" t="n">
+        <v>21.2554</v>
+      </c>
+      <c r="BC40" s="3" t="n">
         <v>21.2554</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily portfolio update 2026-06-30
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -483,9 +483,9 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-29 06:44 IST</t>
+          <t>Generated: 2026-06-30 06:09 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4920365.1738469</v>
+        <v>4900930.8690117</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>450365.1738468995</v>
+        <v>430930.8690117002</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1007528353125055</v>
+        <v>0.09640511611000004</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>546206.5051727295</v>
+        <v>546366.0015945435</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-44575.51482727053</v>
+        <v>-44416.01840545656</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.0754517119990729</v>
+        <v>-0.07518173692127016</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5466571.679019629</v>
+        <v>5447296.870606244</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>405789.6590196295</v>
+        <v>386514.8506062441</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.08018319252162327</v>
+        <v>0.07637453047350261</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-06-29</t>
+          <t>Last snapshot: 2026-06-30</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB19"/>
+  <dimension ref="A1:BC19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -673,6 +673,7 @@
     <col width="21" customWidth="1" min="52" max="52"/>
     <col width="21" customWidth="1" min="53" max="53"/>
     <col width="21" customWidth="1" min="54" max="54"/>
+    <col width="21" customWidth="1" min="55" max="55"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -946,6 +947,11 @@
           <t>2026-06-29</t>
         </is>
       </c>
+      <c r="BC1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -965,13 +971,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>539.9000244140625</v>
+        <v>537</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>43192.001953125</v>
+        <v>42960</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>-625.508046875002</v>
+        <v>-857.510000000002</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1110,6 +1116,9 @@
       </c>
       <c r="BB2" s="3" t="n">
         <v>539.9000244140625</v>
+      </c>
+      <c r="BC2" s="3" t="n">
+        <v>537</v>
       </c>
     </row>
     <row r="3">
@@ -1157,13 +1166,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1358</v>
+        <v>1354.099975585938</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>27160</v>
+        <v>27081.99951171875</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-4944.580000000002</v>
+        <v>-5022.580488281252</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1305,6 +1314,9 @@
       </c>
       <c r="BB4" s="3" t="n">
         <v>1358</v>
+      </c>
+      <c r="BC4" s="3" t="n">
+        <v>1354.099975585938</v>
       </c>
     </row>
     <row r="5">
@@ -1325,13 +1337,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>642.4500122070312</v>
+        <v>643.3499755859375</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>12849.00024414062</v>
+        <v>12866.99951171875</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1364.099755859375</v>
+        <v>-1346.10048828125</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1473,6 +1485,9 @@
       </c>
       <c r="BB5" s="3" t="n">
         <v>642.4500122070312</v>
+      </c>
+      <c r="BC5" s="3" t="n">
+        <v>643.3499755859375</v>
       </c>
     </row>
     <row r="6">
@@ -1493,13 +1508,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>374.3999938964844</v>
+        <v>372.5</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>14975.99975585938</v>
+        <v>14900</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2526.240244140627</v>
+        <v>-2602.240000000002</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1641,6 +1656,9 @@
       </c>
       <c r="BB6" s="3" t="n">
         <v>374.3999938964844</v>
+      </c>
+      <c r="BC6" s="3" t="n">
+        <v>372.5</v>
       </c>
     </row>
     <row r="7">
@@ -1661,13 +1679,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>244.5299987792969</v>
+        <v>240.0299987792969</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>24452.99987792969</v>
+        <v>24002.99987792969</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-1980.820122070312</v>
+        <v>-2430.820122070312</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1809,6 +1827,9 @@
       </c>
       <c r="BB7" s="3" t="n">
         <v>244.5299987792969</v>
+      </c>
+      <c r="BC7" s="3" t="n">
+        <v>240.0299987792969</v>
       </c>
     </row>
     <row r="8">
@@ -1856,13 +1877,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>17.79999923706055</v>
+        <v>17.69000053405762</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>26699.99885559082</v>
+        <v>26535.00080108643</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-4350.171144409178</v>
+        <v>-4515.169198913572</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -2004,6 +2025,9 @@
       </c>
       <c r="BB9" s="3" t="n">
         <v>17.79999923706055</v>
+      </c>
+      <c r="BC9" s="3" t="n">
+        <v>17.69000053405762</v>
       </c>
     </row>
     <row r="10">
@@ -2024,13 +2048,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>411.2000122070312</v>
+        <v>417</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>41120.00122070312</v>
+        <v>41700</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-10378.47877929688</v>
+        <v>-9798.480000000003</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -2172,6 +2196,9 @@
       </c>
       <c r="BB10" s="3" t="n">
         <v>411.2000122070312</v>
+      </c>
+      <c r="BC10" s="3" t="n">
+        <v>417</v>
       </c>
     </row>
     <row r="11">
@@ -2192,13 +2219,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>8.520000457763672</v>
+        <v>8.770000457763672</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>8520.000457763672</v>
+        <v>8770.000457763672</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-1321.209542236327</v>
+        <v>-1071.209542236327</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -2340,6 +2367,9 @@
       </c>
       <c r="BB11" s="3" t="n">
         <v>8.520000457763672</v>
+      </c>
+      <c r="BC11" s="3" t="n">
+        <v>8.770000457763672</v>
       </c>
     </row>
     <row r="12">
@@ -2360,13 +2390,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2553.60009765625</v>
+        <v>2537</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25536.0009765625</v>
+        <v>25370</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2187.2490234375</v>
+        <v>-2353.25</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -2508,6 +2538,9 @@
       </c>
       <c r="BB12" s="3" t="n">
         <v>2553.60009765625</v>
+      </c>
+      <c r="BC12" s="3" t="n">
+        <v>2537</v>
       </c>
     </row>
     <row r="13">
@@ -2528,13 +2561,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>57.25</v>
+        <v>57.7599983215332</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>34350</v>
+        <v>34655.99899291992</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-681.760000000002</v>
+        <v>-375.7610070800802</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -2676,6 +2709,9 @@
       </c>
       <c r="BB13" s="3" t="n">
         <v>57.25</v>
+      </c>
+      <c r="BC13" s="3" t="n">
+        <v>57.7599983215332</v>
       </c>
     </row>
     <row r="14">
@@ -2696,13 +2732,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>729.9000244140625</v>
+        <v>724.1500244140625</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>36495.00122070312</v>
+        <v>36207.50122070312</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-5967.508779296877</v>
+        <v>-6255.008779296877</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -2844,6 +2880,9 @@
       </c>
       <c r="BB14" s="3" t="n">
         <v>729.9000244140625</v>
+      </c>
+      <c r="BC14" s="3" t="n">
+        <v>724.1500244140625</v>
       </c>
     </row>
     <row r="15">
@@ -2918,13 +2957,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>602.7999877929688</v>
+        <v>619.2000122070312</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>30139.99938964844</v>
+        <v>30960.00061035156</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>8385.469389648439</v>
+        <v>9205.470610351564</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -3066,6 +3105,9 @@
       </c>
       <c r="BB17" s="3" t="n">
         <v>602.7999877929688</v>
+      </c>
+      <c r="BC17" s="3" t="n">
+        <v>619.2000122070312</v>
       </c>
     </row>
     <row r="18">
@@ -3086,13 +3128,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>389.4500122070312</v>
+        <v>385.8500061035156</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>38945.00122070312</v>
+        <v>38585.00061035156</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-7695.818779296875</v>
+        <v>-8055.819389648437</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -3234,6 +3276,9 @@
       </c>
       <c r="BB18" s="3" t="n">
         <v>389.4500122070312</v>
+      </c>
+      <c r="BC18" s="3" t="n">
+        <v>385.8500061035156</v>
       </c>
     </row>
     <row r="19">
@@ -3246,10 +3291,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>546206.5051727295</v>
+        <v>546366.0015945435</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-44575.51482727052</v>
+        <v>-44416.01840545655</v>
       </c>
     </row>
   </sheetData>
@@ -3263,7 +3308,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BC41"/>
+  <dimension ref="A1:BD41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3321,6 +3366,7 @@
     <col width="13" customWidth="1" min="53" max="53"/>
     <col width="13" customWidth="1" min="54" max="54"/>
     <col width="13" customWidth="1" min="55" max="55"/>
+    <col width="13" customWidth="1" min="56" max="56"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3599,6 +3645,11 @@
           <t>2026-06-29</t>
         </is>
       </c>
+      <c r="BD1" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3623,16 +3674,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.0634</v>
+        <v>56.4098</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>62930.1573588</v>
+        <v>63318.9851236</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>12930.1573588</v>
+        <v>13318.9851236</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.2586031471760001</v>
+        <v>0.2663797024719999</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -3771,6 +3822,9 @@
       </c>
       <c r="BC2" s="3" t="n">
         <v>56.0634</v>
+      </c>
+      <c r="BD2" s="3" t="n">
+        <v>56.4098</v>
       </c>
     </row>
     <row r="3">
@@ -3796,16 +3850,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.0798</v>
+        <v>25.0331</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>61576.2509974</v>
+        <v>61461.59255030001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>1576.250997399999</v>
+        <v>1461.592550300011</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.02627084995666664</v>
+        <v>0.02435987583833351</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -3938,6 +3992,9 @@
       </c>
       <c r="BC3" s="3" t="n">
         <v>25.0798</v>
+      </c>
+      <c r="BD3" s="3" t="n">
+        <v>25.0331</v>
       </c>
     </row>
     <row r="4">
@@ -3963,16 +4020,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.05</v>
+        <v>11.87</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>231433.42065</v>
+        <v>227976.32391</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>51433.42065000001</v>
+        <v>47976.32391000001</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.2857412258333334</v>
+        <v>0.2665351328333334</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -4105,6 +4162,9 @@
       </c>
       <c r="BC4" s="3" t="n">
         <v>12.05</v>
+      </c>
+      <c r="BD4" s="3" t="n">
+        <v>11.87</v>
       </c>
     </row>
     <row r="5">
@@ -4130,16 +4190,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.372</v>
+        <v>9.3001</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>172014.512736</v>
+        <v>170694.8538088</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-37985.487264</v>
+        <v>-39305.14619119998</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1808832726857143</v>
+        <v>-0.187167362815238</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -4272,6 +4332,9 @@
       </c>
       <c r="BC5" s="3" t="n">
         <v>9.372</v>
+      </c>
+      <c r="BD5" s="3" t="n">
+        <v>9.3001</v>
       </c>
     </row>
     <row r="6">
@@ -4297,16 +4360,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.148</v>
+        <v>12.1758</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>51373.612596</v>
+        <v>51491.1781566</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>1373.612595999999</v>
+        <v>1491.178156599999</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.02747225191999998</v>
+        <v>0.02982356313199998</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -4445,6 +4508,9 @@
       </c>
       <c r="BC6" s="3" t="n">
         <v>12.148</v>
+      </c>
+      <c r="BD6" s="3" t="n">
+        <v>12.1758</v>
       </c>
     </row>
     <row r="7">
@@ -4470,16 +4536,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.621</v>
+        <v>33.6281</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>74169.27084</v>
+        <v>74184.933724</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>14169.27084</v>
+        <v>14184.933724</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.236154514</v>
+        <v>0.2364155620666667</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -4612,6 +4678,9 @@
       </c>
       <c r="BC7" s="3" t="n">
         <v>33.621</v>
+      </c>
+      <c r="BD7" s="3" t="n">
+        <v>33.6281</v>
       </c>
     </row>
     <row r="8">
@@ -4637,16 +4706,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>33.2869</v>
+        <v>33.4275</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>53411.9267317</v>
+        <v>53637.53250750001</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>3411.926731700005</v>
+        <v>3637.532507500007</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.06823853463400009</v>
+        <v>0.07275065015000015</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -4785,6 +4854,9 @@
       </c>
       <c r="BC8" s="3" t="n">
         <v>33.2869</v>
+      </c>
+      <c r="BD8" s="3" t="n">
+        <v>33.4275</v>
       </c>
     </row>
     <row r="9">
@@ -4810,16 +4882,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>40.8271</v>
+        <v>41.3016</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>131438.4799503</v>
+        <v>132966.0819288</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>31438.47995030001</v>
+        <v>32966.08192880001</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3143847995030001</v>
+        <v>0.3296608192880001</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -4952,6 +5024,9 @@
       </c>
       <c r="BC9" s="3" t="n">
         <v>40.8271</v>
+      </c>
+      <c r="BD9" s="3" t="n">
+        <v>41.3016</v>
       </c>
     </row>
     <row r="10">
@@ -4977,16 +5052,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>47.4092</v>
+        <v>47.2178</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>134957.8258628</v>
+        <v>134412.9753302</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>34957.8258628</v>
+        <v>34412.97533019999</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.349578258628</v>
+        <v>0.3441297533019999</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -5119,6 +5194,9 @@
       </c>
       <c r="BC10" s="3" t="n">
         <v>47.4092</v>
+      </c>
+      <c r="BD10" s="3" t="n">
+        <v>47.2178</v>
       </c>
     </row>
     <row r="11">
@@ -5144,16 +5222,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>102.6766</v>
+        <v>104.1402</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>30897.3397954</v>
+        <v>31337.7648438</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>897.3397953999956</v>
+        <v>1337.764843799996</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.02991132651333319</v>
+        <v>0.04459216145999987</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -5286,6 +5364,9 @@
       </c>
       <c r="BC11" s="3" t="n">
         <v>102.6766</v>
+      </c>
+      <c r="BD11" s="3" t="n">
+        <v>104.1402</v>
       </c>
     </row>
     <row r="12">
@@ -5311,16 +5392,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>226.915</v>
+        <v>225.317</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>105633.92463</v>
+        <v>104890.020474</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>5633.924629999994</v>
+        <v>4890.020474000004</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.05633924629999994</v>
+        <v>0.04890020474000004</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -5459,6 +5540,9 @@
       </c>
       <c r="BC12" s="3" t="n">
         <v>226.915</v>
+      </c>
+      <c r="BD12" s="3" t="n">
+        <v>225.317</v>
       </c>
     </row>
     <row r="13">
@@ -5484,16 +5568,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>20.753</v>
+        <v>20.924</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>240477.566565</v>
+        <v>242459.04702</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>40477.56656499999</v>
+        <v>42459.04702</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.2023878328249999</v>
+        <v>0.2122952351</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -5632,6 +5716,9 @@
       </c>
       <c r="BC13" s="3" t="n">
         <v>20.753</v>
+      </c>
+      <c r="BD13" s="3" t="n">
+        <v>20.924</v>
       </c>
     </row>
     <row r="14">
@@ -5657,16 +5744,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>39.3784</v>
+        <v>37.9691</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>142061.7521104</v>
+        <v>136977.5529746</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>42061.7521104</v>
+        <v>36977.5529746</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.420617521104</v>
+        <v>0.369775529746</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -5799,6 +5886,9 @@
       </c>
       <c r="BC14" s="3" t="n">
         <v>39.3784</v>
+      </c>
+      <c r="BD14" s="3" t="n">
+        <v>37.9691</v>
       </c>
     </row>
     <row r="15">
@@ -5824,16 +5914,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.94</v>
+        <v>11.9</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>116342.72718</v>
+        <v>115952.9693</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>16342.72718</v>
+        <v>15952.96930000001</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1634272718</v>
+        <v>0.1595296930000001</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -5972,6 +6062,9 @@
       </c>
       <c r="BC15" s="3" t="n">
         <v>11.94</v>
+      </c>
+      <c r="BD15" s="3" t="n">
+        <v>11.9</v>
       </c>
     </row>
     <row r="16">
@@ -5997,16 +6090,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.2127</v>
+        <v>24.4531</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>138567.5387856</v>
+        <v>139943.3306768</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>38567.53878560002</v>
+        <v>39943.33067679999</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.3856753878560001</v>
+        <v>0.3994333067679999</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -6139,6 +6232,9 @@
       </c>
       <c r="BC16" s="3" t="n">
         <v>24.2127</v>
+      </c>
+      <c r="BD16" s="3" t="n">
+        <v>24.4531</v>
       </c>
     </row>
     <row r="17">
@@ -6164,16 +6260,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.796</v>
+        <v>16.7695</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55528.53337199999</v>
+        <v>55440.9228615</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5528.533371999991</v>
+        <v>5440.922861499996</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1105706674399998</v>
+        <v>0.1088184572299999</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -6306,6 +6402,9 @@
       </c>
       <c r="BC17" s="3" t="n">
         <v>16.796</v>
+      </c>
+      <c r="BD17" s="3" t="n">
+        <v>16.7695</v>
       </c>
     </row>
     <row r="18">
@@ -6331,16 +6430,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>46.28</v>
+        <v>46.38</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>87304.25808</v>
+        <v>87492.90168</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>7304.25808</v>
+        <v>7492.901679999995</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.091303226</v>
+        <v>0.09366127099999995</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -6479,6 +6578,9 @@
       </c>
       <c r="BC18" s="3" t="n">
         <v>46.28</v>
+      </c>
+      <c r="BD18" s="3" t="n">
+        <v>46.38</v>
       </c>
     </row>
     <row r="19">
@@ -6504,16 +6606,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>14.7596</v>
+        <v>14.4768</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>213523.6794536</v>
+        <v>209432.4780288</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>63523.67945359999</v>
+        <v>59432.47802880002</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.4234911963573333</v>
+        <v>0.3962165201920001</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -6646,6 +6748,9 @@
       </c>
       <c r="BC19" s="3" t="n">
         <v>14.7596</v>
+      </c>
+      <c r="BD19" s="3" t="n">
+        <v>14.4768</v>
       </c>
     </row>
     <row r="20">
@@ -6671,16 +6776,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.31</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>244441.52593</v>
+        <v>241553.3876</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-5558.474069999997</v>
+        <v>-8446.612400000013</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.02223389627999999</v>
+        <v>-0.03378644960000005</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -6819,6 +6924,9 @@
       </c>
       <c r="BC20" s="3" t="n">
         <v>9.31</v>
+      </c>
+      <c r="BD20" s="3" t="n">
+        <v>9.199999999999999</v>
       </c>
     </row>
     <row r="21">
@@ -6844,16 +6952,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>111.8968</v>
+        <v>111.5854</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>170000.2204712</v>
-      </c>
-      <c r="H21" s="4" t="n">
-        <v>0.2204712000093423</v>
-      </c>
-      <c r="I21" s="12" t="n">
-        <v>1.29688941181966e-06</v>
+        <v>169527.1232186</v>
+      </c>
+      <c r="H21" s="6" t="n">
+        <v>-472.8767814000021</v>
+      </c>
+      <c r="I21" s="13" t="n">
+        <v>-0.002781628125882365</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -6992,6 +7100,9 @@
       </c>
       <c r="BC21" s="3" t="n">
         <v>111.8968</v>
+      </c>
+      <c r="BD21" s="3" t="n">
+        <v>111.5854</v>
       </c>
     </row>
     <row r="22">
@@ -7017,16 +7128,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>45.142</v>
+        <v>43.655</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>69268.59332</v>
+        <v>66986.85130000001</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>9268.59332</v>
+        <v>6986.851300000009</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1544765553333333</v>
+        <v>0.1164475216666668</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -7159,6 +7270,9 @@
       </c>
       <c r="BC22" s="3" t="n">
         <v>45.142</v>
+      </c>
+      <c r="BD22" s="3" t="n">
+        <v>43.655</v>
       </c>
     </row>
     <row r="23">
@@ -7184,16 +7298,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>63.8459</v>
+        <v>63.542</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>173435.2804353</v>
+        <v>172609.746114</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>23435.2804353</v>
+        <v>22609.74611400001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.156235202902</v>
+        <v>0.1507316407600001</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -7332,6 +7446,9 @@
       </c>
       <c r="BC23" s="3" t="n">
         <v>63.8459</v>
+      </c>
+      <c r="BD23" s="3" t="n">
+        <v>63.542</v>
       </c>
     </row>
     <row r="24">
@@ -7357,16 +7474,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>27.957</v>
+        <v>27.7279</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>101578.572402</v>
+        <v>100746.1636694</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>1578.572402000005</v>
+        <v>746.1636694000044</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.01578572402000005</v>
+        <v>0.007461636694000045</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -7499,6 +7616,9 @@
       </c>
       <c r="BC24" s="3" t="n">
         <v>27.957</v>
+      </c>
+      <c r="BD24" s="3" t="n">
+        <v>27.7279</v>
       </c>
     </row>
     <row r="25">
@@ -7524,16 +7644,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.6432</v>
+        <v>11.5302</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>191200.8347168</v>
+        <v>189345.1855548</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-8799.165283200011</v>
+        <v>-10654.8144452</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.04399582641600006</v>
+        <v>-0.05327407222599999</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -7669,6 +7789,9 @@
       </c>
       <c r="BC25" s="3" t="n">
         <v>11.6432</v>
+      </c>
+      <c r="BD25" s="3" t="n">
+        <v>11.5302</v>
       </c>
     </row>
     <row r="26">
@@ -7694,16 +7817,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>9.124599999999999</v>
+        <v>9.0952</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>108963.372689</v>
+        <v>108612.286268</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>-1036.627311000004</v>
+        <v>-1387.713732000004</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>-0.009423884645454581</v>
+        <v>-0.01261557938181822</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -7839,6 +7962,9 @@
       </c>
       <c r="BC26" s="3" t="n">
         <v>9.124599999999999</v>
+      </c>
+      <c r="BD26" s="3" t="n">
+        <v>9.0952</v>
       </c>
     </row>
     <row r="27">
@@ -7864,16 +7990,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>64.77970000000001</v>
+        <v>64.8481</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>104351.027542</v>
+        <v>104461.210366</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-5648.972458000004</v>
+        <v>-5538.789634000001</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.0513542950727273</v>
+        <v>-0.05035263303636364</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -8012,6 +8138,9 @@
       </c>
       <c r="BC27" s="3" t="n">
         <v>64.77970000000001</v>
+      </c>
+      <c r="BD27" s="3" t="n">
+        <v>64.8481</v>
       </c>
     </row>
     <row r="28">
@@ -8037,16 +8166,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>108.3414</v>
+        <v>107.8072</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>358247.8486998</v>
+        <v>356481.4325304</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-21752.15130020003</v>
+        <v>-23518.56746960001</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.05724250342157902</v>
+        <v>-0.06189096702526317</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -8185,6 +8314,9 @@
       </c>
       <c r="BC28" s="3" t="n">
         <v>108.3414</v>
+      </c>
+      <c r="BD28" s="3" t="n">
+        <v>107.8072</v>
       </c>
     </row>
     <row r="29">
@@ -8210,16 +8342,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.314</v>
+        <v>12.3051</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>118259.998742</v>
+        <v>118174.5257853</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>18259.998742</v>
+        <v>18174.52578529999</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.18259998742</v>
+        <v>0.1817452578529999</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -8352,6 +8484,9 @@
       </c>
       <c r="BC29" s="3" t="n">
         <v>12.314</v>
+      </c>
+      <c r="BD29" s="3" t="n">
+        <v>12.3051</v>
       </c>
     </row>
     <row r="30">
@@ -8377,16 +8512,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>16.5235</v>
+        <v>16.4715</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>122205.5092335</v>
+        <v>121820.9244615</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>22205.50923349999</v>
+        <v>21820.92446149999</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.2220550923349999</v>
+        <v>0.2182092446149999</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -8519,6 +8654,9 @@
       </c>
       <c r="BC30" s="3" t="n">
         <v>16.5235</v>
+      </c>
+      <c r="BD30" s="3" t="n">
+        <v>16.4715</v>
       </c>
     </row>
     <row r="31">
@@ -8544,16 +8682,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>420.0282</v>
+        <v>418.7475</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>111761.103456</v>
+        <v>111420.3348</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>11761.103456</v>
+        <v>11420.3348</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.11761103456</v>
+        <v>0.114203348</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -8689,6 +8827,9 @@
       </c>
       <c r="BC31" s="3" t="n">
         <v>420.0282</v>
+      </c>
+      <c r="BD31" s="3" t="n">
+        <v>418.7475</v>
       </c>
     </row>
     <row r="32">
@@ -8714,16 +8855,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.51</v>
+        <v>10.48</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>222180.9796</v>
+        <v>221546.7808</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>22180.97959999999</v>
+        <v>21546.78080000001</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.110904898</v>
+        <v>0.107733904</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -8862,6 +9003,9 @@
       </c>
       <c r="BC32" s="3" t="n">
         <v>10.51</v>
+      </c>
+      <c r="BD32" s="3" t="n">
+        <v>10.48</v>
       </c>
     </row>
     <row r="33">
@@ -8887,16 +9031,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>18.69</v>
+        <v>18.71</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>66978.2316</v>
+        <v>67049.9044</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>6978.231599999999</v>
+        <v>7049.904399999999</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.11630386</v>
+        <v>0.1174984066666667</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -9029,6 +9173,9 @@
       </c>
       <c r="BC33" s="3" t="n">
         <v>18.69</v>
+      </c>
+      <c r="BD33" s="3" t="n">
+        <v>18.71</v>
       </c>
     </row>
     <row r="34">
@@ -9054,16 +9201,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>205.4291</v>
+        <v>205.3031</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>72214.6969521</v>
+        <v>72170.4040461</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-7785.303047900001</v>
+        <v>-7829.595953900003</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.09731628809875001</v>
+        <v>-0.09786994942375005</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -9199,6 +9346,9 @@
       </c>
       <c r="BC34" s="3" t="n">
         <v>205.4291</v>
+      </c>
+      <c r="BD34" s="3" t="n">
+        <v>205.3031</v>
       </c>
     </row>
     <row r="35">
@@ -9224,16 +9374,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>14.96</v>
+        <v>15.09</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>106745.92808</v>
+        <v>107673.53307</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>6745.928079999998</v>
+        <v>7673.53306999999</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.06745928079999998</v>
+        <v>0.07673533069999991</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -9369,6 +9519,9 @@
       </c>
       <c r="BC35" s="3" t="n">
         <v>14.96</v>
+      </c>
+      <c r="BD35" s="3" t="n">
+        <v>15.09</v>
       </c>
     </row>
     <row r="36">
@@ -9394,16 +9547,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>364.9704</v>
+        <v>367.1375</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>169968.9051024</v>
+        <v>170978.136575</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>19968.90510239999</v>
+        <v>20978.13657500001</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.133126034016</v>
+        <v>0.1398542438333334</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -9539,6 +9692,9 @@
       </c>
       <c r="BC36" s="3" t="n">
         <v>364.9704</v>
+      </c>
+      <c r="BD36" s="3" t="n">
+        <v>367.1375</v>
       </c>
     </row>
     <row r="37">
@@ -9564,16 +9720,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>16.306</v>
+        <v>16.508</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>61357.668034</v>
+        <v>62117.771612</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>11357.668034</v>
+        <v>12117.771612</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.2271533606800001</v>
+        <v>0.2423554322399999</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -9709,6 +9865,9 @@
       </c>
       <c r="BC37" s="3" t="n">
         <v>16.306</v>
+      </c>
+      <c r="BD37" s="3" t="n">
+        <v>16.508</v>
       </c>
     </row>
     <row r="38">
@@ -9734,16 +9893,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>14.2898</v>
+        <v>14.2291</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>85459.8916836</v>
+        <v>85096.8764262</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>5459.891683599999</v>
+        <v>5096.876426200004</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.06824864604499999</v>
+        <v>0.06371095532750005</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -9876,6 +10035,9 @@
       </c>
       <c r="BC38" s="3" t="n">
         <v>14.2898</v>
+      </c>
+      <c r="BD38" s="3" t="n">
+        <v>14.2291</v>
       </c>
     </row>
     <row r="39">
@@ -9901,16 +10063,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1021.4944</v>
+        <v>1022.2323</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50953.1621664</v>
+        <v>50989.9693563</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>953.1621664000049</v>
+        <v>989.9693563000037</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.0190632433280001</v>
+        <v>0.01979938712600007</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -10043,6 +10205,9 @@
       </c>
       <c r="BC39" s="3" t="n">
         <v>1021.4944</v>
+      </c>
+      <c r="BD39" s="3" t="n">
+        <v>1022.2323</v>
       </c>
     </row>
     <row r="40">
@@ -10068,16 +10233,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>21.2554</v>
+        <v>21.3244</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>107149.0452958</v>
+        <v>107496.8761588</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>7149.04529580001</v>
+        <v>7496.876158800005</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.07149045295800009</v>
+        <v>0.07496876158800005</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -10213,6 +10378,9 @@
       </c>
       <c r="BC40" s="3" t="n">
         <v>21.2554</v>
+      </c>
+      <c r="BD40" s="3" t="n">
+        <v>21.3244</v>
       </c>
     </row>
     <row r="41">
@@ -10225,13 +10393,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4920365.1738469</v>
+        <v>4900930.8690117</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>450365.1738469</v>
+        <v>430930.8690117</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1007528353125056</v>
+        <v>0.09640511611000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-07-01
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-30 06:09 IST</t>
+          <t>Generated: 2026-07-01 06:24 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4900930.8690117</v>
+        <v>4938543.4856034</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>430930.8690117002</v>
+        <v>468543.4856033996</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.09640511611000004</v>
+        <v>0.1048195717233556</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>546366.0015945435</v>
+        <v>546248.9931945801</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-44416.01840545656</v>
+        <v>-44533.02680541994</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.07518173692127016</v>
+        <v>-0.07537979372733777</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5447296.870606244</v>
+        <v>5484792.47879798</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>386514.8506062441</v>
+        <v>424010.4587979801</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.07637453047350261</v>
+        <v>0.08378358465595009</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-06-30</t>
+          <t>Last snapshot: 2026-07-01</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BC19"/>
+  <dimension ref="A1:BD19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -674,6 +674,7 @@
     <col width="21" customWidth="1" min="53" max="53"/>
     <col width="21" customWidth="1" min="54" max="54"/>
     <col width="21" customWidth="1" min="55" max="55"/>
+    <col width="21" customWidth="1" min="56" max="56"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -952,6 +953,11 @@
           <t>2026-06-30</t>
         </is>
       </c>
+      <c r="BD1" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -971,13 +977,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>537</v>
+        <v>542.0999755859375</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>42960</v>
+        <v>43367.998046875</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>-857.510000000002</v>
+        <v>-449.511953125002</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1119,6 +1125,9 @@
       </c>
       <c r="BC2" s="3" t="n">
         <v>537</v>
+      </c>
+      <c r="BD2" s="3" t="n">
+        <v>542.0999755859375</v>
       </c>
     </row>
     <row r="3">
@@ -1166,13 +1175,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1354.099975585938</v>
+        <v>1351.199951171875</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>27081.99951171875</v>
+        <v>27023.9990234375</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-5022.580488281252</v>
+        <v>-5080.580976562502</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1317,6 +1326,9 @@
       </c>
       <c r="BC4" s="3" t="n">
         <v>1354.099975585938</v>
+      </c>
+      <c r="BD4" s="3" t="n">
+        <v>1351.199951171875</v>
       </c>
     </row>
     <row r="5">
@@ -1337,13 +1349,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>643.3499755859375</v>
+        <v>650.75</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>12866.99951171875</v>
+        <v>13015</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1346.10048828125</v>
+        <v>-1198.1</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1488,6 +1500,9 @@
       </c>
       <c r="BC5" s="3" t="n">
         <v>643.3499755859375</v>
+      </c>
+      <c r="BD5" s="3" t="n">
+        <v>650.75</v>
       </c>
     </row>
     <row r="6">
@@ -1508,13 +1523,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>372.5</v>
+        <v>369.5</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>14900</v>
+        <v>14780</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2602.240000000002</v>
+        <v>-2722.240000000002</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1659,6 +1674,9 @@
       </c>
       <c r="BC6" s="3" t="n">
         <v>372.5</v>
+      </c>
+      <c r="BD6" s="3" t="n">
+        <v>369.5</v>
       </c>
     </row>
     <row r="7">
@@ -1679,13 +1697,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>240.0299987792969</v>
+        <v>242.1399993896484</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>24002.99987792969</v>
+        <v>24213.99993896484</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-2430.820122070312</v>
+        <v>-2219.820061035156</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1830,6 +1848,9 @@
       </c>
       <c r="BC7" s="3" t="n">
         <v>240.0299987792969</v>
+      </c>
+      <c r="BD7" s="3" t="n">
+        <v>242.1399993896484</v>
       </c>
     </row>
     <row r="8">
@@ -1877,13 +1898,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>17.69000053405762</v>
+        <v>18.07999992370605</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>26535.00080108643</v>
+        <v>27119.99988555908</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-4515.169198913572</v>
+        <v>-3930.170114440916</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -2028,6 +2049,9 @@
       </c>
       <c r="BC9" s="3" t="n">
         <v>17.69000053405762</v>
+      </c>
+      <c r="BD9" s="3" t="n">
+        <v>18.07999992370605</v>
       </c>
     </row>
     <row r="10">
@@ -2048,13 +2072,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>417</v>
+        <v>416.7999877929688</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>41700</v>
+        <v>41679.99877929688</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-9798.480000000003</v>
+        <v>-9818.481220703128</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -2199,6 +2223,9 @@
       </c>
       <c r="BC10" s="3" t="n">
         <v>417</v>
+      </c>
+      <c r="BD10" s="3" t="n">
+        <v>416.7999877929688</v>
       </c>
     </row>
     <row r="11">
@@ -2219,13 +2246,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>8.770000457763672</v>
+        <v>8.789999961853027</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>8770.000457763672</v>
+        <v>8789.999961853027</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-1071.209542236327</v>
+        <v>-1051.210038146972</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -2370,6 +2397,9 @@
       </c>
       <c r="BC11" s="3" t="n">
         <v>8.770000457763672</v>
+      </c>
+      <c r="BD11" s="3" t="n">
+        <v>8.789999961853027</v>
       </c>
     </row>
     <row r="12">
@@ -2390,13 +2420,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2537</v>
+        <v>2489</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25370</v>
+        <v>24890</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2353.25</v>
+        <v>-2833.25</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -2541,6 +2571,9 @@
       </c>
       <c r="BC12" s="3" t="n">
         <v>2537</v>
+      </c>
+      <c r="BD12" s="3" t="n">
+        <v>2489</v>
       </c>
     </row>
     <row r="13">
@@ -2561,13 +2594,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>57.7599983215332</v>
+        <v>58.75</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>34655.99899291992</v>
-      </c>
-      <c r="G13" s="6" t="n">
-        <v>-375.7610070800802</v>
+        <v>35250</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>218.239999999998</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -2712,6 +2745,9 @@
       </c>
       <c r="BC13" s="3" t="n">
         <v>57.7599983215332</v>
+      </c>
+      <c r="BD13" s="3" t="n">
+        <v>58.75</v>
       </c>
     </row>
     <row r="14">
@@ -2732,13 +2768,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>724.1500244140625</v>
+        <v>706.8499755859375</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>36207.50122070312</v>
+        <v>35342.49877929688</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-6255.008779296877</v>
+        <v>-7120.011220703127</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -2883,6 +2919,9 @@
       </c>
       <c r="BC14" s="3" t="n">
         <v>724.1500244140625</v>
+      </c>
+      <c r="BD14" s="3" t="n">
+        <v>706.8499755859375</v>
       </c>
     </row>
     <row r="15">
@@ -2957,13 +2996,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>619.2000122070312</v>
+        <v>614.0999755859375</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>30960.00061035156</v>
+        <v>30704.99877929688</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>9205.470610351564</v>
+        <v>8950.468779296876</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -3108,6 +3147,9 @@
       </c>
       <c r="BC17" s="3" t="n">
         <v>619.2000122070312</v>
+      </c>
+      <c r="BD17" s="3" t="n">
+        <v>614.0999755859375</v>
       </c>
     </row>
     <row r="18">
@@ -3128,13 +3170,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>385.8500061035156</v>
+        <v>383</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>38585.00061035156</v>
+        <v>38300</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-8055.819389648437</v>
+        <v>-8340.82</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -3279,6 +3321,9 @@
       </c>
       <c r="BC18" s="3" t="n">
         <v>385.8500061035156</v>
+      </c>
+      <c r="BD18" s="3" t="n">
+        <v>383</v>
       </c>
     </row>
     <row r="19">
@@ -3291,10 +3336,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>546366.0015945435</v>
+        <v>546248.9931945801</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-44416.01840545655</v>
+        <v>-44533.02680541993</v>
       </c>
     </row>
   </sheetData>
@@ -3308,7 +3353,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BD41"/>
+  <dimension ref="A1:BE41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3319,7 +3364,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
@@ -3367,6 +3412,7 @@
     <col width="13" customWidth="1" min="54" max="54"/>
     <col width="13" customWidth="1" min="55" max="55"/>
     <col width="13" customWidth="1" min="56" max="56"/>
+    <col width="13" customWidth="1" min="57" max="57"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3650,6 +3696,11 @@
           <t>2026-06-30</t>
         </is>
       </c>
+      <c r="BE1" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3674,16 +3725,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.4098</v>
+        <v>56.8613</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>63318.9851236</v>
+        <v>63825.7857466</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>13318.9851236</v>
+        <v>13825.7857466</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.2663797024719999</v>
+        <v>0.276515714932</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -3825,6 +3876,9 @@
       </c>
       <c r="BD2" s="3" t="n">
         <v>56.4098</v>
+      </c>
+      <c r="BE2" s="3" t="n">
+        <v>56.8613</v>
       </c>
     </row>
     <row r="3">
@@ -3850,16 +3904,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.0331</v>
+        <v>25.2087</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>61461.59255030001</v>
+        <v>61892.7279531</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>1461.592550300011</v>
+        <v>1892.727953100002</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.02435987583833351</v>
+        <v>0.03154546588500003</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -3995,6 +4049,9 @@
       </c>
       <c r="BD3" s="3" t="n">
         <v>25.0331</v>
+      </c>
+      <c r="BE3" s="3" t="n">
+        <v>25.2087</v>
       </c>
     </row>
     <row r="4">
@@ -4020,16 +4077,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>11.87</v>
+        <v>12.01</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>227976.32391</v>
+        <v>230665.17693</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>47976.32391000001</v>
+        <v>50665.17693000002</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.2665351328333334</v>
+        <v>0.2814732051666667</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -4165,6 +4222,9 @@
       </c>
       <c r="BD4" s="3" t="n">
         <v>11.87</v>
+      </c>
+      <c r="BE4" s="3" t="n">
+        <v>12.01</v>
       </c>
     </row>
     <row r="5">
@@ -4190,16 +4250,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.3001</v>
+        <v>9.275700000000001</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>170694.8538088</v>
+        <v>170247.0140616</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-39305.14619119998</v>
+        <v>-39752.9859384</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.187167362815238</v>
+        <v>-0.18929993304</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -4335,6 +4395,9 @@
       </c>
       <c r="BD5" s="3" t="n">
         <v>9.3001</v>
+      </c>
+      <c r="BE5" s="3" t="n">
+        <v>9.275700000000001</v>
       </c>
     </row>
     <row r="6">
@@ -4360,16 +4423,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.1758</v>
+        <v>12.1877</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>51491.1781566</v>
+        <v>51541.5029829</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>1491.178156599999</v>
+        <v>1541.502982899998</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.02982356313199998</v>
+        <v>0.03083005965799995</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -4511,6 +4574,9 @@
       </c>
       <c r="BD6" s="3" t="n">
         <v>12.1758</v>
+      </c>
+      <c r="BE6" s="3" t="n">
+        <v>12.1877</v>
       </c>
     </row>
     <row r="7">
@@ -4536,16 +4602,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>33.6281</v>
+        <v>34.0629</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>74184.933724</v>
+        <v>75144.119916</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>14184.933724</v>
+        <v>15144.119916</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2364155620666667</v>
+        <v>0.2524019986</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -4681,6 +4747,9 @@
       </c>
       <c r="BD7" s="3" t="n">
         <v>33.6281</v>
+      </c>
+      <c r="BE7" s="3" t="n">
+        <v>34.0629</v>
       </c>
     </row>
     <row r="8">
@@ -4706,16 +4775,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>33.4275</v>
+        <v>33.7365</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>53637.53250750001</v>
+        <v>54133.3517445</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>3637.532507500007</v>
+        <v>4133.351744500003</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.07275065015000015</v>
+        <v>0.08266703489000007</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -4857,6 +4926,9 @@
       </c>
       <c r="BD8" s="3" t="n">
         <v>33.4275</v>
+      </c>
+      <c r="BE8" s="3" t="n">
+        <v>33.7365</v>
       </c>
     </row>
     <row r="9">
@@ -4882,16 +4954,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>41.3016</v>
+        <v>43.5124</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>132966.0819288</v>
+        <v>140083.5159732</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>32966.08192880001</v>
+        <v>40083.5159732</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3296608192880001</v>
+        <v>0.400835159732</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -5027,6 +5099,9 @@
       </c>
       <c r="BD9" s="3" t="n">
         <v>41.3016</v>
+      </c>
+      <c r="BE9" s="3" t="n">
+        <v>43.5124</v>
       </c>
     </row>
     <row r="10">
@@ -5052,16 +5127,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>47.2178</v>
+        <v>47.3505</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>134412.9753302</v>
+        <v>134790.7269795</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>34412.97533019999</v>
+        <v>34790.7269795</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3441297533019999</v>
+        <v>0.347907269795</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -5197,6 +5272,9 @@
       </c>
       <c r="BD10" s="3" t="n">
         <v>47.2178</v>
+      </c>
+      <c r="BE10" s="3" t="n">
+        <v>47.3505</v>
       </c>
     </row>
     <row r="11">
@@ -5222,16 +5300,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>104.1402</v>
+        <v>106.3735</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31337.7648438</v>
+        <v>32009.8072465</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1337.764843799996</v>
+        <v>2009.8072465</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.04459216145999987</v>
+        <v>0.06699357488333335</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -5367,6 +5445,9 @@
       </c>
       <c r="BD11" s="3" t="n">
         <v>104.1402</v>
+      </c>
+      <c r="BE11" s="3" t="n">
+        <v>106.3735</v>
       </c>
     </row>
     <row r="12">
@@ -5392,16 +5473,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>225.317</v>
+        <v>226.765</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>104890.020474</v>
+        <v>105564.09633</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>4890.020474000004</v>
+        <v>5564.096329999986</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.04890020474000004</v>
+        <v>0.05564096329999986</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -5543,6 +5624,9 @@
       </c>
       <c r="BD12" s="3" t="n">
         <v>225.317</v>
+      </c>
+      <c r="BE12" s="3" t="n">
+        <v>226.765</v>
       </c>
     </row>
     <row r="13">
@@ -5568,16 +5652,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>20.924</v>
+        <v>21.079</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>242459.04702</v>
+        <v>244255.125795</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>42459.04702</v>
+        <v>44255.125795</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.2122952351</v>
+        <v>0.221275628975</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -5719,6 +5803,9 @@
       </c>
       <c r="BD13" s="3" t="n">
         <v>20.924</v>
+      </c>
+      <c r="BE13" s="3" t="n">
+        <v>21.079</v>
       </c>
     </row>
     <row r="14">
@@ -5744,16 +5831,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>37.9691</v>
+        <v>38.6195</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>136977.5529746</v>
+        <v>139323.939917</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>36977.5529746</v>
+        <v>39323.93991700001</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.369775529746</v>
+        <v>0.3932393991700001</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -5889,6 +5976,9 @@
       </c>
       <c r="BD14" s="3" t="n">
         <v>37.9691</v>
+      </c>
+      <c r="BE14" s="3" t="n">
+        <v>38.6195</v>
       </c>
     </row>
     <row r="15">
@@ -5914,16 +6004,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.9</v>
+        <v>11.92</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>115952.9693</v>
+        <v>116147.84824</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>15952.96930000001</v>
+        <v>16147.84824000001</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1595296930000001</v>
+        <v>0.1614784824000001</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -6065,6 +6155,9 @@
       </c>
       <c r="BD15" s="3" t="n">
         <v>11.9</v>
+      </c>
+      <c r="BE15" s="3" t="n">
+        <v>11.92</v>
       </c>
     </row>
     <row r="16">
@@ -6090,16 +6183,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.4531</v>
+        <v>24.9297</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>139943.3306768</v>
+        <v>142670.8781616</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>39943.33067679999</v>
+        <v>42670.87816160001</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.3994333067679999</v>
+        <v>0.4267087816160001</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -6235,6 +6328,9 @@
       </c>
       <c r="BD16" s="3" t="n">
         <v>24.4531</v>
+      </c>
+      <c r="BE16" s="3" t="n">
+        <v>24.9297</v>
       </c>
     </row>
     <row r="17">
@@ -6260,16 +6356,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.7695</v>
+        <v>16.7545</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55440.9228615</v>
+        <v>55391.33200649999</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5440.922861499996</v>
+        <v>5391.332006499993</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1088184572299999</v>
+        <v>0.1078266401299999</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -6405,6 +6501,9 @@
       </c>
       <c r="BD17" s="3" t="n">
         <v>16.7695</v>
+      </c>
+      <c r="BE17" s="3" t="n">
+        <v>16.7545</v>
       </c>
     </row>
     <row r="18">
@@ -6430,16 +6529,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>46.38</v>
+        <v>46.75</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>87492.90168</v>
+        <v>88190.883</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>7492.901679999995</v>
+        <v>8190.883000000002</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.09366127099999995</v>
+        <v>0.1023860375</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -6581,6 +6680,9 @@
       </c>
       <c r="BD18" s="3" t="n">
         <v>46.38</v>
+      </c>
+      <c r="BE18" s="3" t="n">
+        <v>46.75</v>
       </c>
     </row>
     <row r="19">
@@ -6606,16 +6708,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>14.4768</v>
+        <v>14.7451</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>209432.4780288</v>
+        <v>213313.9113466</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>59432.47802880002</v>
+        <v>63313.91134660001</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.3962165201920001</v>
+        <v>0.4220927423106667</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -6751,6 +6853,9 @@
       </c>
       <c r="BD19" s="3" t="n">
         <v>14.4768</v>
+      </c>
+      <c r="BE19" s="3" t="n">
+        <v>14.7451</v>
       </c>
     </row>
     <row r="20">
@@ -6776,16 +6881,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.199999999999999</v>
+        <v>9.16</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>241553.3876</v>
+        <v>240503.15548</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-8446.612400000013</v>
+        <v>-9496.844519999984</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.03378644960000005</v>
+        <v>-0.03798737807999994</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -6927,6 +7032,9 @@
       </c>
       <c r="BD20" s="3" t="n">
         <v>9.199999999999999</v>
+      </c>
+      <c r="BE20" s="3" t="n">
+        <v>9.16</v>
       </c>
     </row>
     <row r="21">
@@ -6952,16 +7060,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>111.5854</v>
+        <v>111.8505</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>169527.1232186</v>
+        <v>169929.8787795</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-472.8767814000021</v>
+        <v>-70.12122050000471</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.002781628125882365</v>
+        <v>-0.0004124777676470865</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -7103,6 +7211,9 @@
       </c>
       <c r="BD21" s="3" t="n">
         <v>111.5854</v>
+      </c>
+      <c r="BE21" s="3" t="n">
+        <v>111.8505</v>
       </c>
     </row>
     <row r="22">
@@ -7128,16 +7239,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>43.655</v>
+        <v>44.502</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>66986.85130000001</v>
+        <v>68286.53892000001</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>6986.851300000009</v>
+        <v>8286.538920000006</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1164475216666668</v>
+        <v>0.1381089820000001</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -7273,6 +7384,9 @@
       </c>
       <c r="BD22" s="3" t="n">
         <v>43.655</v>
+      </c>
+      <c r="BE22" s="3" t="n">
+        <v>44.502</v>
       </c>
     </row>
     <row r="23">
@@ -7298,16 +7412,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>63.542</v>
+        <v>63.725</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>172609.746114</v>
+        <v>173106.859575</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>22609.74611400001</v>
+        <v>23106.85957500001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.1507316407600001</v>
+        <v>0.1540457305000001</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -7449,6 +7563,9 @@
       </c>
       <c r="BD23" s="3" t="n">
         <v>63.542</v>
+      </c>
+      <c r="BE23" s="3" t="n">
+        <v>63.725</v>
       </c>
     </row>
     <row r="24">
@@ -7474,16 +7591,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>27.7279</v>
+        <v>27.7393</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>100746.1636694</v>
+        <v>100787.5842698</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>746.1636694000044</v>
+        <v>787.5842698000051</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.007461636694000045</v>
+        <v>0.007875842698000051</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -7619,6 +7736,9 @@
       </c>
       <c r="BD24" s="3" t="n">
         <v>27.7279</v>
+      </c>
+      <c r="BE24" s="3" t="n">
+        <v>27.7393</v>
       </c>
     </row>
     <row r="25">
@@ -7644,16 +7764,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.5302</v>
+        <v>11.612</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>189345.1855548</v>
+        <v>190688.478488</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-10654.8144452</v>
+        <v>-9311.521512000007</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.05327407222599999</v>
+        <v>-0.04655760756000003</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -7792,6 +7912,9 @@
       </c>
       <c r="BD25" s="3" t="n">
         <v>11.5302</v>
+      </c>
+      <c r="BE25" s="3" t="n">
+        <v>11.612</v>
       </c>
     </row>
     <row r="26">
@@ -7817,16 +7940,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>9.0952</v>
+        <v>9.0871</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>108612.286268</v>
+        <v>108515.5583765</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>-1387.713732000004</v>
+        <v>-1484.44162350001</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>-0.01261557938181822</v>
+        <v>-0.01349492385000009</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -7965,6 +8088,9 @@
       </c>
       <c r="BD26" s="3" t="n">
         <v>9.0952</v>
+      </c>
+      <c r="BE26" s="3" t="n">
+        <v>9.0871</v>
       </c>
     </row>
     <row r="27">
@@ -7990,16 +8116,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>64.8481</v>
+        <v>65.4199</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>104461.210366</v>
+        <v>105382.300114</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-5538.789634000001</v>
+        <v>-4617.699886000002</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.05035263303636364</v>
+        <v>-0.04197908987272729</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -8141,6 +8267,9 @@
       </c>
       <c r="BD27" s="3" t="n">
         <v>64.8481</v>
+      </c>
+      <c r="BE27" s="3" t="n">
+        <v>65.4199</v>
       </c>
     </row>
     <row r="28">
@@ -8166,16 +8295,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>107.8072</v>
+        <v>108.5221</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>356481.4325304</v>
+        <v>358845.3616197</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-23518.56746960001</v>
+        <v>-21154.63838030002</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.06189096702526317</v>
+        <v>-0.05567010100078953</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -8317,6 +8446,9 @@
       </c>
       <c r="BD28" s="3" t="n">
         <v>107.8072</v>
+      </c>
+      <c r="BE28" s="3" t="n">
+        <v>108.5221</v>
       </c>
     </row>
     <row r="29">
@@ -8342,16 +8474,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.3051</v>
+        <v>12.4709</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>118174.5257853</v>
+        <v>119766.8197427</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>18174.52578529999</v>
+        <v>19766.8197427</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.1817452578529999</v>
+        <v>0.197668197427</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -8487,6 +8619,9 @@
       </c>
       <c r="BD29" s="3" t="n">
         <v>12.3051</v>
+      </c>
+      <c r="BE29" s="3" t="n">
+        <v>12.4709</v>
       </c>
     </row>
     <row r="30">
@@ -8512,16 +8647,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>16.4715</v>
+        <v>16.5541</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>121820.9244615</v>
+        <v>122431.8225801</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>21820.92446149999</v>
+        <v>22431.82258009998</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.2182092446149999</v>
+        <v>0.2243182258009998</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -8657,6 +8792,9 @@
       </c>
       <c r="BD30" s="3" t="n">
         <v>16.4715</v>
+      </c>
+      <c r="BE30" s="3" t="n">
+        <v>16.5541</v>
       </c>
     </row>
     <row r="31">
@@ -8682,16 +8820,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>418.7475</v>
+        <v>419.3814</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>111420.3348</v>
+        <v>111589.002912</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>11420.3348</v>
+        <v>11589.002912</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.114203348</v>
+        <v>0.11589002912</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -8830,6 +8968,9 @@
       </c>
       <c r="BD31" s="3" t="n">
         <v>418.7475</v>
+      </c>
+      <c r="BE31" s="3" t="n">
+        <v>419.3814</v>
       </c>
     </row>
     <row r="32">
@@ -8855,16 +8996,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.48</v>
+        <v>10.52</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>221546.7808</v>
+        <v>222392.3792</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>21546.78080000001</v>
+        <v>22392.3792</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.107733904</v>
+        <v>0.111961896</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -9006,6 +9147,9 @@
       </c>
       <c r="BD32" s="3" t="n">
         <v>10.48</v>
+      </c>
+      <c r="BE32" s="3" t="n">
+        <v>10.52</v>
       </c>
     </row>
     <row r="33">
@@ -9031,16 +9175,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>18.71</v>
+        <v>18.89</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>67049.9044</v>
+        <v>67694.9596</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>7049.904399999999</v>
+        <v>7694.959600000002</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.1174984066666667</v>
+        <v>0.1282493266666667</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -9176,6 +9320,9 @@
       </c>
       <c r="BD33" s="3" t="n">
         <v>18.71</v>
+      </c>
+      <c r="BE33" s="3" t="n">
+        <v>18.89</v>
       </c>
     </row>
     <row r="34">
@@ -9201,16 +9348,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>205.3031</v>
+        <v>203.8247</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>72170.4040461</v>
+        <v>71650.7006157</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-7829.595953900003</v>
+        <v>-8349.2993843</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.09786994942375005</v>
+        <v>-0.10436624230375</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -9349,6 +9496,9 @@
       </c>
       <c r="BD34" s="3" t="n">
         <v>205.3031</v>
+      </c>
+      <c r="BE34" s="3" t="n">
+        <v>203.8247</v>
       </c>
     </row>
     <row r="35">
@@ -9374,16 +9524,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>15.09</v>
+        <v>15.16</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>107673.53307</v>
+        <v>108173.01268</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>7673.53306999999</v>
+        <v>8173.01268</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.07673533069999991</v>
+        <v>0.0817301268</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -9522,6 +9672,9 @@
       </c>
       <c r="BD35" s="3" t="n">
         <v>15.09</v>
+      </c>
+      <c r="BE35" s="3" t="n">
+        <v>15.16</v>
       </c>
     </row>
     <row r="36">
@@ -9547,16 +9700,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>367.1375</v>
+        <v>371.1337</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>170978.136575</v>
+        <v>172839.1908922</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>20978.13657500001</v>
+        <v>22839.19089219999</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1398542438333334</v>
+        <v>0.1522612726146666</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -9695,6 +9848,9 @@
       </c>
       <c r="BD36" s="3" t="n">
         <v>367.1375</v>
+      </c>
+      <c r="BE36" s="3" t="n">
+        <v>371.1337</v>
       </c>
     </row>
     <row r="37">
@@ -9720,16 +9876,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>16.508</v>
+        <v>16.632</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>62117.771612</v>
+        <v>62584.36984800001</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>12117.771612</v>
+        <v>12584.36984800001</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.2423554322399999</v>
+        <v>0.2516873969600002</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -9868,6 +10024,9 @@
       </c>
       <c r="BD37" s="3" t="n">
         <v>16.508</v>
+      </c>
+      <c r="BE37" s="3" t="n">
+        <v>16.632</v>
       </c>
     </row>
     <row r="38">
@@ -9893,16 +10052,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>14.2291</v>
+        <v>14.2426</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>85096.8764262</v>
+        <v>85177.6129332</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>5096.876426200004</v>
+        <v>5177.612933199998</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.06371095532750005</v>
+        <v>0.06472016166499998</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -10038,6 +10197,9 @@
       </c>
       <c r="BD38" s="3" t="n">
         <v>14.2291</v>
+      </c>
+      <c r="BE38" s="3" t="n">
+        <v>14.2426</v>
       </c>
     </row>
     <row r="39">
@@ -10063,16 +10225,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1022.2323</v>
+        <v>1021.951</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50989.9693563</v>
+        <v>50975.937831</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>989.9693563000037</v>
+        <v>975.9378310000029</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.01979938712600007</v>
+        <v>0.01951875662000006</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -10208,6 +10370,9 @@
       </c>
       <c r="BD39" s="3" t="n">
         <v>1022.2323</v>
+      </c>
+      <c r="BE39" s="3" t="n">
+        <v>1021.951</v>
       </c>
     </row>
     <row r="40">
@@ -10233,16 +10398,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>21.3244</v>
+        <v>21.4302</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>107496.8761588</v>
+        <v>108030.2168154</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>7496.876158800005</v>
+        <v>8030.216815399996</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.07496876158800005</v>
+        <v>0.08030216815399996</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -10381,6 +10546,9 @@
       </c>
       <c r="BD40" s="3" t="n">
         <v>21.3244</v>
+      </c>
+      <c r="BE40" s="3" t="n">
+        <v>21.4302</v>
       </c>
     </row>
     <row r="41">
@@ -10393,13 +10561,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4900930.8690117</v>
+        <v>4938543.4856034</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>430930.8690117</v>
+        <v>468543.4856034</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.09640511611000001</v>
+        <v>0.1048195717233557</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-07-02
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -483,8 +483,8 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-01 06:24 IST</t>
+          <t>Generated: 2026-07-02 05:57 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4938543.4856034</v>
+        <v>4949302.8839843</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>468543.4856033996</v>
+        <v>479302.8839843003</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1048195717233556</v>
+        <v>0.1072265959696421</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>546248.9931945801</v>
+        <v>543934.9988632202</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-44533.02680541994</v>
+        <v>-46847.0211367798</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.07537979372733777</v>
+        <v>-0.07929662642200892</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5484792.47879798</v>
+        <v>5493237.882847521</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>424010.4587979801</v>
+        <v>432455.862847521</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.08378358465595009</v>
+        <v>0.08545237892848841</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-07-01</t>
+          <t>Last snapshot: 2026-07-02</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BD19"/>
+  <dimension ref="A1:BE19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -675,6 +675,7 @@
     <col width="21" customWidth="1" min="54" max="54"/>
     <col width="21" customWidth="1" min="55" max="55"/>
     <col width="21" customWidth="1" min="56" max="56"/>
+    <col width="21" customWidth="1" min="57" max="57"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -958,6 +959,11 @@
           <t>2026-07-01</t>
         </is>
       </c>
+      <c r="BE1" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -977,13 +983,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>542.0999755859375</v>
+        <v>543.1500244140625</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>43367.998046875</v>
+        <v>43452.001953125</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>-449.511953125002</v>
+        <v>-365.508046875002</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1128,6 +1134,9 @@
       </c>
       <c r="BD2" s="3" t="n">
         <v>542.0999755859375</v>
+      </c>
+      <c r="BE2" s="3" t="n">
+        <v>543.1500244140625</v>
       </c>
     </row>
     <row r="3">
@@ -1175,13 +1184,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1351.199951171875</v>
+        <v>1363</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>27023.9990234375</v>
+        <v>27260</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-5080.580976562502</v>
+        <v>-4844.580000000002</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1329,6 +1338,9 @@
       </c>
       <c r="BD4" s="3" t="n">
         <v>1351.199951171875</v>
+      </c>
+      <c r="BE4" s="3" t="n">
+        <v>1363</v>
       </c>
     </row>
     <row r="5">
@@ -1349,13 +1361,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>650.75</v>
+        <v>645.8499755859375</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13015</v>
+        <v>12916.99951171875</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1198.1</v>
+        <v>-1296.10048828125</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1503,6 +1515,9 @@
       </c>
       <c r="BD5" s="3" t="n">
         <v>650.75</v>
+      </c>
+      <c r="BE5" s="3" t="n">
+        <v>645.8499755859375</v>
       </c>
     </row>
     <row r="6">
@@ -1523,13 +1538,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>369.5</v>
+        <v>364.75</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>14780</v>
+        <v>14590</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2722.240000000002</v>
+        <v>-2912.240000000002</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1677,6 +1692,9 @@
       </c>
       <c r="BD6" s="3" t="n">
         <v>369.5</v>
+      </c>
+      <c r="BE6" s="3" t="n">
+        <v>364.75</v>
       </c>
     </row>
     <row r="7">
@@ -1697,13 +1715,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>242.1399993896484</v>
+        <v>236.1000061035156</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>24213.99993896484</v>
+        <v>23610.00061035156</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-2219.820061035156</v>
+        <v>-2823.819389648437</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1851,6 +1869,9 @@
       </c>
       <c r="BD7" s="3" t="n">
         <v>242.1399993896484</v>
+      </c>
+      <c r="BE7" s="3" t="n">
+        <v>236.1000061035156</v>
       </c>
     </row>
     <row r="8">
@@ -1898,13 +1919,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>18.07999992370605</v>
+        <v>17.98999977111816</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>27119.99988555908</v>
+        <v>26984.99965667725</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-3930.170114440916</v>
+        <v>-4065.170343322752</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -2052,6 +2073,9 @@
       </c>
       <c r="BD9" s="3" t="n">
         <v>18.07999992370605</v>
+      </c>
+      <c r="BE9" s="3" t="n">
+        <v>17.98999977111816</v>
       </c>
     </row>
     <row r="10">
@@ -2072,13 +2096,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>416.7999877929688</v>
+        <v>419.7999877929688</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>41679.99877929688</v>
+        <v>41979.99877929688</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-9818.481220703128</v>
+        <v>-9518.481220703128</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -2226,6 +2250,9 @@
       </c>
       <c r="BD10" s="3" t="n">
         <v>416.7999877929688</v>
+      </c>
+      <c r="BE10" s="3" t="n">
+        <v>419.7999877929688</v>
       </c>
     </row>
     <row r="11">
@@ -2246,13 +2273,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>8.789999961853027</v>
+        <v>9.270000457763672</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>8789.999961853027</v>
+        <v>9270.000457763672</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-1051.210038146972</v>
+        <v>-571.2095422363273</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -2400,6 +2427,9 @@
       </c>
       <c r="BD11" s="3" t="n">
         <v>8.789999961853027</v>
+      </c>
+      <c r="BE11" s="3" t="n">
+        <v>9.270000457763672</v>
       </c>
     </row>
     <row r="12">
@@ -2420,13 +2450,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2489</v>
+        <v>2468</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>24890</v>
+        <v>24680</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2833.25</v>
+        <v>-3043.25</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -2574,6 +2604,9 @@
       </c>
       <c r="BD12" s="3" t="n">
         <v>2489</v>
+      </c>
+      <c r="BE12" s="3" t="n">
+        <v>2468</v>
       </c>
     </row>
     <row r="13">
@@ -2594,13 +2627,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>58.75</v>
+        <v>58.22999954223633</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>35250</v>
-      </c>
-      <c r="G13" s="4" t="n">
-        <v>218.239999999998</v>
+        <v>34937.9997253418</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>-93.76027465820516</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -2748,6 +2781,9 @@
       </c>
       <c r="BD13" s="3" t="n">
         <v>58.75</v>
+      </c>
+      <c r="BE13" s="3" t="n">
+        <v>58.22999954223633</v>
       </c>
     </row>
     <row r="14">
@@ -2768,13 +2804,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>706.8499755859375</v>
+        <v>689.8499755859375</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>35342.49877929688</v>
+        <v>34492.49877929688</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-7120.011220703127</v>
+        <v>-7970.011220703127</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -2922,6 +2958,9 @@
       </c>
       <c r="BD14" s="3" t="n">
         <v>706.8499755859375</v>
+      </c>
+      <c r="BE14" s="3" t="n">
+        <v>689.8499755859375</v>
       </c>
     </row>
     <row r="15">
@@ -2996,13 +3035,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>614.0999755859375</v>
+        <v>608.7999877929688</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>30704.99877929688</v>
+        <v>30439.99938964844</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>8950.468779296876</v>
+        <v>8685.469389648439</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -3150,6 +3189,9 @@
       </c>
       <c r="BD17" s="3" t="n">
         <v>614.0999755859375</v>
+      </c>
+      <c r="BE17" s="3" t="n">
+        <v>608.7999877929688</v>
       </c>
     </row>
     <row r="18">
@@ -3170,13 +3212,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>383</v>
+        <v>375.5</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>38300</v>
+        <v>37550</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-8340.82</v>
+        <v>-9090.82</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -3324,6 +3366,9 @@
       </c>
       <c r="BD18" s="3" t="n">
         <v>383</v>
+      </c>
+      <c r="BE18" s="3" t="n">
+        <v>375.5</v>
       </c>
     </row>
     <row r="19">
@@ -3336,10 +3381,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>546248.9931945801</v>
+        <v>543934.9988632202</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-44533.02680541993</v>
+        <v>-46847.0211367798</v>
       </c>
     </row>
   </sheetData>
@@ -3353,7 +3398,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE41"/>
+  <dimension ref="A1:BF41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3364,7 +3409,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
@@ -3413,6 +3458,7 @@
     <col width="13" customWidth="1" min="55" max="55"/>
     <col width="13" customWidth="1" min="56" max="56"/>
     <col width="13" customWidth="1" min="57" max="57"/>
+    <col width="13" customWidth="1" min="58" max="58"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3701,6 +3747,11 @@
           <t>2026-07-01</t>
         </is>
       </c>
+      <c r="BF1" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3725,16 +3776,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.8613</v>
+        <v>56.818</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>63825.7857466</v>
+        <v>63777.182276</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>13825.7857466</v>
+        <v>13777.182276</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.276515714932</v>
+        <v>0.27554364552</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -3879,6 +3930,9 @@
       </c>
       <c r="BE2" s="3" t="n">
         <v>56.8613</v>
+      </c>
+      <c r="BF2" s="3" t="n">
+        <v>56.818</v>
       </c>
     </row>
     <row r="3">
@@ -3904,16 +3958,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.2087</v>
+        <v>25.3951</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>61892.7279531</v>
+        <v>62350.37965630001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>1892.727953100002</v>
+        <v>2350.379656300007</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.03154546588500003</v>
+        <v>0.03917299427166678</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -4052,6 +4106,9 @@
       </c>
       <c r="BE3" s="3" t="n">
         <v>25.2087</v>
+      </c>
+      <c r="BF3" s="3" t="n">
+        <v>25.3951</v>
       </c>
     </row>
     <row r="4">
@@ -4226,6 +4283,9 @@
       <c r="BE4" s="3" t="n">
         <v>12.01</v>
       </c>
+      <c r="BF4" s="3" t="n">
+        <v>12.01</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4250,16 +4310,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.275700000000001</v>
+        <v>9.323399999999999</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>170247.0140616</v>
+        <v>171122.5040592</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-39752.9859384</v>
+        <v>-38877.4959408</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.18929993304</v>
+        <v>-0.1851309330514286</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -4398,6 +4458,9 @@
       </c>
       <c r="BE5" s="3" t="n">
         <v>9.275700000000001</v>
+      </c>
+      <c r="BF5" s="3" t="n">
+        <v>9.323399999999999</v>
       </c>
     </row>
     <row r="6">
@@ -4423,16 +4486,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.1877</v>
+        <v>12.1012</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>51541.5029829</v>
+        <v>51175.6964724</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>1541.502982899998</v>
+        <v>1175.696472399999</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.03083005965799995</v>
+        <v>0.02351392944799998</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -4577,6 +4640,9 @@
       </c>
       <c r="BE6" s="3" t="n">
         <v>12.1877</v>
+      </c>
+      <c r="BF6" s="3" t="n">
+        <v>12.1012</v>
       </c>
     </row>
     <row r="7">
@@ -4602,16 +4668,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>34.0629</v>
+        <v>34.0402</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>75144.119916</v>
+        <v>75094.042808</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>15144.119916</v>
+        <v>15094.042808</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2524019986</v>
+        <v>0.2515673801333333</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -4750,6 +4816,9 @@
       </c>
       <c r="BE7" s="3" t="n">
         <v>34.0629</v>
+      </c>
+      <c r="BF7" s="3" t="n">
+        <v>34.0402</v>
       </c>
     </row>
     <row r="8">
@@ -4775,16 +4844,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>33.7365</v>
+        <v>33.9583</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>54133.3517445</v>
+        <v>54489.25047190001</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>4133.351744500003</v>
+        <v>4489.250471900006</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.08266703489000007</v>
+        <v>0.08978500943800012</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -4929,6 +4998,9 @@
       </c>
       <c r="BE8" s="3" t="n">
         <v>33.7365</v>
+      </c>
+      <c r="BF8" s="3" t="n">
+        <v>33.9583</v>
       </c>
     </row>
     <row r="9">
@@ -4954,16 +5026,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>43.5124</v>
+        <v>43.416</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>140083.5159732</v>
+        <v>139773.166488</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>40083.5159732</v>
+        <v>39773.16648799999</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.400835159732</v>
+        <v>0.3977316648799999</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -5102,6 +5174,9 @@
       </c>
       <c r="BE9" s="3" t="n">
         <v>43.5124</v>
+      </c>
+      <c r="BF9" s="3" t="n">
+        <v>43.416</v>
       </c>
     </row>
     <row r="10">
@@ -5127,16 +5202,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>47.3505</v>
+        <v>47.4194</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>134790.7269795</v>
+        <v>134986.8617846</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>34790.7269795</v>
+        <v>34986.86178460001</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.347907269795</v>
+        <v>0.3498686178460002</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -5275,6 +5350,9 @@
       </c>
       <c r="BE10" s="3" t="n">
         <v>47.3505</v>
+      </c>
+      <c r="BF10" s="3" t="n">
+        <v>47.4194</v>
       </c>
     </row>
     <row r="11">
@@ -5300,16 +5378,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>106.3735</v>
+        <v>105.5166</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>32009.8072465</v>
+        <v>31751.9497554</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>2009.8072465</v>
+        <v>1751.949755399997</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.06699357488333335</v>
+        <v>0.0583983251799999</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -5448,6 +5526,9 @@
       </c>
       <c r="BE11" s="3" t="n">
         <v>106.3735</v>
+      </c>
+      <c r="BF11" s="3" t="n">
+        <v>105.5166</v>
       </c>
     </row>
     <row r="12">
@@ -5473,16 +5554,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>226.765</v>
+        <v>227.179</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>105564.09633</v>
+        <v>105756.822438</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>5564.096329999986</v>
+        <v>5756.822438000003</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.05564096329999986</v>
+        <v>0.05756822438000003</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -5627,6 +5708,9 @@
       </c>
       <c r="BE12" s="3" t="n">
         <v>226.765</v>
+      </c>
+      <c r="BF12" s="3" t="n">
+        <v>227.179</v>
       </c>
     </row>
     <row r="13">
@@ -5652,16 +5736,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>21.079</v>
+        <v>21.034</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>244255.125795</v>
+        <v>243733.68357</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>44255.125795</v>
+        <v>43733.68356999996</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.221275628975</v>
+        <v>0.2186684178499998</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -5806,6 +5890,9 @@
       </c>
       <c r="BE13" s="3" t="n">
         <v>21.079</v>
+      </c>
+      <c r="BF13" s="3" t="n">
+        <v>21.034</v>
       </c>
     </row>
     <row r="14">
@@ -5980,6 +6067,9 @@
       <c r="BE14" s="3" t="n">
         <v>38.6195</v>
       </c>
+      <c r="BF14" s="3" t="n">
+        <v>38.6195</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -6159,6 +6249,9 @@
       <c r="BE15" s="3" t="n">
         <v>11.92</v>
       </c>
+      <c r="BF15" s="3" t="n">
+        <v>11.92</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -6183,16 +6276,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.9297</v>
+        <v>24.5808</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>142670.8781616</v>
+        <v>140674.1485824</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>42670.87816160001</v>
+        <v>40674.1485824</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4267087816160001</v>
+        <v>0.406741485824</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -6331,6 +6424,9 @@
       </c>
       <c r="BE16" s="3" t="n">
         <v>24.9297</v>
+      </c>
+      <c r="BF16" s="3" t="n">
+        <v>24.5808</v>
       </c>
     </row>
     <row r="17">
@@ -6356,16 +6452,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.7545</v>
+        <v>16.7895</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55391.33200649999</v>
+        <v>55507.0440015</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5391.332006499993</v>
+        <v>5507.044001499999</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1078266401299999</v>
+        <v>0.11014088003</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -6504,6 +6600,9 @@
       </c>
       <c r="BE17" s="3" t="n">
         <v>16.7545</v>
+      </c>
+      <c r="BF17" s="3" t="n">
+        <v>16.7895</v>
       </c>
     </row>
     <row r="18">
@@ -6529,16 +6628,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>46.75</v>
+        <v>46.59</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>88190.883</v>
+        <v>87889.05324000001</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>8190.883000000002</v>
+        <v>7889.053240000008</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.1023860375</v>
+        <v>0.0986131655000001</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -6683,6 +6782,9 @@
       </c>
       <c r="BE18" s="3" t="n">
         <v>46.75</v>
+      </c>
+      <c r="BF18" s="3" t="n">
+        <v>46.59</v>
       </c>
     </row>
     <row r="19">
@@ -6708,16 +6810,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>14.7451</v>
+        <v>15.0717</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>213313.9113466</v>
+        <v>218038.7571222</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>63313.91134660001</v>
+        <v>68038.75712219998</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.4220927423106667</v>
+        <v>0.4535917141479999</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -6856,6 +6958,9 @@
       </c>
       <c r="BE19" s="3" t="n">
         <v>14.7451</v>
+      </c>
+      <c r="BF19" s="3" t="n">
+        <v>15.0717</v>
       </c>
     </row>
     <row r="20">
@@ -6881,16 +6986,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.16</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>240503.15548</v>
+        <v>239715.48139</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-9496.844519999984</v>
+        <v>-10284.51860999997</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.03798737807999994</v>
+        <v>-0.04113807443999988</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -7035,6 +7140,9 @@
       </c>
       <c r="BE20" s="3" t="n">
         <v>9.16</v>
+      </c>
+      <c r="BF20" s="3" t="n">
+        <v>9.130000000000001</v>
       </c>
     </row>
     <row r="21">
@@ -7060,16 +7168,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>111.8505</v>
+        <v>112.2987</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>169929.8787795</v>
-      </c>
-      <c r="H21" s="6" t="n">
-        <v>-70.12122050000471</v>
-      </c>
-      <c r="I21" s="13" t="n">
-        <v>-0.0004124777676470865</v>
+        <v>170610.8106633</v>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>610.8106632999843</v>
+      </c>
+      <c r="I21" s="12" t="n">
+        <v>0.003593003901764613</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -7214,6 +7322,9 @@
       </c>
       <c r="BE21" s="3" t="n">
         <v>111.8505</v>
+      </c>
+      <c r="BF21" s="3" t="n">
+        <v>112.2987</v>
       </c>
     </row>
     <row r="22">
@@ -7388,6 +7499,9 @@
       <c r="BE22" s="3" t="n">
         <v>44.502</v>
       </c>
+      <c r="BF22" s="3" t="n">
+        <v>44.502</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -7412,16 +7526,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>63.725</v>
+        <v>63.9487</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>173106.859575</v>
+        <v>173714.5332429</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>23106.85957500001</v>
+        <v>23714.53324290001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.1540457305000001</v>
+        <v>0.1580968882860001</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -7566,6 +7680,9 @@
       </c>
       <c r="BE23" s="3" t="n">
         <v>63.725</v>
+      </c>
+      <c r="BF23" s="3" t="n">
+        <v>63.9487</v>
       </c>
     </row>
     <row r="24">
@@ -7591,16 +7708,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>27.7393</v>
+        <v>27.7429</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>100787.5842698</v>
+        <v>100800.6644594</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>787.5842698000051</v>
+        <v>800.6644593999954</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.007875842698000051</v>
+        <v>0.008006644593999954</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -7739,6 +7856,9 @@
       </c>
       <c r="BE24" s="3" t="n">
         <v>27.7393</v>
+      </c>
+      <c r="BF24" s="3" t="n">
+        <v>27.7429</v>
       </c>
     </row>
     <row r="25">
@@ -7764,16 +7884,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.612</v>
+        <v>11.6549</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>190688.478488</v>
+        <v>191392.9683026</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-9311.521512000007</v>
+        <v>-8607.031697400031</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.04655760756000003</v>
+        <v>-0.04303515848700015</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -7915,6 +8035,9 @@
       </c>
       <c r="BE25" s="3" t="n">
         <v>11.612</v>
+      </c>
+      <c r="BF25" s="3" t="n">
+        <v>11.6549</v>
       </c>
     </row>
     <row r="26">
@@ -7940,16 +8063,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>9.0871</v>
+        <v>9.2058</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>108515.5583765</v>
+        <v>109933.039947</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>-1484.44162350001</v>
+        <v>-66.96005300000252</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>-0.01349492385000009</v>
+        <v>-0.0006087277545454774</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -8091,6 +8214,9 @@
       </c>
       <c r="BE26" s="3" t="n">
         <v>9.0871</v>
+      </c>
+      <c r="BF26" s="3" t="n">
+        <v>9.2058</v>
       </c>
     </row>
     <row r="27">
@@ -8116,16 +8242,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>65.4199</v>
+        <v>65.5801</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>105382.300114</v>
+        <v>105640.359886</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-4617.699886000002</v>
+        <v>-4359.640114000009</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.04197908987272729</v>
+        <v>-0.03963309194545463</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -8270,6 +8396,9 @@
       </c>
       <c r="BE27" s="3" t="n">
         <v>65.4199</v>
+      </c>
+      <c r="BF27" s="3" t="n">
+        <v>65.5801</v>
       </c>
     </row>
     <row r="28">
@@ -8295,16 +8424,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>108.5221</v>
+        <v>109.2744</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>358845.3616197</v>
+        <v>361332.9596808</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-21154.63838030002</v>
+        <v>-18667.04031919996</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.05567010100078953</v>
+        <v>-0.04912379031368412</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -8449,6 +8578,9 @@
       </c>
       <c r="BE28" s="3" t="n">
         <v>108.5221</v>
+      </c>
+      <c r="BF28" s="3" t="n">
+        <v>109.2744</v>
       </c>
     </row>
     <row r="29">
@@ -8474,16 +8606,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.4709</v>
+        <v>12.518</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>119766.8197427</v>
+        <v>120219.154154</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>19766.8197427</v>
+        <v>20219.154154</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.197668197427</v>
+        <v>0.20219154154</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -8622,6 +8754,9 @@
       </c>
       <c r="BE29" s="3" t="n">
         <v>12.4709</v>
+      </c>
+      <c r="BF29" s="3" t="n">
+        <v>12.518</v>
       </c>
     </row>
     <row r="30">
@@ -8647,16 +8782,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>16.5541</v>
+        <v>16.6816</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>122431.8225801</v>
+        <v>123374.7948576</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>22431.82258009998</v>
+        <v>23374.79485759999</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.2243182258009998</v>
+        <v>0.2337479485759999</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -8795,6 +8930,9 @@
       </c>
       <c r="BE30" s="3" t="n">
         <v>16.5541</v>
+      </c>
+      <c r="BF30" s="3" t="n">
+        <v>16.6816</v>
       </c>
     </row>
     <row r="31">
@@ -8820,16 +8958,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>419.3814</v>
+        <v>419.6801</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>111589.002912</v>
+        <v>111668.481008</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>11589.002912</v>
+        <v>11668.48100799999</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.11589002912</v>
+        <v>0.1166848100799999</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -8971,6 +9109,9 @@
       </c>
       <c r="BE31" s="3" t="n">
         <v>419.3814</v>
+      </c>
+      <c r="BF31" s="3" t="n">
+        <v>419.6801</v>
       </c>
     </row>
     <row r="32">
@@ -8996,16 +9137,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.52</v>
+        <v>10.58</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>222392.3792</v>
+        <v>223660.7768</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>22392.3792</v>
+        <v>23660.77679999999</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.111961896</v>
+        <v>0.118303884</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -9150,6 +9291,9 @@
       </c>
       <c r="BE32" s="3" t="n">
         <v>10.52</v>
+      </c>
+      <c r="BF32" s="3" t="n">
+        <v>10.58</v>
       </c>
     </row>
     <row r="33">
@@ -9175,16 +9319,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>18.89</v>
+        <v>18.99</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>67694.9596</v>
+        <v>68053.32359999999</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>7694.959600000002</v>
+        <v>8053.323599999989</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.1282493266666667</v>
+        <v>0.1342220599999998</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -9323,6 +9467,9 @@
       </c>
       <c r="BE33" s="3" t="n">
         <v>18.89</v>
+      </c>
+      <c r="BF33" s="3" t="n">
+        <v>18.99</v>
       </c>
     </row>
     <row r="34">
@@ -9348,16 +9495,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>203.8247</v>
+        <v>204.8743</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>71650.7006157</v>
+        <v>72019.66755330001</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-8349.2993843</v>
+        <v>-7980.332446699991</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.10436624230375</v>
+        <v>-0.09975415558374989</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -9499,6 +9646,9 @@
       </c>
       <c r="BE34" s="3" t="n">
         <v>203.8247</v>
+      </c>
+      <c r="BF34" s="3" t="n">
+        <v>204.8743</v>
       </c>
     </row>
     <row r="35">
@@ -9524,16 +9674,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>15.16</v>
+        <v>15.04</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>108173.01268</v>
+        <v>107316.76192</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>8173.01268</v>
+        <v>7316.76191999999</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.0817301268</v>
+        <v>0.07316761919999989</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -9675,6 +9825,9 @@
       </c>
       <c r="BE35" s="3" t="n">
         <v>15.16</v>
+      </c>
+      <c r="BF35" s="3" t="n">
+        <v>15.04</v>
       </c>
     </row>
     <row r="36">
@@ -9700,16 +9853,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>371.1337</v>
+        <v>370.0029</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>172839.1908922</v>
+        <v>172312.5705474</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>22839.19089219999</v>
+        <v>22312.57054740001</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1522612726146666</v>
+        <v>0.1487504703160001</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -9851,6 +10004,9 @@
       </c>
       <c r="BE36" s="3" t="n">
         <v>371.1337</v>
+      </c>
+      <c r="BF36" s="3" t="n">
+        <v>370.0029</v>
       </c>
     </row>
     <row r="37">
@@ -9876,16 +10032,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>16.632</v>
+        <v>16.582</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>62584.36984800001</v>
+        <v>62396.225398</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>12584.36984800001</v>
+        <v>12396.225398</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.2516873969600002</v>
+        <v>0.24792450796</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -10027,6 +10183,9 @@
       </c>
       <c r="BE37" s="3" t="n">
         <v>16.632</v>
+      </c>
+      <c r="BF37" s="3" t="n">
+        <v>16.582</v>
       </c>
     </row>
     <row r="38">
@@ -10052,16 +10211,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>14.2426</v>
+        <v>14.3009</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>85177.6129332</v>
+        <v>85526.2750338</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>5177.612933199998</v>
+        <v>5526.275033800004</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.06472016166499998</v>
+        <v>0.06907843792250005</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -10200,6 +10359,9 @@
       </c>
       <c r="BE38" s="3" t="n">
         <v>14.2426</v>
+      </c>
+      <c r="BF38" s="3" t="n">
+        <v>14.3009</v>
       </c>
     </row>
     <row r="39">
@@ -10225,16 +10387,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1021.951</v>
+        <v>1022.1898</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50975.937831</v>
+        <v>50987.8494138</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>975.9378310000029</v>
+        <v>987.8494138000024</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.01951875662000006</v>
+        <v>0.01975698827600005</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -10373,6 +10535,9 @@
       </c>
       <c r="BE39" s="3" t="n">
         <v>1021.951</v>
+      </c>
+      <c r="BF39" s="3" t="n">
+        <v>1022.1898</v>
       </c>
     </row>
     <row r="40">
@@ -10398,16 +10563,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>21.4302</v>
+        <v>21.4405</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>108030.2168154</v>
+        <v>108082.1393935</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>8030.216815399996</v>
+        <v>8082.139393500009</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.08030216815399996</v>
+        <v>0.08082139393500008</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -10549,6 +10714,9 @@
       </c>
       <c r="BE40" s="3" t="n">
         <v>21.4302</v>
+      </c>
+      <c r="BF40" s="3" t="n">
+        <v>21.4405</v>
       </c>
     </row>
     <row r="41">
@@ -10561,13 +10729,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4938543.4856034</v>
+        <v>4949302.8839843</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>468543.4856034</v>
+        <v>479302.8839843</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1048195717233557</v>
+        <v>0.1072265959696421</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-07-03
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -483,8 +483,8 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-02 05:57 IST</t>
+          <t>Generated: 2026-07-03 05:51 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4949302.8839843</v>
+        <v>4973326.7211613</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>479302.8839843003</v>
+        <v>503326.7211613003</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1072265959696421</v>
+        <v>0.1126010561882104</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>543934.9988632202</v>
+        <v>544960.0008850098</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-46847.0211367798</v>
+        <v>-45822.01911499025</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.07929662642200892</v>
+        <v>-0.07756163451790603</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5493237.882847521</v>
+        <v>5518286.72204631</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>432455.862847521</v>
+        <v>457504.7020463105</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.08545237892848841</v>
+        <v>0.09040197744899327</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-07-02</t>
+          <t>Last snapshot: 2026-07-03</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE19"/>
+  <dimension ref="A1:BF19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -676,6 +676,7 @@
     <col width="21" customWidth="1" min="55" max="55"/>
     <col width="21" customWidth="1" min="56" max="56"/>
     <col width="21" customWidth="1" min="57" max="57"/>
+    <col width="21" customWidth="1" min="58" max="58"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -964,6 +965,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="BF1" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -983,13 +989,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>543.1500244140625</v>
+        <v>541.4000244140625</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>43452.001953125</v>
+        <v>43312.001953125</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>-365.508046875002</v>
+        <v>-505.508046875002</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1137,6 +1143,9 @@
       </c>
       <c r="BE2" s="3" t="n">
         <v>543.1500244140625</v>
+      </c>
+      <c r="BF2" s="3" t="n">
+        <v>541.4000244140625</v>
       </c>
     </row>
     <row r="3">
@@ -1184,13 +1193,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1363</v>
+        <v>1363.599975585938</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>27260</v>
+        <v>27271.99951171875</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-4844.580000000002</v>
+        <v>-4832.580488281252</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1341,6 +1350,9 @@
       </c>
       <c r="BE4" s="3" t="n">
         <v>1363</v>
+      </c>
+      <c r="BF4" s="3" t="n">
+        <v>1363.599975585938</v>
       </c>
     </row>
     <row r="5">
@@ -1361,13 +1373,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>645.8499755859375</v>
+        <v>657.75</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>12916.99951171875</v>
+        <v>13155</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1296.10048828125</v>
+        <v>-1058.1</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1518,6 +1530,9 @@
       </c>
       <c r="BE5" s="3" t="n">
         <v>645.8499755859375</v>
+      </c>
+      <c r="BF5" s="3" t="n">
+        <v>657.75</v>
       </c>
     </row>
     <row r="6">
@@ -1538,13 +1553,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>364.75</v>
+        <v>369.5499877929688</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>14590</v>
+        <v>14781.99951171875</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2912.240000000002</v>
+        <v>-2720.240488281252</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1695,6 +1710,9 @@
       </c>
       <c r="BE6" s="3" t="n">
         <v>364.75</v>
+      </c>
+      <c r="BF6" s="3" t="n">
+        <v>369.5499877929688</v>
       </c>
     </row>
     <row r="7">
@@ -1715,13 +1733,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>236.1000061035156</v>
+        <v>237.6100006103516</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>23610.00061035156</v>
+        <v>23761.00006103516</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-2823.819389648437</v>
+        <v>-2672.819938964843</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1872,6 +1890,9 @@
       </c>
       <c r="BE7" s="3" t="n">
         <v>236.1000061035156</v>
+      </c>
+      <c r="BF7" s="3" t="n">
+        <v>237.6100006103516</v>
       </c>
     </row>
     <row r="8">
@@ -1919,13 +1940,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>17.98999977111816</v>
+        <v>17.82999992370605</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>26984.99965667725</v>
+        <v>26744.99988555908</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-4065.170343322752</v>
+        <v>-4305.170114440916</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -2076,6 +2097,9 @@
       </c>
       <c r="BE9" s="3" t="n">
         <v>17.98999977111816</v>
+      </c>
+      <c r="BF9" s="3" t="n">
+        <v>17.82999992370605</v>
       </c>
     </row>
     <row r="10">
@@ -2096,13 +2120,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>419.7999877929688</v>
+        <v>424.3999938964844</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>41979.99877929688</v>
+        <v>42439.99938964844</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-9518.481220703128</v>
+        <v>-9058.480610351566</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -2253,6 +2277,9 @@
       </c>
       <c r="BE10" s="3" t="n">
         <v>419.7999877929688</v>
+      </c>
+      <c r="BF10" s="3" t="n">
+        <v>424.3999938964844</v>
       </c>
     </row>
     <row r="11">
@@ -2273,13 +2300,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>9.270000457763672</v>
+        <v>10.13000011444092</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>9270.000457763672</v>
-      </c>
-      <c r="G11" s="6" t="n">
-        <v>-571.2095422363273</v>
+        <v>10130.00011444092</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>288.7901144409188</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -2430,6 +2457,9 @@
       </c>
       <c r="BE11" s="3" t="n">
         <v>9.270000457763672</v>
+      </c>
+      <c r="BF11" s="3" t="n">
+        <v>10.13000011444092</v>
       </c>
     </row>
     <row r="12">
@@ -2450,13 +2480,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2468</v>
+        <v>2496.10009765625</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>24680</v>
+        <v>24961.0009765625</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-3043.25</v>
+        <v>-2762.2490234375</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -2607,6 +2637,9 @@
       </c>
       <c r="BE12" s="3" t="n">
         <v>2468</v>
+      </c>
+      <c r="BF12" s="3" t="n">
+        <v>2496.10009765625</v>
       </c>
     </row>
     <row r="13">
@@ -2627,13 +2660,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>58.22999954223633</v>
+        <v>57.09000015258789</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>34937.9997253418</v>
+        <v>34254.00009155273</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-93.76027465820516</v>
+        <v>-777.7599084472677</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -2784,6 +2817,9 @@
       </c>
       <c r="BE13" s="3" t="n">
         <v>58.22999954223633</v>
+      </c>
+      <c r="BF13" s="3" t="n">
+        <v>57.09000015258789</v>
       </c>
     </row>
     <row r="14">
@@ -2804,13 +2840,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>689.8499755859375</v>
+        <v>696.7999877929688</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>34492.49877929688</v>
+        <v>34839.99938964844</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-7970.011220703127</v>
+        <v>-7622.510610351565</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -2961,6 +2997,9 @@
       </c>
       <c r="BE14" s="3" t="n">
         <v>689.8499755859375</v>
+      </c>
+      <c r="BF14" s="3" t="n">
+        <v>696.7999877929688</v>
       </c>
     </row>
     <row r="15">
@@ -3035,13 +3074,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>608.7999877929688</v>
+        <v>595.9500122070312</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>30439.99938964844</v>
+        <v>29797.50061035156</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>8685.469389648439</v>
+        <v>8042.970610351564</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -3192,6 +3231,9 @@
       </c>
       <c r="BE17" s="3" t="n">
         <v>608.7999877929688</v>
+      </c>
+      <c r="BF17" s="3" t="n">
+        <v>595.9500122070312</v>
       </c>
     </row>
     <row r="18">
@@ -3212,13 +3254,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>375.5</v>
+        <v>377.3999938964844</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>37550</v>
+        <v>37739.99938964844</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-9090.82</v>
+        <v>-8900.820610351562</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -3369,6 +3411,9 @@
       </c>
       <c r="BE18" s="3" t="n">
         <v>375.5</v>
+      </c>
+      <c r="BF18" s="3" t="n">
+        <v>377.3999938964844</v>
       </c>
     </row>
     <row r="19">
@@ -3381,10 +3426,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>543934.9988632202</v>
+        <v>544960.0008850098</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-46847.0211367798</v>
+        <v>-45822.01911499025</v>
       </c>
     </row>
   </sheetData>
@@ -3398,7 +3443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BF41"/>
+  <dimension ref="A1:BG41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3409,7 +3454,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
@@ -3459,6 +3504,7 @@
     <col width="13" customWidth="1" min="56" max="56"/>
     <col width="13" customWidth="1" min="57" max="57"/>
     <col width="13" customWidth="1" min="58" max="58"/>
+    <col width="13" customWidth="1" min="59" max="59"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3752,6 +3798,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="BG1" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3776,16 +3827,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.818</v>
+        <v>56.7917</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>63777.182276</v>
+        <v>63747.6609994</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>13777.182276</v>
+        <v>13747.6609994</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.27554364552</v>
+        <v>0.2749532199879999</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -3933,6 +3984,9 @@
       </c>
       <c r="BF2" s="3" t="n">
         <v>56.818</v>
+      </c>
+      <c r="BG2" s="3" t="n">
+        <v>56.7917</v>
       </c>
     </row>
     <row r="3">
@@ -3958,16 +4012,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.3951</v>
+        <v>25.7336</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>62350.37965630001</v>
+        <v>63181.4692568</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>2350.379656300007</v>
+        <v>3181.469256800003</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.03917299427166678</v>
+        <v>0.05302448761333338</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -4109,6 +4163,9 @@
       </c>
       <c r="BF3" s="3" t="n">
         <v>25.3951</v>
+      </c>
+      <c r="BG3" s="3" t="n">
+        <v>25.7336</v>
       </c>
     </row>
     <row r="4">
@@ -4134,16 +4191,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.01</v>
+        <v>12.18</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>230665.17693</v>
+        <v>233930.21274</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>50665.17693000002</v>
+        <v>53930.21274000002</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.2814732051666667</v>
+        <v>0.2996122930000001</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -4285,6 +4342,9 @@
       </c>
       <c r="BF4" s="3" t="n">
         <v>12.01</v>
+      </c>
+      <c r="BG4" s="3" t="n">
+        <v>12.18</v>
       </c>
     </row>
     <row r="5">
@@ -4310,16 +4370,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.323399999999999</v>
+        <v>9.435499999999999</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>171122.5040592</v>
+        <v>173179.997324</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-38877.4959408</v>
+        <v>-36820.002676</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1851309330514286</v>
+        <v>-0.1753333460761905</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -4461,6 +4521,9 @@
       </c>
       <c r="BF5" s="3" t="n">
         <v>9.323399999999999</v>
+      </c>
+      <c r="BG5" s="3" t="n">
+        <v>9.435499999999999</v>
       </c>
     </row>
     <row r="6">
@@ -4486,16 +4549,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.1012</v>
+        <v>12.0868</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>51175.6964724</v>
+        <v>51114.7992036</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>1175.696472399999</v>
+        <v>1114.7992036</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.02351392944799998</v>
+        <v>0.02229598407199999</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -4643,6 +4706,9 @@
       </c>
       <c r="BF6" s="3" t="n">
         <v>12.1012</v>
+      </c>
+      <c r="BG6" s="3" t="n">
+        <v>12.0868</v>
       </c>
     </row>
     <row r="7">
@@ -4668,16 +4734,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>34.0402</v>
+        <v>34.6981</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>75094.042808</v>
+        <v>76545.396524</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>15094.042808</v>
+        <v>16545.396524</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2515673801333333</v>
+        <v>0.2757566087333332</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -4819,6 +4885,9 @@
       </c>
       <c r="BF7" s="3" t="n">
         <v>34.0402</v>
+      </c>
+      <c r="BG7" s="3" t="n">
+        <v>34.6981</v>
       </c>
     </row>
     <row r="8">
@@ -4844,16 +4913,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>33.9583</v>
+        <v>34.1008</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>54489.25047190001</v>
+        <v>54717.9049744</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>4489.250471900006</v>
+        <v>4717.9049744</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.08978500943800012</v>
+        <v>0.094358099488</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -5001,6 +5070,9 @@
       </c>
       <c r="BF8" s="3" t="n">
         <v>33.9583</v>
+      </c>
+      <c r="BG8" s="3" t="n">
+        <v>34.1008</v>
       </c>
     </row>
     <row r="9">
@@ -5026,16 +5098,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>43.416</v>
+        <v>43.3305</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>139773.166488</v>
+        <v>139497.9083865</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>39773.16648799999</v>
+        <v>39497.9083865</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3977316648799999</v>
+        <v>0.394979083865</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -5177,6 +5249,9 @@
       </c>
       <c r="BF9" s="3" t="n">
         <v>43.416</v>
+      </c>
+      <c r="BG9" s="3" t="n">
+        <v>43.3305</v>
       </c>
     </row>
     <row r="10">
@@ -5202,16 +5277,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>47.4194</v>
+        <v>48.1528</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>134986.8617846</v>
+        <v>137074.6014952</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>34986.86178460001</v>
+        <v>37074.60149520001</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3498686178460002</v>
+        <v>0.3707460149520001</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -5353,6 +5428,9 @@
       </c>
       <c r="BF10" s="3" t="n">
         <v>47.4194</v>
+      </c>
+      <c r="BG10" s="3" t="n">
+        <v>48.1528</v>
       </c>
     </row>
     <row r="11">
@@ -5378,16 +5456,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>105.5166</v>
+        <v>104.2946</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31751.9497554</v>
+        <v>31384.2267374</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1751.949755399997</v>
+        <v>1384.2267374</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.0583983251799999</v>
+        <v>0.04614089124666668</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -5529,6 +5607,9 @@
       </c>
       <c r="BF11" s="3" t="n">
         <v>105.5166</v>
+      </c>
+      <c r="BG11" s="3" t="n">
+        <v>104.2946</v>
       </c>
     </row>
     <row r="12">
@@ -5554,16 +5635,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>227.179</v>
+        <v>229.575</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>105756.822438</v>
+        <v>106872.21315</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>5756.822438000003</v>
+        <v>6872.213149999996</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.05756822438000003</v>
+        <v>0.06872213149999996</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -5711,6 +5792,9 @@
       </c>
       <c r="BF12" s="3" t="n">
         <v>227.179</v>
+      </c>
+      <c r="BG12" s="3" t="n">
+        <v>229.575</v>
       </c>
     </row>
     <row r="13">
@@ -5736,16 +5820,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>21.034</v>
+        <v>21.216</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>243733.68357</v>
+        <v>245842.62768</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>43733.68356999996</v>
+        <v>45842.62768000001</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.2186684178499998</v>
+        <v>0.2292131384</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -5893,6 +5977,9 @@
       </c>
       <c r="BF13" s="3" t="n">
         <v>21.034</v>
+      </c>
+      <c r="BG13" s="3" t="n">
+        <v>21.216</v>
       </c>
     </row>
     <row r="14">
@@ -5918,16 +6005,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>38.6195</v>
+        <v>37.9283</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>139323.939917</v>
+        <v>136830.3626498</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>39323.93991700001</v>
+        <v>36830.36264980002</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.3932393991700001</v>
+        <v>0.3683036264980002</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -6069,6 +6156,9 @@
       </c>
       <c r="BF14" s="3" t="n">
         <v>38.6195</v>
+      </c>
+      <c r="BG14" s="3" t="n">
+        <v>37.9283</v>
       </c>
     </row>
     <row r="15">
@@ -6094,16 +6184,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.92</v>
+        <v>11.93</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>116147.84824</v>
+        <v>116245.28771</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>16147.84824000001</v>
+        <v>16245.28771</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1614784824000001</v>
+        <v>0.1624528771</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -6251,6 +6341,9 @@
       </c>
       <c r="BF15" s="3" t="n">
         <v>11.92</v>
+      </c>
+      <c r="BG15" s="3" t="n">
+        <v>11.93</v>
       </c>
     </row>
     <row r="16">
@@ -6276,16 +6369,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.5808</v>
+        <v>24.3227</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>140674.1485824</v>
+        <v>139197.0608656</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>40674.1485824</v>
+        <v>39197.06086560001</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.406741485824</v>
+        <v>0.3919706086560001</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -6427,6 +6520,9 @@
       </c>
       <c r="BF16" s="3" t="n">
         <v>24.5808</v>
+      </c>
+      <c r="BG16" s="3" t="n">
+        <v>24.3227</v>
       </c>
     </row>
     <row r="17">
@@ -6452,16 +6548,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.7895</v>
+        <v>16.8976</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55507.0440015</v>
+        <v>55864.4287632</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5507.044001499999</v>
+        <v>5864.428763199998</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.11014088003</v>
+        <v>0.117288575264</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -6603,6 +6699,9 @@
       </c>
       <c r="BF17" s="3" t="n">
         <v>16.7895</v>
+      </c>
+      <c r="BG17" s="3" t="n">
+        <v>16.8976</v>
       </c>
     </row>
     <row r="18">
@@ -6628,16 +6727,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>46.59</v>
+        <v>46.8</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>87889.05324000001</v>
+        <v>88285.20479999999</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>7889.053240000008</v>
+        <v>8285.204799999992</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.0986131655000001</v>
+        <v>0.1035650599999999</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -6785,6 +6884,9 @@
       </c>
       <c r="BF18" s="3" t="n">
         <v>46.59</v>
+      </c>
+      <c r="BG18" s="3" t="n">
+        <v>46.8</v>
       </c>
     </row>
     <row r="19">
@@ -6810,16 +6912,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>15.0717</v>
+        <v>14.5742</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>218038.7571222</v>
+        <v>210841.5410372</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>68038.75712219998</v>
+        <v>60841.54103719999</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.4535917141479999</v>
+        <v>0.4056102735813333</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -6961,6 +7063,9 @@
       </c>
       <c r="BF19" s="3" t="n">
         <v>15.0717</v>
+      </c>
+      <c r="BG19" s="3" t="n">
+        <v>14.5742</v>
       </c>
     </row>
     <row r="20">
@@ -6986,16 +7091,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.130000000000001</v>
+        <v>9.32</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>239715.48139</v>
+        <v>244704.08396</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-10284.51860999997</v>
+        <v>-5295.916039999982</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.04113807443999988</v>
+        <v>-0.02118366415999993</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -7143,6 +7248,9 @@
       </c>
       <c r="BF20" s="3" t="n">
         <v>9.130000000000001</v>
+      </c>
+      <c r="BG20" s="3" t="n">
+        <v>9.32</v>
       </c>
     </row>
     <row r="21">
@@ -7168,16 +7276,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>112.2987</v>
+        <v>113.2332</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>170610.8106633</v>
+        <v>172030.5581988</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>610.8106632999843</v>
+        <v>2030.55819879999</v>
       </c>
       <c r="I21" s="12" t="n">
-        <v>0.003593003901764613</v>
+        <v>0.01194445999294112</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -7325,6 +7433,9 @@
       </c>
       <c r="BF21" s="3" t="n">
         <v>112.2987</v>
+      </c>
+      <c r="BG21" s="3" t="n">
+        <v>113.2332</v>
       </c>
     </row>
     <row r="22">
@@ -7350,16 +7461,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>44.502</v>
+        <v>43.288</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>68286.53892000001</v>
+        <v>66423.70448</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>8286.538920000006</v>
+        <v>6423.70448</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1381089820000001</v>
+        <v>0.1070617413333333</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -7501,6 +7612,9 @@
       </c>
       <c r="BF22" s="3" t="n">
         <v>44.502</v>
+      </c>
+      <c r="BG22" s="3" t="n">
+        <v>43.288</v>
       </c>
     </row>
     <row r="23">
@@ -7526,16 +7640,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>63.9487</v>
+        <v>64.1413</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>173714.5332429</v>
+        <v>174237.7247871</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>23714.53324290001</v>
+        <v>24237.72478710001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.1580968882860001</v>
+        <v>0.1615848319140001</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -7683,6 +7797,9 @@
       </c>
       <c r="BF23" s="3" t="n">
         <v>63.9487</v>
+      </c>
+      <c r="BG23" s="3" t="n">
+        <v>64.1413</v>
       </c>
     </row>
     <row r="24">
@@ -7708,16 +7825,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>27.7429</v>
+        <v>27.8205</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>100800.6644594</v>
+        <v>101082.615213</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>800.6644593999954</v>
+        <v>1082.615212999997</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.008006644593999954</v>
+        <v>0.01082615212999997</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -7859,6 +7976,9 @@
       </c>
       <c r="BF24" s="3" t="n">
         <v>27.7429</v>
+      </c>
+      <c r="BG24" s="3" t="n">
+        <v>27.8205</v>
       </c>
     </row>
     <row r="25">
@@ -7884,16 +8004,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.6549</v>
+        <v>11.8009</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>191392.9683026</v>
+        <v>193790.5327066</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-8607.031697400031</v>
+        <v>-6209.467293399997</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.04303515848700015</v>
+        <v>-0.03104733646699999</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -8038,6 +8158,9 @@
       </c>
       <c r="BF25" s="3" t="n">
         <v>11.6549</v>
+      </c>
+      <c r="BG25" s="3" t="n">
+        <v>11.8009</v>
       </c>
     </row>
     <row r="26">
@@ -8063,16 +8186,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>9.2058</v>
+        <v>9.4598</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>109933.039947</v>
-      </c>
-      <c r="H26" s="6" t="n">
-        <v>-66.96005300000252</v>
-      </c>
-      <c r="I26" s="13" t="n">
-        <v>-0.0006087277545454774</v>
+        <v>112966.235557</v>
+      </c>
+      <c r="H26" s="4" t="n">
+        <v>2966.235556999993</v>
+      </c>
+      <c r="I26" s="12" t="n">
+        <v>0.02696577779090903</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -8217,6 +8340,9 @@
       </c>
       <c r="BF26" s="3" t="n">
         <v>9.2058</v>
+      </c>
+      <c r="BG26" s="3" t="n">
+        <v>9.4598</v>
       </c>
     </row>
     <row r="27">
@@ -8242,16 +8368,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>65.5801</v>
+        <v>65.875</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>105640.359886</v>
+        <v>106115.4025</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-4359.640114000009</v>
+        <v>-3884.597500000003</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.03963309194545463</v>
+        <v>-0.03531452272727276</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -8399,6 +8525,9 @@
       </c>
       <c r="BF27" s="3" t="n">
         <v>65.5801</v>
+      </c>
+      <c r="BG27" s="3" t="n">
+        <v>65.875</v>
       </c>
     </row>
     <row r="28">
@@ -8424,16 +8553,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>109.2744</v>
+        <v>110.107</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>361332.9596808</v>
+        <v>364086.082299</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-18667.04031919996</v>
+        <v>-15913.917701</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.04912379031368412</v>
+        <v>-0.04187873079210526</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -8581,6 +8710,9 @@
       </c>
       <c r="BF28" s="3" t="n">
         <v>109.2744</v>
+      </c>
+      <c r="BG28" s="3" t="n">
+        <v>110.107</v>
       </c>
     </row>
     <row r="29">
@@ -8606,16 +8738,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.518</v>
+        <v>12.5823</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>120219.154154</v>
+        <v>120836.6722569</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>20219.154154</v>
+        <v>20836.6722569</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.20219154154</v>
+        <v>0.208366722569</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -8757,6 +8889,9 @@
       </c>
       <c r="BF29" s="3" t="n">
         <v>12.518</v>
+      </c>
+      <c r="BG29" s="3" t="n">
+        <v>12.5823</v>
       </c>
     </row>
     <row r="30">
@@ -8782,16 +8917,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>16.6816</v>
+        <v>16.8422</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>123374.7948576</v>
+        <v>124562.5701342</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>23374.79485759999</v>
+        <v>24562.57013419998</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.2337479485759999</v>
+        <v>0.2456257013419998</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -8933,6 +9068,9 @@
       </c>
       <c r="BF30" s="3" t="n">
         <v>16.6816</v>
+      </c>
+      <c r="BG30" s="3" t="n">
+        <v>16.8422</v>
       </c>
     </row>
     <row r="31">
@@ -8958,16 +9096,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>419.6801</v>
+        <v>419.6335</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>111668.481008</v>
+        <v>111656.08168</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>11668.48100799999</v>
+        <v>11656.08168</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.1166848100799999</v>
+        <v>0.1165608168</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -9112,6 +9250,9 @@
       </c>
       <c r="BF31" s="3" t="n">
         <v>419.6801</v>
+      </c>
+      <c r="BG31" s="3" t="n">
+        <v>419.6335</v>
       </c>
     </row>
     <row r="32">
@@ -9137,16 +9278,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.58</v>
+        <v>10.66</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>223660.7768</v>
+        <v>225351.9736</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>23660.77679999999</v>
+        <v>25351.9736</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.118303884</v>
+        <v>0.126759868</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -9294,6 +9435,9 @@
       </c>
       <c r="BF32" s="3" t="n">
         <v>10.58</v>
+      </c>
+      <c r="BG32" s="3" t="n">
+        <v>10.66</v>
       </c>
     </row>
     <row r="33">
@@ -9319,16 +9463,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>18.99</v>
+        <v>19.11</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>68053.32359999999</v>
+        <v>68483.36039999999</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>8053.323599999989</v>
+        <v>8483.36039999999</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.1342220599999998</v>
+        <v>0.1413893399999998</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -9470,6 +9614,9 @@
       </c>
       <c r="BF33" s="3" t="n">
         <v>18.99</v>
+      </c>
+      <c r="BG33" s="3" t="n">
+        <v>19.11</v>
       </c>
     </row>
     <row r="34">
@@ -9495,16 +9642,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>204.8743</v>
+        <v>209.343</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>72019.66755330001</v>
+        <v>73590.554133</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-7980.332446699991</v>
+        <v>-6409.445867000002</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.09975415558374989</v>
+        <v>-0.08011807333750003</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -9649,6 +9796,9 @@
       </c>
       <c r="BF34" s="3" t="n">
         <v>204.8743</v>
+      </c>
+      <c r="BG34" s="3" t="n">
+        <v>209.343</v>
       </c>
     </row>
     <row r="35">
@@ -9674,16 +9824,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>15.04</v>
+        <v>14.98</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>107316.76192</v>
+        <v>106888.63654</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>7316.76191999999</v>
+        <v>6888.636540000007</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.07316761919999989</v>
+        <v>0.06888636540000007</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -9828,6 +9978,9 @@
       </c>
       <c r="BF35" s="3" t="n">
         <v>15.04</v>
+      </c>
+      <c r="BG35" s="3" t="n">
+        <v>14.98</v>
       </c>
     </row>
     <row r="36">
@@ -9853,16 +10006,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>370.0029</v>
+        <v>371.7018</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>172312.5705474</v>
+        <v>173103.7584708</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>22312.57054740001</v>
+        <v>23103.75847080001</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1487504703160001</v>
+        <v>0.154025056472</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -10007,6 +10160,9 @@
       </c>
       <c r="BF36" s="3" t="n">
         <v>370.0029</v>
+      </c>
+      <c r="BG36" s="3" t="n">
+        <v>371.7018</v>
       </c>
     </row>
     <row r="37">
@@ -10032,16 +10188,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>16.582</v>
+        <v>16.739</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>62396.225398</v>
+        <v>62986.99897100001</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>12396.225398</v>
+        <v>12986.99897100001</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.24792450796</v>
+        <v>0.2597399794200002</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -10186,6 +10342,9 @@
       </c>
       <c r="BF37" s="3" t="n">
         <v>16.582</v>
+      </c>
+      <c r="BG37" s="3" t="n">
+        <v>16.739</v>
       </c>
     </row>
     <row r="38">
@@ -10211,16 +10370,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>14.3009</v>
+        <v>14.3831</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>85526.2750338</v>
+        <v>86017.8706542</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>5526.275033800004</v>
+        <v>6017.8706542</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.06907843792250005</v>
+        <v>0.07522338317750001</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -10362,6 +10521,9 @@
       </c>
       <c r="BF38" s="3" t="n">
         <v>14.3009</v>
+      </c>
+      <c r="BG38" s="3" t="n">
+        <v>14.3831</v>
       </c>
     </row>
     <row r="39">
@@ -10387,16 +10549,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1022.1898</v>
+        <v>1021.9951</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50987.8494138</v>
+        <v>50978.1375831</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>987.8494138000024</v>
+        <v>978.1375830999968</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.01975698827600005</v>
+        <v>0.01956275166199994</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -10538,6 +10700,9 @@
       </c>
       <c r="BF39" s="3" t="n">
         <v>1022.1898</v>
+      </c>
+      <c r="BG39" s="3" t="n">
+        <v>1021.9951</v>
       </c>
     </row>
     <row r="40">
@@ -10563,16 +10728,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>21.4405</v>
+        <v>21.6385</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>108082.1393935</v>
+        <v>109080.2627395</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>8082.139393500009</v>
+        <v>9080.262739500002</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.08082139393500008</v>
+        <v>0.09080262739500002</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -10717,6 +10882,9 @@
       </c>
       <c r="BF40" s="3" t="n">
         <v>21.4405</v>
+      </c>
+      <c r="BG40" s="3" t="n">
+        <v>21.6385</v>
       </c>
     </row>
     <row r="41">
@@ -10729,13 +10897,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4949302.8839843</v>
+        <v>4973326.7211613</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>479302.8839843</v>
+        <v>503326.7211613</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1072265959696421</v>
+        <v>0.1126010561882103</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-07-04
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-03 05:51 IST</t>
+          <t>Generated: 2026-07-04 05:44 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4973326.7211613</v>
+        <v>4979687.3004521</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>503326.7211613003</v>
+        <v>509687.3004521001</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1126010561882104</v>
+        <v>0.1140240045754139</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>544960.0008850098</v>
+        <v>544721.5007858276</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-45822.01911499025</v>
+        <v>-46060.51921417238</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.07756163451790603</v>
+        <v>-0.07796533688376701</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5518286.72204631</v>
+        <v>5524408.801237928</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>457504.7020463105</v>
+        <v>463626.7812379282</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.09040197744899327</v>
+        <v>0.09161168756245468</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-07-03</t>
+          <t>Last snapshot: 2026-07-04</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BF19"/>
+  <dimension ref="A1:BG19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -677,6 +677,7 @@
     <col width="21" customWidth="1" min="56" max="56"/>
     <col width="21" customWidth="1" min="57" max="57"/>
     <col width="21" customWidth="1" min="58" max="58"/>
+    <col width="21" customWidth="1" min="59" max="59"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -970,6 +971,11 @@
           <t>2026-07-03</t>
         </is>
       </c>
+      <c r="BG1" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -989,13 +995,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>541.4000244140625</v>
+        <v>540.9000244140625</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>43312.001953125</v>
+        <v>43272.001953125</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>-505.508046875002</v>
+        <v>-545.508046875002</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1146,6 +1152,9 @@
       </c>
       <c r="BF2" s="3" t="n">
         <v>541.4000244140625</v>
+      </c>
+      <c r="BG2" s="3" t="n">
+        <v>540.9000244140625</v>
       </c>
     </row>
     <row r="3">
@@ -1193,13 +1202,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1363.599975585938</v>
+        <v>1385</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>27271.99951171875</v>
+        <v>27700</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-4832.580488281252</v>
+        <v>-4404.580000000002</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1353,6 +1362,9 @@
       </c>
       <c r="BF4" s="3" t="n">
         <v>1363.599975585938</v>
+      </c>
+      <c r="BG4" s="3" t="n">
+        <v>1385</v>
       </c>
     </row>
     <row r="5">
@@ -1373,13 +1385,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>657.75</v>
+        <v>662.2000122070312</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13155</v>
+        <v>13244.00024414062</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1058.1</v>
+        <v>-969.0997558593754</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1533,6 +1545,9 @@
       </c>
       <c r="BF5" s="3" t="n">
         <v>657.75</v>
+      </c>
+      <c r="BG5" s="3" t="n">
+        <v>662.2000122070312</v>
       </c>
     </row>
     <row r="6">
@@ -1553,13 +1568,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>369.5499877929688</v>
+        <v>366.8500061035156</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>14781.99951171875</v>
+        <v>14674.00024414062</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2720.240488281252</v>
+        <v>-2828.239755859377</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1713,6 +1728,9 @@
       </c>
       <c r="BF6" s="3" t="n">
         <v>369.5499877929688</v>
+      </c>
+      <c r="BG6" s="3" t="n">
+        <v>366.8500061035156</v>
       </c>
     </row>
     <row r="7">
@@ -1733,13 +1751,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>237.6100006103516</v>
+        <v>237.4900054931641</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>23761.00006103516</v>
+        <v>23749.00054931641</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-2672.819938964843</v>
+        <v>-2684.819450683593</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1893,6 +1911,9 @@
       </c>
       <c r="BF7" s="3" t="n">
         <v>237.6100006103516</v>
+      </c>
+      <c r="BG7" s="3" t="n">
+        <v>237.4900054931641</v>
       </c>
     </row>
     <row r="8">
@@ -1940,13 +1961,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>17.82999992370605</v>
+        <v>17.79999923706055</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>26744.99988555908</v>
+        <v>26699.99885559082</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-4305.170114440916</v>
+        <v>-4350.171144409178</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -2100,6 +2121,9 @@
       </c>
       <c r="BF9" s="3" t="n">
         <v>17.82999992370605</v>
+      </c>
+      <c r="BG9" s="3" t="n">
+        <v>17.79999923706055</v>
       </c>
     </row>
     <row r="10">
@@ -2120,13 +2144,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>424.3999938964844</v>
+        <v>422.1000061035156</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>42439.99938964844</v>
+        <v>42210.00061035156</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-9058.480610351566</v>
+        <v>-9288.479389648441</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -2280,6 +2304,9 @@
       </c>
       <c r="BF10" s="3" t="n">
         <v>424.3999938964844</v>
+      </c>
+      <c r="BG10" s="3" t="n">
+        <v>422.1000061035156</v>
       </c>
     </row>
     <row r="11">
@@ -2300,13 +2327,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>10.13000011444092</v>
+        <v>10.30000019073486</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>10130.00011444092</v>
+        <v>10300.00019073486</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>288.7901144409188</v>
+        <v>458.7901907348642</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -2460,6 +2487,9 @@
       </c>
       <c r="BF11" s="3" t="n">
         <v>10.13000011444092</v>
+      </c>
+      <c r="BG11" s="3" t="n">
+        <v>10.30000019073486</v>
       </c>
     </row>
     <row r="12">
@@ -2480,13 +2510,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2496.10009765625</v>
+        <v>2512.5</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>24961.0009765625</v>
+        <v>25125</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2762.2490234375</v>
+        <v>-2598.25</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -2640,6 +2670,9 @@
       </c>
       <c r="BF12" s="3" t="n">
         <v>2496.10009765625</v>
+      </c>
+      <c r="BG12" s="3" t="n">
+        <v>2512.5</v>
       </c>
     </row>
     <row r="13">
@@ -2660,13 +2693,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>57.09000015258789</v>
+        <v>56.86999893188477</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>34254.00009155273</v>
+        <v>34121.99935913086</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-777.7599084472677</v>
+        <v>-909.7606408691427</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -2820,6 +2853,9 @@
       </c>
       <c r="BF13" s="3" t="n">
         <v>57.09000015258789</v>
+      </c>
+      <c r="BG13" s="3" t="n">
+        <v>56.86999893188477</v>
       </c>
     </row>
     <row r="14">
@@ -2840,13 +2876,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>696.7999877929688</v>
+        <v>693.0999755859375</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>34839.99938964844</v>
+        <v>34654.99877929688</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-7622.510610351565</v>
+        <v>-7807.511220703127</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -3000,6 +3036,9 @@
       </c>
       <c r="BF14" s="3" t="n">
         <v>696.7999877929688</v>
+      </c>
+      <c r="BG14" s="3" t="n">
+        <v>693.0999755859375</v>
       </c>
     </row>
     <row r="15">
@@ -3074,13 +3113,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>595.9500122070312</v>
+        <v>593.5999755859375</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>29797.50061035156</v>
+        <v>29679.99877929688</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>8042.970610351564</v>
+        <v>7925.468779296876</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -3234,6 +3273,9 @@
       </c>
       <c r="BF17" s="3" t="n">
         <v>595.9500122070312</v>
+      </c>
+      <c r="BG17" s="3" t="n">
+        <v>593.5999755859375</v>
       </c>
     </row>
     <row r="18">
@@ -3254,13 +3296,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>377.3999938964844</v>
+        <v>375.2000122070312</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>37739.99938964844</v>
+        <v>37520.00122070312</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-8900.820610351562</v>
+        <v>-9120.818779296875</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -3414,6 +3456,9 @@
       </c>
       <c r="BF18" s="3" t="n">
         <v>377.3999938964844</v>
+      </c>
+      <c r="BG18" s="3" t="n">
+        <v>375.2000122070312</v>
       </c>
     </row>
     <row r="19">
@@ -3426,10 +3471,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>544960.0008850098</v>
+        <v>544721.5007858276</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-45822.01911499025</v>
+        <v>-46060.51921417237</v>
       </c>
     </row>
   </sheetData>
@@ -3443,7 +3488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BG41"/>
+  <dimension ref="A1:BH41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3505,6 +3550,7 @@
     <col width="13" customWidth="1" min="57" max="57"/>
     <col width="13" customWidth="1" min="58" max="58"/>
     <col width="13" customWidth="1" min="59" max="59"/>
+    <col width="13" customWidth="1" min="60" max="60"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3803,6 +3849,11 @@
           <t>2026-07-03</t>
         </is>
       </c>
+      <c r="BH1" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3827,16 +3878,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.7917</v>
+        <v>56.762</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>63747.6609994</v>
+        <v>63714.323284</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>13747.6609994</v>
+        <v>13714.323284</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.2749532199879999</v>
+        <v>0.27428646568</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -3987,6 +4038,9 @@
       </c>
       <c r="BG2" s="3" t="n">
         <v>56.7917</v>
+      </c>
+      <c r="BH2" s="3" t="n">
+        <v>56.762</v>
       </c>
     </row>
     <row r="3">
@@ -4167,6 +4221,9 @@
       <c r="BG3" s="3" t="n">
         <v>25.7336</v>
       </c>
+      <c r="BH3" s="3" t="n">
+        <v>25.7336</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4346,6 +4403,9 @@
       <c r="BG4" s="3" t="n">
         <v>12.18</v>
       </c>
+      <c r="BH4" s="3" t="n">
+        <v>12.18</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4370,16 +4430,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.435499999999999</v>
+        <v>9.4689</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>173179.997324</v>
+        <v>173793.0238632</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-36820.002676</v>
+        <v>-36206.97613680002</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1753333460761905</v>
+        <v>-0.1724141720800001</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -4524,6 +4584,9 @@
       </c>
       <c r="BG5" s="3" t="n">
         <v>9.435499999999999</v>
+      </c>
+      <c r="BH5" s="3" t="n">
+        <v>9.4689</v>
       </c>
     </row>
     <row r="6">
@@ -4549,16 +4612,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.0868</v>
+        <v>11.9457</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>51114.7992036</v>
+        <v>50518.0905489</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>1114.7992036</v>
+        <v>518.0905488999997</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.02229598407199999</v>
+        <v>0.01036181097799999</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -4709,6 +4772,9 @@
       </c>
       <c r="BG6" s="3" t="n">
         <v>12.0868</v>
+      </c>
+      <c r="BH6" s="3" t="n">
+        <v>11.9457</v>
       </c>
     </row>
     <row r="7">
@@ -4734,16 +4800,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>34.6981</v>
+        <v>35.0445</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>76545.396524</v>
+        <v>77309.56878</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>16545.396524</v>
+        <v>17309.56878</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2757566087333332</v>
+        <v>0.288492813</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -4888,6 +4954,9 @@
       </c>
       <c r="BG7" s="3" t="n">
         <v>34.6981</v>
+      </c>
+      <c r="BH7" s="3" t="n">
+        <v>35.0445</v>
       </c>
     </row>
     <row r="8">
@@ -4913,16 +4982,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>34.1008</v>
+        <v>33.8955</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>54717.9049744</v>
+        <v>54388.4820315</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>4717.9049744</v>
+        <v>4388.482031500003</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.094358099488</v>
+        <v>0.08776964063000006</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -5073,6 +5142,9 @@
       </c>
       <c r="BG8" s="3" t="n">
         <v>34.1008</v>
+      </c>
+      <c r="BH8" s="3" t="n">
+        <v>33.8955</v>
       </c>
     </row>
     <row r="9">
@@ -5253,6 +5325,9 @@
       <c r="BG9" s="3" t="n">
         <v>43.3305</v>
       </c>
+      <c r="BH9" s="3" t="n">
+        <v>43.3305</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5432,6 +5507,9 @@
       <c r="BG10" s="3" t="n">
         <v>48.1528</v>
       </c>
+      <c r="BH10" s="3" t="n">
+        <v>48.1528</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5611,6 +5689,9 @@
       <c r="BG11" s="3" t="n">
         <v>104.2946</v>
       </c>
+      <c r="BH11" s="3" t="n">
+        <v>104.2946</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5635,16 +5716,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>229.575</v>
+        <v>229.594</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>106872.21315</v>
+        <v>106881.058068</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>6872.213149999996</v>
+        <v>6881.058067999998</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.06872213149999996</v>
+        <v>0.06881058067999998</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -5795,6 +5876,9 @@
       </c>
       <c r="BG12" s="3" t="n">
         <v>229.575</v>
+      </c>
+      <c r="BH12" s="3" t="n">
+        <v>229.594</v>
       </c>
     </row>
     <row r="13">
@@ -5820,16 +5904,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>21.216</v>
+        <v>21.409</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>245842.62768</v>
+        <v>248079.035445</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>45842.62768000001</v>
+        <v>48079.03544499999</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.2292131384</v>
+        <v>0.2403951772249999</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -5980,6 +6064,9 @@
       </c>
       <c r="BG13" s="3" t="n">
         <v>21.216</v>
+      </c>
+      <c r="BH13" s="3" t="n">
+        <v>21.409</v>
       </c>
     </row>
     <row r="14">
@@ -6005,16 +6092,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>37.9283</v>
+        <v>38.7629</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>136830.3626498</v>
+        <v>139841.2706174</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>36830.36264980002</v>
+        <v>39841.2706174</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.3683036264980002</v>
+        <v>0.398412706174</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -6159,6 +6246,9 @@
       </c>
       <c r="BG14" s="3" t="n">
         <v>37.9283</v>
+      </c>
+      <c r="BH14" s="3" t="n">
+        <v>38.7629</v>
       </c>
     </row>
     <row r="15">
@@ -6184,16 +6274,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.93</v>
+        <v>11.79</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>116245.28771</v>
+        <v>114881.13513</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>16245.28771</v>
+        <v>14881.13513</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1624528771</v>
+        <v>0.1488113512999999</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -6344,6 +6434,9 @@
       </c>
       <c r="BG15" s="3" t="n">
         <v>11.93</v>
+      </c>
+      <c r="BH15" s="3" t="n">
+        <v>11.79</v>
       </c>
     </row>
     <row r="16">
@@ -6524,6 +6617,9 @@
       <c r="BG16" s="3" t="n">
         <v>24.3227</v>
       </c>
+      <c r="BH16" s="3" t="n">
+        <v>24.3227</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -6703,6 +6799,9 @@
       <c r="BG17" s="3" t="n">
         <v>16.8976</v>
       </c>
+      <c r="BH17" s="3" t="n">
+        <v>16.8976</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -6727,16 +6826,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>46.8</v>
+        <v>47.31</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>88285.20479999999</v>
+        <v>89247.28716000001</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>8285.204799999992</v>
+        <v>9247.287160000007</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.1035650599999999</v>
+        <v>0.1155910895000001</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -6887,6 +6986,9 @@
       </c>
       <c r="BG18" s="3" t="n">
         <v>46.8</v>
+      </c>
+      <c r="BH18" s="3" t="n">
+        <v>47.31</v>
       </c>
     </row>
     <row r="19">
@@ -7067,6 +7169,9 @@
       <c r="BG19" s="3" t="n">
         <v>14.5742</v>
       </c>
+      <c r="BH19" s="3" t="n">
+        <v>14.5742</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -7252,6 +7357,9 @@
       <c r="BG20" s="3" t="n">
         <v>9.32</v>
       </c>
+      <c r="BH20" s="3" t="n">
+        <v>9.32</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -7276,16 +7384,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>113.2332</v>
+        <v>113.0168</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>172030.5581988</v>
+        <v>171701.7905512</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>2030.55819879999</v>
+        <v>1701.790551200014</v>
       </c>
       <c r="I21" s="12" t="n">
-        <v>0.01194445999294112</v>
+        <v>0.01001053265411773</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -7436,6 +7544,9 @@
       </c>
       <c r="BG21" s="3" t="n">
         <v>113.2332</v>
+      </c>
+      <c r="BH21" s="3" t="n">
+        <v>113.0168</v>
       </c>
     </row>
     <row r="22">
@@ -7461,16 +7572,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>43.288</v>
+        <v>44.15</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>66423.70448</v>
+        <v>67746.409</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>6423.70448</v>
+        <v>7746.409</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1070617413333333</v>
+        <v>0.1291068166666667</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -7615,6 +7726,9 @@
       </c>
       <c r="BG22" s="3" t="n">
         <v>43.288</v>
+      </c>
+      <c r="BH22" s="3" t="n">
+        <v>44.15</v>
       </c>
     </row>
     <row r="23">
@@ -7640,16 +7754,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>64.1413</v>
+        <v>63.8309</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>174237.7247871</v>
+        <v>173394.5334303</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>24237.72478710001</v>
+        <v>23394.53343030001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.1615848319140001</v>
+        <v>0.1559635562020001</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -7800,6 +7914,9 @@
       </c>
       <c r="BG23" s="3" t="n">
         <v>64.1413</v>
+      </c>
+      <c r="BH23" s="3" t="n">
+        <v>63.8309</v>
       </c>
     </row>
     <row r="24">
@@ -7825,16 +7942,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>27.8205</v>
+        <v>27.732</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>101082.615213</v>
+        <v>100761.060552</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>1082.615212999997</v>
+        <v>761.0605519999954</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.01082615212999997</v>
+        <v>0.007610605519999954</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -7979,6 +8096,9 @@
       </c>
       <c r="BG24" s="3" t="n">
         <v>27.8205</v>
+      </c>
+      <c r="BH24" s="3" t="n">
+        <v>27.732</v>
       </c>
     </row>
     <row r="25">
@@ -8004,16 +8124,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.8009</v>
+        <v>11.8619</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>193790.5327066</v>
+        <v>194792.2548206</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-6209.467293399997</v>
+        <v>-5207.745179399994</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.03104733646699999</v>
+        <v>-0.02603872589699997</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -8161,6 +8281,9 @@
       </c>
       <c r="BG25" s="3" t="n">
         <v>11.8009</v>
+      </c>
+      <c r="BH25" s="3" t="n">
+        <v>11.8619</v>
       </c>
     </row>
     <row r="26">
@@ -8186,16 +8309,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>9.4598</v>
+        <v>9.526199999999999</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>112966.235557</v>
+        <v>113759.165433</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>2966.235556999993</v>
+        <v>3759.165432999987</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.02696577779090903</v>
+        <v>0.03417423120909079</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -8343,6 +8466,9 @@
       </c>
       <c r="BG26" s="3" t="n">
         <v>9.4598</v>
+      </c>
+      <c r="BH26" s="3" t="n">
+        <v>9.526199999999999</v>
       </c>
     </row>
     <row r="27">
@@ -8368,16 +8494,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>65.875</v>
+        <v>65.61020000000001</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>106115.4025</v>
+        <v>105688.846772</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-3884.597500000003</v>
+        <v>-4311.153227999996</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.03531452272727276</v>
+        <v>-0.03919230207272723</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -8528,6 +8654,9 @@
       </c>
       <c r="BG27" s="3" t="n">
         <v>65.875</v>
+      </c>
+      <c r="BH27" s="3" t="n">
+        <v>65.61020000000001</v>
       </c>
     </row>
     <row r="28">
@@ -8553,16 +8682,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>110.107</v>
+        <v>110.2185</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>364086.082299</v>
+        <v>364454.7745545001</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-15913.917701</v>
+        <v>-15545.22544549993</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.04187873079210526</v>
+        <v>-0.04090848801447351</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -8713,6 +8842,9 @@
       </c>
       <c r="BG28" s="3" t="n">
         <v>110.107</v>
+      </c>
+      <c r="BH28" s="3" t="n">
+        <v>110.2185</v>
       </c>
     </row>
     <row r="29">
@@ -8738,16 +8870,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.5823</v>
+        <v>12.5477</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>120836.6722569</v>
+        <v>120504.3841331</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>20836.6722569</v>
+        <v>20504.3841331</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.208366722569</v>
+        <v>0.205043841331</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -8892,6 +9024,9 @@
       </c>
       <c r="BG29" s="3" t="n">
         <v>12.5823</v>
+      </c>
+      <c r="BH29" s="3" t="n">
+        <v>12.5477</v>
       </c>
     </row>
     <row r="30">
@@ -8917,16 +9052,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>16.8422</v>
+        <v>16.7276</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>124562.5701342</v>
+        <v>123715.0044636</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>24562.57013419998</v>
+        <v>23715.00446359999</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.2456257013419998</v>
+        <v>0.237150044636</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -9071,6 +9206,9 @@
       </c>
       <c r="BG30" s="3" t="n">
         <v>16.8422</v>
+      </c>
+      <c r="BH30" s="3" t="n">
+        <v>16.7276</v>
       </c>
     </row>
     <row r="31">
@@ -9096,16 +9234,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>419.6335</v>
+        <v>417.1665</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>111656.08168</v>
+        <v>110999.66232</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>11656.08168</v>
+        <v>10999.66231999999</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.1165608168</v>
+        <v>0.1099966231999999</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -9253,6 +9391,9 @@
       </c>
       <c r="BG31" s="3" t="n">
         <v>419.6335</v>
+      </c>
+      <c r="BH31" s="3" t="n">
+        <v>417.1665</v>
       </c>
     </row>
     <row r="32">
@@ -9278,16 +9419,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.66</v>
+        <v>10.64</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>225351.9736</v>
+        <v>224929.1744</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>25351.9736</v>
+        <v>24929.17439999999</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.126759868</v>
+        <v>0.1246458719999999</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -9438,6 +9579,9 @@
       </c>
       <c r="BG32" s="3" t="n">
         <v>10.66</v>
+      </c>
+      <c r="BH32" s="3" t="n">
+        <v>10.64</v>
       </c>
     </row>
     <row r="33">
@@ -9463,16 +9607,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>19.11</v>
+        <v>19</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>68483.36039999999</v>
+        <v>68089.16</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>8483.36039999999</v>
+        <v>8089.160000000003</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.1413893399999998</v>
+        <v>0.1348193333333334</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -9617,6 +9761,9 @@
       </c>
       <c r="BG33" s="3" t="n">
         <v>19.11</v>
+      </c>
+      <c r="BH33" s="3" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="34">
@@ -9642,16 +9789,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>209.343</v>
+        <v>210.8218</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>73590.554133</v>
+        <v>74110.3981758</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-6409.445867000002</v>
+        <v>-5889.601824199999</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.08011807333750003</v>
+        <v>-0.07362002280249999</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -9799,6 +9946,9 @@
       </c>
       <c r="BG34" s="3" t="n">
         <v>209.343</v>
+      </c>
+      <c r="BH34" s="3" t="n">
+        <v>210.8218</v>
       </c>
     </row>
     <row r="35">
@@ -9824,16 +9974,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>14.98</v>
+        <v>14.83</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>106888.63654</v>
+        <v>105818.32309</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>6888.636540000007</v>
+        <v>5818.323089999991</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.06888636540000007</v>
+        <v>0.05818323089999991</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -9981,6 +10131,9 @@
       </c>
       <c r="BG35" s="3" t="n">
         <v>14.98</v>
+      </c>
+      <c r="BH35" s="3" t="n">
+        <v>14.83</v>
       </c>
     </row>
     <row r="36">
@@ -10006,16 +10159,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>371.7018</v>
+        <v>374.9716</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>173103.7584708</v>
+        <v>174626.5239496</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>23103.75847080001</v>
+        <v>24626.52394960003</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.154025056472</v>
+        <v>0.1641768263306669</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -10163,6 +10316,9 @@
       </c>
       <c r="BG36" s="3" t="n">
         <v>371.7018</v>
+      </c>
+      <c r="BH36" s="3" t="n">
+        <v>374.9716</v>
       </c>
     </row>
     <row r="37">
@@ -10188,16 +10344,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>16.739</v>
+        <v>16.901</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>62986.99897100001</v>
+        <v>63596.586989</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>12986.99897100001</v>
+        <v>13596.586989</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.2597399794200002</v>
+        <v>0.2719317397800001</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -10345,6 +10501,9 @@
       </c>
       <c r="BG37" s="3" t="n">
         <v>16.739</v>
+      </c>
+      <c r="BH37" s="3" t="n">
+        <v>16.901</v>
       </c>
     </row>
     <row r="38">
@@ -10370,16 +10529,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>14.3831</v>
+        <v>14.3909</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>86017.8706542</v>
+        <v>86064.5184138</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>6017.8706542</v>
+        <v>6064.518413800004</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.07522338317750001</v>
+        <v>0.07580648017250005</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -10524,6 +10683,9 @@
       </c>
       <c r="BG38" s="3" t="n">
         <v>14.3831</v>
+      </c>
+      <c r="BH38" s="3" t="n">
+        <v>14.3909</v>
       </c>
     </row>
     <row r="39">
@@ -10549,16 +10711,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1021.9951</v>
+        <v>1022.3097</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50978.1375831</v>
+        <v>50993.8301457</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>978.1375830999968</v>
+        <v>993.830145699998</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.01956275166199994</v>
+        <v>0.01987660291399996</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -10703,6 +10865,9 @@
       </c>
       <c r="BG39" s="3" t="n">
         <v>1021.9951</v>
+      </c>
+      <c r="BH39" s="3" t="n">
+        <v>1022.3097</v>
       </c>
     </row>
     <row r="40">
@@ -10728,16 +10893,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>21.6385</v>
+        <v>21.744</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>109080.2627395</v>
+        <v>109612.091088</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>9080.262739500002</v>
+        <v>9612.091088000001</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.09080262739500002</v>
+        <v>0.09612091088000001</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -10885,6 +11050,9 @@
       </c>
       <c r="BG40" s="3" t="n">
         <v>21.6385</v>
+      </c>
+      <c r="BH40" s="3" t="n">
+        <v>21.744</v>
       </c>
     </row>
     <row r="41">
@@ -10897,13 +11065,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4973326.7211613</v>
+        <v>4979687.3004521</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>503326.7211613</v>
+        <v>509687.3004521001</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1126010561882103</v>
+        <v>0.1140240045754139</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-07-05
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-04 05:44 IST</t>
+          <t>Generated: 2026-07-05 06:03 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4979687.3004521</v>
+        <v>4983336.4581221</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>509687.3004521001</v>
+        <v>513336.4581220997</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1140240045754139</v>
+        <v>0.1148403709445413</v>
       </c>
     </row>
     <row r="6">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5524408.801237928</v>
+        <v>5528057.958907927</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>463626.7812379282</v>
+        <v>467275.9389079278</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.09161168756245468</v>
+        <v>0.09233275352727559</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-07-04</t>
+          <t>Last snapshot: 2026-07-05</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BG19"/>
+  <dimension ref="A1:BH19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -678,6 +678,7 @@
     <col width="21" customWidth="1" min="57" max="57"/>
     <col width="21" customWidth="1" min="58" max="58"/>
     <col width="21" customWidth="1" min="59" max="59"/>
+    <col width="21" customWidth="1" min="60" max="60"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -976,6 +977,11 @@
           <t>2026-07-04</t>
         </is>
       </c>
+      <c r="BH1" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1156,6 +1162,9 @@
       <c r="BG2" s="3" t="n">
         <v>540.9000244140625</v>
       </c>
+      <c r="BH2" s="3" t="n">
+        <v>540.9000244140625</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1366,6 +1375,9 @@
       <c r="BG4" s="3" t="n">
         <v>1385</v>
       </c>
+      <c r="BH4" s="3" t="n">
+        <v>1385</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1549,6 +1561,9 @@
       <c r="BG5" s="3" t="n">
         <v>662.2000122070312</v>
       </c>
+      <c r="BH5" s="3" t="n">
+        <v>662.2000122070312</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1732,6 +1747,9 @@
       <c r="BG6" s="3" t="n">
         <v>366.8500061035156</v>
       </c>
+      <c r="BH6" s="3" t="n">
+        <v>366.8500061035156</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1915,6 +1933,9 @@
       <c r="BG7" s="3" t="n">
         <v>237.4900054931641</v>
       </c>
+      <c r="BH7" s="3" t="n">
+        <v>237.4900054931641</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2125,6 +2146,9 @@
       <c r="BG9" s="3" t="n">
         <v>17.79999923706055</v>
       </c>
+      <c r="BH9" s="3" t="n">
+        <v>17.79999923706055</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2308,6 +2332,9 @@
       <c r="BG10" s="3" t="n">
         <v>422.1000061035156</v>
       </c>
+      <c r="BH10" s="3" t="n">
+        <v>422.1000061035156</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2491,6 +2518,9 @@
       <c r="BG11" s="3" t="n">
         <v>10.30000019073486</v>
       </c>
+      <c r="BH11" s="3" t="n">
+        <v>10.30000019073486</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2674,6 +2704,9 @@
       <c r="BG12" s="3" t="n">
         <v>2512.5</v>
       </c>
+      <c r="BH12" s="3" t="n">
+        <v>2512.5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2857,6 +2890,9 @@
       <c r="BG13" s="3" t="n">
         <v>56.86999893188477</v>
       </c>
+      <c r="BH13" s="3" t="n">
+        <v>56.86999893188477</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3040,6 +3076,9 @@
       <c r="BG14" s="3" t="n">
         <v>693.0999755859375</v>
       </c>
+      <c r="BH14" s="3" t="n">
+        <v>693.0999755859375</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3277,6 +3316,9 @@
       <c r="BG17" s="3" t="n">
         <v>593.5999755859375</v>
       </c>
+      <c r="BH17" s="3" t="n">
+        <v>593.5999755859375</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3458,6 +3500,9 @@
         <v>377.3999938964844</v>
       </c>
       <c r="BG18" s="3" t="n">
+        <v>375.2000122070312</v>
+      </c>
+      <c r="BH18" s="3" t="n">
         <v>375.2000122070312</v>
       </c>
     </row>
@@ -3488,7 +3533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BH41"/>
+  <dimension ref="A1:BI41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3551,6 +3596,7 @@
     <col width="13" customWidth="1" min="58" max="58"/>
     <col width="13" customWidth="1" min="59" max="59"/>
     <col width="13" customWidth="1" min="60" max="60"/>
+    <col width="13" customWidth="1" min="61" max="61"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3854,6 +3900,11 @@
           <t>2026-07-04</t>
         </is>
       </c>
+      <c r="BI1" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -4042,6 +4093,9 @@
       <c r="BH2" s="3" t="n">
         <v>56.762</v>
       </c>
+      <c r="BI2" s="3" t="n">
+        <v>56.762</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4224,6 +4278,9 @@
       <c r="BH3" s="3" t="n">
         <v>25.7336</v>
       </c>
+      <c r="BI3" s="3" t="n">
+        <v>25.7336</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4248,16 +4305,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.18</v>
+        <v>12.37</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>233930.21274</v>
+        <v>237579.37041</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>53930.21274000002</v>
+        <v>57579.37041</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.2996122930000001</v>
+        <v>0.3198853911666667</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -4405,6 +4462,9 @@
       </c>
       <c r="BH4" s="3" t="n">
         <v>12.18</v>
+      </c>
+      <c r="BI4" s="3" t="n">
+        <v>12.37</v>
       </c>
     </row>
     <row r="5">
@@ -4588,6 +4648,9 @@
       <c r="BH5" s="3" t="n">
         <v>9.4689</v>
       </c>
+      <c r="BI5" s="3" t="n">
+        <v>9.4689</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4776,6 +4839,9 @@
       <c r="BH6" s="3" t="n">
         <v>11.9457</v>
       </c>
+      <c r="BI6" s="3" t="n">
+        <v>11.9457</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4958,6 +5024,9 @@
       <c r="BH7" s="3" t="n">
         <v>35.0445</v>
       </c>
+      <c r="BI7" s="3" t="n">
+        <v>35.0445</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5146,6 +5215,9 @@
       <c r="BH8" s="3" t="n">
         <v>33.8955</v>
       </c>
+      <c r="BI8" s="3" t="n">
+        <v>33.8955</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5328,6 +5400,9 @@
       <c r="BH9" s="3" t="n">
         <v>43.3305</v>
       </c>
+      <c r="BI9" s="3" t="n">
+        <v>43.3305</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5510,6 +5585,9 @@
       <c r="BH10" s="3" t="n">
         <v>48.1528</v>
       </c>
+      <c r="BI10" s="3" t="n">
+        <v>48.1528</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5692,6 +5770,9 @@
       <c r="BH11" s="3" t="n">
         <v>104.2946</v>
       </c>
+      <c r="BI11" s="3" t="n">
+        <v>104.2946</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5880,6 +5961,9 @@
       <c r="BH12" s="3" t="n">
         <v>229.594</v>
       </c>
+      <c r="BI12" s="3" t="n">
+        <v>229.594</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6068,6 +6152,9 @@
       <c r="BH13" s="3" t="n">
         <v>21.409</v>
       </c>
+      <c r="BI13" s="3" t="n">
+        <v>21.409</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -6250,6 +6337,9 @@
       <c r="BH14" s="3" t="n">
         <v>38.7629</v>
       </c>
+      <c r="BI14" s="3" t="n">
+        <v>38.7629</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -6438,6 +6528,9 @@
       <c r="BH15" s="3" t="n">
         <v>11.79</v>
       </c>
+      <c r="BI15" s="3" t="n">
+        <v>11.79</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -6620,6 +6713,9 @@
       <c r="BH16" s="3" t="n">
         <v>24.3227</v>
       </c>
+      <c r="BI16" s="3" t="n">
+        <v>24.3227</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -6802,6 +6898,9 @@
       <c r="BH17" s="3" t="n">
         <v>16.8976</v>
       </c>
+      <c r="BI17" s="3" t="n">
+        <v>16.8976</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -6990,6 +7089,9 @@
       <c r="BH18" s="3" t="n">
         <v>47.31</v>
       </c>
+      <c r="BI18" s="3" t="n">
+        <v>47.31</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -7172,6 +7274,9 @@
       <c r="BH19" s="3" t="n">
         <v>14.5742</v>
       </c>
+      <c r="BI19" s="3" t="n">
+        <v>14.5742</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -7360,6 +7465,9 @@
       <c r="BH20" s="3" t="n">
         <v>9.32</v>
       </c>
+      <c r="BI20" s="3" t="n">
+        <v>9.32</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -7548,6 +7656,9 @@
       <c r="BH21" s="3" t="n">
         <v>113.0168</v>
       </c>
+      <c r="BI21" s="3" t="n">
+        <v>113.0168</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -7730,6 +7841,9 @@
       <c r="BH22" s="3" t="n">
         <v>44.15</v>
       </c>
+      <c r="BI22" s="3" t="n">
+        <v>44.15</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -7918,6 +8032,9 @@
       <c r="BH23" s="3" t="n">
         <v>63.8309</v>
       </c>
+      <c r="BI23" s="3" t="n">
+        <v>63.8309</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -8100,6 +8217,9 @@
       <c r="BH24" s="3" t="n">
         <v>27.732</v>
       </c>
+      <c r="BI24" s="3" t="n">
+        <v>27.732</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -8285,6 +8405,9 @@
       <c r="BH25" s="3" t="n">
         <v>11.8619</v>
       </c>
+      <c r="BI25" s="3" t="n">
+        <v>11.8619</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -8470,6 +8593,9 @@
       <c r="BH26" s="3" t="n">
         <v>9.526199999999999</v>
       </c>
+      <c r="BI26" s="3" t="n">
+        <v>9.526199999999999</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -8658,6 +8784,9 @@
       <c r="BH27" s="3" t="n">
         <v>65.61020000000001</v>
       </c>
+      <c r="BI27" s="3" t="n">
+        <v>65.61020000000001</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -8846,6 +8975,9 @@
       <c r="BH28" s="3" t="n">
         <v>110.2185</v>
       </c>
+      <c r="BI28" s="3" t="n">
+        <v>110.2185</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -9028,6 +9160,9 @@
       <c r="BH29" s="3" t="n">
         <v>12.5477</v>
       </c>
+      <c r="BI29" s="3" t="n">
+        <v>12.5477</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -9210,6 +9345,9 @@
       <c r="BH30" s="3" t="n">
         <v>16.7276</v>
       </c>
+      <c r="BI30" s="3" t="n">
+        <v>16.7276</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -9395,6 +9533,9 @@
       <c r="BH31" s="3" t="n">
         <v>417.1665</v>
       </c>
+      <c r="BI31" s="3" t="n">
+        <v>417.1665</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -9583,6 +9724,9 @@
       <c r="BH32" s="3" t="n">
         <v>10.64</v>
       </c>
+      <c r="BI32" s="3" t="n">
+        <v>10.64</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -9765,6 +9909,9 @@
       <c r="BH33" s="3" t="n">
         <v>19</v>
       </c>
+      <c r="BI33" s="3" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -9950,6 +10097,9 @@
       <c r="BH34" s="3" t="n">
         <v>210.8218</v>
       </c>
+      <c r="BI34" s="3" t="n">
+        <v>210.8218</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -10135,6 +10285,9 @@
       <c r="BH35" s="3" t="n">
         <v>14.83</v>
       </c>
+      <c r="BI35" s="3" t="n">
+        <v>14.83</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -10320,6 +10473,9 @@
       <c r="BH36" s="3" t="n">
         <v>374.9716</v>
       </c>
+      <c r="BI36" s="3" t="n">
+        <v>374.9716</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -10505,6 +10661,9 @@
       <c r="BH37" s="3" t="n">
         <v>16.901</v>
       </c>
+      <c r="BI37" s="3" t="n">
+        <v>16.901</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -10687,6 +10846,9 @@
       <c r="BH38" s="3" t="n">
         <v>14.3909</v>
       </c>
+      <c r="BI38" s="3" t="n">
+        <v>14.3909</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -10869,6 +11031,9 @@
       <c r="BH39" s="3" t="n">
         <v>1022.3097</v>
       </c>
+      <c r="BI39" s="3" t="n">
+        <v>1022.3097</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -11054,6 +11219,9 @@
       <c r="BH40" s="3" t="n">
         <v>21.744</v>
       </c>
+      <c r="BI40" s="3" t="n">
+        <v>21.744</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
@@ -11065,13 +11233,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4979687.3004521</v>
+        <v>4983336.4581221</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>509687.3004521001</v>
+        <v>513336.4581221001</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1140240045754139</v>
+        <v>0.1148403709445414</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-07-06
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-05 06:03 IST</t>
+          <t>Generated: 2026-07-06 06:26 IST</t>
         </is>
       </c>
     </row>
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>544721.5007858276</v>
+        <v>542757.4957733154</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-46060.51921417238</v>
+        <v>-48024.52422668459</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.07796533688376701</v>
+        <v>-0.08128975256674972</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5528057.958907927</v>
+        <v>5526093.953895415</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>467275.9389079278</v>
+        <v>465311.9338954156</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.09233275352727559</v>
+        <v>0.09194467022221511</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-07-05</t>
+          <t>Last snapshot: 2026-07-06</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BH19"/>
+  <dimension ref="A1:BI19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -679,6 +679,7 @@
     <col width="21" customWidth="1" min="58" max="58"/>
     <col width="21" customWidth="1" min="59" max="59"/>
     <col width="21" customWidth="1" min="60" max="60"/>
+    <col width="21" customWidth="1" min="61" max="61"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -982,6 +983,11 @@
           <t>2026-07-05</t>
         </is>
       </c>
+      <c r="BI1" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1001,13 +1007,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>540.9000244140625</v>
+        <v>534.0499877929688</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>43272.001953125</v>
+        <v>42723.9990234375</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>-545.508046875002</v>
+        <v>-1093.510976562502</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1164,6 +1170,9 @@
       </c>
       <c r="BH2" s="3" t="n">
         <v>540.9000244140625</v>
+      </c>
+      <c r="BI2" s="3" t="n">
+        <v>534.0499877929688</v>
       </c>
     </row>
     <row r="3">
@@ -1211,13 +1220,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1385</v>
+        <v>1383.199951171875</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>27700</v>
+        <v>27663.9990234375</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-4404.580000000002</v>
+        <v>-4440.580976562502</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1377,6 +1386,9 @@
       </c>
       <c r="BH4" s="3" t="n">
         <v>1385</v>
+      </c>
+      <c r="BI4" s="3" t="n">
+        <v>1383.199951171875</v>
       </c>
     </row>
     <row r="5">
@@ -1397,13 +1409,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>662.2000122070312</v>
+        <v>653.6500244140625</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13244.00024414062</v>
+        <v>13073.00048828125</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-969.0997558593754</v>
+        <v>-1140.09951171875</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1563,6 +1575,9 @@
       </c>
       <c r="BH5" s="3" t="n">
         <v>662.2000122070312</v>
+      </c>
+      <c r="BI5" s="3" t="n">
+        <v>653.6500244140625</v>
       </c>
     </row>
     <row r="6">
@@ -1583,13 +1598,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>366.8500061035156</v>
+        <v>368.7999877929688</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>14674.00024414062</v>
+        <v>14751.99951171875</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2828.239755859377</v>
+        <v>-2750.240488281252</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1749,6 +1764,9 @@
       </c>
       <c r="BH6" s="3" t="n">
         <v>366.8500061035156</v>
+      </c>
+      <c r="BI6" s="3" t="n">
+        <v>368.7999877929688</v>
       </c>
     </row>
     <row r="7">
@@ -1769,13 +1787,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>237.4900054931641</v>
+        <v>243.0099945068359</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>23749.00054931641</v>
+        <v>24300.99945068359</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-2684.819450683593</v>
+        <v>-2132.820549316406</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1935,6 +1953,9 @@
       </c>
       <c r="BH7" s="3" t="n">
         <v>237.4900054931641</v>
+      </c>
+      <c r="BI7" s="3" t="n">
+        <v>243.0099945068359</v>
       </c>
     </row>
     <row r="8">
@@ -1982,13 +2003,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>17.79999923706055</v>
+        <v>17.73999977111816</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>26699.99885559082</v>
+        <v>26609.99965667725</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-4350.171144409178</v>
+        <v>-4440.170343322752</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -2148,6 +2169,9 @@
       </c>
       <c r="BH9" s="3" t="n">
         <v>17.79999923706055</v>
+      </c>
+      <c r="BI9" s="3" t="n">
+        <v>17.73999977111816</v>
       </c>
     </row>
     <row r="10">
@@ -2168,13 +2192,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>422.1000061035156</v>
+        <v>423.0499877929688</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>42210.00061035156</v>
+        <v>42304.99877929688</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-9288.479389648441</v>
+        <v>-9193.481220703128</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -2334,6 +2358,9 @@
       </c>
       <c r="BH10" s="3" t="n">
         <v>422.1000061035156</v>
+      </c>
+      <c r="BI10" s="3" t="n">
+        <v>423.0499877929688</v>
       </c>
     </row>
     <row r="11">
@@ -2354,13 +2381,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>10.30000019073486</v>
+        <v>9.470000267028809</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>10300.00019073486</v>
-      </c>
-      <c r="G11" s="4" t="n">
-        <v>458.7901907348642</v>
+        <v>9470.000267028809</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>-371.2097329711905</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -2520,6 +2547,9 @@
       </c>
       <c r="BH11" s="3" t="n">
         <v>10.30000019073486</v>
+      </c>
+      <c r="BI11" s="3" t="n">
+        <v>9.470000267028809</v>
       </c>
     </row>
     <row r="12">
@@ -2540,13 +2570,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2512.5</v>
+        <v>2566.39990234375</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25125</v>
+        <v>25663.9990234375</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2598.25</v>
+        <v>-2059.2509765625</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -2706,6 +2736,9 @@
       </c>
       <c r="BH12" s="3" t="n">
         <v>2512.5</v>
+      </c>
+      <c r="BI12" s="3" t="n">
+        <v>2566.39990234375</v>
       </c>
     </row>
     <row r="13">
@@ -2726,13 +2759,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>56.86999893188477</v>
+        <v>55.54000091552734</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>34121.99935913086</v>
+        <v>33324.00054931641</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-909.7606408691427</v>
+        <v>-1707.759450683596</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -2892,6 +2925,9 @@
       </c>
       <c r="BH13" s="3" t="n">
         <v>56.86999893188477</v>
+      </c>
+      <c r="BI13" s="3" t="n">
+        <v>55.54000091552734</v>
       </c>
     </row>
     <row r="14">
@@ -2912,13 +2948,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>693.0999755859375</v>
+        <v>690.9000244140625</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>34654.99877929688</v>
+        <v>34545.00122070312</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-7807.511220703127</v>
+        <v>-7917.508779296877</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -3078,6 +3114,9 @@
       </c>
       <c r="BH14" s="3" t="n">
         <v>693.0999755859375</v>
+      </c>
+      <c r="BI14" s="3" t="n">
+        <v>690.9000244140625</v>
       </c>
     </row>
     <row r="15">
@@ -3152,13 +3191,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>593.5999755859375</v>
+        <v>576</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>29679.99877929688</v>
+        <v>28800</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>7925.468779296876</v>
+        <v>7045.470000000001</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -3318,6 +3357,9 @@
       </c>
       <c r="BH17" s="3" t="n">
         <v>593.5999755859375</v>
+      </c>
+      <c r="BI17" s="3" t="n">
+        <v>576</v>
       </c>
     </row>
     <row r="18">
@@ -3338,13 +3380,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>375.2000122070312</v>
+        <v>377.5499877929688</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>37520.00122070312</v>
+        <v>37754.99877929688</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-9120.818779296875</v>
+        <v>-8885.821220703125</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -3504,6 +3546,9 @@
       </c>
       <c r="BH18" s="3" t="n">
         <v>375.2000122070312</v>
+      </c>
+      <c r="BI18" s="3" t="n">
+        <v>377.5499877929688</v>
       </c>
     </row>
     <row r="19">
@@ -3516,10 +3561,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>544721.5007858276</v>
+        <v>542757.4957733154</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-46060.51921417237</v>
+        <v>-48024.52422668458</v>
       </c>
     </row>
   </sheetData>
@@ -3533,7 +3578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BI41"/>
+  <dimension ref="A1:BJ41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3597,6 +3642,7 @@
     <col width="13" customWidth="1" min="59" max="59"/>
     <col width="13" customWidth="1" min="60" max="60"/>
     <col width="13" customWidth="1" min="61" max="61"/>
+    <col width="13" customWidth="1" min="62" max="62"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3905,6 +3951,11 @@
           <t>2026-07-05</t>
         </is>
       </c>
+      <c r="BJ1" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -4096,6 +4147,9 @@
       <c r="BI2" s="3" t="n">
         <v>56.762</v>
       </c>
+      <c r="BJ2" s="3" t="n">
+        <v>56.762</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4281,6 +4335,9 @@
       <c r="BI3" s="3" t="n">
         <v>25.7336</v>
       </c>
+      <c r="BJ3" s="3" t="n">
+        <v>25.7336</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4466,6 +4523,9 @@
       <c r="BI4" s="3" t="n">
         <v>12.37</v>
       </c>
+      <c r="BJ4" s="3" t="n">
+        <v>12.37</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4651,6 +4711,9 @@
       <c r="BI5" s="3" t="n">
         <v>9.4689</v>
       </c>
+      <c r="BJ5" s="3" t="n">
+        <v>9.4689</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4842,6 +4905,9 @@
       <c r="BI6" s="3" t="n">
         <v>11.9457</v>
       </c>
+      <c r="BJ6" s="3" t="n">
+        <v>11.9457</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -5027,6 +5093,9 @@
       <c r="BI7" s="3" t="n">
         <v>35.0445</v>
       </c>
+      <c r="BJ7" s="3" t="n">
+        <v>35.0445</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5218,6 +5287,9 @@
       <c r="BI8" s="3" t="n">
         <v>33.8955</v>
       </c>
+      <c r="BJ8" s="3" t="n">
+        <v>33.8955</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5403,6 +5475,9 @@
       <c r="BI9" s="3" t="n">
         <v>43.3305</v>
       </c>
+      <c r="BJ9" s="3" t="n">
+        <v>43.3305</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5588,6 +5663,9 @@
       <c r="BI10" s="3" t="n">
         <v>48.1528</v>
       </c>
+      <c r="BJ10" s="3" t="n">
+        <v>48.1528</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5773,6 +5851,9 @@
       <c r="BI11" s="3" t="n">
         <v>104.2946</v>
       </c>
+      <c r="BJ11" s="3" t="n">
+        <v>104.2946</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5964,6 +6045,9 @@
       <c r="BI12" s="3" t="n">
         <v>229.594</v>
       </c>
+      <c r="BJ12" s="3" t="n">
+        <v>229.594</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6155,6 +6239,9 @@
       <c r="BI13" s="3" t="n">
         <v>21.409</v>
       </c>
+      <c r="BJ13" s="3" t="n">
+        <v>21.409</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -6340,6 +6427,9 @@
       <c r="BI14" s="3" t="n">
         <v>38.7629</v>
       </c>
+      <c r="BJ14" s="3" t="n">
+        <v>38.7629</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -6531,6 +6621,9 @@
       <c r="BI15" s="3" t="n">
         <v>11.79</v>
       </c>
+      <c r="BJ15" s="3" t="n">
+        <v>11.79</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -6716,6 +6809,9 @@
       <c r="BI16" s="3" t="n">
         <v>24.3227</v>
       </c>
+      <c r="BJ16" s="3" t="n">
+        <v>24.3227</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -6901,6 +6997,9 @@
       <c r="BI17" s="3" t="n">
         <v>16.8976</v>
       </c>
+      <c r="BJ17" s="3" t="n">
+        <v>16.8976</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -7092,6 +7191,9 @@
       <c r="BI18" s="3" t="n">
         <v>47.31</v>
       </c>
+      <c r="BJ18" s="3" t="n">
+        <v>47.31</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -7277,6 +7379,9 @@
       <c r="BI19" s="3" t="n">
         <v>14.5742</v>
       </c>
+      <c r="BJ19" s="3" t="n">
+        <v>14.5742</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -7468,6 +7573,9 @@
       <c r="BI20" s="3" t="n">
         <v>9.32</v>
       </c>
+      <c r="BJ20" s="3" t="n">
+        <v>9.32</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -7659,6 +7767,9 @@
       <c r="BI21" s="3" t="n">
         <v>113.0168</v>
       </c>
+      <c r="BJ21" s="3" t="n">
+        <v>113.0168</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -7844,6 +7955,9 @@
       <c r="BI22" s="3" t="n">
         <v>44.15</v>
       </c>
+      <c r="BJ22" s="3" t="n">
+        <v>44.15</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -8035,6 +8149,9 @@
       <c r="BI23" s="3" t="n">
         <v>63.8309</v>
       </c>
+      <c r="BJ23" s="3" t="n">
+        <v>63.8309</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -8220,6 +8337,9 @@
       <c r="BI24" s="3" t="n">
         <v>27.732</v>
       </c>
+      <c r="BJ24" s="3" t="n">
+        <v>27.732</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -8408,6 +8528,9 @@
       <c r="BI25" s="3" t="n">
         <v>11.8619</v>
       </c>
+      <c r="BJ25" s="3" t="n">
+        <v>11.8619</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -8596,6 +8719,9 @@
       <c r="BI26" s="3" t="n">
         <v>9.526199999999999</v>
       </c>
+      <c r="BJ26" s="3" t="n">
+        <v>9.526199999999999</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -8787,6 +8913,9 @@
       <c r="BI27" s="3" t="n">
         <v>65.61020000000001</v>
       </c>
+      <c r="BJ27" s="3" t="n">
+        <v>65.61020000000001</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -8978,6 +9107,9 @@
       <c r="BI28" s="3" t="n">
         <v>110.2185</v>
       </c>
+      <c r="BJ28" s="3" t="n">
+        <v>110.2185</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -9163,6 +9295,9 @@
       <c r="BI29" s="3" t="n">
         <v>12.5477</v>
       </c>
+      <c r="BJ29" s="3" t="n">
+        <v>12.5477</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -9348,6 +9483,9 @@
       <c r="BI30" s="3" t="n">
         <v>16.7276</v>
       </c>
+      <c r="BJ30" s="3" t="n">
+        <v>16.7276</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -9536,6 +9674,9 @@
       <c r="BI31" s="3" t="n">
         <v>417.1665</v>
       </c>
+      <c r="BJ31" s="3" t="n">
+        <v>417.1665</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -9727,6 +9868,9 @@
       <c r="BI32" s="3" t="n">
         <v>10.64</v>
       </c>
+      <c r="BJ32" s="3" t="n">
+        <v>10.64</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -9912,6 +10056,9 @@
       <c r="BI33" s="3" t="n">
         <v>19</v>
       </c>
+      <c r="BJ33" s="3" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -10100,6 +10247,9 @@
       <c r="BI34" s="3" t="n">
         <v>210.8218</v>
       </c>
+      <c r="BJ34" s="3" t="n">
+        <v>210.8218</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -10288,6 +10438,9 @@
       <c r="BI35" s="3" t="n">
         <v>14.83</v>
       </c>
+      <c r="BJ35" s="3" t="n">
+        <v>14.83</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -10476,6 +10629,9 @@
       <c r="BI36" s="3" t="n">
         <v>374.9716</v>
       </c>
+      <c r="BJ36" s="3" t="n">
+        <v>374.9716</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -10664,6 +10820,9 @@
       <c r="BI37" s="3" t="n">
         <v>16.901</v>
       </c>
+      <c r="BJ37" s="3" t="n">
+        <v>16.901</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -10849,6 +11008,9 @@
       <c r="BI38" s="3" t="n">
         <v>14.3909</v>
       </c>
+      <c r="BJ38" s="3" t="n">
+        <v>14.3909</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -11034,6 +11196,9 @@
       <c r="BI39" s="3" t="n">
         <v>1022.3097</v>
       </c>
+      <c r="BJ39" s="3" t="n">
+        <v>1022.3097</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -11220,6 +11385,9 @@
         <v>21.744</v>
       </c>
       <c r="BI40" s="3" t="n">
+        <v>21.744</v>
+      </c>
+      <c r="BJ40" s="3" t="n">
         <v>21.744</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily portfolio update 2026-07-07
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -485,7 +485,7 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-06 06:26 IST</t>
+          <t>Generated: 2026-07-07 06:05 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4983336.4581221</v>
+        <v>4989918.8116697</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>513336.4581220997</v>
+        <v>519918.8116696998</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1148403709445413</v>
+        <v>0.1163129332594407</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>542757.4957733154</v>
+        <v>540070.0023727417</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-48024.52422668459</v>
+        <v>-50712.01762725832</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.08128975256674972</v>
+        <v>-0.08583879656198461</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5526093.953895415</v>
+        <v>5529988.814042442</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>465311.9338954156</v>
+        <v>469206.794042442</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.09194467022221511</v>
+        <v>0.09271428648540014</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-07-06</t>
+          <t>Last snapshot: 2026-07-07</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BI19"/>
+  <dimension ref="A1:BJ19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -680,6 +680,7 @@
     <col width="21" customWidth="1" min="59" max="59"/>
     <col width="21" customWidth="1" min="60" max="60"/>
     <col width="21" customWidth="1" min="61" max="61"/>
+    <col width="21" customWidth="1" min="62" max="62"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -988,6 +989,11 @@
           <t>2026-07-06</t>
         </is>
       </c>
+      <c r="BJ1" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1007,13 +1013,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>534.0499877929688</v>
+        <v>533.7000122070312</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>42723.9990234375</v>
+        <v>42696.0009765625</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>-1093.510976562502</v>
+        <v>-1121.509023437502</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1173,6 +1179,9 @@
       </c>
       <c r="BI2" s="3" t="n">
         <v>534.0499877929688</v>
+      </c>
+      <c r="BJ2" s="3" t="n">
+        <v>533.7000122070312</v>
       </c>
     </row>
     <row r="3">
@@ -1220,13 +1229,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1383.199951171875</v>
+        <v>1363.599975585938</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>27663.9990234375</v>
+        <v>27271.99951171875</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-4440.580976562502</v>
+        <v>-4832.580488281252</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1389,6 +1398,9 @@
       </c>
       <c r="BI4" s="3" t="n">
         <v>1383.199951171875</v>
+      </c>
+      <c r="BJ4" s="3" t="n">
+        <v>1363.599975585938</v>
       </c>
     </row>
     <row r="5">
@@ -1409,13 +1421,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>653.6500244140625</v>
+        <v>651.0499877929688</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13073.00048828125</v>
+        <v>13020.99975585938</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1140.09951171875</v>
+        <v>-1192.100244140625</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1578,6 +1590,9 @@
       </c>
       <c r="BI5" s="3" t="n">
         <v>653.6500244140625</v>
+      </c>
+      <c r="BJ5" s="3" t="n">
+        <v>651.0499877929688</v>
       </c>
     </row>
     <row r="6">
@@ -1598,13 +1613,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>368.7999877929688</v>
+        <v>366.2999877929688</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>14751.99951171875</v>
+        <v>14651.99951171875</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2750.240488281252</v>
+        <v>-2850.240488281252</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1767,6 +1782,9 @@
       </c>
       <c r="BI6" s="3" t="n">
         <v>368.7999877929688</v>
+      </c>
+      <c r="BJ6" s="3" t="n">
+        <v>366.2999877929688</v>
       </c>
     </row>
     <row r="7">
@@ -1787,13 +1805,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>243.0099945068359</v>
+        <v>239.6199951171875</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>24300.99945068359</v>
+        <v>23961.99951171875</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-2132.820549316406</v>
+        <v>-2471.82048828125</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1956,6 +1974,9 @@
       </c>
       <c r="BI7" s="3" t="n">
         <v>243.0099945068359</v>
+      </c>
+      <c r="BJ7" s="3" t="n">
+        <v>239.6199951171875</v>
       </c>
     </row>
     <row r="8">
@@ -2003,13 +2024,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>17.73999977111816</v>
+        <v>17.39999961853027</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>26609.99965667725</v>
+        <v>26099.99942779541</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-4440.170343322752</v>
+        <v>-4950.170572204588</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -2172,6 +2193,9 @@
       </c>
       <c r="BI9" s="3" t="n">
         <v>17.73999977111816</v>
+      </c>
+      <c r="BJ9" s="3" t="n">
+        <v>17.39999961853027</v>
       </c>
     </row>
     <row r="10">
@@ -2192,13 +2216,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>423.0499877929688</v>
+        <v>422.8500061035156</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>42304.99877929688</v>
+        <v>42285.00061035156</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-9193.481220703128</v>
+        <v>-9213.479389648441</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -2361,6 +2385,9 @@
       </c>
       <c r="BI10" s="3" t="n">
         <v>423.0499877929688</v>
+      </c>
+      <c r="BJ10" s="3" t="n">
+        <v>422.8500061035156</v>
       </c>
     </row>
     <row r="11">
@@ -2381,13 +2408,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>9.470000267028809</v>
+        <v>9.239999771118164</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>9470.000267028809</v>
+        <v>9239.999771118164</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-371.2097329711905</v>
+        <v>-601.2102288818351</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -2550,6 +2577,9 @@
       </c>
       <c r="BI11" s="3" t="n">
         <v>9.470000267028809</v>
+      </c>
+      <c r="BJ11" s="3" t="n">
+        <v>9.239999771118164</v>
       </c>
     </row>
     <row r="12">
@@ -2570,13 +2600,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2566.39990234375</v>
+        <v>2610.300048828125</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>25663.9990234375</v>
+        <v>26103.00048828125</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-2059.2509765625</v>
+        <v>-1620.24951171875</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -2739,6 +2769,9 @@
       </c>
       <c r="BI12" s="3" t="n">
         <v>2566.39990234375</v>
+      </c>
+      <c r="BJ12" s="3" t="n">
+        <v>2610.300048828125</v>
       </c>
     </row>
     <row r="13">
@@ -2759,13 +2792,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>55.54000091552734</v>
+        <v>54.61000061035156</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>33324.00054931641</v>
+        <v>32766.00036621094</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-1707.759450683596</v>
+        <v>-2265.759633789065</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -2928,6 +2961,9 @@
       </c>
       <c r="BI13" s="3" t="n">
         <v>55.54000091552734</v>
+      </c>
+      <c r="BJ13" s="3" t="n">
+        <v>54.61000061035156</v>
       </c>
     </row>
     <row r="14">
@@ -2948,13 +2984,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>690.9000244140625</v>
+        <v>704.7000122070312</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>34545.00122070312</v>
+        <v>35235.00061035156</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-7917.508779296877</v>
+        <v>-7227.50938964844</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -3117,6 +3153,9 @@
       </c>
       <c r="BI14" s="3" t="n">
         <v>690.9000244140625</v>
+      </c>
+      <c r="BJ14" s="3" t="n">
+        <v>704.7000122070312</v>
       </c>
     </row>
     <row r="15">
@@ -3191,13 +3230,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>576</v>
+        <v>547.9500122070312</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>28800</v>
+        <v>27397.50061035156</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>7045.470000000001</v>
+        <v>5642.970610351564</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -3360,6 +3399,9 @@
       </c>
       <c r="BI17" s="3" t="n">
         <v>576</v>
+      </c>
+      <c r="BJ17" s="3" t="n">
+        <v>547.9500122070312</v>
       </c>
     </row>
     <row r="18">
@@ -3380,13 +3422,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>377.5499877929688</v>
+        <v>375.7000122070312</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>37754.99877929688</v>
+        <v>37570.00122070312</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-8885.821220703125</v>
+        <v>-9070.818779296875</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -3549,6 +3591,9 @@
       </c>
       <c r="BI18" s="3" t="n">
         <v>377.5499877929688</v>
+      </c>
+      <c r="BJ18" s="3" t="n">
+        <v>375.7000122070312</v>
       </c>
     </row>
     <row r="19">
@@ -3561,10 +3606,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>542757.4957733154</v>
+        <v>540070.0023727417</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-48024.52422668458</v>
+        <v>-50712.01762725831</v>
       </c>
     </row>
   </sheetData>
@@ -3578,7 +3623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BJ41"/>
+  <dimension ref="A1:BK41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3643,6 +3688,7 @@
     <col width="13" customWidth="1" min="60" max="60"/>
     <col width="13" customWidth="1" min="61" max="61"/>
     <col width="13" customWidth="1" min="62" max="62"/>
+    <col width="13" customWidth="1" min="63" max="63"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3956,6 +4002,11 @@
           <t>2026-07-06</t>
         </is>
       </c>
+      <c r="BK1" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3980,16 +4031,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.762</v>
+        <v>57.3631</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>63714.323284</v>
+        <v>64389.0472142</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>13714.323284</v>
+        <v>14389.0472142</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.27428646568</v>
+        <v>0.287780944284</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -4149,6 +4200,9 @@
       </c>
       <c r="BJ2" s="3" t="n">
         <v>56.762</v>
+      </c>
+      <c r="BK2" s="3" t="n">
+        <v>57.3631</v>
       </c>
     </row>
     <row r="3">
@@ -4174,16 +4228,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.7336</v>
+        <v>25.7229</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>63181.4692568</v>
+        <v>63155.1984777</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>3181.469256800003</v>
+        <v>3155.198477700003</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.05302448761333338</v>
+        <v>0.05258664129500006</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -4337,6 +4391,9 @@
       </c>
       <c r="BJ3" s="3" t="n">
         <v>25.7336</v>
+      </c>
+      <c r="BK3" s="3" t="n">
+        <v>25.7229</v>
       </c>
     </row>
     <row r="4">
@@ -4362,16 +4419,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.37</v>
+        <v>12.3</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>237579.37041</v>
+        <v>236234.9439</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>57579.37041</v>
+        <v>56234.94390000001</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3198853911666667</v>
+        <v>0.3124163550000001</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -4525,6 +4582,9 @@
       </c>
       <c r="BJ4" s="3" t="n">
         <v>12.37</v>
+      </c>
+      <c r="BK4" s="3" t="n">
+        <v>12.3</v>
       </c>
     </row>
     <row r="5">
@@ -4550,16 +4610,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.4689</v>
+        <v>9.519299999999999</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>173793.0238632</v>
+        <v>174718.0698984</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-36206.97613680002</v>
+        <v>-35281.93010160001</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1724141720800001</v>
+        <v>-0.1680091909600001</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -4713,6 +4773,9 @@
       </c>
       <c r="BJ5" s="3" t="n">
         <v>9.4689</v>
+      </c>
+      <c r="BK5" s="3" t="n">
+        <v>9.519299999999999</v>
       </c>
     </row>
     <row r="6">
@@ -4738,16 +4801,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>11.9457</v>
+        <v>12.008</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>50518.0905489</v>
+        <v>50781.55581599999</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>518.0905488999997</v>
+        <v>781.5558159999928</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.01036181097799999</v>
+        <v>0.01563111631999986</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -4907,6 +4970,9 @@
       </c>
       <c r="BJ6" s="3" t="n">
         <v>11.9457</v>
+      </c>
+      <c r="BK6" s="3" t="n">
+        <v>12.008</v>
       </c>
     </row>
     <row r="7">
@@ -4932,16 +4998,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>35.0445</v>
+        <v>34.8705</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>77309.56878</v>
+        <v>76925.71782000001</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>17309.56878</v>
+        <v>16925.71782000001</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.288492813</v>
+        <v>0.2820952970000001</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -5095,6 +5161,9 @@
       </c>
       <c r="BJ7" s="3" t="n">
         <v>35.0445</v>
+      </c>
+      <c r="BK7" s="3" t="n">
+        <v>34.8705</v>
       </c>
     </row>
     <row r="8">
@@ -5120,16 +5189,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>33.8955</v>
+        <v>33.7515</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>54388.4820315</v>
+        <v>54157.4206395</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>4388.482031500003</v>
+        <v>4157.4206395</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.08776964063000006</v>
+        <v>0.08314841279</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -5289,6 +5358,9 @@
       </c>
       <c r="BJ8" s="3" t="n">
         <v>33.8955</v>
+      </c>
+      <c r="BK8" s="3" t="n">
+        <v>33.7515</v>
       </c>
     </row>
     <row r="9">
@@ -5314,16 +5386,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>43.3305</v>
+        <v>42.5258</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>139497.9083865</v>
+        <v>136907.2628394</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>39497.9083865</v>
+        <v>36907.26283939998</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.394979083865</v>
+        <v>0.3690726283939998</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -5477,6 +5549,9 @@
       </c>
       <c r="BJ9" s="3" t="n">
         <v>43.3305</v>
+      </c>
+      <c r="BK9" s="3" t="n">
+        <v>42.5258</v>
       </c>
     </row>
     <row r="10">
@@ -5502,16 +5577,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48.1528</v>
+        <v>48.2855</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>137074.6014952</v>
+        <v>137452.3531445</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>37074.60149520001</v>
+        <v>37452.3531445</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3707460149520001</v>
+        <v>0.3745235314449999</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -5665,6 +5740,9 @@
       </c>
       <c r="BJ10" s="3" t="n">
         <v>48.1528</v>
+      </c>
+      <c r="BK10" s="3" t="n">
+        <v>48.2855</v>
       </c>
     </row>
     <row r="11">
@@ -5690,16 +5768,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>104.2946</v>
+        <v>105.6646</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31384.2267374</v>
+        <v>31796.4857674</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1384.2267374</v>
+        <v>1796.485767399998</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.04614089124666668</v>
+        <v>0.05988285891333326</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -5853,6 +5931,9 @@
       </c>
       <c r="BJ11" s="3" t="n">
         <v>104.2946</v>
+      </c>
+      <c r="BK11" s="3" t="n">
+        <v>105.6646</v>
       </c>
     </row>
     <row r="12">
@@ -5878,16 +5959,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>229.594</v>
+        <v>230.395</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>106881.058068</v>
+        <v>107253.94119</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>6881.058067999998</v>
+        <v>7253.941189999998</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.06881058067999998</v>
+        <v>0.07253941189999998</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -6047,6 +6128,9 @@
       </c>
       <c r="BJ12" s="3" t="n">
         <v>229.594</v>
+      </c>
+      <c r="BK12" s="3" t="n">
+        <v>230.395</v>
       </c>
     </row>
     <row r="13">
@@ -6072,16 +6156,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>21.409</v>
+        <v>21.389</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>248079.035445</v>
+        <v>247847.283345</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>48079.03544499999</v>
+        <v>47847.28334499997</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.2403951772249999</v>
+        <v>0.2392364167249999</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -6241,6 +6325,9 @@
       </c>
       <c r="BJ13" s="3" t="n">
         <v>21.409</v>
+      </c>
+      <c r="BK13" s="3" t="n">
+        <v>21.389</v>
       </c>
     </row>
     <row r="14">
@@ -6266,16 +6353,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>38.7629</v>
+        <v>38.8716</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>139841.2706174</v>
+        <v>140233.4173896</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>39841.2706174</v>
+        <v>40233.41738960001</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.398412706174</v>
+        <v>0.4023341738960001</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -6429,6 +6516,9 @@
       </c>
       <c r="BJ14" s="3" t="n">
         <v>38.7629</v>
+      </c>
+      <c r="BK14" s="3" t="n">
+        <v>38.8716</v>
       </c>
     </row>
     <row r="15">
@@ -6454,16 +6544,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.79</v>
+        <v>11.86</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>114881.13513</v>
+        <v>115563.21142</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>14881.13513</v>
+        <v>15563.21141999999</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1488113512999999</v>
+        <v>0.1556321141999999</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -6623,6 +6713,9 @@
       </c>
       <c r="BJ15" s="3" t="n">
         <v>11.79</v>
+      </c>
+      <c r="BK15" s="3" t="n">
+        <v>11.86</v>
       </c>
     </row>
     <row r="16">
@@ -6648,16 +6741,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.3227</v>
+        <v>24.6581</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>139197.0608656</v>
+        <v>141116.5309168</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>39197.06086560001</v>
+        <v>41116.53091679999</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.3919706086560001</v>
+        <v>0.4111653091679999</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -6811,6 +6904,9 @@
       </c>
       <c r="BJ16" s="3" t="n">
         <v>24.3227</v>
+      </c>
+      <c r="BK16" s="3" t="n">
+        <v>24.6581</v>
       </c>
     </row>
     <row r="17">
@@ -6836,16 +6932,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.8976</v>
+        <v>17.0198</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55864.4287632</v>
+        <v>56268.4289286</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5864.428763199998</v>
+        <v>6268.428928599998</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.117288575264</v>
+        <v>0.125368578572</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -6999,6 +7095,9 @@
       </c>
       <c r="BJ17" s="3" t="n">
         <v>16.8976</v>
+      </c>
+      <c r="BK17" s="3" t="n">
+        <v>17.0198</v>
       </c>
     </row>
     <row r="18">
@@ -7024,16 +7123,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>47.31</v>
+        <v>47.33</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>89247.28716000001</v>
+        <v>89285.01587999999</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>9247.287160000007</v>
+        <v>9285.015879999992</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.1155910895000001</v>
+        <v>0.1160626984999999</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -7193,6 +7292,9 @@
       </c>
       <c r="BJ18" s="3" t="n">
         <v>47.31</v>
+      </c>
+      <c r="BK18" s="3" t="n">
+        <v>47.33</v>
       </c>
     </row>
     <row r="19">
@@ -7218,16 +7320,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>14.5742</v>
+        <v>14.1948</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>210841.5410372</v>
+        <v>205352.8500168</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>60841.54103719999</v>
+        <v>55352.85001680002</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.4056102735813333</v>
+        <v>0.3690190001120001</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -7381,6 +7483,9 @@
       </c>
       <c r="BJ19" s="3" t="n">
         <v>14.5742</v>
+      </c>
+      <c r="BK19" s="3" t="n">
+        <v>14.1948</v>
       </c>
     </row>
     <row r="20">
@@ -7406,16 +7511,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.32</v>
+        <v>9.34</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>244704.08396</v>
+        <v>245229.20002</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-5295.916039999982</v>
+        <v>-4770.799980000011</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.02118366415999993</v>
+        <v>-0.01908319992000004</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -7575,6 +7680,9 @@
       </c>
       <c r="BJ20" s="3" t="n">
         <v>9.32</v>
+      </c>
+      <c r="BK20" s="3" t="n">
+        <v>9.34</v>
       </c>
     </row>
     <row r="21">
@@ -7600,16 +7708,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>113.0168</v>
+        <v>113.3446</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>171701.7905512</v>
+        <v>172199.8036514</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>1701.790551200014</v>
+        <v>2199.803651399998</v>
       </c>
       <c r="I21" s="12" t="n">
-        <v>0.01001053265411773</v>
+        <v>0.01294002147882352</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -7769,6 +7877,9 @@
       </c>
       <c r="BJ21" s="3" t="n">
         <v>113.0168</v>
+      </c>
+      <c r="BK21" s="3" t="n">
+        <v>113.3446</v>
       </c>
     </row>
     <row r="22">
@@ -7794,16 +7905,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>44.15</v>
+        <v>44.183</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>67746.409</v>
+        <v>67797.04618</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>7746.409</v>
+        <v>7797.046180000005</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1291068166666667</v>
+        <v>0.1299507696666667</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -7957,6 +8068,9 @@
       </c>
       <c r="BJ22" s="3" t="n">
         <v>44.15</v>
+      </c>
+      <c r="BK22" s="3" t="n">
+        <v>44.183</v>
       </c>
     </row>
     <row r="23">
@@ -7982,16 +8096,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>63.8309</v>
+        <v>64.0916</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>173394.5334303</v>
+        <v>174102.7163772</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>23394.53343030001</v>
+        <v>24102.71637720001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.1559635562020001</v>
+        <v>0.160684775848</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -8151,6 +8265,9 @@
       </c>
       <c r="BJ23" s="3" t="n">
         <v>63.8309</v>
+      </c>
+      <c r="BK23" s="3" t="n">
+        <v>64.0916</v>
       </c>
     </row>
     <row r="24">
@@ -8176,16 +8293,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>27.732</v>
+        <v>27.7996</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>100761.060552</v>
+        <v>101006.6774456</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>761.0605519999954</v>
+        <v>1006.677445599998</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.007610605519999954</v>
+        <v>0.01006677445599998</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -8339,6 +8456,9 @@
       </c>
       <c r="BJ24" s="3" t="n">
         <v>27.732</v>
+      </c>
+      <c r="BK24" s="3" t="n">
+        <v>27.7996</v>
       </c>
     </row>
     <row r="25">
@@ -8364,16 +8484,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.8619</v>
+        <v>11.9148</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>194792.2548206</v>
+        <v>195660.9613752</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-5207.745179399994</v>
+        <v>-4339.038624800014</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.02603872589699997</v>
+        <v>-0.02169519312400007</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -8530,6 +8650,9 @@
       </c>
       <c r="BJ25" s="3" t="n">
         <v>11.8619</v>
+      </c>
+      <c r="BK25" s="3" t="n">
+        <v>11.9148</v>
       </c>
     </row>
     <row r="26">
@@ -8555,16 +8678,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>9.526199999999999</v>
+        <v>9.4506</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>113759.165433</v>
+        <v>112856.371779</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>3759.165432999987</v>
+        <v>2856.371778999994</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.03417423120909079</v>
+        <v>0.02596701617272722</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -8721,6 +8844,9 @@
       </c>
       <c r="BJ26" s="3" t="n">
         <v>9.526199999999999</v>
+      </c>
+      <c r="BK26" s="3" t="n">
+        <v>9.4506</v>
       </c>
     </row>
     <row r="27">
@@ -8746,16 +8872,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>65.61020000000001</v>
+        <v>65.8224</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>105688.846772</v>
+        <v>106030.671264</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-4311.153227999996</v>
+        <v>-3969.32873600001</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.03919230207272723</v>
+        <v>-0.03608480669090919</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -8915,6 +9041,9 @@
       </c>
       <c r="BJ27" s="3" t="n">
         <v>65.61020000000001</v>
+      </c>
+      <c r="BK27" s="3" t="n">
+        <v>65.8224</v>
       </c>
     </row>
     <row r="28">
@@ -8940,16 +9069,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>110.2185</v>
+        <v>110.5037</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>364454.7745545001</v>
+        <v>365397.8331309</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-15545.22544549993</v>
+        <v>-14602.16686910001</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.04090848801447351</v>
+        <v>-0.03842675491868423</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -9109,6 +9238,9 @@
       </c>
       <c r="BJ28" s="3" t="n">
         <v>110.2185</v>
+      </c>
+      <c r="BK28" s="3" t="n">
+        <v>110.5037</v>
       </c>
     </row>
     <row r="29">
@@ -9134,16 +9266,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.5477</v>
+        <v>12.6358</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>120504.3841331</v>
+        <v>121350.4703674</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>20504.3841331</v>
+        <v>21350.47036739999</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.205043841331</v>
+        <v>0.2135047036739999</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -9297,6 +9429,9 @@
       </c>
       <c r="BJ29" s="3" t="n">
         <v>12.5477</v>
+      </c>
+      <c r="BK29" s="3" t="n">
+        <v>12.6358</v>
       </c>
     </row>
     <row r="30">
@@ -9322,16 +9457,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>16.7276</v>
+        <v>16.8348</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>123715.0044636</v>
+        <v>124507.8407628</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>23715.00446359999</v>
+        <v>24507.84076280001</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.237150044636</v>
+        <v>0.2450784076280001</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -9485,6 +9620,9 @@
       </c>
       <c r="BJ30" s="3" t="n">
         <v>16.7276</v>
+      </c>
+      <c r="BK30" s="3" t="n">
+        <v>16.8348</v>
       </c>
     </row>
     <row r="31">
@@ -9510,16 +9648,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>417.1665</v>
+        <v>419.1787</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>110999.66232</v>
+        <v>111535.068496</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>10999.66231999999</v>
+        <v>11535.06849599999</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.1099966231999999</v>
+        <v>0.1153506849599999</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -9676,6 +9814,9 @@
       </c>
       <c r="BJ31" s="3" t="n">
         <v>417.1665</v>
+      </c>
+      <c r="BK31" s="3" t="n">
+        <v>419.1787</v>
       </c>
     </row>
     <row r="32">
@@ -9701,16 +9842,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.64</v>
+        <v>10.72</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>224929.1744</v>
+        <v>226620.3712</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>24929.17439999999</v>
+        <v>26620.37119999999</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.1246458719999999</v>
+        <v>0.133101856</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -9870,6 +10011,9 @@
       </c>
       <c r="BJ32" s="3" t="n">
         <v>10.64</v>
+      </c>
+      <c r="BK32" s="3" t="n">
+        <v>10.72</v>
       </c>
     </row>
     <row r="33">
@@ -9895,16 +10039,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>19</v>
+        <v>19.03</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>68089.16</v>
+        <v>68196.6692</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>8089.160000000003</v>
+        <v>8196.669200000004</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.1348193333333334</v>
+        <v>0.1366111533333334</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -10058,6 +10202,9 @@
       </c>
       <c r="BJ33" s="3" t="n">
         <v>19</v>
+      </c>
+      <c r="BK33" s="3" t="n">
+        <v>19.03</v>
       </c>
     </row>
     <row r="34">
@@ -10083,16 +10230,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>210.8218</v>
+        <v>210.9021</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>74110.3981758</v>
+        <v>74138.62611509999</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-5889.601824199999</v>
+        <v>-5861.373884900007</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.07362002280249999</v>
+        <v>-0.07326717356125009</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -10249,6 +10396,9 @@
       </c>
       <c r="BJ34" s="3" t="n">
         <v>210.8218</v>
+      </c>
+      <c r="BK34" s="3" t="n">
+        <v>210.9021</v>
       </c>
     </row>
     <row r="35">
@@ -10274,16 +10424,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>14.83</v>
+        <v>14.97</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>105818.32309</v>
+        <v>106817.28231</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>5818.323089999991</v>
+        <v>6817.282309999995</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.05818323089999991</v>
+        <v>0.06817282309999995</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -10440,6 +10590,9 @@
       </c>
       <c r="BJ35" s="3" t="n">
         <v>14.83</v>
+      </c>
+      <c r="BK35" s="3" t="n">
+        <v>14.97</v>
       </c>
     </row>
     <row r="36">
@@ -10465,16 +10618,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>374.9716</v>
+        <v>375.5278</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>174626.5239496</v>
+        <v>174885.5496268</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>24626.52394960003</v>
+        <v>24885.5496268</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1641768263306669</v>
+        <v>0.1659036641786667</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -10631,6 +10784,9 @@
       </c>
       <c r="BJ36" s="3" t="n">
         <v>374.9716</v>
+      </c>
+      <c r="BK36" s="3" t="n">
+        <v>375.5278</v>
       </c>
     </row>
     <row r="37">
@@ -10656,16 +10812,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>16.901</v>
+        <v>16.836</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>63596.586989</v>
+        <v>63351.999204</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>13596.586989</v>
+        <v>13351.999204</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.2719317397800001</v>
+        <v>0.26703998408</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -10822,6 +10978,9 @@
       </c>
       <c r="BJ37" s="3" t="n">
         <v>16.901</v>
+      </c>
+      <c r="BK37" s="3" t="n">
+        <v>16.836</v>
       </c>
     </row>
     <row r="38">
@@ -10847,16 +11006,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>14.3909</v>
+        <v>14.4664</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>86064.5184138</v>
+        <v>86516.0448048</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>6064.518413800004</v>
+        <v>6516.044804799996</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.07580648017250005</v>
+        <v>0.08145056005999995</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -11010,6 +11169,9 @@
       </c>
       <c r="BJ38" s="3" t="n">
         <v>14.3909</v>
+      </c>
+      <c r="BK38" s="3" t="n">
+        <v>14.4664</v>
       </c>
     </row>
     <row r="39">
@@ -11035,16 +11197,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1022.3097</v>
+        <v>1023.125</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50993.8301457</v>
+        <v>51034.498125</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>993.830145699998</v>
+        <v>1034.498124999998</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.01987660291399996</v>
+        <v>0.02068996249999996</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -11198,6 +11360,9 @@
       </c>
       <c r="BJ39" s="3" t="n">
         <v>1022.3097</v>
+      </c>
+      <c r="BK39" s="3" t="n">
+        <v>1023.125</v>
       </c>
     </row>
     <row r="40">
@@ -11223,16 +11388,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>21.744</v>
+        <v>22.0678</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>109612.091088</v>
+        <v>111244.3756306</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>9612.091088000001</v>
+        <v>11244.3756306</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.09612091088000001</v>
+        <v>0.112443756306</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -11389,6 +11554,9 @@
       </c>
       <c r="BJ40" s="3" t="n">
         <v>21.744</v>
+      </c>
+      <c r="BK40" s="3" t="n">
+        <v>22.0678</v>
       </c>
     </row>
     <row r="41">
@@ -11401,13 +11569,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4983336.4581221</v>
+        <v>4989918.8116697</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>513336.4581221001</v>
+        <v>519918.8116696999</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1148403709445414</v>
+        <v>0.1163129332594407</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-07-08
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -483,9 +483,9 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-07 06:05 IST</t>
+          <t>Generated: 2026-07-08 05:19 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4989918.8116697</v>
+        <v>4954844.2160715</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>519918.8116696998</v>
+        <v>484844.2160714995</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1163129332594407</v>
+        <v>0.1084662675775167</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>540070.0023727417</v>
+        <v>540565.9973220825</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-50712.01762725832</v>
+        <v>-50216.0226779175</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.08583879656198461</v>
+        <v>-0.08499923995303292</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5529988.814042442</v>
+        <v>5495410.213393582</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>469206.794042442</v>
+        <v>434628.1933935825</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.09271428648540014</v>
+        <v>0.08588162692563125</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-07-07</t>
+          <t>Last snapshot: 2026-07-08</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BJ19"/>
+  <dimension ref="A1:BK19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -681,6 +681,7 @@
     <col width="21" customWidth="1" min="60" max="60"/>
     <col width="21" customWidth="1" min="61" max="61"/>
     <col width="21" customWidth="1" min="62" max="62"/>
+    <col width="21" customWidth="1" min="63" max="63"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -994,6 +995,11 @@
           <t>2026-07-07</t>
         </is>
       </c>
+      <c r="BK1" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1013,13 +1019,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>533.7000122070312</v>
+        <v>525.5</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>42696.0009765625</v>
+        <v>42040</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>-1121.509023437502</v>
+        <v>-1777.510000000002</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1182,6 +1188,9 @@
       </c>
       <c r="BJ2" s="3" t="n">
         <v>533.7000122070312</v>
+      </c>
+      <c r="BK2" s="3" t="n">
+        <v>525.5</v>
       </c>
     </row>
     <row r="3">
@@ -1229,13 +1238,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1363.599975585938</v>
+        <v>1350.699951171875</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>27271.99951171875</v>
+        <v>27013.9990234375</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-4832.580488281252</v>
+        <v>-5090.580976562502</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1401,6 +1410,9 @@
       </c>
       <c r="BJ4" s="3" t="n">
         <v>1363.599975585938</v>
+      </c>
+      <c r="BK4" s="3" t="n">
+        <v>1350.699951171875</v>
       </c>
     </row>
     <row r="5">
@@ -1421,13 +1433,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>651.0499877929688</v>
+        <v>643.25</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>13020.99975585938</v>
+        <v>12865</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1192.100244140625</v>
+        <v>-1348.1</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1593,6 +1605,9 @@
       </c>
       <c r="BJ5" s="3" t="n">
         <v>651.0499877929688</v>
+      </c>
+      <c r="BK5" s="3" t="n">
+        <v>643.25</v>
       </c>
     </row>
     <row r="6">
@@ -1613,13 +1628,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>366.2999877929688</v>
+        <v>364.5</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>14651.99951171875</v>
+        <v>14580</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2850.240488281252</v>
+        <v>-2922.240000000002</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1785,6 +1800,9 @@
       </c>
       <c r="BJ6" s="3" t="n">
         <v>366.2999877929688</v>
+      </c>
+      <c r="BK6" s="3" t="n">
+        <v>364.5</v>
       </c>
     </row>
     <row r="7">
@@ -1805,13 +1823,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>239.6199951171875</v>
+        <v>243.0299987792969</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>23961.99951171875</v>
+        <v>24302.99987792969</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-2471.82048828125</v>
+        <v>-2130.820122070312</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1977,6 +1995,9 @@
       </c>
       <c r="BJ7" s="3" t="n">
         <v>239.6199951171875</v>
+      </c>
+      <c r="BK7" s="3" t="n">
+        <v>243.0299987792969</v>
       </c>
     </row>
     <row r="8">
@@ -2024,13 +2045,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>17.39999961853027</v>
+        <v>17.3700008392334</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>26099.99942779541</v>
+        <v>26055.0012588501</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-4950.170572204588</v>
+        <v>-4995.168741149901</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -2196,6 +2217,9 @@
       </c>
       <c r="BJ9" s="3" t="n">
         <v>17.39999961853027</v>
+      </c>
+      <c r="BK9" s="3" t="n">
+        <v>17.3700008392334</v>
       </c>
     </row>
     <row r="10">
@@ -2216,13 +2240,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>422.8500061035156</v>
+        <v>424.5</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>42285.00061035156</v>
+        <v>42450</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-9213.479389648441</v>
+        <v>-9048.480000000003</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -2388,6 +2412,9 @@
       </c>
       <c r="BJ10" s="3" t="n">
         <v>422.8500061035156</v>
+      </c>
+      <c r="BK10" s="3" t="n">
+        <v>424.5</v>
       </c>
     </row>
     <row r="11">
@@ -2408,13 +2435,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>9.239999771118164</v>
+        <v>9.729999542236328</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>9239.999771118164</v>
+        <v>9729.999542236328</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-601.2102288818351</v>
+        <v>-111.210457763671</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -2580,6 +2607,9 @@
       </c>
       <c r="BJ11" s="3" t="n">
         <v>9.239999771118164</v>
+      </c>
+      <c r="BK11" s="3" t="n">
+        <v>9.729999542236328</v>
       </c>
     </row>
     <row r="12">
@@ -2600,13 +2630,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2610.300048828125</v>
+        <v>2620</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>26103.00048828125</v>
+        <v>26200</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-1620.24951171875</v>
+        <v>-1523.25</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -2772,6 +2802,9 @@
       </c>
       <c r="BJ12" s="3" t="n">
         <v>2610.300048828125</v>
+      </c>
+      <c r="BK12" s="3" t="n">
+        <v>2620</v>
       </c>
     </row>
     <row r="13">
@@ -2792,13 +2825,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>54.61000061035156</v>
+        <v>54.20999908447266</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>32766.00036621094</v>
+        <v>32525.99945068359</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-2265.759633789065</v>
+        <v>-2505.760549316408</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -2964,6 +2997,9 @@
       </c>
       <c r="BJ13" s="3" t="n">
         <v>54.61000061035156</v>
+      </c>
+      <c r="BK13" s="3" t="n">
+        <v>54.20999908447266</v>
       </c>
     </row>
     <row r="14">
@@ -2984,13 +3020,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>704.7000122070312</v>
+        <v>717.7999877929688</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>35235.00061035156</v>
+        <v>35889.99938964844</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-7227.50938964844</v>
+        <v>-6572.510610351565</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -3156,6 +3192,9 @@
       </c>
       <c r="BJ14" s="3" t="n">
         <v>704.7000122070312</v>
+      </c>
+      <c r="BK14" s="3" t="n">
+        <v>717.7999877929688</v>
       </c>
     </row>
     <row r="15">
@@ -3230,13 +3269,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>547.9500122070312</v>
+        <v>551.5499877929688</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>27397.50061035156</v>
+        <v>27577.49938964844</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>5642.970610351564</v>
+        <v>5822.969389648439</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -3402,6 +3441,9 @@
       </c>
       <c r="BJ17" s="3" t="n">
         <v>547.9500122070312</v>
+      </c>
+      <c r="BK17" s="3" t="n">
+        <v>551.5499877929688</v>
       </c>
     </row>
     <row r="18">
@@ -3422,13 +3464,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>375.7000122070312</v>
+        <v>375.6499938964844</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>37570.00122070312</v>
+        <v>37564.99938964844</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-9070.818779296875</v>
+        <v>-9075.820610351562</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -3594,6 +3636,9 @@
       </c>
       <c r="BJ18" s="3" t="n">
         <v>375.7000122070312</v>
+      </c>
+      <c r="BK18" s="3" t="n">
+        <v>375.6499938964844</v>
       </c>
     </row>
     <row r="19">
@@ -3606,10 +3651,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>540070.0023727417</v>
+        <v>540565.9973220825</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-50712.01762725831</v>
+        <v>-50216.02267791749</v>
       </c>
     </row>
   </sheetData>
@@ -3623,7 +3668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BK41"/>
+  <dimension ref="A1:BL41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3633,7 +3678,7 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
@@ -3689,6 +3734,7 @@
     <col width="13" customWidth="1" min="61" max="61"/>
     <col width="13" customWidth="1" min="62" max="62"/>
     <col width="13" customWidth="1" min="63" max="63"/>
+    <col width="13" customWidth="1" min="64" max="64"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4007,6 +4053,11 @@
           <t>2026-07-07</t>
         </is>
       </c>
+      <c r="BL1" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -4031,16 +4082,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>57.3631</v>
+        <v>56.662</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>64389.0472142</v>
+        <v>63602.075084</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>14389.0472142</v>
+        <v>13602.075084</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.287780944284</v>
+        <v>0.2720415016799999</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -4203,6 +4254,9 @@
       </c>
       <c r="BK2" s="3" t="n">
         <v>57.3631</v>
+      </c>
+      <c r="BL2" s="3" t="n">
+        <v>56.662</v>
       </c>
     </row>
     <row r="3">
@@ -4228,16 +4282,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.7229</v>
+        <v>25.7378</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>63155.1984777</v>
+        <v>63191.78115140001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>3155.198477700003</v>
+        <v>3191.781151400006</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.05258664129500006</v>
+        <v>0.05319635252333343</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -4394,6 +4448,9 @@
       </c>
       <c r="BK3" s="3" t="n">
         <v>25.7229</v>
+      </c>
+      <c r="BL3" s="3" t="n">
+        <v>25.7378</v>
       </c>
     </row>
     <row r="4">
@@ -4419,16 +4476,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.3</v>
+        <v>12.1</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>236234.9439</v>
+        <v>232393.7253</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>56234.94390000001</v>
+        <v>52393.72529999999</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.3124163550000001</v>
+        <v>0.2910762516666666</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -4585,6 +4642,9 @@
       </c>
       <c r="BK4" s="3" t="n">
         <v>12.3</v>
+      </c>
+      <c r="BL4" s="3" t="n">
+        <v>12.1</v>
       </c>
     </row>
     <row r="5">
@@ -4610,16 +4670,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.519299999999999</v>
+        <v>9.542</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>174718.0698984</v>
+        <v>175134.707696</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-35281.93010160001</v>
+        <v>-34865.292304</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1680091909600001</v>
+        <v>-0.1660252014476191</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -4776,6 +4836,9 @@
       </c>
       <c r="BK5" s="3" t="n">
         <v>9.519299999999999</v>
+      </c>
+      <c r="BL5" s="3" t="n">
+        <v>9.542</v>
       </c>
     </row>
     <row r="6">
@@ -4801,16 +4864,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>12.008</v>
+        <v>11.9114</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>50781.55581599999</v>
+        <v>50373.0366378</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>781.5558159999928</v>
+        <v>373.0366378000035</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.01563111631999986</v>
+        <v>0.00746073275600007</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -4973,6 +5036,9 @@
       </c>
       <c r="BK6" s="3" t="n">
         <v>12.008</v>
+      </c>
+      <c r="BL6" s="3" t="n">
+        <v>11.9114</v>
       </c>
     </row>
     <row r="7">
@@ -4998,16 +5064,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>34.8705</v>
+        <v>34.7166</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>76925.71782000001</v>
+        <v>76586.208264</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>16925.71782000001</v>
+        <v>16586.208264</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2820952970000001</v>
+        <v>0.2764368044</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -5164,6 +5230,9 @@
       </c>
       <c r="BK7" s="3" t="n">
         <v>34.8705</v>
+      </c>
+      <c r="BL7" s="3" t="n">
+        <v>34.7166</v>
       </c>
     </row>
     <row r="8">
@@ -5189,16 +5258,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>33.7515</v>
+        <v>33.5633</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>54157.4206395</v>
+        <v>53855.4362369</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>4157.4206395</v>
+        <v>3855.436236900001</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.08314841279</v>
+        <v>0.07710872473800003</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -5361,6 +5430,9 @@
       </c>
       <c r="BK8" s="3" t="n">
         <v>33.7515</v>
+      </c>
+      <c r="BL8" s="3" t="n">
+        <v>33.5633</v>
       </c>
     </row>
     <row r="9">
@@ -5386,16 +5458,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>42.5258</v>
+        <v>40.9134</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>136907.2628394</v>
+        <v>131716.3135662</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>36907.26283939998</v>
+        <v>31716.3135662</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3690726283939998</v>
+        <v>0.317163135662</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -5552,6 +5624,9 @@
       </c>
       <c r="BK9" s="3" t="n">
         <v>42.5258</v>
+      </c>
+      <c r="BL9" s="3" t="n">
+        <v>40.9134</v>
       </c>
     </row>
     <row r="10">
@@ -5577,16 +5652,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48.2855</v>
+        <v>48.5781</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>137452.3531445</v>
+        <v>138285.2855679</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>37452.3531445</v>
+        <v>38285.28556789999</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3745235314449999</v>
+        <v>0.3828528556789999</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -5743,6 +5818,9 @@
       </c>
       <c r="BK10" s="3" t="n">
         <v>48.2855</v>
+      </c>
+      <c r="BL10" s="3" t="n">
+        <v>48.5781</v>
       </c>
     </row>
     <row r="11">
@@ -5768,16 +5846,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>105.6646</v>
+        <v>103.7456</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31796.4857674</v>
+        <v>31219.0222064</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1796.485767399998</v>
+        <v>1219.022206399997</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.05988285891333326</v>
+        <v>0.04063407354666657</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -5934,6 +6012,9 @@
       </c>
       <c r="BK11" s="3" t="n">
         <v>105.6646</v>
+      </c>
+      <c r="BL11" s="3" t="n">
+        <v>103.7456</v>
       </c>
     </row>
     <row r="12">
@@ -5959,16 +6040,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>230.395</v>
+        <v>231.094</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>107253.94119</v>
+        <v>107579.341068</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>7253.941189999998</v>
+        <v>7579.341067999994</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.07253941189999998</v>
+        <v>0.07579341067999994</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -6131,6 +6212,9 @@
       </c>
       <c r="BK12" s="3" t="n">
         <v>230.395</v>
+      </c>
+      <c r="BL12" s="3" t="n">
+        <v>231.094</v>
       </c>
     </row>
     <row r="13">
@@ -6156,16 +6240,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>21.389</v>
+        <v>21.221</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>247847.283345</v>
+        <v>245900.565705</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>47847.28334499997</v>
+        <v>45900.56570499999</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.2392364167249999</v>
+        <v>0.2295028285249999</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -6328,6 +6412,9 @@
       </c>
       <c r="BK13" s="3" t="n">
         <v>21.389</v>
+      </c>
+      <c r="BL13" s="3" t="n">
+        <v>21.221</v>
       </c>
     </row>
     <row r="14">
@@ -6353,16 +6440,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>38.8716</v>
+        <v>37.9607</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>140233.4173896</v>
+        <v>136947.2490842</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>40233.41738960001</v>
+        <v>36947.24908420001</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.4023341738960001</v>
+        <v>0.3694724908420001</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -6519,6 +6606,9 @@
       </c>
       <c r="BK14" s="3" t="n">
         <v>38.8716</v>
+      </c>
+      <c r="BL14" s="3" t="n">
+        <v>37.9607</v>
       </c>
     </row>
     <row r="15">
@@ -6544,16 +6634,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.86</v>
+        <v>11.72</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>115563.21142</v>
+        <v>114199.05884</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>15563.21141999999</v>
+        <v>14199.05884000001</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1556321141999999</v>
+        <v>0.1419905884000001</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -6716,6 +6806,9 @@
       </c>
       <c r="BK15" s="3" t="n">
         <v>11.86</v>
+      </c>
+      <c r="BL15" s="3" t="n">
+        <v>11.72</v>
       </c>
     </row>
     <row r="16">
@@ -6741,16 +6834,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.6581</v>
+        <v>24.1924</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>141116.5309168</v>
+        <v>138451.3633472</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>41116.53091679999</v>
+        <v>38451.36334719998</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4111653091679999</v>
+        <v>0.3845136334719998</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -6907,6 +7000,9 @@
       </c>
       <c r="BK16" s="3" t="n">
         <v>24.6581</v>
+      </c>
+      <c r="BL16" s="3" t="n">
+        <v>24.1924</v>
       </c>
     </row>
     <row r="17">
@@ -6932,16 +7028,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>17.0198</v>
+        <v>16.9736</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>56268.4289286</v>
+        <v>56115.6890952</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>6268.428928599998</v>
+        <v>6115.689095200003</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.125368578572</v>
+        <v>0.1223137819040001</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -7098,6 +7194,9 @@
       </c>
       <c r="BK17" s="3" t="n">
         <v>17.0198</v>
+      </c>
+      <c r="BL17" s="3" t="n">
+        <v>16.9736</v>
       </c>
     </row>
     <row r="18">
@@ -7123,16 +7222,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>47.33</v>
+        <v>47.05</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>89285.01587999999</v>
+        <v>88756.81379999999</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>9285.015879999992</v>
+        <v>8756.813799999989</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.1160626984999999</v>
+        <v>0.1094601724999999</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -7295,6 +7394,9 @@
       </c>
       <c r="BK18" s="3" t="n">
         <v>47.33</v>
+      </c>
+      <c r="BL18" s="3" t="n">
+        <v>47.05</v>
       </c>
     </row>
     <row r="19">
@@ -7320,16 +7422,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>14.1948</v>
+        <v>13.9999</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>205352.8500168</v>
+        <v>202533.2773234</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>55352.85001680002</v>
+        <v>52533.27732339999</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.3690190001120001</v>
+        <v>0.3502218488226666</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -7486,6 +7588,9 @@
       </c>
       <c r="BK19" s="3" t="n">
         <v>14.1948</v>
+      </c>
+      <c r="BL19" s="3" t="n">
+        <v>13.9999</v>
       </c>
     </row>
     <row r="20">
@@ -7511,16 +7616,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.34</v>
+        <v>9.43</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>245229.20002</v>
+        <v>247592.22229</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-4770.799980000011</v>
+        <v>-2407.777709999995</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.01908319992000004</v>
+        <v>-0.009631110839999979</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -7683,6 +7788,9 @@
       </c>
       <c r="BK20" s="3" t="n">
         <v>9.34</v>
+      </c>
+      <c r="BL20" s="3" t="n">
+        <v>9.43</v>
       </c>
     </row>
     <row r="21">
@@ -7708,16 +7816,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>113.3446</v>
+        <v>112.7556</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>172199.8036514</v>
+        <v>171304.9601004</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>2199.803651399998</v>
+        <v>1304.9601004</v>
       </c>
       <c r="I21" s="12" t="n">
-        <v>0.01294002147882352</v>
+        <v>0.007676235884705881</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -7880,6 +7988,9 @@
       </c>
       <c r="BK21" s="3" t="n">
         <v>113.3446</v>
+      </c>
+      <c r="BL21" s="3" t="n">
+        <v>112.7556</v>
       </c>
     </row>
     <row r="22">
@@ -7905,16 +8016,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>44.183</v>
+        <v>43.098</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>67797.04618</v>
+        <v>66132.15708</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>7797.046180000005</v>
+        <v>6132.157080000004</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1299507696666667</v>
+        <v>0.1022026180000001</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -8071,6 +8182,9 @@
       </c>
       <c r="BK22" s="3" t="n">
         <v>44.183</v>
+      </c>
+      <c r="BL22" s="3" t="n">
+        <v>43.098</v>
       </c>
     </row>
     <row r="23">
@@ -8096,16 +8210,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>64.0916</v>
+        <v>63.4827</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>174102.7163772</v>
+        <v>172448.6596209</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>24102.71637720001</v>
+        <v>22448.6596209</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.160684775848</v>
+        <v>0.149657730806</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -8268,6 +8382,9 @@
       </c>
       <c r="BK23" s="3" t="n">
         <v>64.0916</v>
+      </c>
+      <c r="BL23" s="3" t="n">
+        <v>63.4827</v>
       </c>
     </row>
     <row r="24">
@@ -8293,16 +8410,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>27.7996</v>
+        <v>27.7039</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>101006.6774456</v>
+        <v>100658.9624054</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>1006.677445599998</v>
+        <v>658.9624054000014</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0.01006677445599998</v>
+        <v>0.006589624054000014</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -8459,6 +8576,9 @@
       </c>
       <c r="BK24" s="3" t="n">
         <v>27.7996</v>
+      </c>
+      <c r="BL24" s="3" t="n">
+        <v>27.7039</v>
       </c>
     </row>
     <row r="25">
@@ -8484,16 +8604,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.9148</v>
+        <v>11.8526</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>195660.9613752</v>
+        <v>194639.5332524</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-4339.038624800014</v>
+        <v>-5360.466747600003</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.02169519312400007</v>
+        <v>-0.02680233373800002</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -8653,6 +8773,9 @@
       </c>
       <c r="BK25" s="3" t="n">
         <v>11.9148</v>
+      </c>
+      <c r="BL25" s="3" t="n">
+        <v>11.8526</v>
       </c>
     </row>
     <row r="26">
@@ -8678,16 +8801,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>9.4506</v>
+        <v>9.515000000000001</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>112856.371779</v>
+        <v>113625.418225</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>2856.371778999994</v>
+        <v>3625.418225000001</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.02596701617272722</v>
+        <v>0.03295834750000001</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -8847,6 +8970,9 @@
       </c>
       <c r="BK26" s="3" t="n">
         <v>9.4506</v>
+      </c>
+      <c r="BL26" s="3" t="n">
+        <v>9.515000000000001</v>
       </c>
     </row>
     <row r="27">
@@ -8872,16 +8998,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>65.8224</v>
+        <v>65.2525</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>106030.671264</v>
+        <v>105112.64215</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-3969.32873600001</v>
+        <v>-4887.357850000015</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.03608480669090919</v>
+        <v>-0.04443052590909104</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -9044,6 +9170,9 @@
       </c>
       <c r="BK27" s="3" t="n">
         <v>65.8224</v>
+      </c>
+      <c r="BL27" s="3" t="n">
+        <v>65.2525</v>
       </c>
     </row>
     <row r="28">
@@ -9069,16 +9198,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>110.5037</v>
+        <v>109.7658</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>365397.8331309</v>
+        <v>362957.8509306</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-14602.16686910001</v>
+        <v>-17042.14906939998</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.03842675491868423</v>
+        <v>-0.04484776070894732</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -9241,6 +9370,9 @@
       </c>
       <c r="BK28" s="3" t="n">
         <v>110.5037</v>
+      </c>
+      <c r="BL28" s="3" t="n">
+        <v>109.7658</v>
       </c>
     </row>
     <row r="29">
@@ -9266,16 +9398,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.6358</v>
+        <v>12.4274</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>121350.4703674</v>
+        <v>119349.0586622</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>21350.47036739999</v>
+        <v>19349.0586622</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.2135047036739999</v>
+        <v>0.193490586622</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -9432,6 +9564,9 @@
       </c>
       <c r="BK29" s="3" t="n">
         <v>12.6358</v>
+      </c>
+      <c r="BL29" s="3" t="n">
+        <v>12.4274</v>
       </c>
     </row>
     <row r="30">
@@ -9457,16 +9592,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>16.8348</v>
+        <v>16.8079</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>124507.8407628</v>
+        <v>124308.8921019</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>24507.84076280001</v>
+        <v>24308.8921019</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.2450784076280001</v>
+        <v>0.243088921019</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -9623,6 +9758,9 @@
       </c>
       <c r="BK30" s="3" t="n">
         <v>16.8348</v>
+      </c>
+      <c r="BL30" s="3" t="n">
+        <v>16.8079</v>
       </c>
     </row>
     <row r="31">
@@ -9648,16 +9786,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>419.1787</v>
+        <v>414.2588</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>111535.068496</v>
+        <v>110225.981504</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>11535.06849599999</v>
+        <v>10225.981504</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.1153506849599999</v>
+        <v>0.10225981504</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -9817,6 +9955,9 @@
       </c>
       <c r="BK31" s="3" t="n">
         <v>419.1787</v>
+      </c>
+      <c r="BL31" s="3" t="n">
+        <v>414.2588</v>
       </c>
     </row>
     <row r="32">
@@ -9842,16 +9983,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.72</v>
+        <v>10.67</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>226620.3712</v>
+        <v>225563.3732</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>26620.37119999999</v>
+        <v>25563.3732</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.133101856</v>
+        <v>0.127816866</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -10014,6 +10155,9 @@
       </c>
       <c r="BK32" s="3" t="n">
         <v>10.72</v>
+      </c>
+      <c r="BL32" s="3" t="n">
+        <v>10.67</v>
       </c>
     </row>
     <row r="33">
@@ -10039,16 +10183,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>19.03</v>
+        <v>18.92</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>68196.6692</v>
+        <v>67802.4688</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>8196.669200000004</v>
+        <v>7802.468800000002</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.1366111533333334</v>
+        <v>0.1300411466666667</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -10205,6 +10349,9 @@
       </c>
       <c r="BK33" s="3" t="n">
         <v>19.03</v>
+      </c>
+      <c r="BL33" s="3" t="n">
+        <v>18.92</v>
       </c>
     </row>
     <row r="34">
@@ -10230,16 +10377,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>210.9021</v>
+        <v>215.049</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>74138.62611509999</v>
+        <v>75596.390019</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-5861.373884900007</v>
+        <v>-4403.609981000001</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.07326717356125009</v>
+        <v>-0.05504512476250002</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -10399,6 +10546,9 @@
       </c>
       <c r="BK34" s="3" t="n">
         <v>210.9021</v>
+      </c>
+      <c r="BL34" s="3" t="n">
+        <v>215.049</v>
       </c>
     </row>
     <row r="35">
@@ -10424,16 +10574,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>14.97</v>
+        <v>14.92</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>106817.28231</v>
+        <v>106460.51116</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>6817.282309999995</v>
+        <v>6460.511159999995</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.06817282309999995</v>
+        <v>0.06460511159999995</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -10593,6 +10743,9 @@
       </c>
       <c r="BK35" s="3" t="n">
         <v>14.97</v>
+      </c>
+      <c r="BL35" s="3" t="n">
+        <v>14.92</v>
       </c>
     </row>
     <row r="36">
@@ -10618,16 +10771,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>375.5278</v>
+        <v>372.8502</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>174885.5496268</v>
+        <v>173638.5752412</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>24885.5496268</v>
+        <v>23638.57524119999</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1659036641786667</v>
+        <v>0.1575905016079999</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -10787,6 +10940,9 @@
       </c>
       <c r="BK36" s="3" t="n">
         <v>375.5278</v>
+      </c>
+      <c r="BL36" s="3" t="n">
+        <v>372.8502</v>
       </c>
     </row>
     <row r="37">
@@ -10812,16 +10968,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>16.836</v>
+        <v>16.694</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>63351.999204</v>
+        <v>62817.668966</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>13351.999204</v>
+        <v>12817.668966</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.26703998408</v>
+        <v>0.25635337932</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -10981,6 +11137,9 @@
       </c>
       <c r="BK37" s="3" t="n">
         <v>16.836</v>
+      </c>
+      <c r="BL37" s="3" t="n">
+        <v>16.694</v>
       </c>
     </row>
     <row r="38">
@@ -11006,16 +11165,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>14.4664</v>
+        <v>14.4324</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>86516.0448048</v>
+        <v>86312.7084168</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>6516.044804799996</v>
+        <v>6312.7084168</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.08145056005999995</v>
+        <v>0.07890885521</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -11172,6 +11331,9 @@
       </c>
       <c r="BK38" s="3" t="n">
         <v>14.4664</v>
+      </c>
+      <c r="BL38" s="3" t="n">
+        <v>14.4324</v>
       </c>
     </row>
     <row r="39">
@@ -11197,16 +11359,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1023.125</v>
+        <v>1023.5507</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51034.498125</v>
+        <v>51055.7324667</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1034.498124999998</v>
+        <v>1055.732466699999</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.02068996249999996</v>
+        <v>0.02111464933399999</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -11363,6 +11525,9 @@
       </c>
       <c r="BK39" s="3" t="n">
         <v>1023.125</v>
+      </c>
+      <c r="BL39" s="3" t="n">
+        <v>1023.5507</v>
       </c>
     </row>
     <row r="40">
@@ -11388,16 +11553,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>22.0678</v>
+        <v>21.9002</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>111244.3756306</v>
+        <v>110399.4995054</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>11244.3756306</v>
+        <v>10399.4995054</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.112443756306</v>
+        <v>0.103994995054</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -11557,6 +11722,9 @@
       </c>
       <c r="BK40" s="3" t="n">
         <v>22.0678</v>
+      </c>
+      <c r="BL40" s="3" t="n">
+        <v>21.9002</v>
       </c>
     </row>
     <row r="41">
@@ -11569,13 +11737,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4989918.8116697</v>
+        <v>4954844.2160715</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>519918.8116696999</v>
+        <v>484844.2160714999</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1163129332594407</v>
+        <v>0.1084662675775168</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-07-09
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -484,8 +484,8 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-08 05:19 IST</t>
+          <t>Generated: 2026-07-09 06:02 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4954844.2160715</v>
+        <v>4885303.4984155</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>484844.2160714995</v>
+        <v>415303.4984154999</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1084662675775167</v>
+        <v>0.09290906004821027</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>540565.9973220825</v>
+        <v>539316.0028152466</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-50216.0226779175</v>
+        <v>-51466.01718475344</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.08499923995303292</v>
+        <v>-0.0871150702669547</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5495410.213393582</v>
+        <v>5424619.501230747</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>434628.1933935825</v>
+        <v>363837.481230747</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.08588162692563125</v>
+        <v>0.07189352945708319</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-07-08</t>
+          <t>Last snapshot: 2026-07-09</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BK19"/>
+  <dimension ref="A1:BL19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -682,6 +682,7 @@
     <col width="21" customWidth="1" min="61" max="61"/>
     <col width="21" customWidth="1" min="62" max="62"/>
     <col width="21" customWidth="1" min="63" max="63"/>
+    <col width="21" customWidth="1" min="64" max="64"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1000,6 +1001,11 @@
           <t>2026-07-08</t>
         </is>
       </c>
+      <c r="BL1" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1019,13 +1025,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>525.5</v>
+        <v>528.75</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>42040</v>
+        <v>42300</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>-1777.510000000002</v>
+        <v>-1517.510000000002</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1191,6 +1197,9 @@
       </c>
       <c r="BK2" s="3" t="n">
         <v>525.5</v>
+      </c>
+      <c r="BL2" s="3" t="n">
+        <v>528.75</v>
       </c>
     </row>
     <row r="3">
@@ -1238,13 +1247,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1350.699951171875</v>
+        <v>1332.800048828125</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>27013.9990234375</v>
+        <v>26656.0009765625</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-5090.580976562502</v>
+        <v>-5448.579023437502</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1413,6 +1422,9 @@
       </c>
       <c r="BK4" s="3" t="n">
         <v>1350.699951171875</v>
+      </c>
+      <c r="BL4" s="3" t="n">
+        <v>1332.800048828125</v>
       </c>
     </row>
     <row r="5">
@@ -1433,13 +1445,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>643.25</v>
+        <v>645.5999755859375</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>12865</v>
+        <v>12911.99951171875</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1348.1</v>
+        <v>-1301.10048828125</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1608,6 +1620,9 @@
       </c>
       <c r="BK5" s="3" t="n">
         <v>643.25</v>
+      </c>
+      <c r="BL5" s="3" t="n">
+        <v>645.5999755859375</v>
       </c>
     </row>
     <row r="6">
@@ -1628,13 +1643,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>364.5</v>
+        <v>359</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>14580</v>
+        <v>14360</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2922.240000000002</v>
+        <v>-3142.240000000002</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1803,6 +1818,9 @@
       </c>
       <c r="BK6" s="3" t="n">
         <v>364.5</v>
+      </c>
+      <c r="BL6" s="3" t="n">
+        <v>359</v>
       </c>
     </row>
     <row r="7">
@@ -1823,13 +1841,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>243.0299987792969</v>
+        <v>237.25</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>24302.99987792969</v>
+        <v>23725</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-2130.820122070312</v>
+        <v>-2708.82</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -1998,6 +2016,9 @@
       </c>
       <c r="BK7" s="3" t="n">
         <v>243.0299987792969</v>
+      </c>
+      <c r="BL7" s="3" t="n">
+        <v>237.25</v>
       </c>
     </row>
     <row r="8">
@@ -2045,13 +2066,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>17.3700008392334</v>
+        <v>17.10000038146973</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>26055.0012588501</v>
+        <v>25650.00057220459</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-4995.168741149901</v>
+        <v>-5400.169427795408</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -2220,6 +2241,9 @@
       </c>
       <c r="BK9" s="3" t="n">
         <v>17.3700008392334</v>
+      </c>
+      <c r="BL9" s="3" t="n">
+        <v>17.10000038146973</v>
       </c>
     </row>
     <row r="10">
@@ -2240,13 +2264,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>424.5</v>
+        <v>427.6000061035156</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>42450</v>
+        <v>42760.00061035156</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-9048.480000000003</v>
+        <v>-8738.479389648441</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -2415,6 +2439,9 @@
       </c>
       <c r="BK10" s="3" t="n">
         <v>424.5</v>
+      </c>
+      <c r="BL10" s="3" t="n">
+        <v>427.6000061035156</v>
       </c>
     </row>
     <row r="11">
@@ -2435,13 +2462,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>9.729999542236328</v>
+        <v>10.89999961853027</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>9729.999542236328</v>
-      </c>
-      <c r="G11" s="6" t="n">
-        <v>-111.210457763671</v>
+        <v>10899.99961853027</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>1058.789618530274</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -2610,6 +2637,9 @@
       </c>
       <c r="BK11" s="3" t="n">
         <v>9.729999542236328</v>
+      </c>
+      <c r="BL11" s="3" t="n">
+        <v>10.89999961853027</v>
       </c>
     </row>
     <row r="12">
@@ -2630,13 +2660,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2620</v>
+        <v>2628.300048828125</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>26200</v>
+        <v>26283.00048828125</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-1523.25</v>
+        <v>-1440.24951171875</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -2805,6 +2835,9 @@
       </c>
       <c r="BK12" s="3" t="n">
         <v>2620</v>
+      </c>
+      <c r="BL12" s="3" t="n">
+        <v>2628.300048828125</v>
       </c>
     </row>
     <row r="13">
@@ -2825,13 +2858,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>54.20999908447266</v>
+        <v>53.56999969482422</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>32525.99945068359</v>
+        <v>32141.99981689453</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-2505.760549316408</v>
+        <v>-2889.760183105471</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -3000,6 +3033,9 @@
       </c>
       <c r="BK13" s="3" t="n">
         <v>54.20999908447266</v>
+      </c>
+      <c r="BL13" s="3" t="n">
+        <v>53.56999969482422</v>
       </c>
     </row>
     <row r="14">
@@ -3020,13 +3056,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>717.7999877929688</v>
+        <v>708.4000244140625</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>35889.99938964844</v>
+        <v>35420.00122070312</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-6572.510610351565</v>
+        <v>-7042.508779296877</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -3195,6 +3231,9 @@
       </c>
       <c r="BK14" s="3" t="n">
         <v>717.7999877929688</v>
+      </c>
+      <c r="BL14" s="3" t="n">
+        <v>708.4000244140625</v>
       </c>
     </row>
     <row r="15">
@@ -3269,13 +3308,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>551.5499877929688</v>
+        <v>538.9500122070312</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>27577.49938964844</v>
+        <v>26947.50061035156</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>5822.969389648439</v>
+        <v>5192.970610351564</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -3444,6 +3483,9 @@
       </c>
       <c r="BK17" s="3" t="n">
         <v>551.5499877929688</v>
+      </c>
+      <c r="BL17" s="3" t="n">
+        <v>538.9500122070312</v>
       </c>
     </row>
     <row r="18">
@@ -3464,13 +3506,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>375.6499938964844</v>
+        <v>374.8999938964844</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>37564.99938964844</v>
+        <v>37489.99938964844</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-9075.820610351562</v>
+        <v>-9150.820610351562</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -3639,6 +3681,9 @@
       </c>
       <c r="BK18" s="3" t="n">
         <v>375.6499938964844</v>
+      </c>
+      <c r="BL18" s="3" t="n">
+        <v>374.8999938964844</v>
       </c>
     </row>
     <row r="19">
@@ -3651,10 +3696,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>540565.9973220825</v>
+        <v>539316.0028152466</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-50216.02267791749</v>
+        <v>-51466.01718475343</v>
       </c>
     </row>
   </sheetData>
@@ -3668,7 +3713,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BL41"/>
+  <dimension ref="A1:BM41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3678,7 +3723,7 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
@@ -3735,6 +3780,7 @@
     <col width="13" customWidth="1" min="62" max="62"/>
     <col width="13" customWidth="1" min="63" max="63"/>
     <col width="13" customWidth="1" min="64" max="64"/>
+    <col width="13" customWidth="1" min="65" max="65"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4058,6 +4104,11 @@
           <t>2026-07-08</t>
         </is>
       </c>
+      <c r="BM1" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -4082,16 +4133,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.662</v>
+        <v>56.7992</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>63602.075084</v>
+        <v>63756.0796144</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>13602.075084</v>
+        <v>13756.0796144</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.2720415016799999</v>
+        <v>0.275121592288</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -4257,6 +4308,9 @@
       </c>
       <c r="BL2" s="3" t="n">
         <v>56.662</v>
+      </c>
+      <c r="BM2" s="3" t="n">
+        <v>56.7992</v>
       </c>
     </row>
     <row r="3">
@@ -4282,16 +4336,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.7378</v>
+        <v>25.4644</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>63191.78115140001</v>
+        <v>62520.52591720001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>3191.781151400006</v>
+        <v>2520.525917200008</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.05319635252333343</v>
+        <v>0.0420087652866668</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -4451,6 +4505,9 @@
       </c>
       <c r="BL3" s="3" t="n">
         <v>25.7378</v>
+      </c>
+      <c r="BM3" s="3" t="n">
+        <v>25.4644</v>
       </c>
     </row>
     <row r="4">
@@ -4476,16 +4533,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.1</v>
+        <v>12.07</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>232393.7253</v>
+        <v>231817.54251</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>52393.72529999999</v>
+        <v>51817.54251000003</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.2910762516666666</v>
+        <v>0.2878752361666668</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -4645,6 +4702,9 @@
       </c>
       <c r="BL4" s="3" t="n">
         <v>12.1</v>
+      </c>
+      <c r="BM4" s="3" t="n">
+        <v>12.07</v>
       </c>
     </row>
     <row r="5">
@@ -4670,16 +4730,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.542</v>
+        <v>9.373699999999999</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>175134.707696</v>
+        <v>172045.7146856</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-34865.292304</v>
+        <v>-37954.28531440001</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1660252014476191</v>
+        <v>-0.1807346919733334</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -4839,6 +4899,9 @@
       </c>
       <c r="BL5" s="3" t="n">
         <v>9.542</v>
+      </c>
+      <c r="BM5" s="3" t="n">
+        <v>9.373699999999999</v>
       </c>
     </row>
     <row r="6">
@@ -4864,16 +4927,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>11.9114</v>
+        <v>11.7795</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>50373.0366378</v>
-      </c>
-      <c r="H6" s="4" t="n">
-        <v>373.0366378000035</v>
-      </c>
-      <c r="I6" s="12" t="n">
-        <v>0.00746073275600007</v>
+        <v>49815.2345715</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>-184.7654285000026</v>
+      </c>
+      <c r="I6" s="13" t="n">
+        <v>-0.003695308570000052</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -5039,6 +5102,9 @@
       </c>
       <c r="BL6" s="3" t="n">
         <v>11.9114</v>
+      </c>
+      <c r="BM6" s="3" t="n">
+        <v>11.7795</v>
       </c>
     </row>
     <row r="7">
@@ -5064,16 +5130,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>34.7166</v>
+        <v>34.1904</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>76586.208264</v>
+        <v>75425.39001599999</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>16586.208264</v>
+        <v>15425.39001599999</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2764368044</v>
+        <v>0.2570898335999998</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -5233,6 +5299,9 @@
       </c>
       <c r="BL7" s="3" t="n">
         <v>34.7166</v>
+      </c>
+      <c r="BM7" s="3" t="n">
+        <v>34.1904</v>
       </c>
     </row>
     <row r="8">
@@ -5258,16 +5327,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>33.5633</v>
+        <v>33.2286</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>53855.4362369</v>
+        <v>53318.3789598</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>3855.436236900001</v>
+        <v>3318.3789598</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.07710872473800003</v>
+        <v>0.066367579196</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -5433,6 +5502,9 @@
       </c>
       <c r="BL8" s="3" t="n">
         <v>33.5633</v>
+      </c>
+      <c r="BM8" s="3" t="n">
+        <v>33.2286</v>
       </c>
     </row>
     <row r="9">
@@ -5458,16 +5530,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>40.9134</v>
+        <v>40.6637</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>131716.3135662</v>
+        <v>130912.4311341</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>31716.3135662</v>
+        <v>30912.4311341</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.317163135662</v>
+        <v>0.309124311341</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -5627,6 +5699,9 @@
       </c>
       <c r="BL9" s="3" t="n">
         <v>40.9134</v>
+      </c>
+      <c r="BM9" s="3" t="n">
+        <v>40.6637</v>
       </c>
     </row>
     <row r="10">
@@ -5652,16 +5727,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48.5781</v>
+        <v>48.0914</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>138285.2855679</v>
+        <v>136899.8166326</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>38285.28556789999</v>
+        <v>36899.81663260001</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3828528556789999</v>
+        <v>0.3689981663260001</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -5821,6 +5896,9 @@
       </c>
       <c r="BL10" s="3" t="n">
         <v>48.5781</v>
+      </c>
+      <c r="BM10" s="3" t="n">
+        <v>48.0914</v>
       </c>
     </row>
     <row r="11">
@@ -5846,16 +5924,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>103.7456</v>
+        <v>104.7936</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31219.0222064</v>
+        <v>31534.3853184</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1219.022206399997</v>
+        <v>1534.385318399996</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.04063407354666657</v>
+        <v>0.05114617727999988</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -6015,6 +6093,9 @@
       </c>
       <c r="BL11" s="3" t="n">
         <v>103.7456</v>
+      </c>
+      <c r="BM11" s="3" t="n">
+        <v>104.7936</v>
       </c>
     </row>
     <row r="12">
@@ -6040,16 +6121,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>231.094</v>
+        <v>226.564</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>107579.341068</v>
+        <v>105470.526408</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>7579.341067999994</v>
+        <v>5470.526407999991</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.07579341067999994</v>
+        <v>0.05470526407999991</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -6215,6 +6296,9 @@
       </c>
       <c r="BL12" s="3" t="n">
         <v>231.094</v>
+      </c>
+      <c r="BM12" s="3" t="n">
+        <v>226.564</v>
       </c>
     </row>
     <row r="13">
@@ -6240,16 +6324,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>21.221</v>
+        <v>20.994</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>245900.565705</v>
+        <v>243270.17937</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>45900.56570499999</v>
+        <v>43270.17937</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.2295028285249999</v>
+        <v>0.21635089685</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -6415,6 +6499,9 @@
       </c>
       <c r="BL13" s="3" t="n">
         <v>21.221</v>
+      </c>
+      <c r="BM13" s="3" t="n">
+        <v>20.994</v>
       </c>
     </row>
     <row r="14">
@@ -6440,16 +6527,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>37.9607</v>
+        <v>37.5088</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>136947.2490842</v>
+        <v>135316.9719328</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>36947.24908420001</v>
+        <v>35316.97193280002</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.3694724908420001</v>
+        <v>0.3531697193280002</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -6609,6 +6696,9 @@
       </c>
       <c r="BL14" s="3" t="n">
         <v>37.9607</v>
+      </c>
+      <c r="BM14" s="3" t="n">
+        <v>37.5088</v>
       </c>
     </row>
     <row r="15">
@@ -6634,16 +6724,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.72</v>
+        <v>11.58</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>114199.05884</v>
+        <v>112834.90626</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>14199.05884000001</v>
+        <v>12834.90626</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1419905884000001</v>
+        <v>0.1283490626</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -6809,6 +6899,9 @@
       </c>
       <c r="BL15" s="3" t="n">
         <v>11.72</v>
+      </c>
+      <c r="BM15" s="3" t="n">
+        <v>11.58</v>
       </c>
     </row>
     <row r="16">
@@ -6834,16 +6927,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.1924</v>
+        <v>24.2351</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>138451.3633472</v>
+        <v>138695.7323728</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>38451.36334719998</v>
+        <v>38695.7323728</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.3845136334719998</v>
+        <v>0.3869573237280001</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -7003,6 +7096,9 @@
       </c>
       <c r="BL16" s="3" t="n">
         <v>24.1924</v>
+      </c>
+      <c r="BM16" s="3" t="n">
+        <v>24.2351</v>
       </c>
     </row>
     <row r="17">
@@ -7028,16 +7124,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.9736</v>
+        <v>16.8052</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>56115.6890952</v>
+        <v>55558.94909639999</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>6115.689095200003</v>
+        <v>5558.949096399992</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1223137819040001</v>
+        <v>0.1111789819279999</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -7197,6 +7293,9 @@
       </c>
       <c r="BL17" s="3" t="n">
         <v>16.9736</v>
+      </c>
+      <c r="BM17" s="3" t="n">
+        <v>16.8052</v>
       </c>
     </row>
     <row r="18">
@@ -7222,16 +7321,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>47.05</v>
+        <v>46.52</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>88756.81379999999</v>
+        <v>87757.00272</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>8756.813799999989</v>
+        <v>7757.002720000004</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.1094601724999999</v>
+        <v>0.09696253400000004</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -7397,6 +7496,9 @@
       </c>
       <c r="BL18" s="3" t="n">
         <v>47.05</v>
+      </c>
+      <c r="BM18" s="3" t="n">
+        <v>46.52</v>
       </c>
     </row>
     <row r="19">
@@ -7422,16 +7524,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>13.9999</v>
+        <v>13.413</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>202533.2773234</v>
+        <v>194042.732358</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>52533.27732339999</v>
+        <v>44042.73235800001</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.3502218488226666</v>
+        <v>0.2936182157200001</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -7591,6 +7693,9 @@
       </c>
       <c r="BL19" s="3" t="n">
         <v>13.9999</v>
+      </c>
+      <c r="BM19" s="3" t="n">
+        <v>13.413</v>
       </c>
     </row>
     <row r="20">
@@ -7616,16 +7721,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.43</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>247592.22229</v>
+        <v>244178.9679</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-2407.777709999995</v>
+        <v>-5821.032099999982</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.009631110839999979</v>
+        <v>-0.02328412839999993</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -7791,6 +7896,9 @@
       </c>
       <c r="BL20" s="3" t="n">
         <v>9.43</v>
+      </c>
+      <c r="BM20" s="3" t="n">
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="21">
@@ -7816,16 +7924,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>112.7556</v>
+        <v>110.6174</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>171304.9601004</v>
-      </c>
-      <c r="H21" s="4" t="n">
-        <v>1304.9601004</v>
-      </c>
-      <c r="I21" s="12" t="n">
-        <v>0.007676235884705881</v>
+        <v>168056.4805066</v>
+      </c>
+      <c r="H21" s="6" t="n">
+        <v>-1943.519493400003</v>
+      </c>
+      <c r="I21" s="13" t="n">
+        <v>-0.01143246760823531</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -7991,6 +8099,9 @@
       </c>
       <c r="BL21" s="3" t="n">
         <v>112.7556</v>
+      </c>
+      <c r="BM21" s="3" t="n">
+        <v>110.6174</v>
       </c>
     </row>
     <row r="22">
@@ -8016,16 +8127,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>43.098</v>
+        <v>42.592</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>66132.15708</v>
+        <v>65355.72032</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>6132.157080000004</v>
+        <v>5355.72032</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.1022026180000001</v>
+        <v>0.08926200533333334</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -8185,6 +8296,9 @@
       </c>
       <c r="BL22" s="3" t="n">
         <v>43.098</v>
+      </c>
+      <c r="BM22" s="3" t="n">
+        <v>42.592</v>
       </c>
     </row>
     <row r="23">
@@ -8210,16 +8324,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>63.4827</v>
+        <v>62.3249</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>172448.6596209</v>
+        <v>169303.5341283</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>22448.6596209</v>
+        <v>19303.5341283</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.149657730806</v>
+        <v>0.128690227522</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -8385,6 +8499,9 @@
       </c>
       <c r="BL23" s="3" t="n">
         <v>63.4827</v>
+      </c>
+      <c r="BM23" s="3" t="n">
+        <v>62.3249</v>
       </c>
     </row>
     <row r="24">
@@ -8410,16 +8527,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>27.7039</v>
+        <v>27.1036</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>100658.9624054</v>
-      </c>
-      <c r="H24" s="4" t="n">
-        <v>658.9624054000014</v>
-      </c>
-      <c r="I24" s="12" t="n">
-        <v>0.006589624054000014</v>
+        <v>98477.8407896</v>
+      </c>
+      <c r="H24" s="6" t="n">
+        <v>-1522.159210400001</v>
+      </c>
+      <c r="I24" s="13" t="n">
+        <v>-0.01522159210400001</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -8579,6 +8696,9 @@
       </c>
       <c r="BL24" s="3" t="n">
         <v>27.7039</v>
+      </c>
+      <c r="BM24" s="3" t="n">
+        <v>27.1036</v>
       </c>
     </row>
     <row r="25">
@@ -8604,16 +8724,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.8526</v>
+        <v>11.7068</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>194639.5332524</v>
+        <v>192245.2531832</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-5360.466747600003</v>
+        <v>-7754.746816800034</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.02680233373800002</v>
+        <v>-0.03877373408400017</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -8776,6 +8896,9 @@
       </c>
       <c r="BL25" s="3" t="n">
         <v>11.8526</v>
+      </c>
+      <c r="BM25" s="3" t="n">
+        <v>11.7068</v>
       </c>
     </row>
     <row r="26">
@@ -8801,16 +8924,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>9.515000000000001</v>
+        <v>9.313499999999999</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>113625.418225</v>
+        <v>111219.1626525</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>3625.418225000001</v>
+        <v>1219.162652499988</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.03295834750000001</v>
+        <v>0.01108329684090898</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -8973,6 +9096,9 @@
       </c>
       <c r="BL26" s="3" t="n">
         <v>9.515000000000001</v>
+      </c>
+      <c r="BM26" s="3" t="n">
+        <v>9.313499999999999</v>
       </c>
     </row>
     <row r="27">
@@ -8998,16 +9124,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>65.2525</v>
+        <v>64.4315</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>105112.64215</v>
+        <v>103790.12609</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-4887.357850000015</v>
+        <v>-6209.873910000009</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.04443052590909104</v>
+        <v>-0.05645339918181827</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -9173,6 +9299,9 @@
       </c>
       <c r="BL27" s="3" t="n">
         <v>65.2525</v>
+      </c>
+      <c r="BM27" s="3" t="n">
+        <v>64.4315</v>
       </c>
     </row>
     <row r="28">
@@ -9198,16 +9327,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>109.7658</v>
+        <v>107.9814</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>362957.8509306</v>
+        <v>357057.4521798</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-17042.14906939998</v>
+        <v>-22942.54782019998</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.04484776070894732</v>
+        <v>-0.06037512584263152</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -9373,6 +9502,9 @@
       </c>
       <c r="BL28" s="3" t="n">
         <v>109.7658</v>
+      </c>
+      <c r="BM28" s="3" t="n">
+        <v>107.9814</v>
       </c>
     </row>
     <row r="29">
@@ -9398,16 +9530,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.4274</v>
+        <v>12.2198</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>119349.0586622</v>
+        <v>117355.3299194</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>19349.0586622</v>
+        <v>17355.32991939998</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.193490586622</v>
+        <v>0.1735532991939998</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -9567,6 +9699,9 @@
       </c>
       <c r="BL29" s="3" t="n">
         <v>12.4274</v>
+      </c>
+      <c r="BM29" s="3" t="n">
+        <v>12.2198</v>
       </c>
     </row>
     <row r="30">
@@ -9592,16 +9727,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>16.8079</v>
+        <v>16.5323</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>124308.8921019</v>
+        <v>122270.5928103</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>24308.8921019</v>
+        <v>22270.59281029999</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.243088921019</v>
+        <v>0.2227059281029999</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -9761,6 +9896,9 @@
       </c>
       <c r="BL30" s="3" t="n">
         <v>16.8079</v>
+      </c>
+      <c r="BM30" s="3" t="n">
+        <v>16.5323</v>
       </c>
     </row>
     <row r="31">
@@ -9786,16 +9924,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>414.2588</v>
+        <v>406.6306</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>110225.981504</v>
+        <v>108196.270048</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>10225.981504</v>
+        <v>8196.270047999991</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.10225981504</v>
+        <v>0.08196270047999991</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -9958,6 +10096,9 @@
       </c>
       <c r="BL31" s="3" t="n">
         <v>414.2588</v>
+      </c>
+      <c r="BM31" s="3" t="n">
+        <v>406.6306</v>
       </c>
     </row>
     <row r="32">
@@ -9983,16 +10124,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.67</v>
+        <v>10.51</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>225563.3732</v>
+        <v>222180.9796</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>25563.3732</v>
+        <v>22180.97959999999</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.127816866</v>
+        <v>0.110904898</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -10158,6 +10299,9 @@
       </c>
       <c r="BL32" s="3" t="n">
         <v>10.67</v>
+      </c>
+      <c r="BM32" s="3" t="n">
+        <v>10.51</v>
       </c>
     </row>
     <row r="33">
@@ -10183,16 +10327,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>18.92</v>
+        <v>18.71</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>67802.4688</v>
+        <v>67049.9044</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>7802.468800000002</v>
+        <v>7049.904399999999</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.1300411466666667</v>
+        <v>0.1174984066666667</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -10352,6 +10496,9 @@
       </c>
       <c r="BL33" s="3" t="n">
         <v>18.92</v>
+      </c>
+      <c r="BM33" s="3" t="n">
+        <v>18.71</v>
       </c>
     </row>
     <row r="34">
@@ -10377,16 +10524,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>215.049</v>
+        <v>212.26</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>75596.390019</v>
+        <v>74615.97005999999</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-4403.609981000001</v>
+        <v>-5384.029940000008</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.05504512476250002</v>
+        <v>-0.0673003742500001</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -10549,6 +10696,9 @@
       </c>
       <c r="BL34" s="3" t="n">
         <v>215.049</v>
+      </c>
+      <c r="BM34" s="3" t="n">
+        <v>212.26</v>
       </c>
     </row>
     <row r="35">
@@ -10574,16 +10724,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>14.92</v>
+        <v>14.69</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>106460.51116</v>
+        <v>104819.36387</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>6460.511159999995</v>
+        <v>4819.363869999986</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.06460511159999995</v>
+        <v>0.04819363869999987</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -10746,6 +10896,9 @@
       </c>
       <c r="BL35" s="3" t="n">
         <v>14.92</v>
+      </c>
+      <c r="BM35" s="3" t="n">
+        <v>14.69</v>
       </c>
     </row>
     <row r="36">
@@ -10771,16 +10924,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>372.8502</v>
+        <v>368.3554</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>173638.5752412</v>
+        <v>171545.3199124</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>23638.57524119999</v>
+        <v>21545.31991239998</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1575905016079999</v>
+        <v>0.1436354660826665</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -10943,6 +11096,9 @@
       </c>
       <c r="BL36" s="3" t="n">
         <v>372.8502</v>
+      </c>
+      <c r="BM36" s="3" t="n">
+        <v>368.3554</v>
       </c>
     </row>
     <row r="37">
@@ -10968,16 +11124,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>16.694</v>
+        <v>16.565</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>62817.668966</v>
+        <v>62332.25628500001</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>12817.668966</v>
+        <v>12332.25628500001</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.25635337932</v>
+        <v>0.2466451257000002</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -11140,6 +11296,9 @@
       </c>
       <c r="BL37" s="3" t="n">
         <v>16.694</v>
+      </c>
+      <c r="BM37" s="3" t="n">
+        <v>16.565</v>
       </c>
     </row>
     <row r="38">
@@ -11165,16 +11324,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>14.4324</v>
+        <v>14.1655</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>86312.7084168</v>
+        <v>84716.517771</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>6312.7084168</v>
+        <v>4716.517770999999</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.07890885521</v>
+        <v>0.05895647213749999</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -11334,6 +11493,9 @@
       </c>
       <c r="BL38" s="3" t="n">
         <v>14.4324</v>
+      </c>
+      <c r="BM38" s="3" t="n">
+        <v>14.1655</v>
       </c>
     </row>
     <row r="39">
@@ -11359,16 +11521,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1023.5507</v>
+        <v>1022.3234</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51055.7324667</v>
+        <v>50994.5135154</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1055.732466699999</v>
+        <v>994.5135154000018</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.02111464933399999</v>
+        <v>0.01989027030800004</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -11528,6 +11690,9 @@
       </c>
       <c r="BL39" s="3" t="n">
         <v>1023.5507</v>
+      </c>
+      <c r="BM39" s="3" t="n">
+        <v>1022.3234</v>
       </c>
     </row>
     <row r="40">
@@ -11553,16 +11718,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>21.9002</v>
+        <v>21.5332</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>110399.4995054</v>
+        <v>108549.4425964</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>10399.4995054</v>
+        <v>8549.442596400011</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.103994995054</v>
+        <v>0.08549442596400011</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -11725,6 +11890,9 @@
       </c>
       <c r="BL40" s="3" t="n">
         <v>21.9002</v>
+      </c>
+      <c r="BM40" s="3" t="n">
+        <v>21.5332</v>
       </c>
     </row>
     <row r="41">
@@ -11737,13 +11905,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4954844.2160715</v>
+        <v>4885303.4984155</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>484844.2160714999</v>
+        <v>415303.4984154999</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1084662675775168</v>
+        <v>0.09290906004821027</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-07-10
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -483,9 +483,9 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-09 06:02 IST</t>
+          <t>Generated: 2026-07-10 06:01 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4885303.4984155</v>
+        <v>4956779.4405086</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>415303.4984154999</v>
+        <v>486779.4405086003</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.09290906004821027</v>
+        <v>0.1088992036931992</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>539316.0028152466</v>
+        <v>541778.9984207153</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-51466.01718475344</v>
+        <v>-49003.02157928469</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.0871150702669547</v>
+        <v>-0.08294602733387973</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5424619.501230747</v>
+        <v>5498558.438929316</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>363837.481230747</v>
+        <v>437776.4189293161</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.07189352945708319</v>
+        <v>0.08650370974273185</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-07-09</t>
+          <t>Last snapshot: 2026-07-10</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BL19"/>
+  <dimension ref="A1:BM19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -683,6 +683,7 @@
     <col width="21" customWidth="1" min="62" max="62"/>
     <col width="21" customWidth="1" min="63" max="63"/>
     <col width="21" customWidth="1" min="64" max="64"/>
+    <col width="21" customWidth="1" min="65" max="65"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1006,6 +1007,11 @@
           <t>2026-07-09</t>
         </is>
       </c>
+      <c r="BM1" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1025,13 +1031,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>528.75</v>
+        <v>532.3499755859375</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>42300</v>
+        <v>42587.998046875</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>-1517.510000000002</v>
+        <v>-1229.511953125002</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1200,6 +1206,9 @@
       </c>
       <c r="BL2" s="3" t="n">
         <v>528.75</v>
+      </c>
+      <c r="BM2" s="3" t="n">
+        <v>532.3499755859375</v>
       </c>
     </row>
     <row r="3">
@@ -1247,13 +1256,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1332.800048828125</v>
+        <v>1325</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>26656.0009765625</v>
+        <v>26500</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-5448.579023437502</v>
+        <v>-5604.580000000002</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1425,6 +1434,9 @@
       </c>
       <c r="BL4" s="3" t="n">
         <v>1332.800048828125</v>
+      </c>
+      <c r="BM4" s="3" t="n">
+        <v>1325</v>
       </c>
     </row>
     <row r="5">
@@ -1445,13 +1457,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>645.5999755859375</v>
+        <v>645.2000122070312</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>12911.99951171875</v>
+        <v>12904.00024414062</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1301.10048828125</v>
+        <v>-1309.099755859375</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1623,6 +1635,9 @@
       </c>
       <c r="BL5" s="3" t="n">
         <v>645.5999755859375</v>
+      </c>
+      <c r="BM5" s="3" t="n">
+        <v>645.2000122070312</v>
       </c>
     </row>
     <row r="6">
@@ -1643,13 +1658,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>359</v>
+        <v>367.4500122070312</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>14360</v>
+        <v>14698.00048828125</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-3142.240000000002</v>
+        <v>-2804.239511718752</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1821,6 +1836,9 @@
       </c>
       <c r="BL6" s="3" t="n">
         <v>359</v>
+      </c>
+      <c r="BM6" s="3" t="n">
+        <v>367.4500122070312</v>
       </c>
     </row>
     <row r="7">
@@ -1841,13 +1859,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>237.25</v>
+        <v>238.4199981689453</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>23725</v>
+        <v>23841.99981689453</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-2708.82</v>
+        <v>-2591.820183105468</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -2019,6 +2037,9 @@
       </c>
       <c r="BL7" s="3" t="n">
         <v>237.25</v>
+      </c>
+      <c r="BM7" s="3" t="n">
+        <v>238.4199981689453</v>
       </c>
     </row>
     <row r="8">
@@ -2245,6 +2266,9 @@
       <c r="BL9" s="3" t="n">
         <v>17.10000038146973</v>
       </c>
+      <c r="BM9" s="3" t="n">
+        <v>17.10000038146973</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2264,13 +2288,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>427.6000061035156</v>
+        <v>423.3500061035156</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>42760.00061035156</v>
+        <v>42335.00061035156</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-8738.479389648441</v>
+        <v>-9163.479389648441</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -2442,6 +2466,9 @@
       </c>
       <c r="BL10" s="3" t="n">
         <v>427.6000061035156</v>
+      </c>
+      <c r="BM10" s="3" t="n">
+        <v>423.3500061035156</v>
       </c>
     </row>
     <row r="11">
@@ -2462,13 +2489,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>10.89999961853027</v>
+        <v>10.07999992370605</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>10899.99961853027</v>
+        <v>10079.99992370605</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>1058.789618530274</v>
+        <v>238.7899237060556</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -2640,6 +2667,9 @@
       </c>
       <c r="BL11" s="3" t="n">
         <v>10.89999961853027</v>
+      </c>
+      <c r="BM11" s="3" t="n">
+        <v>10.07999992370605</v>
       </c>
     </row>
     <row r="12">
@@ -2660,13 +2690,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2628.300048828125</v>
+        <v>2687.89990234375</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>26283.00048828125</v>
+        <v>26878.9990234375</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-1440.24951171875</v>
+        <v>-844.2509765625</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -2838,6 +2868,9 @@
       </c>
       <c r="BL12" s="3" t="n">
         <v>2628.300048828125</v>
+      </c>
+      <c r="BM12" s="3" t="n">
+        <v>2687.89990234375</v>
       </c>
     </row>
     <row r="13">
@@ -2858,13 +2891,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>53.56999969482422</v>
+        <v>54.09999847412109</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>32141.99981689453</v>
+        <v>32459.99908447266</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-2889.760183105471</v>
+        <v>-2571.760915527346</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -3036,6 +3069,9 @@
       </c>
       <c r="BL13" s="3" t="n">
         <v>53.56999969482422</v>
+      </c>
+      <c r="BM13" s="3" t="n">
+        <v>54.09999847412109</v>
       </c>
     </row>
     <row r="14">
@@ -3056,13 +3092,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>708.4000244140625</v>
+        <v>723.0499877929688</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>35420.00122070312</v>
+        <v>36152.49938964844</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-7042.508779296877</v>
+        <v>-6310.010610351565</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -3234,6 +3270,9 @@
       </c>
       <c r="BL14" s="3" t="n">
         <v>708.4000244140625</v>
+      </c>
+      <c r="BM14" s="3" t="n">
+        <v>723.0499877929688</v>
       </c>
     </row>
     <row r="15">
@@ -3308,13 +3347,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>538.9500122070312</v>
+        <v>556.7000122070312</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>26947.50061035156</v>
+        <v>27835.00061035156</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>5192.970610351564</v>
+        <v>6080.470610351564</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -3486,6 +3525,9 @@
       </c>
       <c r="BL17" s="3" t="n">
         <v>538.9500122070312</v>
+      </c>
+      <c r="BM17" s="3" t="n">
+        <v>556.7000122070312</v>
       </c>
     </row>
     <row r="18">
@@ -3506,13 +3548,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>374.8999938964844</v>
+        <v>380.8500061035156</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>37489.99938964844</v>
+        <v>38085.00061035156</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-9150.820610351562</v>
+        <v>-8555.819389648437</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -3684,6 +3726,9 @@
       </c>
       <c r="BL18" s="3" t="n">
         <v>374.8999938964844</v>
+      </c>
+      <c r="BM18" s="3" t="n">
+        <v>380.8500061035156</v>
       </c>
     </row>
     <row r="19">
@@ -3696,10 +3741,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>539316.0028152466</v>
+        <v>541778.9984207153</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-51466.01718475343</v>
+        <v>-49003.02157928468</v>
       </c>
     </row>
   </sheetData>
@@ -3713,7 +3758,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BM41"/>
+  <dimension ref="A1:BN41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3724,7 +3769,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
@@ -3781,6 +3826,7 @@
     <col width="13" customWidth="1" min="63" max="63"/>
     <col width="13" customWidth="1" min="64" max="64"/>
     <col width="13" customWidth="1" min="65" max="65"/>
+    <col width="13" customWidth="1" min="66" max="66"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4109,6 +4155,11 @@
           <t>2026-07-09</t>
         </is>
       </c>
+      <c r="BN1" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -4133,16 +4184,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>56.7992</v>
+        <v>57.1723</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>63756.0796144</v>
+        <v>64174.8776486</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>13756.0796144</v>
+        <v>14174.8776486</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.275121592288</v>
+        <v>0.283497552972</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -4311,6 +4362,9 @@
       </c>
       <c r="BM2" s="3" t="n">
         <v>56.7992</v>
+      </c>
+      <c r="BN2" s="3" t="n">
+        <v>57.1723</v>
       </c>
     </row>
     <row r="3">
@@ -4336,16 +4390,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.4644</v>
+        <v>25.5926</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>62520.52591720001</v>
+        <v>62835.28422380001</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>2520.525917200008</v>
+        <v>2835.284223800008</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.0420087652866668</v>
+        <v>0.04725473706333348</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -4508,6 +4562,9 @@
       </c>
       <c r="BM3" s="3" t="n">
         <v>25.4644</v>
+      </c>
+      <c r="BN3" s="3" t="n">
+        <v>25.5926</v>
       </c>
     </row>
     <row r="4">
@@ -4533,16 +4590,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.07</v>
+        <v>12.18</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>231817.54251</v>
+        <v>233930.21274</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>51817.54251000003</v>
+        <v>53930.21274000002</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.2878752361666668</v>
+        <v>0.2996122930000001</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -4705,6 +4762,9 @@
       </c>
       <c r="BM4" s="3" t="n">
         <v>12.07</v>
+      </c>
+      <c r="BN4" s="3" t="n">
+        <v>12.18</v>
       </c>
     </row>
     <row r="5">
@@ -4730,16 +4790,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.373699999999999</v>
+        <v>9.403600000000001</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>172045.7146856</v>
+        <v>172594.5019168</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-37954.28531440001</v>
+        <v>-37405.49808319999</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1807346919733334</v>
+        <v>-0.1781214194438095</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -4902,6 +4962,9 @@
       </c>
       <c r="BM5" s="3" t="n">
         <v>9.373699999999999</v>
+      </c>
+      <c r="BN5" s="3" t="n">
+        <v>9.403600000000001</v>
       </c>
     </row>
     <row r="6">
@@ -4927,16 +4990,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>11.7795</v>
+        <v>11.85</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>49815.2345715</v>
-      </c>
-      <c r="H6" s="6" t="n">
-        <v>-184.7654285000026</v>
-      </c>
-      <c r="I6" s="13" t="n">
-        <v>-0.003695308570000052</v>
+        <v>50113.37745</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>113.37745</v>
+      </c>
+      <c r="I6" s="12" t="n">
+        <v>0.002267548999999999</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -5105,6 +5168,9 @@
       </c>
       <c r="BM6" s="3" t="n">
         <v>11.7795</v>
+      </c>
+      <c r="BN6" s="3" t="n">
+        <v>11.85</v>
       </c>
     </row>
     <row r="7">
@@ -5130,16 +5196,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>34.1904</v>
+        <v>34.4039</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>75425.39001599999</v>
+        <v>75896.379556</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>15425.39001599999</v>
+        <v>15896.379556</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2570898335999998</v>
+        <v>0.2649396592666667</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -5302,6 +5368,9 @@
       </c>
       <c r="BM7" s="3" t="n">
         <v>34.1904</v>
+      </c>
+      <c r="BN7" s="3" t="n">
+        <v>34.4039</v>
       </c>
     </row>
     <row r="8">
@@ -5327,16 +5396,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>33.2286</v>
+        <v>33.7817</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>53318.3789598</v>
+        <v>54205.8793481</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>3318.3789598</v>
+        <v>4205.879348100003</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.066367579196</v>
+        <v>0.08411758696200006</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -5505,6 +5574,9 @@
       </c>
       <c r="BM8" s="3" t="n">
         <v>33.2286</v>
+      </c>
+      <c r="BN8" s="3" t="n">
+        <v>33.7817</v>
       </c>
     </row>
     <row r="9">
@@ -5530,16 +5602,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>40.6637</v>
+        <v>42.2188</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>130912.4311341</v>
+        <v>135918.9091884</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>30912.4311341</v>
+        <v>35918.90918839999</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.309124311341</v>
+        <v>0.3591890918839999</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -5702,6 +5774,9 @@
       </c>
       <c r="BM9" s="3" t="n">
         <v>40.6637</v>
+      </c>
+      <c r="BN9" s="3" t="n">
+        <v>42.2188</v>
       </c>
     </row>
     <row r="10">
@@ -5727,16 +5802,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48.0914</v>
+        <v>48.1125</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>136899.8166326</v>
+        <v>136959.8811375</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>36899.81663260001</v>
+        <v>36959.88113749999</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3689981663260001</v>
+        <v>0.3695988113749999</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -5899,6 +5974,9 @@
       </c>
       <c r="BM10" s="3" t="n">
         <v>48.0914</v>
+      </c>
+      <c r="BN10" s="3" t="n">
+        <v>48.1125</v>
       </c>
     </row>
     <row r="11">
@@ -5924,16 +6002,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>104.7936</v>
+        <v>106.0056</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31534.3853184</v>
+        <v>31899.0991464</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1534.385318399996</v>
+        <v>1899.0991464</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.05114617727999988</v>
+        <v>0.06330330487999999</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -6096,6 +6174,9 @@
       </c>
       <c r="BM11" s="3" t="n">
         <v>104.7936</v>
+      </c>
+      <c r="BN11" s="3" t="n">
+        <v>106.0056</v>
       </c>
     </row>
     <row r="12">
@@ -6121,16 +6202,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>226.564</v>
+        <v>228.93</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>105470.526408</v>
+        <v>106571.95146</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>5470.526407999991</v>
+        <v>6571.951459999997</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.05470526407999991</v>
+        <v>0.06571951459999996</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -6299,6 +6380,9 @@
       </c>
       <c r="BM12" s="3" t="n">
         <v>226.564</v>
+      </c>
+      <c r="BN12" s="3" t="n">
+        <v>228.93</v>
       </c>
     </row>
     <row r="13">
@@ -6324,16 +6408,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>20.994</v>
+        <v>21.313</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>243270.17937</v>
+        <v>246966.625365</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>43270.17937</v>
+        <v>46966.62536499999</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.21635089685</v>
+        <v>0.2348331268249999</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -6502,6 +6586,9 @@
       </c>
       <c r="BM13" s="3" t="n">
         <v>20.994</v>
+      </c>
+      <c r="BN13" s="3" t="n">
+        <v>21.313</v>
       </c>
     </row>
     <row r="14">
@@ -6527,16 +6614,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>37.5088</v>
+        <v>37.888</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>135316.9719328</v>
+        <v>136684.976128</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>35316.97193280002</v>
+        <v>36684.97612800001</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.3531697193280002</v>
+        <v>0.3668497612800001</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -6699,6 +6786,9 @@
       </c>
       <c r="BM14" s="3" t="n">
         <v>37.5088</v>
+      </c>
+      <c r="BN14" s="3" t="n">
+        <v>37.888</v>
       </c>
     </row>
     <row r="15">
@@ -6724,16 +6814,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.58</v>
+        <v>11.66</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>112834.90626</v>
+        <v>113614.42202</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>12834.90626</v>
+        <v>13614.42202</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1283490626</v>
+        <v>0.1361442202</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -6902,6 +6992,9 @@
       </c>
       <c r="BM15" s="3" t="n">
         <v>11.58</v>
+      </c>
+      <c r="BN15" s="3" t="n">
+        <v>11.66</v>
       </c>
     </row>
     <row r="16">
@@ -6927,16 +7020,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.2351</v>
+        <v>24.6669</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>138695.7323728</v>
+        <v>141166.8926832</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>38695.7323728</v>
+        <v>41166.89268319999</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.3869573237280001</v>
+        <v>0.4116689268319998</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -7099,6 +7192,9 @@
       </c>
       <c r="BM16" s="3" t="n">
         <v>24.2351</v>
+      </c>
+      <c r="BN16" s="3" t="n">
+        <v>24.6669</v>
       </c>
     </row>
     <row r="17">
@@ -7124,16 +7220,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.8052</v>
+        <v>16.8767</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55558.94909639999</v>
+        <v>55795.33217189999</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5558.949096399992</v>
+        <v>5795.332171899994</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1111789819279999</v>
+        <v>0.1159066434379999</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -7296,6 +7392,9 @@
       </c>
       <c r="BM17" s="3" t="n">
         <v>16.8052</v>
+      </c>
+      <c r="BN17" s="3" t="n">
+        <v>16.8767</v>
       </c>
     </row>
     <row r="18">
@@ -7321,16 +7420,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>46.52</v>
+        <v>46.92</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>87757.00272</v>
+        <v>88511.57712</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>7757.002720000004</v>
+        <v>8511.577120000002</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.09696253400000004</v>
+        <v>0.106394714</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -7499,6 +7598,9 @@
       </c>
       <c r="BM18" s="3" t="n">
         <v>46.52</v>
+      </c>
+      <c r="BN18" s="3" t="n">
+        <v>46.92</v>
       </c>
     </row>
     <row r="19">
@@ -7524,16 +7626,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>13.413</v>
+        <v>13.8131</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>194042.732358</v>
+        <v>199830.8854346</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>44042.73235800001</v>
+        <v>49830.8854346</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.2936182157200001</v>
+        <v>0.3322059028973333</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -7696,6 +7798,9 @@
       </c>
       <c r="BM19" s="3" t="n">
         <v>13.413</v>
+      </c>
+      <c r="BN19" s="3" t="n">
+        <v>13.8131</v>
       </c>
     </row>
     <row r="20">
@@ -7721,16 +7826,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.300000000000001</v>
+        <v>9.44</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>244178.9679</v>
+        <v>247854.78032</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-5821.032099999982</v>
+        <v>-2145.219680000009</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>-0.02328412839999993</v>
+        <v>-0.008580878720000037</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -7899,6 +8004,9 @@
       </c>
       <c r="BM20" s="3" t="n">
         <v>9.300000000000001</v>
+      </c>
+      <c r="BN20" s="3" t="n">
+        <v>9.44</v>
       </c>
     </row>
     <row r="21">
@@ -7924,16 +8032,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>110.6174</v>
+        <v>111.5191</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>168056.4805066</v>
+        <v>169426.3963469</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-1943.519493400003</v>
+        <v>-573.6036530999991</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>-0.01143246760823531</v>
+        <v>-0.003374139135882347</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -8102,6 +8210,9 @@
       </c>
       <c r="BM21" s="3" t="n">
         <v>110.6174</v>
+      </c>
+      <c r="BN21" s="3" t="n">
+        <v>111.5191</v>
       </c>
     </row>
     <row r="22">
@@ -8127,16 +8238,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>42.592</v>
+        <v>42.955</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>65355.72032</v>
+        <v>65912.72929999999</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>5355.72032</v>
+        <v>5912.729299999992</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.08926200533333334</v>
+        <v>0.09854548833333319</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -8299,6 +8410,9 @@
       </c>
       <c r="BM22" s="3" t="n">
         <v>42.592</v>
+      </c>
+      <c r="BN22" s="3" t="n">
+        <v>42.955</v>
       </c>
     </row>
     <row r="23">
@@ -8324,16 +8438,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>62.3249</v>
+        <v>63.0612</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>169303.5341283</v>
+        <v>171303.6687804</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>19303.5341283</v>
+        <v>21303.66878040001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.128690227522</v>
+        <v>0.1420244585360001</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -8502,6 +8616,9 @@
       </c>
       <c r="BM23" s="3" t="n">
         <v>62.3249</v>
+      </c>
+      <c r="BN23" s="3" t="n">
+        <v>63.0612</v>
       </c>
     </row>
     <row r="24">
@@ -8527,16 +8644,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>27.1036</v>
+        <v>27.3285</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>98477.8407896</v>
+        <v>99294.98930099999</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>-1522.159210400001</v>
+        <v>-705.0106990000058</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>-0.01522159210400001</v>
+        <v>-0.007050106990000058</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -8699,6 +8816,9 @@
       </c>
       <c r="BM24" s="3" t="n">
         <v>27.1036</v>
+      </c>
+      <c r="BN24" s="3" t="n">
+        <v>27.3285</v>
       </c>
     </row>
     <row r="25">
@@ -8724,16 +8844,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11.7068</v>
+        <v>12.0694</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>192245.2531832</v>
+        <v>198199.7521756</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-7754.746816800034</v>
+        <v>-1800.247824400023</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>-0.03877373408400017</v>
+        <v>-0.009001239122000116</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -8899,6 +9019,9 @@
       </c>
       <c r="BM25" s="3" t="n">
         <v>11.7068</v>
+      </c>
+      <c r="BN25" s="3" t="n">
+        <v>12.0694</v>
       </c>
     </row>
     <row r="26">
@@ -8924,16 +9047,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>9.313499999999999</v>
+        <v>9.5106</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>111219.1626525</v>
+        <v>113572.874679</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>1219.162652499988</v>
+        <v>3572.874679</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.01108329684090898</v>
+        <v>0.0324806789</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -9099,6 +9222,9 @@
       </c>
       <c r="BM26" s="3" t="n">
         <v>9.313499999999999</v>
+      </c>
+      <c r="BN26" s="3" t="n">
+        <v>9.5106</v>
       </c>
     </row>
     <row r="27">
@@ -9124,16 +9250,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>64.4315</v>
+        <v>65.92959999999999</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>103790.12609</v>
+        <v>106203.355456</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-6209.873910000009</v>
+        <v>-3796.64454400001</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.05645339918181827</v>
+        <v>-0.03451495040000009</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -9302,6 +9428,9 @@
       </c>
       <c r="BM27" s="3" t="n">
         <v>64.4315</v>
+      </c>
+      <c r="BN27" s="3" t="n">
+        <v>65.92959999999999</v>
       </c>
     </row>
     <row r="28">
@@ -9327,16 +9456,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>107.9814</v>
+        <v>111.2113</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>357057.4521798</v>
+        <v>367737.6236241</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-22942.54782019998</v>
+        <v>-12262.3763759</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.06037512584263152</v>
+        <v>-0.03226941151552631</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -9505,6 +9634,9 @@
       </c>
       <c r="BM28" s="3" t="n">
         <v>107.9814</v>
+      </c>
+      <c r="BN28" s="3" t="n">
+        <v>111.2113</v>
       </c>
     </row>
     <row r="29">
@@ -9530,16 +9662,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.2198</v>
+        <v>12.2003</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>117355.3299194</v>
+        <v>117168.0577109</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>17355.32991939998</v>
+        <v>17168.0577109</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.1735532991939998</v>
+        <v>0.171680577109</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -9702,6 +9834,9 @@
       </c>
       <c r="BM29" s="3" t="n">
         <v>12.2198</v>
+      </c>
+      <c r="BN29" s="3" t="n">
+        <v>12.2003</v>
       </c>
     </row>
     <row r="30">
@@ -9727,16 +9862,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>16.5323</v>
+        <v>16.791</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>122270.5928103</v>
+        <v>124183.902051</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>22270.59281029999</v>
+        <v>24183.902051</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.2227059281029999</v>
+        <v>0.24183902051</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -9899,6 +10034,9 @@
       </c>
       <c r="BM30" s="3" t="n">
         <v>16.5323</v>
+      </c>
+      <c r="BN30" s="3" t="n">
+        <v>16.791</v>
       </c>
     </row>
     <row r="31">
@@ -9924,16 +10062,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>406.6306</v>
+        <v>410.4736</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>108196.270048</v>
+        <v>109218.815488</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>8196.270047999991</v>
+        <v>9218.815487999993</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.08196270047999991</v>
+        <v>0.09218815487999993</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -10099,6 +10237,9 @@
       </c>
       <c r="BM31" s="3" t="n">
         <v>406.6306</v>
+      </c>
+      <c r="BN31" s="3" t="n">
+        <v>410.4736</v>
       </c>
     </row>
     <row r="32">
@@ -10124,16 +10265,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.51</v>
+        <v>10.62</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>222180.9796</v>
+        <v>224506.3752</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>22180.97959999999</v>
+        <v>24506.37519999998</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.110904898</v>
+        <v>0.1225318759999999</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -10302,6 +10443,9 @@
       </c>
       <c r="BM32" s="3" t="n">
         <v>10.51</v>
+      </c>
+      <c r="BN32" s="3" t="n">
+        <v>10.62</v>
       </c>
     </row>
     <row r="33">
@@ -10327,16 +10471,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>18.71</v>
+        <v>19</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>67049.9044</v>
+        <v>68089.16</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>7049.904399999999</v>
+        <v>8089.160000000003</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.1174984066666667</v>
+        <v>0.1348193333333334</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -10499,6 +10643,9 @@
       </c>
       <c r="BM33" s="3" t="n">
         <v>18.71</v>
+      </c>
+      <c r="BN33" s="3" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="34">
@@ -10524,16 +10671,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>212.26</v>
+        <v>214.6803</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>74615.97005999999</v>
+        <v>75466.7805393</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-5384.029940000008</v>
+        <v>-4533.219460699998</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.0673003742500001</v>
+        <v>-0.05666524325874998</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -10699,6 +10846,9 @@
       </c>
       <c r="BM34" s="3" t="n">
         <v>212.26</v>
+      </c>
+      <c r="BN34" s="3" t="n">
+        <v>214.6803</v>
       </c>
     </row>
     <row r="35">
@@ -10724,16 +10874,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>14.69</v>
+        <v>15.01</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>104819.36387</v>
+        <v>107102.69923</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>4819.363869999986</v>
+        <v>7102.699229999998</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.04819363869999987</v>
+        <v>0.07102699229999998</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -10899,6 +11049,9 @@
       </c>
       <c r="BM35" s="3" t="n">
         <v>14.69</v>
+      </c>
+      <c r="BN35" s="3" t="n">
+        <v>15.01</v>
       </c>
     </row>
     <row r="36">
@@ -10924,16 +11077,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>368.3554</v>
+        <v>373.7828</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>171545.3199124</v>
+        <v>174072.8926568</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>21545.31991239998</v>
+        <v>24072.89265680002</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1436354660826665</v>
+        <v>0.1604859510453334</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -11099,6 +11252,9 @@
       </c>
       <c r="BM36" s="3" t="n">
         <v>368.3554</v>
+      </c>
+      <c r="BN36" s="3" t="n">
+        <v>373.7828</v>
       </c>
     </row>
     <row r="37">
@@ -11124,16 +11280,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>16.565</v>
+        <v>16.819</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>62332.25628500001</v>
+        <v>63288.030091</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>12332.25628500001</v>
+        <v>13288.030091</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.2466451257000002</v>
+        <v>0.26576060182</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -11299,6 +11455,9 @@
       </c>
       <c r="BM37" s="3" t="n">
         <v>16.565</v>
+      </c>
+      <c r="BN37" s="3" t="n">
+        <v>16.819</v>
       </c>
     </row>
     <row r="38">
@@ -11324,16 +11483,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>14.1655</v>
+        <v>14.2955</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>84716.517771</v>
+        <v>85493.980431</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>4716.517770999999</v>
+        <v>5493.980431000004</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.05895647213749999</v>
+        <v>0.06867475538750005</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -11496,6 +11655,9 @@
       </c>
       <c r="BM38" s="3" t="n">
         <v>14.1655</v>
+      </c>
+      <c r="BN38" s="3" t="n">
+        <v>14.2955</v>
       </c>
     </row>
     <row r="39">
@@ -11521,16 +11683,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1022.3234</v>
+        <v>1022.5379</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>50994.5135154</v>
+        <v>51005.2129899</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>994.5135154000018</v>
+        <v>1005.212989899999</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.01989027030800004</v>
+        <v>0.02010425979799998</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -11693,6 +11855,9 @@
       </c>
       <c r="BM39" s="3" t="n">
         <v>1022.3234</v>
+      </c>
+      <c r="BN39" s="3" t="n">
+        <v>1022.5379</v>
       </c>
     </row>
     <row r="40">
@@ -11718,16 +11883,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>21.5332</v>
+        <v>21.8222</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>108549.4425964</v>
+        <v>110006.2993994</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>8549.442596400011</v>
+        <v>10006.2993994</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.08549442596400011</v>
+        <v>0.100062993994</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -11893,6 +12058,9 @@
       </c>
       <c r="BM40" s="3" t="n">
         <v>21.5332</v>
+      </c>
+      <c r="BN40" s="3" t="n">
+        <v>21.8222</v>
       </c>
     </row>
     <row r="41">
@@ -11905,13 +12073,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4885303.4984155</v>
+        <v>4956779.4405086</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>415303.4984154999</v>
+        <v>486779.4405086</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.09290906004821027</v>
+        <v>0.1088992036931991</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-07-11
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-10 06:01 IST</t>
+          <t>Generated: 2026-07-11 05:11 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4956779.4405086</v>
+        <v>5008989.9490267</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>486779.4405086003</v>
+        <v>538989.9490267001</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1088992036931992</v>
+        <v>0.1205794069410962</v>
       </c>
     </row>
     <row r="6">
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>541778.9984207153</v>
+        <v>543358.5018615723</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-49003.02157928469</v>
+        <v>-47423.51813842775</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.08294602733387973</v>
+        <v>-0.08027244657585847</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5498558.438929316</v>
+        <v>5552348.450888272</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>437776.4189293161</v>
+        <v>491566.4308882728</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.08650370974273185</v>
+        <v>0.09713250421488671</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-07-10</t>
+          <t>Last snapshot: 2026-07-11</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BM19"/>
+  <dimension ref="A1:BN19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -684,6 +684,7 @@
     <col width="21" customWidth="1" min="63" max="63"/>
     <col width="21" customWidth="1" min="64" max="64"/>
     <col width="21" customWidth="1" min="65" max="65"/>
+    <col width="21" customWidth="1" min="66" max="66"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1012,6 +1013,11 @@
           <t>2026-07-10</t>
         </is>
       </c>
+      <c r="BN1" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1031,13 +1037,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>532.3499755859375</v>
+        <v>545.2000122070312</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>42587.998046875</v>
+        <v>43616.0009765625</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>-1229.511953125002</v>
+        <v>-201.509023437502</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1209,6 +1215,9 @@
       </c>
       <c r="BM2" s="3" t="n">
         <v>532.3499755859375</v>
+      </c>
+      <c r="BN2" s="3" t="n">
+        <v>545.2000122070312</v>
       </c>
     </row>
     <row r="3">
@@ -1256,13 +1265,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1325</v>
+        <v>1333.800048828125</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>26500</v>
+        <v>26676.0009765625</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-5604.580000000002</v>
+        <v>-5428.579023437502</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1437,6 +1446,9 @@
       </c>
       <c r="BM4" s="3" t="n">
         <v>1325</v>
+      </c>
+      <c r="BN4" s="3" t="n">
+        <v>1333.800048828125</v>
       </c>
     </row>
     <row r="5">
@@ -1457,13 +1469,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>645.2000122070312</v>
+        <v>643.2999877929688</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>12904.00024414062</v>
+        <v>12865.99975585938</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1309.099755859375</v>
+        <v>-1347.100244140625</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1638,6 +1650,9 @@
       </c>
       <c r="BM5" s="3" t="n">
         <v>645.2000122070312</v>
+      </c>
+      <c r="BN5" s="3" t="n">
+        <v>643.2999877929688</v>
       </c>
     </row>
     <row r="6">
@@ -1658,13 +1673,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>367.4500122070312</v>
+        <v>368.6499938964844</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>14698.00048828125</v>
+        <v>14745.99975585938</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2804.239511718752</v>
+        <v>-2756.240244140627</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1839,6 +1854,9 @@
       </c>
       <c r="BM6" s="3" t="n">
         <v>367.4500122070312</v>
+      </c>
+      <c r="BN6" s="3" t="n">
+        <v>368.6499938964844</v>
       </c>
     </row>
     <row r="7">
@@ -1859,13 +1877,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>238.4199981689453</v>
+        <v>239.6399993896484</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>23841.99981689453</v>
+        <v>23963.99993896484</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-2591.820183105468</v>
+        <v>-2469.820061035156</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -2040,6 +2058,9 @@
       </c>
       <c r="BM7" s="3" t="n">
         <v>238.4199981689453</v>
+      </c>
+      <c r="BN7" s="3" t="n">
+        <v>239.6399993896484</v>
       </c>
     </row>
     <row r="8">
@@ -2087,13 +2108,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>17.10000038146973</v>
+        <v>17.02000045776367</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>25650.00057220459</v>
+        <v>25530.00068664551</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-5400.169427795408</v>
+        <v>-5520.16931335449</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -2268,6 +2289,9 @@
       </c>
       <c r="BM9" s="3" t="n">
         <v>17.10000038146973</v>
+      </c>
+      <c r="BN9" s="3" t="n">
+        <v>17.02000045776367</v>
       </c>
     </row>
     <row r="10">
@@ -2288,13 +2312,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>423.3500061035156</v>
+        <v>424.9500122070312</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>42335.00061035156</v>
+        <v>42495.00122070312</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-9163.479389648441</v>
+        <v>-9003.478779296878</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -2469,6 +2493,9 @@
       </c>
       <c r="BM10" s="3" t="n">
         <v>423.3500061035156</v>
+      </c>
+      <c r="BN10" s="3" t="n">
+        <v>424.9500122070312</v>
       </c>
     </row>
     <row r="11">
@@ -2489,13 +2516,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>10.07999992370605</v>
+        <v>9.989999771118164</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>10079.99992370605</v>
+        <v>9989.999771118164</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>238.7899237060556</v>
+        <v>148.7897711181649</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -2670,6 +2697,9 @@
       </c>
       <c r="BM11" s="3" t="n">
         <v>10.07999992370605</v>
+      </c>
+      <c r="BN11" s="3" t="n">
+        <v>9.989999771118164</v>
       </c>
     </row>
     <row r="12">
@@ -2690,13 +2720,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2687.89990234375</v>
+        <v>2693.800048828125</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>26878.9990234375</v>
+        <v>26938.00048828125</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-844.2509765625</v>
+        <v>-785.24951171875</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -2871,6 +2901,9 @@
       </c>
       <c r="BM12" s="3" t="n">
         <v>2687.89990234375</v>
+      </c>
+      <c r="BN12" s="3" t="n">
+        <v>2693.800048828125</v>
       </c>
     </row>
     <row r="13">
@@ -2891,13 +2924,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>54.09999847412109</v>
+        <v>53.91999816894531</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>32459.99908447266</v>
+        <v>32351.99890136719</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-2571.760915527346</v>
+        <v>-2679.761098632815</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -3072,6 +3105,9 @@
       </c>
       <c r="BM13" s="3" t="n">
         <v>54.09999847412109</v>
+      </c>
+      <c r="BN13" s="3" t="n">
+        <v>53.91999816894531</v>
       </c>
     </row>
     <row r="14">
@@ -3092,13 +3128,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>723.0499877929688</v>
+        <v>721.0499877929688</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>36152.49938964844</v>
+        <v>36052.49938964844</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-6310.010610351565</v>
+        <v>-6410.010610351565</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -3273,6 +3309,9 @@
       </c>
       <c r="BM14" s="3" t="n">
         <v>723.0499877929688</v>
+      </c>
+      <c r="BN14" s="3" t="n">
+        <v>721.0499877929688</v>
       </c>
     </row>
     <row r="15">
@@ -3347,13 +3386,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>556.7000122070312</v>
+        <v>564.6500244140625</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>27835.00061035156</v>
+        <v>28232.50122070312</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>6080.470610351564</v>
+        <v>6477.971220703126</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -3528,6 +3567,9 @@
       </c>
       <c r="BM17" s="3" t="n">
         <v>556.7000122070312</v>
+      </c>
+      <c r="BN17" s="3" t="n">
+        <v>564.6500244140625</v>
       </c>
     </row>
     <row r="18">
@@ -3548,13 +3590,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>380.8500061035156</v>
+        <v>381.2999877929688</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>38085.00061035156</v>
+        <v>38129.99877929688</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-8555.819389648437</v>
+        <v>-8510.821220703125</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -3729,6 +3771,9 @@
       </c>
       <c r="BM18" s="3" t="n">
         <v>380.8500061035156</v>
+      </c>
+      <c r="BN18" s="3" t="n">
+        <v>381.2999877929688</v>
       </c>
     </row>
     <row r="19">
@@ -3741,10 +3786,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>541778.9984207153</v>
+        <v>543358.5018615723</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-49003.02157928468</v>
+        <v>-47423.51813842775</v>
       </c>
     </row>
   </sheetData>
@@ -3758,7 +3803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BN41"/>
+  <dimension ref="A1:BO41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3769,7 +3814,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
@@ -3827,6 +3872,7 @@
     <col width="13" customWidth="1" min="64" max="64"/>
     <col width="13" customWidth="1" min="65" max="65"/>
     <col width="13" customWidth="1" min="66" max="66"/>
+    <col width="13" customWidth="1" min="67" max="67"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4160,6 +4206,11 @@
           <t>2026-07-10</t>
         </is>
       </c>
+      <c r="BO1" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -4184,16 +4235,16 @@
         <v>50000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>57.1723</v>
+        <v>57.4457</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>64174.8776486</v>
+        <v>64481.7642274</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>14174.8776486</v>
+        <v>14481.7642274</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>0.283497552972</v>
+        <v>0.289635284548</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>56.7408</v>
@@ -4365,6 +4416,9 @@
       </c>
       <c r="BN2" s="3" t="n">
         <v>57.1723</v>
+      </c>
+      <c r="BO2" s="3" t="n">
+        <v>57.4457</v>
       </c>
     </row>
     <row r="3">
@@ -4390,16 +4444,16 @@
         <v>60000</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>25.5926</v>
+        <v>25.7751</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>62835.28422380001</v>
+        <v>63283.3605963</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>2835.284223800008</v>
+        <v>3283.360596300001</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.04725473706333348</v>
+        <v>0.05472267660500001</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>25.2746</v>
@@ -4565,6 +4619,9 @@
       </c>
       <c r="BN3" s="3" t="n">
         <v>25.5926</v>
+      </c>
+      <c r="BO3" s="3" t="n">
+        <v>25.7751</v>
       </c>
     </row>
     <row r="4">
@@ -4590,16 +4647,16 @@
         <v>180000</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>12.18</v>
+        <v>12.22</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>233930.21274</v>
+        <v>234698.45646</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>53930.21274000002</v>
+        <v>54698.45646000002</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>0.2996122930000001</v>
+        <v>0.3038803136666667</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>12.93</v>
@@ -4765,6 +4822,9 @@
       </c>
       <c r="BN4" s="3" t="n">
         <v>12.18</v>
+      </c>
+      <c r="BO4" s="3" t="n">
+        <v>12.22</v>
       </c>
     </row>
     <row r="5">
@@ -4790,16 +4850,16 @@
         <v>210000</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.403600000000001</v>
+        <v>9.4945</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>172594.5019168</v>
+        <v>174262.888516</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>-37405.49808319999</v>
+        <v>-35737.11148399999</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>-0.1781214194438095</v>
+        <v>-0.1701767213523809</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>9.4939</v>
@@ -4965,6 +5025,9 @@
       </c>
       <c r="BN5" s="3" t="n">
         <v>9.403600000000001</v>
+      </c>
+      <c r="BO5" s="3" t="n">
+        <v>9.4945</v>
       </c>
     </row>
     <row r="6">
@@ -4990,16 +5053,16 @@
         <v>50000</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>11.85</v>
+        <v>11.9935</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>50113.37745</v>
+        <v>50720.23564949999</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>113.37745</v>
+        <v>720.2356494999913</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0.002267548999999999</v>
+        <v>0.01440471298999983</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>12.5421</v>
@@ -5171,6 +5234,9 @@
       </c>
       <c r="BN6" s="3" t="n">
         <v>11.85</v>
+      </c>
+      <c r="BO6" s="3" t="n">
+        <v>11.9935</v>
       </c>
     </row>
     <row r="7">
@@ -5372,6 +5438,9 @@
       <c r="BN7" s="3" t="n">
         <v>34.4039</v>
       </c>
+      <c r="BO7" s="3" t="n">
+        <v>34.4039</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5396,16 +5465,16 @@
         <v>50000</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>33.7817</v>
+        <v>33.9865</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>54205.8793481</v>
+        <v>54534.4999945</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>4205.879348100003</v>
+        <v>4534.499994500002</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.08411758696200006</v>
+        <v>0.09068999989000004</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>30.6804</v>
@@ -5577,6 +5646,9 @@
       </c>
       <c r="BN8" s="3" t="n">
         <v>33.7817</v>
+      </c>
+      <c r="BO8" s="3" t="n">
+        <v>33.9865</v>
       </c>
     </row>
     <row r="9">
@@ -5778,6 +5850,9 @@
       <c r="BN9" s="3" t="n">
         <v>42.2188</v>
       </c>
+      <c r="BO9" s="3" t="n">
+        <v>42.2188</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5978,6 +6053,9 @@
       <c r="BN10" s="3" t="n">
         <v>48.1125</v>
       </c>
+      <c r="BO10" s="3" t="n">
+        <v>48.1125</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -6002,16 +6080,16 @@
         <v>30000</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>106.0056</v>
+        <v>105.9243</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31899.0991464</v>
+        <v>31874.6344317</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>1899.0991464</v>
+        <v>1874.6344317</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0.06330330487999999</v>
+        <v>0.06248781439000001</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>103.8679</v>
@@ -6177,6 +6255,9 @@
       </c>
       <c r="BN11" s="3" t="n">
         <v>106.0056</v>
+      </c>
+      <c r="BO11" s="3" t="n">
+        <v>105.9243</v>
       </c>
     </row>
     <row r="12">
@@ -6202,16 +6283,16 @@
         <v>100000</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>228.93</v>
+        <v>231.97</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>106571.95146</v>
+        <v>107987.13834</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>6571.951459999997</v>
+        <v>7987.13833999999</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0.06571951459999996</v>
+        <v>0.0798713833999999</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>218.889</v>
@@ -6383,6 +6464,9 @@
       </c>
       <c r="BN12" s="3" t="n">
         <v>228.93</v>
+      </c>
+      <c r="BO12" s="3" t="n">
+        <v>231.97</v>
       </c>
     </row>
     <row r="13">
@@ -6408,16 +6492,16 @@
         <v>200000</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>21.313</v>
+        <v>21.354</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>246966.625365</v>
+        <v>247441.71717</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>46966.62536499999</v>
+        <v>47441.71716999999</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0.2348331268249999</v>
+        <v>0.2372085858499999</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>19.888</v>
@@ -6589,6 +6673,9 @@
       </c>
       <c r="BN13" s="3" t="n">
         <v>21.313</v>
+      </c>
+      <c r="BO13" s="3" t="n">
+        <v>21.354</v>
       </c>
     </row>
     <row r="14">
@@ -6614,16 +6701,16 @@
         <v>100000</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>37.888</v>
+        <v>38.061</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>136684.976128</v>
+        <v>137309.091966</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>36684.97612800001</v>
+        <v>37309.09196600001</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0.3668497612800001</v>
+        <v>0.3730909196600001</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>38.9826</v>
@@ -6789,6 +6876,9 @@
       </c>
       <c r="BN14" s="3" t="n">
         <v>37.888</v>
+      </c>
+      <c r="BO14" s="3" t="n">
+        <v>38.061</v>
       </c>
     </row>
     <row r="15">
@@ -6814,16 +6904,16 @@
         <v>100000</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>11.66</v>
+        <v>11.78</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>113614.42202</v>
+        <v>114783.69566</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>13614.42202</v>
+        <v>14783.69566</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0.1361442202</v>
+        <v>0.1478369566</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>11.76</v>
@@ -6995,6 +7085,9 @@
       </c>
       <c r="BN15" s="3" t="n">
         <v>11.66</v>
+      </c>
+      <c r="BO15" s="3" t="n">
+        <v>11.78</v>
       </c>
     </row>
     <row r="16">
@@ -7020,16 +7113,16 @@
         <v>100000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.6669</v>
+        <v>24.7318</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>141166.8926832</v>
+        <v>141538.3107104</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>41166.89268319999</v>
+        <v>41538.31071039999</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0.4116689268319998</v>
+        <v>0.4153831071039999</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>24.4436</v>
@@ -7195,6 +7288,9 @@
       </c>
       <c r="BN16" s="3" t="n">
         <v>24.6669</v>
+      </c>
+      <c r="BO16" s="3" t="n">
+        <v>24.7318</v>
       </c>
     </row>
     <row r="17">
@@ -7220,16 +7316,16 @@
         <v>50000</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>16.8767</v>
+        <v>16.974</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>55795.33217189999</v>
+        <v>56117.011518</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>5795.332171899994</v>
+        <v>6117.011517999999</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>0.1159066434379999</v>
+        <v>0.12234023036</v>
       </c>
       <c r="J17" s="3" t="n">
         <v>16.7178</v>
@@ -7395,6 +7491,9 @@
       </c>
       <c r="BN17" s="3" t="n">
         <v>16.8767</v>
+      </c>
+      <c r="BO17" s="3" t="n">
+        <v>16.974</v>
       </c>
     </row>
     <row r="18">
@@ -7420,16 +7519,16 @@
         <v>80000</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>46.92</v>
+        <v>47.31</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>88511.57712</v>
+        <v>89247.28716000001</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>8511.577120000002</v>
+        <v>9247.287160000007</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>0.106394714</v>
+        <v>0.1155910895000001</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>45.31</v>
@@ -7601,6 +7700,9 @@
       </c>
       <c r="BN18" s="3" t="n">
         <v>46.92</v>
+      </c>
+      <c r="BO18" s="3" t="n">
+        <v>47.31</v>
       </c>
     </row>
     <row r="19">
@@ -7626,16 +7728,16 @@
         <v>150000</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>13.8131</v>
+        <v>14.1214</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>199830.8854346</v>
+        <v>204290.9893924</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>49830.8854346</v>
+        <v>54290.98939239999</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0.3322059028973333</v>
+        <v>0.3619399292826666</v>
       </c>
       <c r="J19" s="3" t="n">
         <v>14.6788</v>
@@ -7801,6 +7903,9 @@
       </c>
       <c r="BN19" s="3" t="n">
         <v>13.8131</v>
+      </c>
+      <c r="BO19" s="3" t="n">
+        <v>14.1214</v>
       </c>
     </row>
     <row r="20">
@@ -7826,16 +7931,16 @@
         <v>250000</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9.44</v>
+        <v>9.58</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>247854.78032</v>
-      </c>
-      <c r="H20" s="6" t="n">
-        <v>-2145.219680000009</v>
-      </c>
-      <c r="I20" s="13" t="n">
-        <v>-0.008580878720000037</v>
+        <v>251530.59274</v>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>1530.592739999993</v>
+      </c>
+      <c r="I20" s="12" t="n">
+        <v>0.006122370959999971</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>9.039999999999999</v>
@@ -8007,6 +8112,9 @@
       </c>
       <c r="BN20" s="3" t="n">
         <v>9.44</v>
+      </c>
+      <c r="BO20" s="3" t="n">
+        <v>9.58</v>
       </c>
     </row>
     <row r="21">
@@ -8032,16 +8140,16 @@
         <v>170000</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>111.5191</v>
+        <v>112.7512</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>169426.3963469</v>
-      </c>
-      <c r="H21" s="6" t="n">
-        <v>-573.6036530999991</v>
-      </c>
-      <c r="I21" s="13" t="n">
-        <v>-0.003374139135882347</v>
+        <v>171298.2753608</v>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>1298.275360800006</v>
+      </c>
+      <c r="I21" s="12" t="n">
+        <v>0.007636913887058857</v>
       </c>
       <c r="J21" s="3" t="n">
         <v>107.9031</v>
@@ -8213,6 +8321,9 @@
       </c>
       <c r="BN21" s="3" t="n">
         <v>111.5191</v>
+      </c>
+      <c r="BO21" s="3" t="n">
+        <v>112.7512</v>
       </c>
     </row>
     <row r="22">
@@ -8414,6 +8525,9 @@
       <c r="BN22" s="3" t="n">
         <v>42.955</v>
       </c>
+      <c r="BO22" s="3" t="n">
+        <v>42.955</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -8438,16 +8552,16 @@
         <v>150000</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>63.0612</v>
+        <v>63.6749</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>171303.6687804</v>
+        <v>172970.7645783</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>21303.66878040001</v>
+        <v>22970.7645783</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0.1420244585360001</v>
+        <v>0.153138430522</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>60.3775</v>
@@ -8619,6 +8733,9 @@
       </c>
       <c r="BN23" s="3" t="n">
         <v>63.0612</v>
+      </c>
+      <c r="BO23" s="3" t="n">
+        <v>63.6749</v>
       </c>
     </row>
     <row r="24">
@@ -8644,16 +8761,16 @@
         <v>100000</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>27.3285</v>
+        <v>27.6997</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>99294.98930099999</v>
-      </c>
-      <c r="H24" s="6" t="n">
-        <v>-705.0106990000058</v>
-      </c>
-      <c r="I24" s="13" t="n">
-        <v>-0.007050106990000058</v>
+        <v>100643.7021842</v>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>643.7021841999958</v>
+      </c>
+      <c r="I24" s="12" t="n">
+        <v>0.006437021841999958</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>28.2458</v>
@@ -8819,6 +8936,9 @@
       </c>
       <c r="BN24" s="3" t="n">
         <v>27.3285</v>
+      </c>
+      <c r="BO24" s="3" t="n">
+        <v>27.6997</v>
       </c>
     </row>
     <row r="25">
@@ -8844,16 +8964,16 @@
         <v>200000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>12.0694</v>
+        <v>12.3502</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>198199.7521756</v>
-      </c>
-      <c r="H25" s="6" t="n">
-        <v>-1800.247824400023</v>
-      </c>
-      <c r="I25" s="13" t="n">
-        <v>-0.009001239122000116</v>
+        <v>202810.9582348</v>
+      </c>
+      <c r="H25" s="4" t="n">
+        <v>2810.958234799968</v>
+      </c>
+      <c r="I25" s="12" t="n">
+        <v>0.01405479117399984</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>11.2082</v>
@@ -9022,6 +9142,9 @@
       </c>
       <c r="BN25" s="3" t="n">
         <v>12.0694</v>
+      </c>
+      <c r="BO25" s="3" t="n">
+        <v>12.3502</v>
       </c>
     </row>
     <row r="26">
@@ -9047,16 +9170,16 @@
         <v>110000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>9.5106</v>
+        <v>9.755699999999999</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>113572.874679</v>
+        <v>116499.7890255</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>3572.874679</v>
+        <v>6499.789025499995</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>0.0324806789</v>
+        <v>0.05908899114090904</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>8.626300000000001</v>
@@ -9225,6 +9348,9 @@
       </c>
       <c r="BN26" s="3" t="n">
         <v>9.5106</v>
+      </c>
+      <c r="BO26" s="3" t="n">
+        <v>9.755699999999999</v>
       </c>
     </row>
     <row r="27">
@@ -9250,16 +9376,16 @@
         <v>110000</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>65.92959999999999</v>
+        <v>66.8194</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>106203.355456</v>
+        <v>107636.698684</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-3796.64454400001</v>
+        <v>-2363.301315999997</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>-0.03451495040000009</v>
+        <v>-0.02148455741818179</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>62.0021</v>
@@ -9431,6 +9557,9 @@
       </c>
       <c r="BN27" s="3" t="n">
         <v>65.92959999999999</v>
+      </c>
+      <c r="BO27" s="3" t="n">
+        <v>66.8194</v>
       </c>
     </row>
     <row r="28">
@@ -9456,16 +9585,16 @@
         <v>380000</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>111.2113</v>
+        <v>113.6371</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>367737.6236241</v>
+        <v>375758.9121747</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-12262.3763759</v>
+        <v>-4241.087825299997</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>-0.03226941151552631</v>
+        <v>-0.01116075743499999</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>104.8438</v>
@@ -9637,6 +9766,9 @@
       </c>
       <c r="BN28" s="3" t="n">
         <v>111.2113</v>
+      </c>
+      <c r="BO28" s="3" t="n">
+        <v>113.6371</v>
       </c>
     </row>
     <row r="29">
@@ -9662,16 +9794,16 @@
         <v>100000</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12.2003</v>
+        <v>12.4311</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>117168.0577109</v>
+        <v>119384.5923633</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>17168.0577109</v>
+        <v>19384.59236330001</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.171680577109</v>
+        <v>0.193845923633</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>12.0216</v>
@@ -9837,6 +9969,9 @@
       </c>
       <c r="BN29" s="3" t="n">
         <v>12.2003</v>
+      </c>
+      <c r="BO29" s="3" t="n">
+        <v>12.4311</v>
       </c>
     </row>
     <row r="30">
@@ -9862,16 +9997,16 @@
         <v>100000</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>16.791</v>
+        <v>16.9773</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>124183.902051</v>
+        <v>125561.7509553</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>24183.902051</v>
+        <v>25561.7509553</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.24183902051</v>
+        <v>0.255617509553</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>15.064</v>
@@ -10037,6 +10172,9 @@
       </c>
       <c r="BN30" s="3" t="n">
         <v>16.791</v>
+      </c>
+      <c r="BO30" s="3" t="n">
+        <v>16.9773</v>
       </c>
     </row>
     <row r="31">
@@ -10062,16 +10200,16 @@
         <v>100000</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>410.4736</v>
+        <v>415.9646</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>109218.815488</v>
+        <v>110679.860768</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>9218.815487999993</v>
+        <v>10679.860768</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.09218815487999993</v>
+        <v>0.10679860768</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>413.2552</v>
@@ -10240,6 +10378,9 @@
       </c>
       <c r="BN31" s="3" t="n">
         <v>410.4736</v>
+      </c>
+      <c r="BO31" s="3" t="n">
+        <v>415.9646</v>
       </c>
     </row>
     <row r="32">
@@ -10265,16 +10406,16 @@
         <v>200000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>10.62</v>
+        <v>10.71</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>224506.3752</v>
+        <v>226408.9716</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>24506.37519999998</v>
+        <v>26408.97160000002</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.1225318759999999</v>
+        <v>0.1320448580000001</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>10.1</v>
@@ -10446,6 +10587,9 @@
       </c>
       <c r="BN32" s="3" t="n">
         <v>10.62</v>
+      </c>
+      <c r="BO32" s="3" t="n">
+        <v>10.71</v>
       </c>
     </row>
     <row r="33">
@@ -10471,16 +10615,16 @@
         <v>60000</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>19</v>
+        <v>19.16</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>68089.16</v>
+        <v>68662.54239999999</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>8089.160000000003</v>
+        <v>8662.542399999991</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0.1348193333333334</v>
+        <v>0.1443757066666665</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>17.77</v>
@@ -10646,6 +10790,9 @@
       </c>
       <c r="BN33" s="3" t="n">
         <v>19</v>
+      </c>
+      <c r="BO33" s="3" t="n">
+        <v>19.16</v>
       </c>
     </row>
     <row r="34">
@@ -10671,16 +10818,16 @@
         <v>80000</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>214.6803</v>
+        <v>216.5522</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>75466.7805393</v>
+        <v>76124.8114182</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>-4533.219460699998</v>
+        <v>-3875.188581800001</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>-0.05666524325874998</v>
+        <v>-0.04843985727250001</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>207.806</v>
@@ -10849,6 +10996,9 @@
       </c>
       <c r="BN34" s="3" t="n">
         <v>214.6803</v>
+      </c>
+      <c r="BO34" s="3" t="n">
+        <v>216.5522</v>
       </c>
     </row>
     <row r="35">
@@ -10874,16 +11024,16 @@
         <v>100000</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>15.01</v>
+        <v>15.19</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>107102.69923</v>
+        <v>108387.07537</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>7102.699229999998</v>
+        <v>8387.075369999991</v>
       </c>
       <c r="I35" s="12" t="n">
-        <v>0.07102699229999998</v>
+        <v>0.08387075369999991</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>13.81</v>
@@ -11052,6 +11202,9 @@
       </c>
       <c r="BN35" s="3" t="n">
         <v>15.01</v>
+      </c>
+      <c r="BO35" s="3" t="n">
+        <v>15.19</v>
       </c>
     </row>
     <row r="36">
@@ -11077,16 +11230,16 @@
         <v>150000</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>373.7828</v>
+        <v>375.8957</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>174072.8926568</v>
+        <v>175056.8828642</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>24072.89265680002</v>
+        <v>25056.88286419999</v>
       </c>
       <c r="I36" s="12" t="n">
-        <v>0.1604859510453334</v>
+        <v>0.1670458857613333</v>
       </c>
       <c r="J36" s="3" t="n">
         <v>349.0771</v>
@@ -11255,6 +11408,9 @@
       </c>
       <c r="BN36" s="3" t="n">
         <v>373.7828</v>
+      </c>
+      <c r="BO36" s="3" t="n">
+        <v>375.8957</v>
       </c>
     </row>
     <row r="37">
@@ -11280,16 +11436,16 @@
         <v>50000</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>16.819</v>
+        <v>16.872</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>63288.030091</v>
+        <v>63487.463208</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>13288.030091</v>
+        <v>13487.463208</v>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0.26576060182</v>
+        <v>0.26974926416</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>15.6</v>
@@ -11458,6 +11614,9 @@
       </c>
       <c r="BN37" s="3" t="n">
         <v>16.819</v>
+      </c>
+      <c r="BO37" s="3" t="n">
+        <v>16.872</v>
       </c>
     </row>
     <row r="38">
@@ -11483,16 +11642,16 @@
         <v>80000</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>14.2955</v>
+        <v>14.4706</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>85493.980431</v>
+        <v>86541.1628292</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>5493.980431000004</v>
+        <v>6541.162829199995</v>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0.06867475538750005</v>
+        <v>0.08176453536499993</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>13.9942</v>
@@ -11658,6 +11817,9 @@
       </c>
       <c r="BN38" s="3" t="n">
         <v>14.2955</v>
+      </c>
+      <c r="BO38" s="3" t="n">
+        <v>14.4706</v>
       </c>
     </row>
     <row r="39">
@@ -11683,16 +11845,16 @@
         <v>50000</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1022.5379</v>
+        <v>1023.6046</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>51005.2129899</v>
+        <v>51058.4210526</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>1005.212989899999</v>
+        <v>1058.421052600002</v>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0.02010425979799998</v>
+        <v>0.02116842105200005</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>1008.9183</v>
@@ -11858,6 +12020,9 @@
       </c>
       <c r="BN39" s="3" t="n">
         <v>1022.5379</v>
+      </c>
+      <c r="BO39" s="3" t="n">
+        <v>1023.6046</v>
       </c>
     </row>
     <row r="40">
@@ -11883,16 +12048,16 @@
         <v>100000</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>21.8222</v>
+        <v>22.0645</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>110006.2993994</v>
+        <v>111227.7402415</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>10006.2993994</v>
+        <v>11227.7402415</v>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0.100062993994</v>
+        <v>0.112277402415</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>19.911</v>
@@ -12061,6 +12226,9 @@
       </c>
       <c r="BN40" s="3" t="n">
         <v>21.8222</v>
+      </c>
+      <c r="BO40" s="3" t="n">
+        <v>22.0645</v>
       </c>
     </row>
     <row r="41">
@@ -12073,13 +12241,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>4956779.4405086</v>
+        <v>5008989.9490267</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>486779.4405086</v>
+        <v>538989.9490266999</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1088992036931991</v>
+        <v>0.1205794069410962</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-07-12
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-11 05:11 IST</t>
+          <t>Generated: 2026-07-12 05:25 IST</t>
         </is>
       </c>
     </row>
@@ -544,13 +544,13 @@
         <v>4470000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>5008989.9490267</v>
+        <v>5008308.1836056</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>538989.9490267001</v>
+        <v>538308.1836056001</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1205794069410962</v>
+        <v>0.1204268867126622</v>
       </c>
     </row>
     <row r="6">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5552348.450888272</v>
+        <v>5551666.685467172</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>491566.4308882728</v>
+        <v>490884.6654671729</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.09713250421488671</v>
+        <v>0.09699778878584715</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-07-11</t>
+          <t>Last snapshot: 2026-07-12</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BN19"/>
+  <dimension ref="A1:BO19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -685,6 +685,7 @@
     <col width="21" customWidth="1" min="64" max="64"/>
     <col width="21" customWidth="1" min="65" max="65"/>
     <col width="21" customWidth="1" min="66" max="66"/>
+    <col width="21" customWidth="1" min="67" max="67"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1018,6 +1019,11 @@
           <t>2026-07-11</t>
         </is>
       </c>
+      <c r="BO1" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1219,6 +1225,9 @@
       <c r="BN2" s="3" t="n">
         <v>545.2000122070312</v>
       </c>
+      <c r="BO2" s="3" t="n">
+        <v>545.2000122070312</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1450,6 +1459,9 @@
       <c r="BN4" s="3" t="n">
         <v>1333.800048828125</v>
       </c>
+      <c r="BO4" s="3" t="n">
+        <v>1333.800048828125</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1654,6 +1666,9 @@
       <c r="BN5" s="3" t="n">
         <v>643.2999877929688</v>
       </c>
+      <c r="BO5" s="3" t="n">
+        <v>643.2999877929688</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1858,6 +1873,9 @@
       <c r="BN6" s="3" t="n">
         <v>368.6499938964844</v>
       </c>
+      <c r="BO6" s="3" t="n">
+        <v>368.6499938964844</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2062,6 +2080,9 @@
       <c r="BN7" s="3" t="n">
         <v>239.6399993896484</v>
       </c>
+      <c r="BO7" s="3" t="n">
+        <v>239.6399993896484</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2293,6 +2314,9 @@
       <c r="BN9" s="3" t="n">
         <v>17.02000045776367</v>
       </c>
+      <c r="BO9" s="3" t="n">
+        <v>17.02000045776367</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2497,6 +2521,9 @@
       <c r="BN10" s="3" t="n">
         <v>424.9500122070312</v>
       </c>
+      <c r="BO10" s="3" t="n">
+        <v>424.9500122070312</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2701,6 +2728,9 @@
       <c r="BN11" s="3" t="n">
         <v>9.989999771118164</v>
       </c>
+      <c r="BO11" s="3" t="n">
+        <v>9.989999771118164</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2905,6 +2935,9 @@
       <c r="BN12" s="3" t="n">
         <v>2693.800048828125</v>
       </c>
+      <c r="BO12" s="3" t="n">
+        <v>2693.800048828125</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3109,6 +3142,9 @@
       <c r="BN13" s="3" t="n">
         <v>53.91999816894531</v>
       </c>
+      <c r="BO13" s="3" t="n">
+        <v>53.91999816894531</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3313,6 +3349,9 @@
       <c r="BN14" s="3" t="n">
         <v>721.0499877929688</v>
       </c>
+      <c r="BO14" s="3" t="n">
+        <v>721.0499877929688</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3571,6 +3610,9 @@
       <c r="BN17" s="3" t="n">
         <v>564.6500244140625</v>
       </c>
+      <c r="BO17" s="3" t="n">
+        <v>564.6500244140625</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3773,6 +3815,9 @@
         <v>380.8500061035156</v>
       </c>
       <c r="BN18" s="3" t="n">
+        <v>381.2999877929688</v>
+      </c>
+      <c r="BO18" s="3" t="n">
         <v>381.2999877929688</v>
       </c>
     </row>
@@ -3803,7 +3848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BO41"/>
+  <dimension ref="A1:BP41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3873,6 +3918,7 @@
     <col width="13" customWidth="1" min="65" max="65"/>
     <col width="13" customWidth="1" min="66" max="66"/>
     <col width="13" customWidth="1" min="67" max="67"/>
+    <col width="13" customWidth="1" min="68" max="68"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4211,6 +4257,11 @@
           <t>2026-07-11</t>
         </is>
       </c>
+      <c r="BP1" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -4420,6 +4471,9 @@
       <c r="BO2" s="3" t="n">
         <v>57.4457</v>
       </c>
+      <c r="BP2" s="3" t="n">
+        <v>57.4457</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4623,6 +4677,9 @@
       <c r="BO3" s="3" t="n">
         <v>25.7751</v>
       </c>
+      <c r="BP3" s="3" t="n">
+        <v>25.7751</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4826,6 +4883,9 @@
       <c r="BO4" s="3" t="n">
         <v>12.22</v>
       </c>
+      <c r="BP4" s="3" t="n">
+        <v>12.22</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5029,6 +5089,9 @@
       <c r="BO5" s="3" t="n">
         <v>9.4945</v>
       </c>
+      <c r="BP5" s="3" t="n">
+        <v>9.4945</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -5238,6 +5301,9 @@
       <c r="BO6" s="3" t="n">
         <v>11.9935</v>
       </c>
+      <c r="BP6" s="3" t="n">
+        <v>11.9935</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -5262,16 +5328,16 @@
         <v>60000</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>34.4039</v>
+        <v>34.3308</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>75896.379556</v>
+        <v>75735.11803200001</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>15896.379556</v>
+        <v>15735.11803200001</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.2649396592666667</v>
+        <v>0.2622519672000002</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>33.3317</v>
@@ -5440,6 +5506,9 @@
       </c>
       <c r="BO7" s="3" t="n">
         <v>34.4039</v>
+      </c>
+      <c r="BP7" s="3" t="n">
+        <v>34.3308</v>
       </c>
     </row>
     <row r="8">
@@ -5650,6 +5719,9 @@
       <c r="BO8" s="3" t="n">
         <v>33.9865</v>
       </c>
+      <c r="BP8" s="3" t="n">
+        <v>33.9865</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5674,16 +5746,16 @@
         <v>100000</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>42.2188</v>
+        <v>41.7597</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>135918.9091884</v>
+        <v>134440.8858621</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>35918.90918839999</v>
+        <v>34440.8858621</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0.3591890918839999</v>
+        <v>0.344408858621</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>40.758</v>
@@ -5852,6 +5924,9 @@
       </c>
       <c r="BO9" s="3" t="n">
         <v>42.2188</v>
+      </c>
+      <c r="BP9" s="3" t="n">
+        <v>41.7597</v>
       </c>
     </row>
     <row r="10">
@@ -5877,16 +5952,16 @@
         <v>100000</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>48.1125</v>
+        <v>48.3513</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>136959.8811375</v>
+        <v>137639.6633067</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>36959.88113749999</v>
+        <v>37639.66330670001</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>0.3695988113749999</v>
+        <v>0.3763966330670001</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>45.95</v>
@@ -6055,6 +6130,9 @@
       </c>
       <c r="BO10" s="3" t="n">
         <v>48.1125</v>
+      </c>
+      <c r="BP10" s="3" t="n">
+        <v>48.3513</v>
       </c>
     </row>
     <row r="11">
@@ -6259,6 +6337,9 @@
       <c r="BO11" s="3" t="n">
         <v>105.9243</v>
       </c>
+      <c r="BP11" s="3" t="n">
+        <v>105.9243</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -6468,6 +6549,9 @@
       <c r="BO12" s="3" t="n">
         <v>231.97</v>
       </c>
+      <c r="BP12" s="3" t="n">
+        <v>231.97</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6677,6 +6761,9 @@
       <c r="BO13" s="3" t="n">
         <v>21.354</v>
       </c>
+      <c r="BP13" s="3" t="n">
+        <v>21.354</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -6880,6 +6967,9 @@
       <c r="BO14" s="3" t="n">
         <v>38.061</v>
       </c>
+      <c r="BP14" s="3" t="n">
+        <v>38.061</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -7089,6 +7179,9 @@
       <c r="BO15" s="3" t="n">
         <v>11.78</v>
       </c>
+      <c r="BP15" s="3" t="n">
+        <v>11.78</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -7292,6 +7385,9 @@
       <c r="BO16" s="3" t="n">
         <v>24.7318</v>
       </c>
+      <c r="BP16" s="3" t="n">
+        <v>24.7318</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -7495,6 +7591,9 @@
       <c r="BO17" s="3" t="n">
         <v>16.974</v>
       </c>
+      <c r="BP17" s="3" t="n">
+        <v>16.974</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -7704,6 +7803,9 @@
       <c r="BO18" s="3" t="n">
         <v>47.31</v>
       </c>
+      <c r="BP18" s="3" t="n">
+        <v>47.31</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -7907,6 +8009,9 @@
       <c r="BO19" s="3" t="n">
         <v>14.1214</v>
       </c>
+      <c r="BP19" s="3" t="n">
+        <v>14.1214</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -8116,6 +8221,9 @@
       <c r="BO20" s="3" t="n">
         <v>9.58</v>
       </c>
+      <c r="BP20" s="3" t="n">
+        <v>9.58</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -8325,6 +8433,9 @@
       <c r="BO21" s="3" t="n">
         <v>112.7512</v>
       </c>
+      <c r="BP21" s="3" t="n">
+        <v>112.7512</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -8349,16 +8460,16 @@
         <v>60000</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>42.955</v>
+        <v>43.136</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>65912.72929999999</v>
+        <v>66190.46656</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>5912.729299999992</v>
+        <v>6190.466560000001</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0.09854548833333319</v>
+        <v>0.1031744426666667</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>43.8</v>
@@ -8527,6 +8638,9 @@
       </c>
       <c r="BO22" s="3" t="n">
         <v>42.955</v>
+      </c>
+      <c r="BP22" s="3" t="n">
+        <v>43.136</v>
       </c>
     </row>
     <row r="23">
@@ -8737,6 +8851,9 @@
       <c r="BO23" s="3" t="n">
         <v>63.6749</v>
       </c>
+      <c r="BP23" s="3" t="n">
+        <v>63.6749</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -8940,6 +9057,9 @@
       <c r="BO24" s="3" t="n">
         <v>27.6997</v>
       </c>
+      <c r="BP24" s="3" t="n">
+        <v>27.6997</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -9146,6 +9266,9 @@
       <c r="BO25" s="3" t="n">
         <v>12.3502</v>
       </c>
+      <c r="BP25" s="3" t="n">
+        <v>12.3502</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -9352,6 +9475,9 @@
       <c r="BO26" s="3" t="n">
         <v>9.755699999999999</v>
       </c>
+      <c r="BP26" s="3" t="n">
+        <v>9.755699999999999</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -9561,6 +9687,9 @@
       <c r="BO27" s="3" t="n">
         <v>66.8194</v>
       </c>
+      <c r="BP27" s="3" t="n">
+        <v>66.8194</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -9770,6 +9899,9 @@
       <c r="BO28" s="3" t="n">
         <v>113.6371</v>
       </c>
+      <c r="BP28" s="3" t="n">
+        <v>113.6371</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -9973,6 +10105,9 @@
       <c r="BO29" s="3" t="n">
         <v>12.4311</v>
       </c>
+      <c r="BP29" s="3" t="n">
+        <v>12.4311</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -10176,6 +10311,9 @@
       <c r="BO30" s="3" t="n">
         <v>16.9773</v>
       </c>
+      <c r="BP30" s="3" t="n">
+        <v>16.9773</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -10382,6 +10520,9 @@
       <c r="BO31" s="3" t="n">
         <v>415.9646</v>
       </c>
+      <c r="BP31" s="3" t="n">
+        <v>415.9646</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -10591,6 +10732,9 @@
       <c r="BO32" s="3" t="n">
         <v>10.71</v>
       </c>
+      <c r="BP32" s="3" t="n">
+        <v>10.71</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -10794,6 +10938,9 @@
       <c r="BO33" s="3" t="n">
         <v>19.16</v>
       </c>
+      <c r="BP33" s="3" t="n">
+        <v>19.16</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -11000,6 +11147,9 @@
       <c r="BO34" s="3" t="n">
         <v>216.5522</v>
       </c>
+      <c r="BP34" s="3" t="n">
+        <v>216.5522</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -11206,6 +11356,9 @@
       <c r="BO35" s="3" t="n">
         <v>15.19</v>
       </c>
+      <c r="BP35" s="3" t="n">
+        <v>15.19</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -11412,6 +11565,9 @@
       <c r="BO36" s="3" t="n">
         <v>375.8957</v>
       </c>
+      <c r="BP36" s="3" t="n">
+        <v>375.8957</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -11618,6 +11774,9 @@
       <c r="BO37" s="3" t="n">
         <v>16.872</v>
       </c>
+      <c r="BP37" s="3" t="n">
+        <v>16.872</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -11821,6 +11980,9 @@
       <c r="BO38" s="3" t="n">
         <v>14.4706</v>
       </c>
+      <c r="BP38" s="3" t="n">
+        <v>14.4706</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -12024,6 +12186,9 @@
       <c r="BO39" s="3" t="n">
         <v>1023.6046</v>
       </c>
+      <c r="BP39" s="3" t="n">
+        <v>1023.6046</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -12230,6 +12395,9 @@
       <c r="BO40" s="3" t="n">
         <v>22.0645</v>
       </c>
+      <c r="BP40" s="3" t="n">
+        <v>22.0645</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
@@ -12241,13 +12409,13 @@
         <v>4470000</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>5008989.9490267</v>
+        <v>5008308.1836056</v>
       </c>
       <c r="H41" s="14" t="n">
-        <v>538989.9490266999</v>
+        <v>538308.1836055999</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0.1205794069410962</v>
+        <v>0.1204268867126622</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily portfolio update 2026-07-13
</commit_message>
<xml_diff>
--- a/portfolio_report.xlsx
+++ b/portfolio_report.xlsx
@@ -39,10 +39,10 @@
       <sz val="10"/>
     </font>
     <font>
-      <color rgb="009C0006"/>
+      <color rgb="00006100"/>
     </font>
     <font>
-      <color rgb="00006100"/>
+      <color rgb="009C0006"/>
     </font>
     <font>
       <b val="1"/>
@@ -97,9 +97,9 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -109,8 +109,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-12 05:25 IST</t>
+          <t>Generated: 2026-07-13 05:35 IST</t>
         </is>
       </c>
     </row>
@@ -566,13 +566,13 @@
         <v>590782.02</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>543358.5018615723</v>
+        <v>544374.496887207</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>-47423.51813842775</v>
+        <v>-46407.52311279299</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.08027244657585847</v>
+        <v>-0.07855270055915545</v>
       </c>
     </row>
     <row r="7">
@@ -588,20 +588,20 @@
         <v>5060782.02</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5551666.685467172</v>
+        <v>5552682.680492807</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>490884.6654671729</v>
+        <v>491900.6604928076</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.09699778878584715</v>
+        <v>0.0971985472894973</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Last snapshot: 2026-07-12</t>
+          <t>Last snapshot: 2026-07-13</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BO19"/>
+  <dimension ref="A1:BP19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -686,6 +686,7 @@
     <col width="21" customWidth="1" min="65" max="65"/>
     <col width="21" customWidth="1" min="66" max="66"/>
     <col width="21" customWidth="1" min="67" max="67"/>
+    <col width="21" customWidth="1" min="68" max="68"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1024,6 +1025,11 @@
           <t>2026-07-12</t>
         </is>
       </c>
+      <c r="BP1" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1043,13 +1049,13 @@
         <v>43817.51</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>545.2000122070312</v>
+        <v>585.2999877929688</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>43616.0009765625</v>
-      </c>
-      <c r="G2" s="6" t="n">
-        <v>-201.509023437502</v>
+        <v>46823.9990234375</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>3006.489023437498</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>539.75</v>
@@ -1227,6 +1233,9 @@
       </c>
       <c r="BO2" s="3" t="n">
         <v>545.2000122070312</v>
+      </c>
+      <c r="BP2" s="3" t="n">
+        <v>585.2999877929688</v>
       </c>
     </row>
     <row r="3">
@@ -1274,13 +1283,13 @@
         <v>32104.58</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1333.800048828125</v>
+        <v>1321.599975585938</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>26676.0009765625</v>
+        <v>26431.99951171875</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-5428.579023437502</v>
+        <v>-5672.580488281252</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1561.300048828125</v>
@@ -1461,6 +1470,9 @@
       </c>
       <c r="BO4" s="3" t="n">
         <v>1333.800048828125</v>
+      </c>
+      <c r="BP4" s="3" t="n">
+        <v>1321.599975585938</v>
       </c>
     </row>
     <row r="5">
@@ -1481,13 +1493,13 @@
         <v>14213.1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>643.2999877929688</v>
+        <v>646.75</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>12865.99975585938</v>
+        <v>12935</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>-1347.100244140625</v>
+        <v>-1278.1</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>649.7999877929688</v>
@@ -1668,6 +1680,9 @@
       </c>
       <c r="BO5" s="3" t="n">
         <v>643.2999877929688</v>
+      </c>
+      <c r="BP5" s="3" t="n">
+        <v>646.75</v>
       </c>
     </row>
     <row r="6">
@@ -1688,13 +1703,13 @@
         <v>17502.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>368.6499938964844</v>
+        <v>369.1000061035156</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>14745.99975585938</v>
+        <v>14764.00024414062</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-2756.240244140627</v>
+        <v>-2738.239755859377</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>401</v>
@@ -1875,6 +1890,9 @@
       </c>
       <c r="BO6" s="3" t="n">
         <v>368.6499938964844</v>
+      </c>
+      <c r="BP6" s="3" t="n">
+        <v>369.1000061035156</v>
       </c>
     </row>
     <row r="7">
@@ -1895,13 +1913,13 @@
         <v>26433.82</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>239.6399993896484</v>
+        <v>236.8000030517578</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>23963.99993896484</v>
+        <v>23680.00030517578</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-2469.820061035156</v>
+        <v>-2753.819694824218</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>254.0500030517578</v>
@@ -2082,6 +2100,9 @@
       </c>
       <c r="BO7" s="3" t="n">
         <v>239.6399993896484</v>
+      </c>
+      <c r="BP7" s="3" t="n">
+        <v>236.8000030517578</v>
       </c>
     </row>
     <row r="8">
@@ -2129,13 +2150,13 @@
         <v>31050.17</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>17.02000045776367</v>
+        <v>16.80999946594238</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>25530.00068664551</v>
+        <v>25214.99919891357</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-5520.16931335449</v>
+        <v>-5835.170801086424</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>17.86000061035156</v>
@@ -2316,6 +2337,9 @@
       </c>
       <c r="BO9" s="3" t="n">
         <v>17.02000045776367</v>
+      </c>
+      <c r="BP9" s="3" t="n">
+        <v>16.80999946594238</v>
       </c>
     </row>
     <row r="10">
@@ -2336,13 +2360,13 @@
         <v>51498.48</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>424.9500122070312</v>
+        <v>425.3500061035156</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>42495.00122070312</v>
+        <v>42535.00061035156</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>-9003.478779296878</v>
+        <v>-8963.479389648441</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>517.5499877929688</v>
@@ -2523,6 +2547,9 @@
       </c>
       <c r="BO10" s="3" t="n">
         <v>424.9500122070312</v>
+      </c>
+      <c r="BP10" s="3" t="n">
+        <v>425.3500061035156</v>
       </c>
     </row>
     <row r="11">
@@ -2543,13 +2570,13 @@
         <v>9841.209999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>9.989999771118164</v>
+        <v>9.939999580383301</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>9989.999771118164</v>
+        <v>9939.999580383301</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>148.7897711181649</v>
+        <v>98.78958038330165</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>8.510000228881836</v>
@@ -2730,6 +2757,9 @@
       </c>
       <c r="BO11" s="3" t="n">
         <v>9.989999771118164</v>
+      </c>
+      <c r="BP11" s="3" t="n">
+        <v>9.939999580383301</v>
       </c>
     </row>
     <row r="12">
@@ -2750,13 +2780,13 @@
         <v>27723.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2693.800048828125</v>
+        <v>2710.199951171875</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>26938.00048828125</v>
+        <v>27101.99951171875</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-785.24951171875</v>
+        <v>-621.25048828125</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>2888.60009765625</v>
@@ -2937,6 +2967,9 @@
       </c>
       <c r="BO12" s="3" t="n">
         <v>2693.800048828125</v>
+      </c>
+      <c r="BP12" s="3" t="n">
+        <v>2710.199951171875</v>
       </c>
     </row>
     <row r="13">
@@ -2957,13 +2990,13 @@
         <v>35031.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>53.91999816894531</v>
+        <v>53.16999816894531</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>32351.99890136719</v>
+        <v>31901.99890136719</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>-2679.761098632815</v>
+        <v>-3129.761098632815</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>53.47000122070312</v>
@@ -3144,6 +3177,9 @@
       </c>
       <c r="BO13" s="3" t="n">
         <v>53.91999816894531</v>
+      </c>
+      <c r="BP13" s="3" t="n">
+        <v>53.16999816894531</v>
       </c>
     </row>
     <row r="14">
@@ -3164,13 +3200,13 @@
         <v>42462.51</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>721.0499877929688</v>
+        <v>714.2000122070312</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>36052.49938964844</v>
+        <v>35710.00061035156</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-6410.010610351565</v>
+        <v>-6752.50938964844</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>757.0999755859375</v>
@@ -3351,6 +3387,9 @@
       </c>
       <c r="BO14" s="3" t="n">
         <v>721.0499877929688</v>
+      </c>
+      <c r="BP14" s="3" t="n">
+        <v>714.2000122070312</v>
       </c>
     </row>
     <row r="15">
@@ -3425,13 +3464,13 @@
         <v>21754.53</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>564.6500244140625</v>
+        <v>556</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>28232.50122070312</v>
+        <v>27800</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>6477.971220703126</v>
+        <v>6045.470000000001</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>458.0499877929688</v>
@@ -3612,6 +3651,9 @@
       </c>
       <c r="BO17" s="3" t="n">
         <v>564.6500244140625</v>
+      </c>
+      <c r="BP17" s="3" t="n">
+        <v>556</v>
       </c>
     </row>
     <row r="18">
@@ -3632,13 +3674,13 @@
         <v>46640.82</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>381.2999877929688</v>
+        <v>377.6499938964844</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>38129.99877929688</v>
+        <v>37764.99938964844</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-8510.821220703125</v>
+        <v>-8875.820610351562</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>407.8500061035156</v>
@@ -3819,6 +3861,9 @@
       </c>
       <c r="BO18" s="3" t="n">
         <v>381.2999877929688</v>
+      </c>
+      <c r="BP18" s="3" t="n">
+        <v>377.6499938964844</v>
       </c>
     </row>
     <row r="19">
@@ -3831,10 +3876,10 @@
         <v>590782.02</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>543358.5018615723</v>
+        <v>544374.496887207</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>-47423.51813842775</v>
+        <v>-46407.52311279298</v>
       </c>
     </row>
   </sheetData>
@@ -3848,7 +3893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BP41"/>
+  <dimension ref="A1:BQ41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3919,6 +3964,7 @@
     <col width="13" customWidth="1" min="66" max="66"/>
     <col width="13" customWidth="1" min="67" max="67"/>
     <col width="13" customWidth="1" min="68" max="68"/>
+    <col width="13" customWidth="1" min="69" max="69"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4262,6 +4308,11 @@
           <t>2026-07-12</t>
         </is>
       </c>
+      <c r="BQ1" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -4474,6 +4525,9 @@
       <c r="BP2" s="3" t="n">
         <v>57.4457</v>
       </c>
+      <c r="BQ2" s="3" t="n">
+        <v>57.4457</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4680,6 +4734,9 @@
       <c r="BP3" s="3" t="n">
         <v>25.7751</v>
       </c>
+      <c r="BQ3" s="3" t="n">
+        <v>25.7751</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4886,6 +4943,9 @@
       <c r="BP4" s="3" t="n">
         <v>12.22</v>
       </c>
+      <c r="BQ4" s="3" t="n">
+        <v>12.22</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5092,6 +5152,9 @@
       <c r="BP5" s="3" t="n">
         <v>9.4945</v>
       </c>
+      <c r="BQ5" s="3" t="n">
+        <v>9.4945</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -5304,6 +5367,9 @@
       <c r="BP6" s="3" t="n">
         <v>11.9935</v>
       </c>
+      <c r="BQ6" s="3" t="n">
+        <v>11.9935</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -5510,6 +5576,9 @@
       <c r="BP7" s="3" t="n">
         <v>34.3308</v>
       </c>
+      <c r="BQ7" s="3" t="n">
+        <v>34.3308</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5722,6 +5791,9 @@
       <c r="BP8" s="3" t="n">
         <v>33.9865</v>
       </c>
+      <c r="BQ8" s="3" t="n">
+        <v>33.9865</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5928,6 +6000,9 @@
       <c r="BP9" s="3" t="n">
         <v>41.7597</v>
       </c>
+      <c r="BQ9" s="3" t="n">
+        <v>41.7597</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -6134,6 +6209,9 @@
       <c r="BP10" s="3" t="n">
         <v>48.3513</v>
       </c>
+      <c r="BQ10" s="3" t="n">
+        <v>48.3513</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -6340,6 +6418,9 @@
       <c r="BP11" s="3" t="n">
         <v>105.9243</v>
       </c>
+      <c r="BQ11" s="3" t="n">
+        <v>105.9243</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -6552,6 +6633,9 @@
       <c r="BP12" s="3" t="n">
         <v>231.97</v>
       </c>
+      <c r="BQ12" s="3" t="n">
+        <v>231.97</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6764,6 +6848,9 @@
       <c r="BP13" s="3" t="n">
         <v>21.354</v>
       </c>
+      <c r="BQ13" s="3" t="n">
+        <v>21.354</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -6970,6 +7057,9 @@
       <c r="BP14" s="3" t="n">
         <v>38.061</v>
       </c>
+      <c r="BQ14" s="3" t="n">
+        <v>38.061</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -7182,6 +7272,9 @@
       <c r="BP15" s="3" t="n">
         <v>11.78</v>
       </c>
+      <c r="BQ15" s="3" t="n">
+        <v>11.78</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -7388,6 +7481,9 @@
       <c r="BP16" s="3" t="n">
         <v>24.7318</v>
       </c>
+      <c r="BQ16" s="3" t="n">
+        <v>24.7318</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -7594,6 +7690,9 @@
       <c r="BP17" s="3" t="n">
         <v>16.974</v>
       </c>
+      <c r="BQ17" s="3" t="n">
+        <v>16.974</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -7806,6 +7905,9 @@
       <c r="BP18" s="3" t="n">
         <v>47.31</v>
       </c>
+      <c r="BQ18" s="3" t="n">
+        <v>47.31</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -8012,6 +8114,9 @@
       <c r="BP19" s="3" t="n">
         <v>14.1214</v>
       </c>
+      <c r="BQ19" s="3" t="n">
+        <v>14.1214</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -8224,6 +8329,9 @@
       <c r="BP20" s="3" t="n">
         <v>9.58</v>
       </c>
+      <c r="BQ20" s="3" t="n">
+        <v>9.58</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -8436,6 +8544,9 @@
       <c r="BP21" s="3" t="n">
         <v>112.7512</v>
       </c>
+      <c r="BQ21" s="3" t="n">
+        <v>112.7512</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -8642,6 +8753,9 @@
       <c r="BP22" s="3" t="n">
         <v>43.136</v>
       </c>
+      <c r="BQ22" s="3" t="n">
+        <v>43.136</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -8854,6 +8968,9 @@
       <c r="BP23" s="3" t="n">
         <v>63.6749</v>
       </c>
+      <c r="BQ23" s="3" t="n">
+        <v>63.6749</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -9060,6 +9177,9 @@
       <c r="BP24" s="3" t="n">
         <v>27.6997</v>
       </c>
+      <c r="BQ24" s="3" t="n">
+        <v>27.6997</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -9269,6 +9389,9 @@
       <c r="BP25" s="3" t="n">
         <v>12.3502</v>
       </c>
+      <c r="BQ25" s="3" t="n">
+        <v>12.3502</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -9478,6 +9601,9 @@
       <c r="BP26" s="3" 